<commit_message>
chore: cleanup variable nomenclature
</commit_message>
<xml_diff>
--- a/XL-Int.xlsx
+++ b/XL-Int.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\foolu\Workspace\Excel\xl-int\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2273CAF-7F9F-4B41-9A4D-4B0FE9B4C2E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61FEFC49-7320-41B5-95F3-BA9301FA05E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21220" xr2:uid="{36490472-0618-4E80-9469-F609392FABC8}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="24580" windowHeight="21000" xr2:uid="{36490472-0618-4E80-9469-F609392FABC8}"/>
   </bookViews>
   <sheets>
     <sheet name="Tests" sheetId="1" r:id="rId1"/>
@@ -19,52 +19,52 @@
     <sheet name="Sheet1" sheetId="6" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="BigInt.Abs" comment="Returns the unsigned magnitude of a BigInt string (absolute value)._x000a_@param big_int The BigInt string.">_xlfn.LAMBDA(_xlpm.big_int, _xlfn.LET(_xlpm.num, BigInt.Norm(_xlpm.big_int), IF(LEFT(_xlpm.num) = "-", MID(_xlpm.num, 2, LEN(_xlpm.num) - 1), _xlpm.num)))</definedName>
-    <definedName name="BigInt.Add" comment="Adds two BigInt strings._x000a_@param big_int_a The first BigInt string._x000a_@param big_int_b The second BigInt string.">_xlfn.LAMBDA(_xlpm.big_int_a,_xlpm.big_int_b, _xlfn.LET(_xlpm.norm_a, BigInt.Norm(_xlpm.big_int_a), _xlpm.norm_b, BigInt.Norm(_xlpm.big_int_b), _xlpm.sign_a, BigInt.Sign(_xlpm.norm_a), _xlpm.sign_b, BigInt.Sign(_xlpm.norm_b), _xlpm.k, core_BigInt.SafeK("ADD"), _xlpm.limbs_a, core_BigInt.Split(BigInt.Abs(_xlpm.norm_a), _xlpm.k), _xlpm.limbs_b, core_BigInt.Split(BigInt.Abs(_xlpm.norm_b), _xlpm.k), _xlpm.routed, core_BigInt.AddSubRouter(_xlpm.limbs_a, _xlpm.limbs_b, _xlpm.sign_a, _xlpm.sign_b, _xlpm.k), _xlpm.final_sign, _xlfn.CHOOSEROWS(_xlpm.routed, -1), _xlpm.final_limbs, _xlfn.DROP(_xlpm.routed, -1), _xlpm.merged, core_BigInt.Merge(_xlpm.final_limbs, _xlpm.k), IF(_xlpm.final_sign = -1, "-" &amp; _xlpm.merged, _xlpm.merged)))</definedName>
-    <definedName name="BigInt.Compare" comment="Compares two BigInt strings. Returns 1 (a &gt; b), -1 (a &lt; b), or 0 (a = b)._x000a_Evaluates signs and lengths. If identical, delegates to native limb array comparison._x000a_@param big_int_a The first BigInt string._x000a_@param big_int_b The second BigInt string.">_xlfn.LAMBDA(_xlpm.big_int_a,_xlpm.big_int_b, _xlfn.LET(_xlpm.norm_a, BigInt.Norm(_xlpm.big_int_a), _xlpm.norm_b, BigInt.Norm(_xlpm.big_int_b), _xlpm.sign_a, BigInt.Sign(_xlpm.norm_a), _xlpm.sign_b, BigInt.Sign(_xlpm.norm_b), IF(_xlpm.sign_a &lt;&gt; _xlpm.sign_b, SIGN(_xlpm.sign_a - _xlpm.sign_b), IF(_xlpm.sign_a = 0, 0, _xlfn.LET(_xlpm.len_a, LEN(_xlpm.norm_a), _xlpm.len_b, LEN(_xlpm.norm_b), IF(_xlpm.len_a &lt;&gt; _xlpm.len_b, SIGN(_xlpm.len_a - _xlpm.len_b) * _xlpm.sign_a, _xlfn.LET(_xlpm.k, core_BigInt.SafeK("ADD"), _xlpm.limbs_a, core_BigInt.Split(BigInt.Abs(_xlpm.norm_a), _xlpm.k), _xlpm.limbs_b, core_BigInt.Split(BigInt.Abs(_xlpm.norm_b), _xlpm.k), _xlpm.mag_comparison, core_BigInt.UCompare(_xlpm.limbs_a, _xlpm.limbs_b), _xlpm.mag_comparison * _xlpm.sign_a)))))))</definedName>
-    <definedName name="BigInt.Div" comment="Divides the first BigInt by the second (A / B). _x000a_@param big_int_a The dividend BigInt string._x000a_@param big_int_b The divisor BigInt string._x000a_@param [use_floor] Optional boolean. TRUE for Python-style Floor division. Defaults to FALSE.">_xlfn.LAMBDA(_xlpm.big_int_a,_xlpm.big_int_b,_xlop.use_floor, INDEX(BigInt.DivMod(_xlpm.big_int_a, _xlpm.big_int_b, _xlpm.use_floor), 1, 1))</definedName>
-    <definedName name="BigInt.DivMod" comment="Divides the first BigInt by the second (A / B). _x000a_Returns the quotient and modulus in rows 1 and 2, respectively._x000a_@param big_int_a The dividend BigInt string._x000a_@param big_int_b The divisor BigInt string._x000a_@param [use_floor] Optional boolean. TRUE for Python-">_xlfn.LAMBDA(_xlpm.big_int_a,_xlpm.big_int_b,_xlop.use_floor, _xlfn.LET(_xlpm.norm_a, BigInt.Norm(_xlpm.big_int_a), _xlpm.norm_b, BigInt.Norm(_xlpm.big_int_b), _xlpm.sign_a, BigInt.Sign(_xlpm.norm_a), _xlpm.sign_b, BigInt.Sign(_xlpm.norm_b), _xlpm.is_floor, IF(_xlfn.ISOMITTED(_xlpm.use_floor), FALSE, _xlpm.use_floor), IF(_xlpm.sign_b = 0, #DIV/0!, IF(_xlpm.sign_a = 0, {"0";"0"}, _xlfn.LET(_xlpm.k, core_BigInt.SafeK("DIV"), _xlpm.limbs_a, core_BigInt.Split(BigInt.Abs(_xlpm.norm_a), _xlpm.k), _xlpm.limbs_b, core_BigInt.Split(BigInt.Abs(_xlpm.norm_b), _xlpm.k), _xlpm.packed_result, core_BigInt.DivRouter(_xlpm.limbs_a, _xlpm.limbs_b, _xlpm.k), _xlpm.len_r, INDEX(_xlpm.packed_result, 1, 1), _xlpm.rem_limbs, _xlfn.CHOOSEROWS(_xlpm.packed_result, _xlfn.SEQUENCE(_xlpm.len_r, 1, 2)), _xlpm.quot_limbs, _xlfn.DROP(_xlpm.packed_result, _xlpm.len_r + 1), _xlpm.final_sign, _xlpm.sign_a * _xlpm.sign_b, _xlpm.merged_q, core_BigInt.Merge(_xlpm.quot_limbs, _xlpm.k), _xlpm.merged_r, core_BigInt.Merge(_xlpm.rem_limbs, _xlpm.k), _xlpm.trunc_q, IF(AND(_xlpm.final_sign = -1, _xlpm.merged_q &lt;&gt; "0"), "-" &amp; _xlpm.merged_q, _xlpm.merged_q), _xlpm.trunc_r, IF(AND(_xlpm.sign_a = -1, _xlpm.merged_r &lt;&gt; "0"), "-" &amp; _xlpm.merged_r, _xlpm.merged_r), _xlpm.needs_correction, AND(_xlpm.is_floor, _xlpm.final_sign = -1, _xlpm.merged_r &lt;&gt; "0"), _xlpm.final_q, IF(_xlpm.needs_correction, BigInt.Sub(_xlpm.trunc_q, "1"), _xlpm.trunc_q), _xlpm.final_r, IF(_xlpm.needs_correction, BigInt.Add(_xlpm.trunc_r, _xlpm.norm_b), _xlpm.trunc_r), _xlfn.VSTACK(_xlpm.final_q, _xlpm.final_r))))))</definedName>
-    <definedName name="BigInt.Fact" comment="Computes the factorial of a BigInt (n!) using Peter Luschny's Prime Swing algorithm._x000a_@param big_int The BigInt string. Maximum supported input is 9273.">_xlfn.LAMBDA(_xlpm.big_int, _xlfn.LET(_xlpm.norm_n, BigInt.Norm(_xlpm.big_int), _xlpm.sign_n, BigInt.Sign(_xlpm.norm_n), IF(_xlpm.sign_n = -1, #NUM!, IF(_xlpm.norm_n = "0", "1", IF(_xlpm.norm_n = "1", "1", IF(LEN(_xlpm.norm_n) &gt; 4, #NUM!, IF(VALUE(_xlpm.norm_n) &gt; 9273, #NUM!, _xlfn.LET(_xlpm.n_val, VALUE(_xlpm.norm_n), _xlpm.global_primes, core_BigInt.NativePrimes(_xlpm.n_val), core_BigInt.PrimeSwingKernel(_xlpm.n_val, _xlpm.global_primes)))))))))</definedName>
-    <definedName name="BigInt.IsEven" comment="Returns TRUE if the BigInt is even._x000a_@param big_int The BigInt string.">_xlfn.LAMBDA(_xlpm.big_int, ISEVEN(VALUE(RIGHT(BigInt.Norm(_xlpm.big_int)))))</definedName>
-    <definedName name="BigInt.IsNeg" comment="Returns TRUE if the BigInt is negative._x000a_@param big_int The BigInt string.">_xlfn.LAMBDA(_xlpm.big_int, LEFT(BigInt.Norm(_xlpm.big_int)) = "-")</definedName>
-    <definedName name="BigInt.IsOdd" comment="Returns TRUE if the BigInt is odd._x000a_@param big_int The BigInt string.">_xlfn.LAMBDA(_xlpm.big_int, ISODD(VALUE(RIGHT(BigInt.Norm(_xlpm.big_int)))))</definedName>
-    <definedName name="BigInt.IsZero" comment="Returns TRUE if the BigInt is exactly zero._x000a_@param big_int The BigInt string.">_xlfn.LAMBDA(_xlpm.big_int, BigInt.Norm(_xlpm.big_int) = "0")</definedName>
-    <definedName name="BigInt.Max" comment="Returns the maximum BigInt from an array or range._x000a_@param range A contiguous range or array of BigInt strings.">_xlfn.LAMBDA(_xlpm.range, _xlfn.LET(_xlpm.clean_col, _xlfn.TOCOL(_xlpm.range, 1), IF(OR(ISERROR(_xlpm.clean_col), ROWS(_xlpm.clean_col) = 0), "0", core_BigInt.TreeCompare(_xlfn.MAP(_xlpm.clean_col, BigInt.Norm), 1))))</definedName>
-    <definedName name="BigInt.Min" comment="Returns the minimum BigInt from an array or range._x000a_@param range A contiguous range or array of BigInt strings.">_xlfn.LAMBDA(_xlpm.range, _xlfn.LET(_xlpm.clean_col, _xlfn.TOCOL(_xlpm.range, 1), IF(OR(ISERROR(_xlpm.clean_col), ROWS(_xlpm.clean_col) = 0), "0", core_BigInt.TreeCompare(_xlfn.MAP(_xlpm.clean_col, BigInt.Norm), -1))))</definedName>
-    <definedName name="BigInt.Mod" comment="Computes the remainder of A / B._x000a_@param big_int_a The dividend BigInt string._x000a_@param big_int_b The divisor BigInt string._x000a_@param [use_floor] Optional boolean. TRUE for Python-style Modulo. Defaults to FALSE.">_xlfn.LAMBDA(_xlpm.big_int_a,_xlpm.big_int_b,_xlop.use_floor, INDEX(BigInt.DivMod(_xlpm.big_int_a, _xlpm.big_int_b, _xlpm.use_floor), 2, 1))</definedName>
-    <definedName name="BigInt.Mul" comment="Multiplies two BigInt strings._x000a_@param big_int_a The first BigInt string._x000a_@param big_int_b The second BigInt string.">_xlfn.LAMBDA(_xlpm.big_int_a,_xlpm.big_int_b, _xlfn.LET(_xlpm.norm_a, BigInt.Norm(_xlpm.big_int_a), _xlpm.norm_b, BigInt.Norm(_xlpm.big_int_b), _xlpm.sign_a, BigInt.Sign(_xlpm.norm_a), _xlpm.sign_b, BigInt.Sign(_xlpm.norm_b), _xlpm.len_a, LEN(_xlpm.norm_a), _xlpm.len_b, LEN(_xlpm.norm_b), IF(OR(_xlpm.sign_a = 0, _xlpm.sign_b = 0), "0", IF(_xlpm.len_a + _xlpm.len_b &gt; 32766, #NUM!, _xlfn.LET(_xlpm.k, core_BigInt.SafeK("MUL", MIN(_xlpm.len_a, _xlpm.len_b)), _xlpm.limbs_a, core_BigInt.Split(BigInt.Abs(_xlpm.norm_a), _xlpm.k), _xlpm.limbs_b, core_BigInt.Split(BigInt.Abs(_xlpm.norm_b), _xlpm.k), _xlpm.final_limbs, core_BigInt.UMul(_xlpm.limbs_a, _xlpm.limbs_b, _xlpm.k), _xlpm.final_sign, _xlpm.sign_a * _xlpm.sign_b, _xlpm.merged, core_BigInt.Merge(_xlpm.final_limbs, _xlpm.k), IF(_xlpm.final_sign = -1, "-" &amp; _xlpm.merged, _xlpm.merged))))))</definedName>
-    <definedName name="BigInt.Norm" comment="Normalises a BigInt string. Strips leading zeros, resolves &quot;-0&quot; to &quot;0&quot;, and throws #VALUE! on invalid characters._x000a_@param big_int The BigInt string.">_xlfn.LAMBDA(_xlpm.big_int, _xlfn.LET(_xlpm.str, IF(OR(_xlfn.ISOMITTED(_xlpm.big_int), _xlpm.big_int = ""), "0", _xlpm.big_int &amp; ""), _xlpm.is_valid, _xlfn.REGEXTEST(_xlpm.str, "^-?\d+$"), _xlpm.stripped, _xlfn.REGEXREPLACE(_xlpm.str, "^(-?)0+(?=\d)", "$1"), IF(NOT(_xlpm.is_valid), VALUE("#VALUE!"), IF(_xlpm.stripped = "-0", "0", _xlpm.stripped))))</definedName>
-    <definedName name="BigInt.Pow" comment="Raises a BigInt base to the power of a BigInt exponent._x000a_@param base The base BigInt string._x000a_@param exponent The exponent BigInt string.">_xlfn.LAMBDA(_xlpm.base,_xlpm.exponent, _xlfn.LET(_xlpm.norm_base, BigInt.Norm(_xlpm.base), _xlpm.norm_exp, BigInt.Norm(_xlpm.exponent), _xlpm.sign_base, BigInt.Sign(_xlpm.norm_base), _xlpm.sign_exp, BigInt.Sign(_xlpm.norm_exp), _xlpm.abs_base, BigInt.Abs(_xlpm.norm_base), _xlpm.abs_exp, BigInt.Abs(_xlpm.norm_exp), _xlpm.is_exp_even, ISEVEN(VALUE(RIGHT(_xlpm.norm_exp, 1))), _xlpm.final_sign, IF(_xlpm.sign_base = -1, IF(_xlpm.is_exp_even, 1, -1), _xlpm.sign_base), IF(_xlpm.abs_base = "0", IF(_xlpm.norm_exp = "0", #NUM!, "0"), IF(_xlpm.abs_base = "1", IF(_xlpm.final_sign = -1, "-1", "1"), IF(_xlpm.sign_exp = -1, "0", IF(_xlpm.norm_exp = "0", "1", IF(LEN(_xlpm.norm_exp) &gt; 6, #NUM!, _xlfn.LET(_xlpm.num_exp, VALUE(_xlpm.norm_exp), _xlpm.base_log10,LOG10(VALUE(LEFT(_xlpm.abs_base, 14))) + MAX(0, LEN(_xlpm.abs_base) - 14), _xlpm.approx_digits, _xlpm.num_exp * _xlpm.base_log10, IF(_xlpm.approx_digits &gt; 32766, #NUM!, _xlfn.LET(_xlpm.k, core_BigInt.SafeK("MUL", _xlpm.approx_digits / 2), _xlpm.limbs_base, core_BigInt.Split(_xlpm.abs_base, _xlpm.k), _xlpm.final_limbs, core_BigInt.UPow(_xlpm.limbs_base, _xlpm.norm_exp, _xlpm.k), _xlpm.merged, core_BigInt.Merge(_xlpm.final_limbs, _xlpm.k), IF(_xlpm.final_sign = -1, "-" &amp; _xlpm.merged, _xlpm.merged)))))))))))</definedName>
-    <definedName name="BigInt.RandBigIntArray" comment="[VOLATILE] Generates a dynamic array of integers as text._x000a_@param [num_rows] array height, default 1._x000a_@param [num_cols] array width, default 1._x000a_@param [min_digits] minimum number of digits, default 16 (min 1 digit)_x000a_@param [max_digits] maximum number of dig">_xlfn.LAMBDA(_xlop.num_rows,_xlop.num_cols,_xlop.min_digits,_xlop.max_digits, _xlfn.LET(_xlpm.n_rows, IF(_xlfn.ISOMITTED(_xlpm.num_rows), 1, _xlpm.num_rows), _xlpm.n_cols, IF(_xlfn.ISOMITTED(_xlpm.num_cols), 1, _xlpm.num_cols), _xlpm.min_len, IF(_xlfn.ISOMITTED(_xlpm.min_digits), 16, MIN(32767, MAX(1, _xlpm.min_digits))), _xlpm.max_len, IF(_xlfn.ISOMITTED(_xlpm.max_digits), 50, MAX(1, MIN(32766, _xlpm.max_digits))), _xlfn.MAP(_xlfn.RANDARRAY(_xlpm.n_rows, _xlpm.n_cols, _xlpm.min_len, _xlpm.max_len, TRUE), _xlfn.LAMBDA(_xlpm.length, _xlfn.LET(_xlpm.sign, CHOOSE(RANDBETWEEN(1, 2), "", "-"), _xlpm.digits, _xlfn.CONCAT(_xlfn.RANDARRAY(1, _xlpm.length, 0, 9, TRUE)), _xlpm.sign &amp; _xlfn.REGEXREPLACE(_xlpm.digits, "^0*", ""))))))</definedName>
-    <definedName name="BigInt.Sign" comment="Returns the sign of a BigInt: 1 (positive), -1 (negative), or 0 (zero)._x000a_@param big_int The BigInt string.">_xlfn.LAMBDA(_xlpm.big_int, _xlfn.LET(_xlpm.normed, BigInt.Norm(_xlpm.big_int), _xlfn.SWITCH(LEFT(_xlpm.normed), "0", 0, "-", -1, 1)))</definedName>
-    <definedName name="BigInt.Sqrt" comment="Calculates the integer square root (floor) of a BigInt._x000a_@param big_int The radicand BigInt string.">_xlfn.LAMBDA(_xlpm.big_int, _xlfn.LET(_xlpm.norm_n, BigInt.Norm(_xlpm.big_int), _xlpm.sign_n, BigInt.Sign(_xlpm.norm_n), IF(_xlpm.sign_n = -1, #NUM!, IF(_xlpm.norm_n = "0", "0", IF(_xlpm.norm_n = "1", "1", _xlfn.LET(_xlpm.len_n, LEN(_xlpm.norm_n), _xlpm.take_digits, IF(_xlpm.len_n &lt;= 14, _xlpm.len_n, IF(ISEVEN(_xlpm.len_n), 14, 13)), _xlpm.v_str, LEFT(_xlpm.norm_n, _xlpm.take_digits), _xlpm.v_num, VALUE(_xlpm.v_str), _xlpm.zero_count, (_xlpm.len_n - _xlpm.take_digits) / 2, _xlpm.seed_prefix, TEXT(ROUNDUP(SQRT(_xlpm.v_num), 0) + 1, "0"), _xlpm.seed_str, _xlpm.seed_prefix &amp; REPT("0", _xlpm.zero_count), _xlpm.k, core_BigInt.SafeK("MUL", _xlpm.len_n), _xlpm.limbs_n, core_BigInt.Split(_xlpm.norm_n, _xlpm.k), _xlpm.limbs_seed, core_BigInt.Split(_xlpm.seed_str, _xlpm.k), _xlpm.final_limbs, core_BigInt.USqrt(_xlpm.limbs_n, _xlpm.limbs_seed, _xlpm.k), core_BigInt.Merge(_xlpm.final_limbs, _xlpm.k)))))))</definedName>
-    <definedName name="BigInt.Sub" comment="Subtracts the second BigInt string from the first (A - B)._x000a_@param big_int_a The minuend BigInt string._x000a_@param big_int_b The subtrahend BigInt string.">_xlfn.LAMBDA(_xlpm.big_int_a,_xlpm.big_int_b, _xlfn.LET(_xlpm.norm_b, BigInt.Norm(_xlpm.big_int_b), _xlpm.inv_b, IF(_xlpm.norm_b = "0", "0", IF(LEFT(_xlpm.norm_b) = "-", MID(_xlpm.norm_b, 2, LEN(_xlpm.norm_b)), "-" &amp; _xlpm.norm_b)), BigInt.Add(_xlpm.big_int_a, _xlpm.inv_b)))</definedName>
-    <definedName name="BigInt.Sum" comment="Sums an array or range of BigInt strings via vectorized group matrices._x000a_@param range A contiguous range or array of BigInt strings.">_xlfn.LAMBDA(_xlpm.range, _xlfn.LET(_xlpm.flat, _xlfn.TOROW(_xlpm.range, 1), IF(OR(ISERROR(_xlpm.flat), COLUMNS(_xlpm.flat) = 0), "0", _xlfn.LET(_xlpm.norms, _xlfn.MAP(_xlpm.flat, _xlfn.LAMBDA(_xlpm.x, BigInt.Norm(_xlpm.x))), _xlpm.signs, _xlfn.MAP(LEFT(_xlpm.norms), _xlfn.LAMBDA(_xlpm.x, IF(_xlpm.x = "0", 0, IF(_xlpm.x = "-", -1, 1)))), _xlpm.abs_norms, _xlfn.MAP(_xlpm.norms, _xlpm.signs, _xlfn.LAMBDA(_xlpm.x,_xlpm.sign, IF(_xlpm.sign = -1, MID(_xlpm.x, 2, LEN(_xlpm.x) - 1), _xlpm.x))), _xlpm.pos_strs, _xlfn._xlws.FILTER(_xlpm.abs_norms, _xlpm.signs = 1, {"0"}), _xlpm.neg_strs, _xlfn._xlws.FILTER(_xlpm.abs_norms, _xlpm.signs = -1, {"0"}), _xlpm.unified_k, core_BigInt.SafeK("ADD", COLUMNS(_xlpm.flat)), _xlpm.pos_limbs, core_BigInt.UMatrixSum(_xlpm.pos_strs, _xlpm.unified_k), _xlpm.neg_limbs, core_BigInt.UMatrixSum(_xlpm.neg_strs, _xlpm.unified_k), _xlpm.routed, core_BigInt.AddSubRouter(_xlpm.pos_limbs, _xlpm.neg_limbs, 1, -1, _xlpm.unified_k), _xlpm.final_sign, _xlfn.CHOOSEROWS(_xlpm.routed, -1), _xlpm.final_limbs, _xlfn.DROP(_xlpm.routed, -1), _xlpm.merged, core_BigInt.Merge(_xlpm.final_limbs, _xlpm.unified_k), IF(_xlpm.final_sign = -1, "-" &amp; _xlpm.merged, _xlpm.merged)))))</definedName>
-    <definedName name="core_BigInt.AddSubRouter" comment="[Internal] Routes addition/subtraction based on signs and magnitudes._x000a_Returns a tuple array: VSTACK(limbs, final_sign) where the final row is the scalar sign._x000a_@param limbs_a The first little-endian limb array._x000a_@param limbs_b The second little-endian limb ">_xlfn.LAMBDA(_xlpm.limbs_a,_xlpm.limbs_b,_xlpm.sign_a,_xlpm.sign_b,_xlpm.k, _xlfn.LET(_xlpm.is_same_sign, _xlpm.sign_a = _xlpm.sign_b, IF(_xlpm.is_same_sign, _xlfn.VSTACK(core_BigInt.UAdd(_xlpm.limbs_a, _xlpm.limbs_b, _xlpm.k), _xlpm.sign_a), _xlfn.LET(_xlpm.mag_comp, core_BigInt.UCompare(_xlpm.limbs_a, _xlpm.limbs_b), IF(_xlpm.mag_comp = 0, {0;0}, IF(_xlpm.mag_comp &gt; 0, _xlfn.VSTACK(core_BigInt.USub(_xlpm.limbs_a, _xlpm.limbs_b, _xlpm.k), _xlpm.sign_a), _xlfn.VSTACK(core_BigInt.USub(_xlpm.limbs_b, _xlpm.limbs_a, _xlpm.k), _xlpm.sign_b)))))))</definedName>
-    <definedName name="core_BigInt.Carry" comment="[Internal] Resolves carries right-to-left across a vertical array of base-10^k limbs._x000a_@param limbs The array of numeric limbs._x000a_@param k The limb size.">_xlfn.LAMBDA(_xlpm.limbs,_xlpm.k, _xlfn.LET(_xlpm.n, ROWS(_xlpm.limbs), _xlpm.base, 10 ^ _xlpm.k, _xlpm.scanned, _xlfn.SCAN(0, _xlpm.limbs, _xlfn.LAMBDA(_xlpm.acc,_xlpm.val, _xlpm.val + INT(_xlpm.acc / _xlpm.base))), _xlpm.remainders, MOD(_xlpm.scanned, _xlpm.base), _xlpm.final_carry, INT(INDEX(_xlpm.scanned, _xlpm.n, 1) / _xlpm.base), IF(_xlpm.final_carry &gt; 0, _xlfn.VSTACK(_xlpm.remainders, _xlpm.final_carry), _xlpm.remainders)))</definedName>
-    <definedName name="core_BigInt.DivRouter" comment=" * [Internal] Hybrid Division Router._x000a_ * Directs division to the optimal kernel based on Dividend length._x000a_ * @param limbs_a The dividend array._x000a_ * @param limbs_b The divisor array._x000a_ * @param k The dynamic chunk size context._x000a_ ">_xlfn.LAMBDA(_xlpm.limbs_a,_xlpm.limbs_b,_xlpm.k, _xlfn.LET(_xlpm.digits_a, ROWS(_xlpm.limbs_a) * _xlpm.k, _xlpm.digits_b, ROWS(_xlpm.limbs_b) * _xlpm.k, _xlpm.m, 0.107821194271297, _xlpm.c, -221.902189462068, _xlpm.threshold, (_xlpm.m * _xlpm.digits_a) + _xlpm.c, IF(_xlpm.digits_b &lt;= _xlpm.threshold, core_BigInt.KnuthDiv(_xlpm.limbs_a, _xlpm.limbs_b, _xlpm.k), core_BigInt.NewtonRaphsonDiv(_xlpm.limbs_a, _xlpm.limbs_b, _xlpm.k))))</definedName>
-    <definedName name="core_BigInt.FindQuotientLimb" comment=" * [Internal] Binary search to find the highest scalar quotient limb q (0 &lt;= q &lt; 10^k)_x000a_ * such that B * q &lt;= acc. Eliminates the need for Knuth D float-estimation._x000a_ * @param acc The current remainder array._x000a_ * @param b The divisor array._x000a_ * @param k The d">_xlfn.LAMBDA(_xlpm.acc,_xlpm.b,_xlpm.k, _xlfn.LET(_xlpm.bits, _xlfn.CEILING.MATH(LOG(10 ^ _xlpm.k, 2)), _xlpm.powers, 2 ^ _xlfn.SEQUENCE(_xlpm.bits, 1, _xlpm.bits - 1, -1), _xlfn.REDUCE(0, _xlpm.powers, _xlfn.LAMBDA(_xlpm.curr_q,_xlpm.power, _xlfn.LET(_xlpm.test_q, _xlpm.curr_q + _xlpm.power, IF(_xlpm.test_q &gt;= 10 ^ _xlpm.k, _xlpm.curr_q, _xlfn.LET(_xlpm.test_prod, core_BigInt.Carry(_xlpm.b * _xlpm.test_q, _xlpm.k), _xlpm.comp, core_BigInt.UCompare(_xlpm.acc, _xlpm.test_prod), IF(_xlpm.comp &gt;= 0, _xlpm.test_q, _xlpm.curr_q))))))))</definedName>
-    <definedName name="core_BigInt.KnuthDiv" comment=" * [Internal] Basecase Division via sequential shift-and-subtract._x000a_ * Returns a packed 1D array: VSTACK(Length_R, R_limbs, Q_limbs)._x000a_ * Eliminates 2D array padding to strictly preserve memory efficiency._x000a_ * @param limbs_a The dividend array._x000a_ * @param lim">_xlfn.LAMBDA(_xlpm.limbs_a,_xlpm.limbs_b,_xlpm.k, _xlfn.LET(_xlpm.mag_comp, core_BigInt.UCompare(_xlpm.limbs_a, _xlpm.limbs_b), IF(_xlpm.mag_comp &lt; 0, _xlfn.VSTACK(ROWS(_xlpm.limbs_a), _xlpm.limbs_a, 0), IF(_xlpm.mag_comp = 0, _xlfn.VSTACK(1, 0, 1), _xlfn.LET(_xlpm.len_a, ROWS(_xlpm.limbs_a), _xlpm.reversed_a, _xlfn.CHOOSEROWS(_xlpm.limbs_a, _xlfn.SEQUENCE(_xlpm.len_a, 1, _xlpm.len_a, -1)), _xlpm.initial_state, _xlfn.VSTACK(1, 0, 0), _xlpm.final_state, _xlfn.REDUCE(_xlpm.initial_state, _xlpm.reversed_a, _xlfn.LAMBDA(_xlpm.state,_xlpm.val, _xlfn.LET(_xlpm.len_remainder, INDEX(_xlpm.state, 1, 1), _xlpm.remainder, _xlfn.CHOOSEROWS(_xlpm.state, _xlfn.SEQUENCE(_xlpm.len_remainder, 1, 2)), _xlpm.quotient, _xlfn.DROP(_xlpm.state, _xlpm.len_remainder + 1), _xlpm.extended_remainder, IF(AND(ROWS(_xlpm.remainder) = 1, INDEX(_xlpm.remainder, 1, 1) = 0), _xlpm.val, _xlfn.VSTACK(_xlpm.val, _xlpm.remainder)), _xlpm.next_quotient_limb, core_BigInt.FindQuotientLimb(_xlpm.extended_remainder, _xlpm.limbs_b, _xlpm.k), _xlpm.prod, core_BigInt.Carry(_xlpm.limbs_b * _xlpm.next_quotient_limb, _xlpm.k), _xlpm.new_remainder, core_BigInt.USub(_xlpm.extended_remainder, _xlpm.prod, _xlpm.k), _xlpm.has_quotient, OR(ROWS(_xlpm.quotient) &gt; 1, INDEX(_xlpm.quotient, 1, 1) &gt; 0), _xlpm.next_quot, IF(_xlpm.has_quotient, _xlfn.VSTACK(_xlpm.quotient, _xlpm.next_quotient_limb), _xlpm.next_quotient_limb), _xlfn.VSTACK(ROWS(_xlpm.new_remainder), _xlpm.new_remainder, _xlpm.next_quot)))), _xlpm.len_remainder, INDEX(_xlpm.final_state, 1, 1), _xlpm.remainder, _xlfn.CHOOSEROWS(_xlpm.final_state, _xlfn.SEQUENCE(_xlpm.len_remainder, 1, 2)), _xlpm.reversed_quotient, _xlfn.DROP(_xlpm.final_state, _xlpm.len_remainder + 1), _xlpm.len_quotient, ROWS(_xlpm.reversed_quotient), _xlpm.quotient, _xlfn.CHOOSEROWS(_xlpm.reversed_quotient, _xlfn.SEQUENCE(_xlpm.len_quotient, 1, _xlpm.len_quotient, -1)), _xlfn.VSTACK(_xlpm.len_remainder, _xlpm.remainder, _xlpm.quotient))))))</definedName>
+    <definedName name="BigInt.Abs" comment="Returns the unsigned magnitude of a BigInt string (absolute value)._x000a_@param input The BigInt string.">_xlfn.LAMBDA(_xlpm.input, _xlfn.LET(_xlpm.str_norm, BigInt.Norm(_xlpm.input), IF(LEFT(_xlpm.str_norm) = "-", MID(_xlpm.str_norm, 2, LEN(_xlpm.str_norm) - 1), _xlpm.str_norm)))</definedName>
+    <definedName name="BigInt.Add" comment="Adds two BigInt strings._x000a_@param input_a The first BigInt string._x000a_@param input_b The second BigInt string.">_xlfn.LAMBDA(_xlpm.input_a,_xlpm.input_b, _xlfn.LET(_xlpm.str_norm_a, BigInt.Norm(_xlpm.input_a), _xlpm.str_norm_b, BigInt.Norm(_xlpm.input_b), _xlpm.sign_a, BigInt.Sign(_xlpm.str_norm_a), _xlpm.sign_b, BigInt.Sign(_xlpm.str_norm_b), _xlpm.k, core_BigInt.SafeK("ADD"), _xlpm.limbs_a, core_BigInt.Split(BigInt.Abs(_xlpm.str_norm_a), _xlpm.k), _xlpm.limbs_b, core_BigInt.Split(BigInt.Abs(_xlpm.str_norm_b), _xlpm.k), _xlpm.packed_result, core_BigInt.AddSubRouter(_xlpm.limbs_a, _xlpm.limbs_b, _xlpm.sign_a, _xlpm.sign_b, _xlpm.k), _xlpm.final_sign, _xlfn.CHOOSEROWS(_xlpm.packed_result, -1), _xlpm.final_limbs, _xlfn.DROP(_xlpm.packed_result, -1), _xlpm.str_merged, core_BigInt.Merge(_xlpm.final_limbs, _xlpm.k), IF(_xlpm.final_sign = -1, "-" &amp; _xlpm.str_merged, _xlpm.str_merged)))</definedName>
+    <definedName name="BigInt.Compare" comment="Compares two BigInt strings. Returns 1 (a &gt; b), -1 (a &lt; b), or 0 (a = b)._x000a_Evaluates signs and lengths. If identical, delegates to native limb array comparison._x000a_@param input_a The first BigInt string._x000a_@param input_b The second BigInt string.">_xlfn.LAMBDA(_xlpm.input_a,_xlpm.input_b, _xlfn.LET(_xlpm.str_norm_a, BigInt.Norm(_xlpm.input_a), _xlpm.str_norm_b, BigInt.Norm(_xlpm.input_b), _xlpm.sign_a, BigInt.Sign(_xlpm.str_norm_a), _xlpm.sign_b, BigInt.Sign(_xlpm.str_norm_b), IF(_xlpm.sign_a &lt;&gt; _xlpm.sign_b, SIGN(_xlpm.sign_a - _xlpm.sign_b), IF(_xlpm.sign_a = 0, 0, _xlfn.LET(_xlpm.len_a, LEN(_xlpm.str_norm_a), _xlpm.len_b, LEN(_xlpm.str_norm_b), IF(_xlpm.len_a &lt;&gt; _xlpm.len_b, SIGN(_xlpm.len_a - _xlpm.len_b) * _xlpm.sign_a, _xlfn.LET(_xlpm.k, core_BigInt.SafeK("ADD"), _xlpm.limbs_a, core_BigInt.Split(BigInt.Abs(_xlpm.str_norm_a), _xlpm.k), _xlpm.limbs_b, core_BigInt.Split(BigInt.Abs(_xlpm.str_norm_b), _xlpm.k), _xlpm.magnitude_comparison, core_BigInt.UCompare(_xlpm.limbs_a, _xlpm.limbs_b), _xlpm.magnitude_comparison * _xlpm.sign_a)))))))</definedName>
+    <definedName name="BigInt.Div" comment="Divides the first BigInt by the second (A / B). _x000a_@param input_a The dividend BigInt string._x000a_@param input_b The divisor BigInt string._x000a_@param [use_floor] Optional boolean. TRUE for Python-style Floor division. Defaults to FALSE.">_xlfn.LAMBDA(_xlpm.input_a,_xlpm.input_b,_xlop.use_floor, INDEX(BigInt.DivMod(_xlpm.input_a, _xlpm.input_b, _xlpm.use_floor), 1, 1))</definedName>
+    <definedName name="BigInt.DivMod" comment="Divides the first BigInt by the second (A / B). _x000a_Returns the quotient and modulus in rows 1 and 2, respectively._x000a_@param input_a The dividend BigInt string._x000a_@param input_b The divisor BigInt string._x000a_@param [use_floor] Optional boolean. TRUE for Python-styl">_xlfn.LAMBDA(_xlpm.input_a,_xlpm.input_b,_xlop.use_floor, _xlfn.LET(_xlpm.str_norm_a, BigInt.Norm(_xlpm.input_a), _xlpm.str_norm_b, BigInt.Norm(_xlpm.input_b), _xlpm.sign_a, BigInt.Sign(_xlpm.str_norm_a), _xlpm.sign_b, BigInt.Sign(_xlpm.str_norm_b), _xlpm.is_floor_div, IF(_xlfn.ISOMITTED(_xlpm.use_floor), FALSE, _xlpm.use_floor), IF(_xlpm.sign_b = 0, #DIV/0!, IF(_xlpm.sign_a = 0, {"0";"0"}, _xlfn.LET(_xlpm.k, core_BigInt.SafeK("DIV"), _xlpm.limbs_a, core_BigInt.Split(BigInt.Abs(_xlpm.str_norm_a), _xlpm.k), _xlpm.limbs_b, core_BigInt.Split(BigInt.Abs(_xlpm.str_norm_b), _xlpm.k), _xlpm.packed_result, core_BigInt.DivRouter(_xlpm.limbs_a, _xlpm.limbs_b, _xlpm.k), _xlpm.len_remainder, INDEX(_xlpm.packed_result, 1, 1), _xlpm.limbs_remainder, _xlfn.CHOOSEROWS(_xlpm.packed_result, _xlfn.SEQUENCE(_xlpm.len_remainder, 1, 2)), _xlpm.limbs_quotient, _xlfn.DROP(_xlpm.packed_result, _xlpm.len_remainder + 1), _xlpm.final_sign, _xlpm.sign_a * _xlpm.sign_b, _xlpm.str_merged_q, core_BigInt.Merge(_xlpm.limbs_quotient, _xlpm.k), _xlpm.str_merged_r, core_BigInt.Merge(_xlpm.limbs_remainder, _xlpm.k), _xlpm.str_trunc_q, IF(AND(_xlpm.final_sign = -1, _xlpm.str_merged_q &lt;&gt; "0"), "-" &amp; _xlpm.str_merged_q, _xlpm.str_merged_q), _xlpm.str_trunc_r, IF(AND(_xlpm.sign_a = -1, _xlpm.str_merged_r &lt;&gt; "0"), "-" &amp; _xlpm.str_merged_r, _xlpm.str_merged_r), _xlpm.needs_floor_correction, AND(_xlpm.is_floor_div, _xlpm.final_sign = -1, _xlpm.str_merged_r &lt;&gt; "0"), _xlpm.str_final_q, IF(_xlpm.needs_floor_correction, BigInt.Sub(_xlpm.str_trunc_q, "1"), _xlpm.str_trunc_q), _xlpm.str_final_r, IF(_xlpm.needs_floor_correction, BigInt.Add(_xlpm.str_trunc_r, _xlpm.str_norm_b), _xlpm.str_trunc_r), _xlfn.VSTACK(_xlpm.str_final_q, _xlpm.str_final_r))))))</definedName>
+    <definedName name="BigInt.Fact" comment="Computes the factorial of a BigInt (n!) using Peter Luschny's Prime Swing algorithm._x000a_@param input The BigInt string. Maximum supported input is 9273.">_xlfn.LAMBDA(_xlpm.input, _xlfn.LET(_xlpm.str_norm, BigInt.Norm(_xlpm.input), _xlpm.sign_n, BigInt.Sign(_xlpm.str_norm), IF(_xlpm.sign_n = -1, #NUM!, IF(_xlpm.str_norm = "0", "1", IF(_xlpm.str_norm = "1", "1", IF(LEN(_xlpm.str_norm) &gt; 4, #NUM!, IF(VALUE(_xlpm.str_norm) &gt; 9273, #NUM!, _xlfn.LET(_xlpm.num_n, VALUE(_xlpm.str_norm), _xlpm.global_primes, core_BigInt.NativePrimes(_xlpm.num_n), core_BigInt.PrimeSwingKernel(_xlpm.num_n, _xlpm.global_primes)))))))))</definedName>
+    <definedName name="BigInt.IsEven" comment="Returns TRUE if the BigInt is even._x000a_@param input The BigInt string.">_xlfn.LAMBDA(_xlpm.input, ISEVEN(VALUE(RIGHT(BigInt.Norm(_xlpm.input)))))</definedName>
+    <definedName name="BigInt.IsNeg" comment="Returns TRUE if the BigInt is negative._x000a_@param input The BigInt string.">_xlfn.LAMBDA(_xlpm.input, LEFT(BigInt.Norm(_xlpm.input)) = "-")</definedName>
+    <definedName name="BigInt.IsOdd" comment="Returns TRUE if the BigInt is odd._x000a_@param input The BigInt string.">_xlfn.LAMBDA(_xlpm.input, ISODD(VALUE(RIGHT(BigInt.Norm(_xlpm.input)))))</definedName>
+    <definedName name="BigInt.IsZero" comment="Returns TRUE if the BigInt is exactly zero._x000a_@param input The BigInt string.">_xlfn.LAMBDA(_xlpm.input, BigInt.Norm(_xlpm.input) = "0")</definedName>
+    <definedName name="BigInt.Max" comment="Returns the maximum BigInt from an array or range._x000a_@param range A contiguous range or array of BigInt strings.">_xlfn.LAMBDA(_xlpm.range, _xlfn.LET(_xlpm.flattened_col, _xlfn.TOCOL(_xlpm.range, 1), IF(OR(ISERROR(_xlpm.flattened_col), ROWS(_xlpm.flattened_col) = 0), "0", core_BigInt.TreeCompare(_xlfn.MAP(_xlpm.flattened_col, BigInt.Norm), 1))))</definedName>
+    <definedName name="BigInt.Min" comment="Returns the minimum BigInt from an array or range._x000a_@param range A contiguous range or array of BigInt strings.">_xlfn.LAMBDA(_xlpm.range, _xlfn.LET(_xlpm.flattened_col, _xlfn.TOCOL(_xlpm.range, 1), IF(OR(ISERROR(_xlpm.flattened_col), ROWS(_xlpm.flattened_col) = 0), "0", core_BigInt.TreeCompare(_xlfn.MAP(_xlpm.flattened_col, BigInt.Norm), -1))))</definedName>
+    <definedName name="BigInt.Mod" comment="Computes the remainder of A / B._x000a_@param input_a The dividend BigInt string._x000a_@param input_b The divisor BigInt string._x000a_@param [use_floor] Optional boolean. TRUE for Python-style Modulo. Defaults to FALSE.">_xlfn.LAMBDA(_xlpm.input_a,_xlpm.input_b,_xlop.use_floor, INDEX(BigInt.DivMod(_xlpm.input_a, _xlpm.input_b, _xlpm.use_floor), 2, 1))</definedName>
+    <definedName name="BigInt.Mul" comment="Multiplies two BigInt strings._x000a_@param input_a The first BigInt string._x000a_@param input_b The second BigInt string.">_xlfn.LAMBDA(_xlpm.input_a,_xlpm.input_b, _xlfn.LET(_xlpm.str_norm_a, BigInt.Norm(_xlpm.input_a), _xlpm.str_norm_b, BigInt.Norm(_xlpm.input_b), _xlpm.sign_a, BigInt.Sign(_xlpm.str_norm_a), _xlpm.sign_b, BigInt.Sign(_xlpm.str_norm_b), _xlpm.len_a, LEN(_xlpm.str_norm_a) - IF(_xlpm.sign_a = -1, 1, 0), _xlpm.len_b, LEN(_xlpm.str_norm_b) - IF(_xlpm.sign_b = -1, 1, 0), IF(OR(_xlpm.sign_a = 0, _xlpm.sign_b = 0), "0", IF(_xlpm.len_a + _xlpm.len_b &gt; 32766, #NUM!, _xlfn.LET(_xlpm.k, core_BigInt.SafeK("MUL", MIN(_xlpm.len_a, _xlpm.len_b)), _xlpm.limbs_a, core_BigInt.Split(BigInt.Abs(_xlpm.str_norm_a), _xlpm.k), _xlpm.limbs_b, core_BigInt.Split(BigInt.Abs(_xlpm.str_norm_b), _xlpm.k), _xlpm.final_limbs, core_BigInt.UMul(_xlpm.limbs_a, _xlpm.limbs_b, _xlpm.k), _xlpm.final_sign, _xlpm.sign_a * _xlpm.sign_b, _xlpm.str_merged, core_BigInt.Merge(_xlpm.final_limbs, _xlpm.k), IF(_xlpm.final_sign = -1, "-" &amp; _xlpm.str_merged, _xlpm.str_merged))))))</definedName>
+    <definedName name="BigInt.Norm" comment="Normalises a BigInt string. Strips leading zeros, resolves &quot;-0&quot; to &quot;0&quot;, and throws #VALUE! on invalid characters._x000a_@param input The BigInt string.">_xlfn.LAMBDA(_xlpm.input, _xlfn.LET(_xlpm.str_input, IF(OR(_xlfn.ISOMITTED(_xlpm.input), _xlpm.input = ""), "0", _xlpm.input &amp; ""), _xlpm.is_value_format, _xlfn.REGEXTEST(_xlpm.str_input, "^-?\d+$"), _xlpm.str_norm, _xlfn.REGEXREPLACE(_xlpm.str_input, "^(-?)0+(?=\d)", "$1"), IF(NOT(_xlpm.is_value_format), VALUE("#VALUE!"), IF(_xlpm.str_norm = "-0", "0", _xlpm.str_norm))))</definedName>
+    <definedName name="BigInt.Pow" comment="Raises a BigInt base to the power of a BigInt exponent._x000a_@param base The base BigInt string._x000a_@param exponent The exponent BigInt string.">_xlfn.LAMBDA(_xlpm.base,_xlpm.exponent, _xlfn.LET(_xlpm.str_norm_base, BigInt.Norm(_xlpm.base), _xlpm.str_norm_exp, BigInt.Norm(_xlpm.exponent), _xlpm.sign_base, BigInt.Sign(_xlpm.str_norm_base), _xlpm.sign_exp, BigInt.Sign(_xlpm.str_norm_exp), _xlpm.str_abs_base, BigInt.Abs(_xlpm.str_norm_base), _xlpm.str_abs_exp, BigInt.Abs(_xlpm.str_norm_exp), _xlpm.is_exp_even, ISEVEN(VALUE(RIGHT(_xlpm.str_norm_exp, 1))), _xlpm.final_sign, IF(_xlpm.sign_base = -1, IF(_xlpm.is_exp_even, 1, -1), _xlpm.sign_base), IF(_xlpm.str_abs_base = "0", IF(_xlpm.str_norm_exp = "0", #NUM!, "0"), IF(_xlpm.str_abs_base = "1", IF(_xlpm.final_sign = -1, "-1", "1"), IF(_xlpm.sign_exp = -1, "0", IF(_xlpm.str_norm_exp = "0", "1", IF(LEN(_xlpm.str_norm_exp) &gt; 6, #NUM!, _xlfn.LET(_xlpm.num_exp, VALUE(_xlpm.str_norm_exp), _xlpm.base_log10,LOG10(VALUE(LEFT(_xlpm.str_abs_base, 14))) + MAX(0, LEN(_xlpm.str_abs_base) - 14), _xlpm.approx_digits, _xlpm.num_exp * _xlpm.base_log10, IF(_xlpm.approx_digits &gt; 32766, #NUM!, _xlfn.LET(_xlpm.k, core_BigInt.SafeK("MUL", _xlpm.approx_digits / 2), _xlpm.limbs_base, core_BigInt.Split(_xlpm.str_abs_base, _xlpm.k), _xlpm.limbs_final, core_BigInt.UPow(_xlpm.limbs_base, _xlpm.str_norm_exp, _xlpm.k), _xlpm.str_merged, core_BigInt.Merge(_xlpm.limbs_final, _xlpm.k), IF(_xlpm.final_sign = -1, "-" &amp; _xlpm.str_merged, _xlpm.str_merged)))))))))))</definedName>
+    <definedName name="BigInt.RandArray" comment="[VOLATILE] Generates a dynamic array of integers as text._x000a_@param [num_rows] array height, default 1._x000a_@param [num_cols] array width, default 1._x000a_@param [min_digits] minimum number of digits, default 16 (min 1 digit)_x000a_@param [max_digits] maximum number of dig">_xlfn.LAMBDA(_xlop.num_rows,_xlop.num_cols,_xlop.min_digits,_xlop.max_digits, _xlfn.LET(_xlpm.n_rows, IF(_xlfn.ISOMITTED(_xlpm.num_rows), 1, _xlpm.num_rows), _xlpm.n_cols, IF(_xlfn.ISOMITTED(_xlpm.num_cols), 1, _xlpm.num_cols), _xlpm.min_len, IF(_xlfn.ISOMITTED(_xlpm.min_digits), 16, MIN(32767, MAX(1, _xlpm.min_digits))), _xlpm.max_len, IF(_xlfn.ISOMITTED(_xlpm.max_digits), 50, MAX(1, MIN(32766, _xlpm.max_digits))), _xlfn.MAP(_xlfn.RANDARRAY(_xlpm.n_rows, _xlpm.n_cols, _xlpm.min_len, _xlpm.max_len, TRUE), _xlfn.LAMBDA(_xlpm.length, _xlfn.LET(_xlpm.sign_prefix, CHOOSE(RANDBETWEEN(1, 2), "", "-"), _xlpm.rand_digits, _xlfn.CONCAT(_xlfn.RANDARRAY(1, _xlpm.length, 0, 9, TRUE)), _xlpm.sign_prefix &amp; _xlfn.REGEXREPLACE(_xlpm.rand_digits, "^0*", ""))))))</definedName>
+    <definedName name="BigInt.Sign" comment="Returns the sign of a BigInt: 1 (positive), -1 (negative), or 0 (zero)._x000a_@param big_int The BigInt string.">_xlfn.LAMBDA(_xlpm.input, _xlfn.LET(_xlpm.str_norm, BigInt.Norm(_xlpm.input), _xlfn.SWITCH(LEFT(_xlpm.str_norm), "0", 0, "-", -1, 1)))</definedName>
+    <definedName name="BigInt.Sqrt" comment="Calculates the integer square root (floor) of a BigInt._x000a_@param input The radicand BigInt string.">_xlfn.LAMBDA(_xlpm.input, _xlfn.LET(_xlpm.str_norm, BigInt.Norm(_xlpm.input), _xlpm.sign_n, BigInt.Sign(_xlpm.str_norm), IF(_xlpm.sign_n = -1, #NUM!, IF(_xlpm.str_norm = "0", "0", IF(_xlpm.str_norm = "1", "1", _xlfn.LET(_xlpm.len_norm, LEN(_xlpm.str_norm), _xlpm.num_seed_precision, IF(_xlpm.len_norm &lt;= 14, _xlpm.len_norm, IF(ISEVEN(_xlpm.len_norm), 14, 13)), _xlpm.str_native_precision, LEFT(_xlpm.str_norm, _xlpm.num_seed_precision), _xlpm.num_native_precision, VALUE(_xlpm.str_native_precision), _xlpm.num_magnitude_zeroes, (_xlpm.len_norm - _xlpm.num_seed_precision) / 2, _xlpm.str_prefix, TEXT(ROUNDUP(SQRT(_xlpm.num_native_precision), 0) + 1, "0"), _xlpm.str_seed, _xlpm.str_prefix &amp; REPT("0", _xlpm.num_magnitude_zeroes), _xlpm.k, core_BigInt.SafeK("MUL", _xlpm.len_norm), _xlpm.limbs_radicand, core_BigInt.Split(_xlpm.str_norm, _xlpm.k), _xlpm.limbs_seed, core_BigInt.Split(_xlpm.str_seed, _xlpm.k), _xlpm.limbs_final, core_BigInt.USqrt(_xlpm.limbs_radicand, _xlpm.limbs_seed, _xlpm.k), core_BigInt.Merge(_xlpm.limbs_final, _xlpm.k)))))))</definedName>
+    <definedName name="BigInt.Sub" comment="Subtracts the second BigInt string from the first (A - B)._x000a_@param input_a The minuend BigInt string._x000a_@param input_b The subtrahend BigInt string.">_xlfn.LAMBDA(_xlpm.input_a,_xlpm.input_b, _xlfn.LET(_xlpm.str_norm_b, BigInt.Norm(_xlpm.input_b), _xlpm.str_inverse_b, IF(_xlpm.str_norm_b = "0", "0", IF(LEFT(_xlpm.str_norm_b) = "-", MID(_xlpm.str_norm_b, 2, LEN(_xlpm.str_norm_b)), "-" &amp; _xlpm.str_norm_b)), BigInt.Add(_xlpm.input_a, _xlpm.str_inverse_b)))</definedName>
+    <definedName name="BigInt.Sum" comment="Sums an array or range of BigInt strings via vectorized group matrices._x000a_@param input_range A contiguous range or array of BigInt strings.">_xlfn.LAMBDA(_xlpm.input_range, _xlfn.LET(_xlpm.flattened_input, _xlfn.TOROW(_xlpm.input_range, 1), IF(OR(ISERROR(_xlpm.flattened_input), COLUMNS(_xlpm.flattened_input) = 0), "0", _xlfn.LET(_xlpm.str_norms, _xlfn.MAP(_xlpm.flattened_input, _xlfn.LAMBDA(_xlpm.x, BigInt.Norm(_xlpm.x))), _xlpm.arr_signs, _xlfn.MAP(LEFT(_xlpm.str_norms), _xlfn.LAMBDA(_xlpm.x, IF(_xlpm.x = "0", 0, IF(_xlpm.x = "-", -1, 1)))), _xlpm.str_abs, _xlfn.MAP(_xlpm.str_norms, _xlpm.arr_signs, _xlfn.LAMBDA(_xlpm.x,_xlpm.sign, IF(_xlpm.sign = -1, MID(_xlpm.x, 2, LEN(_xlpm.x) - 1), _xlpm.x))), _xlpm.str_pos, _xlfn._xlws.FILTER(_xlpm.str_abs, _xlpm.arr_signs = 1, {"0"}), _xlpm.str_negs, _xlfn._xlws.FILTER(_xlpm.str_abs, _xlpm.arr_signs = -1, {"0"}), _xlpm.unified_k, core_BigInt.SafeK("ADD", COLUMNS(_xlpm.flattened_input)), _xlpm.limbs_pos_sum, core_BigInt.UMatrixSum(_xlpm.str_pos, _xlpm.unified_k), _xlpm.limbs_neg_sum, core_BigInt.UMatrixSum(_xlpm.str_negs, _xlpm.unified_k), _xlpm.packed_result, core_BigInt.AddSubRouter(_xlpm.limbs_pos_sum, _xlpm.limbs_neg_sum, 1, -1, _xlpm.unified_k), _xlpm.final_sign, _xlfn.CHOOSEROWS(_xlpm.packed_result, -1), _xlpm.final_limbs, _xlfn.DROP(_xlpm.packed_result, -1), _xlpm.str_merged, core_BigInt.Merge(_xlpm.final_limbs, _xlpm.unified_k), IF(_xlpm.final_sign = -1, "-" &amp; _xlpm.str_merged, _xlpm.str_merged)))))</definedName>
+    <definedName name="core_BigInt.AddSubRouter" comment="[Internal] Routes addition/subtraction based on signs and magnitudes._x000a_Returns a tuple array: VSTACK(limbs, final_sign) where the final row is the scalar sign._x000a_@param limbs_a The first little-endian limb array._x000a_@param limbs_b The second little-endian limb ">_xlfn.LAMBDA(_xlpm.limbs_a,_xlpm.limbs_b,_xlpm.sign_a,_xlpm.sign_b,_xlpm.k, _xlfn.LET(_xlpm.is_addition, _xlpm.sign_a = _xlpm.sign_b, IF(_xlpm.is_addition, _xlfn.VSTACK(core_BigInt.UAdd(_xlpm.limbs_a, _xlpm.limbs_b, _xlpm.k), _xlpm.sign_a), _xlfn.LET(_xlpm.magnitude_comparison, core_BigInt.UCompare(_xlpm.limbs_a, _xlpm.limbs_b), IF(_xlpm.magnitude_comparison = 0, {0;0}, IF(_xlpm.magnitude_comparison &gt; 0, _xlfn.VSTACK(core_BigInt.USub(_xlpm.limbs_a, _xlpm.limbs_b, _xlpm.k), _xlpm.sign_a), _xlfn.VSTACK(core_BigInt.USub(_xlpm.limbs_b, _xlpm.limbs_a, _xlpm.k), _xlpm.sign_b)))))))</definedName>
+    <definedName name="core_BigInt.Carry" comment="[Internal] Resolves carries right-to-left across a vertical array of base-10^k limbs._x000a_@param limbs The array of numeric limbs._x000a_@param k The limb size.">_xlfn.LAMBDA(_xlpm.limbs,_xlpm.k, _xlfn.LET(_xlpm.num_limbs, ROWS(_xlpm.limbs), _xlpm.radix_base, 10 ^ _xlpm.k, _xlpm.arr_carries, _xlfn.SCAN(0, _xlpm.limbs, _xlfn.LAMBDA(_xlpm.acc,_xlpm.val, _xlpm.val + INT(_xlpm.acc / _xlpm.radix_base))), _xlpm.remainders, MOD(_xlpm.arr_carries, _xlpm.radix_base), _xlpm.final_carry, INT(INDEX(_xlpm.arr_carries, _xlpm.num_limbs, 1) / _xlpm.radix_base), IF(_xlpm.final_carry &gt; 0, _xlfn.VSTACK(_xlpm.remainders, _xlpm.final_carry), _xlpm.remainders)))</definedName>
+    <definedName name="core_BigInt.DivRouter" comment=" * [Internal] Hybrid Division Router._x000a_ * Directs division to the optimal kernel based on Dividend length._x000a_ * @param limbs_a The dividend array._x000a_ * @param limbs_b The divisor array._x000a_ * @param k The dynamic chunk size context._x000a_ ">_xlfn.LAMBDA(_xlpm.limbs_a,_xlpm.limbs_b,_xlpm.k, _xlfn.LET(_xlpm.approx_digits_a, ROWS(_xlpm.limbs_a) * _xlpm.k, _xlpm.approx_digits_b, ROWS(_xlpm.limbs_b) * _xlpm.k, _xlpm.regression_slope_m, 0.107821194271297, _xlpm.regression_intercept_c, -221.902189462068, _xlpm.threshold_digits, (_xlpm.regression_slope_m * _xlpm.approx_digits_a) + _xlpm.regression_intercept_c, IF(_xlpm.approx_digits_b &lt;= _xlpm.threshold_digits, core_BigInt.KnuthDiv(_xlpm.limbs_a, _xlpm.limbs_b, _xlpm.k), core_BigInt.NewtonRaphsonDiv(_xlpm.limbs_a, _xlpm.limbs_b, _xlpm.k))))</definedName>
+    <definedName name="core_BigInt.FindQuotientLimb" comment=" * [Internal] Binary search to find the highest scalar quotient limb q (0 &lt;= q &lt; 10^k)_x000a_ * such that B * q &lt;= limbs_r. Eliminates the need for Knuth D float-estimation._x000a_ * @param limbs_r The current remainder array._x000a_ * @param b The divisor array._x000a_ * @param">_xlfn.LAMBDA(_xlpm.limbs_r,_xlpm.limbs_b,_xlpm.k, _xlfn.LET(_xlpm.required_bits, _xlfn.CEILING.MATH(LOG(10 ^ _xlpm.k, 2)), _xlpm.powers_of_two, 2 ^ _xlfn.SEQUENCE(_xlpm.required_bits, 1, _xlpm.required_bits - 1, -1), _xlfn.REDUCE(0, _xlpm.powers_of_two, _xlfn.LAMBDA(_xlpm.current_q,_xlpm.current_power, _xlfn.LET(_xlpm.test_q, _xlpm.current_q + _xlpm.current_power, IF(_xlpm.test_q &gt;= 10 ^ _xlpm.k, _xlpm.current_q, _xlfn.LET(_xlpm.limbs_bq, core_BigInt.Carry(_xlpm.limbs_b * _xlpm.test_q, _xlpm.k), _xlpm.magnitude_comparison, core_BigInt.UCompare(_xlpm.limbs_r, _xlpm.limbs_bq), IF(_xlpm.magnitude_comparison &gt;= 0, _xlpm.test_q, _xlpm.current_q))))))))</definedName>
+    <definedName name="core_BigInt.KnuthDiv" comment=" * [Internal] Basecase Division via sequential shift-and-subtract._x000a_ * Returns a packed 1D array: VSTACK(Length_R, R_limbs, Q_limbs)._x000a_ * Eliminates 2D array padding to strictly preserve memory efficiency._x000a_ * @param limbs_a The dividend array._x000a_ * @param lim">_xlfn.LAMBDA(_xlpm.limbs_a,_xlpm.limbs_b,_xlpm.k, _xlfn.LET(_xlpm.magnitude_comparison, core_BigInt.UCompare(_xlpm.limbs_a, _xlpm.limbs_b), IF(_xlpm.magnitude_comparison &lt; 0, _xlfn.VSTACK(ROWS(_xlpm.limbs_a), _xlpm.limbs_a, 0), IF(_xlpm.magnitude_comparison = 0, _xlfn.VSTACK(1, 0, 1), _xlfn.LET(_xlpm.num_limbs_a, ROWS(_xlpm.limbs_a), _xlpm.big_endian_a, _xlfn.CHOOSEROWS(_xlpm.limbs_a, _xlfn.SEQUENCE(_xlpm.num_limbs_a, 1, _xlpm.num_limbs_a, -1)), _xlpm.final_packed_state, _xlfn.REDUCE(_xlfn.VSTACK(1, 0, 0), _xlpm.big_endian_a, _xlfn.LAMBDA(_xlpm.packed_state,_xlpm.val, _xlfn.LET(_xlpm.num_limbs_r, INDEX(_xlpm.packed_state, 1, 1), _xlpm.limbs_r, _xlfn.CHOOSEROWS(_xlpm.packed_state, _xlfn.SEQUENCE(_xlpm.num_limbs_r, 1, 2)), _xlpm.limbs_q, _xlfn.DROP(_xlpm.packed_state, _xlpm.num_limbs_r + 1), _xlpm.limbs_shifted_r, IF(AND(ROWS(_xlpm.limbs_r) = 1, INDEX(_xlpm.limbs_r, 1, 1) = 0), _xlpm.val, _xlfn.VSTACK(_xlpm.val, _xlpm.limbs_r)), _xlpm.q_limb, core_BigInt.FindQuotientLimb(_xlpm.limbs_shifted_r, _xlpm.limbs_b, _xlpm.k), _xlpm.limbs_bq, core_BigInt.Carry(_xlpm.limbs_b * _xlpm.q_limb, _xlpm.k), _xlpm.limbs_next_r, core_BigInt.USub(_xlpm.limbs_shifted_r, _xlpm.limbs_bq, _xlpm.k), _xlpm.has_q, OR(ROWS(_xlpm.limbs_q) &gt; 1, INDEX(_xlpm.limbs_q, 1, 1) &gt; 0), _xlpm.limbs_next_q, IF(_xlpm.has_q, _xlfn.VSTACK(_xlpm.limbs_q, _xlpm.q_limb), _xlpm.q_limb), _xlfn.VSTACK(ROWS(_xlpm.limbs_next_r), _xlpm.limbs_next_r, _xlpm.limbs_next_q)))), _xlpm.num_limbs_r, INDEX(_xlpm.final_packed_state, 1, 1), _xlpm.limbs_r, _xlfn.CHOOSEROWS(_xlpm.final_packed_state, _xlfn.SEQUENCE(_xlpm.num_limbs_r, 1, 2)), _xlpm.big_endian_q, _xlfn.DROP(_xlpm.final_packed_state, _xlpm.num_limbs_r + 1), _xlpm.len_q, ROWS(_xlpm.big_endian_q), _xlpm.limbs_q, _xlfn.CHOOSEROWS(_xlpm.big_endian_q, _xlfn.SEQUENCE(_xlpm.len_q, 1, _xlpm.len_q, -1)), _xlfn.VSTACK(_xlpm.num_limbs_r, _xlpm.limbs_r, _xlpm.limbs_q))))))</definedName>
     <definedName name="core_BigInt.Merge" comment="[Internal] Concatenates an array of numeric limbs into a BigInt string, zero-padding all but the first limb._x000a_@param limbs The vertical array of numeric limbs._x000a_@param k The limb size used during calculation.">_xlfn.LAMBDA(_xlpm.limbs,_xlpm.k, _xlfn.LET(_xlpm.num_limbs, ROWS(_xlpm.limbs), _xlpm.rev_limbs, _xlfn.CHOOSEROWS(_xlpm.limbs, _xlfn.SEQUENCE(_xlpm.num_limbs, 1, _xlpm.num_limbs, -1)), IF(_xlpm.num_limbs = 1, _xlpm.rev_limbs &amp; "", _xlfn.CONCAT(_xlfn.VSTACK(_xlfn.TAKE(_xlpm.rev_limbs, 1) &amp; "", TEXT(_xlfn.DROP(_xlpm.rev_limbs, 1), REPT("0", _xlpm.k)))))))</definedName>
-    <definedName name="core_BigInt.NativePrimes" comment="[Internal] Generates a 1D vertical array of all prime numbers up to n._x000a_Evaluates purely in native C++ using a dynamic sieve._x000a_@param n The upper bound integer (assumed &lt;= 9273).">_xlfn.LAMBDA(_xlpm.n, IF(_xlpm.n &lt; 2, #NUM!, _xlfn.LET(_xlpm.seq, _xlfn.SEQUENCE(_xlpm.n - 1, 1, 2), _xlfn._xlws.FILTER(_xlpm.seq, _xlfn.MAP(_xlpm.seq, _xlfn.LAMBDA(_xlpm.x, _xlfn.LET(_xlpm.limit, INT(SQRT(_xlpm.x)), IF(_xlpm.limit &lt; 2, TRUE, MIN(MOD(_xlpm.x, _xlfn.SEQUENCE(_xlpm.limit - 1, 1, 2))) &gt; 0))))))))</definedName>
-    <definedName name="core_BigInt.NativeSwingExponents" comment="[Internal] Calculates the exponent for an array of primes in the Swing term of a factorial._x000a_@param n The current factorial magnitude (&lt;= 9273)._x000a_@param primes A vertical array of prime numbers (&lt;= n).">_xlfn.LAMBDA(_xlpm.n,_xlpm.primes, _xlfn.MAP(_xlpm.primes, _xlfn.LAMBDA(_xlpm.p, _xlfn.LET(_xlpm.max_k, INT(LOG(_xlpm.n, _xlpm.p)), _xlpm.powers, _xlpm.p ^ _xlfn.SEQUENCE(_xlpm.max_k), SUM(MOD(INT(_xlpm.n / _xlpm.powers), 2))))))</definedName>
-    <definedName name="core_BigInt.NewtonRaphsonDiv" comment="[Internal] Heavyweight Newton-Raphson Division._x000a_Implements progressive scaling bounded to MAX(len_a, len_b)._x000a_@param limbs_a The dividend array._x000a_@param limbs_b The divisor array._x000a_@param k The dynamic chunk size context.">_xlfn.LAMBDA(_xlpm.limbs_a,_xlpm.limbs_b,_xlpm.k, _xlfn.LET(_xlpm.len_a, ROWS(_xlpm.limbs_a), _xlpm.len_b, ROWS(_xlpm.limbs_b), _xlpm.target_len, MAX(_xlpm.len_a, _xlpm.len_b), _xlpm.r, core_BigInt.NewtonRaphsonReciprocal(_xlpm.limbs_b, _xlpm.target_len, _xlpm.k), _xlpm.drop_limbs, 2 * _xlpm.target_len, _xlpm.q_unscaled, core_BigInt.UMul(_xlpm.limbs_a, _xlpm.r, _xlpm.k), _xlpm.q_approx, IF(ROWS(_xlpm.q_unscaled) &lt;= _xlpm.drop_limbs, {0}, _xlfn.DROP(_xlpm.q_unscaled, _xlpm.drop_limbs)), _xlpm.p_baseline, core_BigInt.UMul(_xlpm.limbs_b, _xlpm.q_approx, _xlpm.k), _xlpm.initial_state, _xlfn.VSTACK(ROWS(_xlpm.q_approx), _xlpm.q_approx, _xlpm.p_baseline), _xlpm.sweep_down, _xlfn.REDUCE(_xlpm.initial_state, {1;2}, _xlfn.LAMBDA(_xlpm.state,_xlpm.i, _xlfn.LET(_xlpm.len_q, INDEX(_xlpm.state, 1, 1), _xlpm.curr_q, _xlfn.CHOOSEROWS(_xlpm.state, _xlfn.SEQUENCE(_xlpm.len_q, 1, 2)), _xlpm.curr_p, _xlfn.DROP(_xlpm.state, _xlpm.len_q + 1), IF(core_BigInt.UCompare(_xlpm.curr_p, _xlpm.limbs_a) &gt; 0, _xlfn.LET(_xlpm.next_q, core_BigInt.USub(_xlpm.curr_q, {1}, _xlpm.k), _xlpm.next_p, core_BigInt.USub(_xlpm.curr_p, _xlpm.limbs_b, _xlpm.k), _xlfn.VSTACK(ROWS(_xlpm.next_q), _xlpm.next_q, _xlpm.next_p)), _xlpm.state)))), _xlpm.sweep_up, _xlfn.REDUCE(_xlpm.sweep_down, {1;2}, _xlfn.LAMBDA(_xlpm.state,_xlpm.i, _xlfn.LET(_xlpm.len_q, INDEX(_xlpm.state, 1, 1), _xlpm.curr_q, _xlfn.CHOOSEROWS(_xlpm.state, _xlfn.SEQUENCE(_xlpm.len_q, 1, 2)), _xlpm.curr_p, _xlfn.DROP(_xlpm.state, _xlpm.len_q + 1), _xlpm.next_p_test, core_BigInt.UAdd(_xlpm.curr_p, _xlpm.limbs_b, _xlpm.k), IF(core_BigInt.UCompare(_xlpm.next_p_test, _xlpm.limbs_a) &lt;= 0, _xlfn.LET(_xlpm.next_q, core_BigInt.UAdd(_xlpm.curr_q, {1}, _xlpm.k), _xlfn.VSTACK(ROWS(_xlpm.next_q), _xlpm.next_q, _xlpm.next_p_test)), _xlpm.state)))), _xlpm.final_len_q, INDEX(_xlpm.sweep_up, 1, 1), _xlpm.final_q, _xlfn.CHOOSEROWS(_xlpm.sweep_up, _xlfn.SEQUENCE(_xlpm.final_len_q, 1, 2)), _xlpm.final_p, _xlfn.DROP(_xlpm.sweep_up, _xlpm.final_len_q + 1), _xlpm.final_r, core_BigInt.USub(_xlpm.limbs_a, _xlpm.final_p, _xlpm.k), _xlfn.VSTACK(ROWS(_xlpm.final_r), _xlpm.final_r, _xlpm.final_q)))</definedName>
-    <definedName name="core_BigInt.NewtonRaphsonReciprocal" comment="[Internal] Computes the Reciprocal progressively scaling up to the Dividend's precision._x000a_@param limbs_b The divisor limb array._x000a_@param target_len The limb-length of Dividend A._x000a_@param k The dynamic chunk size context.">_xlfn.LAMBDA(_xlpm.limbs_b,_xlpm.target_len,_xlpm.k, _xlfn.LET(_xlpm.len_b, ROWS(_xlpm.limbs_b), _xlpm.seed_len, MIN(3, _xlpm.len_b), _xlpm.r_seed_limbs, core_BigInt.NewtonRaphsonSeed(_xlpm.limbs_b, _xlpm.k), _xlpm.initial_state, _xlfn.VSTACK(_xlpm.seed_len, _xlpm.r_seed_limbs), _xlpm.req_iters, MAX(0, _xlfn.CEILING.MATH(LN(_xlpm.target_len / _xlpm.seed_len) / LN(2))) + 1, IF(_xlpm.req_iters = 0, _xlpm.r_seed_limbs, _xlfn.LET(_xlpm.iterations, _xlfn.SEQUENCE(_xlpm.req_iters), _xlpm.final_state, _xlfn.REDUCE(_xlpm.initial_state, _xlpm.iterations, _xlfn.LAMBDA(_xlpm.state,_xlpm.iter, _xlfn.LET(_xlpm.curr_len, INDEX(_xlpm.state, 1, 1), _xlpm.curr_r, _xlfn.DROP(_xlpm.state, 1), _xlpm.next_len, MIN(_xlpm.curr_len * 2, _xlpm.target_len), _xlpm.active_curr, MIN(_xlpm.curr_len, _xlpm.len_b), _xlpm.active_next, MIN(_xlpm.next_len, _xlpm.len_b), _xlpm.shift_limbs, 2 * (_xlpm.next_len - _xlpm.curr_len) - (_xlpm.active_next - _xlpm.active_curr), _xlpm.r_prime, IF(_xlpm.shift_limbs &gt; 0, _xlfn.VSTACK(_xlfn.EXPAND(0, _xlpm.shift_limbs, , 0), _xlpm.curr_r), _xlpm.curr_r), _xlpm.b_active, _xlfn.TAKE(_xlpm.limbs_b, -_xlpm.active_next), _xlpm.p, core_BigInt.UMul(_xlpm.b_active, _xlpm.r_prime, _xlpm.k), _xlpm.two_beta, _xlfn.VSTACK(_xlfn.EXPAND(0, 2 * _xlpm.next_len, , 0), 2), _xlpm.err, core_BigInt.USub(_xlpm.two_beta, _xlpm.p, _xlpm.k), _xlpm.next_r_unscaled, core_BigInt.UMul(_xlpm.r_prime, _xlpm.err, _xlpm.k), _xlpm.next_r, IF(ROWS(_xlpm.next_r_unscaled) &lt;= 2 * _xlpm.next_len, {0}, _xlfn.DROP(_xlpm.next_r_unscaled, 2 * _xlpm.next_len)), _xlfn.VSTACK(_xlpm.next_len, _xlpm.next_r)))), _xlfn.DROP(_xlpm.final_state, 1)))))</definedName>
-    <definedName name="core_BigInt.NewtonRaphsonSeed" comment="[Internal] Generates the exact reciprocal seed for Newton-Raphson Division using Knuth Basecase._x000a_Extracts up to the top 3 limbs of B and calculates floor(Beta^(2*len) / B_top)._x000a_@param limbs_b The divisor limb array._x000a_@param k The dynamic chunk size context">_xlfn.LAMBDA(_xlpm.limbs_b,_xlpm.k, _xlfn.LET(_xlpm.len_b, ROWS(_xlpm.limbs_b), _xlpm.seed_len, MIN(3, _xlpm.len_b), _xlpm.b_top, _xlfn.TAKE(_xlpm.limbs_b, -_xlpm.seed_len), _xlpm.beta_2m, _xlfn.VSTACK(_xlfn.EXPAND(0, 2 * _xlpm.seed_len, , 0), 1), _xlpm.packed, core_BigInt.KnuthDiv(_xlpm.beta_2m, _xlpm.b_top, _xlpm.k), _xlpm.len_r, INDEX(_xlpm.packed, 1, 1), _xlfn.DROP(_xlpm.packed, _xlpm.len_r + 1)))</definedName>
-    <definedName name="core_BigInt.PrimeSwingKernel" comment="[Internal] Recursive top-down LAMBDA calculating the Prime Swing factorial._x000a_@param n The current factorial magnitude._x000a_@param global_primes The unified vertical array of all primes up to the target factorial.">_xlfn.LAMBDA(_xlpm.n,_xlpm.global_primes, IF(_xlpm.n &lt; 2, "1", _xlfn.LET(_xlpm.half_n, INT(_xlpm.n / 2), _xlpm.half_fact, core_BigInt.PrimeSwingKernel(_xlpm.half_n, _xlpm.global_primes), _xlpm.squared_half, core_BigInt.UTextMul(_xlpm.half_fact, _xlpm.half_fact), _xlpm.tier_primes, _xlfn._xlws.FILTER(_xlpm.global_primes, _xlpm.global_primes &lt;= _xlpm.n), _xlpm.swing, core_BigInt.SwingTerm(_xlpm.n, _xlpm.tier_primes), core_BigInt.UTextMul(_xlpm.squared_half, _xlpm.swing))))</definedName>
-    <definedName name="core_BigInt.SafeK" comment="[Internal] Computes the maximum safe base-10 limb size (k) to avoid IEEE-754 precision loss._x000a_@param operation: &quot;ADD&quot;, &quot;MUL&quot;, or &quot;DIV&quot;._x000a_@param [max_items] ADD: number of operands. MUL: shortest string digits count.">_xlfn.LAMBDA(_xlpm.operation,_xlop.max_items, _xlfn.LET(_xlpm.items, IF(OR(_xlpm.max_items = "", _xlfn.ISOMITTED(_xlpm.max_items)), 2, MAX(2, _xlpm.max_items)), _xlfn.SWITCH(_xlpm.operation, "ADD", 15 - LEN(_xlpm.items), "MUL", _xlfn.LET(_xlpm.test_k, {7;6;5;4;3;2;1}, _xlpm.max_overlap, ROUNDUP(_xlpm.items / _xlpm.test_k, 0), _xlpm.uncarried_max, _xlpm.max_overlap * (10 ^ _xlpm.test_k - 1) ^ 2, _xlpm.max_carry, INT(_xlpm.uncarried_max / 10 ^ _xlpm.test_k), _xlpm.peak_val, _xlpm.uncarried_max + _xlpm.max_carry, MAX(_xlfn._xlws.FILTER(_xlpm.test_k, _xlpm.peak_val &lt;= (10 ^ 15 - 1)))), "DIV", 7, #NAME?)))</definedName>
-    <definedName name="core_BigInt.Split" comment="[Internal] Unified Splitter. Splits both scalars and arrays into Little-Endian limbs._x000a_Uses MAX() to guarantee scalar inputs to the SEQUENCE engine._x000a_@param big_ints The string or array of strings._x000a_@param k The dynamic chunk size context.">_xlfn.LAMBDA(_xlpm.big_ints,_xlpm.k, _xlfn.LET(_xlpm.big_int_row, _xlfn.TOROW(_xlpm.big_ints), _xlpm.lengths, LEN(_xlpm.big_int_row), _xlpm.max_len, MAX(_xlpm.lengths), _xlpm.pad_len, ROUNDUP(_xlpm.max_len / _xlpm.k, 0) * _xlpm.k, _xlpm.padded, REPT("0", _xlpm.pad_len - _xlpm.lengths) &amp; _xlpm.big_int_row, _xlpm.starts, _xlfn.SEQUENCE(_xlpm.pad_len / _xlpm.k, 1, _xlpm.pad_len - _xlpm.k + 1, -_xlpm.k), --MID(_xlpm.padded, _xlpm.starts, _xlpm.k)))</definedName>
-    <definedName name="core_BigInt.SwingTerm" comment="[Internal] Calculates the massive BigInt string for the Swing term of a factorial._x000a_@param n The current factorial magnitude._x000a_@param tier_primes A vertical array of prime numbers (&lt;= n).">_xlfn.LAMBDA(_xlpm.n,_xlpm.tier_primes, _xlfn.LET(_xlpm.exponents, core_BigInt.NativeSwingExponents(_xlpm.n, _xlpm.tier_primes), _xlpm.is_greater_than_zero, _xlpm.exponents &gt; 0, IF(AND(NOT(_xlpm.is_greater_than_zero)), "1", _xlfn.LET(_xlpm.filtered_primes, _xlfn._xlws.FILTER(_xlpm.tier_primes, _xlpm.is_greater_than_zero), _xlpm.filtered_exps, _xlfn._xlws.FILTER(_xlpm.exponents, _xlpm.is_greater_than_zero), _xlpm.prime_powers, _xlfn.MAP(_xlpm.filtered_primes, _xlpm.filtered_exps, _xlfn.LAMBDA(_xlpm.p,_xlpm.e, IF(_xlpm.e = 1, _xlpm.p &amp; "", BigInt.Pow(_xlpm.p &amp; "", _xlpm.e &amp; "")))), core_BigInt.TextTreeProd(_xlpm.prime_powers)))))</definedName>
-    <definedName name="core_BigInt.TextTreeProd" comment="[Internal] Vectorized logarithmic product of an array of BigInt strings._x000a_Recursively cuts the array in half to bypass REDUCE sequential memory allocations._x000a_@param text_arr A 1D vertical array of BigInt strings.">_xlfn.LAMBDA(_xlpm.text_arr, _xlfn.LET(_xlpm.n, ROWS(_xlpm.text_arr), IF(_xlpm.n = 1, INDEX(_xlpm.text_arr, 1, 1), _xlfn.LET(_xlpm.paired, _xlfn.WRAPROWS(_xlpm.text_arr, 2, "1"), _xlpm.next_arr, _xlfn.BYROW(_xlpm.paired, _xlfn.LAMBDA(_xlpm.row, core_BigInt.UTextMul(INDEX(_xlpm.row, 1, 1), INDEX(_xlpm.row, 1, 2)))), core_BigInt.TextTreeProd(_xlpm.next_arr)))))</definedName>
-    <definedName name="core_BigInt.TreeCompare" comment="[Internal] Recursive tournament tree for Min/Max evaluations._x000a_@param col A 1D vertical array of normalized BigInt strings._x000a_@param mode 1 for Maximum, -1 for Minimum.">_xlfn.LAMBDA(_xlpm.col,_xlpm.mode, _xlfn.LET(_xlpm.n, ROWS(_xlpm.col), IF(_xlpm.n = 1, INDEX(_xlpm.col, 1, 1), _xlfn.LET(_xlpm.paired, _xlfn.WRAPROWS(_xlpm.col, 2, "#PAD#"), _xlpm.col_a, _xlfn.TAKE(_xlpm.paired, , 1), _xlpm.col_b, _xlfn.TAKE(_xlpm.paired, , -1), _xlpm.winners, _xlfn.MAP(_xlpm.col_a, _xlpm.col_b, _xlfn.LAMBDA(_xlpm.a,_xlpm.b, IF(_xlpm.b = "#PAD#", _xlpm.a, _xlfn.LET(_xlpm.comp, BigInt.Compare(_xlpm.a, _xlpm.b), IF(_xlpm.comp * _xlpm.mode &gt;= 0, _xlpm.a, _xlpm.b))))), core_BigInt.TreeCompare(_xlpm.winners, _xlpm.mode)))))</definedName>
-    <definedName name="core_BigInt.UAdd" comment="[Internal] Unsigned addition of two Little-Endian limb arrays._x000a_@param limbs_a The first limb array._x000a_@param limbs_b The second limb array._x000a_@param k The dynamic chunk size context.">_xlfn.LAMBDA(_xlpm.a,_xlpm.b,_xlpm.k, _xlfn.LET(_xlpm.max_rows, MAX(ROWS(_xlpm.a), ROWS(_xlpm.b)), _xlpm.pad_a, _xlfn.EXPAND(_xlpm.a, _xlpm.max_rows, 1, 0), _xlpm.pad_b, _xlfn.EXPAND(_xlpm.b, _xlpm.max_rows, 1, 0), core_BigInt.Carry(_xlpm.pad_a + _xlpm.pad_b, _xlpm.k)))</definedName>
-    <definedName name="core_BigInt.UCompare" comment="[Internal] Unsigned comparison of two Little-Endian limb arrays._x000a_Returns 1 (a &gt; b), -1 (a &lt; b), or 0 (a = b)._x000a_@param limbs_a The first limb array._x000a_@param limbs_b The second limb array.">_xlfn.LAMBDA(_xlpm.limbs_a,_xlpm.limbs_b, _xlfn.LET(_xlpm.max_rows, MAX(ROWS(_xlpm.limbs_a), ROWS(_xlpm.limbs_b)), _xlpm.pad_a, _xlfn.EXPAND(_xlpm.limbs_a, _xlpm.max_rows, 1, 0), _xlpm.pad_b, _xlfn.EXPAND(_xlpm.limbs_b, _xlpm.max_rows, 1, 0), _xlpm.diff, _xlpm.pad_a - _xlpm.pad_b, _xlpm.msd_idx, _xlfn.XMATCH(TRUE, _xlpm.diff &lt;&gt; 0, 0, -1), IF(ISNA(_xlpm.msd_idx), 0, SIGN(INDEX(_xlpm.diff, _xlpm.msd_idx, 1)))))</definedName>
-    <definedName name="core_BigInt.UMatrixSum" comment="[Internal] Vectorized matrix sum of unsigned BigInt strings._x000a_@param ubig_int Horizontal array (1xN) of normalized magnitude strings._x000a_@param k The unified dynamic chunk size context.">_xlfn.LAMBDA(_xlpm.ubig_ints,_xlpm.k, _xlfn.LET(_xlpm.grid, core_BigInt.Split(_xlpm.ubig_ints, _xlpm.k), _xlpm.raw_limbs, _xlfn.BYROW(_xlpm.grid, _xleta.SUM), core_BigInt.Carry(_xlpm.raw_limbs, _xlpm.k)))</definedName>
-    <definedName name="core_BigInt.UMul" comment="[Internal] Unsigned multiplication of two Little-Endian limb arrays._x000a_Utilizes a 1D Discrete Convolution (Cauchy Product) array-slicing strategy._x000a_Zero dynamic memory reallocation. $O(N+M)$ memory footprint._x000a_@param limbs_a The multiplicand limb array._x000a_@para">_xlfn.LAMBDA(_xlpm.limbs_a,_xlpm.limbs_b,_xlpm.k, _xlfn.LET(_xlpm.len_a, ROWS(_xlpm.limbs_a), _xlpm.len_b, ROWS(_xlpm.limbs_b), _xlpm.max_rows, _xlpm.len_a + _xlpm.len_b - 1, _xlpm.raw_limbs, _xlfn.MAKEARRAY(_xlpm.max_rows, 1, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, _xlfn.LET(_xlpm.start_i, MAX(1, _xlpm.r - _xlpm.len_b + 1), _xlpm.end_i, MIN(_xlpm.r, _xlpm.len_a), _xlpm.count, _xlpm.end_i - _xlpm.start_i + 1, _xlpm.seq_i, _xlfn.SEQUENCE(_xlpm.count, 1, _xlpm.start_i, 1), _xlpm.seq_j, _xlfn.SEQUENCE(_xlpm.count, 1, _xlpm.r - _xlpm.start_i + 1, -1), SUM(INDEX(_xlpm.limbs_a, _xlpm.seq_i, 1) * INDEX(_xlpm.limbs_b, _xlpm.seq_j, 1))))), core_BigInt.Carry(_xlpm.raw_limbs, _xlpm.k)))</definedName>
-    <definedName name="core_BigInt.UPow" comment="[Internal] Unsigned Base-10 Left-to-Right Exponentiation._x000a_Evaluates the exponent iteratively using a pre-computed 1-9 cache._x000a_@param limbs_base The little-endian limb array of the base._x000a_@param exp_string The exact text string of the exponent._x000a_@param k The ">_xlfn.LAMBDA(_xlpm.limbs_base,_xlpm.exp_string,_xlpm.k, _xlfn.LET(_xlpm.first, _xlpm.limbs_base, _xlpm.second, core_BigInt.UMul(_xlpm.first, _xlpm.first, _xlpm.k), _xlpm.third, core_BigInt.UMul(_xlpm.second, _xlpm.first, _xlpm.k), _xlpm.fourth, core_BigInt.UMul(_xlpm.second, _xlpm.second, _xlpm.k), _xlpm.fifth, core_BigInt.UMul(_xlpm.fourth, _xlpm.first, _xlpm.k), _xlpm.sixth, core_BigInt.UMul(_xlpm.third, _xlpm.third, _xlpm.k), _xlpm.seventh, core_BigInt.UMul(_xlpm.sixth, _xlpm.first, _xlpm.k), _xlpm.eigth, core_BigInt.UMul(_xlpm.fourth, _xlpm.fourth, _xlpm.k), _xlpm.ninth, core_BigInt.UMul(_xlpm.eigth, _xlpm.first, _xlpm.k), _xlpm.exp_digits, --MID(_xlpm.exp_string, _xlfn.SEQUENCE(LEN(_xlpm.exp_string)), 1), _xlfn.REDUCE(1, _xlpm.exp_digits, _xlfn.LAMBDA(_xlpm.acc,_xlpm.digit, _xlfn.LET(_xlpm.is_one, AND(ROWS(_xlpm.acc) = 1, INDEX(_xlpm.acc, 1, 1) = 1), _xlpm.acc_10, IF(_xlpm.is_one, _xlpm.acc, _xlfn.LET(_xlpm.acc_2, core_BigInt.UMul(_xlpm.acc, _xlpm.acc, _xlpm.k), _xlpm.acc_4, core_BigInt.UMul(_xlpm.acc_2, _xlpm.acc_2, _xlpm.k), _xlpm.acc_8, core_BigInt.UMul(_xlpm.acc_4, _xlpm.acc_4, _xlpm.k), core_BigInt.UMul(_xlpm.acc_8, _xlpm.acc_2, _xlpm.k))), IF(_xlpm.digit = 0, _xlpm.acc_10, _xlfn.LET(_xlpm.cache_val, CHOOSE(_xlpm.digit, _xlpm.first, _xlpm.second, _xlpm.third, _xlpm.fourth, _xlpm.fifth, _xlpm.sixth, _xlpm.seventh, _xlpm.eigth, _xlpm.ninth), IF(_xlpm.is_one, _xlpm.cache_val, core_BigInt.UMul(_xlpm.acc_10, _xlpm.cache_val, _xlpm.k)))))))))</definedName>
-    <definedName name="core_BigInt.USqrt" comment="[Internal] Unsigned Integer Square Root using Newton's Method._x000a_@param limbs_n Radicand little-endian array._x000a_@param limbs_seed Over-estimated little-endian seed array._x000a_@param k The dynamic chunk size context.">_xlfn.LAMBDA(_xlpm.limbs_n,_xlpm.limbs_seed,_xlpm.k, _xlfn.LET(_xlpm.initial_state, _xlfn.VSTACK(0, _xlpm.limbs_seed), _xlpm.max_iters, 35, _xlpm.final_state, _xlfn.REDUCE(_xlpm.initial_state, _xlfn.SEQUENCE(_xlpm.max_iters), _xlfn.LAMBDA(_xlpm.state,_xlpm.i, _xlfn.LET(_xlpm.is_done, INDEX(_xlpm.state, 1, 1), _xlpm.curr_x, _xlfn.DROP(_xlpm.state, 1), IF(_xlpm.is_done, _xlpm.state, _xlfn.LET(_xlpm.div_packed, core_BigInt.DivRouter(_xlpm.limbs_n, _xlpm.curr_x, _xlpm.k), _xlpm.len_r, INDEX(_xlpm.div_packed, 1, 1), _xlpm.q, _xlfn.DROP(_xlpm.div_packed, _xlpm.len_r + 1), _xlpm.sum_xq, core_BigInt.UAdd(_xlpm.curr_x, _xlpm.q, _xlpm.k), _xlpm.div_2_packed, core_BigInt.KnuthDiv(_xlpm.sum_xq, {2}, _xlpm.k), _xlpm.len_r2, INDEX(_xlpm.div_2_packed, 1, 1), _xlpm.x_next, _xlfn.DROP(_xlpm.div_2_packed, _xlpm.len_r2 + 1), _xlpm.comp, core_BigInt.UCompare(_xlpm.x_next, _xlpm.curr_x), IF(_xlpm.comp &gt;= 0, _xlfn.VSTACK(1, _xlpm.curr_x), _xlfn.VSTACK(0, _xlpm.x_next))))))), _xlfn.DROP(_xlpm.final_state, 1)))</definedName>
-    <definedName name="core_BigInt.USub" comment="[Internal] Unsigned subtraction of two Little-Endian limb arrays._x000a_Assumes magnitudes A &gt;= B. Resolves borrows top-to-bottom and trims trailing zeros._x000a_@param limbs_a The minuend limb array (must be &gt;= limbs_b)._x000a_@param limbs_b The subtrahend limb array._x000a_@pa">_xlfn.LAMBDA(_xlpm.limbs_a,_xlpm.limbs_b,_xlpm.k, _xlfn.LET(_xlpm.max_rows, MAX(ROWS(_xlpm.limbs_a), ROWS(_xlpm.limbs_b)), _xlpm.pad_a, _xlfn.EXPAND(_xlpm.limbs_a, _xlpm.max_rows, 1, 0), _xlpm.pad_b, _xlfn.EXPAND(_xlpm.limbs_b, _xlpm.max_rows, 1, 0), _xlpm.diff, _xlpm.pad_a - _xlpm.pad_b, _xlpm.resolved, core_BigInt.Carry(_xlpm.diff, _xlpm.k), _xlpm.msd_idx, _xlfn.XMATCH(TRUE, _xlpm.resolved &lt;&gt; 0, 0, -1), IF(ISNA(_xlpm.msd_idx), {0}, _xlfn.TAKE(_xlpm.resolved, _xlpm.msd_idx))))</definedName>
-    <definedName name="core_BigInt.UTextMul" comment="[Internal] Unsafe, high-performance text multiplication for trusted, positive BigInt strings._x000a_Bypasses Layer 0 validation. Implements strict short-circuits for padding optimization._x000a_@param str_a The first trusted BigInt string._x000a_@param str_b The second tru">_xlfn.LAMBDA(_xlpm.str_a,_xlpm.str_b, IF(OR(_xlpm.str_a = "0", _xlpm.str_b = "0"), "0", IF(_xlpm.str_a = "1", _xlpm.str_b, IF(_xlpm.str_b = "1", _xlpm.str_a, _xlfn.LET(_xlpm.len_a, LEN(_xlpm.str_a), _xlpm.len_b, LEN(_xlpm.str_b), _xlpm.k, core_BigInt.SafeK("MUL", MIN(_xlpm.len_a, _xlpm.len_b)), _xlpm.limbs_a, core_BigInt.Split(_xlpm.str_a, _xlpm.k), _xlpm.limbs_b, core_BigInt.Split(_xlpm.str_b, _xlpm.k), _xlpm.final_limbs, core_BigInt.UMul(_xlpm.limbs_a, _xlpm.limbs_b, _xlpm.k), core_BigInt.Merge(_xlpm.final_limbs, _xlpm.k))))))</definedName>
+    <definedName name="core_BigInt.NativePrimes" comment="[Internal] Generates a 1D vertical array of all prime numbers up to n._x000a_Evaluates purely in native C++ using a dynamic sieve._x000a_@param n The upper bound integer (assumed &lt;= 9273).">_xlfn.LAMBDA(_xlpm.n, IF(_xlpm.n &lt; 2, #NUM!, _xlfn.LET(_xlpm.candidate_sequence, _xlfn.SEQUENCE(_xlpm.n - 1, 1, 2), _xlfn._xlws.FILTER(_xlpm.candidate_sequence, _xlfn.MAP(_xlpm.candidate_sequence, _xlfn.LAMBDA(_xlpm.current_candidate, _xlfn.LET(_xlpm.limit, INT(SQRT(_xlpm.current_candidate)), IF(_xlpm.limit &lt; 2, TRUE, MIN(MOD(_xlpm.current_candidate, _xlfn.SEQUENCE(_xlpm.limit - 1, 1, 2))) &gt; 0))))))))</definedName>
+    <definedName name="core_BigInt.NativeSwingExponents" comment="[Internal] Calculates the exponent for an array of primes in the Swing term of a factorial._x000a_@param n The current factorial magnitude (&lt;= 9273)._x000a_@param primes A vertical array of prime numbers (&lt;= n).">_xlfn.LAMBDA(_xlpm.n,_xlpm.primes, _xlfn.MAP(_xlpm.primes, _xlfn.LAMBDA(_xlpm.p, _xlfn.LET(_xlpm.max_power_k, INT(LOG(_xlpm.n, _xlpm.p)), _xlpm.prime_powers, _xlpm.p ^ _xlfn.SEQUENCE(_xlpm.max_power_k), SUM(MOD(INT(_xlpm.n / _xlpm.prime_powers), 2))))))</definedName>
+    <definedName name="core_BigInt.NewtonRaphsonDiv" comment="[Internal] Heavyweight Newton-Raphson Division._x000a_Implements progressive scaling bounded to MAX(len_a, len_b)._x000a_@param limbs_a The dividend array._x000a_@param limbs_b The divisor array._x000a_@param k The dynamic chunk size context.">_xlfn.LAMBDA(_xlpm.limbs_a,_xlpm.limbs_b,_xlpm.k, _xlfn.LET(_xlpm.num_limbs_a, ROWS(_xlpm.limbs_a), _xlpm.num_limbs_b, ROWS(_xlpm.limbs_b), _xlpm.num_limbs_target, MAX(_xlpm.num_limbs_a, _xlpm.num_limbs_b), _xlpm.limbs_reciprocal, core_BigInt.NewtonRaphsonReciprocal(_xlpm.limbs_b, _xlpm.num_limbs_target, _xlpm.k), _xlpm.right_shift_limbs, 2 * _xlpm.num_limbs_target, _xlpm.limbs_q_unscaled, core_BigInt.UMul(_xlpm.limbs_a, _xlpm.limbs_reciprocal, _xlpm.k), _xlpm.limbs_q_approx, IF(ROWS(_xlpm.limbs_q_unscaled) &lt;= _xlpm.right_shift_limbs, {0}, _xlfn.DROP(_xlpm.limbs_q_unscaled, _xlpm.right_shift_limbs)), _xlpm.limbs_p_baseline, core_BigInt.UMul(_xlpm.limbs_b, _xlpm.limbs_q_approx, _xlpm.k), _xlpm.initial_packed_state, _xlfn.VSTACK(ROWS(_xlpm.limbs_q_approx), _xlpm.limbs_q_approx, _xlpm.limbs_p_baseline), _xlpm.packed_state_swept_down, _xlfn.REDUCE(_xlpm.initial_packed_state, {1;2}, _xlfn.LAMBDA(_xlpm.packed_state,_xlpm.i, _xlfn.LET(_xlpm.len_q, INDEX(_xlpm.packed_state, 1, 1), _xlpm.limbs_current_q, _xlfn.CHOOSEROWS(_xlpm.packed_state, _xlfn.SEQUENCE(_xlpm.len_q, 1, 2)), _xlpm.limbs_current_p, _xlfn.DROP(_xlpm.packed_state, _xlpm.len_q + 1), IF(core_BigInt.UCompare(_xlpm.limbs_current_p, _xlpm.limbs_a) &lt;= 0, _xlpm.packed_state, _xlfn.LET(_xlpm.limbs_next_q, core_BigInt.USub(_xlpm.limbs_current_q, {1}, _xlpm.k), _xlpm.limbs_next_p, core_BigInt.USub(_xlpm.limbs_current_p, _xlpm.limbs_b, _xlpm.k), _xlfn.VSTACK(ROWS(_xlpm.limbs_next_q), _xlpm.limbs_next_q, _xlpm.limbs_next_p)))))), _xlpm.packed_state_swept_up, _xlfn.REDUCE(_xlpm.packed_state_swept_down, {1;2}, _xlfn.LAMBDA(_xlpm.packed_state,_xlpm.i, _xlfn.LET(_xlpm.len_q, INDEX(_xlpm.packed_state, 1, 1), _xlpm.limbs_current_q, _xlfn.CHOOSEROWS(_xlpm.packed_state, _xlfn.SEQUENCE(_xlpm.len_q, 1, 2)), _xlpm.limbs_current_p, _xlfn.DROP(_xlpm.packed_state, _xlpm.len_q + 1), _xlpm.limbs_next_p_test, core_BigInt.UAdd(_xlpm.limbs_current_p, _xlpm.limbs_b, _xlpm.k), IF(core_BigInt.UCompare(_xlpm.limbs_next_p_test, _xlpm.limbs_a) &gt; 0, _xlpm.packed_state, _xlfn.LET(_xlpm.limbs_next_q, core_BigInt.UAdd(_xlpm.limbs_current_q, {1}, _xlpm.k), _xlfn.VSTACK(ROWS(_xlpm.limbs_next_q), _xlpm.limbs_next_q, _xlpm.limbs_next_p_test)))))), _xlpm.len_q, INDEX(_xlpm.packed_state_swept_up, 1, 1), _xlpm.limbs_q, _xlfn.CHOOSEROWS(_xlpm.packed_state_swept_up, _xlfn.SEQUENCE(_xlpm.len_q, 1, 2)), _xlpm.limbs_p, _xlfn.DROP(_xlpm.packed_state_swept_up, _xlpm.len_q + 1), _xlpm.limbs_r, core_BigInt.USub(_xlpm.limbs_a, _xlpm.limbs_p, _xlpm.k), _xlfn.VSTACK(ROWS(_xlpm.limbs_r), _xlpm.limbs_r, _xlpm.limbs_q)))</definedName>
+    <definedName name="core_BigInt.NewtonRaphsonReciprocal" comment="[Internal] Computes the Reciprocal progressively scaling up to the Dividend's precision._x000a_@param limbs_b The divisor limb array._x000a_@param target_len The limb-length of Dividend A._x000a_@param k The dynamic chunk size context.">_xlfn.LAMBDA(_xlpm.limbs_b,_xlpm.target_len,_xlpm.k, _xlfn.LET(_xlpm.num_limbs_b, ROWS(_xlpm.limbs_b), _xlpm.num_seed_limbs, MIN(3, _xlpm.num_limbs_b), _xlpm.limbs_r_seed, core_BigInt.NewtonRaphsonSeed(_xlpm.limbs_b, _xlpm.k), _xlpm.required_iterations, MAX(0, _xlfn.CEILING.MATH(LN(_xlpm.target_len / _xlpm.num_seed_limbs) / LN(2))) + 1, IF(_xlpm.required_iterations = 0, _xlpm.limbs_r_seed, _xlfn.LET(_xlpm.iterations, _xlfn.SEQUENCE(_xlpm.required_iterations), _xlpm.final_packed_state, _xlfn.REDUCE(_xlfn.VSTACK(_xlpm.num_seed_limbs, _xlpm.limbs_r_seed), _xlpm.iterations, _xlfn.LAMBDA(_xlpm.packed_state,_xlpm.i, _xlfn.LET(_xlpm.current_len, INDEX(_xlpm.packed_state, 1, 1), _xlpm.limbs_current_r, _xlfn.DROP(_xlpm.packed_state, 1), _xlpm.next_len, MIN(_xlpm.current_len * 2, _xlpm.target_len), _xlpm.active_b_limbs_current, MIN(_xlpm.current_len, _xlpm.num_limbs_b), _xlpm.active_b_limbs_next, MIN(_xlpm.next_len, _xlpm.num_limbs_b), _xlpm.required_shift_limbs, 2 * (_xlpm.next_len - _xlpm.current_len) - (_xlpm.active_b_limbs_next - _xlpm.active_b_limbs_current), _xlpm.limbs_r_prime, IF(_xlpm.required_shift_limbs &gt; 0, _xlfn.VSTACK(_xlfn.EXPAND(0, _xlpm.required_shift_limbs, , 0), _xlpm.limbs_current_r), _xlpm.limbs_current_r), _xlpm.limbs_b_active, _xlfn.TAKE(_xlpm.limbs_b, -_xlpm.active_b_limbs_next), _xlpm.limbs_p, core_BigInt.UMul(_xlpm.limbs_b_active, _xlpm.limbs_r_prime, _xlpm.k), _xlpm.limbs_two_beta, _xlfn.VSTACK(_xlfn.EXPAND(0, 2 * _xlpm.next_len, , 0), 2), _xlpm.limbs_error_term, core_BigInt.USub(_xlpm.limbs_two_beta, _xlpm.limbs_p, _xlpm.k), _xlpm.limbs_next_r_unscaled, core_BigInt.UMul(_xlpm.limbs_r_prime, _xlpm.limbs_error_term, _xlpm.k), _xlpm.limbs_next_r, IF(ROWS(_xlpm.limbs_next_r_unscaled) &lt;= 2 * _xlpm.next_len, {0}, _xlfn.DROP(_xlpm.limbs_next_r_unscaled, 2 * _xlpm.next_len)), _xlfn.VSTACK(_xlpm.next_len, _xlpm.limbs_next_r)))), _xlfn.DROP(_xlpm.final_packed_state, 1)))))</definedName>
+    <definedName name="core_BigInt.NewtonRaphsonSeed" comment="[Internal] Generates the exact reciprocal seed for Newton-Raphson Division using Knuth Basecase._x000a_Extracts up to the top 3 limbs of B and calculates floor(Beta^(2*len) / B_top)._x000a_@param limbs_b The divisor limb array._x000a_@param k The dynamic chunk size context">_xlfn.LAMBDA(_xlpm.limbs_b,_xlpm.k, _xlfn.LET(_xlpm.num_limbs_b, ROWS(_xlpm.limbs_b), _xlpm.num_seed_limbs, MIN(3, _xlpm.num_limbs_b), _xlpm.limbs_b_top, _xlfn.TAKE(_xlpm.limbs_b, -_xlpm.num_seed_limbs), _xlpm.limbs_beta_2m, _xlfn.VSTACK(_xlfn.EXPAND(0, 2 * _xlpm.num_seed_limbs, , 0), 1), _xlpm.packed_basecase_result, core_BigInt.KnuthDiv(_xlpm.limbs_beta_2m, _xlpm.limbs_b_top, _xlpm.k), _xlpm.num_limbs_r, INDEX(_xlpm.packed_basecase_result, 1, 1), _xlfn.DROP(_xlpm.packed_basecase_result, _xlpm.num_limbs_r + 1)))</definedName>
+    <definedName name="core_BigInt.PrimeSwingKernel" comment="[Internal] Recursive top-down LAMBDA calculating the Prime Swing factorial._x000a_@param n The current factorial magnitude._x000a_@param global_primes The unified vertical array of all primes up to the target factorial.">_xlfn.LAMBDA(_xlpm.n,_xlpm.global_primes, IF(_xlpm.n &lt; 2, "1", _xlfn.LET(_xlpm.floor_half_n, INT(_xlpm.n / 2), _xlpm.factorial_half_n, core_BigInt.PrimeSwingKernel(_xlpm.floor_half_n, _xlpm.global_primes), _xlpm.squared_half_factorial, core_BigInt.UTextMul(_xlpm.factorial_half_n, _xlpm.factorial_half_n), _xlpm.applicable_tier_primes, _xlfn._xlws.FILTER(_xlpm.global_primes, _xlpm.global_primes &lt;= _xlpm.n), _xlpm.str_swing_term, core_BigInt.SwingTerm(_xlpm.n, _xlpm.applicable_tier_primes), core_BigInt.UTextMul(_xlpm.squared_half_factorial, _xlpm.str_swing_term))))</definedName>
+    <definedName name="core_BigInt.SafeK" comment="[Internal] Computes the maximum safe base-10 limb size (k) to avoid IEEE-754 precision loss._x000a_@param operation: &quot;ADD&quot;, &quot;MUL&quot;, or &quot;DIV&quot;._x000a_@param [max_items] ADD: number of operands. MUL: shortest string digits count.">_xlfn.LAMBDA(_xlpm.operation,_xlop.operand_or_digits, _xlfn.LET(_xlpm.resolved_count, IF(OR(_xlpm.operand_or_digits = "", _xlfn.ISOMITTED(_xlpm.operand_or_digits)), 2, MAX(2, _xlpm.operand_or_digits)), _xlfn.SWITCH(_xlpm.operation, "ADD", 15 - LEN(_xlpm.resolved_count), "MUL", _xlfn.LET(_xlpm.test_k, {7;6;5;4;3;2;1}, _xlpm.max_overlap, ROUNDUP(_xlpm.resolved_count / _xlpm.test_k, 0), _xlpm.uncarried_max, _xlpm.max_overlap * (10 ^ _xlpm.test_k - 1) ^ 2, _xlpm.max_carry, INT(_xlpm.uncarried_max / 10 ^ _xlpm.test_k), _xlpm.peak_val, _xlpm.uncarried_max + _xlpm.max_carry, MAX(_xlfn._xlws.FILTER(_xlpm.test_k, _xlpm.peak_val &lt;= (10 ^ 15 - 1)))), "DIV", 7, #NAME?)))</definedName>
+    <definedName name="core_BigInt.Split" comment="[Internal] Unified Splitter. Splits both scalars and arrays into Little-Endian limbs._x000a_Uses MAX() to guarantee scalar inputs to the SEQUENCE engine._x000a_@param big_ints The string or array of strings._x000a_@param k The dynamic chunk size context.">_xlfn.LAMBDA(_xlpm.str_norms,_xlpm.k, _xlfn.LET(_xlpm.flattened_norms, _xlfn.TOROW(_xlpm.str_norms), _xlpm.lengths, LEN(_xlpm.flattened_norms), _xlpm.max_len, MAX(_xlpm.lengths), _xlpm.pad_len, ROUNDUP(_xlpm.max_len / _xlpm.k, 0) * _xlpm.k, _xlpm.padded_norms, REPT("0", _xlpm.pad_len - _xlpm.lengths) &amp; _xlpm.flattened_norms, _xlpm.limb_start_indices, _xlfn.SEQUENCE(_xlpm.pad_len / _xlpm.k, 1, _xlpm.pad_len - _xlpm.k + 1, -_xlpm.k), --MID(_xlpm.padded_norms, _xlpm.limb_start_indices, _xlpm.k)))</definedName>
+    <definedName name="core_BigInt.SwingTerm" comment="[Internal] Calculates the massive BigInt string for the Swing term of a factorial._x000a_@param n The current factorial magnitude._x000a_@param tier_primes A vertical array of prime numbers (&lt;= n).">_xlfn.LAMBDA(_xlpm.n,_xlpm.tier_primes, _xlfn.LET(_xlpm.swing_exponents, core_BigInt.NativeSwingExponents(_xlpm.n, _xlpm.tier_primes), _xlpm.has_native_exponent, _xlpm.swing_exponents &gt; 0, IF(AND(NOT(_xlpm.has_native_exponent)), "1", _xlfn.LET(_xlpm.active_primes, _xlfn._xlws.FILTER(_xlpm.tier_primes, _xlpm.has_native_exponent), _xlpm.active_exponents, _xlfn._xlws.FILTER(_xlpm.swing_exponents, _xlpm.has_native_exponent), _xlpm.evalutated_prime_powers, _xlfn.MAP(_xlpm.active_primes, _xlpm.active_exponents, _xlfn.LAMBDA(_xlpm.p,_xlpm.e, IF(_xlpm.e = 1, _xlpm.p &amp; "", BigInt.Pow(_xlpm.p &amp; "", _xlpm.e &amp; "")))), core_BigInt.TextTreeProd(_xlpm.evalutated_prime_powers)))))</definedName>
+    <definedName name="core_BigInt.TextTreeProd" comment="[Internal] Vectorized logarithmic product of an array of BigInt strings._x000a_Recursively cuts the array in half to bypass REDUCE sequential memory allocations._x000a_@param arr_strings A 1D vertical array of BigInt strings.">_xlfn.LAMBDA(_xlpm.arr_strings, _xlfn.LET(_xlpm.num_elements, ROWS(_xlpm.arr_strings), IF(_xlpm.num_elements = 1, INDEX(_xlpm.arr_strings, 1, 1), _xlfn.LET(_xlpm.paired_strings, _xlfn.WRAPROWS(_xlpm.arr_strings, 2, "1"), _xlpm.reduced_array, _xlfn.BYROW(_xlpm.paired_strings, _xlfn.LAMBDA(_xlpm.row, core_BigInt.UTextMul(INDEX(_xlpm.row, 1, 1), INDEX(_xlpm.row, 1, 2)))), core_BigInt.TextTreeProd(_xlpm.reduced_array)))))</definedName>
+    <definedName name="core_BigInt.TreeCompare" comment="[Internal] Recursive tournament tree for Min/Max evaluations._x000a_@param col A 1D vertical array of normalized BigInt strings._x000a_@param mode 1 for Maximum, -1 for Minimum.">_xlfn.LAMBDA(_xlpm.str_norms,_xlpm.comparison_mode, _xlfn.LET(_xlpm.num_rows, ROWS(_xlpm.str_norms), IF(_xlpm.num_rows = 1, INDEX(_xlpm.str_norms, 1, 1), _xlfn.LET(_xlpm.tournament_pairs, _xlfn.WRAPROWS(_xlpm.str_norms, 2), _xlpm.competitors_a, _xlfn.TAKE(_xlpm.tournament_pairs, , 1), _xlpm.competitors_b, _xlfn.TAKE(_xlpm.tournament_pairs, , -1), _xlpm.round_winners, _xlfn.MAP(_xlpm.competitors_a, _xlpm.competitors_b, _xlfn.LAMBDA(_xlpm.a,_xlpm.b, IF(ISNA(_xlpm.b), _xlpm.a, _xlfn.LET(_xlpm.comparison_result, BigInt.Compare(_xlpm.a, _xlpm.b), IF(_xlpm.comparison_result * _xlpm.comparison_mode &gt;= 0, _xlpm.a, _xlpm.b))))), core_BigInt.TreeCompare(_xlpm.round_winners, _xlpm.comparison_mode)))))</definedName>
+    <definedName name="core_BigInt.UAdd" comment="[Internal] Unsigned addition of two Little-Endian limb arrays._x000a_@param limbs_a The first limb array._x000a_@param limbs_b The second limb array._x000a_@param k The dynamic chunk size context.">_xlfn.LAMBDA(_xlpm.a,_xlpm.b,_xlpm.k, _xlfn.LET(_xlpm.max_rows, MAX(ROWS(_xlpm.a), ROWS(_xlpm.b)), _xlpm.limbs_a_aligned, _xlfn.EXPAND(_xlpm.a, _xlpm.max_rows, 1, 0), _xlpm.limbs_b_aligned, _xlfn.EXPAND(_xlpm.b, _xlpm.max_rows, 1, 0), core_BigInt.Carry(_xlpm.limbs_a_aligned + _xlpm.limbs_b_aligned, _xlpm.k)))</definedName>
+    <definedName name="core_BigInt.UCompare" comment="[Internal] Unsigned comparison of two Little-Endian limb arrays._x000a_Returns 1 (a &gt; b), -1 (a &lt; b), or 0 (a = b)._x000a_@param limbs_a The first limb array._x000a_@param limbs_b The second limb array.">_xlfn.LAMBDA(_xlpm.limbs_a,_xlpm.limbs_b, _xlfn.LET(_xlpm.max_rows, MAX(ROWS(_xlpm.limbs_a), ROWS(_xlpm.limbs_b)), _xlpm.limbs_a_aligned, _xlfn.EXPAND(_xlpm.limbs_a, _xlpm.max_rows, 1, 0), _xlpm.limbs_b_aligned, _xlfn.EXPAND(_xlpm.limbs_b, _xlpm.max_rows, 1, 0), _xlpm.differences, _xlpm.limbs_a_aligned - _xlpm.limbs_b_aligned, _xlpm.highest_non_zero_index, _xlfn.XMATCH(TRUE, _xlpm.differences &lt;&gt; 0, 0, -1), IF(ISNA(_xlpm.highest_non_zero_index), 0, SIGN(INDEX(_xlpm.differences, _xlpm.highest_non_zero_index, 1)))))</definedName>
+    <definedName name="core_BigInt.UMatrixSum" comment="[Internal] Vectorized matrix sum of unsigned BigInt strings._x000a_@param str_norms Horizontal array (1xN) of normalized magnitude strings._x000a_@param k The unified dynamic chunk size context.">_xlfn.LAMBDA(_xlpm.str_norms,_xlpm.k, _xlfn.LET(_xlpm.grid, core_BigInt.Split(_xlpm.str_norms, _xlpm.k), _xlpm.raw_limbs, _xlfn.BYROW(_xlpm.grid, _xleta.SUM), core_BigInt.Carry(_xlpm.raw_limbs, _xlpm.k)))</definedName>
+    <definedName name="core_BigInt.UMul" comment="[Internal] Unsigned multiplication of two Little-Endian limb arrays._x000a_Utilizes a 1D Discrete Convolution (Cauchy Product) array-slicing strategy._x000a_Zero dynamic memory reallocation. $O(N+M)$ memory footprint._x000a_@param limbs_a The multiplicand limb array._x000a_@para">_xlfn.LAMBDA(_xlpm.limbs_a,_xlpm.limbs_b,_xlpm.k, _xlfn.LET(_xlpm.num_limbs_a, ROWS(_xlpm.limbs_a), _xlpm.num_limbs_b, ROWS(_xlpm.limbs_b), _xlpm.convolution_length, _xlpm.num_limbs_a + _xlpm.num_limbs_b - 1, _xlpm.raw_convolution, _xlfn.MAKEARRAY(_xlpm.convolution_length, 1, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, _xlfn.LET(_xlpm.window_start_i, MAX(1, _xlpm.r - _xlpm.num_limbs_b + 1), _xlpm.window_end_i, MIN(_xlpm.r, _xlpm.num_limbs_a), _xlpm.overlap_rows, _xlpm.window_end_i - _xlpm.window_start_i + 1, _xlpm.seq_i, _xlfn.SEQUENCE(_xlpm.overlap_rows, 1, _xlpm.window_start_i, 1), _xlpm.seq_j, _xlfn.SEQUENCE(_xlpm.overlap_rows, 1, _xlpm.r - _xlpm.window_start_i + 1, -1), SUM(INDEX(_xlpm.limbs_a, _xlpm.seq_i, 1) * INDEX(_xlpm.limbs_b, _xlpm.seq_j, 1))))), core_BigInt.Carry(_xlpm.raw_convolution, _xlpm.k)))</definedName>
+    <definedName name="core_BigInt.UPow" comment="[Internal] Unsigned Base-10 Left-to-Right Exponentiation._x000a_Evaluates the exponent iteratively using a pre-computed 1-9 cache._x000a_@param limbs_base The little-endian limb array of the base._x000a_@param exp_string The exact text string of the exponent._x000a_@param k The ">_xlfn.LAMBDA(_xlpm.limbs_base,_xlpm.exponent_string,_xlpm.k, _xlfn.LET(_xlpm.limbs_base1, _xlpm.limbs_base, _xlpm.limbs_base2, core_BigInt.UMul(_xlpm.limbs_base1, _xlpm.limbs_base1, _xlpm.k), _xlpm.limbs_base3, core_BigInt.UMul(_xlpm.limbs_base2, _xlpm.limbs_base1, _xlpm.k), _xlpm.limbs_base4, core_BigInt.UMul(_xlpm.limbs_base2, _xlpm.limbs_base2, _xlpm.k), _xlpm.limbs_base5, core_BigInt.UMul(_xlpm.limbs_base4, _xlpm.limbs_base1, _xlpm.k), _xlpm.limbs_base6, core_BigInt.UMul(_xlpm.limbs_base3, _xlpm.limbs_base3, _xlpm.k), _xlpm.limbs_base7, core_BigInt.UMul(_xlpm.limbs_base6, _xlpm.limbs_base1, _xlpm.k), _xlpm.limbs_base8, core_BigInt.UMul(_xlpm.limbs_base4, _xlpm.limbs_base4, _xlpm.k), _xlpm.limbs_base9, core_BigInt.UMul(_xlpm.limbs_base8, _xlpm.limbs_base1, _xlpm.k), _xlpm.exponent_digits, --MID(_xlpm.exponent_string, _xlfn.SEQUENCE(LEN(_xlpm.exponent_string)), 1), _xlfn.REDUCE(1, _xlpm.exponent_digits, _xlfn.LAMBDA(_xlpm.limbs_accumulator,_xlpm.current_digit, _xlfn.LET(_xlpm.is_one, AND(ROWS(_xlpm.limbs_accumulator) = 1, INDEX(_xlpm.limbs_accumulator, 1, 1) = 1), _xlpm.limbs_acc_10, IF(_xlpm.is_one, _xlpm.limbs_accumulator, _xlfn.LET(_xlpm.limbs_acc_2, core_BigInt.UMul(_xlpm.limbs_accumulator, _xlpm.limbs_accumulator, _xlpm.k), _xlpm.limbs_acc_4, core_BigInt.UMul(_xlpm.limbs_acc_2, _xlpm.limbs_acc_2, _xlpm.k), _xlpm.limbs_acc_8, core_BigInt.UMul(_xlpm.limbs_acc_4, _xlpm.limbs_acc_4, _xlpm.k), core_BigInt.UMul(_xlpm.limbs_acc_8, _xlpm.limbs_acc_2, _xlpm.k))), IF(_xlpm.current_digit = 0, _xlpm.limbs_acc_10, _xlfn.LET(_xlpm.limbs_cache_multiplier, CHOOSE(_xlpm.current_digit, _xlpm.limbs_base1, _xlpm.limbs_base2, _xlpm.limbs_base3, _xlpm.limbs_base4, _xlpm.limbs_base5, _xlpm.limbs_base6, _xlpm.limbs_base7, _xlpm.limbs_base8, _xlpm.limbs_base9), IF(_xlpm.is_one, _xlpm.limbs_cache_multiplier, core_BigInt.UMul(_xlpm.limbs_acc_10, _xlpm.limbs_cache_multiplier, _xlpm.k)))))))))</definedName>
+    <definedName name="core_BigInt.USqrt" comment="[Internal] Unsigned Integer Square Root using Newton's Method._x000a_@param limbs_radicand._x000a_@param limbs_initial_x Over-estimated seed array._x000a_@param k The dynamic chunk size context.">_xlfn.LAMBDA(_xlpm.limbs_radicand,_xlpm.limbs_initial_x,_xlpm.k, _xlfn.LET(_xlpm.maximum_iterations, 35, _xlpm.final_packed_state, _xlfn.REDUCE(_xlfn.VSTACK(0, _xlpm.limbs_initial_x), _xlfn.SEQUENCE(_xlpm.maximum_iterations), _xlfn.LAMBDA(_xlpm.packed_state,_xlpm.i, _xlfn.LET(_xlpm.has_converged, INDEX(_xlpm.packed_state, 1, 1), _xlpm.limbs_current_x, _xlfn.DROP(_xlpm.packed_state, 1), IF(_xlpm.has_converged, _xlpm.packed_state, _xlfn.LET(_xlpm.packed_division_result, core_BigInt.DivRouter(_xlpm.limbs_radicand, _xlpm.limbs_current_x, _xlpm.k), _xlpm.num_limbs_r, INDEX(_xlpm.packed_division_result, 1, 1), _xlpm.limbs_q, _xlfn.DROP(_xlpm.packed_division_result, _xlpm.num_limbs_r + 1), _xlpm.limbs_sum_xq, core_BigInt.UAdd(_xlpm.limbs_current_x, _xlpm.limbs_q, _xlpm.k), _xlpm.packed_half_result, core_BigInt.KnuthDiv(_xlpm.limbs_sum_xq, {2}, _xlpm.k), _xlpm.num_limbs_halfed, INDEX(_xlpm.packed_half_result, 1, 1), _xlpm.limbs_next_x, _xlfn.DROP(_xlpm.packed_half_result, _xlpm.num_limbs_halfed + 1), _xlpm.convergence_comparison, core_BigInt.UCompare(_xlpm.limbs_next_x, _xlpm.limbs_current_x), IF(_xlpm.convergence_comparison &gt;= 0, _xlfn.VSTACK(1, _xlpm.limbs_current_x), _xlfn.VSTACK(0, _xlpm.limbs_next_x))))))), _xlfn.DROP(_xlpm.final_packed_state, 1)))</definedName>
+    <definedName name="core_BigInt.USub" comment="[Internal] Unsigned subtraction of two Little-Endian limb arrays._x000a_Assumes magnitudes A &gt;= B. Resolves borrows top-to-bottom and trims trailing zeros._x000a_@param limbs_a The minuend limb array (must be &gt;= limbs_b)._x000a_@param limbs_b The subtrahend limb array._x000a_@pa">_xlfn.LAMBDA(_xlpm.limbs_a,_xlpm.limbs_b,_xlpm.k, _xlfn.LET(_xlpm.max_rows, MAX(ROWS(_xlpm.limbs_a), ROWS(_xlpm.limbs_b)), _xlpm.limbs_a_aligned, _xlfn.EXPAND(_xlpm.limbs_a, _xlpm.max_rows, 1, 0), _xlpm.limbs_b_aligned, _xlfn.EXPAND(_xlpm.limbs_b, _xlpm.max_rows, 1, 0), _xlpm.differences, _xlpm.limbs_a_aligned - _xlpm.limbs_b_aligned, _xlpm.carried_differences, core_BigInt.Carry(_xlpm.differences, _xlpm.k), _xlpm.highest_non_zero_index, _xlfn.XMATCH(TRUE, _xlpm.carried_differences &lt;&gt; 0, 0, -1), IF(ISNA(_xlpm.highest_non_zero_index), {0}, _xlfn.TAKE(_xlpm.carried_differences, _xlpm.highest_non_zero_index))))</definedName>
+    <definedName name="core_BigInt.UTextMul" comment="[Internal] Unsafe, high-performance text multiplication for normalised, positive BigInt strings._x000a_Bypasses Layer 0 validation. Implements strict short-circuits for padding optimization._x000a_@param norm_a_x000a_@param norm_b">_xlfn.LAMBDA(_xlpm.norm_a,_xlpm.norm_b, IF(OR(_xlpm.norm_a = "0", _xlpm.norm_b = "0"), "0", IF(_xlpm.norm_a = "1", _xlpm.norm_b, IF(_xlpm.norm_b = "1", _xlpm.norm_a, _xlfn.LET(_xlpm.len_a, LEN(_xlpm.norm_a), _xlpm.len_b, LEN(_xlpm.norm_b), _xlpm.k, core_BigInt.SafeK("MUL", MIN(_xlpm.len_a, _xlpm.len_b)), _xlpm.limbs_a, core_BigInt.Split(_xlpm.norm_a, _xlpm.k), _xlpm.limbs_b, core_BigInt.Split(_xlpm.norm_b, _xlpm.k), _xlpm.final_limbs, core_BigInt.UMul(_xlpm.limbs_a, _xlpm.limbs_b, _xlpm.k), core_BigInt.Merge(_xlpm.final_limbs, _xlpm.k))))))</definedName>
     <definedName name="test_BigInt.AsymmetricABGrid">_xlfn.LAMBDA(_xlpm.start_a,_xlpm.max_a,_xlpm.step_a,_xlpm.start_b,_xlpm.max_b,_xlpm.step_b, _xlfn.LET(_xlpm.seq_a, _xlfn.SEQUENCE((_xlpm.max_a - _xlpm.start_a) / _xlpm.step_a + 1, 1, _xlpm.start_a, _xlpm.step_a), _xlpm.seq_b, _xlfn.SEQUENCE((_xlpm.max_b - _xlpm.start_b) / _xlpm.step_b + 1, 1, _xlpm.start_b, _xlpm.step_b), _xlpm.n_a, ROWS(_xlpm.seq_a), _xlpm.n_b, ROWS(_xlpm.seq_b), _xlpm.col_a, _xlfn.TOCOL(IF(_xlfn.SEQUENCE(1, _xlpm.n_b), _xlpm.seq_a)), _xlpm.col_b, _xlfn.TOCOL(IF(_xlfn.SEQUENCE(_xlpm.n_a), _xlfn.TOROW(_xlpm.seq_b))), _xlfn.HSTACK(_xlpm.col_a, _xlpm.col_b)))</definedName>
     <definedName name="test_BigInt.DivisionAlgorithmComparison" comment="Executes a strictly sequential benchmark suite to avoid multi-threading contamination._x000a_@param test_cases An N x 2 array of test lengths: [Length_A, Length_B]_x000a_@param iters Number of iterations per benchmark to smooth NOW() resolution.">_xlfn.LAMBDA(_xlpm.test_cases,_xlpm.iters,_xlpm.repeats, _xlfn.LET(_xlpm.n_tests, ROWS(_xlpm.test_cases), _xlpm.initial, {"Len_A","Len_B","Knuth_ms","NR_ms"}, _xlfn.REDUCE(_xlpm.initial, _xlfn.SEQUENCE(_xlpm.n_tests), _xlfn.LAMBDA(_xlpm.acc,_xlpm.i, _xlfn.LET(_xlpm.len_a, INDEX(_xlpm.test_cases, _xlpm.i, 1), _xlpm.len_b, INDEX(_xlpm.test_cases, _xlpm.i, 2), IF(_xlpm.len_b &gt; _xlpm.len_a, _xlpm.acc, _xlfn.LET(_xlpm.str_a, REPT("9", _xlpm.len_a), _xlpm.str_b, IF(_xlpm.len_b = 1, "7", "7" &amp; REPT("3", _xlpm.len_b - 1)), _xlpm.time_k, test_BigInt.DivisionAlgorithms(_xlpm.str_a, _xlpm.str_b, "KNUTH", _xlpm.iters, _xlpm.repeats), _xlpm.time_nr, test_BigInt.DivisionAlgorithms(_xlpm.str_a, _xlpm.str_b, "NR", _xlpm.iters, _xlpm.repeats), _xlfn.VSTACK(_xlpm.acc, _xlfn.HSTACK(_xlpm.len_a, _xlpm.len_b, _xlpm.time_k, _xlpm.time_nr)))))))))</definedName>
     <definedName name="test_BigInt.DivisionAlgorithms" comment="@param a The dividend string_x000a_@param b The divisor string_x000a_@param mode &quot;KNUTH&quot; or &quot;NR&quot;_x000a_@param iters Inner loop count (to defeat chunky clock resolution)_x000a_@param repeats Outer loop count (to defeat OS/Garbage Collection noise)">_xlfn.LAMBDA(_xlpm.a,_xlpm.b,_xlpm.mode,_xlpm.iters,_xlpm.repeats, _xlfn.LET(_xlpm.batch_times, _xlfn.MAP(_xlfn.SEQUENCE(_xlpm.repeats), _xlfn.LAMBDA(_xlpm.r, _xlfn.LET(_xlpm.start, NOW(), _xlpm.run, IF(_xlpm.mode = "KNUTH", _xlfn.MAP(_xlfn.SEQUENCE(_xlpm.iters), _xlfn.LAMBDA(_xlpm.i, test_BigInt.KnuthDivision(_xlpm.a, _xlpm.b))), _xlfn.MAP(_xlfn.SEQUENCE(_xlpm.iters), _xlfn.LAMBDA(_xlpm.i, test_BigInt.NewtonRaphsonDivision(_xlpm.a, _xlpm.b)))), _xlpm.stop, NOW() + (0 * LEN(INDEX(_xlpm.run, 1, 1))), (_xlpm.stop - _xlpm.start) * 86400000))), MIN(_xlpm.batch_times) / _xlpm.iters))</definedName>
@@ -12235,7 +12235,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="1805" row="6">
+  <wetp:taskpane dockstate="right" visibility="0" width="1659" row="6">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -21597,7 +21597,7 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAHQAZQBzAHQAXwBCAGkAZwBJAG4AdAAiACwAIgB0AGUAeAB0ACIAOgAiAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAFwAbgAvAC8AIABCAGkAZwAgAEkAbgB0AGUAZwBlAHIAIABBAHIAaQB0AGgAbQBlAHQAaQBjACAATABpAGIAcgBhAHIAeQAgAC8ALwBcAG4ALwAvACAAIAAgACAAIAAgACAAdABlAHMAdABfAEIAaQBnAEkAbgB0ACAATQBvAGQAdQBsAGUAIAAgACAAIAAgACAAIAAvAC8AXABuAC8ALwAgACAAIAAgACAAIAAgAFAAcgBpAHYAYQB0AGUAIABUAGUAcwB0AGkAbgBnACAAQQBQAEkAIAAgACAAIAAgACAALwAvAFwAbgAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwBcAG4AXABuAEsAbgB1AHQAaABEAGkAdgBpAHMAaQBvAG4APQBMAEEATQBCAEQAQQAoAGEALAAgAGIALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAawAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwBhAGYAZQBLACgAXAAiAEQASQBWAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABwAGEAYwBrAGUAZAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4ASwBuAHUAdABoAEQAaQB2ACgAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwBwAGwAaQB0ACgAYQAsACAAawApACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBTAHAAbABpAHQAKABiACwAIABrACkALAAgAGsAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAE0AZQByAGcAZQAoAEQAUgBPAFAAKABwAGEAYwBrAGUAZAAsACAASQBOAEQARQBYACgAcABhAGMAawBlAGQALAAgADEALAAgADEAKQAgACsAIAAxACkALAAgAGsAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBOAGUAdwB0AG8AbgBSAGEAcABoAHMAbwBuAEQAaQB2AGkAcwBpAG8AbgAgAD0AIABMAEEATQBCAEQAQQAoAGEALAAgAGIALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAawAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwBhAGYAZQBLACgAXAAiAEQASQBWAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABwAGEAYwBrAGUAZAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4ATgBlAHcAdABvAG4AUgBhAHAAaABzAG8AbgBEAGkAdgAoAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFMAcABsAGkAdAAoAGEALAAgAGsAKQAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwBwAGwAaQB0ACgAYgAsACAAawApACwAIABrACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBNAGUAcgBnAGUAKABEAFIATwBQACgAcABhAGMAawBlAGQALAAgAEkATgBEAEUAWAAoAHAAYQBjAGsAZQBkACwAIAAxACwAIAAxACkAIAArACAAMQApACwAIABrACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAEAAcABhAHIAYQBtACAAYQAgAFQAaABlACAAZABpAHYAaQBkAGUAbgBkACAAcwB0AHIAaQBuAGcAXABuACAAKgAgAEAAcABhAHIAYQBtACAAYgAgAFQAaABlACAAZABpAHYAaQBzAG8AcgAgAHMAdAByAGkAbgBnAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAG0AbwBkAGUAIABcACIASwBOAFUAVABIAFwAIgAgAG8AcgAgAFwAIgBOAFIAXAAiAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGkAdABlAHIAcwAgAEkAbgBuAGUAcgAgAGwAbwBvAHAAIABjAG8AdQBuAHQAIAAoAHQAbwAgAGQAZQBmAGUAYQB0ACAAYwBoAHUAbgBrAHkAIABjAGwAbwBjAGsAIAByAGUAcwBvAGwAdQB0AGkAbwBuACkAXABuACAAKgAgAEAAcABhAHIAYQBtACAAcgBlAHAAZQBhAHQAcwAgAE8AdQB0AGUAcgAgAGwAbwBvAHAAIABjAG8AdQBuAHQAIAAoAHQAbwAgAGQAZQBmAGUAYQB0ACAATwBTAC8ARwBhAHIAYgBhAGcAZQAgAEMAbwBsAGwAZQBjAHQAaQBvAG4AIABuAG8AaQBzAGUAKQBcAG4AIAAqAC8AXABuAEQAaQB2AGkAcwBpAG8AbgBBAGwAZwBvAHIAaQB0AGgAbQBzACAAPQAgAEwAQQBNAEIARABBACgAYQAsACAAYgAsACAAbQBvAGQAZQAsACAAaQB0AGUAcgBzACwAIAByAGUAcABlAGEAdABzACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAC8ALwAgAE0AYQBwACAAdABoAGUAIABvAHUAdABlAHIAIAByAGUAcABlAGEAdABzACAAbABvAG8AcABcAG4AIAAgACAAIAAgACAAIAAgAGIAYQB0AGMAaABfAHQAaQBtAGUAcwAsACAATQBBAFAAKABTAEUAUQBVAEUATgBDAEUAKAByAGUAcABlAGEAdABzACkALAAgAEwAQQBNAEIARABBACgAcgAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHMAdABhAHIAdAAsACAATgBPAFcAKAApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAATQBhAHAAIAB0AGgAZQAgAGkAbgBuAGUAcgAgAGUAeABlAGMAdQB0AGkAbwBuACAAbABvAG8AcABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAByAHUAbgAsACAASQBGACgAbQBvAGQAZQAgAD0AIABcACIASwBOAFUAVABIAFwAIgAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAE0AQQBQACgAUwBFAFEAVQBFAE4AQwBFACgAaQB0AGUAcgBzACkALAAgAEwAQQBNAEIARABBACgAaQAsACAASwBuAHUAdABoAEQAaQB2AGkAcwBpAG8AbgAoAGEALAAgAGIAKQApACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBBAFAAKABTAEUAUQBVAEUATgBDAEUAKABpAHQAZQByAHMAKQAsACAATABBAE0AQgBEAEEAKABpACwAIABOAGUAdwB0AG8AbgBSAGEAcABoAHMAbwBuAEQAaQB2AGkAcwBpAG8AbgAoAGEALAAgAGIAKQApACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAEYAbwByAGMAZQAgAGUAdgBhAGwAdQBhAHQAaQBvAG4AIABiAGUAZgBvAHIAZQAgAHAAdQBsAGwAaQBuAGcAIABzAHQAbwBwACAAdABpAG0AZQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABzAHQAbwBwACwAIABOAE8AVwAoACkAIAArACAAKAAwACAAKgAgAEwARQBOACgASQBOAEQARQBYACgAcgB1AG4ALAAgADEALAAgADEAKQApACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIABUAG8AdABhAGwAIABiAGEAdABjAGgAIAB0AGkAbQBlACAAaQBuACAAbQBpAGwAbABpAHMAZQBjAG8AbgBkAHMAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABzAHQAbwBwACAALQAgAHMAdABhAHIAdAApACAAKgAgADgANgA0ADAAMAAwADAAMABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABFAHgAdAByAGEAYwB0ACAAdABoAGUAIABjAGwAZQBhAG4AZQBzAHQAIAByAHUAbgAgAGEAbgBkACAAYQB2AGUAcgBhAGcAZQAgAGkAdAAgAGQAbwB3AG4AIAB0AG8AIABhACAAcwBpAG4AZwBsAGUAIABlAHgAZQBjAHUAdABpAG8AbgAgAHQAaQBtAGUAXABuACAAIAAgACAAIAAgACAAIABNAEkATgAoAGIAYQB0AGMAaABfAHQAaQBtAGUAcwApACAALwAgAGkAdABlAHIAcwBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAARQB4AGUAYwB1AHQAZQBzACAAYQAgAHMAdAByAGkAYwB0AGwAeQAgAHMAZQBxAHUAZQBuAHQAaQBhAGwAIABiAGUAbgBjAGgAbQBhAHIAawAgAHMAdQBpAHQAZQAgAHQAbwAgAGEAdgBvAGkAZAAgAG0AdQBsAHQAaQAtAHQAaAByAGUAYQBkAGkAbgBnACAAYwBvAG4AdABhAG0AaQBuAGEAdABpAG8AbgAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAHQAZQBzAHQAXwBjAGEAcwBlAHMAIABBAG4AIABOACAAeAAgADIAIABhAHIAcgBhAHkAIABvAGYAIAB0AGUAcwB0ACAAbABlAG4AZwB0AGgAcwA6ACAAWwBMAGUAbgBnAHQAaABfAEEALAAgAEwAZQBuAGcAdABoAF8AQgBdAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGkAdABlAHIAcwAgAE4AdQBtAGIAZQByACAAbwBmACAAaQB0AGUAcgBhAHQAaQBvAG4AcwAgAHAAZQByACAAYgBlAG4AYwBoAG0AYQByAGsAIAB0AG8AIABzAG0AbwBvAHQAaAAgAE4ATwBXACgAKQAgAHIAZQBzAG8AbAB1AHQAaQBvAG4ALgBcAG4AIAAqAC8AXABuAEQAaQB2AGkAcwBpAG8AbgBBAGwAZwBvAHIAaQB0AGgAbQBDAG8AbQBwAGEAcgBpAHMAbwBuACAAPQAgAEwAQQBNAEIARABBACgAdABlAHMAdABfAGMAYQBzAGUAcwAsACAAaQB0AGUAcgBzACwAIAByAGUAcABlAGEAdABzACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG4AXwB0AGUAcwB0AHMALAAgAFIATwBXAFMAKAB0AGUAcwB0AF8AYwBhAHMAZQBzACkALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAALwAvACAASQBuAGkAdABpAGEAbAAgAHMAdABhAHQAZQA6ACAARABhAHQAYQAgAGgAZQBhAGQAZQByAHMAIABmAG8AcgAgAEMAUwBWACAAZQB4AHAAbwByAHQAXABuACAAIAAgACAAIAAgACAAIABpAG4AaQB0AGkAYQBsACwAIAB7AFwAIgBMAGUAbgBfAEEAXAAiACwAIABcACIATABlAG4AXwBCAFwAIgAsACAAXAAiAEsAbgB1AHQAaABfAG0AcwBcACIALAAgAFwAIgBOAFIAXwBtAHMAXAAiAH0ALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAUgBFAEQAVQBDAEUAKABpAG4AaQB0AGkAYQBsACwAIABTAEUAUQBVAEUATgBDAEUAKABuAF8AdABlAHMAdABzACkALAAgAEwAQQBNAEIARABBACgAYQBjAGMALAAgAGkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGUAbgBfAGEALAAgAEkATgBEAEUAWAAoAHQAZQBzAHQAXwBjAGEAcwBlAHMALAAgAGkALAAgADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAZQBuAF8AYgAsACAASQBOAEQARQBYACgAdABlAHMAdABfAGMAYQBzAGUAcwAsACAAaQAsACAAMgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAAUwBrAGkAcAAgAEQAaQB2AGkAcwBvAHIAIAA+ACAARABpAHYAaQBkAGUAbgBkABQgaQB0ACcAcwAgAG4AZQB2AGUAcgAgAGEAbgAgAGkAbgB0AGUAZwBlAHIAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgAbABlAG4AXwBiACAAPgAgAGwAZQBuAF8AYQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABhAGMAYwAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAARwBlAG4AZQByAGEAdABlACAAZQB4AGEAYwB0AC0AbABlAG4AZwB0AGgAIAB0AGUAcwB0ACAAcwB0AHIAaQBuAGcAcwAgAG4AYQB0AGkAdgBlAGwAeQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcwB0AHIAXwBhACwAIABSAEUAUABUACgAXAAiADkAXAAiACwAIABsAGUAbgBfAGEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABzAHQAcgBfAGIALAAgAEkARgAoAGwAZQBuAF8AYgAgAD0AIAAxACwAIABcACIANwBcACIALAAgAFwAIgA3AFwAIgAgACYAIABSAEUAUABUACgAXAAiADMAXAAiACwAIABsAGUAbgBfAGIAIAAtACAAMQApACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAEUAeABlAGMAdQB0AGUAIABiAGUAbgBjAGgAbQBhAHIAawBzACAAcwB0AHIAaQBjAHQAbAB5ACAAbwBuAGUAIABhAGYAdABlAHIAIAB0AGgAZQAgAG8AdABoAGUAcgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAdABpAG0AZQBfAGsALAAgAEQAaQB2AGkAcwBpAG8AbgBBAGwAZwBvAHIAaQB0AGgAbQBzACgAcwB0AHIAXwBhACwAIABzAHQAcgBfAGIALAAgAFwAIgBLAE4AVQBUAEgAXAAiACwAIABpAHQAZQByAHMALAAgAHIAZQBwAGUAYQB0AHMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAB0AGkAbQBlAF8AbgByACwAIABEAGkAdgBpAHMAaQBvAG4AQQBsAGcAbwByAGkAdABoAG0AcwAoAHMAdAByAF8AYQAsACAAcwB0AHIAXwBiACwAIABcACIATgBSAFwAIgAsACAAaQB0AGUAcgBzACwAIAByAGUAcABlAGEAdABzACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAEEAcABwAGUAbgBkACAAdABoAGUAIAByAGUAcwB1AGwAdABzAC4AIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAAUgBlAGEAbABsAG8AYwBhAHQAaQBvAG4AIABkAGUAbABhAHkAIABvAGMAYwB1AHIAcwAgAGgAZQByAGUALAAgAHMAYQBmAGUAbAB5ACAAbwB1AHQAcwBpAGQAZQAgAHQAaABlACAAdABpAG0AZQBkACAAdwBpAG4AZABvAHcALgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAVgBTAFQAQQBDAEsAKABhAGMAYwAsACAASABTAFQAQQBDAEsAKABsAGUAbgBfAGEALAAgAGwAZQBuAF8AYgAsACAAdABpAG0AZQBfAGsALAAgAHQAaQBtAGUAXwBuAHIAKQApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8ALwAgAEcAZQBuAGUAcgBhAHQAZQBzACAAYQAgADIALQBjAG8AbAB1AG0AbgAgAGEAcgByAGEAeQAgAG8AZgAgAGUAdgBlAHIAeQAgAGMAbwBtAGIAaQBuAGEAdABpAG8AbgAgAG8AZgAgAGwAZQBuAGcAdABoAHMAXABuAEQAaQB2AGkAcwBpAG8AbgBCAGUAbgBjAGgAbQBhAHIAawBDAGEAcwBlAHMAIAA9ACAATABBAE0AQgBEAEEAKABzAHQAYQByAHQAXwBsAGUAbgAsACAAbQBhAHgAXwBsAGUAbgAsACAAcwB0AGUAcAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABzAGUAcQAsACAAUwBFAFEAVQBFAE4AQwBFACgAKABtAGEAeABfAGwAZQBuACAALQAgAHMAdABhAHIAdABfAGwAZQBuACkAIAAvACAAcwB0AGUAcAAgACsAIAAxACwAIAAxACwAIABzAHQAYQByAHQAXwBsAGUAbgAsACAAcwB0AGUAcAApACwAXABuACAAIAAgACAAIAAgACAAIABuACwAIABSAE8AVwBTACgAcwBlAHEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABDAGEAcgB0AGUAcwBpAGEAbgAgAEoAbwBpAG4AXABuACAAIAAgACAAIAAgACAAIABjAG8AbABfAGEALAAgAFQATwBDAE8ATAAoAEkARgAoAFMARQBRAFUARQBOAEMARQAoADEALAAgAG4AKQAsACAAcwBlAHEAKQApACwAXABuACAAIAAgACAAIAAgACAAIABjAG8AbABfAGIALAAgAFQATwBDAE8ATAAoAEkARgAoAFMARQBRAFUARQBOAEMARQAoAG4ALAAgADEAKQAsACAAVABPAFIATwBXACgAcwBlAHEAKQApACkALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAASABTAFQAQQBDAEsAKABjAG8AbABfAGEALAAgAGMAbwBsAF8AYgApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8ALwAgAEcAZQBuAGUAcgBhAHQAZQBzACAAYQAgAEMAYQByAHQAZQBzAGkAYQBuACAAZwByAGkAZAAgAGYAcgBvAG0AIAB0AHcAbwAgAGkAbgBkAGUAcABlAG4AZABlAG4AdAAgAHMAZQBxAHUAZQBuAGMAZQBzAFwAbgBBAHMAeQBtAG0AZQB0AHIAaQBjAEEAQgBHAHIAaQBkACAAPQAgAEwAQQBNAEIARABBACgAcwB0AGEAcgB0AF8AYQAsACAAbQBhAHgAXwBhACwAIABzAHQAZQBwAF8AYQAsACAAcwB0AGEAcgB0AF8AYgAsACAAbQBhAHgAXwBiACwAIABzAHQAZQBwAF8AYgAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABzAGUAcQBfAGEALAAgAFMARQBRAFUARQBOAEMARQAoACgAbQBhAHgAXwBhACAALQAgAHMAdABhAHIAdABfAGEAKQAgAC8AIABzAHQAZQBwAF8AYQAgACsAIAAxACwAIAAxACwAIABzAHQAYQByAHQAXwBhACwAIABzAHQAZQBwAF8AYQApACwAXABuACAAIAAgACAAIAAgACAAIABzAGUAcQBfAGIALAAgAFMARQBRAFUARQBOAEMARQAoACgAbQBhAHgAXwBiACAALQAgAHMAdABhAHIAdABfAGIAKQAgAC8AIABzAHQAZQBwAF8AYgAgACsAIAAxACwAIAAxACwAIABzAHQAYQByAHQAXwBiACwAIABzAHQAZQBwAF8AYgApACwAXABuACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgAG4AXwBhACwAIABSAE8AVwBTACgAcwBlAHEAXwBhACkALABcAG4AIAAgACAAIAAgACAAIAAgAG4AXwBiACwAIABSAE8AVwBTACgAcwBlAHEAXwBiACkALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAALwAvACAATwByAHQAaABvAGcAbwBuAGEAbAAgAGIAcgBvAGEAZABjAGEAcwB0ACAAdQBzAGkAbgBnACAAaQBuAGQAZQBwAGUAbgBkAGUAbgB0ACAAZABpAG0AZQBuAHMAaQBvAG4AcwBcAG4AIAAgACAAIAAgACAAIAAgAGMAbwBsAF8AYQAsACAAVABPAEMATwBMACgASQBGACgAUwBFAFEAVQBFAE4AQwBFACgAMQAsACAAbgBfAGIAKQAsACAAcwBlAHEAXwBhACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAYwBvAGwAXwBiACwAIABUAE8AQwBPAEwAKABJAEYAKABTAEUAUQBVAEUATgBDAEUAKABuAF8AYQApACwAIABUAE8AUgBPAFcAKABzAGUAcQBfAGIAKQApACkALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAASABTAFQAQQBDAEsAKABjAG8AbABfAGEALAAgAGMAbwBsAF8AYgApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAEYAYQBjAHQAbwByAGkAYQBsAEEAbABnAG8AcgBpAHQAaABtAHMAIAA9ACAATABBAE0AQgBEAEEAKABpAG4AcAB1AHQALAAgAG0AbwBkAGUALAAgAGkAdABlAHIAcwAsACAAcgBlAHAAZQBhAHQAcwAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABNAGEAcAAgAHQAaABlACAAbwB1AHQAZQByACAAcgBlAHAAZQBhAHQAcwAgAGwAbwBvAHAAXABuACAAIAAgACAAIAAgACAAIABiAGEAdABjAGgAXwB0AGkAbQBlAHMALAAgAE0AQQBQACgAUwBFAFEAVQBFAE4AQwBFACgAcgBlAHAAZQBhAHQAcwApACwAIABMAEEATQBCAEQAQQAoAHIALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQALAAgAE4ATwBXACgAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAE0AYQBwACAAdABoAGUAIABpAG4AbgBlAHIAIABlAHgAZQBjAHUAdABpAG8AbgAgAGwAbwBvAHAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcgB1AG4ALAAgAEkARgAoAG0AbwBkAGUAIAA9ACAAXAAiAEwAZQBnAGUAbgBkAHIAZQBcACIALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEEAUAAoAFMARQBRAFUARQBOAEMARQAoAGkAdABlAHIAcwApACwAIABMAEEATQBCAEQAQQAoAGkALAAgAEIAaQBnAEkAbgB0AC4ARgBhAGMAdAAoAGkAbgBwAHUAdAApACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEEAUAAoAFMARQBRAFUARQBOAEMARQAoAGkAdABlAHIAcwApACwAIABMAEEATQBCAEQAQQAoAGkALAAgAEIAaQBnAEkAbgB0AC4ARgBhAGMAdABTAHcAaQBuAGcAKABpAG4AcAB1AHQAKQApACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAEYAbwByAGMAZQAgAGUAdgBhAGwAdQBhAHQAaQBvAG4AIABiAGUAZgBvAHIAZQAgAHAAdQBsAGwAaQBuAGcAIABzAHQAbwBwACAAdABpAG0AZQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABzAHQAbwBwACwAIABOAE8AVwAoACkAIAArACAAKAAwACAAKgAgAEwARQBOACgASQBOAEQARQBYACgAcgB1AG4ALAAgADEALAAgADEAKQApACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIABUAG8AdABhAGwAIABiAGEAdABjAGgAIAB0AGkAbQBlACAAaQBuACAAbQBpAGwAbABpAHMAZQBjAG8AbgBkAHMAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABzAHQAbwBwACAALQAgAHMAdABhAHIAdAApACAAKgAgADgANgA0ADAAMAAwADAAMABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABFAHgAdAByAGEAYwB0ACAAdABoAGUAIABjAGwAZQBhAG4AZQBzAHQAIAByAHUAbgAgAGEAbgBkACAAYQB2AGUAcgBhAGcAZQAgAGkAdAAgAGQAbwB3AG4AIAB0AG8AIABhACAAcwBpAG4AZwBsAGUAIABlAHgAZQBjAHUAdABpAG8AbgAgAHQAaQBtAGUAXABuACAAIAAgACAAIAAgACAAIABNAEkATgAoAGIAYQB0AGMAaABfAHQAaQBtAGUAcwApACAALwAgAGkAdABlAHIAcwBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAARQB4AGUAYwB1AHQAZQBzACAAYQAgAHMAdAByAGkAYwB0AGwAeQAgAHMAZQBxAHUAZQBuAHQAaQBhAGwAIABiAGUAbgBjAGgAbQBhAHIAawAgAHMAdQBpAHQAZQAgAHQAbwAgAGEAdgBvAGkAZAAgAG0AdQBsAHQAaQAtAHQAaAByAGUAYQBkAGkAbgBnACAAYwBvAG4AdABhAG0AaQBuAGEAdABpAG8AbgAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAHQAZQBzAHQAXwBjAGEAcwBlAHMAIABBAG4AIABOACAAeAAgADEAIABhAHIAcgBhAHkAIABvAGYAIAB0AGUAcwB0ACAAaQBuAHAAdQB0AHMAXABuACAAKgAgAEAAcABhAHIAYQBtACAAaQB0AGUAcgBzACAATgB1AG0AYgBlAHIAIABvAGYAIABpAHQAZQByAGEAdABpAG8AbgBzACAAcABlAHIAIABzAGEAbQBwAGwAZQAgAHQAbwAgAHMAbQBvAG8AdABoACAATgBPAFcAKAApACAAcgBlAHMAbwBsAHUAdABpAG8AbgAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAHIAZQBwAGUAYQB0AHMAIABOAHUAbQBiAGUAcgAgAG8AZgAgAGkAdABlAHIAYQB0AGkAbwBuAHMAIABwAGUAcgAgAGIAZQBuAGMAaABtAGEAcgBrACAAdABvACAAcwBtAG8AbwB0AGgAIABPAFMAIABhAG4AZAAgAGIAYQBjAGsAZwByAG8AdQBuAGQAIABuAG8AaQBzAGUALgBcAG4AIAAqAC8AXABuAEYAYQBjAHQAbwByAGkAYQBsAEMAbwBtAHAAYQByAGkAcwBvAG4AIAA9ACAATABBAE0AQgBEAEEAKAB0AGUAcwB0AF8AYwBhAHMAZQBzACwAIABpAHQAZQByAHMALAAgAHIAZQBwAGUAYQB0AHMALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbgBfAHQAZQBzAHQAcwAsACAAUgBPAFcAUwAoAHQAZQBzAHQAXwBjAGEAcwBlAHMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABJAG4AaQB0AGkAYQBsACAAcwB0AGEAdABlADoAIABEAGEAdABhACAAaABlAGEAZABlAHIAcwAgAGYAbwByACAAQwBTAFYAIABlAHgAcABvAHIAdABcAG4AIAAgACAAIAAgACAAIAAgAGkAbgBpAHQAaQBhAGwALAAgAHsAXAAiAE4AXAAiACwAIABcACIATABlAGcAZQBuAGQAcgBlAFwAIgAsACAAXAAiAFMAdwBpAG4AZwBcACIAfQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIABSAEUARABVAEMARQAoAGkAbgBpAHQAaQBhAGwALAAgAFMARQBRAFUARQBOAEMARQAoAG4AXwB0AGUAcwB0AHMAKQAsACAATABBAE0AQgBEAEEAKABhAGMAYwAsACAAaQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGkAbgBwAHUAdAAsACAASQBOAEQARQBYACgAdABlAHMAdABfAGMAYQBzAGUAcwAsACAAaQAsACAAMQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAARQB4AGUAYwB1AHQAZQAgAGIAZQBuAGMAaABtAGEAcgBrAHMAIABzAHQAcgBpAGMAdABsAHkAIABvAG4AZQAgAGEAZgB0AGUAcgAgAHQAaABlACAAbwB0AGgAZQByAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHQAaQBtAGUAXwBsAGUAZwBlAG4AZAByAGUALAAgAEYAYQBjAHQAbwByAGkAYQBsAEEAbABnAG8AcgBpAHQAaABtAHMAKABpAG4AcAB1AHQALAAgAFwAIgBMAGUAZwBlAG4AZAByAGUAXAAiACwAIABpAHQAZQByAHMALAAgAHIAZQBwAGUAYQB0AHMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHQAaQBtAGUAXwBzAHcAaQBuAGcALAAgAEYAYQBjAHQAbwByAGkAYQBsAEEAbABnAG8AcgBpAHQAaABtAHMAKABpAG4AcAB1AHQALAAgAFwAIgBTAHcAaQBuAGcAXAAiACwAIABpAHQAZQByAHMALAAgAHIAZQBwAGUAYQB0AHMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAEEAcABwAGUAbgBkACAAdABoAGUAIAByAGUAcwB1AGwAdABzAC4AIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIABSAGUAYQBsAGwAbwBjAGEAdABpAG8AbgAgAGQAZQBsAGEAeQAgAG8AYwBjAHUAcgBzACAAaABlAHIAZQAsACAAcwBhAGYAZQBsAHkAIABvAHUAdABzAGkAZABlACAAdABoAGUAIAB0AGkAbQBlAGQAIAB3AGkAbgBkAG8AdwAuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFYAUwBUAEEAQwBLACgAYQBjAGMALAAgAEgAUwBUAEEAQwBLACgAaQBuAHAAdQB0ACwAIAB0AGkAbQBlAF8AbABlAGcAZQBuAGQAcgBlACwAIAB0AGkAbQBlAF8AcwB3AGkAbgBnACkAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBjAG8AcgBlAF8AQgBpAGcASQBuAHQAIgAsACIAdABlAHgAdAAiADoAIgAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwBcAG4ALwAvACAAQgBpAGcAIABJAG4AdABlAGcAZQByACAAQQByAGkAdABoAG0AZQB0AGkAYwAgAEwAaQBiAHIAYQByAHkAIAAvAC8AXABuAC8ALwAgACAAIAAgACAAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQAIABNAG8AZAB1AGwAZQAgACAAIAAgACAAIAAgACAALwAvAFwAbgAvAC8AIAAgACAAIAAgACAAIAAgACAAIABQAHIAaQB2AGEAdABlACAAQQBQAEkAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwBcAG4ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8AXABuAFwAbgAvACoAKgBcAG4AIAAqACAAWwBJAG4AdABlAHIAbgBhAGwAXQAgAEMAbwBtAHAAdQB0AGUAcwAgAHQAaABlACAAbQBhAHgAaQBtAHUAbQAgAHMAYQBmAGUAIABiAGEAcwBlAC0AMQAwACAAbABpAG0AYgAgAHMAaQB6AGUAIAAoAGsAKQAgAHQAbwAgAGEAdgBvAGkAZAAgAEkARQBFAEUALQA3ADUANAAgAHAAcgBlAGMAaQBzAGkAbwBuACAAbABvAHMAcwAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAG8AcABlAHIAYQB0AGkAbwBuADoAIABcACIAQQBEAEQAXAAiACwAIABcACIATQBVAEwAXAAiACwAIABvAHIAIABcACIARABJAFYAXAAiAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAWwBtAGEAeABfAGkAdABlAG0AcwBdACAAQQBEAEQAOgAgAG4AdQBtAGIAZQByACAAbwBmACAAbwBwAGUAcgBhAG4AZABzAC4AIABNAFUATAA6ACAAcwBoAG8AcgB0AGUAcwB0ACAAcwB0AHIAaQBuAGcAIABkAGkAZwBpAHQAcwAgAGMAbwB1AG4AdAAuAFwAbgAgACoALwBcAG4AUwBhAGYAZQBLACAAPQAgAEwAQQBNAEIARABBACgAbwBwAGUAcgBhAHQAaQBvAG4ALAAgAFsAbQBhAHgAXwBpAHQAZQBtAHMAXQAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABpAHQAZQBtAHMALAAgAEkARgAoAE8AUgAoAG0AYQB4AF8AaQB0AGUAbQBzACAAPQAgAFwAIgBcACIALAAgAEkAUwBPAE0ASQBUAFQARQBEACgAbQBhAHgAXwBpAHQAZQBtAHMAKQApACwAIAAyACwAIABNAEEAWAAoADIALAAgAG0AYQB4AF8AaQB0AGUAbQBzACkAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAFMAVwBJAFQAQwBIACgAbwBwAGUAcgBhAHQAaQBvAG4ALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEARABEAFwAIgAsACAAMQA1ACAALQAgAEwARQBOACgAaQB0AGUAbQBzACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAFUATABcACIALAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAARQB2AGEAbAB1AGEAdABlACAAcABvAHMAcwBpAGIAbABlACAAawAgAHYAYQBsAHUAZQBzACAAZAB5AG4AYQBtAGkAYwBhAGwAbAB5AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHQAZQBzAHQAXwBrACwAIAB7ADcAOwAgADYAOwAgADUAOwAgADQAOwAgADMAOwAgADIAOwAgADEAfQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAG0AYQB4AF8AbwB2AGUAcgBsAGEAcAAsACAAUgBPAFUATgBEAFUAUAAoAGkAdABlAG0AcwAgAC8AIAB0AGUAcwB0AF8AawAsACAAMAApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAAQwBhAGwAYwB1AGwAYQB0AGUAIAB0AGgAZQAgAGEAYgBzAG8AbAB1AHQAZQAgAHAAZQBhAGsAIAB2AGEAbAB1AGUAIABpAG4AcwBpAGQAZQAgAHQAaABlACAAZQBuAGcAaQBuAGUAIAAoAEMAbwBuAHYAbwBsAHUAdABpAG8AbgAgACsAIABDAGEAcgByAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAB1AG4AYwBhAHIAcgBpAGUAZABfAG0AYQB4ACwAIABtAGEAeABfAG8AdgBlAHIAbABhAHAAIAAqACAAKAAxADAAXgB0AGUAcwB0AF8AawAgAC0AIAAxACkAXgAyACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbQBhAHgAXwBjAGEAcgByAHkALAAgAEkATgBUACgAdQBuAGMAYQByAHIAaQBlAGQAXwBtAGEAeAAgAC8AIAAxADAAXgB0AGUAcwB0AF8AawApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcABlAGEAawBfAHYAYQBsACwAIAB1AG4AYwBhAHIAcgBpAGUAZABfAG0AYQB4ACAAKwAgAG0AYQB4AF8AYwBhAHIAcgB5ACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAAUgBlAHQAdQByAG4AIAB0AGgAZQAgAG0AYQB4ACAAawAgADwAPQAgAEUAeABjAGUAbAAnAHMAIAAxADUALQBkAGkAZwBpAHQAIABjAGUAaQBsAGkAbgBnAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAE0AQQBYACgARgBJAEwAVABFAFIAKAB0AGUAcwB0AF8AawAsACAAcABlAGEAawBfAHYAYQBsACAAPAA9ACAAKAAxADAAXgAxADUAIAAtACAAMQApACkAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQASQBWAFwAIgAsACAANwAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAjAE4AQQBNAEUAPwBcAG4AIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFsASQBuAHQAZQByAG4AYQBsAF0AIABVAG4AaQBmAGkAZQBkACAAUwBwAGwAaQB0AHQAZQByAC4AIABTAHAAbABpAHQAcwAgAGIAbwB0AGgAIABzAGMAYQBsAGEAcgBzACAAYQBuAGQAIABhAHIAcgBhAHkAcwAgAGkAbgB0AG8AIABMAGkAdAB0AGwAZQAtAEUAbgBkAGkAYQBuACAAbABpAG0AYgBzAC4AXABuACAAKgAgAFUAcwBlAHMAIABNAEEAWAAoACkAIAB0AG8AIABnAHUAYQByAGEAbgB0AGUAZQAgAHMAYwBhAGwAYQByACAAaQBuAHAAdQB0AHMAIAB0AG8AIAB0AGgAZQAgAFMARQBRAFUARQBOAEMARQAgAGUAbgBnAGkAbgBlAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAYgBpAGcAXwBpAG4AdABzACAAVABoAGUAIABzAHQAcgBpAG4AZwAgAG8AcgAgAGEAcgByAGEAeQAgAG8AZgAgAHMAdAByAGkAbgBnAHMALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABrACAAVABoAGUAIABkAHkAbgBhAG0AaQBjACAAYwBoAHUAbgBrACAAcwBpAHoAZQAgAGMAbwBuAHQAZQB4AHQALgBcAG4AIAAqAC8AXABuAFMAcABsAGkAdAAgAD0AIABMAEEATQBCAEQAQQAoAGIAaQBnAF8AaQBuAHQAcwAsACAAawAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABiAGkAZwBfAGkAbgB0AF8AcgBvAHcALAAgAFQATwBSAE8AVwAoAGIAaQBnAF8AaQBuAHQAcwApACwAXABuACAAIAAgACAAIAAgACAAIABsAGUAbgBnAHQAaABzACwAIABMAEUATgAoAGIAaQBnAF8AaQBuAHQAXwByAG8AdwApACwAXABuACAAIAAgACAAIAAgACAAIABtAGEAeABfAGwAZQBuACwAIABNAEEAWAAoAGwAZQBuAGcAdABoAHMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcABhAGQAXwBsAGUAbgAsACAAUgBPAFUATgBEAFUAUAAoAG0AYQB4AF8AbABlAG4AIAAvACAAawAsACAAMAApACAAKgAgAGsALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAcABhAGQAZABlAGQALAAgAFIARQBQAFQAKABcACIAMABcACIALAAgAHAAYQBkAF8AbABlAG4AIAAtACAAbABlAG4AZwB0AGgAcwApACAAJgAgAGIAaQBnAF8AaQBuAHQAXwByAG8AdwAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AGEAcgB0AHMALAAgAFMARQBRAFUARQBOAEMARQAoAHAAYQBkAF8AbABlAG4AIAAvACAAawAsACAAMQAsACAAcABhAGQAXwBsAGUAbgAgAC0AIABrACAAKwAgADEALAAgAC0AawApACwAXABuACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgAC0ALQBNAEkARAAoAHAAYQBkAGQAZQBkACwAIABzAHQAYQByAHQAcwAsACAAawApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABbAEkAbgB0AGUAcgBuAGEAbABdACAAQwBvAG4AYwBhAHQAZQBuAGEAdABlAHMAIABhAG4AIABhAHIAcgBhAHkAIABvAGYAIABuAHUAbQBlAHIAaQBjACAAbABpAG0AYgBzACAAaQBuAHQAbwAgAGEAIABCAGkAZwBJAG4AdAAgAHMAdAByAGkAbgBnACwAIAB6AGUAcgBvAC0AcABhAGQAZABpAG4AZwAgAGEAbABsACAAYgB1AHQAIAB0AGgAZQAgAGYAaQByAHMAdAAgAGwAaQBtAGIALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABsAGkAbQBiAHMAIABUAGgAZQAgAHYAZQByAHQAaQBjAGEAbAAgAGEAcgByAGEAeQAgAG8AZgAgAG4AdQBtAGUAcgBpAGMAIABsAGkAbQBiAHMALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABrACAAVABoAGUAIABsAGkAbQBiACAAcwBpAHoAZQAgAHUAcwBlAGQAIABkAHUAcgBpAG4AZwAgAGMAYQBsAGMAdQBsAGEAdABpAG8AbgAuAFwAbgAgACoALwBcAG4ATQBlAHIAZwBlACAAPQAgAEwAQQBNAEIARABBACgAbABpAG0AYgBzACwAIABrACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG4AdQBtAF8AbABpAG0AYgBzACwAIABSAE8AVwBTACgAbABpAG0AYgBzACkALABcAG4AIAAgACAAIAAgACAAIAAgAHIAZQB2AF8AbABpAG0AYgBzACwAIABDAEgATwBPAFMARQBSAE8AVwBTACgAbABpAG0AYgBzACwAIABTAEUAUQBVAEUATgBDAEUAKABuAHUAbQBfAGwAaQBtAGIAcwAsACAAMQAsACAAbgB1AG0AXwBsAGkAbQBiAHMALAAgAC0AMQApACkALABcAG4AIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAG4AdQBtAF8AbABpAG0AYgBzACAAPQAgADEALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAcgBlAHYAXwBsAGkAbQBiAHMAIAAmACAAXAAiAFwAIgAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABDAE8ATgBDAEEAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFYAUwBUAEEAQwBLACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABUAEEASwBFACgAcgBlAHYAXwBsAGkAbQBiAHMALAAgADEAKQAgACYAIABcACIAXAAiACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABUAEUAWABUACgARABSAE8AUAAoAHIAZQB2AF8AbABpAG0AYgBzACwAIAAxACkALAAgAFIARQBQAFQAKABcACIAMABcACIALAAgAGsAKQApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABbAEkAbgB0AGUAcgBuAGEAbABdACAAUgBlAHMAbwBsAHYAZQBzACAAYwBhAHIAcgBpAGUAcwAgAHIAaQBnAGgAdAAtAHQAbwAtAGwAZQBmAHQAIABhAGMAcgBvAHMAcwAgAGEAIAB2AGUAcgB0AGkAYwBhAGwAIABhAHIAcgBhAHkAIABvAGYAIABiAGEAcwBlAC0AMQAwAF4AawAgAGwAaQBtAGIAcwAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGwAaQBtAGIAcwAgAFQAaABlACAAYQByAHIAYQB5ACAAbwBmACAAbgB1AG0AZQByAGkAYwAgAGwAaQBtAGIAcwAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGsAIABUAGgAZQAgAGwAaQBtAGIAIABzAGkAegBlAC4AXABuACAAKgAvAFwAbgBDAGEAcgByAHkAIAA9ACAATABBAE0AQgBEAEEAKABsAGkAbQBiAHMALAAgAGsALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbgAsACAAUgBPAFcAUwAoAGwAaQBtAGIAcwApACwAXABuACAAIAAgACAAIAAgACAAIABiAGEAcwBlACwAIAAxADAAXgBrACwAXABuACAAIAAgACAAIAAgACAAIABzAGMAYQBuAG4AZQBkACwAIABTAEMAQQBOACgAMAAsACAAbABpAG0AYgBzACwAIABMAEEATQBCAEQAQQAoAGEAYwBjACwAIAB2AGEAbAAsACAAdgBhAGwAIAArACAASQBOAFQAKABhAGMAYwAgAC8AIABiAGEAcwBlACkAKQApACwAXABuACAAIAAgACAAIAAgACAAIAByAGUAbQBhAGkAbgBkAGUAcgBzACwAIABNAE8ARAAoAHMAYwBhAG4AbgBlAGQALAAgAGIAYQBzAGUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAG4AYQBsAF8AYwBhAHIAcgB5ACwAIABJAE4AVAAoAEkATgBEAEUAWAAoAHMAYwBhAG4AbgBlAGQALAAgAG4ALAAgADEAKQAgAC8AIABiAGEAcwBlACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIABJAEYAKABmAGkAbgBhAGwAXwBjAGEAcgByAHkAIAA+ACAAMAAsACAAVgBTAFQAQQBDAEsAKAByAGUAbQBhAGkAbgBkAGUAcgBzACwAIABmAGkAbgBhAGwAXwBjAGEAcgByAHkAKQAsACAAcgBlAG0AYQBpAG4AZABlAHIAcwApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8ALwAgAC0ALQAtACAAVQBuAHMAaQBnAG4AZQBkACAASwBlAHIAbgBlAGwAcwAgAC0ALQAtACAAXABcAFwAXABcAG4AXABuAC8AKgAqAFwAbgAgACoAIABbAEkAbgB0AGUAcgBuAGEAbABdACAAVQBuAHMAaQBnAG4AZQBkACAAYwBvAG0AcABhAHIAaQBzAG8AbgAgAG8AZgAgAHQAdwBvACAATABpAHQAdABsAGUALQBFAG4AZABpAGEAbgAgAGwAaQBtAGIAIABhAHIAcgBhAHkAcwAuAFwAbgAgACoAIABSAGUAdAB1AHIAbgBzACAAMQAgACgAYQAgAD4AIABiACkALAAgAC0AMQAgACgAYQAgADwAIABiACkALAAgAG8AcgAgADAAIAAoAGEAIAA9ACAAYgApAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAbABpAG0AYgBzAF8AYQAgAFQAaABlACAAZgBpAHIAcwB0ACAAbABpAG0AYgAgAGEAcgByAGEAeQAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGwAaQBtAGIAcwBfAGIAIABUAGgAZQAgAHMAZQBjAG8AbgBkACAAbABpAG0AYgAgAGEAcgByAGEAeQAuAFwAbgAgACoALwBcAG4AVQBDAG8AbQBwAGEAcgBlACAAPQAgAEwAQQBNAEIARABBACgAbABpAG0AYgBzAF8AYQAsACAAbABpAG0AYgBzAF8AYgAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABtAGEAeABfAHIAbwB3AHMALAAgAE0AQQBYACgAUgBPAFcAUwAoAGwAaQBtAGIAcwBfAGEAKQAsACAAUgBPAFcAUwAoAGwAaQBtAGIAcwBfAGIAKQApACwAXABuACAAIAAgACAAIAAgACAAIABwAGEAZABfAGEALAAgAEUAWABQAEEATgBEACgAbABpAG0AYgBzAF8AYQAsACAAbQBhAHgAXwByAG8AdwBzACwAIAAxACwAIAAwACkALABcAG4AIAAgACAAIAAgACAAIAAgAHAAYQBkAF8AYgAsACAARQBYAFAAQQBOAEQAKABsAGkAbQBiAHMAXwBiACwAIABtAGEAeABfAHIAbwB3AHMALAAgADEALAAgADAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIABkAGkAZgBmACwAIABwAGEAZABfAGEAIAAtACAAcABhAGQAXwBiACwAXABuACAAIAAgACAAIAAgACAAIABtAHMAZABfAGkAZAB4ACwAIABYAE0AQQBUAEMASAAoAFQAUgBVAEUALAAgAGQAaQBmAGYAIAA8AD4AIAAwACwAIAAwACwAIAAtADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATgBBACgAbQBzAGQAXwBpAGQAeAApACwAIAAwACwAIABTAEkARwBOACgASQBOAEQARQBYACgAZABpAGYAZgAsACAAbQBzAGQAXwBpAGQAeAAsACAAMQApACkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAAWwBJAG4AdABlAHIAbgBhAGwAXQAgAFUAbgBzAGkAZwBuAGUAZAAgAGEAZABkAGkAdABpAG8AbgAgAG8AZgAgAHQAdwBvACAATABpAHQAdABsAGUALQBFAG4AZABpAGEAbgAgAGwAaQBtAGIAIABhAHIAcgBhAHkAcwAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGwAaQBtAGIAcwBfAGEAIABUAGgAZQAgAGYAaQByAHMAdAAgAGwAaQBtAGIAIABhAHIAcgBhAHkALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABsAGkAbQBiAHMAXwBiACAAVABoAGUAIABzAGUAYwBvAG4AZAAgAGwAaQBtAGIAIABhAHIAcgBhAHkALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABrACAAVABoAGUAIABkAHkAbgBhAG0AaQBjACAAYwBoAHUAbgBrACAAcwBpAHoAZQAgAGMAbwBuAHQAZQB4AHQALgBcAG4AIAAqAC8AXABuAFUAQQBkAGQAIAA9ACAATABBAE0AQgBEAEEAKABhACwAIABiACwAIABrACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQB4AF8AcgBvAHcAcwAsACAATQBBAFgAKABSAE8AVwBTACgAYQApACwAIABSAE8AVwBTACgAYgApACkALABcAG4AIAAgACAAIAAgACAAIAAgAHAAYQBkAF8AYQAsACAARQBYAFAAQQBOAEQAKABhACwAIABtAGEAeABfAHIAbwB3AHMALAAgADEALAAgADAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcABhAGQAXwBiACwAIABFAFgAUABBAE4ARAAoAGIALAAgAG0AYQB4AF8AcgBvAHcAcwAsACAAMQAsACAAMAApACwAXABuACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAYQByAHIAeQAoAHAAYQBkAF8AYQAgACsAIABwAGEAZABfAGIALAAgAGsAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAAWwBJAG4AdABlAHIAbgBhAGwAXQAgAFUAbgBzAGkAZwBuAGUAZAAgAHMAdQBiAHQAcgBhAGMAdABpAG8AbgAgAG8AZgAgAHQAdwBvACAATABpAHQAdABsAGUALQBFAG4AZABpAGEAbgAgAGwAaQBtAGIAIABhAHIAcgBhAHkAcwAuAFwAbgAgACoAIABBAHMAcwB1AG0AZQBzACAAbQBhAGcAbgBpAHQAdQBkAGUAcwAgAEEAIAA+AD0AIABCAC4AIABSAGUAcwBvAGwAdgBlAHMAIABiAG8AcgByAG8AdwBzACAAdABvAHAALQB0AG8ALQBiAG8AdAB0AG8AbQAgAGEAbgBkACAAdAByAGkAbQBzACAAdAByAGEAaQBsAGkAbgBnACAAegBlAHIAbwBzAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAbABpAG0AYgBzAF8AYQAgAFQAaABlACAAbQBpAG4AdQBlAG4AZAAgAGwAaQBtAGIAIABhAHIAcgBhAHkAIAAoAG0AdQBzAHQAIABiAGUAIAA+AD0AIABsAGkAbQBiAHMAXwBiACkALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABsAGkAbQBiAHMAXwBiACAAVABoAGUAIABzAHUAYgB0AHIAYQBoAGUAbgBkACAAbABpAG0AYgAgAGEAcgByAGEAeQAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGsAIABUAGgAZQAgAGQAeQBuAGEAbQBpAGMAIABjAGgAdQBuAGsAIABzAGkAegBlACAAYwBvAG4AdABlAHgAdAAuAFwAbgAgACoALwBcAG4AVQBTAHUAYgAgAD0AIABMAEEATQBCAEQAQQAoAGwAaQBtAGIAcwBfAGEALAAgAGwAaQBtAGIAcwBfAGIALAAgAGsALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHgAXwByAG8AdwBzACwAIABNAEEAWAAoAFIATwBXAFMAKABsAGkAbQBiAHMAXwBhACkALAAgAFIATwBXAFMAKABsAGkAbQBiAHMAXwBiACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcABhAGQAXwBhACwAIABFAFgAUABBAE4ARAAoAGwAaQBtAGIAcwBfAGEALAAgAG0AYQB4AF8AcgBvAHcAcwAsACAAMQAsACAAMAApACwAXABuACAAIAAgACAAIAAgACAAIABwAGEAZABfAGIALAAgAEUAWABQAEEATgBEACgAbABpAG0AYgBzAF8AYgAsACAAbQBhAHgAXwByAG8AdwBzACwAIAAxACwAIAAwACkALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAZABpAGYAZgAsACAAcABhAGQAXwBhACAALQAgAHAAYQBkAF8AYgAsAFwAbgAgACAAIAAgACAAIAAgACAAcgBlAHMAbwBsAHYAZQBkACwAIABDAGEAcgByAHkAKABkAGkAZgBmACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAbQBzAGQAXwBpAGQAeAAsACAAWABNAEEAVABDAEgAKABUAFIAVQBFACwAIAByAGUAcwBvAGwAdgBlAGQAIAA8AD4AIAAwACwAIAAwACwAIAAtADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATgBBACgAbQBzAGQAXwBpAGQAeAApACwAIAB7ADAAfQAsACAAVABBAEsARQAoAHIAZQBzAG8AbAB2AGUAZAAsACAAbQBzAGQAXwBpAGQAeAApACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFsASQBuAHQAZQByAG4AYQBsAF0AIABWAGUAYwB0AG8AcgBpAHoAZQBkACAAbQBhAHQAcgBpAHgAIABzAHUAbQAgAG8AZgAgAHUAbgBzAGkAZwBuAGUAZAAgAEIAaQBnAEkAbgB0ACAAcwB0AHIAaQBuAGcAcwAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAHUAYgBpAGcAXwBpAG4AdAAgAEgAbwByAGkAegBvAG4AdABhAGwAIABhAHIAcgBhAHkAIAAoADEAeABOACkAIABvAGYAIABuAG8AcgBtAGEAbABpAHoAZQBkACAAbQBhAGcAbgBpAHQAdQBkAGUAIABzAHQAcgBpAG4AZwBzAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAawAgAFQAaABlACAAdQBuAGkAZgBpAGUAZAAgAGQAeQBuAGEAbQBpAGMAIABjAGgAdQBuAGsAIABzAGkAegBlACAAYwBvAG4AdABlAHgAdAAuAFwAbgAgACoALwBcAG4AVQBNAGEAdAByAGkAeABTAHUAbQAgAD0AIABMAEEATQBCAEQAQQAoAHUAYgBpAGcAXwBpAG4AdABzACwAIABrACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAGcAcgBpAGQALAAgAFMAcABsAGkAdAAoAHUAYgBpAGcAXwBpAG4AdABzACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgAHIAYQB3AF8AbABpAG0AYgBzACwAIABCAFkAUgBPAFcAKABnAHIAaQBkACwAIABTAFUATQApACwAXABuACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAYQByAHIAeQAoAHIAYQB3AF8AbABpAG0AYgBzACwAIABrACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFsASQBuAHQAZQByAG4AYQBsAF0AIABSAG8AdQB0AGUAcwAgAGEAZABkAGkAdABpAG8AbgAvAHMAdQBiAHQAcgBhAGMAdABpAG8AbgAgAGIAYQBzAGUAZAAgAG8AbgAgAHMAaQBnAG4AcwAgAGEAbgBkACAAbQBhAGcAbgBpAHQAdQBkAGUAcwAuAFwAbgAgACoAIABSAGUAdAB1AHIAbgBzACAAYQAgAHQAdQBwAGwAZQAgAGEAcgByAGEAeQA6ACAAVgBTAFQAQQBDAEsAKABsAGkAbQBiAHMALAAgAGYAaQBuAGEAbABfAHMAaQBnAG4AKQAgAHcAaABlAHIAZQAgAHQAaABlACAAZgBpAG4AYQBsACAAcgBvAHcAIABpAHMAIAB0AGgAZQAgAHMAYwBhAGwAYQByACAAcwBpAGcAbgAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGwAaQBtAGIAcwBfAGEAIABUAGgAZQAgAGYAaQByAHMAdAAgAGwAaQB0AHQAbABlAC0AZQBuAGQAaQBhAG4AIABsAGkAbQBiACAAYQByAHIAYQB5AC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAbABpAG0AYgBzAF8AYgAgAFQAaABlACAAcwBlAGMAbwBuAGQAIABsAGkAdAB0AGwAZQAtAGUAbgBkAGkAYQBuACAAbABpAG0AYgAgAGEAcgByAGEAeQAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAHMAaQBnAG4AXwBhACAAVABoAGUAIABzAGkAZwBuACAAbwBmACAAdABoAGUAIABmAGkAcgBzAHQAIABhAHIAcgBhAHkAIAAoADEALAAgAC0AMQAsACAAMAApAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAcwBpAGcAbgBfAGIAIABUAGgAZQAgAHMAaQBnAG4AIABvAGYAIAB0AGgAZQAgAHMAZQBjAG8AbgBkACAAYQByAHIAYQB5ACAAKAAxACwAIAAtADEALAAgADAAKQAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGsAIABUAGgAZQAgAGQAeQBuAGEAbQBpAGMAIABjAGgAdQBuAGsAIABzAGkAegBlACAAYwBvAG4AdABlAHgAdAAuAFwAbgAgACoALwBcAG4AQQBkAGQAUwB1AGIAUgBvAHUAdABlAHIAIAA9ACAATABBAE0AQgBEAEEAKABsAGkAbQBiAHMAXwBhACwAIABsAGkAbQBiAHMAXwBiACwAIABzAGkAZwBuAF8AYQAsACAAcwBpAGcAbgBfAGIALAAgAGsALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAaQBzAF8AcwBhAG0AZQBfAHMAaQBnAG4ALAAgAHMAaQBnAG4AXwBhACAAPQAgAHMAaQBnAG4AXwBiACwAXABuACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAGkAcwBfAHMAYQBtAGUAXwBzAGkAZwBuACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAEEAZABkAGkAdABpAG8AbgA6ACAAbQBhAGcAbgBpAHQAdQBkAGUAcwAgAGMAbwBtAGIAaQBuAGUALAAgAHMAaQBnAG4AIAByAGUAbQBhAGkAbgBzACAAdABoAGUAIABzAGEAbQBlAC4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFYAUwBUAEEAQwBLACgAVQBBAGQAZAAoAGwAaQBtAGIAcwBfAGEALAAgAGwAaQBtAGIAcwBfAGIALAAgAGsAKQAsACAAcwBpAGcAbgBfAGEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAAUwB1AGIAdAByAGEAYwB0AGkAbwBuADoAIABlAHYAYQBsAHUAYQB0AGUAIABtAGEAZwBuAGkAdAB1AGQAZQBzACAAdABvACAAcwBhAHQAaQBzAGYAeQAgAFUAUwB1AGIAIAAoAEEAIAA+AD0AIABCACkAIABwAHIAZQBjAG8AbgBkAGkAdABpAG8AbgAuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAG0AYQBnAF8AYwBvAG0AcAAsACAAVQBDAG8AbQBwAGEAcgBlACgAbABpAG0AYgBzAF8AYQAsACAAbABpAG0AYgBzAF8AYgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgAbQBhAGcAXwBjAG8AbQBwACAAPQAgADAALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAFQAbwB0AGEAbAAgAGMAYQBuAGMAZQBsAGwAYQB0AGkAbwBuADoAIAByAGUAdAB1AHIAbgAgAHsAMAB9ACAAbABpAG0AYgAgAGEAbgBkACAAMAAgAHMAaQBnAG4ALgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHsAMAA7ADAAfQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABtAGEAZwBfAGMAbwBtAHAAIAA+ACAAMAAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIABBACAAaQBzACAAbABhAHIAZwBlAHIAOgAgAHMAaQBnAG4AIABiAGUAbABvAG4AZwBzACAAdABvACAAQQAuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABWAFMAVABBAEMASwAoAFUAUwB1AGIAKABsAGkAbQBiAHMAXwBhACwAIABsAGkAbQBiAHMAXwBiACwAIABrACkALAAgAHMAaQBnAG4AXwBhACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAEIAIABpAHMAIABsAGEAcgBnAGUAcgA6ACAAcgBvAHUAdABlACAAQgAgAGYAaQByAHMAdAAsACAAcwBpAGcAbgAgAGIAZQBsAG8AbgBnAHMAIAB0AG8AIABCAC4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFYAUwBUAEEAQwBLACgAVQBTAHUAYgAoAGwAaQBtAGIAcwBfAGIALAAgAGwAaQBtAGIAcwBfAGEALAAgAGsAKQAsACAAcwBpAGcAbgBfAGIAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFsASQBuAHQAZQByAG4AYQBsAF0AIABVAG4AcwBpAGcAbgBlAGQAIABtAHUAbAB0AGkAcABsAGkAYwBhAHQAaQBvAG4AIABvAGYAIAB0AHcAbwAgAEwAaQB0AHQAbABlAC0ARQBuAGQAaQBhAG4AIABsAGkAbQBiACAAYQByAHIAYQB5AHMALgBcAG4AIAAqACAAVQB0AGkAbABpAHoAZQBzACAAYQAgADEARAAgAEQAaQBzAGMAcgBlAHQAZQAgAEMAbwBuAHYAbwBsAHUAdABpAG8AbgAgACgAQwBhAHUAYwBoAHkAIABQAHIAbwBkAHUAYwB0ACkAIABhAHIAcgBhAHkALQBzAGwAaQBjAGkAbgBnACAAcwB0AHIAYQB0AGUAZwB5AC4AXABuACAAKgAgAFoAZQByAG8AIABkAHkAbgBhAG0AaQBjACAAbQBlAG0AbwByAHkAIAByAGUAYQBsAGwAbwBjAGEAdABpAG8AbgAuACAAJABPACgATgArAE0AKQAkACAAbQBlAG0AbwByAHkAIABmAG8AbwB0AHAAcgBpAG4AdAAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGwAaQBtAGIAcwBfAGEAIABUAGgAZQAgAG0AdQBsAHQAaQBwAGwAaQBjAGEAbgBkACAAbABpAG0AYgAgAGEAcgByAGEAeQAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGwAaQBtAGIAcwBfAGIAIABUAGgAZQAgAG0AdQBsAHQAaQBwAGwAaQBlAHIAIABsAGkAbQBiACAAYQByAHIAYQB5AC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAawAgAFQAaABlACAAZAB5AG4AYQBtAGkAYwAgAGMAaAB1AG4AawAgAHMAaQB6AGUAIABjAG8AbgB0AGUAeAB0AC4AXABuACAAKgAvAFwAbgBVAE0AdQBsACAAPQAgAEwAQQBNAEIARABBACgAbABpAG0AYgBzAF8AYQAsACAAbABpAG0AYgBzAF8AYgAsACAAawAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABsAGUAbgBfAGEALAAgAFIATwBXAFMAKABsAGkAbQBiAHMAXwBhACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAZQBuAF8AYgAsACAAUgBPAFcAUwAoAGwAaQBtAGIAcwBfAGIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHgAXwByAG8AdwBzACwAIABsAGUAbgBfAGEAIAArACAAbABlAG4AXwBiACAALQAgADEALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAALwAvACAATABvAG8AcAAgAHAAdQByAGUAbAB5ACAAbwB2AGUAcgAgAHQAaABlACAAbABlAG4AZwB0AGgAIABvAGYAIAB0AGgAZQAgAGYAaQBuAGEAbAAgAG8AdQB0AHAAdQB0ACAAYQByAHIAYQB5AFwAbgAgACAAIAAgACAAIAAgACAAcgBhAHcAXwBsAGkAbQBiAHMALAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAbQBhAHgAXwByAG8AdwBzACwAIAAxACwAIABMAEEATQBCAEQAQQAoAHIALAAgAGMALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIABDAGEAbABjAHUAbABhAHQAZQAgAHQAaABlACAAdgBhAGwAaQBkACAAbwB2AGUAcgBsAGEAcABwAGkAbgBnACAAdwBpAG4AZABvAHcAIABvAGYAIABpAG4AZABpAGMAZQBzACAAZgBvAHIAIAB0AGgAaQBzACAAbQBhAGcAbgBpAHQAdQBkAGUAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcwB0AGEAcgB0AF8AaQAsACAATQBBAFgAKAAxACwAIAByACAALQAgAGwAZQBuAF8AYgAgACsAIAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABlAG4AZABfAGkALAAgAE0ASQBOACgAcgAsACAAbABlAG4AXwBhACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABjAG8AdQBuAHQALAAgAGUAbgBkAF8AaQAgAC0AIABzAHQAYQByAHQAXwBpACAAKwAgADEALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIABTAGUAcQB1AGUAbgBjAGUAIABpACAAYwBvAHUAbgB0AHMAIABVAFAALgAgAFMAZQBxAHUAZQBuAGMAZQAgAGoAIABjAG8AdQBuAHQAcwAgAEQATwBXAE4ALgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABzAGUAcQBfAGkALAAgAFMARQBRAFUARQBOAEMARQAoAGMAbwB1AG4AdAAsACAAMQAsACAAcwB0AGEAcgB0AF8AaQAsACAAMQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcwBlAHEAXwBqACwAIABTAEUAUQBVAEUATgBDAEUAKABjAG8AdQBuAHQALAAgADEALAAgAHIAIAAtACAAcwB0AGEAcgB0AF8AaQAgACsAIAAxACwAIAAtADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAFMAbABpAGMAZQAgAHQAaABlACAAZQB4AGEAYwB0ACAAaQBuAHQAZQByAHMAZQBjAHQAaQBuAGcAIABsAGkAbQBiAHMALAAgAG0AdQBsAHQAaQBwAGwAeQAsACAAYQBuAGQAIABzAHUAbQAgAG4AYQB0AGkAdgBlAGwAeQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABTAFUATQAoAEkATgBEAEUAWAAoAGwAaQBtAGIAcwBfAGEALAAgAHMAZQBxAF8AaQAsACAAMQApACAAKgAgAEkATgBEAEUAWAAoAGwAaQBtAGIAcwBfAGIALAAgAHMAZQBxAF8AagAsACAAMQApACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAApACkALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAALwAvACAAUgBlAHMAbwBsAHYAZQAgAGEAbABsACAAYwBhAHIAcgBpAGUAcwAgAGIAbwB0AHQAbwBtAC0AdABvAC0AdABvAHAAIABlAHgAYQBjAHQAbAB5ACAAbwBuAGMAZQBcAG4AIAAgACAAIAAgACAAIAAgAEMAYQByAHIAeQAoAHIAYQB3AF8AbABpAG0AYgBzACwAIABrACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuAKAAKgAgAFsASQBuAHQAZQByAG4AYQBsAF0AIABCAGkAbgBhAHIAeQAgAHMAZQBhAHIAYwBoACAAdABvACAAZgBpAG4AZAAgAHQAaABlACAAaABpAGcAaABlAHMAdAAgAHMAYwBhAGwAYQByACAAcQB1AG8AdABpAGUAbgB0ACAAbABpAG0AYgAgAHEAIAAoADAAIAA8AD0AIABxACAAPAAgADEAMABeAGsAKQBcAG4AoAAqACAAcwB1AGMAaAAgAHQAaABhAHQAIABCACAAKgAgAHEAIAA8AD0AIABhAGMAYwAuACAARQBsAGkAbQBpAG4AYQB0AGUAcwAgAHQAaABlACAAbgBlAGUAZAAgAGYAbwByACAASwBuAHUAdABoACAARAAgAGYAbABvAGEAdAAtAGUAcwB0AGkAbQBhAHQAaQBvAG4ALgBcAG4AoAAqACAAQABwAGEAcgBhAG0AIABhAGMAYwAgAFQAaABlACAAYwB1AHIAcgBlAG4AdAAgAHIAZQBtAGEAaQBuAGQAZQByACAAYQByAHIAYQB5AC4AXABuAKAAKgAgAEAAcABhAHIAYQBtACAAYgAgAFQAaABlACAAZABpAHYAaQBzAG8AcgAgAGEAcgByAGEAeQAuAFwAbgCgACoAIABAAHAAYQByAGEAbQAgAGsAIABUAGgAZQAgAGQAeQBuAGEAbQBpAGMAIABjAGgAdQBuAGsAIABzAGkAegBlACAAYwBvAG4AdABlAHgAdAAuAFwAbgCgACoALwBcAG4ARgBpAG4AZABRAHUAbwB0AGkAZQBuAHQATABpAG0AYgAgAD0AIABMAEEATQBCAEQAQQAoAGEAYwBjACwAIABiACwAIABrACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAC8ALwAgAEMAYQBsAGMAdQBsAGEAdABlACAAcgBlAHEAdQBpAHIAZQBkACAAYgBpAHQAcwAgAGQAeQBuAGEAbQBpAGMAYQBsAGwAeQAuACAARgBvAHIAIABtAGEAeAAgAGsAPQA3ACwAIAB0AGgAaQBzACAAZQB2AGEAbAB1AGEAdABlAHMAIAB0AG8AIAAyADQAIABiAGkAdABzAC4AXABuACAAIAAgACAAIAAgACAAIABiAGkAdABzACwAIABDAEUASQBMAEkATgBHAC4ATQBBAFQASAAoAEwATwBHACgAMQAwAF4AawAsACAAMgApACkALABcAG4AIAAgACAAIAAgACAAIAAgAHAAbwB3AGUAcgBzACwAIAAyACAAXgAgAFMARQBRAFUARQBOAEMARQAoAGIAaQB0AHMALAAgADEALAAgAGIAaQB0AHMAIAAtACAAMQAsACAALQAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAUgBFAEQAVQBDAEUAKAAwACwAIABwAG8AdwBlAHIAcwAsACAATABBAE0AQgBEAEEAKABjAHUAcgByAF8AcQAsACAAcABvAHcAZQByACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAdABlAHMAdABfAHEALAAgAGMAdQByAHIAXwBxACAAKwAgAHAAbwB3AGUAcgAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAFMAawBpAHAAIABpAGYAIAB0AGUAcwB0AF8AcQAgAGUAeABjAGUAZQBkAHMAIAB0AGgAZQAgAGwAaQBtAGIAIABiAGEAcwBlAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEkARgAoAHQAZQBzAHQAXwBxACAAPgA9ACAAMQAwAF4AawAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABjAHUAcgByAF8AcQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAATQB1AGwAdABpAHAAbAB5ACAAQgAgAGIAeQAgAHMAYwBhAGwAYQByACAAdABlAHMAdABfAHEAIABhAG4AZAAgAHIAZQBzAG8AbAB2AGUAIABjAGEAcgByAGkAZQBzACAAbgBhAHQAaQB2AGUAbAB5AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAB0AGUAcwB0AF8AcAByAG8AZAAsACAAQwBhAHIAcgB5ACgAYgAgACoAIAB0AGUAcwB0AF8AcQAsACAAawApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGMAbwBtAHAALAAgAFUAQwBvAG0AcABhAHIAZQAoAGEAYwBjACwAIAB0AGUAcwB0AF8AcAByAG8AZAApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABjAG8AbQBwACAAPgA9ACAAMAAsACAAdABlAHMAdABfAHEALAAgAGMAdQByAHIAXwBxACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAApACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuAKAAKgAgAFsASQBuAHQAZQByAG4AYQBsAF0AIABCAGEAcwBlAGMAYQBzAGUAIABEAGkAdgBpAHMAaQBvAG4AIAB2AGkAYQAgAHMAZQBxAHUAZQBuAHQAaQBhAGwAIABzAGgAaQBmAHQALQBhAG4AZAAtAHMAdQBiAHQAcgBhAGMAdAAuAFwAbgCgACoAIABSAGUAdAB1AHIAbgBzACAAYQAgAHAAYQBjAGsAZQBkACAAMQBEACAAYQByAHIAYQB5ADoAIABWAFMAVABBAEMASwAoAEwAZQBuAGcAdABoAF8AUgAsACAAUgBfAGwAaQBtAGIAcwAsACAAUQBfAGwAaQBtAGIAcwApAC4AXABuAKAAKgAgAEUAbABpAG0AaQBuAGEAdABlAHMAIAAyAEQAIABhAHIAcgBhAHkAIABwAGEAZABkAGkAbgBnACAAdABvACAAcwB0AHIAaQBjAHQAbAB5ACAAcAByAGUAcwBlAHIAdgBlACAAbQBlAG0AbwByAHkAIABlAGYAZgBpAGMAaQBlAG4AYwB5AC4AXABuAKAAKgAgAEAAcABhAHIAYQBtACAAbABpAG0AYgBzAF8AYQAgAFQAaABlACAAZABpAHYAaQBkAGUAbgBkACAAYQByAHIAYQB5AC4AXABuAKAAKgAgAEAAcABhAHIAYQBtACAAbABpAG0AYgBzAF8AYgAgAFQAaABlACAAZABpAHYAaQBzAG8AcgAgAGEAcgByAGEAeQAgACgAYQBzAHMAdQBtAGUAZAAgAG4AbwBuAC0AegBlAHIAbwApAC4AXABuAKAAKgAgAEAAcABhAHIAYQBtACAAawAgAFQAaABlACAAZAB5AG4AYQBtAGkAYwAgAGMAaAB1AG4AawAgAHMAaQB6AGUAIABjAG8AbgB0AGUAeAB0AC4AXABuAKAAKgAvAFwAbgBLAG4AdQB0AGgARABpAHYAIAA9ACAATABBAE0AQgBEAEEAKABsAGkAbQBiAHMAXwBhACwAIABsAGkAbQBiAHMAXwBiACwAIABrACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQBnAF8AYwBvAG0AcAAsACAAVQBDAG8AbQBwAGEAcgBlACgAbABpAG0AYgBzAF8AYQAsACAAbABpAG0AYgBzAF8AYgApACwAXABuACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgAC8ALwAgAFMAaABvAHIAdAAtAGMAaQByAGMAdQBpAHQAIAByAG8AdQB0AGkAbgBnACAAdwBpAHQAaAAgAHQAaABlACAAbgBlAHcAIABwAGEAYwBrAGUAZAAgAG0AZQBtAG8AcgB5ACAAYwBvAG4AdAByAGEAYwB0AFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAbQBhAGcAXwBjAG8AbQBwACAAPAAgADAALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAVgBTAFQAQQBDAEsAKABSAE8AVwBTACgAbABpAG0AYgBzAF8AYQApACwAIABsAGkAbQBiAHMAXwBhACwAIAAwACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgAbQBhAGcAXwBjAG8AbQBwACAAPQAgADAALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABWAFMAVABBAEMASwAoADEALAAgADAALAAgADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGUAbgBfAGEALAAgAFIATwBXAFMAKABsAGkAbQBiAHMAXwBhACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAEkAdABlAHIAYQB0AGUAIABvAHYAZQByACAAQQAgAGYAcgBvAG0AIABNAFMAQgAgACgAdABvAHAAKQAgAHQAbwAgAEwAUwBCACAAKABiAG8AdAB0AG8AbQApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcgBlAHYAZQByAHMAZQBkAF8AYQAsACAAQwBIAE8ATwBTAEUAUgBPAFcAUwAoAGwAaQBtAGIAcwBfAGEALAAgAFMARQBRAFUARQBOAEMARQAoAGwAZQBuAF8AYQAsACAAMQAsACAAbABlAG4AXwBhACwAIAAtADEAKQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAFMAdABhAHQAZQAgAHMAZQBwAGEAcgBhAHQAbwByADoAIABWAFMAVABBAEMASwAoAGwAZQBuAF8AcgBlAG0AYQBpAG4AZABlAHIALAAgAHIAZQBtAGEAaQBuAGQAZQByACwAIABxAHUAbwB0AGkAZQBuAHQAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGkAbgBpAHQAaQBhAGwAXwBzAHQAYQB0AGUALAAgAFYAUwBUAEEAQwBLACgAMQAsACAAMAAsACAAMAApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGYAaQBuAGEAbABfAHMAdABhAHQAZQAsACAAUgBFAEQAVQBDAEUAKABpAG4AaQB0AGkAYQBsAF8AcwB0AGEAdABlACwAIAByAGUAdgBlAHIAcwBlAGQAXwBhACwAIABMAEEATQBCAEQAQQAoAHMAdABhAHQAZQAsACAAdgBhAGwALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGUAbgBfAHIAZQBtAGEAaQBuAGQAZQByACwAIABJAE4ARABFAFgAKABzAHQAYQB0AGUALAAgADEALAAgADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHIAZQBtAGEAaQBuAGQAZQByACwAIABDAEgATwBPAFMARQBSAE8AVwBTACgAcwB0AGEAdABlACwAIABTAEUAUQBVAEUATgBDAEUAKABsAGUAbgBfAHIAZQBtAGEAaQBuAGQAZQByACwAIAAxACwAIAAyACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHEAdQBvAHQAaQBlAG4AdAAsACAARABSAE8AUAAoAHMAdABhAHQAZQAsACAAbABlAG4AXwByAGUAbQBhAGkAbgBkAGUAcgAgACsAIAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIABTAGgAaQBmAHQAIABhAGMAYwAgAHUAcAAgAGIAeQAgADEAIABsAGkAbQBiACAAKABMAGkAdAB0AGwAZQAtAEUAbgBkAGkAYQBuADoAIABpAG4AcwBlAHIAdAAgAGEAdAAgAGkAbgBkAGUAeAAgADEAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABlAHgAdABlAG4AZABlAGQAXwByAGUAbQBhAGkAbgBkAGUAcgAsACAASQBGACgAQQBOAEQAKABSAE8AVwBTACgAcgBlAG0AYQBpAG4AZABlAHIAKQAgAD0AIAAxACwAIABJAE4ARABFAFgAKAByAGUAbQBhAGkAbgBkAGUAcgAsACAAMQAsACAAMQApACAAPQAgADAAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAB2AGEAbAAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABWAFMAVABBAEMASwAoAHYAYQBsACwAIAByAGUAbQBhAGkAbgBkAGUAcgApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABuAGUAeAB0AF8AcQB1AG8AdABpAGUAbgB0AF8AbABpAG0AYgAsACAARgBpAG4AZABRAHUAbwB0AGkAZQBuAHQATABpAG0AYgAoAGUAeAB0AGUAbgBkAGUAZABfAHIAZQBtAGEAaQBuAGQAZQByACwAIABsAGkAbQBiAHMAXwBiACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABwAHIAbwBkACwAIABDAGEAcgByAHkAKABsAGkAbQBiAHMAXwBiACAAKgAgAG4AZQB4AHQAXwBxAHUAbwB0AGkAZQBuAHQAXwBsAGkAbQBiACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABuAGUAdwBfAHIAZQBtAGEAaQBuAGQAZQByACwAIABVAFMAdQBiACgAZQB4AHQAZQBuAGQAZQBkAF8AcgBlAG0AYQBpAG4AZABlAHIALAAgAHAAcgBvAGQALAAgAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGgAYQBzAF8AcQB1AG8AdABpAGUAbgB0ACwAIABPAFIAKABSAE8AVwBTACgAcQB1AG8AdABpAGUAbgB0ACkAIAA+ACAAMQAsACAASQBOAEQARQBYACgAcQB1AG8AdABpAGUAbgB0ACwAMQAsADEAKQAgAD4AIAAwACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABuAGUAeAB0AF8AcQB1AG8AdAAsACAASQBGACgAaABhAHMAXwBxAHUAbwB0AGkAZQBuAHQALAAgAFYAUwBUAEEAQwBLACgAcQB1AG8AdABpAGUAbgB0ACwAIABuAGUAeAB0AF8AcQB1AG8AdABpAGUAbgB0AF8AbABpAG0AYgApACwAIABuAGUAeAB0AF8AcQB1AG8AdABpAGUAbgB0AF8AbABpAG0AYgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAVgBTAFQAQQBDAEsAKABSAE8AVwBTACgAbgBlAHcAXwByAGUAbQBhAGkAbgBkAGUAcgApACwAIABuAGUAdwBfAHIAZQBtAGEAaQBuAGQAZQByACwAIABuAGUAeAB0AF8AcQB1AG8AdAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAZQBuAF8AcgBlAG0AYQBpAG4AZABlAHIALAAgAEkATgBEAEUAWAAoAGYAaQBuAGEAbABfAHMAdABhAHQAZQAsACAAMQAsACAAMQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAByAGUAbQBhAGkAbgBkAGUAcgAsACAAQwBIAE8ATwBTAEUAUgBPAFcAUwAoAGYAaQBuAGEAbABfAHMAdABhAHQAZQAsACAAUwBFAFEAVQBFAE4AQwBFACgAbABlAG4AXwByAGUAbQBhAGkAbgBkAGUAcgAsACAAMQAsACAAMgApACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHIAZQB2AGUAcgBzAGUAZABfAHEAdQBvAHQAaQBlAG4AdAAsACAARABSAE8AUAAoAGYAaQBuAGEAbABfAHMAdABhAHQAZQAsACAAbABlAG4AXwByAGUAbQBhAGkAbgBkAGUAcgAgACsAIAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAAcQB1AG8AdABfAHIAYQB3ACAAdwBhAHMAIABiAHUAaQBsAHQAIABNAFMAQgAgAHQAbwAgAEwAUwBCACAAKABCAGkAZwAtAEUAbgBkAGkAYQBuACkALgAgAFIAZQB2AGUAcgBzAGUAIAB0AG8AIABpAG4AdABlAHIAbgBhAGwAIABMAGkAdAB0AGwAZQAtAEUAbgBkAGkAYQBuAC4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGUAbgBfAHEAdQBvAHQAaQBlAG4AdAAsACAAUgBPAFcAUwAoAHIAZQB2AGUAcgBzAGUAZABfAHEAdQBvAHQAaQBlAG4AdAApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABxAHUAbwB0AGkAZQBuAHQALAAgAEMASABPAE8AUwBFAFIATwBXAFMAKAByAGUAdgBlAHIAcwBlAGQAXwBxAHUAbwB0AGkAZQBuAHQALAAgAFMARQBRAFUARQBOAEMARQAoAGwAZQBuAF8AcQB1AG8AdABpAGUAbgB0ACwAIAAxACwAIABsAGUAbgBfAHEAdQBvAHQAaQBlAG4AdAAsACAALQAxACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIABSAGUAdAB1AHIAbgAgAHMAdAByAGkAYwB0AGwAeQAgAHAAYQBjAGsAZQBkACAAMQBEACAAYQByAHIAYQB5AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAVgBTAFQAQQBDAEsAKABsAGUAbgBfAHIAZQBtAGEAaQBuAGQAZQByACwAIAByAGUAbQBhAGkAbgBkAGUAcgAsACAAcQB1AG8AdABpAGUAbgB0ACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuAKAAKgAgAFsASQBuAHQAZQByAG4AYQBsAF0AIABIAHkAYgByAGkAZAAgAEQAaQB2AGkAcwBpAG8AbgAgAFIAbwB1AHQAZQByAC4AXABuAKAAKgAgAEQAaQByAGUAYwB0AHMAIABkAGkAdgBpAHMAaQBvAG4AIAB0AG8AIAB0AGgAZQAgAG8AcAB0AGkAbQBhAGwAIABrAGUAcgBuAGUAbAAgAGIAYQBzAGUAZAAgAG8AbgAgAEQAaQB2AGkAZABlAG4AZAAgAGwAZQBuAGcAdABoAC4AXABuAKAAKgAgAEAAcABhAHIAYQBtACAAbABpAG0AYgBzAF8AYQAgAFQAaABlACAAZABpAHYAaQBkAGUAbgBkACAAYQByAHIAYQB5AC4AXABuAKAAKgAgAEAAcABhAHIAYQBtACAAbABpAG0AYgBzAF8AYgAgAFQAaABlACAAZABpAHYAaQBzAG8AcgAgAGEAcgByAGEAeQAuAFwAbgCgACoAIABAAHAAYQByAGEAbQAgAGsAIABUAGgAZQAgAGQAeQBuAGEAbQBpAGMAIABjAGgAdQBuAGsAIABzAGkAegBlACAAYwBvAG4AdABlAHgAdAAuAFwAbgCgACoALwBcAG4ARABpAHYAUgBvAHUAdABlAHIAIAA9ACAATABBAE0AQgBEAEEAKABsAGkAbQBiAHMAXwBhACwAIABsAGkAbQBiAHMAXwBiACwAIABrACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAC8ALwAgAEQAaQBnAGkAdAAgAGMAbwB1AG4AdABzACAAYQByAGUAIABhAHAAcAByAG8AeABpAG0AYQB0AGUALAAgAGIAdQB0ACAAcwB1AGYAZgBpAGMAaQBlAG4AdABcAG4AIAAgACAAIAAgACAAIAAgAGQAaQBnAGkAdABzAF8AYQAsACAAUgBPAFcAUwAoAGwAaQBtAGIAcwBfAGEAKQAgACoAIABrACwAXABuACAAIAAgACAAIAAgACAAIABkAGkAZwBpAHQAcwBfAGIALAAgAFIATwBXAFMAKABsAGkAbQBiAHMAXwBiACkAIAAqACAAawAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABNAGEAYwBoAGkAbgBlAC0AbABlAGEAcgBuAGUAZAAgAGMAbwBlAGYAZgBpAGMAaQBlAG4AdABzACAAZgByAG8AbQAgAEwAbwBnAGkAcwB0AGkAYwAgAFIAZQBnAHIAZQBzAHMAaQBvAG4AXABuACAAIAAgACAAIAAgACAAIABtACwAIAAwAC4AMQAwADcAOAAyADEAMQA5ADQAMgA3ADEAMgA5ADcALABcAG4AIAAgACAAIAAgACAAIAAgAGMALAAgAC0AMgAyADEALgA5ADAAMgAxADgAOQA0ADYAMgAwADYAOAAsAFwAbgAgACAAIAAgACAAIAAgACAAdABoAHIAZQBzAGgAbwBsAGQALAAgACgAbQAgACoAIABkAGkAZwBpAHQAcwBfAGEAKQAgACsAIABjACwAXABuACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAGQAaQBnAGkAdABzAF8AYgAgADwAPQAgAHQAaAByAGUAcwBoAG8AbABkACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEsAbgB1AHQAaABEAGkAdgAoAGwAaQBtAGIAcwBfAGEALAAgAGwAaQBtAGIAcwBfAGIALAAgAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABOAGUAdwB0AG8AbgBSAGEAcABoAHMAbwBuAEQAaQB2ACgAbABpAG0AYgBzAF8AYQAsACAAbABpAG0AYgBzAF8AYgAsACAAawApAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAAWwBJAG4AdABlAHIAbgBhAGwAXQAgAEcAZQBuAGUAcgBhAHQAZQBzACAAdABoAGUAIABlAHgAYQBjAHQAIAByAGUAYwBpAHAAcgBvAGMAYQBsACAAcwBlAGUAZAAgAGYAbwByACAATgBlAHcAdABvAG4ALQBSAGEAcABoAHMAbwBuACAARABpAHYAaQBzAGkAbwBuACAAdQBzAGkAbgBnACAASwBuAHUAdABoACAAQgBhAHMAZQBjAGEAcwBlAC4AXABuACAAKgAgAEUAeAB0AHIAYQBjAHQAcwAgAHUAcAAgAHQAbwAgAHQAaABlACAAdABvAHAAIAAzACAAbABpAG0AYgBzACAAbwBmACAAQgAgAGEAbgBkACAAYwBhAGwAYwB1AGwAYQB0AGUAcwAgAGYAbABvAG8AcgAoAEIAZQB0AGEAXgAoADIAKgBsAGUAbgApACAALwAgAEIAXwB0AG8AcAApAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAbABpAG0AYgBzAF8AYgAgAFQAaABlACAAZABpAHYAaQBzAG8AcgAgAGwAaQBtAGIAIABhAHIAcgBhAHkALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABrACAAVABoAGUAIABkAHkAbgBhAG0AaQBjACAAYwBoAHUAbgBrACAAcwBpAHoAZQAgAGMAbwBuAHQAZQB4AHQALgBcAG4AIAAqAC8AXABuAE4AZQB3AHQAbwBuAFIAYQBwAGgAcwBvAG4AUwBlAGUAZAAgAD0AIABMAEEATQBCAEQAQQAoAGwAaQBtAGIAcwBfAGIALAAgAGsALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbABlAG4AXwBiACwAIABSAE8AVwBTACgAbABpAG0AYgBzAF8AYgApACwAXABuACAAIAAgACAAIAAgACAAIABzAGUAZQBkAF8AbABlAG4ALAAgAE0ASQBOACgAMwAsACAAbABlAG4AXwBiACkALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAALwAvACAARQB4AHQAcgBhAGMAdAAgAHQAbwBwACAAJwBzAGUAZQBkAF8AbABlAG4AJwAgAGwAaQBtAGIAcwAgACgATABpAHQAdABsAGUALQBFAG4AZABpAGEAbgA6ACAAdABhAGsAZQAgAGYAcgBvAG0AIAB0AGgAZQAgAGIAbwB0AHQAbwBtACkAXABuACAAIAAgACAAIAAgACAAIABiAF8AdABvAHAALAAgAFQAQQBLAEUAKABsAGkAbQBiAHMAXwBiACwAIAAtAHMAZQBlAGQAXwBsAGUAbgApACwAXABuACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgAC8ALwAgAEMAbwBuAHMAdAByAHUAYwB0ACAAQgBlAHQAYQBeACgAMgAgACoAIABzAGUAZQBkAF8AbABlAG4AKQAgAG4AYQB0AGkAdgBlAGwAeQBcAG4AIAAgACAAIAAgACAAIAAgAC8ALwAgAGUALgBnAC4ALAAgAGkAZgAgAHMAZQBlAGQAXwBsAGUAbgAgAD0AIAAxACwAIAB0AGgAZQBuACAAMQAgAGYAbwBsAGwAbwB3AGUAZAAgAGIAeQAgAHQAdwBvACAAegBlAHIAbwAgAGwAaQBtAGIAcwA6ACAAVgBTAFQAQQBDAEsAKAAwACwAIAAwACwAIAAxACkAXABuACAAIAAgACAAIAAgACAAIABiAGUAdABhAF8AMgBtACwAIABWAFMAVABBAEMASwAoAEUAWABQAEEATgBEACgAMAAsACAAMgAgACoAIABzAGUAZQBkAF8AbABlAG4ALAAgACwAIAAwACkALAAgADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABLAG4AdQB0AGgAIABEAGkAdgBpAHMAaQBvAG4AIAB5AGkAZQBsAGQAcwAgAGUAeABhAGMAdAAgAGkAbgBpAHQAaQBhAGwAIAByAGUAYwBpAHAAcgBvAGMAYQBsAFwAbgAgACAAIAAgACAAIAAgACAAcABhAGMAawBlAGQALAAgAEsAbgB1AHQAaABEAGkAdgAoAGIAZQB0AGEAXwAyAG0ALAAgAGIAXwB0AG8AcAAsACAAawApACwAXABuACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgAC8ALwAgAEUAeAB0AHIAYQBjAHQAIABRAHUAbwB0AGkAZQBuAHQAIABhAHIAcgBhAHkAIABmAHIAbwBtACAAdABoAGUAIABwAGEAYwBrAGUAZAAgAFYAUwBUAEEAQwBLAFwAbgAgACAAIAAgACAAIAAgACAAbABlAG4AXwByACwAIABJAE4ARABFAFgAKABwAGEAYwBrAGUAZAAsACAAMQAsACAAMQApACwAXABuACAAIAAgACAAIAAgACAAIABEAFIATwBQACgAcABhAGMAawBlAGQALAAgAGwAZQBuAF8AcgAgACsAIAAxACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFsASQBuAHQAZQByAG4AYQBsAF0AIABDAG8AbQBwAHUAdABlAHMAIAB0AGgAZQAgAFIAZQBjAGkAcAByAG8AYwBhAGwAIABwAHIAbwBnAHIAZQBzAHMAaQB2AGUAbAB5ACAAcwBjAGEAbABpAG4AZwAgAHUAcAAgAHQAbwAgAHQAaABlACAARABpAHYAaQBkAGUAbgBkACcAcwAgAHAAcgBlAGMAaQBzAGkAbwBuAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAbABpAG0AYgBzAF8AYgAgAFQAaABlACAAZABpAHYAaQBzAG8AcgAgAGwAaQBtAGIAIABhAHIAcgBhAHkALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIAB0AGEAcgBnAGUAdABfAGwAZQBuACAAVABoAGUAIABsAGkAbQBiAC0AbABlAG4AZwB0AGgAIABvAGYAIABEAGkAdgBpAGQAZQBuAGQAIABBAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAawAgAFQAaABlACAAZAB5AG4AYQBtAGkAYwAgAGMAaAB1AG4AawAgAHMAaQB6AGUAIABjAG8AbgB0AGUAeAB0AC4AXABuACAAKgAvAFwAbgBOAGUAdwB0AG8AbgBSAGEAcABoAHMAbwBuAFIAZQBjAGkAcAByAG8AYwBhAGwAIAA9ACAATABBAE0AQgBEAEEAKABsAGkAbQBiAHMAXwBiACwAIAB0AGEAcgBnAGUAdABfAGwAZQBuACwAIABrACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAGwAZQBuAF8AYgAsACAAUgBPAFcAUwAoAGwAaQBtAGIAcwBfAGIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwBlAGUAZABfAGwAZQBuACwAIABNAEkATgAoADMALAAgAGwAZQBuAF8AYgApACwAXABuACAAIAAgACAAIAAgACAAIAByAF8AcwBlAGUAZABfAGwAaQBtAGIAcwAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4ATgBlAHcAdABvAG4AUgBhAHAAaABzAG8AbgBTAGUAZQBkACgAbABpAG0AYgBzAF8AYgAsACAAawApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAaQBuAGkAdABpAGEAbABfAHMAdABhAHQAZQAsACAAVgBTAFQAQQBDAEsAKABzAGUAZQBkAF8AbABlAG4ALAAgAHIAXwBzAGUAZQBkAF8AbABpAG0AYgBzACkALABcAG4AIAAgACAAIAAgACAAIAAgAHIAZQBxAF8AaQB0AGUAcgBzACwAIABNAEEAWAAoADAALAAgAEMARQBJAEwASQBOAEcALgBNAEEAVABIACgATABOACgAdABhAHIAZwBlAHQAXwBsAGUAbgAgAC8AIABzAGUAZQBkAF8AbABlAG4AKQAgAC8AIABMAE4AKAAyACkAKQApACAAKwAgADEALABcAG4AXABuACAAIAAgACAAIAAgACAAIABJAEYAKAByAGUAcQBfAGkAdABlAHIAcwAgAD0AIAAwACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHIAXwBzAGUAZQBkAF8AbABpAG0AYgBzACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAaQB0AGUAcgBhAHQAaQBvAG4AcwAsACAAUwBFAFEAVQBFAE4AQwBFACgAcgBlAHEAXwBpAHQAZQByAHMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGYAaQBuAGEAbABfAHMAdABhAHQAZQAsACAAUgBFAEQAVQBDAEUAKABpAG4AaQB0AGkAYQBsAF8AcwB0AGEAdABlACwAIABpAHQAZQByAGEAdABpAG8AbgBzACwAIABMAEEATQBCAEQAQQAoAHMAdABhAHQAZQAsACAAaQB0AGUAcgAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAYwB1AHIAcgBfAGwAZQBuACwAIABJAE4ARABFAFgAKABzAHQAYQB0AGUALAAgADEALAAgADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABjAHUAcgByAF8AcgAsACAARABSAE8AUAAoAHMAdABhAHQAZQAsACAAMQApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABuAGUAeAB0AF8AbABlAG4ALAAgAE0ASQBOACgAYwB1AHIAcgBfAGwAZQBuACAAKgAgADIALAAgAHQAYQByAGcAZQB0AF8AbABlAG4AKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAARAB5AG4AYQBtAGkAYwAgAFMAYwBhAGwAaQBuAGcAIABTAGgAaQBmAHQAOgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAASQBmACAAQgAgAGgAYQBzACAAcABsAGEAdABlAGEAdQBlAGQALAAgAFIAIABtAHUAcwB0ACAAcwBjAGEAbABlACAAYgB5ACAAMgAqACgAbgAtAG0AKQAuACAASQBmACAAQgAgAGkAcwAgAGcAcgBvAHcAaQBuAGcALAAgAFIAIABzAGMAYQBsAGUAcwAgAGIAeQAgACgAbgAtAG0AKQAuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABhAGMAdABpAHYAZQBfAGMAdQByAHIALAAgAE0ASQBOACgAYwB1AHIAcgBfAGwAZQBuACwAIABsAGUAbgBfAGIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABhAGMAdABpAHYAZQBfAG4AZQB4AHQALAAgAE0ASQBOACgAbgBlAHgAdABfAGwAZQBuACwAIABsAGUAbgBfAGIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABzAGgAaQBmAHQAXwBsAGkAbQBiAHMALAAgADIAIAAqACAAKABuAGUAeAB0AF8AbABlAG4AIAAtACAAYwB1AHIAcgBfAGwAZQBuACkAIAAtACAAKABhAGMAdABpAHYAZQBfAG4AZQB4AHQAIAAtACAAYQBjAHQAaQB2AGUAXwBjAHUAcgByACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHIAXwBwAHIAaQBtAGUALAAgAEkARgAoAHMAaABpAGYAdABfAGwAaQBtAGIAcwAgAD4AIAAwACwAIABWAFMAVABBAEMASwAoAEUAWABQAEEATgBEACgAMAAsACAAcwBoAGkAZgB0AF8AbABpAG0AYgBzACwAIAAsACAAMAApACwAIABjAHUAcgByAF8AcgApACwAIABjAHUAcgByAF8AcgApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABiAF8AYQBjAHQAaQB2AGUALAAgAFQAQQBLAEUAKABsAGkAbQBiAHMAXwBiACwAIAAtAGEAYwB0AGkAdgBlAF8AbgBlAHgAdAApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIABQACAAaQBzACAAbgBhAHQAaQB2AGUAbAB5ACAAYQBsAGkAZwBuAGUAZAAgAHQAbwAgADIAKgBuAGUAeAB0AF8AbABlAG4AIABiAGUAYwBhAHUAcwBlACAAbwBmACAAdABoAGUAIABjAG8AcgByAGUAYwB0AGUAZAAgAHMAaABpAGYAdABfAGwAaQBtAGIAcwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBNAHUAbAAoAGIAXwBhAGMAdABpAHYAZQAsACAAcgBfAHAAcgBpAG0AZQAsACAAawApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAB0AHcAbwBfAGIAZQB0AGEALAAgAFYAUwBUAEEAQwBLACgARQBYAFAAQQBOAEQAKAAwACwAIAAyACAAKgAgAG4AZQB4AHQAXwBsAGUAbgAsACAALAAgADAAKQAsACAAMgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGUAcgByACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAFMAdQBiACgAdAB3AG8AXwBiAGUAdABhACwAIABwACwAIABrACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAG4AZQB4AHQAXwByAF8AdQBuAHMAYwBhAGwAZQBkACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAE0AdQBsACgAcgBfAHAAcgBpAG0AZQAsACAAZQByAHIALAAgAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABuAGUAeAB0AF8AcgAsACAASQBGACgAUgBPAFcAUwAoAG4AZQB4AHQAXwByAF8AdQBuAHMAYwBhAGwAZQBkACkAIAA8AD0AIAAyACAAKgAgAG4AZQB4AHQAXwBsAGUAbgAsACAAewAwAH0ALAAgAEQAUgBPAFAAKABuAGUAeAB0AF8AcgBfAHUAbgBzAGMAYQBsAGUAZAAsACAAMgAgACoAIABuAGUAeAB0AF8AbABlAG4AKQApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABWAFMAVABBAEMASwAoAG4AZQB4AHQAXwBsAGUAbgAsACAAbgBlAHgAdABfAHIAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAARABSAE8AUAAoAGYAaQBuAGEAbABfAHMAdABhAHQAZQAsACAAMQApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAAWwBJAG4AdABlAHIAbgBhAGwAXQAgAEgAZQBhAHYAeQB3AGUAaQBnAGgAdAAgAE4AZQB3AHQAbwBuAC0AUgBhAHAAaABzAG8AbgAgAEQAaQB2AGkAcwBpAG8AbgAuAFwAbgAgACoAIABJAG0AcABsAGUAbQBlAG4AdABzACAAcAByAG8AZwByAGUAcwBzAGkAdgBlACAAcwBjAGEAbABpAG4AZwAgAGIAbwB1AG4AZABlAGQAIAB0AG8AIABNAEEAWAAoAGwAZQBuAF8AYQAsACAAbABlAG4AXwBiACkALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABsAGkAbQBiAHMAXwBhACAAVABoAGUAIABkAGkAdgBpAGQAZQBuAGQAIABhAHIAcgBhAHkALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABsAGkAbQBiAHMAXwBiACAAVABoAGUAIABkAGkAdgBpAHMAbwByACAAYQByAHIAYQB5AC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAawAgAFQAaABlACAAZAB5AG4AYQBtAGkAYwAgAGMAaAB1AG4AawAgAHMAaQB6AGUAIABjAG8AbgB0AGUAeAB0AC4AXABuACAAKgAvAFwAbgBOAGUAdwB0AG8AbgBSAGEAcABoAHMAbwBuAEQAaQB2ACAAPQAgAEwAQQBNAEIARABBACgAbABpAG0AYgBzAF8AYQAsACAAbABpAG0AYgBzAF8AYgAsACAAawAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABsAGUAbgBfAGEALAAgAFIATwBXAFMAKABsAGkAbQBiAHMAXwBhACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAZQBuAF8AYgAsACAAUgBPAFcAUwAoAGwAaQBtAGIAcwBfAGIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAdABhAHIAZwBlAHQAXwBsAGUAbgAsACAATQBBAFgAKABsAGUAbgBfAGEALAAgAGwAZQBuAF8AYgApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAALwAvACAAMQAuACAAQwBhAGwAYwB1AGwAYQB0AGUAIAByAGUAYwBpAHAAcgBvAGMAYQBsACAAUgAgAHMAYwBhAGwAZQBkACAAZAB5AG4AYQBtAGkAYwBhAGwAbAB5ACAAdABvACAAMgAgACoAIAB0AGEAcgBnAGUAdABfAGwAZQBuAFwAbgAgACAAIAAgACAAIAAgACAAcgAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4ATgBlAHcAdABvAG4AUgBhAHAAaABzAG8AbgBSAGUAYwBpAHAAcgBvAGMAYQBsACgAbABpAG0AYgBzAF8AYgAsACAAdABhAHIAZwBlAHQAXwBsAGUAbgAsACAAawApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAALwAvACAAMgAuACAAQQBwAHAAcgBvAHgAaQBtAGEAdABlACAAUQB1AG8AdABpAGUAbgB0ADoAIABRAF8AYQBwAHAAcgBvAHgAIAA9ACAAQQAgACoAIABSACAALwAgAEIAZQB0AGEAXgAoADIAIAAqACAAdABhAHIAZwBlAHQAXwBsAGUAbgApAFwAbgAgACAAIAAgACAAIAAgACAAZAByAG8AcABfAGwAaQBtAGIAcwAsACAAMgAgACoAIAB0AGEAcgBnAGUAdABfAGwAZQBuACwAXABuACAAIAAgACAAIAAgACAAIABxAF8AdQBuAHMAYwBhAGwAZQBkACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAE0AdQBsACgAbABpAG0AYgBzAF8AYQAsACAAcgAsACAAawApACwAXABuACAAIAAgACAAIAAgACAAIABxAF8AYQBwAHAAcgBvAHgALAAgAEkARgAoAFIATwBXAFMAKABxAF8AdQBuAHMAYwBhAGwAZQBkACkAIAA8AD0AIABkAHIAbwBwAF8AbABpAG0AYgBzACwAIAB7ADAAfQAsACAARABSAE8AUAAoAHEAXwB1AG4AcwBjAGEAbABlAGQALAAgAGQAcgBvAHAAXwBsAGkAbQBiAHMAKQApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAALwAvACAAQwBhAGwAYwB1AGwAYQB0AGUAIAB0AGgAZQAgAG0AYQBzAHMAaQB2AGUAIABiAGEAcwBlAGwAaQBuAGUAIABwAHIAbwBkAHUAYwB0ACAAZQB4AGEAYwB0AGwAeQAgAE8ATgBDAEUAXABuACAAIAAgACAAIAAgACAAIABwAF8AYgBhAHMAZQBsAGkAbgBlACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAE0AdQBsACgAbABpAG0AYgBzAF8AYgAsACAAcQBfAGEAcABwAHIAbwB4ACwAIABrACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAvAC8AIAAzAC4AIABCAG8AdQBuAGQAZQBkACAARQByAHIAbwByACAAQwBvAHIAcgBlAGMAdABpAG8AbgAgAFMAdwBlAGUAcAAgACgATwBwAHQAaQBtAGkAegBlAGQAIABPACgATgApACAAUwB0AGUAcABwAGkAbgBnACkAXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABTAHQAYQB0AGUAIABwAGEAYwBrAGkAbgBnADoAIABWAFMAVABBAEMASwAoAEwAZQBuAGcAdABoAF8AUQAsACAAUQBfAGwAaQBtAGIAcwAsACAAUABfAGwAaQBtAGIAcwApAFwAbgAgACAAIAAgACAAIAAgACAAaQBuAGkAdABpAGEAbABfAHMAdABhAHQAZQAsACAAVgBTAFQAQQBDAEsAKABSAE8AVwBTACgAcQBfAGEAcABwAHIAbwB4ACkALAAgAHEAXwBhAHAAcAByAG8AeAAsACAAcABfAGIAYQBzAGUAbABpAG4AZQApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAALwAvACAAUwB3AGUAZQBwACAARABvAHcAbgA6ACAASQBmACAAUAAgAD4AIABBACwAIABRACAAaQBzACAAdABvAG8AIABiAGkAZwAuACAAUwB0AGUAcAAgAFEAIABkAG8AdwBuACAAYgB5ACAAMQAsACAAYQBuAGQAIABQACAAZABvAHcAbgAgAGIAeQAgAEIALgBcAG4AIAAgACAAIAAgACAAIAAgAHMAdwBlAGUAcABfAGQAbwB3AG4ALAAgAFIARQBEAFUAQwBFACgAaQBuAGkAdABpAGEAbABfAHMAdABhAHQAZQAsACAAewAxADsAIAAyAH0ALAAgAEwAQQBNAEIARABBACgAcwB0AGEAdABlACwAIABpACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABlAG4AXwBxACwAIABJAE4ARABFAFgAKABzAHQAYQB0AGUALAAgADEALAAgADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGMAdQByAHIAXwBxACwAIABDAEgATwBPAFMARQBSAE8AVwBTACgAcwB0AGEAdABlACwAIABTAEUAUQBVAEUATgBDAEUAKABsAGUAbgBfAHEALAAgADEALAAgADIAKQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAYwB1AHIAcgBfAHAALAAgAEQAUgBPAFAAKABzAHQAYQB0AGUALAAgAGwAZQBuAF8AcQAgACsAIAAxACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBDAG8AbQBwAGEAcgBlACgAYwB1AHIAcgBfAHAALAAgAGwAaQBtAGIAcwBfAGEAKQAgAD4AIAAwACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABuAGUAeAB0AF8AcQAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBTAHUAYgAoAGMAdQByAHIAXwBxACwAIAB7ADEAfQAsACAAawApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAG4AZQB4AHQAXwBwACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAFMAdQBiACgAYwB1AHIAcgBfAHAALAAgAGwAaQBtAGIAcwBfAGIALAAgAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABWAFMAVABBAEMASwAoAFIATwBXAFMAKABuAGUAeAB0AF8AcQApACwAIABuAGUAeAB0AF8AcQAsACAAbgBlAHgAdABfAHAAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHMAdABhAHQAZQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAKQApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAALwAvACAAUwB3AGUAZQBwACAAVQBwADoAIABJAGYAIABQACAAKwAgAEIAIAA8AD0AIABBACwAIABRACAAaQBzACAAdABvAG8AIABzAG0AYQBsAGwALgAgAFMAdABlAHAAIABRACAAdQBwACAAYgB5ACAAMQAsACAAYQBuAGQAIABQACAAdQBwACAAYgB5ACAAQgAuAFwAbgAgACAAIAAgACAAIAAgACAAcwB3AGUAZQBwAF8AdQBwACwAIABSAEUARABVAEMARQAoAHMAdwBlAGUAcABfAGQAbwB3AG4ALAAgAHsAMQA7ACAAMgB9ACwAIABMAEEATQBCAEQAQQAoAHMAdABhAHQAZQAsACAAaQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAZQBuAF8AcQAsACAASQBOAEQARQBYACgAcwB0AGEAdABlACwAIAAxACwAIAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABjAHUAcgByAF8AcQAsACAAQwBIAE8ATwBTAEUAUgBPAFcAUwAoAHMAdABhAHQAZQAsACAAUwBFAFEAVQBFAE4AQwBFACgAbABlAG4AXwBxACwAIAAxACwAIAAyACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGMAdQByAHIAXwBwACwAIABEAFIATwBQACgAcwB0AGEAdABlACwAIABsAGUAbgBfAHEAIAArACAAMQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbgBlAHgAdABfAHAAXwB0AGUAcwB0ACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAEEAZABkACgAYwB1AHIAcgBfAHAALAAgAGwAaQBtAGIAcwBfAGIALAAgAGsAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAEMAbwBtAHAAYQByAGUAKABuAGUAeAB0AF8AcABfAHQAZQBzAHQALAAgAGwAaQBtAGIAcwBfAGEAKQAgADwAPQAgADAALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAG4AZQB4AHQAXwBxACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAEEAZABkACgAYwB1AHIAcgBfAHEALAAgAHsAMQB9ACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAVgBTAFQAQQBDAEsAKABSAE8AVwBTACgAbgBlAHgAdABfAHEAKQAsACAAbgBlAHgAdABfAHEALAAgAG4AZQB4AHQAXwBwAF8AdABlAHMAdAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcwB0AGEAdABlAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAApACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABFAHgAdAByAGEAYwB0ACAARgBpAG4AYQBsACAAUQAgAGEAbgBkACAAUABcAG4AIAAgACAAIAAgACAAIAAgAGYAaQBuAGEAbABfAGwAZQBuAF8AcQAsACAASQBOAEQARQBYACgAcwB3AGUAZQBwAF8AdQBwACwAIAAxACwAIAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAGYAaQBuAGEAbABfAHEALAAgAEMASABPAE8AUwBFAFIATwBXAFMAKABzAHcAZQBlAHAAXwB1AHAALAAgAFMARQBRAFUARQBOAEMARQAoAGYAaQBuAGEAbABfAGwAZQBuAF8AcQAsACAAMQAsACAAMgApACkALABcAG4AIAAgACAAIAAgACAAIAAgAGYAaQBuAGEAbABfAHAALAAgAEQAUgBPAFAAKABzAHcAZQBlAHAAXwB1AHAALAAgAGYAaQBuAGEAbABfAGwAZQBuAF8AcQAgACsAIAAxACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAvAC8AIAA0AC4AIABFAHgAdAByAGEAYwB0ACAAVAByAHUAZQAgAFIAZQBtAGEAaQBuAGQAZQByACAAUwBhAGYAZQBsAHkAIAAoAEEAIAAtACAARgBpAG4AYQBsAF8AUAApAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAG4AYQBsAF8AcgAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBTAHUAYgAoAGwAaQBtAGIAcwBfAGEALAAgAGYAaQBuAGEAbABfAHAALAAgAGsAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAFYAUwBUAEEAQwBLACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIATwBXAFMAKABmAGkAbgBhAGwAXwByACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAZgBpAG4AYQBsAF8AcgAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABmAGkAbgBhAGwAXwBxAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAAWwBJAG4AdABlAHIAbgBhAGwAXQAgAFUAbgBzAGkAZwBuAGUAZAAgAEIAYQBzAGUALQAxADAAIABMAGUAZgB0AC0AdABvAC0AUgBpAGcAaAB0ACAARQB4AHAAbwBuAGUAbgB0AGkAYQB0AGkAbwBuAC4AXABuACAAKgAgAEUAdgBhAGwAdQBhAHQAZQBzACAAdABoAGUAIABlAHgAcABvAG4AZQBuAHQAIABpAHQAZQByAGEAdABpAHYAZQBsAHkAIAB1AHMAaQBuAGcAIABhACAAcAByAGUALQBjAG8AbQBwAHUAdABlAGQAIAAxAC0AOQAgAGMAYQBjAGgAZQAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGwAaQBtAGIAcwBfAGIAYQBzAGUAIABUAGgAZQAgAGwAaQB0AHQAbABlAC0AZQBuAGQAaQBhAG4AIABsAGkAbQBiACAAYQByAHIAYQB5ACAAbwBmACAAdABoAGUAIABiAGEAcwBlAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAZQB4AHAAXwBzAHQAcgBpAG4AZwAgAFQAaABlACAAZQB4AGEAYwB0ACAAdABlAHgAdAAgAHMAdAByAGkAbgBnACAAbwBmACAAdABoAGUAIABlAHgAcABvAG4AZQBuAHQALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABrACAAVABoAGUAIABkAHkAbgBhAG0AaQBjACAAYwBoAHUAbgBrACAAcwBpAHoAZQAgAGMAbwBuAHQAZQB4AHQALgBcAG4AIAAqAC8AXABuAFUAUABvAHcAIAA9ACAATABBAE0AQgBEAEEAKABsAGkAbQBiAHMAXwBiAGEAcwBlACwAIABlAHgAcABfAHMAdAByAGkAbgBnACwAIABrACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAC8ALwAgAFAAcgBlAC0AYwBvAG0AcAB1AHQAZQAgAHAAbwB3AGUAcgBzACAAMQAgAHQAaAByAG8AdQBnAGgAIAA5AC4AXABuACAAIAAgACAAIAAgACAAIABmAGkAcgBzAHQALAAgAGwAaQBtAGIAcwBfAGIAYQBzAGUALABcAG4AIAAgACAAIAAgACAAIAAgAHMAZQBjAG8AbgBkACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAE0AdQBsACgAZgBpAHIAcwB0ACwAIABmAGkAcgBzAHQALAAgAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAdABoAGkAcgBkACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAE0AdQBsACgAcwBlAGMAbwBuAGQALAAgAGYAaQByAHMAdAAsACAAawApACwAXABuACAAIAAgACAAIAAgACAAIABmAG8AdQByAHQAaAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBNAHUAbAAoAHMAZQBjAG8AbgBkACwAIABzAGUAYwBvAG4AZAAsACAAawApACwAXABuACAAIAAgACAAIAAgACAAIABmAGkAZgB0AGgALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFUATQB1AGwAKABmAG8AdQByAHQAaAAsACAAZgBpAHIAcwB0ACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAaQB4AHQAaAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBNAHUAbAAoAHQAaABpAHIAZAAsACAAdABoAGkAcgBkACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAZQB2AGUAbgB0AGgALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFUATQB1AGwAKABzAGkAeAB0AGgALAAgAGYAaQByAHMAdAAsACAAawApACwAXABuACAAIAAgACAAIAAgACAAIABlAGkAZwB0AGgALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFUATQB1AGwAKABmAG8AdQByAHQAaAAsACAAZgBvAHUAcgB0AGgALAAgAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbgBpAG4AdABoACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAE0AdQBsACgAZQBpAGcAdABoACwAIABmAGkAcgBzAHQALAAgAGsAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAGUAeABwAF8AZABpAGcAaQB0AHMALAAgAC0ALQBNAEkARAAoAGUAeABwAF8AcwB0AHIAaQBuAGcALAAgAFMARQBRAFUARQBOAEMARQAoAEwARQBOACgAZQB4AHAAXwBzAHQAcgBpAG4AZwApACkALAAgADEAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAFIARQBEAFUAQwBFACgAMQAsACAAZQB4AHAAXwBkAGkAZwBpAHQAcwAsACAATABBAE0AQgBEAEEAKABhAGMAYwAsACAAZABpAGcAaQB0ACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAAUwBoAG8AcgB0AC0AYwBpAHIAYwB1AGkAdAA6ACAAUwBrAGkAcAAgAGMAYQBsAGMAdQBsAGEAdABpAG4AZwAgADEAXgAxADAAIABkAHUAcgBpAG4AZwAgAGwAZQBhAGQAaQBuAGcAIABpAHQAZQByAGEAdABpAG8AbgBzAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGkAcwBfAG8AbgBlACwAIABBAE4ARAAoAFIATwBXAFMAKABhAGMAYwApACAAPQAgADEALAAgAEkATgBEAEUAWAAoAGEAYwBjACwAIAAxACwAIAAxACkAIAA9ACAAMQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAAMQAuACAAUgBhAGkAcwBlACAAQQBjAGMAIAB0AG8AIAB0AGgAZQAgADEAMAB0AGgAIABwAG8AdwBlAHIAIAB1AHMAaQBuAGcAIABlAHgAYQBjAHQAbAB5ACAANAAgAG0AdQBsAHQAaQBwAGwAaQBjAGEAdABpAG8AbgBzAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGEAYwBjAF8AMQAwACwAIABJAEYAKABpAHMAXwBvAG4AZQAsACAAYQBjAGMALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGEAYwBjAF8AMgAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBNAHUAbAAoAGEAYwBjACwAIABhAGMAYwAsACAAawApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGEAYwBjAF8ANAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBNAHUAbAAoAGEAYwBjAF8AMgAsACAAYQBjAGMAXwAyACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAYQBjAGMAXwA4ACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAE0AdQBsACgAYQBjAGMAXwA0ACwAIABhAGMAYwBfADQALAAgAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAE0AdQBsACgAYQBjAGMAXwA4ACwAIABhAGMAYwBfADIALAAgAGsAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIAAyAC4AIABNAHUAbAB0AGkAcABsAHkAIABiAHkAIAB0AGgAZQAgAGMAbwByAHIAZQBzAHAAbwBuAGQAaQBuAGcAIABwAHIAZQAtAGMAbwBtAHAAdQB0AGUAZAAgAGMAYQBjAGgAZQAgAHYAYQBsAHUAZQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABkAGkAZwBpAHQAIAA9ACAAMAAsACAAYQBjAGMAXwAxADAALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGMAYQBjAGgAZQBfAHYAYQBsACwAIABDAEgATwBPAFMARQAoAGQAaQBnAGkAdAAsACAAZgBpAHIAcwB0ACwAIABzAGUAYwBvAG4AZAAsACAAdABoAGkAcgBkACwAIABmAG8AdQByAHQAaAAsACAAZgBpAGYAdABoACwAIABzAGkAeAB0AGgALAAgAHMAZQB2AGUAbgB0AGgALAAgAGUAaQBnAHQAaAAsACAAbgBpAG4AdABoACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgAaQBzAF8AbwBuAGUALAAgAGMAYQBjAGgAZQBfAHYAYQBsACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAE0AdQBsACgAYQBjAGMAXwAxADAALAAgAGMAYQBjAGgAZQBfAHYAYQBsACwAIABrACkAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAAWwBJAG4AdABlAHIAbgBhAGwAXQAgAFUAbgBzAGkAZwBuAGUAZAAgAEkAbgB0AGUAZwBlAHIAIABTAHEAdQBhAHIAZQAgAFIAbwBvAHQAIAB1AHMAaQBuAGcAIABOAGUAdwB0AG8AbgAnAHMAIABNAGUAdABoAG8AZAAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGwAaQBtAGIAcwBfAG4AIABSAGEAZABpAGMAYQBuAGQAIABsAGkAdAB0AGwAZQAtAGUAbgBkAGkAYQBuACAAYQByAHIAYQB5AC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAbABpAG0AYgBzAF8AcwBlAGUAZAAgAE8AdgBlAHIALQBlAHMAdABpAG0AYQB0AGUAZAAgAGwAaQB0AHQAbABlAC0AZQBuAGQAaQBhAG4AIABzAGUAZQBkACAAYQByAHIAYQB5AC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAawAgAFQAaABlACAAZAB5AG4AYQBtAGkAYwAgAGMAaAB1AG4AawAgAHMAaQB6AGUAIABjAG8AbgB0AGUAeAB0AC4AXABuACAAKgAvAFwAbgBVAFMAcQByAHQAIAA9ACAATABBAE0AQgBEAEEAKABsAGkAbQBiAHMAXwBuACwAIABsAGkAbQBiAHMAXwBzAGUAZQBkACwAIABrACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAC8ALwAgAFMAdABhAHQAZQAgAGkAcwAgAHAAYQBjAGsAZQBkADoAIABWAFMAVABBAEMASwAoAGkAcwBfAGQAbwBuAGUAXwBmAGwAYQBnACwAIABjAHUAcgByAGUAbgB0AF8AeAApAFwAbgAgACAAIAAgACAAIAAgACAAaQBuAGkAdABpAGEAbABfAHMAdABhAHQAZQAsACAAVgBTAFQAQQBDAEsAKAAwACwAIABsAGkAbQBiAHMAXwBzAGUAZQBkACkALABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQB4AF8AaQB0AGUAcgBzACwAIAAzADUALABcAG4AXABuACAAIAAgACAAIAAgACAAIABmAGkAbgBhAGwAXwBzAHQAYQB0AGUALAAgAFIARQBEAFUAQwBFACgAaQBuAGkAdABpAGEAbABfAHMAdABhAHQAZQAsACAAUwBFAFEAVQBFAE4AQwBFACgAbQBhAHgAXwBpAHQAZQByAHMAKQAsACAATABBAE0AQgBEAEEAKABzAHQAYQB0AGUALAAgAGkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABpAHMAXwBkAG8AbgBlACwAIABJAE4ARABFAFgAKABzAHQAYQB0AGUALAAgADEALAAgADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGMAdQByAHIAXwB4ACwAIABEAFIATwBQACgAcwB0AGEAdABlACwAIAAxACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgAaQBzAF8AZABvAG4AZQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcwB0AGEAdABlACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIAAxAC4AIABEAGkAdgBpAHMAaQBvAG4AOgAgAG4AIAAvACAAeABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAZABpAHYAXwBwAGEAYwBrAGUAZAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4ARABpAHYAUgBvAHUAdABlAHIAKABsAGkAbQBiAHMAXwBuACwAIABjAHUAcgByAF8AeAAsACAAawApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAZQBuAF8AcgAsACAASQBOAEQARQBYACgAZABpAHYAXwBwAGEAYwBrAGUAZAAsACAAMQAsACAAMQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHEALAAgAEQAUgBPAFAAKABkAGkAdgBfAHAAYQBjAGsAZQBkACwAIABsAGUAbgBfAHIAIAArACAAMQApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIAAyAC4AIABBAGQAZABpAHQAaQBvAG4AOgAgAHgAIAArACAAKABuACAALwAgAHgAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcwB1AG0AXwB4AHEALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFUAQQBkAGQAKABjAHUAcgByAF8AeAAsACAAcQAsACAAawApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIAAzAC4AIABIAGEAbAB2AGkAbgBnADoAIAAoAHgAIAArACAAKABuACAALwAgAHgAKQApACAALwAgADIAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAEsAbgB1AHQAaABEAGkAdgAgAGkAbgBoAGUAcgBlAG4AdABsAHkAIABzAHUAcABwAG8AcgB0AHMAIABzAGMAYQBsAGEAcgAgAGQAaQB2AGkAcwBvAHIAcwAgAHcAaQB0AGgAIAB6AGUAcgBvACAAbwB2AGUAcgBoAGUAYQBkAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABkAGkAdgBfADIAXwBwAGEAYwBrAGUAZAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4ASwBuAHUAdABoAEQAaQB2ACgAcwB1AG0AXwB4AHEALAAgAHsAMgB9ACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABlAG4AXwByADIALAAgAEkATgBEAEUAWAAoAGQAaQB2AF8AMgBfAHAAYQBjAGsAZQBkACwAIAAxACwAIAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAeABfAG4AZQB4AHQALAAgAEQAUgBPAFAAKABkAGkAdgBfADIAXwBwAGEAYwBrAGUAZAAsACAAbABlAG4AXwByADIAIAArACAAMQApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIAA0AC4AIABDAG8AbgB2AGUAcgBnAGUAbgBjAGUAIABDAGgAZQBjAGsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGMAbwBtAHAALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFUAQwBvAG0AcABhAHIAZQAoAHgAXwBuAGUAeAB0ACwAIABjAHUAcgByAF8AeAApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIABOAGUAdwB0AG8AbgAnAHMAIABtAGUAdABoAG8AZAAgAGMAbwBuAHYAZQByAGcAZQBzACAAbwBuACAAdABoAGUAIABmAGwAbwBvAHIAIAByAG8AbwB0ACwAIABhAG4AZAAgAHMAdABhAGIAaQBsAGkAegBlAHMAIABvAHIAIABvAHMAYwBpAGwAbABhAHQAZQBzACAAdQBwACAAYgB5ACAAMQAuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIABUAGgAZQByAGUAZgBvAHIAZQAsACAAaQBmACAAeABfAG4AZQB4AHQAIAA+AD0AIABjAHUAcgByAF8AeAAsACAAdABoAGUAIABhAGwAZwBvAHIAaQB0AGgAbQAgAGgAYQBzACAAYwBvAG4AdgBlAHIAZwBlAGQALgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgAYwBvAG0AcAAgAD4APQAgADAALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABWAFMAVABBAEMASwAoADEALAAgAGMAdQByAHIAXwB4ACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABWAFMAVABBAEMASwAoADAALAAgAHgAXwBuAGUAeAB0ACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAApACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIABEAFIATwBQACgAZgBpAG4AYQBsAF8AcwB0AGEAdABlACwAIAAxACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFsASQBuAHQAZQByAG4AYQBsAF0AIABHAGUAbgBlAHIAYQB0AGUAcwAgAGEAIAAxAEQAIAB2AGUAcgB0AGkAYwBhAGwAIABhAHIAcgBhAHkAIABvAGYAIABhAGwAbAAgAHAAcgBpAG0AZQAgAG4AdQBtAGIAZQByAHMAIAB1AHAAIAB0AG8AIABuAC4AXABuACAAKgAgAEUAdgBhAGwAdQBhAHQAZQBzACAAcAB1AHIAZQBsAHkAIABpAG4AIABuAGEAdABpAHYAZQAgAEMAKwArACAAdQBzAGkAbgBnACAAYQAgAGQAeQBuAGEAbQBpAGMAIABzAGkAZQB2AGUALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABuACAAVABoAGUAIAB1AHAAcABlAHIAIABiAG8AdQBuAGQAIABpAG4AdABlAGcAZQByACAAKABhAHMAcwB1AG0AZQBkACAAPAA9ACAAOQAyADcAMwApAC4AXABuACAAKgAvAFwAbgBOAGEAdABpAHYAZQBQAHIAaQBtAGUAcwAgAD0AIABMAEEATQBCAEQAQQAoAG4ALABcAG4AIAAgACAAIABJAEYAKABuACAAPAAgADIALAAgACMATgBVAE0AIQAsAFwAbgAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAcwBlAHEALAAgAFMARQBRAFUARQBOAEMARQAoAG4AIAAtACAAMQAsACAAMQAsACAAMgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSACgAcwBlAHEALAAgAE0AQQBQACgAcwBlAHEALAAgAEwAQQBNAEIARABBACgAeAAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGkAbQBpAHQALAAgAEkATgBUACgAUwBRAFIAVAAoAHgAKQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABsAGkAbQBpAHQAIAA8ACAAMgAsACAAVABSAFUARQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEkATgAoAE0ATwBEACgAeAAsACAAUwBFAFEAVQBFAE4AQwBFACgAbABpAG0AaQB0ACAALQAgADEALAAgADEALAAgADIAKQApACkAIAA+ACAAMABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQApACkAXABuACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABbAEkAbgB0AGUAcgBuAGEAbABdACAAVQBuAHMAYQBmAGUALAAgAGgAaQBnAGgALQBwAGUAcgBmAG8AcgBtAGEAbgBjAGUAIAB0AGUAeAB0ACAAbQB1AGwAdABpAHAAbABpAGMAYQB0AGkAbwBuACAAZgBvAHIAIAB0AHIAdQBzAHQAZQBkACwAIABwAG8AcwBpAHQAaQB2AGUAIABCAGkAZwBJAG4AdAAgAHMAdAByAGkAbgBnAHMALgBcAG4AIAAqACAAQgB5AHAAYQBzAHMAZQBzACAATABhAHkAZQByACAAMAAgAHYAYQBsAGkAZABhAHQAaQBvAG4ALgAgAEkAbQBwAGwAZQBtAGUAbgB0AHMAIABzAHQAcgBpAGMAdAAgAHMAaABvAHIAdAAtAGMAaQByAGMAdQBpAHQAcwAgAGYAbwByACAAcABhAGQAZABpAG4AZwAgAG8AcAB0AGkAbQBpAHoAYQB0AGkAbwBuAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAcwB0AHIAXwBhACAAVABoAGUAIABmAGkAcgBzAHQAIAB0AHIAdQBzAHQAZQBkACAAQgBpAGcASQBuAHQAIABzAHQAcgBpAG4AZwAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAHMAdAByAF8AYgAgAFQAaABlACAAcwBlAGMAbwBuAGQAIAB0AHIAdQBzAHQAZQBkACAAQgBpAGcASQBuAHQAIABzAHQAcgBpAG4AZwAuAFwAbgAgACoALwBcAG4AVQBUAGUAeAB0AE0AdQBsACAAPQAgAEwAQQBNAEIARABBACgAcwB0AHIAXwBhACwAIABzAHQAcgBfAGIALABcAG4AIAAgACAAIABJAEYAKABPAFIAKABzAHQAcgBfAGEAIAA9ACAAXAAiADAAXAAiACwAIABzAHQAcgBfAGIAIAA9ACAAXAAiADAAXAAiACkALAAgAFwAIgAwAFwAIgAsAFwAbgAgACAAIAAgAEkARgAoAHMAdAByAF8AYQAgAD0AIABcACIAMQBcACIALAAgAHMAdAByAF8AYgAsAFwAbgAgACAAIAAgAEkARgAoAHMAdAByAF8AYgAgAD0AIABcACIAMQBcACIALAAgAHMAdAByAF8AYQAsAFwAbgAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABlAG4AXwBhACwAIABMAEUATgAoAHMAdAByAF8AYQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAZQBuAF8AYgAsACAATABFAE4AKABzAHQAcgBfAGIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABrACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBTAGEAZgBlAEsAKABcACIATQBVAEwAXAAiACwAIABNAEkATgAoAGwAZQBuAF8AYQAsACAAbABlAG4AXwBiACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYQAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwBwAGwAaQB0ACgAcwB0AHIAXwBhACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYgAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwBwAGwAaQB0ACgAcwB0AHIAXwBiACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGYAaQBuAGEAbABfAGwAaQBtAGIAcwAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBNAHUAbAAoAGwAaQBtAGIAcwBfAGEALAAgAGwAaQBtAGIAcwBfAGIALAAgAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4ATQBlAHIAZwBlACgAZgBpAG4AYQBsAF8AbABpAG0AYgBzACwAIABrACkAXABuACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAKQApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAAWwBJAG4AdABlAHIAbgBhAGwAXQAgAFYAZQBjAHQAbwByAGkAegBlAGQAIABsAG8AZwBhAHIAaQB0AGgAbQBpAGMAIABwAHIAbwBkAHUAYwB0ACAAbwBmACAAYQBuACAAYQByAHIAYQB5ACAAbwBmACAAQgBpAGcASQBuAHQAIABzAHQAcgBpAG4AZwBzAC4AXABuACAAKgAgAFIAZQBjAHUAcgBzAGkAdgBlAGwAeQAgAGMAdQB0AHMAIAB0AGgAZQAgAGEAcgByAGEAeQAgAGkAbgAgAGgAYQBsAGYAIAB0AG8AIABiAHkAcABhAHMAcwAgAFIARQBEAFUAQwBFACAAcwBlAHEAdQBlAG4AdABpAGEAbAAgAG0AZQBtAG8AcgB5ACAAYQBsAGwAbwBjAGEAdABpAG8AbgBzAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAdABlAHgAdABfAGEAcgByACAAQQAgADEARAAgAHYAZQByAHQAaQBjAGEAbAAgAGEAcgByAGEAeQAgAG8AZgAgAEIAaQBnAEkAbgB0ACAAcwB0AHIAaQBuAGcAcwAuAFwAbgAgACoALwBcAG4AVABlAHgAdABUAHIAZQBlAFAAcgBvAGQAIAA9ACAATABBAE0AQgBEAEEAKAB0AGUAeAB0AF8AYQByAHIALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbgAsACAAUgBPAFcAUwAoAHQAZQB4AHQAXwBhAHIAcgApACwAXABuACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAG4AIAA9ACAAMQAsACAASQBOAEQARQBYACgAdABlAHgAdABfAGEAcgByACwAIAAxACwAIAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIABSAGUAcwBoAGEAcABlACAAYQByAHIAYQB5ACAAaQBuAHQAbwAgAHAAYQBpAHIAcwAuACAATwBkAGQALQBsAGUAbgBnAHQAaAAgAGEAcgByAGEAeQBzACAAYQByAGUAIABzAGEAZgBlAGwAeQAgAHAAYQBkAGQAZQBkACAAdwBpAHQAaAAgAHQAaABlACAAbQB1AGwAdABpAHAAbABpAGMAYQB0AGkAdgBlACAAaQBkAGUAbgB0AGkAdAB5ACAAXAAiADEAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHAAYQBpAHIAZQBkACwAIABXAFIAQQBQAFIATwBXAFMAKAB0AGUAeAB0AF8AYQByAHIALAAgADIALAAgAFwAIgAxAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAAVgBlAGMAdABvAHIAaQB6AGUAZAAgAG0AdQBsAHQAaQBwAGwAaQBjAGEAdABpAG8AbgAgAGEAYwByAG8AcwBzACAAYQBsAGwAIABwAGEAaQByAHMAIABzAGkAbQB1AGwAdABhAG4AZQBvAHUAcwBsAHkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbgBlAHgAdABfAGEAcgByACwAIABCAFkAUgBPAFcAKABwAGEAaQByAGUAZAAsACAATABBAE0AQgBEAEEAKAByAG8AdwAsACAAVQBUAGUAeAB0AE0AdQBsACgASQBOAEQARQBYACgAcgBvAHcALAAgADEALAAgADEAKQAsACAASQBOAEQARQBYACgAcgBvAHcALAAgADEALAAgADIAKQApACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAFMAaABhAGwAbABvAHcAIAByAGUAYwB1AHIAcwBpAG8AbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBUAGUAeAB0AFQAcgBlAGUAUAByAG8AZAAoAG4AZQB4AHQAXwBhAHIAcgApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAAWwBJAG4AdABlAHIAbgBhAGwAXQAgAEMAYQBsAGMAdQBsAGEAdABlAHMAIAB0AGgAZQAgAGUAeABwAG8AbgBlAG4AdAAgAGYAbwByACAAYQBuACAAYQByAHIAYQB5ACAAbwBmACAAcAByAGkAbQBlAHMAIABpAG4AIAB0AGgAZQAgAFMAdwBpAG4AZwAgAHQAZQByAG0AIABvAGYAIABhACAAZgBhAGMAdABvAHIAaQBhAGwALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABuACAAVABoAGUAIABjAHUAcgByAGUAbgB0ACAAZgBhAGMAdABvAHIAaQBhAGwAIABtAGEAZwBuAGkAdAB1AGQAZQAgACgAPAA9ACAAOQAyADcAMwApAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAcAByAGkAbQBlAHMAIABBACAAdgBlAHIAdABpAGMAYQBsACAAYQByAHIAYQB5ACAAbwBmACAAcAByAGkAbQBlACAAbgB1AG0AYgBlAHIAcwAgACgAPAA9ACAAbgApAC4AXABuACAAKgAvAFwAbgBOAGEAdABpAHYAZQBTAHcAaQBuAGcARQB4AHAAbwBuAGUAbgB0AHMAIAA9ACAATABBAE0AQgBEAEEAKABuACwAIABwAHIAaQBtAGUAcwAsAFwAbgAgACAAIAAgAE0AQQBQACgAcAByAGkAbQBlAHMALAAgAEwAQQBNAEIARABBACgAcAAsAFwAbgAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAbQBhAHgAXwBrACwAIABJAE4AVAAoAEwATwBHACgAbgAsACAAcAApACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAcABvAHcAZQByAHMALAAgAHAAIABeACAAUwBFAFEAVQBFAE4AQwBFACgAbQBhAHgAXwBrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUwBVAE0AKABNAE8ARAAoAEkATgBUACgAbgAgAC8AIABwAG8AdwBlAHIAcwApACwAIAAyACkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAAWwBJAG4AdABlAHIAbgBhAGwAXQAgAEMAYQBsAGMAdQBsAGEAdABlAHMAIAB0AGgAZQAgAG0AYQBzAHMAaQB2AGUAIABCAGkAZwBJAG4AdAAgAHMAdAByAGkAbgBnACAAZgBvAHIAIAB0AGgAZQAgAFMAdwBpAG4AZwAgAHQAZQByAG0AIABvAGYAIABhACAAZgBhAGMAdABvAHIAaQBhAGwALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABuACAAVABoAGUAIABjAHUAcgByAGUAbgB0ACAAZgBhAGMAdABvAHIAaQBhAGwAIABtAGEAZwBuAGkAdAB1AGQAZQAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAHQAaQBlAHIAXwBwAHIAaQBtAGUAcwAgAEEAIAB2AGUAcgB0AGkAYwBhAGwAIABhAHIAcgBhAHkAIABvAGYAIABwAHIAaQBtAGUAIABuAHUAbQBiAGUAcgBzACAAKAA8AD0AIABuACkALgBcAG4AIAAqAC8AXABuAFMAdwBpAG4AZwBUAGUAcgBtACAAPQAgAEwAQQBNAEIARABBACgAbgAsACAAdABpAGUAcgBfAHAAcgBpAG0AZQBzACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAGUAeABwAG8AbgBlAG4AdABzACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBOAGEAdABpAHYAZQBTAHcAaQBuAGcARQB4AHAAbwBuAGUAbgB0AHMAKABuACwAIAB0AGkAZQByAF8AcAByAGkAbQBlAHMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAaQBzAF8AZwByAGUAYQB0AGUAcgBfAHQAaABhAG4AXwB6AGUAcgBvACwAIABlAHgAcABvAG4AZQBuAHQAcwAgAD4AIAAwACwAXABuACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgAC8ALwAgAEkAZgAgAGEAbABsACAAZQB4AHAAbwBuAGUAbgB0AHMAIABhAHIAZQAgADAALAAgAHQAaABlACAAcwB3AGkAbgBnACAAdABlAHIAbQAgAGkAcwAgADEALgBcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAEEATgBEACgATgBPAFQAKABpAHMAXwBnAHIAZQBhAHQAZQByAF8AdABoAGEAbgBfAHoAZQByAG8AKQApACwAIABcACIAMQBcACIALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABmAGkAbAB0AGUAcgBlAGQAXwBwAHIAaQBtAGUAcwAsACAARgBJAEwAVABFAFIAKAB0AGkAZQByAF8AcAByAGkAbQBlAHMALAAgAGkAcwBfAGcAcgBlAGEAdABlAHIAXwB0AGgAYQBuAF8AegBlAHIAbwApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAZgBpAGwAdABlAHIAZQBkAF8AZQB4AHAAcwAsACAARgBJAEwAVABFAFIAKABlAHgAcABvAG4AZQBuAHQAcwAsACAAaQBzAF8AZwByAGUAYQB0AGUAcgBfAHQAaABhAG4AXwB6AGUAcgBvACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABwAHIAaQBtAGUAXwBwAG8AdwBlAHIAcwAsACAATQBBAFAAKABmAGkAbAB0AGUAcgBlAGQAXwBwAHIAaQBtAGUAcwAsACAAZgBpAGwAdABlAHIAZQBkAF8AZQB4AHAAcwAsACAATABBAE0AQgBEAEEAKABwACwAIABlACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEkARgAoAGUAIAA9ACAAMQAsACAAcAAgACYAIABcACIAXAAiACwAIABCAGkAZwBJAG4AdAAuAFAAbwB3ACgAcAAgACYAIABcACIAXAAiACwAIABlACAAJgAgAFwAIgBcACIAKQApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFQAZQB4AHQAVAByAGUAZQBQAHIAbwBkACgAcAByAGkAbQBlAF8AcABvAHcAZQByAHMAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFsASQBuAHQAZQByAG4AYQBsAF0AIABSAGUAYwB1AHIAcwBpAHYAZQAgAHQAbwBwAC0AZABvAHcAbgAgAEwAQQBNAEIARABBACAAYwBhAGwAYwB1AGwAYQB0AGkAbgBnACAAdABoAGUAIABQAHIAaQBtAGUAIABTAHcAaQBuAGcAIABmAGEAYwB0AG8AcgBpAGEAbAAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAG4AIABUAGgAZQAgAGMAdQByAHIAZQBuAHQAIABmAGEAYwB0AG8AcgBpAGEAbAAgAG0AYQBnAG4AaQB0AHUAZABlAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAZwBsAG8AYgBhAGwAXwBwAHIAaQBtAGUAcwAgAFQAaABlACAAdQBuAGkAZgBpAGUAZAAgAHYAZQByAHQAaQBjAGEAbAAgAGEAcgByAGEAeQAgAG8AZgAgAGEAbABsACAAcAByAGkAbQBlAHMAIAB1AHAAIAB0AG8AIAB0AGgAZQAgAHQAYQByAGcAZQB0ACAAZgBhAGMAdABvAHIAaQBhAGwALgBcAG4AIAAqAC8AXABuAFAAcgBpAG0AZQBTAHcAaQBuAGcASwBlAHIAbgBlAGwAIAA9ACAATABBAE0AQgBEAEEAKABuACwAIABnAGwAbwBiAGEAbABfAHAAcgBpAG0AZQBzACwAXABuACAAIAAgACAASQBGACgAbgAgADwAIAAyACwAIABcACIAMQBcACIALABcAG4AIAAgACAAIAAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGgAYQBsAGYAXwBuACwAIABJAE4AVAAoAG4AIAAvACAAMgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGgAYQBsAGYAXwBmAGEAYwB0ACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBQAHIAaQBtAGUAUwB3AGkAbgBnAEsAZQByAG4AZQBsACgAaABhAGwAZgBfAG4ALAAgAGcAbABvAGIAYQBsAF8AcAByAGkAbQBlAHMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAAUwBxAHUAYQByAGUAIAB0AGgAZQAgAGgAYQBsAGYAdwBhAHkAIABwAG8AaQBuAHQAIAB1AHMAaQBuAGcAIAB0AGgAZQAgAHUAbgBzAGEAZgBlACAAawBlAHIAbgBlAGwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHMAcQB1AGEAcgBlAGQAXwBoAGEAbABmACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAFQAZQB4AHQATQB1AGwAKABoAGEAbABmAF8AZgBhAGMAdAAsACAAaABhAGwAZgBfAGYAYQBjAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAASQBzAG8AbABhAHQAZQAgAHQAaABlACAAcAByAGkAbQBlAHMAIABuAGUAZQBkAGUAZAAgAGYAbwByACAAdABoAGkAcwAgAHQAaQBlAHIAIABhAG4AZAAgAGMAYQBsAGMAdQBsAGEAdABlACAAdABoAGUAIABzAHcAaQBuAGcAIAB0AGUAcgBtAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAB0AGkAZQByAF8AcAByAGkAbQBlAHMALAAgAEYASQBMAFQARQBSACgAZwBsAG8AYgBhAGwAXwBwAHIAaQBtAGUAcwAsACAAZwBsAG8AYgBhAGwAXwBwAHIAaQBtAGUAcwAgADwAPQAgAG4AKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABzAHcAaQBuAGcALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFMAdwBpAG4AZwBUAGUAcgBtACgAbgAsACAAdABpAGUAcgBfAHAAcgBpAG0AZQBzACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFUAVABlAHgAdABNAHUAbAAoAHMAcQB1AGEAcgBlAGQAXwBoAGEAbABmACwAIABzAHcAaQBuAGcAKQBcAG4AIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFsASQBuAHQAZQByAG4AYQBsAF0AIABSAGUAYwB1AHIAcwBpAHYAZQAgAHQAbwB1AHIAbgBhAG0AZQBuAHQAIAB0AHIAZQBlACAAZgBvAHIAIABNAGkAbgAvAE0AYQB4ACAAZQB2AGEAbAB1AGEAdABpAG8AbgBzAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAYwBvAGwAIABBACAAMQBEACAAdgBlAHIAdABpAGMAYQBsACAAYQByAHIAYQB5ACAAbwBmACAAbgBvAHIAbQBhAGwAaQB6AGUAZAAgAEIAaQBnAEkAbgB0ACAAcwB0AHIAaQBuAGcAcwAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAG0AbwBkAGUAIAAxACAAZgBvAHIAIABNAGEAeABpAG0AdQBtACwAIAAtADEAIABmAG8AcgAgAE0AaQBuAGkAbQB1AG0ALgBcAG4AIAAqAC8AXABuAFQAcgBlAGUAQwBvAG0AcABhAHIAZQAgAD0AIABMAEEATQBCAEQAQQAoAGMAbwBsACwAIABtAG8AZABlACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG4ALAAgAFIATwBXAFMAKABjAG8AbAApACwAXABuACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAG4AIAA9ACAAMQAsACAASQBOAEQARQBYACgAYwBvAGwALAAgADEALAAgADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHAAYQBpAHIAZQBkACwAIABXAFIAQQBQAFIATwBXAFMAKABjAG8AbAAsACAAMgAsACAAXAAiACMAUABBAEQAIwBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGMAbwBsAF8AYQAsACAAVABBAEsARQAoAHAAYQBpAHIAZQBkACwAIAAsACAAMQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAYwBvAGwAXwBiACwAIABUAEEASwBFACgAcABhAGkAcgBlAGQALAAgACwAIAAtADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHcAaQBuAG4AZQByAHMALAAgAE0AQQBQACgAYwBvAGwAXwBhACwAIABjAG8AbABfAGIALAAgAEwAQQBNAEIARABBACgAYQAsACAAYgAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgAYgAgAD0AIABcACIAIwBQAEEARAAjAFwAIgAsACAAYQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGMAbwBtAHAALAAgAEIAaQBnAEkAbgB0AC4AQwBvAG0AcABhAHIAZQAoAGEALAAgAGIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEkARgAoAGMAbwBtAHAAIAAqACAAbQBvAGQAZQAgAD4APQAgADAALAAgAGEALAAgAGIAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVAByAGUAZQBDAG8AbQBwAGEAcgBlACgAdwBpAG4AbgBlAHIAcwAsACAAbQBvAGQAZQApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBCAGkAZwBJAG4AdAAiACwAIgB0AGUAeAB0ACIAOgAiAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAFwAbgAvAC8AIABCAGkAZwAgAEkAbgB0AGUAZwBlAHIAIABBAHIAaQB0AGgAbQBlAHQAaQBjACAATABpAGIAcgBhAHIAeQAgAC8ALwBcAG4ALwAvACAAIAAgACAAIAAgACAAIABCAGkAZwBJAG4AdAAgAE0AbwBkAHUAbABlACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AXABuAC8ALwAgACAAIAAgACAAIAAgACAAIAAgAFAAdQBiAGwAaQBjACAAQQBQAEkAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvAFwAbgAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABOAG8AcgBtAGEAbABpAHMAZQBzACAAYQAgAEIAaQBnAEkAbgB0ACAAcwB0AHIAaQBuAGcALgAgAFMAdAByAGkAcABzACAAbABlAGEAZABpAG4AZwAgAHoAZQByAG8AcwAsACAAcgBlAHMAbwBsAHYAZQBzACAAXAAiAC0AMABcACIAIAB0AG8AIABcACIAMABcACIALAAgAGEAbgBkACAAdABoAHIAbwB3AHMAIAAjAFYAQQBMAFUARQAhACAAbwBuACAAaQBuAHYAYQBsAGkAZAAgAGMAaABhAHIAYQBjAHQAZQByAHMALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABiAGkAZwBfAGkAbgB0ACAAVABoAGUAIABCAGkAZwBJAG4AdAAgAHMAdAByAGkAbgBnAC4AXABuACAAKgAvAFwAbgBOAG8AcgBtACAAPQAgAEwAQQBNAEIARABBACgAYgBpAGcAXwBpAG4AdAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABzAHQAcgAsACAASQBGACgATwBSACgASQBTAE8ATQBJAFQAVABFAEQAKABiAGkAZwBfAGkAbgB0ACkALAAgAGIAaQBnAF8AaQBuAHQAIAA9ACAAXAAiAFwAIgApACwAIABcACIAMABcACIALAAgAGIAaQBnAF8AaQBuAHQAIAAmACAAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABpAHMAXwB2AGEAbABpAGQALAAgAFIARQBHAEUAWABUAEUAUwBUACgAcwB0AHIALAAgAFwAIgBeAC0APwBcAFwAZAArACQAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAdAByAGkAcABwAGUAZAAsACAAUgBFAEcARQBYAFIARQBQAEwAQQBDAEUAKABzAHQAcgAsACAAXAAiAF4AKAAtAD8AKQAwACsAKAA/AD0AXABcAGQAKQBcACIALAAgAFwAIgAkADEAXAAiACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIABJAEYAKABOAE8AVAAoAGkAcwBfAHYAYQBsAGkAZAApACwAIABWAEEATABVAEUAKABcACIAIwBWAEEATABVAEUAIQBcACIAKQAsACAASQBGACgAcwB0AHIAaQBwAHAAZQBkACAAPQAgAFwAIgAtADAAXAAiACwAIABcACIAMABcACIALAAgAHMAdAByAGkAcABwAGUAZAApACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFIAZQB0AHUAcgBuAHMAIAB0AGgAZQAgAHMAaQBnAG4AIABvAGYAIABhACAAQgBpAGcASQBuAHQAOgAgADEAIAAoAHAAbwBzAGkAdABpAHYAZQApACwAIAAtADEAIAAoAG4AZQBnAGEAdABpAHYAZQApACwAIABvAHIAIAAwACAAKAB6AGUAcgBvACkALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABiAGkAZwBfAGkAbgB0ACAAVABoAGUAIABCAGkAZwBJAG4AdAAgAHMAdAByAGkAbgBnAC4AXABuACAAKgAvAFwAbgBTAGkAZwBuACAAPQAgAEwAQQBNAEIARABBACgAYgBpAGcAXwBpAG4AdAAsACAAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG4AbwByAG0AZQBkACwAIABOAG8AcgBtACgAYgBpAGcAXwBpAG4AdAApACwAXABuACAAIAAgACAAIAAgACAAIABTAFcASQBUAEMASAAoAEwARQBGAFQAKABuAG8AcgBtAGUAZAApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAwAFwAIgAsACAAMAAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIALQBcACIALAAgAC0AMQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvAC8AIAAtAC0ALQAgAFAAcgBlAGQAaQBjAGEAdABlAHMAIAAtAC0ALQAgAFwAXABcAFwAXABuAFwAbgAvACoAKgBcAG4AIAAqACAAUgBlAHQAdQByAG4AcwAgAFQAUgBVAEUAIABpAGYAIAB0AGgAZQAgAEIAaQBnAEkAbgB0ACAAaQBzACAAZQB4AGEAYwB0AGwAeQAgAHoAZQByAG8ALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABiAGkAZwBfAGkAbgB0ACAAVABoAGUAIABCAGkAZwBJAG4AdAAgAHMAdAByAGkAbgBnAC4AXABuACAAKgAvAFwAbgBJAHMAWgBlAHIAbwAgAD0AIABMAEEATQBCAEQAQQAoAGIAaQBnAF8AaQBuAHQALAAgAE4AbwByAG0AKABiAGkAZwBfAGkAbgB0ACkAIAA9ACAAXAAiADAAXAAiACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABSAGUAdAB1AHIAbgBzACAAVABSAFUARQAgAGkAZgAgAHQAaABlACAAQgBpAGcASQBuAHQAIABpAHMAIABuAGUAZwBhAHQAaQB2AGUALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABiAGkAZwBfAGkAbgB0ACAAVABoAGUAIABCAGkAZwBJAG4AdAAgAHMAdAByAGkAbgBnAC4AXABuACAAKgAvAFwAbgBJAHMATgBlAGcAIAA9ACAATABBAE0AQgBEAEEAKABiAGkAZwBfAGkAbgB0ACwAIABMAEUARgBUACgATgBvAHIAbQAoAGIAaQBnAF8AaQBuAHQAKQApACAAPQAgAFwAIgAtAFwAIgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAAUgBlAHQAdQByAG4AcwAgAFQAUgBVAEUAIABpAGYAIAB0AGgAZQAgAEIAaQBnAEkAbgB0ACAAaQBzACAAZQB2AGUAbgAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGIAaQBnAF8AaQBuAHQAIABUAGgAZQAgAEIAaQBnAEkAbgB0ACAAcwB0AHIAaQBuAGcALgBcAG4AIAAqAC8AXABuAEkAcwBFAHYAZQBuACAAPQAgAEwAQQBNAEIARABBACgAYgBpAGcAXwBpAG4AdAAsACAASQBTAEUAVgBFAE4AKABWAEEATABVAEUAKABSAEkARwBIAFQAKABOAG8AcgBtACgAYgBpAGcAXwBpAG4AdAApACkAKQApACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABSAGUAdAB1AHIAbgBzACAAVABSAFUARQAgAGkAZgAgAHQAaABlACAAQgBpAGcASQBuAHQAIABpAHMAIABvAGQAZAAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGIAaQBnAF8AaQBuAHQAIABUAGgAZQAgAEIAaQBnAEkAbgB0ACAAcwB0AHIAaQBuAGcALgBcAG4AIAAqAC8AXABuAEkAcwBPAGQAZAAgAD0AIABMAEEATQBCAEQAQQAoAGIAaQBnAF8AaQBuAHQALAAgAEkAUwBPAEQARAAoAFYAQQBMAFUARQAoAFIASQBHAEgAVAAoAE4AbwByAG0AKABiAGkAZwBfAGkAbgB0ACkAKQApACkAKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFIAZQB0AHUAcgBuAHMAIAB0AGgAZQAgAHUAbgBzAGkAZwBuAGUAZAAgAG0AYQBnAG4AaQB0AHUAZABlACAAbwBmACAAYQAgAEIAaQBnAEkAbgB0ACAAcwB0AHIAaQBuAGcAIAAoAGEAYgBzAG8AbAB1AHQAZQAgAHYAYQBsAHUAZQApAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAYgBpAGcAXwBpAG4AdAAgAFQAaABlACAAQgBpAGcASQBuAHQAIABzAHQAcgBpAG4AZwAuAFwAbgAgACoALwBcAG4AQQBiAHMAIAA9ACAATABBAE0AQgBEAEEAKABiAGkAZwBfAGkAbgB0ACwAIABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbgB1AG0ALAAgAE4AbwByAG0AKABiAGkAZwBfAGkAbgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAEwARQBGAFQAKABuAHUAbQApACAAPQAgAFwAIgAtAFwAIgAsACAATQBJAEQAKABuAHUAbQAsACAAMgAsACAATABFAE4AKABuAHUAbQApACAALQAgADEAKQAsACAAbgB1AG0AKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAAQwBvAG0AcABhAHIAZQBzACAAdAB3AG8AIABCAGkAZwBJAG4AdAAgAHMAdAByAGkAbgBnAHMALgAgAFIAZQB0AHUAcgBuAHMAIAAxACAAKABhACAAPgAgAGIAKQAsACAALQAxACAAKABhACAAPAAgAGIAKQAsACAAbwByACAAMAAgACgAYQAgAD0AIABiACkALgBcAG4AIAAqACAARQB2AGEAbAB1AGEAdABlAHMAIABzAGkAZwBuAHMAIABhAG4AZAAgAGwAZQBuAGcAdABoAHMALgAgAEkAZgAgAGkAZABlAG4AdABpAGMAYQBsACwAIABkAGUAbABlAGcAYQB0AGUAcwAgAHQAbwAgAG4AYQB0AGkAdgBlACAAbABpAG0AYgAgAGEAcgByAGEAeQAgAGMAbwBtAHAAYQByAGkAcwBvAG4ALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABiAGkAZwBfAGkAbgB0AF8AYQAgAFQAaABlACAAZgBpAHIAcwB0ACAAQgBpAGcASQBuAHQAIABzAHQAcgBpAG4AZwAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGIAaQBnAF8AaQBuAHQAXwBiACAAVABoAGUAIABzAGUAYwBvAG4AZAAgAEIAaQBnAEkAbgB0ACAAcwB0AHIAaQBuAGcALgBcAG4AIAAqAC8AXABuAEMAbwBtAHAAYQByAGUAIAA9ACAATABBAE0AQgBEAEEAKABiAGkAZwBfAGkAbgB0AF8AYQAsACAAYgBpAGcAXwBpAG4AdABfAGIALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbgBvAHIAbQBfAGEALAAgAE4AbwByAG0AKABiAGkAZwBfAGkAbgB0AF8AYQApACwAXABuACAAIAAgACAAIAAgACAAIABuAG8AcgBtAF8AYgAsACAATgBvAHIAbQAoAGIAaQBnAF8AaQBuAHQAXwBiACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAaQBnAG4AXwBhACwAIABCAGkAZwBJAG4AdAAuAFMAaQBnAG4AKABuAG8AcgBtAF8AYQApACwAXABuACAAIAAgACAAIAAgACAAIABzAGkAZwBuAF8AYgAsACAAQgBpAGcAaQBuAHQALgBTAGkAZwBuACgAbgBvAHIAbQBfAGIAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAHMAaQBnAG4AXwBhACAAPAA+ACAAcwBpAGcAbgBfAGIALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUwBJAEcATgAoAHMAaQBnAG4AXwBhACAALQAgAHMAaQBnAG4AXwBiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgAcwBpAGcAbgBfAGEAIAA9ACAAMAAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgADAALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABlAG4AXwBhACwAIABMAEUATgAoAG4AbwByAG0AXwBhACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAZQBuAF8AYgAsACAATABFAE4AKABuAG8AcgBtAF8AYgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEkARgAoAGwAZQBuAF8AYQAgADwAPgAgAGwAZQBuAF8AYgAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABTAEkARwBOACgAbABlAG4AXwBhACAALQAgAGwAZQBuAF8AYgApACAAKgAgAHMAaQBnAG4AXwBhACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAawAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwBhAGYAZQBLACgAXAAiAEEARABEAFwAIgApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBhACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBTAHAAbABpAHQAKABCAGkAZwBJAG4AdAAuAEEAYgBzACgAbgBvAHIAbQBfAGEAKQAsACAAawApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYgAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwBwAGwAaQB0ACgAQgBpAGcASQBuAHQALgBBAGIAcwAoAG4AbwByAG0AXwBiACkALAAgAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAG0AYQBnAF8AYwBvAG0AcABhAHIAaQBzAG8AbgAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBDAG8AbQBwAGEAcgBlACgAbABpAG0AYgBzAF8AYQAsACAAbABpAG0AYgBzAF8AYgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbQBhAGcAXwBjAG8AbQBwAGEAcgBpAHMAbwBuACAAKgAgAHMAaQBnAG4AXwBhAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvAC8AIAAgACAAIAAgACAAIAAgACAAIAAtACAAQQBkAGQAaQB0AGkAbwBuACAAJgAgAFMAdQBiAHQAcgBhAGMAdABpAG8AbgAgAC0AIAAgACAAIAAgACAAIABcAFwAXABcAFwAbgBcAG4ALwAqACoAXABuACAAKgAgAEEAZABkAHMAIAB0AHcAbwAgAEIAaQBnAEkAbgB0ACAAcwB0AHIAaQBuAGcAcwAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGIAaQBnAF8AaQBuAHQAXwBhACAAVABoAGUAIABmAGkAcgBzAHQAIABCAGkAZwBJAG4AdAAgAHMAdAByAGkAbgBnAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAYgBpAGcAXwBpAG4AdABfAGIAIABUAGgAZQAgAHMAZQBjAG8AbgBkACAAQgBpAGcASQBuAHQAIABzAHQAcgBpAG4AZwAuAFwAbgAgACoALwBcAG4AQQBkAGQAIAA9ACAATABBAE0AQgBEAEEAKABiAGkAZwBfAGkAbgB0AF8AYQAsACAAYgBpAGcAXwBpAG4AdABfAGIALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbgBvAHIAbQBfAGEALAAgAE4AbwByAG0AKABiAGkAZwBfAGkAbgB0AF8AYQApACwAXABuACAAIAAgACAAIAAgACAAIABuAG8AcgBtAF8AYgAsACAATgBvAHIAbQAoAGIAaQBnAF8AaQBuAHQAXwBiACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAaQBnAG4AXwBhACwAIABCAGkAZwBpAG4AdAAuAFMAaQBnAG4AKABuAG8AcgBtAF8AYQApACwAXABuACAAIAAgACAAIAAgACAAIABzAGkAZwBuAF8AYgAsACAAQgBpAGcASQBuAHQALgBTAGkAZwBuACgAbgBvAHIAbQBfAGIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIABrACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBTAGEAZgBlAEsAKABcACIAQQBEAEQAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGEALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFMAcABsAGkAdAAoAEIAaQBnAEkAbgB0AC4AQQBiAHMAKABuAG8AcgBtAF8AYQApACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGIALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFMAcABsAGkAdAAoAEIAaQBnAEkAbgB0AC4AQQBiAHMAKABuAG8AcgBtAF8AYgApACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAcgBvAHUAdABlAGQALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAEEAZABkAFMAdQBiAFIAbwB1AHQAZQByACgAbABpAG0AYgBzAF8AYQAsACAAbABpAG0AYgBzAF8AYgAsACAAcwBpAGcAbgBfAGEALAAgAHMAaQBnAG4AXwBiACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgAGYAaQBuAGEAbABfAHMAaQBnAG4ALAAgAEMASABPAE8AUwBFAFIATwBXAFMAKAByAG8AdQB0AGUAZAAsACAALQAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAGYAaQBuAGEAbABfAGwAaQBtAGIAcwAsACAARABSAE8AUAAoAHIAbwB1AHQAZQBkACwAIAAtADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIABtAGUAcgBnAGUAZAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4ATQBlAHIAZwBlACgAZgBpAG4AYQBsAF8AbABpAG0AYgBzACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAZgBpAG4AYQBsAF8AcwBpAGcAbgAgAD0AIAAtADEALAAgAFwAIgAtAFwAIgAgACYAIABtAGUAcgBnAGUAZAAsACAAbQBlAHIAZwBlAGQAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAAUwB1AGIAdAByAGEAYwB0AHMAIAB0AGgAZQAgAHMAZQBjAG8AbgBkACAAQgBpAGcASQBuAHQAIABzAHQAcgBpAG4AZwAgAGYAcgBvAG0AIAB0AGgAZQAgAGYAaQByAHMAdAAgACgAQQAgAC0AIABCACkALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABiAGkAZwBfAGkAbgB0AF8AYQAgAFQAaABlACAAbQBpAG4AdQBlAG4AZAAgAEIAaQBnAEkAbgB0ACAAcwB0AHIAaQBuAGcALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABiAGkAZwBfAGkAbgB0AF8AYgAgAFQAaABlACAAcwB1AGIAdAByAGEAaABlAG4AZAAgAEIAaQBnAEkAbgB0ACAAcwB0AHIAaQBuAGcALgBcAG4AIAAqAC8AXABuAFMAdQBiACAAPQAgAEwAQQBNAEIARABBACgAYgBpAGcAXwBpAG4AdABfAGEALAAgAGIAaQBnAF8AaQBuAHQAXwBiACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG4AbwByAG0AXwBiACwAIABOAG8AcgBtACgAYgBpAGcAXwBpAG4AdABfAGIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABJAG4AdgBlAHIAdAAgAHQAaABlACAAcwBpAGcAbgAgAG8AZgAgAEIAIABhAHQAIAB0AGgAZQAgAHQAZQB4AHQAIABsAGUAdgBlAGwAXABuACAAIAAgACAAIAAgACAAIABpAG4AdgBfAGIALAAgAEkARgAoAG4AbwByAG0AXwBiACAAPQAgAFwAIgAwAFwAIgAsACAAXAAiADAAXAAiACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgATABFAEYAVAAoAG4AbwByAG0AXwBiACkAIAA9ACAAXAAiAC0AXAAiACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEkARAAoAG4AbwByAG0AXwBiACwAIAAyACwAIABMAEUATgAoAG4AbwByAG0AXwBiACkAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAC0AXAAiACAAJgAgAG4AbwByAG0AXwBiAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABQAGEAcwBzACAAdABvACAAQQBkAGQAXABuACAAIAAgACAAIAAgACAAIABBAGQAZAAoAGIAaQBnAF8AaQBuAHQAXwBhACwAIABpAG4AdgBfAGIAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAAUwB1AG0AcwAgAGEAbgAgAGEAcgByAGEAeQAgAG8AcgAgAHIAYQBuAGcAZQAgAG8AZgAgAEIAaQBnAEkAbgB0ACAAcwB0AHIAaQBuAGcAcwAgAHYAaQBhACAAdgBlAGMAdABvAHIAaQB6AGUAZAAgAGcAcgBvAHUAcAAgAG0AYQB0AHIAaQBjAGUAcwAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAHIAYQBuAGcAZQAgAEEAIABjAG8AbgB0AGkAZwB1AG8AdQBzACAAcgBhAG4AZwBlACAAbwByACAAYQByAHIAYQB5ACAAbwBmACAAQgBpAGcASQBuAHQAIABzAHQAcgBpAG4AZwBzAC4AXABuACAAKgAvAFwAbgBTAHUAbQAgAD0AIABMAEEATQBCAEQAQQAoAHIAYQBuAGcAZQAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABmAGwAYQB0ACwAIABUAE8AUgBPAFcAKAByAGEAbgBnAGUALAAgADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABPAFIAKABJAFMARQBSAFIATwBSACgAZgBsAGEAdAApACwAIABDAE8ATABVAE0ATgBTACgAZgBsAGEAdAApACAAPQAgADAAKQAsACAAXAAiADAAXAAiACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbgBvAHIAbQBzACwAIABNAEEAUAAoAGYAbABhAHQALAAgAEwAQQBNAEIARABBACgAeAAsACAATgBvAHIAbQAoAHgAKQApACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABzAGkAZwBuAHMALAAgAE0AQQBQACgATABFAEYAVAAoAG4AbwByAG0AcwApACwAIABMAEEATQBCAEQAQQAoAHgALAAgAEkARgAoAHgAIAA9ACAAXAAiADAAXAAiACwAIAAwACwAIABpAGYAKAB4ACAAPQAgAFwAIgAtAFwAIgAsACAALQAxACwAIAAxACkAKQApACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABhAGIAcwBfAG4AbwByAG0AcwAsACAATQBBAFAAKABuAG8AcgBtAHMALAAgAHMAaQBnAG4AcwAsACAATABBAE0AQgBEAEEAKAB4ACwAIABzAGkAZwBuACwAIABJAEYAKABzAGkAZwBuACAAPQAgAC0AMQAsACAATQBJAEQAKAB4ACwAIAAyACwAIABMAEUATgAoAHgAKQAtADEAKQAsACAAeAApACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHAAbwBzAF8AcwB0AHIAcwAsACAARgBJAEwAVABFAFIAKABhAGIAcwBfAG4AbwByAG0AcwAsACAAcwBpAGcAbgBzACAAPQAgADEALAAgAHsAXAAiADAAXAAiAH0AKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAG4AZQBnAF8AcwB0AHIAcwAsACAARgBJAEwAVABFAFIAKABhAGIAcwBfAG4AbwByAG0AcwAsACAAcwBpAGcAbgBzACAAPQAgAC0AMQAsACAAewBcACIAMABcACIAfQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAdQBuAGkAZgBpAGUAZABfAGsALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFMAYQBmAGUASwAoAFwAIgBBAEQARABcACIALAAgAEMATwBMAFUATQBOAFMAKABmAGwAYQB0ACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHAAbwBzAF8AbABpAG0AYgBzACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAE0AYQB0AHIAaQB4AFMAdQBtACgAcABvAHMAXwBzAHQAcgBzACwAIAB1AG4AaQBmAGkAZQBkAF8AawApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbgBlAGcAXwBsAGkAbQBiAHMALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFUATQBhAHQAcgBpAHgAUwB1AG0AKABuAGUAZwBfAHMAdAByAHMALAAgAHUAbgBpAGYAaQBlAGQAXwBrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAByAG8AdQB0AGUAZAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AQQBkAGQAUwB1AGIAUgBvAHUAdABlAHIAKABwAG8AcwBfAGwAaQBtAGIAcwAsACAAbgBlAGcAXwBsAGkAbQBiAHMALAAgADEALAAgAC0AMQAsACAAdQBuAGkAZgBpAGUAZABfAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGYAaQBuAGEAbABfAHMAaQBnAG4ALAAgAEMASABPAE8AUwBFAFIATwBXAFMAKAByAG8AdQB0AGUAZAAsACAALQAxACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABmAGkAbgBhAGwAXwBsAGkAbQBiAHMALAAgAEQAUgBPAFAAKAByAG8AdQB0AGUAZAAsACAALQAxACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABtAGUAcgBnAGUAZAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4ATQBlAHIAZwBlACgAZgBpAG4AYQBsAF8AbABpAG0AYgBzACwAIAB1AG4AaQBmAGkAZQBkAF8AawApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgAZgBpAG4AYQBsAF8AcwBpAGcAbgAgAD0AIAAtADEALAAgAFwAIgAtAFwAIgAgACYAIABtAGUAcgBnAGUAZAAsACAAbQBlAHIAZwBlAGQAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAE0AdQBsAHQAaQBwAGwAaQBlAHMAIAB0AHcAbwAgAEIAaQBnAEkAbgB0ACAAcwB0AHIAaQBuAGcAcwAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGIAaQBnAF8AaQBuAHQAXwBhACAAVABoAGUAIABmAGkAcgBzAHQAIABCAGkAZwBJAG4AdAAgAHMAdAByAGkAbgBnAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAYgBpAGcAXwBpAG4AdABfAGIAIABUAGgAZQAgAHMAZQBjAG8AbgBkACAAQgBpAGcASQBuAHQAIABzAHQAcgBpAG4AZwAuAFwAbgAgACoALwBcAG4ATQB1AGwAIAA9ACAATABBAE0AQgBEAEEAKABiAGkAZwBfAGkAbgB0AF8AYQAsACAAYgBpAGcAXwBpAG4AdABfAGIALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbgBvAHIAbQBfAGEALAAgAE4AbwByAG0AKABiAGkAZwBfAGkAbgB0AF8AYQApACwAXABuACAAIAAgACAAIAAgACAAIABuAG8AcgBtAF8AYgAsACAATgBvAHIAbQAoAGIAaQBnAF8AaQBuAHQAXwBiACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAaQBnAG4AXwBhACwAIABCAGkAZwBJAG4AdAAuAFMAaQBnAG4AKABuAG8AcgBtAF8AYQApACwAXABuACAAIAAgACAAIAAgACAAIABzAGkAZwBuAF8AYgAsACAAQgBpAGcASQBuAHQALgBTAGkAZwBuACgAbgBvAHIAbQBfAGIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABlAG4AXwBhACwAIABMAEUATgAoAG4AbwByAG0AXwBhACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAZQBuAF8AYgAsACAATABFAE4AKABuAG8AcgBtAF8AYgApACwAXABuACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgAC8ALwAgAFMAaABvAHIAdAAtAGMAaQByAGMAdQBpAHQAOgAgADAAIABtAHUAbAB0AGkAcABsAGkAZQBkACAAYgB5ACAAYQBuAHkAdABoAGkAbgBnACAAaQBzACAAMABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAE8AUgAoAHMAaQBnAG4AXwBhACAAPQAgADAALAAgAHMAaQBnAG4AXwBiACAAPQAgADAAKQAsACAAXAAiADAAXAAiACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABsAGUAbgBfAGEAIAArACAAbABlAG4AXwBiACAAPgAgADMAMgA3ADYANgAsACAAIwBOAFUATQAhACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAAQwBhAGwAYwB1AGwAYQB0AGUAIABkAHkAbgBhAG0AaQBjACAAcwBhAGYAZQAgAEsAIABiAGEAcwBlAGQAIABvAG4AIAB0AGgAZQAgAHMAaABvAHIAdABlAHMAdAAgAHMAdAByAGkAbgBnAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGsALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFMAYQBmAGUASwAoAFwAIgBNAFUATABcACIALAAgAE0ASQBOACgAbABlAG4AXwBhACwAIABsAGUAbgBfAGIAKQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAAUwBwAGwAaQB0ACAAYQBiAHMAbwBsAHUAdABlACAAcwB0AHIAaQBuAGcAcwAgAGkAbgB0AG8AIABsAGkAdAB0AGwAZQAtAGUAbgBkAGkAYQBuACAAYQByAHIAYQB5AHMAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYQAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwBwAGwAaQB0ACgAQgBpAGcASQBuAHQALgBBAGIAcwAoAG4AbwByAG0AXwBhACkALAAgAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGIALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFMAcABsAGkAdAAoAEIAaQBnAEkAbgB0AC4AQQBiAHMAKABuAG8AcgBtAF8AYgApACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIABDAGEAbABjAHUAbABhAHQAZQAgAG0AYQBnAG4AaQB0AHUAZABlACAAYQBuAGQAIAByAGUAcwBvAGwAdgBlACAAcwBpAGcAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABmAGkAbgBhAGwAXwBsAGkAbQBiAHMALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFUATQB1AGwAKABsAGkAbQBiAHMAXwBhACwAIABsAGkAbQBiAHMAXwBiACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABmAGkAbgBhAGwAXwBzAGkAZwBuACwAIABzAGkAZwBuAF8AYQAgACoAIABzAGkAZwBuAF8AYgAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAG0AZQByAGcAZQBkACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBNAGUAcgBnAGUAKABmAGkAbgBhAGwAXwBsAGkAbQBiAHMALAAgAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEkARgAoAGYAaQBuAGEAbABfAHMAaQBnAG4AIAA9ACAALQAxACwAIABcACIALQBcACIAIAAmACAAbQBlAHIAZwBlAGQALAAgAG0AZQByAGcAZQBkACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAApACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFsAVgBPAEwAQQBUAEkATABFAF0AIABHAGUAbgBlAHIAYQB0AGUAcwAgAGEAIABkAHkAbgBhAG0AaQBjACAAYQByAHIAYQB5ACAAbwBmACAAaQBuAHQAZQBnAGUAcgBzACAAYQBzACAAdABlAHgAdAAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAFsAbgB1AG0AXwByAG8AdwBzAF0AIABhAHIAcgBhAHkAIABoAGUAaQBnAGgAdAAsACAAZABlAGYAYQB1AGwAdAAgADEALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABbAG4AdQBtAF8AYwBvAGwAcwBdACAAYQByAHIAYQB5ACAAdwBpAGQAdABoACwAIABkAGUAZgBhAHUAbAB0ACAAMQAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAFsAbQBpAG4AXwBkAGkAZwBpAHQAcwBdACAAbQBpAG4AaQBtAHUAbQAgAG4AdQBtAGIAZQByACAAbwBmACAAZABpAGcAaQB0AHMALAAgAGQAZQBmAGEAdQBsAHQAIAAxADYAIAAoAG0AaQBuACAAMQAgAGQAaQBnAGkAdAApAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAFsAbQBhAHgAXwBkAGkAZwBpAHQAcwBdACAAbQBhAHgAaQBtAHUAbQAgAG4AdQBtAGIAZQByACAAbwBmACAAZABpAGcAaQB0AHMALAAgAGQAZQBmAGEAdQBsAHQAIAA1ADAAIAAoAG0AYQB4ACAAMwAyACwANwA2ADcAIABjAGgAYQByAHMALAAgAGkAbgBjAGwAdQBkAGkAbgBnACAAcwBpAGcAbgApAFwAbgAgACoALwBcAG4AUgBhAG4AZABCAGkAZwBJAG4AdABBAHIAcgBhAHkAIAA9ACAATABBAE0AQgBEAEEAKABbAG4AdQBtAF8AcgBvAHcAcwBdACwAIABbAG4AdQBtAF8AYwBvAGwAcwBdACwAIABbAG0AaQBuAF8AZABpAGcAaQB0AHMAXQAsACAAWwBtAGEAeABfAGQAaQBnAGkAdABzAF0ALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbgBfAHIAbwB3AHMALAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAbgB1AG0AXwByAG8AdwBzACkALAAgADEALAAgAG4AdQBtAF8AcgBvAHcAcwApACwAXABuACAAIAAgACAAIAAgACAAIABuAF8AYwBvAGwAcwAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABuAHUAbQBfAGMAbwBsAHMAKQAsACAAMQAsACAAbgB1AG0AXwBjAG8AbABzACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAbQBpAG4AXwBsAGUAbgAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABtAGkAbgBfAGQAaQBnAGkAdABzACkALAAgADEANgAsACAATQBJAE4AKAAzADIANwA2ADcALAAgAE0AQQBYACgAMQAsACAAbQBpAG4AXwBkAGkAZwBpAHQAcwApACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHgAXwBsAGUAbgAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABtAGEAeABfAGQAaQBnAGkAdABzACkALAAgADUAMAAsACAATQBBAFgAKAAxACwAIABNAEkATgAoADMAMgA3ADYANgAsACAAbQBhAHgAXwBkAGkAZwBpAHQAcwApACkAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAE0AQQBQACgAUgBBAE4ARABBAFIAUgBBAFkAKABuAF8AcgBvAHcAcwAsACAAbgBfAGMAbwBsAHMALAAgAG0AaQBuAF8AbABlAG4ALAAgAG0AYQB4AF8AbABlAG4ALAAgAFQAUgBVAEUAKQAsACAATABBAE0AQgBEAEEAKABsAGUAbgBnAHQAaAAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHMAaQBnAG4ALAAgAEMASABPAE8AUwBFACgAUgBBAE4ARABCAEUAVABXAEUARQBOACgAMQAsACAAMgApACwAIABcACIAXAAiACwAIABcACIALQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGQAaQBnAGkAdABzACwAIABDAE8ATgBDAEEAVAAoAFIAQQBOAEQAQQBSAFIAQQBZACgAMQAsACAAbABlAG4AZwB0AGgALAAgADAALAAgADkALAAgAFQAUgBVAEUAKQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcwBpAGcAbgAgACYAIABSAEUARwBFAFgAUgBFAFAATABBAEMARQAoAGQAaQBnAGkAdABzACwAIABcACIAXgAwACoAXAAiACwAIABcACIAXAAiACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAApACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAEQAaQB2AGkAZABlAHMAIAB0AGgAZQAgAGYAaQByAHMAdAAgAEIAaQBnAEkAbgB0ACAAYgB5ACAAdABoAGUAIABzAGUAYwBvAG4AZAAgACgAQQAgAC8AIABCACkALgAgAFwAbgAgACoAIABSAGUAdAB1AHIAbgBzACAAdABoAGUAIABxAHUAbwB0AGkAZQBuAHQAIABhAG4AZAAgAG0AbwBkAHUAbAB1AHMAIABpAG4AIAByAG8AdwBzACAAMQAgAGEAbgBkACAAMgAsACAAcgBlAHMAcABlAGMAdABpAHYAZQBsAHkALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABiAGkAZwBfAGkAbgB0AF8AYQAgAFQAaABlACAAZABpAHYAaQBkAGUAbgBkACAAQgBpAGcASQBuAHQAIABzAHQAcgBpAG4AZwAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGIAaQBnAF8AaQBuAHQAXwBiACAAVABoAGUAIABkAGkAdgBpAHMAbwByACAAQgBpAGcASQBuAHQAIABzAHQAcgBpAG4AZwAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAFsAdQBzAGUAXwBmAGwAbwBvAHIAXQAgAE8AcAB0AGkAbwBuAGEAbAAgAGIAbwBvAGwAZQBhAG4ALgAgAFQAUgBVAEUAIABmAG8AcgAgAFAAeQB0AGgAbwBuAC0AcwB0AHkAbABlACAARgBsAG8AbwByACAAZABpAHYAaQBzAGkAbwBuACwAIABGAEEATABTAEUAIABmAG8AcgAgAFQAcgB1AG4AYwBhAHQAZQBkAC4AIABEAGUAZgBhAHUAbAB0AHMAIAB0AG8AIABGAEEATABTAEUALgBcAG4AIAAqAC8AXABuAEQAaQB2AE0AbwBkACAAPQAgAEwAQQBNAEIARABBACgAYgBpAGcAXwBpAG4AdABfAGEALAAgAGIAaQBnAF8AaQBuAHQAXwBiACwAIABbAHUAcwBlAF8AZgBsAG8AbwByAF0ALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbgBvAHIAbQBfAGEALAAgAE4AbwByAG0AKABiAGkAZwBfAGkAbgB0AF8AYQApACwAXABuACAAIAAgACAAIAAgACAAIABuAG8AcgBtAF8AYgAsACAATgBvAHIAbQAoAGIAaQBnAF8AaQBuAHQAXwBiACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAaQBnAG4AXwBhACwAIABCAGkAZwBJAG4AdAAuAFMAaQBnAG4AKABuAG8AcgBtAF8AYQApACwAXABuACAAIAAgACAAIAAgACAAIABzAGkAZwBuAF8AYgAsACAAQgBpAGcASQBuAHQALgBTAGkAZwBuACgAbgBvAHIAbQBfAGIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAaQBzAF8AZgBsAG8AbwByACwAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAHUAcwBlAF8AZgBsAG8AbwByACkALAAgAEYAQQBMAFMARQAsACAAdQBzAGUAXwBmAGwAbwBvAHIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABzAGkAZwBuAF8AYgAgAD0AIAAwACwAIAAjAEQASQBWAC8AMAAhACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEkARgAoAHMAaQBnAG4AXwBhACAAPQAgADAALAAgAHsAXAAiADAAXAAiADsAXAAiADAAXAAiAH0ALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAawAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwBhAGYAZQBLACgAXAAiAEQASQBWAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBhACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBTAHAAbABpAHQAKABCAGkAZwBJAG4AdAAuAEEAYgBzACgAbgBvAHIAbQBfAGEAKQAsACAAawApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBiACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBTAHAAbABpAHQAKABCAGkAZwBJAG4AdAAuAEEAYgBzACgAbgBvAHIAbQBfAGIAKQAsACAAawApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHAAYQBjAGsAZQBkAF8AcgBlAHMAdQBsAHQALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAEQAaQB2AFIAbwB1AHQAZQByACgAbABpAG0AYgBzAF8AYQAsACAAbABpAG0AYgBzAF8AYgAsACAAawApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAEUAeAB0AHIAYQBjAHQAIABSAGUAbQBhAGkAbgBkAGUAcgAgAGEAbgBkACAAUQB1AG8AdABpAGUAbgB0ACAAYQByAHIAYQB5AHMAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGUAbgBfAHIALAAgAEkATgBEAEUAWAAoAHAAYQBjAGsAZQBkAF8AcgBlAHMAdQBsAHQALAAgADEALAAgADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcgBlAG0AXwBsAGkAbQBiAHMALAAgAEMASABPAE8AUwBFAFIATwBXAFMAKABwAGEAYwBrAGUAZABfAHIAZQBzAHUAbAB0ACwAIABTAEUAUQBVAEUATgBDAEUAKABsAGUAbgBfAHIALAAgADEALAAgADIAKQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABxAHUAbwB0AF8AbABpAG0AYgBzACwAIABEAFIATwBQACgAcABhAGMAawBlAGQAXwByAGUAcwB1AGwAdAAsACAAbABlAG4AXwByACAAKwAgADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIABSAGUAcwBvAGwAdgBlACAAVAByAHUAbgBjAGEAdABlAGQAIABzAGkAZwBuAHMAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABmAGkAbgBhAGwAXwBzAGkAZwBuACwAIABzAGkAZwBuAF8AYQAgACoAIABzAGkAZwBuAF8AYgAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbQBlAHIAZwBlAGQAXwBxACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBNAGUAcgBnAGUAKABxAHUAbwB0AF8AbABpAG0AYgBzACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAG0AZQByAGcAZQBkAF8AcgAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4ATQBlAHIAZwBlACgAcgBlAG0AXwBsAGkAbQBiAHMALAAgAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAB0AHIAdQBuAGMAXwBxACwAIABJAEYAKABBAE4ARAAoAGYAaQBuAGEAbABfAHMAaQBnAG4AIAA9ACAALQAxACwAIABtAGUAcgBnAGUAZABfAHEAIAA8AD4AIABcACIAMABcACIAKQAgACwAIABcACIALQBcACIAIAAmACAAbQBlAHIAZwBlAGQAXwBxACwAIABtAGUAcgBnAGUAZABfAHEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAdAByAHUAbgBjAF8AcgAsACAASQBGACgAYQBuAGQAKABzAGkAZwBuAF8AYQAgAD0AIAAtADEALAAgAG0AZQByAGcAZQBkAF8AcgAgADwAPgAgAFwAIgAwAFwAIgApACwAIABcACIALQBcACIAIAAmACAAbQBlAHIAZwBlAGQAXwByACwAIABtAGUAcgBnAGUAZABfAHIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIABGAGwAbwBvAHIAIABDAG8AcgByAGUAYwB0AGkAbwBuADoAIABUAHIAaQBnAGcAZQByACAATwBOAEwAWQAgAGkAZgAgAGYAbABvAG8AcgAgAGkAcwAgAHIAZQBxAHUAZQBzAHQAZQBkACwAIABzAGkAZwBuAHMAIABkAGkAZgBmAGUAcgAsACAAYQBuAGQAIAByAGUAbQBhAGkAbgBkAGUAcgAgAGkAcwAgAG4AbwBuAC0AegBlAHIAbwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAG4AZQBlAGQAcwBfAGMAbwByAHIAZQBjAHQAaQBvAG4ALAAgAEEATgBEACgAaQBzAF8AZgBsAG8AbwByACwAIABmAGkAbgBhAGwAXwBzAGkAZwBuACAAPQAgAC0AMQAsACAAbQBlAHIAZwBlAGQAXwByACAAPAA+ACAAXAAiADAAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAZgBpAG4AYQBsAF8AcQAsACAASQBGACgAbgBlAGUAZABzAF8AYwBvAHIAcgBlAGMAdABpAG8AbgAsACAAUwB1AGIAKAB0AHIAdQBuAGMAXwBxACwAIABcACIAMQBcACIAKQAsACAAdAByAHUAbgBjAF8AcQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABmAGkAbgBhAGwAXwByACwAIABJAEYAKABuAGUAZQBkAHMAXwBjAG8AcgByAGUAYwB0AGkAbwBuACwAIABBAGQAZAAoAHQAcgB1AG4AYwBfAHIALAAgAG4AbwByAG0AXwBiACkALAAgAHQAcgB1AG4AYwBfAHIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABWAFMAVABBAEMASwAoAGYAaQBuAGEAbABfAHEALAAgAGYAaQBuAGEAbABfAHIAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAARABpAHYAaQBkAGUAcwAgAHQAaABlACAAZgBpAHIAcwB0ACAAQgBpAGcASQBuAHQAIABiAHkAIAB0AGgAZQAgAHMAZQBjAG8AbgBkACAAKABBACAALwAgAEIAKQAuACAAXABuACAAKgAgAEAAcABhAHIAYQBtACAAYgBpAGcAXwBpAG4AdABfAGEAIABUAGgAZQAgAGQAaQB2AGkAZABlAG4AZAAgAEIAaQBnAEkAbgB0ACAAcwB0AHIAaQBuAGcALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABiAGkAZwBfAGkAbgB0AF8AYgAgAFQAaABlACAAZABpAHYAaQBzAG8AcgAgAEIAaQBnAEkAbgB0ACAAcwB0AHIAaQBuAGcALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABbAHUAcwBlAF8AZgBsAG8AbwByAF0AIABPAHAAdABpAG8AbgBhAGwAIABiAG8AbwBsAGUAYQBuAC4AIABUAFIAVQBFACAAZgBvAHIAIABQAHkAdABoAG8AbgAtAHMAdAB5AGwAZQAgAEYAbABvAG8AcgAgAGQAaQB2AGkAcwBpAG8AbgAuACAARABlAGYAYQB1AGwAdABzACAAdABvACAARgBBAEwAUwBFAC4AXABuACAAKgAvAFwAbgBEAGkAdgAgAD0AIABMAEEATQBCAEQAQQAoAGIAaQBnAF8AaQBuAHQAXwBhACwAIABiAGkAZwBfAGkAbgB0AF8AYgAsACAAWwB1AHMAZQBfAGYAbABvAG8AcgBdACwAXABuACAAIAAgACAASQBOAEQARQBYACgARABpAHYATQBvAGQAKABiAGkAZwBfAGkAbgB0AF8AYQAsACAAYgBpAGcAXwBpAG4AdABfAGIALAAgAHUAcwBlAF8AZgBsAG8AbwByACkALAAgADEALAAgADEAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAEMAbwBtAHAAdQB0AGUAcwAgAHQAaABlACAAcgBlAG0AYQBpAG4AZABlAHIAIABvAGYAIABBACAALwAgAEIALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABiAGkAZwBfAGkAbgB0AF8AYQAgAFQAaABlACAAZABpAHYAaQBkAGUAbgBkACAAQgBpAGcASQBuAHQAIABzAHQAcgBpAG4AZwAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGIAaQBnAF8AaQBuAHQAXwBiACAAVABoAGUAIABkAGkAdgBpAHMAbwByACAAQgBpAGcASQBuAHQAIABzAHQAcgBpAG4AZwAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAFsAdQBzAGUAXwBmAGwAbwBvAHIAXQAgAE8AcAB0AGkAbwBuAGEAbAAgAGIAbwBvAGwAZQBhAG4ALgAgAFQAUgBVAEUAIABmAG8AcgAgAFAAeQB0AGgAbwBuAC0AcwB0AHkAbABlACAATQBvAGQAdQBsAG8ALgAgAEQAZQBmAGEAdQBsAHQAcwAgAHQAbwAgAEYAQQBMAFMARQAuAFwAbgAgACoALwBcAG4ATQBvAGQAIAA9ACAATABBAE0AQgBEAEEAKABiAGkAZwBfAGkAbgB0AF8AYQAsACAAYgBpAGcAXwBpAG4AdABfAGIALAAgAFsAdQBzAGUAXwBmAGwAbwBvAHIAXQAsAFwAbgAgACAAIAAgAEkATgBEAEUAWAAoAEQAaQB2AE0AbwBkACgAYgBpAGcAXwBpAG4AdABfAGEALAAgAGIAaQBnAF8AaQBuAHQAXwBiACwAIAB1AHMAZQBfAGYAbABvAG8AcgApACwAIAAyACwAIAAxACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABSAGEAaQBzAGUAcwAgAGEAIABCAGkAZwBJAG4AdAAgAGIAYQBzAGUAIAB0AG8AIAB0AGgAZQAgAHAAbwB3AGUAcgAgAG8AZgAgAGEAIABCAGkAZwBJAG4AdAAgAGUAeABwAG8AbgBlAG4AdAAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGIAYQBzAGUAIABUAGgAZQAgAGIAYQBzAGUAIABCAGkAZwBJAG4AdAAgAHMAdAByAGkAbgBnAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAZQB4AHAAbwBuAGUAbgB0ACAAVABoAGUAIABlAHgAcABvAG4AZQBuAHQAIABCAGkAZwBJAG4AdAAgAHMAdAByAGkAbgBnAC4AXABuACAAKgAvAFwAbgBQAG8AdwAgAD0AIABMAEEATQBCAEQAQQAoAGIAYQBzAGUALAAgAGUAeABwAG8AbgBlAG4AdAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABuAG8AcgBtAF8AYgBhAHMAZQAsACAATgBvAHIAbQAoAGIAYQBzAGUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbgBvAHIAbQBfAGUAeABwACwAIABOAG8AcgBtACgAZQB4AHAAbwBuAGUAbgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAaQBnAG4AXwBiAGEAcwBlACwAIABCAGkAZwBJAG4AdAAuAFMAaQBnAG4AKABuAG8AcgBtAF8AYgBhAHMAZQApACwAXABuACAAIAAgACAAIAAgACAAIABzAGkAZwBuAF8AZQB4AHAALAAgAEIAaQBnAEkAbgB0AC4AUwBpAGcAbgAoAG4AbwByAG0AXwBlAHgAcAApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAYQBiAHMAXwBiAGEAcwBlACwAIABCAGkAZwBJAG4AdAAuAEEAYgBzACgAbgBvAHIAbQBfAGIAYQBzAGUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAYQBiAHMAXwBlAHgAcAAsACAAQgBpAGcASQBuAHQALgBBAGIAcwAoAG4AbwByAG0AXwBlAHgAcAApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAaQBzAF8AZQB4AHAAXwBlAHYAZQBuACwAIABJAFMARQBWAEUATgAoAFYAQQBMAFUARQAoAFIASQBHAEgAVAAoAG4AbwByAG0AXwBlAHgAcAAsACAAMQApACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAG4AYQBsAF8AcwBpAGcAbgAsACAASQBGACgAcwBpAGcAbgBfAGIAYQBzAGUAIAA9ACAALQAxACwAIABJAEYAKABpAHMAXwBlAHgAcABfAGUAdgBlAG4ALAAgADEALAAgAC0AMQApACwAIABzAGkAZwBuAF8AYgBhAHMAZQApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAALwAvACAASABhAG4AZABsAGUAIABtAGEAdABoAGUAbQBhAHQAaQBjAGEAbAAgAGIAbwB1AG4AZABhAHIAaQBlAHMAIABhAG4AZAAgAGIAYQBzAGUAIABsAGkAbQBpAHQAcwBcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAGEAYgBzAF8AYgBhAHMAZQAgAD0AIABcACIAMABcACIALAAgAEkARgAoAG4AbwByAG0AXwBlAHgAcAAgAD0AIABcACIAMABcACIALAAgACMATgBVAE0AIQAsACAAXAAiADAAXAAiACkALAAgAC8ALwAgADAAXgAwACAAaQBzACAAdQBuAGQAZQBmAGkAbgBlAGQAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABhAGIAcwBfAGIAYQBzAGUAIAA9ACAAXAAiADEAXAAiACwAIABJAEYAKABmAGkAbgBhAGwAXwBzAGkAZwBuACAAPQAgAC0AMQAsACAAXAAiAC0AMQBcACIALAAgAFwAIgAxAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABzAGkAZwBuAF8AZQB4AHAAIAA9ACAALQAxACwAIABcACIAMABcACIALAAgAC8ALwAgAEkAbgB0AGUAZwBlAHIAIAB0AHIAdQBuAGMAYQB0AGkAbwBuADoAIABuAGUAZwBhAHQAaQB2AGUAIABlAHgAcABvAG4AZQBuAHQAcwAgAHkAaQBlAGwAZAAgADAAIABmAG8AcgAgAGIAYQBzAGUAcwAgAD4APQAgADIAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABuAG8AcgBtAF8AZQB4AHAAIAA9ACAAXAAiADAAXAAiACwAIABcACIAMQBcACIALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABSAGUAcwB1AGwAdABzACAAZgByAG8AbQAgAGUAeABwAG8AbgBlAG4AdABzACAAZwByAGUAYQB0AGUAcgAgAHQAaABhAG4AIAA2ACAAZABpAGcAaQB0AHMAIABjAGEAbgBuAG8AdAAgAGIAZQAgAGQAaQBzAHAAbABhAHkAZQBkAC4AXABuACAAIAAgACAAIAAgACAAIABJAEYAKABMAEUATgAoAG4AbwByAG0AXwBlAHgAcAApACAAPgAgADYALAAgACMATgBVAE0AIQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAG4AdQBtAF8AZQB4AHAALAAgAFYAQQBMAFUARQAoAG4AbwByAG0AXwBlAHgAcAApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAAQQBwAHAAcgBvAHgAaQBtAGEAdABlACAAdABoAGUAIABmAGkAbgBhAGwAIABjAGgAYQByAGEAYwB0AGUAcgAgAGMAbwB1AG4AdAA6ACAAQgAgACoAIABMAG8AZwAxADAAKABBACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAYgBhAHMAZQBfAGwAbwBnADEAMAAsACAATABPAEcAMQAwACgAVgBBAEwAVQBFACgATABFAEYAVAAoAGEAYgBzAF8AYgBhAHMAZQAsACAAMQA0ACkAKQApACAAKwAgAE0AQQBYACgAMAAsACAATABFAE4AKABhAGIAcwBfAGIAYQBzAGUAKQAgAC0AIAAxADQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGEAcABwAHIAbwB4AF8AZABpAGcAaQB0AHMALAAgAG4AdQBtAF8AZQB4AHAAIAAqACAAYgBhAHMAZQBfAGwAbwBnADEAMAAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABhAHAAcAByAG8AeABfAGQAaQBnAGkAdABzACAAPgAgADMAMgA3ADYANgAsACAAIwBOAFUATQAhACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABrACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBTAGEAZgBlAEsAKABcACIATQBVAEwAXAAiACwAIABhAHAAcAByAG8AeABfAGQAaQBnAGkAdABzACAALwAgADIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBiAGEAcwBlACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBTAHAAbABpAHQAKABhAGIAcwBfAGIAYQBzAGUALAAgAGsAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAZgBpAG4AYQBsAF8AbABpAG0AYgBzACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAFAAbwB3ACgAbABpAG0AYgBzAF8AYgBhAHMAZQAsACAAbgBvAHIAbQBfAGUAeABwACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbQBlAHIAZwBlAGQALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAE0AZQByAGcAZQAoAGYAaQBuAGEAbABfAGwAaQBtAGIAcwAsACAAawApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABmAGkAbgBhAGwAXwBzAGkAZwBuACAAPQAgAC0AMQAsACAAXAAiAC0AXAAiACAAJgAgAG0AZQByAGcAZQBkACwAIABtAGUAcgBnAGUAZAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAKQApACkAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABDAGEAbABjAHUAbABhAHQAZQBzACAAdABoAGUAIABpAG4AdABlAGcAZQByACAAcwBxAHUAYQByAGUAIAByAG8AbwB0ACAAKABmAGwAbwBvAHIAKQAgAG8AZgAgAGEAIABCAGkAZwBJAG4AdAAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGIAaQBnAF8AaQBuAHQAIABUAGgAZQAgAHIAYQBkAGkAYwBhAG4AZAAgAEIAaQBnAEkAbgB0ACAAcwB0AHIAaQBuAGcALgBcAG4AIAAqAC8AXABuAFMAcQByAHQAIAA9ACAATABBAE0AQgBEAEEAKABiAGkAZwBfAGkAbgB0ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG4AbwByAG0AXwBuACwAIABOAG8AcgBtACgAYgBpAGcAXwBpAG4AdAApACwAXABuACAAIAAgACAAIAAgACAAIABzAGkAZwBuAF8AbgAsACAAQgBpAGcASQBuAHQALgBTAGkAZwBuACgAbgBvAHIAbQBfAG4AKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAHMAaQBnAG4AXwBuACAAPQAgAC0AMQAsACAAIwBOAFUATQAhACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABuAG8AcgBtAF8AbgAgAD0AIABcACIAMABcACIALAAgAFwAIgAwAFwAIgAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAbgBvAHIAbQBfAG4AIAA9ACAAXAAiADEAXAAiACwAIABcACIAMQBcACIALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGUAbgBfAG4ALAAgAEwARQBOACgAbgBvAHIAbQBfAG4AKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHQAYQBrAGUAXwBkAGkAZwBpAHQAcwAsACAASQBGACgAbABlAG4AXwBuACAAPAA9ACAAMQA0ACwAIABsAGUAbgBfAG4ALAAgAEkARgAoAEkAUwBFAFYARQBOACgAbABlAG4AXwBuACkALAAgADEANAAsACAAMQAzACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHYAXwBzAHQAcgAsACAATABFAEYAVAAoAG4AbwByAG0AXwBuACwAIAB0AGEAawBlAF8AZABpAGcAaQB0AHMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHYAXwBuAHUAbQAsACAAVgBBAEwAVQBFACgAdgBfAHMAdAByACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAB6AGUAcgBvAF8AYwBvAHUAbgB0ACwAIAAoAGwAZQBuAF8AbgAgAC0AIAB0AGEAawBlAF8AZABpAGcAaQB0AHMAKQAgAC8AIAAyACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHMAZQBlAGQAXwBwAHIAZQBmAGkAeAAsACAAVABFAFgAVAAoAFIATwBVAE4ARABVAFAAKABTAFEAUgBUACgAdgBfAG4AdQBtACkALAAgADAAKQAgACsAIAAxACwAIABcACIAMABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHMAZQBlAGQAXwBzAHQAcgAsACAAcwBlAGUAZABfAHAAcgBlAGYAaQB4ACAAJgAgAFIARQBQAFQAKABcACIAMABcACIALAAgAHoAZQByAG8AXwBjAG8AdQBuAHQAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIABTAGMAYQBsAGUAcwAgAGsAIABiAHkAIAB0AGgAZQAgAG0AYQB4AGkAbQB1AG0AIABvAHYAZQByAGwAYQBwACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAawAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwBhAGYAZQBLACgAXAAiAE0AVQBMAFwAIgAsACAAbABlAG4AXwBuACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBuACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBTAHAAbABpAHQAKABuAG8AcgBtAF8AbgAsACAAawApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AcwBlAGUAZAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwBwAGwAaQB0ACgAcwBlAGUAZABfAHMAdAByACwAIABrACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAZgBpAG4AYQBsAF8AbABpAG0AYgBzACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAFMAcQByAHQAKABsAGkAbQBiAHMAXwBuACwAIABsAGkAbQBiAHMAXwBzAGUAZQBkACwAIABrACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4ATQBlAHIAZwBlACgAZgBpAG4AYQBsAF8AbABpAG0AYgBzACwAIABrACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAApACkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAAQwBvAG0AcAB1AHQAZQBzACAAdABoAGUAIABmAGEAYwB0AG8AcgBpAGEAbAAgAG8AZgAgAGEAIABCAGkAZwBJAG4AdAAgACgAbgAhACkAIAB1AHMAaQBuAGcAIABQAGUAdABlAHIAIABMAHUAcwBjAGgAbgB5ACcAcwAgAFAAcgBpAG0AZQAgAFMAdwBpAG4AZwAgAGEAbABnAG8AcgBpAHQAaABtAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAYgBpAGcAXwBpAG4AdAAgAFQAaABlACAAQgBpAGcASQBuAHQAIABzAHQAcgBpAG4AZwAuACAATQBhAHgAaQBtAHUAbQAgAHMAdQBwAHAAbwByAHQAZQBkACAAaQBuAHAAdQB0ACAAaQBzACAAOQAyADcAMwAuAFwAbgAgACoALwBcAG4ARgBhAGMAdAAgAD0AIABMAEEATQBCAEQAQQAoAGIAaQBnAF8AaQBuAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbgBvAHIAbQBfAG4ALAAgAE4AbwByAG0AKABiAGkAZwBfAGkAbgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAaQBnAG4AXwBuACwAIABCAGkAZwBJAG4AdAAuAFMAaQBnAG4AKABuAG8AcgBtAF8AbgApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAcwBpAGcAbgBfAG4AIAA9ACAALQAxACwAIAAjAE4AVQBNACEALABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAG4AbwByAG0AXwBuACAAPQAgAFwAIgAwAFwAIgAsACAAXAAiADEAXAAiACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABuAG8AcgBtAF8AbgAgAD0AIABcACIAMQBcACIALAAgAFwAIgAxAFwAIgAsAFwAbgAgACAAIAAgACAAIAAgACAALwAvACAARgBpAHIAZQB3AGEAbABsACAAMQA6ACAAVAByAGEAcAAgAG0AYQBzAHMAaQB2AGUAIABzAHQAcgBpAG4AZwBzACAAYgBlAGYAbwByAGUAIAB0AGgAZQB5ACAAaABpAHQAIABWAEEATABVAEUAKAApAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgATABFAE4AKABuAG8AcgBtAF8AbgApACAAPgAgADQALAAgACMATgBVAE0AIQAsACAAXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABGAGkAcgBlAHcAYQBsAGwAIAAyADoAIABUAHIAYQBwACAAbQBhAHQAaABlAG0AYQB0AGkAYwBhAGwAIABjAGUAaQBsAGkAbgBnAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAVgBBAEwAVQBFACgAbgBvAHIAbQBfAG4AKQAgAD4AIAA5ADIANwAzACwAIAAjAE4AVQBNACEALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABuAF8AdgBhAGwALAAgAFYAQQBMAFUARQAoAG4AbwByAG0AXwBuACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABnAGwAbwBiAGEAbABfAHAAcgBpAG0AZQBzACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBOAGEAdABpAHYAZQBQAHIAaQBtAGUAcwAoAG4AXwB2AGEAbAApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUAByAGkAbQBlAFMAdwBpAG4AZwBLAGUAcgBuAGUAbAAoAG4AXwB2AGEAbAAsACAAZwBsAG8AYgBhAGwAXwBwAHIAaQBtAGUAcwApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAKQApACkAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABSAGUAdAB1AHIAbgBzACAAdABoAGUAIABtAGkAbgBpAG0AdQBtACAAQgBpAGcASQBuAHQAIABmAHIAbwBtACAAYQBuACAAYQByAHIAYQB5ACAAbwByACAAcgBhAG4AZwBlAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAcgBhAG4AZwBlACAAQQAgAGMAbwBuAHQAaQBnAHUAbwB1AHMAIAByAGEAbgBnAGUAIABvAHIAIABhAHIAcgBhAHkAIABvAGYAIABCAGkAZwBJAG4AdAAgAHMAdAByAGkAbgBnAHMALgBcAG4AIAAqAC8AXABuAE0AaQBuACAAPQAgAEwAQQBNAEIARABBACgAcgBhAG4AZwBlACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAGMAbABlAGEAbgBfAGMAbwBsACwAIABUAE8AQwBPAEwAKAByAGEAbgBnAGUALAAgADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABPAFIAKABJAFMARQBSAFIATwBSACgAYwBsAGUAYQBuAF8AYwBvAGwAKQAsACAAUgBPAFcAUwAoAGMAbABlAGEAbgBfAGMAbwBsACkAIAA9ACAAMAApACwAIABcACIAMABcACIALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVAByAGUAZQBDAG8AbQBwAGEAcgBlACgATQBBAFAAKABjAGwAZQBhAG4AXwBjAG8AbAAsACAAQgBpAGcASQBuAHQALgBOAG8AcgBtACkALAAgAC0AMQApAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAAUgBlAHQAdQByAG4AcwAgAHQAaABlACAAbQBhAHgAaQBtAHUAbQAgAEIAaQBnAEkAbgB0ACAAZgByAG8AbQAgAGEAbgAgAGEAcgByAGEAeQAgAG8AcgAgAHIAYQBuAGcAZQAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAHIAYQBuAGcAZQAgAEEAIABjAG8AbgB0AGkAZwB1AG8AdQBzACAAcgBhAG4AZwBlACAAbwByACAAYQByAHIAYQB5ACAAbwBmACAAQgBpAGcASQBuAHQAIABzAHQAcgBpAG4AZwBzAC4AXABuACAAKgAvAFwAbgBNAGEAeAAgAD0AIABMAEEATQBCAEQAQQAoAHIAYQBuAGcAZQAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABjAGwAZQBhAG4AXwBjAG8AbAAsACAAVABPAEMATwBMACgAcgBhAG4AZwBlACwAIAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgATwBSACgASQBTAEUAUgBSAE8AUgAoAGMAbABlAGEAbgBfAGMAbwBsACkALAAgAFIATwBXAFMAKABjAGwAZQBhAG4AXwBjAG8AbAApACAAPQAgADAAKQAsACAAXAAiADAAXAAiACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFQAcgBlAGUAQwBvAG0AcABhAHIAZQAoAE0AQQBQACgAYwBsAGUAYQBuAF8AYwBvAGwALAAgAEIAaQBnAEkAbgB0AC4ATgBvAHIAbQApACwAIAAxACkAXABuACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACkAOwAiAH0AXQAsACIAcAByAG8AagBlAGMAdABOAGEAbQBlAHMAIgA6AFsAIgB0AGUAcwB0AF8AQgBpAGcASQBuAHQALgBLAG4AdQB0AGgARABpAHYAaQBzAGkAbwBuACIALAAiAHQAZQBzAHQAXwBCAGkAZwBJAG4AdAAuAE4AZQB3AHQAbwBuAFIAYQBwAGgAcwBvAG4ARABpAHYAaQBzAGkAbwBuACIALAAiAHQAZQBzAHQAXwBCAGkAZwBJAG4AdAAuAEQAaQB2AGkAcwBpAG8AbgBBAGwAZwBvAHIAaQB0AGgAbQBzACIALAAiAHQAZQBzAHQAXwBCAGkAZwBJAG4AdAAuAEQAaQB2AGkAcwBpAG8AbgBBAGwAZwBvAHIAaQB0AGgAbQBDAG8AbQBwAGEAcgBpAHMAbwBuACIALAAiAHQAZQBzAHQAXwBCAGkAZwBJAG4AdAAuAEQAaQB2AGkAcwBpAG8AbgBCAGUAbgBjAGgAbQBhAHIAawBDAGEAcwBlAHMAIgAsACIAdABlAHMAdABfAEIAaQBnAEkAbgB0AC4AQQBzAHkAbQBtAGUAdAByAGkAYwBBAEIARwByAGkAZAAiACwAIgB0AGUAcwB0AF8AQgBpAGcASQBuAHQALgBGAGEAYwB0AG8AcgBpAGEAbABBAGwAZwBvAHIAaQB0AGgAbQBzACIALAAiAHQAZQBzAHQAXwBCAGkAZwBJAG4AdAAuAEYAYQBjAHQAbwByAGkAYQBsAEMAbwBtAHAAYQByAGkAcwBvAG4AIgAsACIAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwBhAGYAZQBLACIALAAiAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFMAcABsAGkAdAAiACwAIgBjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBNAGUAcgBnAGUAIgAsACIAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AQwBhAHIAcgB5ACIALAAiAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFUAQwBvAG0AcABhAHIAZQAiACwAIgBjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAEEAZABkACIALAAiAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFUAUwB1AGIAIgAsACIAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBNAGEAdAByAGkAeABTAHUAbQAiACwAIgBjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBBAGQAZABTAHUAYgBSAG8AdQB0AGUAcgAiACwAIgBjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAE0AdQBsACIALAAiAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAEYAaQBuAGQAUQB1AG8AdABpAGUAbgB0AEwAaQBtAGIAIgAsACIAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4ASwBuAHUAdABoAEQAaQB2ACIALAAiAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAEQAaQB2AFIAbwB1AHQAZQByACIALAAiAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAE4AZQB3AHQAbwBuAFIAYQBwAGgAcwBvAG4AUwBlAGUAZAAiACwAIgBjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBOAGUAdwB0AG8AbgBSAGEAcABoAHMAbwBuAFIAZQBjAGkAcAByAG8AYwBhAGwAIgAsACIAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4ATgBlAHcAdABvAG4AUgBhAHAAaABzAG8AbgBEAGkAdgAiACwAIgBjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAFAAbwB3ACIALAAiAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFUAUwBxAHIAdAAiACwAIgBjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBOAGEAdABpAHYAZQBQAHIAaQBtAGUAcwAiACwAIgBjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAFQAZQB4AHQATQB1AGwAIgAsACIAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVABlAHgAdABUAHIAZQBlAFAAcgBvAGQAIgAsACIAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4ATgBhAHQAaQB2AGUAUwB3AGkAbgBnAEUAeABwAG8AbgBlAG4AdABzACIALAAiAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFMAdwBpAG4AZwBUAGUAcgBtACIALAAiAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFAAcgBpAG0AZQBTAHcAaQBuAGcASwBlAHIAbgBlAGwAIgAsACIAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVAByAGUAZQBDAG8AbQBwAGEAcgBlACIALAAiAEIAaQBnAEkAbgB0AC4ATgBvAHIAbQAiACwAIgBCAGkAZwBJAG4AdAAuAFMAaQBnAG4AIgAsACIAQgBpAGcASQBuAHQALgBJAHMAWgBlAHIAbwAiACwAIgBCAGkAZwBJAG4AdAAuAEkAcwBOAGUAZwAiACwAIgBCAGkAZwBJAG4AdAAuAEkAcwBFAHYAZQBuACIALAAiAEIAaQBnAEkAbgB0AC4ASQBzAE8AZABkACIALAAiAEIAaQBnAEkAbgB0AC4AQQBiAHMAIgAsACIAQgBpAGcASQBuAHQALgBDAG8AbQBwAGEAcgBlACIALAAiAEIAaQBnAEkAbgB0AC4AQQBkAGQAIgAsACIAQgBpAGcASQBuAHQALgBTAHUAYgAiACwAIgBCAGkAZwBJAG4AdAAuAFMAdQBtACIALAAiAEIAaQBnAEkAbgB0AC4ATQB1AGwAIgAsACIAQgBpAGcASQBuAHQALgBSAGEAbgBkAEIAaQBnAEkAbgB0AEEAcgByAGEAeQAiACwAIgBCAGkAZwBJAG4AdAAuAEQAaQB2AE0AbwBkACIALAAiAEIAaQBnAEkAbgB0AC4ARABpAHYAIgAsACIAQgBpAGcASQBuAHQALgBNAG8AZAAiACwAIgBCAGkAZwBJAG4AdAAuAFAAbwB3ACIALAAiAEIAaQBnAEkAbgB0AC4AUwBxAHIAdAAiACwAIgBCAGkAZwBJAG4AdAAuAEYAYQBjAHQAIgAsACIAQgBpAGcASQBuAHQALgBNAGkAbgAiACwAIgBCAGkAZwBJAG4AdAAuAE0AYQB4ACIAXQAsACIAbABvAGMAYQBsAGUAIgA6AHsAIgBsAGkAcwB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAcgBvAHcAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIAOwAiACwAIgBjAG8AbAB1AG0AbgBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHQAaABvAHUAcwBhAG4AZABzAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUABvAHMAaQB0AGkAbwBuAHMAIgA6AFsAMwBdACwAIgBkAGUAYwBpAG0AYQBsAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiAC4AIgAsACIAZABhAHQAZQBPAHIAZABlAHIAIgA6ACIARABNAFkAIgAsACIAYwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsACIAOgAiACQAIgAsACIAaQBzAEMAdQByAHIAZQBuAGMAeQBTAHkAbQBiAG8AbABMAGUAYQBkACIAOgB0AHIAdQBlACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAZQBwAEIAeQBTAHAAYQBjAGUAIgA6AGYAYQBsAHMAZQAsACIAcgBvAHcATABlAHQAdABlAHIAIgA6ACIAUgAiACwAIgBjAG8AbAB1AG0AbgBMAGUAdAB0AGUAcgAiADoAIgBDACIALAAiAHIAYwBMAGUAZgB0AEIAcgBhAGMAawBlAHQAIgA6ACIAWwAiACwAIgByAGMAUgBpAGcAaAB0AEIAcgBhAGMAawBlAHQAIgA6ACIAXQAiACwAIgBzAHQAYQB0AGUAbQBlAG4AdABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGwAbwBjAGEAbABlAE4AYQBtAGUAIgA6ACIAZQBuAC0AdQBzACIAfQB9AA==</AFEJSONBlob>
+<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAHQAZQBzAHQAXwBCAGkAZwBJAG4AdAAiACwAIgB0AGUAeAB0ACIAOgAiAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAFwAbgAvAC8AIABCAGkAZwAgAEkAbgB0AGUAZwBlAHIAIABBAHIAaQB0AGgAbQBlAHQAaQBjACAATABpAGIAcgBhAHIAeQAgAC8ALwBcAG4ALwAvACAAIAAgACAAIAAgACAAdABlAHMAdABfAEIAaQBnAEkAbgB0ACAATQBvAGQAdQBsAGUAIAAgACAAIAAgACAAIAAvAC8AXABuAC8ALwAgACAAIAAgACAAIAAgAFAAcgBpAHYAYQB0AGUAIABUAGUAcwB0AGkAbgBnACAAQQBQAEkAIAAgACAAIAAgACAALwAvAFwAbgAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwBcAG4AXABuAEsAbgB1AHQAaABEAGkAdgBpAHMAaQBvAG4APQBMAEEATQBCAEQAQQAoAGEALAAgAGIALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAawAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwBhAGYAZQBLACgAXAAiAEQASQBWAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABwAGEAYwBrAGUAZAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4ASwBuAHUAdABoAEQAaQB2ACgAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwBwAGwAaQB0ACgAYQAsACAAawApACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBTAHAAbABpAHQAKABiACwAIABrACkALAAgAGsAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAE0AZQByAGcAZQAoAEQAUgBPAFAAKABwAGEAYwBrAGUAZAAsACAASQBOAEQARQBYACgAcABhAGMAawBlAGQALAAgADEALAAgADEAKQAgACsAIAAxACkALAAgAGsAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBOAGUAdwB0AG8AbgBSAGEAcABoAHMAbwBuAEQAaQB2AGkAcwBpAG8AbgAgAD0AIABMAEEATQBCAEQAQQAoAGEALAAgAGIALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAawAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwBhAGYAZQBLACgAXAAiAEQASQBWAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABwAGEAYwBrAGUAZAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4ATgBlAHcAdABvAG4AUgBhAHAAaABzAG8AbgBEAGkAdgAoAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFMAcABsAGkAdAAoAGEALAAgAGsAKQAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwBwAGwAaQB0ACgAYgAsACAAawApACwAIABrACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBNAGUAcgBnAGUAKABEAFIATwBQACgAcABhAGMAawBlAGQALAAgAEkATgBEAEUAWAAoAHAAYQBjAGsAZQBkACwAIAAxACwAIAAxACkAIAArACAAMQApACwAIABrACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAEAAcABhAHIAYQBtACAAYQAgAFQAaABlACAAZABpAHYAaQBkAGUAbgBkACAAcwB0AHIAaQBuAGcAXABuACAAKgAgAEAAcABhAHIAYQBtACAAYgAgAFQAaABlACAAZABpAHYAaQBzAG8AcgAgAHMAdAByAGkAbgBnAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAG0AbwBkAGUAIABcACIASwBOAFUAVABIAFwAIgAgAG8AcgAgAFwAIgBOAFIAXAAiAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGkAdABlAHIAcwAgAEkAbgBuAGUAcgAgAGwAbwBvAHAAIABjAG8AdQBuAHQAIAAoAHQAbwAgAGQAZQBmAGUAYQB0ACAAYwBoAHUAbgBrAHkAIABjAGwAbwBjAGsAIAByAGUAcwBvAGwAdQB0AGkAbwBuACkAXABuACAAKgAgAEAAcABhAHIAYQBtACAAcgBlAHAAZQBhAHQAcwAgAE8AdQB0AGUAcgAgAGwAbwBvAHAAIABjAG8AdQBuAHQAIAAoAHQAbwAgAGQAZQBmAGUAYQB0ACAATwBTAC8ARwBhAHIAYgBhAGcAZQAgAEMAbwBsAGwAZQBjAHQAaQBvAG4AIABuAG8AaQBzAGUAKQBcAG4AIAAqAC8AXABuAEQAaQB2AGkAcwBpAG8AbgBBAGwAZwBvAHIAaQB0AGgAbQBzACAAPQAgAEwAQQBNAEIARABBACgAYQAsACAAYgAsACAAbQBvAGQAZQAsACAAaQB0AGUAcgBzACwAIAByAGUAcABlAGEAdABzACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAC8ALwAgAE0AYQBwACAAdABoAGUAIABvAHUAdABlAHIAIAByAGUAcABlAGEAdABzACAAbABvAG8AcABcAG4AIAAgACAAIAAgACAAIAAgAGIAYQB0AGMAaABfAHQAaQBtAGUAcwAsACAATQBBAFAAKABTAEUAUQBVAEUATgBDAEUAKAByAGUAcABlAGEAdABzACkALAAgAEwAQQBNAEIARABBACgAcgAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHMAdABhAHIAdAAsACAATgBPAFcAKAApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAATQBhAHAAIAB0AGgAZQAgAGkAbgBuAGUAcgAgAGUAeABlAGMAdQB0AGkAbwBuACAAbABvAG8AcABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAByAHUAbgAsACAASQBGACgAbQBvAGQAZQAgAD0AIABcACIASwBOAFUAVABIAFwAIgAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAE0AQQBQACgAUwBFAFEAVQBFAE4AQwBFACgAaQB0AGUAcgBzACkALAAgAEwAQQBNAEIARABBACgAaQAsACAASwBuAHUAdABoAEQAaQB2AGkAcwBpAG8AbgAoAGEALAAgAGIAKQApACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBBAFAAKABTAEUAUQBVAEUATgBDAEUAKABpAHQAZQByAHMAKQAsACAATABBAE0AQgBEAEEAKABpACwAIABOAGUAdwB0AG8AbgBSAGEAcABoAHMAbwBuAEQAaQB2AGkAcwBpAG8AbgAoAGEALAAgAGIAKQApACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAEYAbwByAGMAZQAgAGUAdgBhAGwAdQBhAHQAaQBvAG4AIABiAGUAZgBvAHIAZQAgAHAAdQBsAGwAaQBuAGcAIABzAHQAbwBwACAAdABpAG0AZQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABzAHQAbwBwACwAIABOAE8AVwAoACkAIAArACAAKAAwACAAKgAgAEwARQBOACgASQBOAEQARQBYACgAcgB1AG4ALAAgADEALAAgADEAKQApACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIABUAG8AdABhAGwAIABiAGEAdABjAGgAIAB0AGkAbQBlACAAaQBuACAAbQBpAGwAbABpAHMAZQBjAG8AbgBkAHMAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABzAHQAbwBwACAALQAgAHMAdABhAHIAdAApACAAKgAgADgANgA0ADAAMAAwADAAMABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABFAHgAdAByAGEAYwB0ACAAdABoAGUAIABjAGwAZQBhAG4AZQBzAHQAIAByAHUAbgAgAGEAbgBkACAAYQB2AGUAcgBhAGcAZQAgAGkAdAAgAGQAbwB3AG4AIAB0AG8AIABhACAAcwBpAG4AZwBsAGUAIABlAHgAZQBjAHUAdABpAG8AbgAgAHQAaQBtAGUAXABuACAAIAAgACAAIAAgACAAIABNAEkATgAoAGIAYQB0AGMAaABfAHQAaQBtAGUAcwApACAALwAgAGkAdABlAHIAcwBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAARQB4AGUAYwB1AHQAZQBzACAAYQAgAHMAdAByAGkAYwB0AGwAeQAgAHMAZQBxAHUAZQBuAHQAaQBhAGwAIABiAGUAbgBjAGgAbQBhAHIAawAgAHMAdQBpAHQAZQAgAHQAbwAgAGEAdgBvAGkAZAAgAG0AdQBsAHQAaQAtAHQAaAByAGUAYQBkAGkAbgBnACAAYwBvAG4AdABhAG0AaQBuAGEAdABpAG8AbgAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAHQAZQBzAHQAXwBjAGEAcwBlAHMAIABBAG4AIABOACAAeAAgADIAIABhAHIAcgBhAHkAIABvAGYAIAB0AGUAcwB0ACAAbABlAG4AZwB0AGgAcwA6ACAAWwBMAGUAbgBnAHQAaABfAEEALAAgAEwAZQBuAGcAdABoAF8AQgBdAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGkAdABlAHIAcwAgAE4AdQBtAGIAZQByACAAbwBmACAAaQB0AGUAcgBhAHQAaQBvAG4AcwAgAHAAZQByACAAYgBlAG4AYwBoAG0AYQByAGsAIAB0AG8AIABzAG0AbwBvAHQAaAAgAE4ATwBXACgAKQAgAHIAZQBzAG8AbAB1AHQAaQBvAG4ALgBcAG4AIAAqAC8AXABuAEQAaQB2AGkAcwBpAG8AbgBBAGwAZwBvAHIAaQB0AGgAbQBDAG8AbQBwAGEAcgBpAHMAbwBuACAAPQAgAEwAQQBNAEIARABBACgAdABlAHMAdABfAGMAYQBzAGUAcwAsACAAaQB0AGUAcgBzACwAIAByAGUAcABlAGEAdABzACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG4AXwB0AGUAcwB0AHMALAAgAFIATwBXAFMAKAB0AGUAcwB0AF8AYwBhAHMAZQBzACkALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAALwAvACAASQBuAGkAdABpAGEAbAAgAHMAdABhAHQAZQA6ACAARABhAHQAYQAgAGgAZQBhAGQAZQByAHMAIABmAG8AcgAgAEMAUwBWACAAZQB4AHAAbwByAHQAXABuACAAIAAgACAAIAAgACAAIABpAG4AaQB0AGkAYQBsACwAIAB7AFwAIgBMAGUAbgBfAEEAXAAiACwAIABcACIATABlAG4AXwBCAFwAIgAsACAAXAAiAEsAbgB1AHQAaABfAG0AcwBcACIALAAgAFwAIgBOAFIAXwBtAHMAXAAiAH0ALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAUgBFAEQAVQBDAEUAKABpAG4AaQB0AGkAYQBsACwAIABTAEUAUQBVAEUATgBDAEUAKABuAF8AdABlAHMAdABzACkALAAgAEwAQQBNAEIARABBACgAYQBjAGMALAAgAGkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGUAbgBfAGEALAAgAEkATgBEAEUAWAAoAHQAZQBzAHQAXwBjAGEAcwBlAHMALAAgAGkALAAgADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAZQBuAF8AYgAsACAASQBOAEQARQBYACgAdABlAHMAdABfAGMAYQBzAGUAcwAsACAAaQAsACAAMgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAAUwBrAGkAcAAgAEQAaQB2AGkAcwBvAHIAIAA+ACAARABpAHYAaQBkAGUAbgBkABQgaQB0ACcAcwAgAG4AZQB2AGUAcgAgAGEAbgAgAGkAbgB0AGUAZwBlAHIAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgAbABlAG4AXwBiACAAPgAgAGwAZQBuAF8AYQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABhAGMAYwAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAARwBlAG4AZQByAGEAdABlACAAZQB4AGEAYwB0AC0AbABlAG4AZwB0AGgAIAB0AGUAcwB0ACAAcwB0AHIAaQBuAGcAcwAgAG4AYQB0AGkAdgBlAGwAeQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcwB0AHIAXwBhACwAIABSAEUAUABUACgAXAAiADkAXAAiACwAIABsAGUAbgBfAGEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABzAHQAcgBfAGIALAAgAEkARgAoAGwAZQBuAF8AYgAgAD0AIAAxACwAIABcACIANwBcACIALAAgAFwAIgA3AFwAIgAgACYAIABSAEUAUABUACgAXAAiADMAXAAiACwAIABsAGUAbgBfAGIAIAAtACAAMQApACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAEUAeABlAGMAdQB0AGUAIABiAGUAbgBjAGgAbQBhAHIAawBzACAAcwB0AHIAaQBjAHQAbAB5ACAAbwBuAGUAIABhAGYAdABlAHIAIAB0AGgAZQAgAG8AdABoAGUAcgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAdABpAG0AZQBfAGsALAAgAEQAaQB2AGkAcwBpAG8AbgBBAGwAZwBvAHIAaQB0AGgAbQBzACgAcwB0AHIAXwBhACwAIABzAHQAcgBfAGIALAAgAFwAIgBLAE4AVQBUAEgAXAAiACwAIABpAHQAZQByAHMALAAgAHIAZQBwAGUAYQB0AHMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAB0AGkAbQBlAF8AbgByACwAIABEAGkAdgBpAHMAaQBvAG4AQQBsAGcAbwByAGkAdABoAG0AcwAoAHMAdAByAF8AYQAsACAAcwB0AHIAXwBiACwAIABcACIATgBSAFwAIgAsACAAaQB0AGUAcgBzACwAIAByAGUAcABlAGEAdABzACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAEEAcABwAGUAbgBkACAAdABoAGUAIAByAGUAcwB1AGwAdABzAC4AIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAAUgBlAGEAbABsAG8AYwBhAHQAaQBvAG4AIABkAGUAbABhAHkAIABvAGMAYwB1AHIAcwAgAGgAZQByAGUALAAgAHMAYQBmAGUAbAB5ACAAbwB1AHQAcwBpAGQAZQAgAHQAaABlACAAdABpAG0AZQBkACAAdwBpAG4AZABvAHcALgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAVgBTAFQAQQBDAEsAKABhAGMAYwAsACAASABTAFQAQQBDAEsAKABsAGUAbgBfAGEALAAgAGwAZQBuAF8AYgAsACAAdABpAG0AZQBfAGsALAAgAHQAaQBtAGUAXwBuAHIAKQApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8ALwAgAEcAZQBuAGUAcgBhAHQAZQBzACAAYQAgADIALQBjAG8AbAB1AG0AbgAgAGEAcgByAGEAeQAgAG8AZgAgAGUAdgBlAHIAeQAgAGMAbwBtAGIAaQBuAGEAdABpAG8AbgAgAG8AZgAgAGwAZQBuAGcAdABoAHMAXABuAEQAaQB2AGkAcwBpAG8AbgBCAGUAbgBjAGgAbQBhAHIAawBDAGEAcwBlAHMAIAA9ACAATABBAE0AQgBEAEEAKABzAHQAYQByAHQAXwBsAGUAbgAsACAAbQBhAHgAXwBsAGUAbgAsACAAcwB0AGUAcAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABzAGUAcQAsACAAUwBFAFEAVQBFAE4AQwBFACgAKABtAGEAeABfAGwAZQBuACAALQAgAHMAdABhAHIAdABfAGwAZQBuACkAIAAvACAAcwB0AGUAcAAgACsAIAAxACwAIAAxACwAIABzAHQAYQByAHQAXwBsAGUAbgAsACAAcwB0AGUAcAApACwAXABuACAAIAAgACAAIAAgACAAIABuACwAIABSAE8AVwBTACgAcwBlAHEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABDAGEAcgB0AGUAcwBpAGEAbgAgAEoAbwBpAG4AXABuACAAIAAgACAAIAAgACAAIABjAG8AbABfAGEALAAgAFQATwBDAE8ATAAoAEkARgAoAFMARQBRAFUARQBOAEMARQAoADEALAAgAG4AKQAsACAAcwBlAHEAKQApACwAXABuACAAIAAgACAAIAAgACAAIABjAG8AbABfAGIALAAgAFQATwBDAE8ATAAoAEkARgAoAFMARQBRAFUARQBOAEMARQAoAG4ALAAgADEAKQAsACAAVABPAFIATwBXACgAcwBlAHEAKQApACkALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAASABTAFQAQQBDAEsAKABjAG8AbABfAGEALAAgAGMAbwBsAF8AYgApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8ALwAgAEcAZQBuAGUAcgBhAHQAZQBzACAAYQAgAEMAYQByAHQAZQBzAGkAYQBuACAAZwByAGkAZAAgAGYAcgBvAG0AIAB0AHcAbwAgAGkAbgBkAGUAcABlAG4AZABlAG4AdAAgAHMAZQBxAHUAZQBuAGMAZQBzAFwAbgBBAHMAeQBtAG0AZQB0AHIAaQBjAEEAQgBHAHIAaQBkACAAPQAgAEwAQQBNAEIARABBACgAcwB0AGEAcgB0AF8AYQAsACAAbQBhAHgAXwBhACwAIABzAHQAZQBwAF8AYQAsACAAcwB0AGEAcgB0AF8AYgAsACAAbQBhAHgAXwBiACwAIABzAHQAZQBwAF8AYgAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABzAGUAcQBfAGEALAAgAFMARQBRAFUARQBOAEMARQAoACgAbQBhAHgAXwBhACAALQAgAHMAdABhAHIAdABfAGEAKQAgAC8AIABzAHQAZQBwAF8AYQAgACsAIAAxACwAIAAxACwAIABzAHQAYQByAHQAXwBhACwAIABzAHQAZQBwAF8AYQApACwAXABuACAAIAAgACAAIAAgACAAIABzAGUAcQBfAGIALAAgAFMARQBRAFUARQBOAEMARQAoACgAbQBhAHgAXwBiACAALQAgAHMAdABhAHIAdABfAGIAKQAgAC8AIABzAHQAZQBwAF8AYgAgACsAIAAxACwAIAAxACwAIABzAHQAYQByAHQAXwBiACwAIABzAHQAZQBwAF8AYgApACwAXABuACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgAG4AXwBhACwAIABSAE8AVwBTACgAcwBlAHEAXwBhACkALABcAG4AIAAgACAAIAAgACAAIAAgAG4AXwBiACwAIABSAE8AVwBTACgAcwBlAHEAXwBiACkALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAALwAvACAATwByAHQAaABvAGcAbwBuAGEAbAAgAGIAcgBvAGEAZABjAGEAcwB0ACAAdQBzAGkAbgBnACAAaQBuAGQAZQBwAGUAbgBkAGUAbgB0ACAAZABpAG0AZQBuAHMAaQBvAG4AcwBcAG4AIAAgACAAIAAgACAAIAAgAGMAbwBsAF8AYQAsACAAVABPAEMATwBMACgASQBGACgAUwBFAFEAVQBFAE4AQwBFACgAMQAsACAAbgBfAGIAKQAsACAAcwBlAHEAXwBhACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAYwBvAGwAXwBiACwAIABUAE8AQwBPAEwAKABJAEYAKABTAEUAUQBVAEUATgBDAEUAKABuAF8AYQApACwAIABUAE8AUgBPAFcAKABzAGUAcQBfAGIAKQApACkALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAASABTAFQAQQBDAEsAKABjAG8AbABfAGEALAAgAGMAbwBsAF8AYgApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAEYAYQBjAHQAbwByAGkAYQBsAEEAbABnAG8AcgBpAHQAaABtAHMAIAA9ACAATABBAE0AQgBEAEEAKABpAG4AcAB1AHQALAAgAG0AbwBkAGUALAAgAGkAdABlAHIAcwAsACAAcgBlAHAAZQBhAHQAcwAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABNAGEAcAAgAHQAaABlACAAbwB1AHQAZQByACAAcgBlAHAAZQBhAHQAcwAgAGwAbwBvAHAAXABuACAAIAAgACAAIAAgACAAIABiAGEAdABjAGgAXwB0AGkAbQBlAHMALAAgAE0AQQBQACgAUwBFAFEAVQBFAE4AQwBFACgAcgBlAHAAZQBhAHQAcwApACwAIABMAEEATQBCAEQAQQAoAHIALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQALAAgAE4ATwBXACgAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAE0AYQBwACAAdABoAGUAIABpAG4AbgBlAHIAIABlAHgAZQBjAHUAdABpAG8AbgAgAGwAbwBvAHAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcgB1AG4ALAAgAEkARgAoAG0AbwBkAGUAIAA9ACAAXAAiAEwAZQBnAGUAbgBkAHIAZQBcACIALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEEAUAAoAFMARQBRAFUARQBOAEMARQAoAGkAdABlAHIAcwApACwAIABMAEEATQBCAEQAQQAoAGkALAAgAEIAaQBnAEkAbgB0AC4ARgBhAGMAdAAoAGkAbgBwAHUAdAApACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEEAUAAoAFMARQBRAFUARQBOAEMARQAoAGkAdABlAHIAcwApACwAIABMAEEATQBCAEQAQQAoAGkALAAgAEIAaQBnAEkAbgB0AC4ARgBhAGMAdABTAHcAaQBuAGcAKABpAG4AcAB1AHQAKQApACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAEYAbwByAGMAZQAgAGUAdgBhAGwAdQBhAHQAaQBvAG4AIABiAGUAZgBvAHIAZQAgAHAAdQBsAGwAaQBuAGcAIABzAHQAbwBwACAAdABpAG0AZQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABzAHQAbwBwACwAIABOAE8AVwAoACkAIAArACAAKAAwACAAKgAgAEwARQBOACgASQBOAEQARQBYACgAcgB1AG4ALAAgADEALAAgADEAKQApACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIABUAG8AdABhAGwAIABiAGEAdABjAGgAIAB0AGkAbQBlACAAaQBuACAAbQBpAGwAbABpAHMAZQBjAG8AbgBkAHMAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABzAHQAbwBwACAALQAgAHMAdABhAHIAdAApACAAKgAgADgANgA0ADAAMAAwADAAMABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABFAHgAdAByAGEAYwB0ACAAdABoAGUAIABjAGwAZQBhAG4AZQBzAHQAIAByAHUAbgAgAGEAbgBkACAAYQB2AGUAcgBhAGcAZQAgAGkAdAAgAGQAbwB3AG4AIAB0AG8AIABhACAAcwBpAG4AZwBsAGUAIABlAHgAZQBjAHUAdABpAG8AbgAgAHQAaQBtAGUAXABuACAAIAAgACAAIAAgACAAIABNAEkATgAoAGIAYQB0AGMAaABfAHQAaQBtAGUAcwApACAALwAgAGkAdABlAHIAcwBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAARQB4AGUAYwB1AHQAZQBzACAAYQAgAHMAdAByAGkAYwB0AGwAeQAgAHMAZQBxAHUAZQBuAHQAaQBhAGwAIABiAGUAbgBjAGgAbQBhAHIAawAgAHMAdQBpAHQAZQAgAHQAbwAgAGEAdgBvAGkAZAAgAG0AdQBsAHQAaQAtAHQAaAByAGUAYQBkAGkAbgBnACAAYwBvAG4AdABhAG0AaQBuAGEAdABpAG8AbgAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAHQAZQBzAHQAXwBjAGEAcwBlAHMAIABBAG4AIABOACAAeAAgADEAIABhAHIAcgBhAHkAIABvAGYAIAB0AGUAcwB0ACAAaQBuAHAAdQB0AHMAXABuACAAKgAgAEAAcABhAHIAYQBtACAAaQB0AGUAcgBzACAATgB1AG0AYgBlAHIAIABvAGYAIABpAHQAZQByAGEAdABpAG8AbgBzACAAcABlAHIAIABzAGEAbQBwAGwAZQAgAHQAbwAgAHMAbQBvAG8AdABoACAATgBPAFcAKAApACAAcgBlAHMAbwBsAHUAdABpAG8AbgAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAHIAZQBwAGUAYQB0AHMAIABOAHUAbQBiAGUAcgAgAG8AZgAgAGkAdABlAHIAYQB0AGkAbwBuAHMAIABwAGUAcgAgAGIAZQBuAGMAaABtAGEAcgBrACAAdABvACAAcwBtAG8AbwB0AGgAIABPAFMAIABhAG4AZAAgAGIAYQBjAGsAZwByAG8AdQBuAGQAIABuAG8AaQBzAGUALgBcAG4AIAAqAC8AXABuAEYAYQBjAHQAbwByAGkAYQBsAEMAbwBtAHAAYQByAGkAcwBvAG4AIAA9ACAATABBAE0AQgBEAEEAKAB0AGUAcwB0AF8AYwBhAHMAZQBzACwAIABpAHQAZQByAHMALAAgAHIAZQBwAGUAYQB0AHMALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbgBfAHQAZQBzAHQAcwAsACAAUgBPAFcAUwAoAHQAZQBzAHQAXwBjAGEAcwBlAHMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABJAG4AaQB0AGkAYQBsACAAcwB0AGEAdABlADoAIABEAGEAdABhACAAaABlAGEAZABlAHIAcwAgAGYAbwByACAAQwBTAFYAIABlAHgAcABvAHIAdABcAG4AIAAgACAAIAAgACAAIAAgAGkAbgBpAHQAaQBhAGwALAAgAHsAXAAiAE4AXAAiACwAIABcACIATABlAGcAZQBuAGQAcgBlAFwAIgAsACAAXAAiAFMAdwBpAG4AZwBcACIAfQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIABSAEUARABVAEMARQAoAGkAbgBpAHQAaQBhAGwALAAgAFMARQBRAFUARQBOAEMARQAoAG4AXwB0AGUAcwB0AHMAKQAsACAATABBAE0AQgBEAEEAKABhAGMAYwAsACAAaQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGkAbgBwAHUAdAAsACAASQBOAEQARQBYACgAdABlAHMAdABfAGMAYQBzAGUAcwAsACAAaQAsACAAMQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAARQB4AGUAYwB1AHQAZQAgAGIAZQBuAGMAaABtAGEAcgBrAHMAIABzAHQAcgBpAGMAdABsAHkAIABvAG4AZQAgAGEAZgB0AGUAcgAgAHQAaABlACAAbwB0AGgAZQByAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHQAaQBtAGUAXwBsAGUAZwBlAG4AZAByAGUALAAgAEYAYQBjAHQAbwByAGkAYQBsAEEAbABnAG8AcgBpAHQAaABtAHMAKABpAG4AcAB1AHQALAAgAFwAIgBMAGUAZwBlAG4AZAByAGUAXAAiACwAIABpAHQAZQByAHMALAAgAHIAZQBwAGUAYQB0AHMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHQAaQBtAGUAXwBzAHcAaQBuAGcALAAgAEYAYQBjAHQAbwByAGkAYQBsAEEAbABnAG8AcgBpAHQAaABtAHMAKABpAG4AcAB1AHQALAAgAFwAIgBTAHcAaQBuAGcAXAAiACwAIABpAHQAZQByAHMALAAgAHIAZQBwAGUAYQB0AHMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAEEAcABwAGUAbgBkACAAdABoAGUAIAByAGUAcwB1AGwAdABzAC4AIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIABSAGUAYQBsAGwAbwBjAGEAdABpAG8AbgAgAGQAZQBsAGEAeQAgAG8AYwBjAHUAcgBzACAAaABlAHIAZQAsACAAcwBhAGYAZQBsAHkAIABvAHUAdABzAGkAZABlACAAdABoAGUAIAB0AGkAbQBlAGQAIAB3AGkAbgBkAG8AdwAuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFYAUwBUAEEAQwBLACgAYQBjAGMALAAgAEgAUwBUAEEAQwBLACgAaQBuAHAAdQB0ACwAIAB0AGkAbQBlAF8AbABlAGcAZQBuAGQAcgBlACwAIAB0AGkAbQBlAF8AcwB3AGkAbgBnACkAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBjAG8AcgBlAF8AQgBpAGcASQBuAHQAIgAsACIAdABlAHgAdAAiADoAIgAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwBcAG4ALwAvACAAQgBpAGcAIABJAG4AdABlAGcAZQByACAAQQByAGkAdABoAG0AZQB0AGkAYwAgAEwAaQBiAHIAYQByAHkAIAAvAC8AXABuAC8ALwAgACAAIAAgACAAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQAIABNAG8AZAB1AGwAZQAgACAAIAAgACAAIAAgACAALwAvAFwAbgAvAC8AIAAgACAAIAAgACAAIAAgACAAIABQAHIAaQB2AGEAdABlACAAQQBQAEkAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwBcAG4ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8AXABuAFwAbgAvACoAKgBcAG4AIAAqACAAWwBJAG4AdABlAHIAbgBhAGwAXQAgAEMAbwBtAHAAdQB0AGUAcwAgAHQAaABlACAAbQBhAHgAaQBtAHUAbQAgAHMAYQBmAGUAIABiAGEAcwBlAC0AMQAwACAAbABpAG0AYgAgAHMAaQB6AGUAIAAoAGsAKQAgAHQAbwAgAGEAdgBvAGkAZAAgAEkARQBFAEUALQA3ADUANAAgAHAAcgBlAGMAaQBzAGkAbwBuACAAbABvAHMAcwAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAG8AcABlAHIAYQB0AGkAbwBuADoAIABcACIAQQBEAEQAXAAiACwAIABcACIATQBVAEwAXAAiACwAIABvAHIAIABcACIARABJAFYAXAAiAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAWwBtAGEAeABfAGkAdABlAG0AcwBdACAAQQBEAEQAOgAgAG4AdQBtAGIAZQByACAAbwBmACAAbwBwAGUAcgBhAG4AZABzAC4AIABNAFUATAA6ACAAcwBoAG8AcgB0AGUAcwB0ACAAcwB0AHIAaQBuAGcAIABkAGkAZwBpAHQAcwAgAGMAbwB1AG4AdAAuAFwAbgAgACoALwBcAG4AUwBhAGYAZQBLACAAPQAgAEwAQQBNAEIARABBACgAbwBwAGUAcgBhAHQAaQBvAG4ALAAgAFsAbwBwAGUAcgBhAG4AZABfAG8AcgBfAGQAaQBnAGkAdABzAF0ALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAcgBlAHMAbwBsAHYAZQBkAF8AYwBvAHUAbgB0ACwAIABJAEYAKABPAFIAKABvAHAAZQByAGEAbgBkAF8AbwByAF8AZABpAGcAaQB0AHMAIAA9ACAAXAAiAFwAIgAsACAASQBTAE8ATQBJAFQAVABFAEQAKABvAHAAZQByAGEAbgBkAF8AbwByAF8AZABpAGcAaQB0AHMAKQApACwAIAAyACwAIABNAEEAWAAoADIALAAgAG8AcABlAHIAYQBuAGQAXwBvAHIAXwBkAGkAZwBpAHQAcwApACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIABTAFcASQBUAEMASAAoAG8AcABlAHIAYQB0AGkAbwBuACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAEQARABcACIALAAgADEANQAgAC0AIABMAEUATgAoAHIAZQBzAG8AbAB2AGUAZABfAGMAbwB1AG4AdAApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIATQBVAEwAXAAiACwAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHQAZQBzAHQAXwBrACwAIAB7ADcAOwAgADYAOwAgADUAOwAgADQAOwAgADMAOwAgADIAOwAgADEAfQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAG0AYQB4AF8AbwB2AGUAcgBsAGEAcAAsACAAUgBPAFUATgBEAFUAUAAoAHIAZQBzAG8AbAB2AGUAZABfAGMAbwB1AG4AdAAgAC8AIAB0AGUAcwB0AF8AawAsACAAMAApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAAQwBhAGwAYwB1AGwAYQB0AGUAIAB0AGgAZQAgAGEAYgBzAG8AbAB1AHQAZQAgAHAAZQBhAGsAIAB2AGEAbAB1AGUAIABpAG4AcwBpAGQAZQAgAHQAaABlACAAZQBuAGcAaQBuAGUAIAAoAEMAbwBuAHYAbwBsAHUAdABpAG8AbgAgACsAIABDAGEAcgByAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAB1AG4AYwBhAHIAcgBpAGUAZABfAG0AYQB4ACwAIABtAGEAeABfAG8AdgBlAHIAbABhAHAAIAAqACAAKAAxADAAXgB0AGUAcwB0AF8AawAgAC0AIAAxACkAXgAyACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbQBhAHgAXwBjAGEAcgByAHkALAAgAEkATgBUACgAdQBuAGMAYQByAHIAaQBlAGQAXwBtAGEAeAAgAC8AIAAxADAAXgB0AGUAcwB0AF8AawApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcABlAGEAawBfAHYAYQBsACwAIAB1AG4AYwBhAHIAcgBpAGUAZABfAG0AYQB4ACAAKwAgAG0AYQB4AF8AYwBhAHIAcgB5ACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAAUgBlAHQAdQByAG4AIAB0AGgAZQAgAG0AYQB4ACAAawAgADwAPQAgAEUAeABjAGUAbAAnAHMAIAAxADUALQBkAGkAZwBpAHQAIABjAGUAaQBsAGkAbgBnAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAE0AQQBYACgARgBJAEwAVABFAFIAKAB0AGUAcwB0AF8AawAsACAAcABlAGEAawBfAHYAYQBsACAAPAA9ACAAKAAxADAAXgAxADUAIAAtACAAMQApACkAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQASQBWAFwAIgAsACAANwAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAjAE4AQQBNAEUAPwBcAG4AIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFsASQBuAHQAZQByAG4AYQBsAF0AIABVAG4AaQBmAGkAZQBkACAAUwBwAGwAaQB0AHQAZQByAC4AIABTAHAAbABpAHQAcwAgAGIAbwB0AGgAIABzAGMAYQBsAGEAcgBzACAAYQBuAGQAIABhAHIAcgBhAHkAcwAgAGkAbgB0AG8AIABMAGkAdAB0AGwAZQAtAEUAbgBkAGkAYQBuACAAbABpAG0AYgBzAC4AXABuACAAKgAgAFUAcwBlAHMAIABNAEEAWAAoACkAIAB0AG8AIABnAHUAYQByAGEAbgB0AGUAZQAgAHMAYwBhAGwAYQByACAAaQBuAHAAdQB0AHMAIAB0AG8AIAB0AGgAZQAgAFMARQBRAFUARQBOAEMARQAgAGUAbgBnAGkAbgBlAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAYgBpAGcAXwBpAG4AdABzACAAVABoAGUAIABzAHQAcgBpAG4AZwAgAG8AcgAgAGEAcgByAGEAeQAgAG8AZgAgAHMAdAByAGkAbgBnAHMALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABrACAAVABoAGUAIABkAHkAbgBhAG0AaQBjACAAYwBoAHUAbgBrACAAcwBpAHoAZQAgAGMAbwBuAHQAZQB4AHQALgBcAG4AIAAqAC8AXABuAFMAcABsAGkAdAAgAD0AIABMAEEATQBCAEQAQQAoAHMAdAByAF8AbgBvAHIAbQBzACwAIABrACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAGYAbABhAHQAdABlAG4AZQBkAF8AbgBvAHIAbQBzACwAIABUAE8AUgBPAFcAKABzAHQAcgBfAG4AbwByAG0AcwApACwAXABuACAAIAAgACAAIAAgACAAIABsAGUAbgBnAHQAaABzACwAIABMAEUATgAoAGYAbABhAHQAdABlAG4AZQBkAF8AbgBvAHIAbQBzACkALABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQB4AF8AbABlAG4ALAAgAE0AQQBYACgAbABlAG4AZwB0AGgAcwApACwAXABuACAAIAAgACAAIAAgACAAIABwAGEAZABfAGwAZQBuACwAIABSAE8AVQBOAEQAVQBQACgAbQBhAHgAXwBsAGUAbgAgAC8AIABrACwAIAAwACkAIAAqACAAawAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIABwAGEAZABkAGUAZABfAG4AbwByAG0AcwAsACAAUgBFAFAAVAAoAFwAIgAwAFwAIgAsACAAcABhAGQAXwBsAGUAbgAgAC0AIABsAGUAbgBnAHQAaABzACkAIAAmACAAZgBsAGEAdAB0AGUAbgBlAGQAXwBuAG8AcgBtAHMALABcAG4AIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAXwBzAHQAYQByAHQAXwBpAG4AZABpAGMAZQBzACwAIABTAEUAUQBVAEUATgBDAEUAKABwAGEAZABfAGwAZQBuACAALwAgAGsALAAgADEALAAgAHAAYQBkAF8AbABlAG4AIAAtACAAawAgACsAIAAxACwAIAAtAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAtAC0ATQBJAEQAKABwAGEAZABkAGUAZABfAG4AbwByAG0AcwAsACAAbABpAG0AYgBfAHMAdABhAHIAdABfAGkAbgBkAGkAYwBlAHMALAAgAGsAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAAWwBJAG4AdABlAHIAbgBhAGwAXQAgAEMAbwBuAGMAYQB0AGUAbgBhAHQAZQBzACAAYQBuACAAYQByAHIAYQB5ACAAbwBmACAAbgB1AG0AZQByAGkAYwAgAGwAaQBtAGIAcwAgAGkAbgB0AG8AIABhACAAQgBpAGcASQBuAHQAIABzAHQAcgBpAG4AZwAsACAAegBlAHIAbwAtAHAAYQBkAGQAaQBuAGcAIABhAGwAbAAgAGIAdQB0ACAAdABoAGUAIABmAGkAcgBzAHQAIABsAGkAbQBiAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAbABpAG0AYgBzACAAVABoAGUAIAB2AGUAcgB0AGkAYwBhAGwAIABhAHIAcgBhAHkAIABvAGYAIABuAHUAbQBlAHIAaQBjACAAbABpAG0AYgBzAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAawAgAFQAaABlACAAbABpAG0AYgAgAHMAaQB6AGUAIAB1AHMAZQBkACAAZAB1AHIAaQBuAGcAIABjAGEAbABjAHUAbABhAHQAaQBvAG4ALgBcAG4AIAAqAC8AXABuAE0AZQByAGcAZQAgAD0AIABMAEEATQBCAEQAQQAoAGwAaQBtAGIAcwAsACAAawAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABuAHUAbQBfAGwAaQBtAGIAcwAsACAAUgBPAFcAUwAoAGwAaQBtAGIAcwApACwAXABuACAAIAAgACAAIAAgACAAIAByAGUAdgBfAGwAaQBtAGIAcwAsACAAQwBIAE8ATwBTAEUAUgBPAFcAUwAoAGwAaQBtAGIAcwAsACAAUwBFAFEAVQBFAE4AQwBFACgAbgB1AG0AXwBsAGkAbQBiAHMALAAgADEALAAgAG4AdQBtAF8AbABpAG0AYgBzACwAIAAtADEAKQApACwAXABuACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABuAHUAbQBfAGwAaQBtAGIAcwAgAD0AIAAxACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHIAZQB2AF8AbABpAG0AYgBzACAAJgAgAFwAIgBcACIALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAQwBPAE4AQwBBAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABWAFMAVABBAEMASwAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAVABBAEsARQAoAHIAZQB2AF8AbABpAG0AYgBzACwAIAAxACkAIAAmACAAXAAiAFwAIgAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAVABFAFgAVAAoAEQAUgBPAFAAKAByAGUAdgBfAGwAaQBtAGIAcwAsACAAMQApACwAIABSAEUAUABUACgAXAAiADAAXAAiACwAIABrACkAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAAWwBJAG4AdABlAHIAbgBhAGwAXQAgAFIAZQBzAG8AbAB2AGUAcwAgAGMAYQByAHIAaQBlAHMAIAByAGkAZwBoAHQALQB0AG8ALQBsAGUAZgB0ACAAYQBjAHIAbwBzAHMAIABhACAAdgBlAHIAdABpAGMAYQBsACAAYQByAHIAYQB5ACAAbwBmACAAYgBhAHMAZQAtADEAMABeAGsAIABsAGkAbQBiAHMALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABsAGkAbQBiAHMAIABUAGgAZQAgAGEAcgByAGEAeQAgAG8AZgAgAG4AdQBtAGUAcgBpAGMAIABsAGkAbQBiAHMALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABrACAAVABoAGUAIABsAGkAbQBiACAAcwBpAHoAZQAuAFwAbgAgACoALwBcAG4AQwBhAHIAcgB5ACAAPQAgAEwAQQBNAEIARABBACgAbABpAG0AYgBzACwAIABrACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG4AdQBtAF8AbABpAG0AYgBzACwAIABSAE8AVwBTACgAbABpAG0AYgBzACkALABcAG4AIAAgACAAIAAgACAAIAAgAHIAYQBkAGkAeABfAGIAYQBzAGUALAAgADEAMABeAGsALABcAG4AIAAgACAAIAAgACAAIAAgAGEAcgByAF8AYwBhAHIAcgBpAGUAcwAsACAAUwBDAEEATgAoADAALAAgAGwAaQBtAGIAcwAsACAATABBAE0AQgBEAEEAKABhAGMAYwAsACAAdgBhAGwALAAgAHYAYQBsACAAKwAgAEkATgBUACgAYQBjAGMAIAAvACAAcgBhAGQAaQB4AF8AYgBhAHMAZQApACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcgBlAG0AYQBpAG4AZABlAHIAcwAsACAATQBPAEQAKABhAHIAcgBfAGMAYQByAHIAaQBlAHMALAAgAHIAYQBkAGkAeABfAGIAYQBzAGUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAG4AYQBsAF8AYwBhAHIAcgB5ACwAIABJAE4AVAAoAEkATgBEAEUAWAAoAGEAcgByAF8AYwBhAHIAcgBpAGUAcwAsACAAbgB1AG0AXwBsAGkAbQBiAHMALAAgADEAKQAgAC8AIAByAGEAZABpAHgAXwBiAGEAcwBlACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIABJAEYAKABmAGkAbgBhAGwAXwBjAGEAcgByAHkAIAA+ACAAMAAsACAAVgBTAFQAQQBDAEsAKAByAGUAbQBhAGkAbgBkAGUAcgBzACwAIABmAGkAbgBhAGwAXwBjAGEAcgByAHkAKQAsACAAcgBlAG0AYQBpAG4AZABlAHIAcwApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8ALwAgAC0ALQAtACAAVQBuAHMAaQBnAG4AZQBkACAASwBlAHIAbgBlAGwAcwAgAC0ALQAtACAAXABcAFwAXABcAG4AXABuAC8AKgAqAFwAbgAgACoAIABbAEkAbgB0AGUAcgBuAGEAbABdACAAVQBuAHMAaQBnAG4AZQBkACAAYwBvAG0AcABhAHIAaQBzAG8AbgAgAG8AZgAgAHQAdwBvACAATABpAHQAdABsAGUALQBFAG4AZABpAGEAbgAgAGwAaQBtAGIAIABhAHIAcgBhAHkAcwAuAFwAbgAgACoAIABSAGUAdAB1AHIAbgBzACAAMQAgACgAYQAgAD4AIABiACkALAAgAC0AMQAgACgAYQAgADwAIABiACkALAAgAG8AcgAgADAAIAAoAGEAIAA9ACAAYgApAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAbABpAG0AYgBzAF8AYQAgAFQAaABlACAAZgBpAHIAcwB0ACAAbABpAG0AYgAgAGEAcgByAGEAeQAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGwAaQBtAGIAcwBfAGIAIABUAGgAZQAgAHMAZQBjAG8AbgBkACAAbABpAG0AYgAgAGEAcgByAGEAeQAuAFwAbgAgACoALwBcAG4AVQBDAG8AbQBwAGEAcgBlACAAPQAgAEwAQQBNAEIARABBACgAbABpAG0AYgBzAF8AYQAsACAAbABpAG0AYgBzAF8AYgAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABtAGEAeABfAHIAbwB3AHMALAAgAE0AQQBYACgAUgBPAFcAUwAoAGwAaQBtAGIAcwBfAGEAKQAsACAAUgBPAFcAUwAoAGwAaQBtAGIAcwBfAGIAKQApACwAXABuACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBhAF8AYQBsAGkAZwBuAGUAZAAsACAARQBYAFAAQQBOAEQAKABsAGkAbQBiAHMAXwBhACwAIABtAGEAeABfAHIAbwB3AHMALAAgADEALAAgADAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYgBfAGEAbABpAGcAbgBlAGQALAAgAEUAWABQAEEATgBEACgAbABpAG0AYgBzAF8AYgAsACAAbQBhAHgAXwByAG8AdwBzACwAIAAxACwAIAAwACkALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAZABpAGYAZgBlAHIAZQBuAGMAZQBzACwAIABsAGkAbQBiAHMAXwBhAF8AYQBsAGkAZwBuAGUAZAAgAC0AIABsAGkAbQBiAHMAXwBiAF8AYQBsAGkAZwBuAGUAZAAsAFwAbgAgACAAIAAgACAAIAAgACAAaABpAGcAaABlAHMAdABfAG4AbwBuAF8AegBlAHIAbwBfAGkAbgBkAGUAeAAsACAAWABNAEEAVABDAEgAKABUAFIAVQBFACwAIABkAGkAZgBmAGUAcgBlAG4AYwBlAHMAIAA8AD4AIAAwACwAIAAwACwAIAAtADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATgBBACgAaABpAGcAaABlAHMAdABfAG4AbwBuAF8AegBlAHIAbwBfAGkAbgBkAGUAeAApACwAIAAwACwAIABTAEkARwBOACgASQBOAEQARQBYACgAZABpAGYAZgBlAHIAZQBuAGMAZQBzACwAIABoAGkAZwBoAGUAcwB0AF8AbgBvAG4AXwB6AGUAcgBvAF8AaQBuAGQAZQB4ACwAIAAxACkAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABbAEkAbgB0AGUAcgBuAGEAbABdACAAVQBuAHMAaQBnAG4AZQBkACAAYQBkAGQAaQB0AGkAbwBuACAAbwBmACAAdAB3AG8AIABMAGkAdAB0AGwAZQAtAEUAbgBkAGkAYQBuACAAbABpAG0AYgAgAGEAcgByAGEAeQBzAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAbABpAG0AYgBzAF8AYQAgAFQAaABlACAAZgBpAHIAcwB0ACAAbABpAG0AYgAgAGEAcgByAGEAeQAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGwAaQBtAGIAcwBfAGIAIABUAGgAZQAgAHMAZQBjAG8AbgBkACAAbABpAG0AYgAgAGEAcgByAGEAeQAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGsAIABUAGgAZQAgAGQAeQBuAGEAbQBpAGMAIABjAGgAdQBuAGsAIABzAGkAegBlACAAYwBvAG4AdABlAHgAdAAuAFwAbgAgACoALwBcAG4AVQBBAGQAZAAgAD0AIABMAEEATQBCAEQAQQAoAGEALAAgAGIALAAgAGsALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHgAXwByAG8AdwBzACwAIABNAEEAWAAoAFIATwBXAFMAKABhACkALAAgAFIATwBXAFMAKABiACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYQBfAGEAbABpAGcAbgBlAGQALAAgAEUAWABQAEEATgBEACgAYQAsACAAbQBhAHgAXwByAG8AdwBzACwAIAAxACwAIAAwACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGIAXwBhAGwAaQBnAG4AZQBkACwAIABFAFgAUABBAE4ARAAoAGIALAAgAG0AYQB4AF8AcgBvAHcAcwAsACAAMQAsACAAMAApACwAXABuACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAYQByAHIAeQAoAGwAaQBtAGIAcwBfAGEAXwBhAGwAaQBnAG4AZQBkACAAKwAgAGwAaQBtAGIAcwBfAGIAXwBhAGwAaQBnAG4AZQBkACwAIABrACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFsASQBuAHQAZQByAG4AYQBsAF0AIABVAG4AcwBpAGcAbgBlAGQAIABzAHUAYgB0AHIAYQBjAHQAaQBvAG4AIABvAGYAIAB0AHcAbwAgAEwAaQB0AHQAbABlAC0ARQBuAGQAaQBhAG4AIABsAGkAbQBiACAAYQByAHIAYQB5AHMALgBcAG4AIAAqACAAQQBzAHMAdQBtAGUAcwAgAG0AYQBnAG4AaQB0AHUAZABlAHMAIABBACAAPgA9ACAAQgAuACAAUgBlAHMAbwBsAHYAZQBzACAAYgBvAHIAcgBvAHcAcwAgAHQAbwBwAC0AdABvAC0AYgBvAHQAdABvAG0AIABhAG4AZAAgAHQAcgBpAG0AcwAgAHQAcgBhAGkAbABpAG4AZwAgAHoAZQByAG8AcwAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGwAaQBtAGIAcwBfAGEAIABUAGgAZQAgAG0AaQBuAHUAZQBuAGQAIABsAGkAbQBiACAAYQByAHIAYQB5ACAAKABtAHUAcwB0ACAAYgBlACAAPgA9ACAAbABpAG0AYgBzAF8AYgApAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAbABpAG0AYgBzAF8AYgAgAFQAaABlACAAcwB1AGIAdAByAGEAaABlAG4AZAAgAGwAaQBtAGIAIABhAHIAcgBhAHkALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABrACAAVABoAGUAIABkAHkAbgBhAG0AaQBjACAAYwBoAHUAbgBrACAAcwBpAHoAZQAgAGMAbwBuAHQAZQB4AHQALgBcAG4AIAAqAC8AXABuAFUAUwB1AGIAIAA9ACAATABBAE0AQgBEAEEAKABsAGkAbQBiAHMAXwBhACwAIABsAGkAbQBiAHMAXwBiACwAIABrACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQB4AF8AcgBvAHcAcwAsACAATQBBAFgAKABSAE8AVwBTACgAbABpAG0AYgBzAF8AYQApACwAIABSAE8AVwBTACgAbABpAG0AYgBzAF8AYgApACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGEAXwBhAGwAaQBnAG4AZQBkACwAIABFAFgAUABBAE4ARAAoAGwAaQBtAGIAcwBfAGEALAAgAG0AYQB4AF8AcgBvAHcAcwAsACAAMQAsACAAMAApACwAXABuACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBiAF8AYQBsAGkAZwBuAGUAZAAsACAARQBYAFAAQQBOAEQAKABsAGkAbQBiAHMAXwBiACwAIABtAGEAeABfAHIAbwB3AHMALAAgADEALAAgADAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIABkAGkAZgBmAGUAcgBlAG4AYwBlAHMALAAgAGwAaQBtAGIAcwBfAGEAXwBhAGwAaQBnAG4AZQBkACAALQAgAGwAaQBtAGIAcwBfAGIAXwBhAGwAaQBnAG4AZQBkACwAXABuACAAIAAgACAAIAAgACAAIABjAGEAcgByAGkAZQBkAF8AZABpAGYAZgBlAHIAZQBuAGMAZQBzACwAIABDAGEAcgByAHkAKABkAGkAZgBmAGUAcgBlAG4AYwBlAHMALAAgAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIABoAGkAZwBoAGUAcwB0AF8AbgBvAG4AXwB6AGUAcgBvAF8AaQBuAGQAZQB4ACwAIABYAE0AQQBUAEMASAAoAFQAUgBVAEUALAAgAGMAYQByAHIAaQBlAGQAXwBkAGkAZgBmAGUAcgBlAG4AYwBlAHMAIAA8AD4AIAAwACwAIAAwACwAIAAtADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATgBBACgAaABpAGcAaABlAHMAdABfAG4AbwBuAF8AegBlAHIAbwBfAGkAbgBkAGUAeAApACwAIAB7ADAAfQAsACAAVABBAEsARQAoAGMAYQByAHIAaQBlAGQAXwBkAGkAZgBmAGUAcgBlAG4AYwBlAHMALAAgAGgAaQBnAGgAZQBzAHQAXwBuAG8AbgBfAHoAZQByAG8AXwBpAG4AZABlAHgAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABbAEkAbgB0AGUAcgBuAGEAbABdACAAVgBlAGMAdABvAHIAaQB6AGUAZAAgAG0AYQB0AHIAaQB4ACAAcwB1AG0AIABvAGYAIAB1AG4AcwBpAGcAbgBlAGQAIABCAGkAZwBJAG4AdAAgAHMAdAByAGkAbgBnAHMALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABzAHQAcgBfAG4AbwByAG0AcwAgAEgAbwByAGkAegBvAG4AdABhAGwAIABhAHIAcgBhAHkAIAAoADEAeABOACkAIABvAGYAIABuAG8AcgBtAGEAbABpAHoAZQBkACAAbQBhAGcAbgBpAHQAdQBkAGUAIABzAHQAcgBpAG4AZwBzAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAawAgAFQAaABlACAAdQBuAGkAZgBpAGUAZAAgAGQAeQBuAGEAbQBpAGMAIABjAGgAdQBuAGsAIABzAGkAegBlACAAYwBvAG4AdABlAHgAdAAuAFwAbgAgACoALwBcAG4AVQBNAGEAdAByAGkAeABTAHUAbQAgAD0AIABMAEEATQBCAEQAQQAoAHMAdAByAF8AbgBvAHIAbQBzACwAIABrACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAGcAcgBpAGQALAAgAFMAcABsAGkAdAAoAHMAdAByAF8AbgBvAHIAbQBzACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgAHIAYQB3AF8AbABpAG0AYgBzACwAIABCAFkAUgBPAFcAKABnAHIAaQBkACwAIABTAFUATQApACwAXABuACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAYQByAHIAeQAoAHIAYQB3AF8AbABpAG0AYgBzACwAIABrACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFsASQBuAHQAZQByAG4AYQBsAF0AIABSAG8AdQB0AGUAcwAgAGEAZABkAGkAdABpAG8AbgAvAHMAdQBiAHQAcgBhAGMAdABpAG8AbgAgAGIAYQBzAGUAZAAgAG8AbgAgAHMAaQBnAG4AcwAgAGEAbgBkACAAbQBhAGcAbgBpAHQAdQBkAGUAcwAuAFwAbgAgACoAIABSAGUAdAB1AHIAbgBzACAAYQAgAHQAdQBwAGwAZQAgAGEAcgByAGEAeQA6ACAAVgBTAFQAQQBDAEsAKABsAGkAbQBiAHMALAAgAGYAaQBuAGEAbABfAHMAaQBnAG4AKQAgAHcAaABlAHIAZQAgAHQAaABlACAAZgBpAG4AYQBsACAAcgBvAHcAIABpAHMAIAB0AGgAZQAgAHMAYwBhAGwAYQByACAAcwBpAGcAbgAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGwAaQBtAGIAcwBfAGEAIABUAGgAZQAgAGYAaQByAHMAdAAgAGwAaQB0AHQAbABlAC0AZQBuAGQAaQBhAG4AIABsAGkAbQBiACAAYQByAHIAYQB5AC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAbABpAG0AYgBzAF8AYgAgAFQAaABlACAAcwBlAGMAbwBuAGQAIABsAGkAdAB0AGwAZQAtAGUAbgBkAGkAYQBuACAAbABpAG0AYgAgAGEAcgByAGEAeQAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAHMAaQBnAG4AXwBhACAAVABoAGUAIABzAGkAZwBuACAAbwBmACAAdABoAGUAIABmAGkAcgBzAHQAIABhAHIAcgBhAHkAIAAoADEALAAgAC0AMQAsACAAMAApAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAcwBpAGcAbgBfAGIAIABUAGgAZQAgAHMAaQBnAG4AIABvAGYAIAB0AGgAZQAgAHMAZQBjAG8AbgBkACAAYQByAHIAYQB5ACAAKAAxACwAIAAtADEALAAgADAAKQAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGsAIABUAGgAZQAgAGQAeQBuAGEAbQBpAGMAIABjAGgAdQBuAGsAIABzAGkAegBlACAAYwBvAG4AdABlAHgAdAAuAFwAbgAgACoALwBcAG4AQQBkAGQAUwB1AGIAUgBvAHUAdABlAHIAIAA9ACAATABBAE0AQgBEAEEAKABsAGkAbQBiAHMAXwBhACwAIABsAGkAbQBiAHMAXwBiACwAIABzAGkAZwBuAF8AYQAsACAAcwBpAGcAbgBfAGIALAAgAGsALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAaQBzAF8AYQBkAGQAaQB0AGkAbwBuACwAIABzAGkAZwBuAF8AYQAgAD0AIABzAGkAZwBuAF8AYgAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABpAHMAXwBhAGQAZABpAHQAaQBvAG4ALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAVgBTAFQAQQBDAEsAKABVAEEAZABkACgAbABpAG0AYgBzAF8AYQAsACAAbABpAG0AYgBzAF8AYgAsACAAawApACwAIABzAGkAZwBuAF8AYQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAG0AYQBnAG4AaQB0AHUAZABlAF8AYwBvAG0AcABhAHIAaQBzAG8AbgAsACAAVQBDAG8AbQBwAGEAcgBlACgAbABpAG0AYgBzAF8AYQAsACAAbABpAG0AYgBzAF8AYgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgAbQBhAGcAbgBpAHQAdQBkAGUAXwBjAG8AbQBwAGEAcgBpAHMAbwBuACAAPQAgADAALAAgAC8ALwAgAFQAbwB0AGEAbAAgAGMAYQBuAGMAZQBsAGwAYQB0AGkAbwBuADoAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAB7ADAAOwAwAH0ALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgAbQBhAGcAbgBpAHQAdQBkAGUAXwBjAG8AbQBwAGEAcgBpAHMAbwBuACAAPgAgADAALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAAQQAgAGkAcwAgAGwAYQByAGcAZQByADoAIABzAGkAZwBuACAAYgBlAGwAbwBuAGcAcwAgAHQAbwAgAEEALgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAVgBTAFQAQQBDAEsAKABVAFMAdQBiACgAbABpAG0AYgBzAF8AYQAsACAAbABpAG0AYgBzAF8AYgAsACAAawApACwAIABzAGkAZwBuAF8AYQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIABCACAAaQBzACAAbABhAHIAZwBlAHIAOgAgAHIAbwB1AHQAZQAgAEIAIABmAGkAcgBzAHQALAAgAHMAaQBnAG4AIABiAGUAbABvAG4AZwBzACAAdABvACAAQgAuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABWAFMAVABBAEMASwAoAFUAUwB1AGIAKABsAGkAbQBiAHMAXwBiACwAIABsAGkAbQBiAHMAXwBhACwAIABrACkALAAgAHMAaQBnAG4AXwBiACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABbAEkAbgB0AGUAcgBuAGEAbABdACAAVQBuAHMAaQBnAG4AZQBkACAAbQB1AGwAdABpAHAAbABpAGMAYQB0AGkAbwBuACAAbwBmACAAdAB3AG8AIABMAGkAdAB0AGwAZQAtAEUAbgBkAGkAYQBuACAAbABpAG0AYgAgAGEAcgByAGEAeQBzAC4AXABuACAAKgAgAFUAdABpAGwAaQB6AGUAcwAgAGEAIAAxAEQAIABEAGkAcwBjAHIAZQB0AGUAIABDAG8AbgB2AG8AbAB1AHQAaQBvAG4AIAAoAEMAYQB1AGMAaAB5ACAAUAByAG8AZAB1AGMAdAApACAAYQByAHIAYQB5AC0AcwBsAGkAYwBpAG4AZwAgAHMAdAByAGEAdABlAGcAeQAuAFwAbgAgACoAIABaAGUAcgBvACAAZAB5AG4AYQBtAGkAYwAgAG0AZQBtAG8AcgB5ACAAcgBlAGEAbABsAG8AYwBhAHQAaQBvAG4ALgAgACQATwAoAE4AKwBNACkAJAAgAG0AZQBtAG8AcgB5ACAAZgBvAG8AdABwAHIAaQBuAHQALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABsAGkAbQBiAHMAXwBhACAAVABoAGUAIABtAHUAbAB0AGkAcABsAGkAYwBhAG4AZAAgAGwAaQBtAGIAIABhAHIAcgBhAHkALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABsAGkAbQBiAHMAXwBiACAAVABoAGUAIABtAHUAbAB0AGkAcABsAGkAZQByACAAbABpAG0AYgAgAGEAcgByAGEAeQAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGsAIABUAGgAZQAgAGQAeQBuAGEAbQBpAGMAIABjAGgAdQBuAGsAIABzAGkAegBlACAAYwBvAG4AdABlAHgAdAAuAFwAbgAgACoALwBcAG4AVQBNAHUAbAAgAD0AIABMAEEATQBCAEQAQQAoAGwAaQBtAGIAcwBfAGEALAAgAGwAaQBtAGIAcwBfAGIALAAgAGsALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbgB1AG0AXwBsAGkAbQBiAHMAXwBhACwAIABSAE8AVwBTACgAbABpAG0AYgBzAF8AYQApACwAXABuACAAIAAgACAAIAAgACAAIABuAHUAbQBfAGwAaQBtAGIAcwBfAGIALAAgAFIATwBXAFMAKABsAGkAbQBiAHMAXwBiACkALABcAG4AIAAgACAAIAAgACAAIAAgAGMAbwBuAHYAbwBsAHUAdABpAG8AbgBfAGwAZQBuAGcAdABoACwAIABuAHUAbQBfAGwAaQBtAGIAcwBfAGEAIAArACAAbgB1AG0AXwBsAGkAbQBiAHMAXwBiACAALQAgADEALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAcgBhAHcAXwBjAG8AbgB2AG8AbAB1AHQAaQBvAG4ALAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAYwBvAG4AdgBvAGwAdQB0AGkAbwBuAF8AbABlAG4AZwB0AGgALAAgADEALAAgAEwAQQBNAEIARABBACgAcgAsACAAYwAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHcAaQBuAGQAbwB3AF8AcwB0AGEAcgB0AF8AaQAsACAATQBBAFgAKAAxACwAIAByACAALQAgAG4AdQBtAF8AbABpAG0AYgBzAF8AYgAgACsAIAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAB3AGkAbgBkAG8AdwBfAGUAbgBkAF8AaQAsACAATQBJAE4AKAByACwAIABuAHUAbQBfAGwAaQBtAGIAcwBfAGEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAG8AdgBlAHIAbABhAHAAXwByAG8AdwBzACwAIAB3AGkAbgBkAG8AdwBfAGUAbgBkAF8AaQAgAC0AIAB3AGkAbgBkAG8AdwBfAHMAdABhAHIAdABfAGkAIAArACAAMQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHMAZQBxAF8AaQAsACAAUwBFAFEAVQBFAE4AQwBFACgAbwB2AGUAcgBsAGEAcABfAHIAbwB3AHMALAAgADEALAAgAHcAaQBuAGQAbwB3AF8AcwB0AGEAcgB0AF8AaQAsACAAMQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcwBlAHEAXwBqACwAIABTAEUAUQBVAEUATgBDAEUAKABvAHYAZQByAGwAYQBwAF8AcgBvAHcAcwAsACAAMQAsACAAcgAgAC0AIAB3AGkAbgBkAG8AdwBfAHMAdABhAHIAdABfAGkAIAArACAAMQAsACAALQAxACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABTAFUATQAoAEkATgBEAEUAWAAoAGwAaQBtAGIAcwBfAGEALAAgAHMAZQBxAF8AaQAsACAAMQApACAAKgAgAEkATgBEAEUAWAAoAGwAaQBtAGIAcwBfAGIALAAgAHMAZQBxAF8AagAsACAAMQApACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAApACkALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBhAHIAcgB5ACgAcgBhAHcAXwBjAG8AbgB2AG8AbAB1AHQAaQBvAG4ALAAgAGsAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AoAAqACAAWwBJAG4AdABlAHIAbgBhAGwAXQAgAEIAaQBuAGEAcgB5ACAAcwBlAGEAcgBjAGgAIAB0AG8AIABmAGkAbgBkACAAdABoAGUAIABoAGkAZwBoAGUAcwB0ACAAcwBjAGEAbABhAHIAIABxAHUAbwB0AGkAZQBuAHQAIABsAGkAbQBiACAAcQAgACgAMAAgADwAPQAgAHEAIAA8ACAAMQAwAF4AawApAFwAbgCgACoAIABzAHUAYwBoACAAdABoAGEAdAAgAEIAIAAqACAAcQAgADwAPQAgAGwAaQBtAGIAcwBfAHIALgAgAEUAbABpAG0AaQBuAGEAdABlAHMAIAB0AGgAZQAgAG4AZQBlAGQAIABmAG8AcgAgAEsAbgB1AHQAaAAgAEQAIABmAGwAbwBhAHQALQBlAHMAdABpAG0AYQB0AGkAbwBuAC4AXABuAKAAKgAgAEAAcABhAHIAYQBtACAAbABpAG0AYgBzAF8AcgAgAFQAaABlACAAYwB1AHIAcgBlAG4AdAAgAHIAZQBtAGEAaQBuAGQAZQByACAAYQByAHIAYQB5AC4AXABuAKAAKgAgAEAAcABhAHIAYQBtACAAYgAgAFQAaABlACAAZABpAHYAaQBzAG8AcgAgAGEAcgByAGEAeQAuAFwAbgCgACoAIABAAHAAYQByAGEAbQAgAGsAIABUAGgAZQAgAGQAeQBuAGEAbQBpAGMAIABjAGgAdQBuAGsAIABzAGkAegBlACAAYwBvAG4AdABlAHgAdAAuAFwAbgCgACoALwBcAG4ARgBpAG4AZABRAHUAbwB0AGkAZQBuAHQATABpAG0AYgAgAD0AIABMAEEATQBCAEQAQQAoAGwAaQBtAGIAcwBfAHIALAAgAGwAaQBtAGIAcwBfAGIALAAgAGsALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAcgBlAHEAdQBpAHIAZQBkAF8AYgBpAHQAcwAsACAAQwBFAEkATABJAE4ARwAuAE0AQQBUAEgAKABMAE8ARwAoADEAMABeAGsALAAgADIAKQApACwAXABuACAAIAAgACAAIAAgACAAIABwAG8AdwBlAHIAcwBfAG8AZgBfAHQAdwBvACwAIAAyACAAXgAgAFMARQBRAFUARQBOAEMARQAoAHIAZQBxAHUAaQByAGUAZABfAGIAaQB0AHMALAAgADEALAAgAHIAZQBxAHUAaQByAGUAZABfAGIAaQB0AHMAIAAtACAAMQAsACAALQAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAUgBFAEQAVQBDAEUAKAAwACwAIABwAG8AdwBlAHIAcwBfAG8AZgBfAHQAdwBvACwAIABMAEEATQBCAEQAQQAoAGMAdQByAHIAZQBuAHQAXwBxACwAIABjAHUAcgByAGUAbgB0AF8AcABvAHcAZQByACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAdABlAHMAdABfAHEALAAgAGMAdQByAHIAZQBuAHQAXwBxACAAKwAgAGMAdQByAHIAZQBuAHQAXwBwAG8AdwBlAHIALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKAB0AGUAcwB0AF8AcQAgAD4APQAgADEAMABeAGsALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAYwB1AHIAcgBlAG4AdABfAHEALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGIAcQAsACAAQwBhAHIAcgB5ACgAbABpAG0AYgBzAF8AYgAgACoAIAB0AGUAcwB0AF8AcQAsACAAawApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAG0AYQBnAG4AaQB0AHUAZABlAF8AYwBvAG0AcABhAHIAaQBzAG8AbgAsACAAVQBDAG8AbQBwAGEAcgBlACgAbABpAG0AYgBzAF8AcgAsACAAbABpAG0AYgBzAF8AYgBxACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEkARgAoAG0AYQBnAG4AaQB0AHUAZABlAF8AYwBvAG0AcABhAHIAaQBzAG8AbgAgAD4APQAgADAALAAgAHQAZQBzAHQAXwBxACwAIABjAHUAcgByAGUAbgB0AF8AcQApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgCgACoAIABbAEkAbgB0AGUAcgBuAGEAbABdACAAQgBhAHMAZQBjAGEAcwBlACAARABpAHYAaQBzAGkAbwBuACAAdgBpAGEAIABzAGUAcQB1AGUAbgB0AGkAYQBsACAAcwBoAGkAZgB0AC0AYQBuAGQALQBzAHUAYgB0AHIAYQBjAHQALgBcAG4AoAAqACAAUgBlAHQAdQByAG4AcwAgAGEAIABwAGEAYwBrAGUAZAAgADEARAAgAGEAcgByAGEAeQA6ACAAVgBTAFQAQQBDAEsAKABMAGUAbgBnAHQAaABfAFIALAAgAFIAXwBsAGkAbQBiAHMALAAgAFEAXwBsAGkAbQBiAHMAKQAuAFwAbgCgACoAIABFAGwAaQBtAGkAbgBhAHQAZQBzACAAMgBEACAAYQByAHIAYQB5ACAAcABhAGQAZABpAG4AZwAgAHQAbwAgAHMAdAByAGkAYwB0AGwAeQAgAHAAcgBlAHMAZQByAHYAZQAgAG0AZQBtAG8AcgB5ACAAZQBmAGYAaQBjAGkAZQBuAGMAeQAuAFwAbgCgACoAIABAAHAAYQByAGEAbQAgAGwAaQBtAGIAcwBfAGEAIABUAGgAZQAgAGQAaQB2AGkAZABlAG4AZAAgAGEAcgByAGEAeQAuAFwAbgCgACoAIABAAHAAYQByAGEAbQAgAGwAaQBtAGIAcwBfAGIAIABUAGgAZQAgAGQAaQB2AGkAcwBvAHIAIABhAHIAcgBhAHkAIAAoAGEAcwBzAHUAbQBlAGQAIABuAG8AbgAtAHoAZQByAG8AKQAuAFwAbgCgACoAIABAAHAAYQByAGEAbQAgAGsAIABUAGgAZQAgAGQAeQBuAGEAbQBpAGMAIABjAGgAdQBuAGsAIABzAGkAegBlACAAYwBvAG4AdABlAHgAdAAuAFwAbgCgACoALwBcAG4ASwBuAHUAdABoAEQAaQB2ACAAPQAgAEwAQQBNAEIARABBACgAbABpAG0AYgBzAF8AYQAsACAAbABpAG0AYgBzAF8AYgAsACAAawAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABtAGEAZwBuAGkAdAB1AGQAZQBfAGMAbwBtAHAAYQByAGkAcwBvAG4ALAAgAFUAQwBvAG0AcABhAHIAZQAoAGwAaQBtAGIAcwBfAGEALAAgAGwAaQBtAGIAcwBfAGIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABtAGEAZwBuAGkAdAB1AGQAZQBfAGMAbwBtAHAAYQByAGkAcwBvAG4AIAA8ACAAMAAsACAAVgBTAFQAQQBDAEsAKABSAE8AVwBTACgAbABpAG0AYgBzAF8AYQApACwAIABsAGkAbQBiAHMAXwBhACwAIAAwACkALABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAG0AYQBnAG4AaQB0AHUAZABlAF8AYwBvAG0AcABhAHIAaQBzAG8AbgAgAD0AIAAwACwAIABWAFMAVABBAEMASwAoADEALAAgADAALAAgADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAG4AdQBtAF8AbABpAG0AYgBzAF8AYQAsACAAUgBPAFcAUwAoAGwAaQBtAGIAcwBfAGEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGIAaQBnAF8AZQBuAGQAaQBhAG4AXwBhACwAIABDAEgATwBPAFMARQBSAE8AVwBTACgAbABpAG0AYgBzAF8AYQAsACAAUwBFAFEAVQBFAE4AQwBFACgAbgB1AG0AXwBsAGkAbQBiAHMAXwBhACwAIAAxACwAIABuAHUAbQBfAGwAaQBtAGIAcwBfAGEALAAgAC0AMQApACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABmAGkAbgBhAGwAXwBwAGEAYwBrAGUAZABfAHMAdABhAHQAZQAsACAAUgBFAEQAVQBDAEUAKABWAFMAVABBAEMASwAoADEALAAgADAALAAgADAAKQAsACAAYgBpAGcAXwBlAG4AZABpAGEAbgBfAGEALAAgAEwAQQBNAEIARABBACgAcABhAGMAawBlAGQAXwBzAHQAYQB0AGUALAAgAHYAYQBsACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABuAHUAbQBfAGwAaQBtAGIAcwBfAHIALAAgAEkATgBEAEUAWAAoAHAAYQBjAGsAZQBkAF8AcwB0AGEAdABlACwAIAAxACwAIAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AcgAsACAAQwBIAE8ATwBTAEUAUgBPAFcAUwAoAHAAYQBjAGsAZQBkAF8AcwB0AGEAdABlACwAIABTAEUAUQBVAEUATgBDAEUAKABuAHUAbQBfAGwAaQBtAGIAcwBfAHIALAAgADEALAAgADIAKQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAHEALAAgAEQAUgBPAFAAKABwAGEAYwBrAGUAZABfAHMAdABhAHQAZQAsACAAbgB1AG0AXwBsAGkAbQBiAHMAXwByACAAKwAgADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AcwBoAGkAZgB0AGUAZABfAHIALAAgAEkARgAoAEEATgBEACgAUgBPAFcAUwAoAGwAaQBtAGIAcwBfAHIAKQAgAD0AIAAxACwAIABJAE4ARABFAFgAKABsAGkAbQBiAHMAXwByACwAIAAxACwAIAAxACkAIAA9ACAAMAApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAB2AGEAbAAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAVgBTAFQAQQBDAEsAKAB2AGEAbAAsACAAbABpAG0AYgBzAF8AcgApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABxAF8AbABpAG0AYgAsACAARgBpAG4AZABRAHUAbwB0AGkAZQBuAHQATABpAG0AYgAoAGwAaQBtAGIAcwBfAHMAaABpAGYAdABlAGQAXwByACwAIABsAGkAbQBiAHMAXwBiACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYgBxACwAIABDAGEAcgByAHkAKABsAGkAbQBiAHMAXwBiACAAKgAgAHEAXwBsAGkAbQBiACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AbgBlAHgAdABfAHIALAAgAFUAUwB1AGIAKABsAGkAbQBiAHMAXwBzAGgAaQBmAHQAZQBkAF8AcgAsACAAbABpAG0AYgBzAF8AYgBxACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAaABhAHMAXwBxACwAIABPAFIAKABSAE8AVwBTACgAbABpAG0AYgBzAF8AcQApACAAPgAgADEALAAgAEkATgBEAEUAWAAoAGwAaQBtAGIAcwBfAHEALAAxACwAMQApACAAPgAgADAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AbgBlAHgAdABfAHEALAAgAEkARgAoAGgAYQBzAF8AcQAsACAAVgBTAFQAQQBDAEsAKABsAGkAbQBiAHMAXwBxACwAIABxAF8AbABpAG0AYgApACwAIABxAF8AbABpAG0AYgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABWAFMAVABBAEMASwAoAFIATwBXAFMAKABsAGkAbQBiAHMAXwBuAGUAeAB0AF8AcgApACwAIABsAGkAbQBiAHMAXwBuAGUAeAB0AF8AcgAsACAAbABpAG0AYgBzAF8AbgBlAHgAdABfAHEAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbgB1AG0AXwBsAGkAbQBiAHMAXwByACwAIABJAE4ARABFAFgAKABmAGkAbgBhAGwAXwBwAGEAYwBrAGUAZABfAHMAdABhAHQAZQAsACAAMQAsACAAMQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AcgAsACAAQwBIAE8ATwBTAEUAUgBPAFcAUwAoAGYAaQBuAGEAbABfAHAAYQBjAGsAZQBkAF8AcwB0AGEAdABlACwAIABTAEUAUQBVAEUATgBDAEUAKABuAHUAbQBfAGwAaQBtAGIAcwBfAHIALAAgADEALAAgADIAKQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAYgBpAGcAXwBlAG4AZABpAGEAbgBfAHEALAAgAEQAUgBPAFAAKABmAGkAbgBhAGwAXwBwAGEAYwBrAGUAZABfAHMAdABhAHQAZQAsACAAbgB1AG0AXwBsAGkAbQBiAHMAXwByACAAKwAgADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAZQBuAF8AcQAsACAAUgBPAFcAUwAoAGIAaQBnAF8AZQBuAGQAaQBhAG4AXwBxACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBxACwAIABDAEgATwBPAFMARQBSAE8AVwBTACgAYgBpAGcAXwBlAG4AZABpAGEAbgBfAHEALAAgAFMARQBRAFUARQBOAEMARQAoAGwAZQBuAF8AcQAsACAAMQAsACAAbABlAG4AXwBxACwAIAAtADEAKQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAVgBTAFQAQQBDAEsAKABuAHUAbQBfAGwAaQBtAGIAcwBfAHIALAAgAGwAaQBtAGIAcwBfAHIALAAgAGwAaQBtAGIAcwBfAHEAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AoAAqACAAWwBJAG4AdABlAHIAbgBhAGwAXQAgAEgAeQBiAHIAaQBkACAARABpAHYAaQBzAGkAbwBuACAAUgBvAHUAdABlAHIALgBcAG4AoAAqACAARABpAHIAZQBjAHQAcwAgAGQAaQB2AGkAcwBpAG8AbgAgAHQAbwAgAHQAaABlACAAbwBwAHQAaQBtAGEAbAAgAGsAZQByAG4AZQBsACAAYgBhAHMAZQBkACAAbwBuACAARABpAHYAaQBkAGUAbgBkACAAbABlAG4AZwB0AGgALgBcAG4AoAAqACAAQABwAGEAcgBhAG0AIABsAGkAbQBiAHMAXwBhACAAVABoAGUAIABkAGkAdgBpAGQAZQBuAGQAIABhAHIAcgBhAHkALgBcAG4AoAAqACAAQABwAGEAcgBhAG0AIABsAGkAbQBiAHMAXwBiACAAVABoAGUAIABkAGkAdgBpAHMAbwByACAAYQByAHIAYQB5AC4AXABuAKAAKgAgAEAAcABhAHIAYQBtACAAawAgAFQAaABlACAAZAB5AG4AYQBtAGkAYwAgAGMAaAB1AG4AawAgAHMAaQB6AGUAIABjAG8AbgB0AGUAeAB0AC4AXABuAKAAKgAvAFwAbgBEAGkAdgBSAG8AdQB0AGUAcgAgAD0AIABMAEEATQBCAEQAQQAoAGwAaQBtAGIAcwBfAGEALAAgAGwAaQBtAGIAcwBfAGIALAAgAGsALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAYQBwAHAAcgBvAHgAXwBkAGkAZwBpAHQAcwBfAGEALAAgAFIATwBXAFMAKABsAGkAbQBiAHMAXwBhACkAIAAqACAAawAsAFwAbgAgACAAIAAgACAAIAAgACAAYQBwAHAAcgBvAHgAXwBkAGkAZwBpAHQAcwBfAGIALAAgAFIATwBXAFMAKABsAGkAbQBiAHMAXwBiACkAIAAqACAAawAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABMAG8AZwBpAHMAdABpAGMAIABSAGUAZwByAGUAcwBzAGkAbwBuACAAYwBvAGUAZgBmAGkAYwBpAGUAbgB0AHMAXABuACAAIAAgACAAIAAgACAAIAByAGUAZwByAGUAcwBzAGkAbwBuAF8AcwBsAG8AcABlAF8AbQAsACAAMAAuADEAMAA3ADgAMgAxADEAOQA0ADIANwAxADIAOQA3ACwAXABuACAAIAAgACAAIAAgACAAIAByAGUAZwByAGUAcwBzAGkAbwBuAF8AaQBuAHQAZQByAGMAZQBwAHQAXwBjACwAIAAtADIAMgAxAC4AOQAwADIAMQA4ADkANAA2ADIAMAA2ADgALABcAG4AIAAgACAAIAAgACAAIAAgAHQAaAByAGUAcwBoAG8AbABkAF8AZABpAGcAaQB0AHMALAAgACgAcgBlAGcAcgBlAHMAcwBpAG8AbgBfAHMAbABvAHAAZQBfAG0AIAAqACAAYQBwAHAAcgBvAHgAXwBkAGkAZwBpAHQAcwBfAGEAKQAgACsAIAByAGUAZwByAGUAcwBzAGkAbwBuAF8AaQBuAHQAZQByAGMAZQBwAHQAXwBjACwAXABuACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAGEAcABwAHIAbwB4AF8AZABpAGcAaQB0AHMAXwBiACAAPAA9ACAAdABoAHIAZQBzAGgAbwBsAGQAXwBkAGkAZwBpAHQAcwAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABLAG4AdQB0AGgARABpAHYAKABsAGkAbQBiAHMAXwBhACwAIABsAGkAbQBiAHMAXwBiACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATgBlAHcAdABvAG4AUgBhAHAAaABzAG8AbgBEAGkAdgAoAGwAaQBtAGIAcwBfAGEALAAgAGwAaQBtAGIAcwBfAGIALAAgAGsAKQBcAG4AIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFsASQBuAHQAZQByAG4AYQBsAF0AIABHAGUAbgBlAHIAYQB0AGUAcwAgAHQAaABlACAAZQB4AGEAYwB0ACAAcgBlAGMAaQBwAHIAbwBjAGEAbAAgAHMAZQBlAGQAIABmAG8AcgAgAE4AZQB3AHQAbwBuAC0AUgBhAHAAaABzAG8AbgAgAEQAaQB2AGkAcwBpAG8AbgAgAHUAcwBpAG4AZwAgAEsAbgB1AHQAaAAgAEIAYQBzAGUAYwBhAHMAZQAuAFwAbgAgACoAIABFAHgAdAByAGEAYwB0AHMAIAB1AHAAIAB0AG8AIAB0AGgAZQAgAHQAbwBwACAAMwAgAGwAaQBtAGIAcwAgAG8AZgAgAEIAIABhAG4AZAAgAGMAYQBsAGMAdQBsAGEAdABlAHMAIABmAGwAbwBvAHIAKABCAGUAdABhAF4AKAAyACoAbABlAG4AKQAgAC8AIABCAF8AdABvAHAAKQAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGwAaQBtAGIAcwBfAGIAIABUAGgAZQAgAGQAaQB2AGkAcwBvAHIAIABsAGkAbQBiACAAYQByAHIAYQB5AC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAawAgAFQAaABlACAAZAB5AG4AYQBtAGkAYwAgAGMAaAB1AG4AawAgAHMAaQB6AGUAIABjAG8AbgB0AGUAeAB0AC4AXABuACAAKgAvAFwAbgBOAGUAdwB0AG8AbgBSAGEAcABoAHMAbwBuAFMAZQBlAGQAIAA9ACAATABBAE0AQgBEAEEAKABsAGkAbQBiAHMAXwBiACwAIABrACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG4AdQBtAF8AbABpAG0AYgBzAF8AYgAsACAAUgBPAFcAUwAoAGwAaQBtAGIAcwBfAGIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbgB1AG0AXwBzAGUAZQBkAF8AbABpAG0AYgBzACwAIABNAEkATgAoADMALAAgAG4AdQBtAF8AbABpAG0AYgBzAF8AYgApACwAXABuACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgAC8ALwAgAEUAeAB0AHIAYQBjAHQAIAB0AG8AcAAgACcAcwBlAGUAZABfAGwAZQBuACcAIABsAGkAbQBiAHMAIAAoAEwAaQB0AHQAbABlAC0ARQBuAGQAaQBhAG4AOgAgAHQAYQBrAGUAIABmAHIAbwBtACAAdABoAGUAIABiAG8AdAB0AG8AbQApAFwAbgAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYgBfAHQAbwBwACwAIABUAEEASwBFACgAbABpAG0AYgBzAF8AYgAsACAALQBuAHUAbQBfAHMAZQBlAGQAXwBsAGkAbQBiAHMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABDAG8AbgBzAHQAcgB1AGMAdAAgAEIAZQB0AGEAXgAoADIAIAAqACAAcwBlAGUAZABfAGwAZQBuACkAIABuAGEAdABpAHYAZQBsAHkAXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABlAC4AZwAuACwAIABpAGYAIABzAGUAZQBkAF8AbABlAG4AIAA9ACAAMQAsACAAdABoAGUAbgAgADEAIABmAG8AbABsAG8AdwBlAGQAIABiAHkAIAB0AHcAbwAgAHoAZQByAG8AIABsAGkAbQBiAHMAOgAgAFYAUwBUAEEAQwBLACgAMAAsACAAMAAsACAAMQApAFwAbgAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYgBlAHQAYQBfADIAbQAsACAAVgBTAFQAQQBDAEsAKABFAFgAUABBAE4ARAAoADAALAAgADIAIAAqACAAbgB1AG0AXwBzAGUAZQBkAF8AbABpAG0AYgBzACwAIAAsACAAMAApACwAIAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAALwAvACAASwBuAHUAdABoACAARABpAHYAaQBzAGkAbwBuACAAeQBpAGUAbABkAHMAIABlAHgAYQBjAHQAIABpAG4AaQB0AGkAYQBsACAAcgBlAGMAaQBwAHIAbwBjAGEAbABcAG4AIAAgACAAIAAgACAAIAAgAHAAYQBjAGsAZQBkAF8AYgBhAHMAZQBjAGEAcwBlAF8AcgBlAHMAdQBsAHQALAAgAEsAbgB1AHQAaABEAGkAdgAoAGwAaQBtAGIAcwBfAGIAZQB0AGEAXwAyAG0ALAAgAGwAaQBtAGIAcwBfAGIAXwB0AG8AcAAsACAAawApACwAXABuACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgAC8ALwAgAEUAeAB0AHIAYQBjAHQAIABRAHUAbwB0AGkAZQBuAHQAIABhAHIAcgBhAHkAIABmAHIAbwBtACAAdABoAGUAIABwAGEAYwBrAGUAZAAgAFYAUwBUAEEAQwBLAFwAbgAgACAAIAAgACAAIAAgACAAbgB1AG0AXwBsAGkAbQBiAHMAXwByACwAIABJAE4ARABFAFgAKABwAGEAYwBrAGUAZABfAGIAYQBzAGUAYwBhAHMAZQBfAHIAZQBzAHUAbAB0ACwAIAAxACwAIAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAEQAUgBPAFAAKABwAGEAYwBrAGUAZABfAGIAYQBzAGUAYwBhAHMAZQBfAHIAZQBzAHUAbAB0ACwAIABuAHUAbQBfAGwAaQBtAGIAcwBfAHIAIAArACAAMQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABbAEkAbgB0AGUAcgBuAGEAbABdACAAQwBvAG0AcAB1AHQAZQBzACAAdABoAGUAIABSAGUAYwBpAHAAcgBvAGMAYQBsACAAcAByAG8AZwByAGUAcwBzAGkAdgBlAGwAeQAgAHMAYwBhAGwAaQBuAGcAIAB1AHAAIAB0AG8AIAB0AGgAZQAgAEQAaQB2AGkAZABlAG4AZAAnAHMAIABwAHIAZQBjAGkAcwBpAG8AbgAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGwAaQBtAGIAcwBfAGIAIABUAGgAZQAgAGQAaQB2AGkAcwBvAHIAIABsAGkAbQBiACAAYQByAHIAYQB5AC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAdABhAHIAZwBlAHQAXwBsAGUAbgAgAFQAaABlACAAbABpAG0AYgAtAGwAZQBuAGcAdABoACAAbwBmACAARABpAHYAaQBkAGUAbgBkACAAQQAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGsAIABUAGgAZQAgAGQAeQBuAGEAbQBpAGMAIABjAGgAdQBuAGsAIABzAGkAegBlACAAYwBvAG4AdABlAHgAdAAuAFwAbgAgACoALwBcAG4ATgBlAHcAdABvAG4AUgBhAHAAaABzAG8AbgBSAGUAYwBpAHAAcgBvAGMAYQBsACAAPQAgAEwAQQBNAEIARABBACgAbABpAG0AYgBzAF8AYgAsACAAdABhAHIAZwBlAHQAXwBsAGUAbgAsACAAawAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABuAHUAbQBfAGwAaQBtAGIAcwBfAGIALAAgAFIATwBXAFMAKABsAGkAbQBiAHMAXwBiACkALABcAG4AIAAgACAAIAAgACAAIAAgAG4AdQBtAF8AcwBlAGUAZABfAGwAaQBtAGIAcwAsACAATQBJAE4AKAAzACwAIABuAHUAbQBfAGwAaQBtAGIAcwBfAGIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AcgBfAHMAZQBlAGQALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAE4AZQB3AHQAbwBuAFIAYQBwAGgAcwBvAG4AUwBlAGUAZAAoAGwAaQBtAGIAcwBfAGIALAAgAGsAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAHIAZQBxAHUAaQByAGUAZABfAGkAdABlAHIAYQB0AGkAbwBuAHMALAAgAE0AQQBYACgAMAAsACAAQwBFAEkATABJAE4ARwAuAE0AQQBUAEgAKABMAE4AKAB0AGEAcgBnAGUAdABfAGwAZQBuACAALwAgAG4AdQBtAF8AcwBlAGUAZABfAGwAaQBtAGIAcwApACAALwAgAEwATgAoADIAKQApACkAIAArACAAMQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAHIAZQBxAHUAaQByAGUAZABfAGkAdABlAHIAYQB0AGkAbwBuAHMAIAA9ACAAMAAsACAAbABpAG0AYgBzAF8AcgBfAHMAZQBlAGQALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABpAHQAZQByAGEAdABpAG8AbgBzACwAIABTAEUAUQBVAEUATgBDAEUAKAByAGUAcQB1AGkAcgBlAGQAXwBpAHQAZQByAGEAdABpAG8AbgBzACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABmAGkAbgBhAGwAXwBwAGEAYwBrAGUAZABfAHMAdABhAHQAZQAsACAAUgBFAEQAVQBDAEUAKABWAFMAVABBAEMASwAoAG4AdQBtAF8AcwBlAGUAZABfAGwAaQBtAGIAcwAsACAAbABpAG0AYgBzAF8AcgBfAHMAZQBlAGQAKQAsACAAaQB0AGUAcgBhAHQAaQBvAG4AcwAsACAATABBAE0AQgBEAEEAKABwAGEAYwBrAGUAZABfAHMAdABhAHQAZQAsACAAaQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAYwB1AHIAcgBlAG4AdABfAGwAZQBuACwAIABJAE4ARABFAFgAKABwAGEAYwBrAGUAZABfAHMAdABhAHQAZQAsACAAMQAsACAAMQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGMAdQByAHIAZQBuAHQAXwByACwAIABEAFIATwBQACgAcABhAGMAawBlAGQAXwBzAHQAYQB0AGUALAAgADEAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbgBlAHgAdABfAGwAZQBuACwAIABNAEkATgAoAGMAdQByAHIAZQBuAHQAXwBsAGUAbgAgACoAIAAyACwAIAB0AGEAcgBnAGUAdABfAGwAZQBuACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAEQAeQBuAGEAbQBpAGMAIABTAGMAYQBsAGkAbgBnACAAUwBoAGkAZgB0ADoAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAEkAZgAgAEIAIABoAGEAcwAgAHAAbABhAHQAZQBhAHUAZQBkACwAIABSACAAbQB1AHMAdAAgAHMAYwBhAGwAZQAgAGIAeQAgADIAKgAoAG4ALQBtACkALgAgAEkAZgAgAEIAIABpAHMAIABnAHIAbwB3AGkAbgBnACwAIABSACAAcwBjAGEAbABlAHMAIABiAHkAIAAoAG4ALQBtACkALgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAYQBjAHQAaQB2AGUAXwBiAF8AbABpAG0AYgBzAF8AYwB1AHIAcgBlAG4AdAAsACAATQBJAE4AKABjAHUAcgByAGUAbgB0AF8AbABlAG4ALAAgAG4AdQBtAF8AbABpAG0AYgBzAF8AYgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGEAYwB0AGkAdgBlAF8AYgBfAGwAaQBtAGIAcwBfAG4AZQB4AHQALAAgAE0ASQBOACgAbgBlAHgAdABfAGwAZQBuACwAIABuAHUAbQBfAGwAaQBtAGIAcwBfAGIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAByAGUAcQB1AGkAcgBlAGQAXwBzAGgAaQBmAHQAXwBsAGkAbQBiAHMALAAgADIAIAAqACAAKABuAGUAeAB0AF8AbABlAG4AIAAtACAAYwB1AHIAcgBlAG4AdABfAGwAZQBuACkAIAAtACAAKABhAGMAdABpAHYAZQBfAGIAXwBsAGkAbQBiAHMAXwBuAGUAeAB0ACAALQAgAGEAYwB0AGkAdgBlAF8AYgBfAGwAaQBtAGIAcwBfAGMAdQByAHIAZQBuAHQAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AcgBfAHAAcgBpAG0AZQAsACAASQBGACgAcgBlAHEAdQBpAHIAZQBkAF8AcwBoAGkAZgB0AF8AbABpAG0AYgBzACAAPgAgADAALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABWAFMAVABBAEMASwAoAEUAWABQAEEATgBEACgAMAAsACAAcgBlAHEAdQBpAHIAZQBkAF8AcwBoAGkAZgB0AF8AbABpAG0AYgBzACwAIAAsACAAMAApACwAIABsAGkAbQBiAHMAXwBjAHUAcgByAGUAbgB0AF8AcgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYwB1AHIAcgBlAG4AdABfAHIAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGIAXwBhAGMAdABpAHYAZQAsACAAVABBAEsARQAoAGwAaQBtAGIAcwBfAGIALAAgAC0AYQBjAHQAaQB2AGUAXwBiAF8AbABpAG0AYgBzAF8AbgBlAHgAdAApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIABQACAAaQBzACAAbgBhAHQAaQB2AGUAbAB5ACAAYQBsAGkAZwBuAGUAZAAgAHQAbwAgADIAKgBuAGUAeAB0AF8AbABlAG4AIABiAGUAYwBhAHUAcwBlACAAbwBmACAAdABoAGUAIABjAG8AcgByAGUAYwB0AGUAZAAgAHMAaABpAGYAdABfAGwAaQBtAGIAcwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AcAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBNAHUAbAAoAGwAaQBtAGIAcwBfAGIAXwBhAGMAdABpAHYAZQAsACAAbABpAG0AYgBzAF8AcgBfAHAAcgBpAG0AZQAsACAAawApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwB0AHcAbwBfAGIAZQB0AGEALAAgAFYAUwBUAEEAQwBLACgARQBYAFAAQQBOAEQAKAAwACwAIAAyACAAKgAgAG4AZQB4AHQAXwBsAGUAbgAsACAALAAgADAAKQAsACAAMgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGUAcgByAG8AcgBfAHQAZQByAG0ALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFUAUwB1AGIAKABsAGkAbQBiAHMAXwB0AHcAbwBfAGIAZQB0AGEALAAgAGwAaQBtAGIAcwBfAHAALAAgAGsAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AbgBlAHgAdABfAHIAXwB1AG4AcwBjAGEAbABlAGQALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFUATQB1AGwAKABsAGkAbQBiAHMAXwByAF8AcAByAGkAbQBlACwAIABsAGkAbQBiAHMAXwBlAHIAcgBvAHIAXwB0AGUAcgBtACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AbgBlAHgAdABfAHIALAAgAEkARgAoAFIATwBXAFMAKABsAGkAbQBiAHMAXwBuAGUAeAB0AF8AcgBfAHUAbgBzAGMAYQBsAGUAZAApACAAPAA9ACAAMgAgACoAIABuAGUAeAB0AF8AbABlAG4ALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAB7ADAAfQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEQAUgBPAFAAKABsAGkAbQBiAHMAXwBuAGUAeAB0AF8AcgBfAHUAbgBzAGMAYQBsAGUAZAAsACAAMgAgACoAIABuAGUAeAB0AF8AbABlAG4AKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAVgBTAFQAQQBDAEsAKABuAGUAeAB0AF8AbABlAG4ALAAgAGwAaQBtAGIAcwBfAG4AZQB4AHQAXwByACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEQAUgBPAFAAKABmAGkAbgBhAGwAXwBwAGEAYwBrAGUAZABfAHMAdABhAHQAZQAsACAAMQApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAAWwBJAG4AdABlAHIAbgBhAGwAXQAgAEgAZQBhAHYAeQB3AGUAaQBnAGgAdAAgAE4AZQB3AHQAbwBuAC0AUgBhAHAAaABzAG8AbgAgAEQAaQB2AGkAcwBpAG8AbgAuAFwAbgAgACoAIABJAG0AcABsAGUAbQBlAG4AdABzACAAcAByAG8AZwByAGUAcwBzAGkAdgBlACAAcwBjAGEAbABpAG4AZwAgAGIAbwB1AG4AZABlAGQAIAB0AG8AIABNAEEAWAAoAGwAZQBuAF8AYQAsACAAbABlAG4AXwBiACkALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABsAGkAbQBiAHMAXwBhACAAVABoAGUAIABkAGkAdgBpAGQAZQBuAGQAIABhAHIAcgBhAHkALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABsAGkAbQBiAHMAXwBiACAAVABoAGUAIABkAGkAdgBpAHMAbwByACAAYQByAHIAYQB5AC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAawAgAFQAaABlACAAZAB5AG4AYQBtAGkAYwAgAGMAaAB1AG4AawAgAHMAaQB6AGUAIABjAG8AbgB0AGUAeAB0AC4AXABuACAAKgAvAFwAbgBOAGUAdwB0AG8AbgBSAGEAcABoAHMAbwBuAEQAaQB2ACAAPQAgAEwAQQBNAEIARABBACgAbABpAG0AYgBzAF8AYQAsACAAbABpAG0AYgBzAF8AYgAsACAAawAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABuAHUAbQBfAGwAaQBtAGIAcwBfAGEALAAgAFIATwBXAFMAKABsAGkAbQBiAHMAXwBhACkALABcAG4AIAAgACAAIAAgACAAIAAgAG4AdQBtAF8AbABpAG0AYgBzAF8AYgAsACAAUgBPAFcAUwAoAGwAaQBtAGIAcwBfAGIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbgB1AG0AXwBsAGkAbQBiAHMAXwB0AGEAcgBnAGUAdAAsACAATQBBAFgAKABuAHUAbQBfAGwAaQBtAGIAcwBfAGEALAAgAG4AdQBtAF8AbABpAG0AYgBzAF8AYgApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAALwAvACAAMQAuACAAQwBhAGwAYwB1AGwAYQB0AGUAIAByAGUAYwBpAHAAcgBvAGMAYQBsACAAUgAgAHMAYwBhAGwAZQBkACAAZAB5AG4AYQBtAGkAYwBhAGwAbAB5ACAAdABvACAAMgAgACoAIAB0AGEAcgBnAGUAdABfAGwAZQBuAFwAbgAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AcgBlAGMAaQBwAHIAbwBjAGEAbAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4ATgBlAHcAdABvAG4AUgBhAHAAaABzAG8AbgBSAGUAYwBpAHAAcgBvAGMAYQBsACgAbABpAG0AYgBzAF8AYgAsACAAbgB1AG0AXwBsAGkAbQBiAHMAXwB0AGEAcgBnAGUAdAAsACAAawApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAALwAvACAAMgAuACAAQQBwAHAAcgBvAHgAaQBtAGEAdABlACAAUQB1AG8AdABpAGUAbgB0ADoAIABRAF8AYQBwAHAAcgBvAHgAIAA9ACAAQQAgACoAIABSACAALwAgAEIAZQB0AGEAXgAoADIAIAAqACAAdABhAHIAZwBlAHQAXwBsAGUAbgApAFwAbgAgACAAIAAgACAAIAAgACAAcgBpAGcAaAB0AF8AcwBoAGkAZgB0AF8AbABpAG0AYgBzACwAIAAyACAAKgAgAG4AdQBtAF8AbABpAG0AYgBzAF8AdABhAHIAZwBlAHQALABcAG4AIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAHEAXwB1AG4AcwBjAGEAbABlAGQALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFUATQB1AGwAKABsAGkAbQBiAHMAXwBhACwAIABsAGkAbQBiAHMAXwByAGUAYwBpAHAAcgBvAGMAYQBsACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAHEAXwBhAHAAcAByAG8AeAAsACAASQBGACgAUgBPAFcAUwAoAGwAaQBtAGIAcwBfAHEAXwB1AG4AcwBjAGEAbABlAGQAKQAgADwAPQAgAHIAaQBnAGgAdABfAHMAaABpAGYAdABfAGwAaQBtAGIAcwAsACAAewAwAH0ALAAgAEQAUgBPAFAAKABsAGkAbQBiAHMAXwBxAF8AdQBuAHMAYwBhAGwAZQBkACwAIAByAGkAZwBoAHQAXwBzAGgAaQBmAHQAXwBsAGkAbQBiAHMAKQApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAALwAvACAAQwBhAGwAYwB1AGwAYQB0AGUAIAB0AGgAZQAgAG0AYQBzAHMAaQB2AGUAIABiAGEAcwBlAGwAaQBuAGUAIABwAHIAbwBkAHUAYwB0ACAAZQB4AGEAYwB0AGwAeQAgAE8ATgBDAEUAXABuACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBwAF8AYgBhAHMAZQBsAGkAbgBlACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAE0AdQBsACgAbABpAG0AYgBzAF8AYgAsACAAbABpAG0AYgBzAF8AcQBfAGEAcABwAHIAbwB4ACwAIABrACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAvAC8AIAAzAC4AIABCAG8AdQBuAGQAZQBkACAARQByAHIAbwByACAAQwBvAHIAcgBlAGMAdABpAG8AbgAgAFMAdwBlAGUAcAAgACgATwBwAHQAaQBtAGkAegBlAGQAIABPACgATgApACAAUwB0AGUAcABwAGkAbgBnACkAXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABTAHQAYQB0AGUAIABwAGEAYwBrAGkAbgBnADoAIABWAFMAVABBAEMASwAoAEwAZQBuAGcAdABoAF8AUQAsACAAUQBfAGwAaQBtAGIAcwAsACAAUABfAGwAaQBtAGIAcwApAFwAbgAgACAAIAAgACAAIAAgACAAaQBuAGkAdABpAGEAbABfAHAAYQBjAGsAZQBkAF8AcwB0AGEAdABlACwAIABWAFMAVABBAEMASwAoAFIATwBXAFMAKABsAGkAbQBiAHMAXwBxAF8AYQBwAHAAcgBvAHgAKQAsACAAbABpAG0AYgBzAF8AcQBfAGEAcABwAHIAbwB4ACwAIABsAGkAbQBiAHMAXwBwAF8AYgBhAHMAZQBsAGkAbgBlACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABTAHcAZQBlAHAAIABEAG8AdwBuADoAIABJAGYAIABQACAAPgAgAEEALAAgAFEAIABpAHMAIAB0AG8AbwAgAGIAaQBnAC4AIABTAHQAZQBwACAAUQAgAGQAbwB3AG4AIABiAHkAIAAxACwAIABhAG4AZAAgAFAAIABkAG8AdwBuACAAYgB5ACAAQgAuAFwAbgAgACAAIAAgACAAIAAgACAAcABhAGMAawBlAGQAXwBzAHQAYQB0AGUAXwBzAHcAZQBwAHQAXwBkAG8AdwBuACwAIABSAEUARABVAEMARQAoAGkAbgBpAHQAaQBhAGwAXwBwAGEAYwBrAGUAZABfAHMAdABhAHQAZQAsACAAewAxADsAIAAyAH0ALAAgAEwAQQBNAEIARABBACgAcABhAGMAawBlAGQAXwBzAHQAYQB0AGUALAAgAGkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGUAbgBfAHEALAAgAEkATgBEAEUAWAAoAHAAYQBjAGsAZQBkAF8AcwB0AGEAdABlACwAIAAxACwAIAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBjAHUAcgByAGUAbgB0AF8AcQAsACAAQwBIAE8ATwBTAEUAUgBPAFcAUwAoAHAAYQBjAGsAZQBkAF8AcwB0AGEAdABlACwAIABTAEUAUQBVAEUATgBDAEUAKABsAGUAbgBfAHEALAAgADEALAAgADIAKQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYwB1AHIAcgBlAG4AdABfAHAALAAgAEQAUgBPAFAAKABwAGEAYwBrAGUAZABfAHMAdABhAHQAZQAsACAAbABlAG4AXwBxACAAKwAgADEAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAEMAbwBtAHAAYQByAGUAKABsAGkAbQBiAHMAXwBjAHUAcgByAGUAbgB0AF8AcAAsACAAbABpAG0AYgBzAF8AYQApACAAPAA9ACAAMAAsACAAcABhAGMAawBlAGQAXwBzAHQAYQB0AGUALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAG4AZQB4AHQAXwBxACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAFMAdQBiACgAbABpAG0AYgBzAF8AYwB1AHIAcgBlAG4AdABfAHEALAAgAHsAMQB9ACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AbgBlAHgAdABfAHAALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFUAUwB1AGIAKABsAGkAbQBiAHMAXwBjAHUAcgByAGUAbgB0AF8AcAAsACAAbABpAG0AYgBzAF8AYgAsACAAawApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFYAUwBUAEEAQwBLACgAUgBPAFcAUwAoAGwAaQBtAGIAcwBfAG4AZQB4AHQAXwBxACkALAAgAGwAaQBtAGIAcwBfAG4AZQB4AHQAXwBxACwAIABsAGkAbQBiAHMAXwBuAGUAeAB0AF8AcAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACkAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAC8ALwAgAFMAdwBlAGUAcAAgAFUAcAA6ACAASQBmACAAUAAgACsAIABCACAAPAA9ACAAQQAsACAAUQAgAGkAcwAgAHQAbwBvACAAcwBtAGEAbABsAC4AIABTAHQAZQBwACAAUQAgAHUAcAAgAGIAeQAgADEALAAgAGEAbgBkACAAUAAgAHUAcAAgAGIAeQAgAEIALgBcAG4AIAAgACAAIAAgACAAIAAgAHAAYQBjAGsAZQBkAF8AcwB0AGEAdABlAF8AcwB3AGUAcAB0AF8AdQBwACwAIABSAEUARABVAEMARQAoAHAAYQBjAGsAZQBkAF8AcwB0AGEAdABlAF8AcwB3AGUAcAB0AF8AZABvAHcAbgAsACAAewAxADsAIAAyAH0ALAAgAEwAQQBNAEIARABBACgAcABhAGMAawBlAGQAXwBzAHQAYQB0AGUALAAgAGkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGUAbgBfAHEALAAgAEkATgBEAEUAWAAoAHAAYQBjAGsAZQBkAF8AcwB0AGEAdABlACwAIAAxACwAIAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBjAHUAcgByAGUAbgB0AF8AcQAsACAAQwBIAE8ATwBTAEUAUgBPAFcAUwAoAHAAYQBjAGsAZQBkAF8AcwB0AGEAdABlACwAIABTAEUAUQBVAEUATgBDAEUAKABsAGUAbgBfAHEALAAgADEALAAgADIAKQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYwB1AHIAcgBlAG4AdABfAHAALAAgAEQAUgBPAFAAKABwAGEAYwBrAGUAZABfAHMAdABhAHQAZQAsACAAbABlAG4AXwBxACAAKwAgADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAG4AZQB4AHQAXwBwAF8AdABlAHMAdAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBBAGQAZAAoAGwAaQBtAGIAcwBfAGMAdQByAHIAZQBuAHQAXwBwACwAIABsAGkAbQBiAHMAXwBiACwAIABrACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBDAG8AbQBwAGEAcgBlACgAbABpAG0AYgBzAF8AbgBlAHgAdABfAHAAXwB0AGUAcwB0ACwAIABsAGkAbQBiAHMAXwBhACkAIAA+ACAAMAAsACAAcABhAGMAawBlAGQAXwBzAHQAYQB0AGUALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAG4AZQB4AHQAXwBxACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAEEAZABkACgAbABpAG0AYgBzAF8AYwB1AHIAcgBlAG4AdABfAHEALAAgAHsAMQB9ACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAVgBTAFQAQQBDAEsAKABSAE8AVwBTACgAbABpAG0AYgBzAF8AbgBlAHgAdABfAHEAKQAsACAAbABpAG0AYgBzAF8AbgBlAHgAdABfAHEALAAgAGwAaQBtAGIAcwBfAG4AZQB4AHQAXwBwAF8AdABlAHMAdAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACkAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAC8ALwAgAEUAeAB0AHIAYQBjAHQAIABGAGkAbgBhAGwAIABRACAAYQBuAGQAIABQAFwAbgAgACAAIAAgACAAIAAgACAAbABlAG4AXwBxACwAIABJAE4ARABFAFgAKABwAGEAYwBrAGUAZABfAHMAdABhAHQAZQBfAHMAdwBlAHAAdABfAHUAcAAsACAAMQAsACAAMQApACwAXABuACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBxACwAIABDAEgATwBPAFMARQBSAE8AVwBTACgAcABhAGMAawBlAGQAXwBzAHQAYQB0AGUAXwBzAHcAZQBwAHQAXwB1AHAALAAgAFMARQBRAFUARQBOAEMARQAoAGwAZQBuAF8AcQAsACAAMQAsACAAMgApACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAHAALAAgAEQAUgBPAFAAKABwAGEAYwBrAGUAZABfAHMAdABhAHQAZQBfAHMAdwBlAHAAdABfAHUAcAAsACAAbABlAG4AXwBxACAAKwAgADEAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAC8ALwAgADQALgAgAEUAeAB0AHIAYQBjAHQAIABUAHIAdQBlACAAUgBlAG0AYQBpAG4AZABlAHIAIABTAGEAZgBlAGwAeQAgACgAQQAgAC0AIABGAGkAbgBhAGwAXwBQACkAXABuACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwByACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAFMAdQBiACgAbABpAG0AYgBzAF8AYQAsACAAbABpAG0AYgBzAF8AcAAsACAAawApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAVgBTAFQAQQBDAEsAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBPAFcAUwAoAGwAaQBtAGIAcwBfAHIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwByACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAHEAXABuACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABbAEkAbgB0AGUAcgBuAGEAbABdACAAVQBuAHMAaQBnAG4AZQBkACAAQgBhAHMAZQAtADEAMAAgAEwAZQBmAHQALQB0AG8ALQBSAGkAZwBoAHQAIABFAHgAcABvAG4AZQBuAHQAaQBhAHQAaQBvAG4ALgBcAG4AIAAqACAARQB2AGEAbAB1AGEAdABlAHMAIAB0AGgAZQAgAGUAeABwAG8AbgBlAG4AdAAgAGkAdABlAHIAYQB0AGkAdgBlAGwAeQAgAHUAcwBpAG4AZwAgAGEAIABwAHIAZQAtAGMAbwBtAHAAdQB0AGUAZAAgADEALQA5ACAAYwBhAGMAaABlAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAbABpAG0AYgBzAF8AYgBhAHMAZQAgAFQAaABlACAAbABpAHQAdABsAGUALQBlAG4AZABpAGEAbgAgAGwAaQBtAGIAIABhAHIAcgBhAHkAIABvAGYAIAB0AGgAZQAgAGIAYQBzAGUALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABlAHgAcABfAHMAdAByAGkAbgBnACAAVABoAGUAIABlAHgAYQBjAHQAIAB0AGUAeAB0ACAAcwB0AHIAaQBuAGcAIABvAGYAIAB0AGgAZQAgAGUAeABwAG8AbgBlAG4AdAAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGsAIABUAGgAZQAgAGQAeQBuAGEAbQBpAGMAIABjAGgAdQBuAGsAIABzAGkAegBlACAAYwBvAG4AdABlAHgAdAAuAFwAbgAgACoALwBcAG4AVQBQAG8AdwAgAD0AIABMAEEATQBCAEQAQQAoAGwAaQBtAGIAcwBfAGIAYQBzAGUALAAgAGUAeABwAG8AbgBlAG4AdABfAHMAdAByAGkAbgBnACwAIABrACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAC8ALwAgAFAAcgBlAC0AYwBvAG0AcAB1AHQAZQAgAHAAbwB3AGUAcgBzACAAMQAgAHQAaAByAG8AdQBnAGgAIAA5AC4AXABuACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBiAGEAcwBlADEALAAgAGwAaQBtAGIAcwBfAGIAYQBzAGUALABcAG4AIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGIAYQBzAGUAMgAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBNAHUAbAAoAGwAaQBtAGIAcwBfAGIAYQBzAGUAMQAsACAAbABpAG0AYgBzAF8AYgBhAHMAZQAxACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGIAYQBzAGUAMwAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBNAHUAbAAoAGwAaQBtAGIAcwBfAGIAYQBzAGUAMgAsACAAbABpAG0AYgBzAF8AYgBhAHMAZQAxACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGIAYQBzAGUANAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBNAHUAbAAoAGwAaQBtAGIAcwBfAGIAYQBzAGUAMgAsACAAbABpAG0AYgBzAF8AYgBhAHMAZQAyACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGIAYQBzAGUANQAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBNAHUAbAAoAGwAaQBtAGIAcwBfAGIAYQBzAGUANAAsACAAbABpAG0AYgBzAF8AYgBhAHMAZQAxACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGIAYQBzAGUANgAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBNAHUAbAAoAGwAaQBtAGIAcwBfAGIAYQBzAGUAMwAsACAAbABpAG0AYgBzAF8AYgBhAHMAZQAzACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGIAYQBzAGUANwAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBNAHUAbAAoAGwAaQBtAGIAcwBfAGIAYQBzAGUANgAsACAAbABpAG0AYgBzAF8AYgBhAHMAZQAxACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGIAYQBzAGUAOAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBNAHUAbAAoAGwAaQBtAGIAcwBfAGIAYQBzAGUANAAsACAAbABpAG0AYgBzAF8AYgBhAHMAZQA0ACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGIAYQBzAGUAOQAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBNAHUAbAAoAGwAaQBtAGIAcwBfAGIAYQBzAGUAOAAsACAAbABpAG0AYgBzAF8AYgBhAHMAZQAxACwAIABrACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIABlAHgAcABvAG4AZQBuAHQAXwBkAGkAZwBpAHQAcwAsACAALQAtAE0ASQBEACgAZQB4AHAAbwBuAGUAbgB0AF8AcwB0AHIAaQBuAGcALAAgAFMARQBRAFUARQBOAEMARQAoAEwARQBOACgAZQB4AHAAbwBuAGUAbgB0AF8AcwB0AHIAaQBuAGcAKQApACwAIAAxACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIABSAEUARABVAEMARQAoADEALAAgAGUAeABwAG8AbgBlAG4AdABfAGQAaQBnAGkAdABzACwAIABMAEEATQBCAEQAQQAoAGwAaQBtAGIAcwBfAGEAYwBjAHUAbQB1AGwAYQB0AG8AcgAsACAAYwB1AHIAcgBlAG4AdABfAGQAaQBnAGkAdAAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAFMAaABvAHIAdAAtAGMAaQByAGMAdQBpAHQAOgAgAFMAawBpAHAAIABjAGEAbABjAHUAbABhAHQAaQBuAGcAIAAxAF4AMQAwACAAZAB1AHIAaQBuAGcAIABsAGUAYQBkAGkAbgBnACAAaQB0AGUAcgBhAHQAaQBvAG4AcwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABpAHMAXwBvAG4AZQAsACAAQQBOAEQAKABSAE8AVwBTACgAbABpAG0AYgBzAF8AYQBjAGMAdQBtAHUAbABhAHQAbwByACkAIAA9ACAAMQAsACAASQBOAEQARQBYACgAbABpAG0AYgBzAF8AYQBjAGMAdQBtAHUAbABhAHQAbwByACwAIAAxACwAIAAxACkAIAA9ACAAMQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAAMQAuACAAUgBhAGkAcwBlACAAQQBjAGMAIAB0AG8AIAB0AGgAZQAgADEAMAB0AGgAIABwAG8AdwBlAHIAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYQBjAGMAXwAxADAALAAgAEkARgAoAGkAcwBfAG8AbgBlACwAIABsAGkAbQBiAHMAXwBhAGMAYwB1AG0AdQBsAGEAdABvAHIALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGEAYwBjAF8AMgAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBNAHUAbAAoAGwAaQBtAGIAcwBfAGEAYwBjAHUAbQB1AGwAYQB0AG8AcgAsACAAbABpAG0AYgBzAF8AYQBjAGMAdQBtAHUAbABhAHQAbwByACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYQBjAGMAXwA0ACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAE0AdQBsACgAbABpAG0AYgBzAF8AYQBjAGMAXwAyACwAIABsAGkAbQBiAHMAXwBhAGMAYwBfADIALAAgAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBhAGMAYwBfADgALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFUATQB1AGwAKABsAGkAbQBiAHMAXwBhAGMAYwBfADQALAAgAGwAaQBtAGIAcwBfAGEAYwBjAF8ANAAsACAAawApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFUATQB1AGwAKABsAGkAbQBiAHMAXwBhAGMAYwBfADgALAAgAGwAaQBtAGIAcwBfAGEAYwBjAF8AMgAsACAAawApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgADIALgAgAE0AdQBsAHQAaQBwAGwAeQAgAGIAeQAgAHQAaABlACAAYwBvAHIAcgBlAHMAcABvAG4AZABpAG4AZwAgAGMAYQBjAGgAZQBkACAAdgBhAGwAdQBlAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEkARgAoAGMAdQByAHIAZQBuAHQAXwBkAGkAZwBpAHQAIAA9ACAAMAAsACAAbABpAG0AYgBzAF8AYQBjAGMAXwAxADAALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGMAYQBjAGgAZQBfAG0AdQBsAHQAaQBwAGwAaQBlAHIALAAgAEMASABPAE8AUwBFACgAYwB1AHIAcgBlAG4AdABfAGQAaQBnAGkAdAAsACAAbABpAG0AYgBzAF8AYgBhAHMAZQAxACwAIABsAGkAbQBiAHMAXwBiAGEAcwBlADIALAAgAGwAaQBtAGIAcwBfAGIAYQBzAGUAMwAsACAAbABpAG0AYgBzAF8AYgBhAHMAZQA0ACwAIABsAGkAbQBiAHMAXwBiAGEAcwBlADUALAAgAGwAaQBtAGIAcwBfAGIAYQBzAGUANgAsACAAbABpAG0AYgBzAF8AYgBhAHMAZQA3ACwAIABsAGkAbQBiAHMAXwBiAGEAcwBlADgALAAgAGwAaQBtAGIAcwBfAGIAYQBzAGUAOQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEkARgAoAGkAcwBfAG8AbgBlACwAIABsAGkAbQBiAHMAXwBjAGEAYwBoAGUAXwBtAHUAbAB0AGkAcABsAGkAZQByACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAE0AdQBsACgAbABpAG0AYgBzAF8AYQBjAGMAXwAxADAALAAgAGwAaQBtAGIAcwBfAGMAYQBjAGgAZQBfAG0AdQBsAHQAaQBwAGwAaQBlAHIALAAgAGsAKQApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABbAEkAbgB0AGUAcgBuAGEAbABdACAAVQBuAHMAaQBnAG4AZQBkACAASQBuAHQAZQBnAGUAcgAgAFMAcQB1AGEAcgBlACAAUgBvAG8AdAAgAHUAcwBpAG4AZwAgAE4AZQB3AHQAbwBuACcAcwAgAE0AZQB0AGgAbwBkAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAbABpAG0AYgBzAF8AcgBhAGQAaQBjAGEAbgBkAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAbABpAG0AYgBzAF8AaQBuAGkAdABpAGEAbABfAHgAIABPAHYAZQByAC0AZQBzAHQAaQBtAGEAdABlAGQAIABzAGUAZQBkACAAYQByAHIAYQB5AC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAawAgAFQAaABlACAAZAB5AG4AYQBtAGkAYwAgAGMAaAB1AG4AawAgAHMAaQB6AGUAIABjAG8AbgB0AGUAeAB0AC4AXABuACAAKgAvAFwAbgBVAFMAcQByAHQAIAA9ACAATABBAE0AQgBEAEEAKABsAGkAbQBiAHMAXwByAGEAZABpAGMAYQBuAGQALAAgAGwAaQBtAGIAcwBfAGkAbgBpAHQAaQBhAGwAXwB4ACwAIABrACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQB4AGkAbQB1AG0AXwBpAHQAZQByAGEAdABpAG8AbgBzACwAIAAzADUALABcAG4AXABuACAAIAAgACAAIAAgACAAIABmAGkAbgBhAGwAXwBwAGEAYwBrAGUAZABfAHMAdABhAHQAZQAsACAAUgBFAEQAVQBDAEUAKABWAFMAVABBAEMASwAoADAALAAgAGwAaQBtAGIAcwBfAGkAbgBpAHQAaQBhAGwAXwB4ACkALAAgAFMARQBRAFUARQBOAEMARQAoAG0AYQB4AGkAbQB1AG0AXwBpAHQAZQByAGEAdABpAG8AbgBzACkALAAgAEwAQQBNAEIARABBACgAcABhAGMAawBlAGQAXwBzAHQAYQB0AGUALAAgAGkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABoAGEAcwBfAGMAbwBuAHYAZQByAGcAZQBkACwAIABJAE4ARABFAFgAKABwAGEAYwBrAGUAZABfAHMAdABhAHQAZQAsACAAMQAsACAAMQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYwB1AHIAcgBlAG4AdABfAHgALAAgAEQAUgBPAFAAKABwAGEAYwBrAGUAZABfAHMAdABhAHQAZQAsACAAMQApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEkARgAoAGgAYQBzAF8AYwBvAG4AdgBlAHIAZwBlAGQALAAgAHAAYQBjAGsAZQBkAF8AcwB0AGEAdABlACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIAAxAC4AIABEAGkAdgBpAHMAaQBvAG4AOgAgAG4AIAAvACAAeABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcABhAGMAawBlAGQAXwBkAGkAdgBpAHMAaQBvAG4AXwByAGUAcwB1AGwAdAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4ARABpAHYAUgBvAHUAdABlAHIAKABsAGkAbQBiAHMAXwByAGEAZABpAGMAYQBuAGQALAAgAGwAaQBtAGIAcwBfAGMAdQByAHIAZQBuAHQAXwB4ACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbgB1AG0AXwBsAGkAbQBiAHMAXwByACwAIABJAE4ARABFAFgAKABwAGEAYwBrAGUAZABfAGQAaQB2AGkAcwBpAG8AbgBfAHIAZQBzAHUAbAB0ACwAIAAxACwAIAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AcQAsACAARABSAE8AUAAoAHAAYQBjAGsAZQBkAF8AZABpAHYAaQBzAGkAbwBuAF8AcgBlAHMAdQBsAHQALAAgAG4AdQBtAF8AbABpAG0AYgBzAF8AcgAgACsAIAAxACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgADIALgAgAEEAZABkAGkAdABpAG8AbgA6ACAAeAAgACsAIAAoAG4AIAAvACAAeAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBzAHUAbQBfAHgAcQAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBBAGQAZAAoAGwAaQBtAGIAcwBfAGMAdQByAHIAZQBuAHQAXwB4ACwAIABsAGkAbQBiAHMAXwBxACwAIABrACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgADMALgAgAEgAYQBsAHYAaQBuAGcAOgAgACgAeAAgACsAIAAoAG4AIAAvACAAeAApACkAIAAvACAAMgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAASwBuAHUAdABoAEQAaQB2ACAAaQBuAGgAZQByAGUAbgB0AGwAeQAgAHMAdQBwAHAAbwByAHQAcwAgAHMAYwBhAGwAYQByACAAZABpAHYAaQBzAG8AcgBzACAAdwBpAHQAaAAgAHoAZQByAG8AIABvAHYAZQByAGgAZQBhAGQAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHAAYQBjAGsAZQBkAF8AaABhAGwAZgBfAHIAZQBzAHUAbAB0ACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBLAG4AdQB0AGgARABpAHYAKABsAGkAbQBiAHMAXwBzAHUAbQBfAHgAcQAsACAAewAyAH0ALAAgAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABuAHUAbQBfAGwAaQBtAGIAcwBfAGgAYQBsAGYAZQBkACwAIABJAE4ARABFAFgAKABwAGEAYwBrAGUAZABfAGgAYQBsAGYAXwByAGUAcwB1AGwAdAAsACAAMQAsACAAMQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAG4AZQB4AHQAXwB4ACwAIABEAFIATwBQACgAcABhAGMAawBlAGQAXwBoAGEAbABmAF8AcgBlAHMAdQBsAHQALAAgAG4AdQBtAF8AbABpAG0AYgBzAF8AaABhAGwAZgBlAGQAIAArACAAMQApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIAA0AC4AIABDAG8AbgB2AGUAcgBnAGUAbgBjAGUAIABDAGgAZQBjAGsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGMAbwBuAHYAZQByAGcAZQBuAGMAZQBfAGMAbwBtAHAAYQByAGkAcwBvAG4ALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFUAQwBvAG0AcABhAHIAZQAoAGwAaQBtAGIAcwBfAG4AZQB4AHQAXwB4ACwAIABsAGkAbQBiAHMAXwBjAHUAcgByAGUAbgB0AF8AeAApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIABOAGUAdwB0AG8AbgAnAHMAIABtAGUAdABoAG8AZAAgAGMAbwBuAHYAZQByAGcAZQBzACAAbwBuACAAdABoAGUAIABmAGwAbwBvAHIAIAByAG8AbwB0ACwAIABhAG4AZAAgAHMAdABhAGIAaQBsAGkAegBlAHMAIABvAHIAIABvAHMAYwBpAGwAbABhAHQAZQBzACAAdQBwACAAYgB5ACAAMQAuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIABUAGgAZQByAGUAZgBvAHIAZQAsACAAaQBmACAAeABfAG4AZQB4AHQAIAA+AD0AIABjAHUAcgByAF8AeAAsACAAdABoAGUAIABhAGwAZwBvAHIAaQB0AGgAbQAgAGgAYQBzACAAYwBvAG4AdgBlAHIAZwBlAGQALgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgAYwBvAG4AdgBlAHIAZwBlAG4AYwBlAF8AYwBvAG0AcABhAHIAaQBzAG8AbgAgAD4APQAgADAALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABWAFMAVABBAEMASwAoADEALAAgAGwAaQBtAGIAcwBfAGMAdQByAHIAZQBuAHQAXwB4ACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABWAFMAVABBAEMASwAoADAALAAgAGwAaQBtAGIAcwBfAG4AZQB4AHQAXwB4ACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAApACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIABEAFIATwBQACgAZgBpAG4AYQBsAF8AcABhAGMAawBlAGQAXwBzAHQAYQB0AGUALAAgADEAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAAWwBJAG4AdABlAHIAbgBhAGwAXQAgAEcAZQBuAGUAcgBhAHQAZQBzACAAYQAgADEARAAgAHYAZQByAHQAaQBjAGEAbAAgAGEAcgByAGEAeQAgAG8AZgAgAGEAbABsACAAcAByAGkAbQBlACAAbgB1AG0AYgBlAHIAcwAgAHUAcAAgAHQAbwAgAG4ALgBcAG4AIAAqACAARQB2AGEAbAB1AGEAdABlAHMAIABwAHUAcgBlAGwAeQAgAGkAbgAgAG4AYQB0AGkAdgBlACAAQwArACsAIAB1AHMAaQBuAGcAIABhACAAZAB5AG4AYQBtAGkAYwAgAHMAaQBlAHYAZQAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAG4AIABUAGgAZQAgAHUAcABwAGUAcgAgAGIAbwB1AG4AZAAgAGkAbgB0AGUAZwBlAHIAIAAoAGEAcwBzAHUAbQBlAGQAIAA8AD0AIAA5ADIANwAzACkALgBcAG4AIAAqAC8AXABuAE4AYQB0AGkAdgBlAFAAcgBpAG0AZQBzACAAPQAgAEwAQQBNAEIARABBACgAbgAsAFwAbgAgACAAIAAgAEkARgAoAG4AIAA8ACAAMgAsACAAIwBOAFUATQAhACwAXABuACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABjAGEAbgBkAGkAZABhAHQAZQBfAHMAZQBxAHUAZQBuAGMAZQAsACAAUwBFAFEAVQBFAE4AQwBFACgAbgAgAC0AIAAxACwAIAAxACwAIAAyACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABjAGEAbgBkAGkAZABhAHQAZQBfAHMAZQBxAHUAZQBuAGMAZQAsACAATQBBAFAAKABjAGEAbgBkAGkAZABhAHQAZQBfAHMAZQBxAHUAZQBuAGMAZQAsACAATABBAE0AQgBEAEEAKABjAHUAcgByAGUAbgB0AF8AYwBhAG4AZABpAGQAYQB0AGUALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AaQB0ACwAIABJAE4AVAAoAFMAUQBSAFQAKABjAHUAcgByAGUAbgB0AF8AYwBhAG4AZABpAGQAYQB0AGUAKQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABsAGkAbQBpAHQAIAA8ACAAMgAsACAAVABSAFUARQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEkATgAoAE0ATwBEACgAYwB1AHIAcgBlAG4AdABfAGMAYQBuAGQAaQBkAGEAdABlACwAIABTAEUAUQBVAEUATgBDAEUAKABsAGkAbQBpAHQAIAAtACAAMQAsACAAMQAsACAAMgApACkAKQAgAD4AIAAwAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAApACkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFsASQBuAHQAZQByAG4AYQBsAF0AIABVAG4AcwBhAGYAZQAsACAAaABpAGcAaAAtAHAAZQByAGYAbwByAG0AYQBuAGMAZQAgAHQAZQB4AHQAIABtAHUAbAB0AGkAcABsAGkAYwBhAHQAaQBvAG4AIABmAG8AcgAgAG4AbwByAG0AYQBsAGkAcwBlAGQALAAgAHAAbwBzAGkAdABpAHYAZQAgAEIAaQBnAEkAbgB0ACAAcwB0AHIAaQBuAGcAcwAuAFwAbgAgACoAIABCAHkAcABhAHMAcwBlAHMAIABMAGEAeQBlAHIAIAAwACAAdgBhAGwAaQBkAGEAdABpAG8AbgAuACAASQBtAHAAbABlAG0AZQBuAHQAcwAgAHMAdAByAGkAYwB0ACAAcwBoAG8AcgB0AC0AYwBpAHIAYwB1AGkAdABzACAAZgBvAHIAIABwAGEAZABkAGkAbgBnACAAbwBwAHQAaQBtAGkAegBhAHQAaQBvAG4ALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABuAG8AcgBtAF8AYQBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABuAG8AcgBtAF8AYgBcAG4AIAAqAC8AXABuAFUAVABlAHgAdABNAHUAbAAgAD0AIABMAEEATQBCAEQAQQAoAG4AbwByAG0AXwBhACwAIABuAG8AcgBtAF8AYgAsAFwAbgAgACAAIAAgAEkARgAoAE8AUgAoAG4AbwByAG0AXwBhACAAPQAgAFwAIgAwAFwAIgAsACAAbgBvAHIAbQBfAGIAIAA9ACAAXAAiADAAXAAiACkALAAgAFwAIgAwAFwAIgAsAFwAbgAgACAAIAAgAEkARgAoAG4AbwByAG0AXwBhACAAPQAgAFwAIgAxAFwAIgAsACAAbgBvAHIAbQBfAGIALABcAG4AIAAgACAAIABJAEYAKABuAG8AcgBtAF8AYgAgAD0AIABcACIAMQBcACIALAAgAG4AbwByAG0AXwBhACwAXABuACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGUAbgBfAGEALAAgAEwARQBOACgAbgBvAHIAbQBfAGEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGUAbgBfAGIALAAgAEwARQBOACgAbgBvAHIAbQBfAGIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABrACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBTAGEAZgBlAEsAKABcACIATQBVAEwAXAAiACwAIABNAEkATgAoAGwAZQBuAF8AYQAsACAAbABlAG4AXwBiACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYQAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwBwAGwAaQB0ACgAbgBvAHIAbQBfAGEALAAgAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBiACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBTAHAAbABpAHQAKABuAG8AcgBtAF8AYgAsACAAawApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABmAGkAbgBhAGwAXwBsAGkAbQBiAHMALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFUATQB1AGwAKABsAGkAbQBiAHMAXwBhACwAIABsAGkAbQBiAHMAXwBiACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAE0AZQByAGcAZQAoAGYAaQBuAGEAbABfAGwAaQBtAGIAcwAsACAAawApAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApACkAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFsASQBuAHQAZQByAG4AYQBsAF0AIABWAGUAYwB0AG8AcgBpAHoAZQBkACAAbABvAGcAYQByAGkAdABoAG0AaQBjACAAcAByAG8AZAB1AGMAdAAgAG8AZgAgAGEAbgAgAGEAcgByAGEAeQAgAG8AZgAgAEIAaQBnAEkAbgB0ACAAcwB0AHIAaQBuAGcAcwAuAFwAbgAgACoAIABSAGUAYwB1AHIAcwBpAHYAZQBsAHkAIABjAHUAdABzACAAdABoAGUAIABhAHIAcgBhAHkAIABpAG4AIABoAGEAbABmACAAdABvACAAYgB5AHAAYQBzAHMAIABSAEUARABVAEMARQAgAHMAZQBxAHUAZQBuAHQAaQBhAGwAIABtAGUAbQBvAHIAeQAgAGEAbABsAG8AYwBhAHQAaQBvAG4AcwAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGEAcgByAF8AcwB0AHIAaQBuAGcAcwAgAEEAIAAxAEQAIAB2AGUAcgB0AGkAYwBhAGwAIABhAHIAcgBhAHkAIABvAGYAIABCAGkAZwBJAG4AdAAgAHMAdAByAGkAbgBnAHMALgBcAG4AIAAqAC8AXABuAFQAZQB4AHQAVAByAGUAZQBQAHIAbwBkACAAPQAgAEwAQQBNAEIARABBACgAYQByAHIAXwBzAHQAcgBpAG4AZwBzACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG4AdQBtAF8AZQBsAGUAbQBlAG4AdABzACwAIABSAE8AVwBTACgAYQByAHIAXwBzAHQAcgBpAG4AZwBzACkALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAbgB1AG0AXwBlAGwAZQBtAGUAbgB0AHMAIAA9ACAAMQAsACAASQBOAEQARQBYACgAYQByAHIAXwBzAHQAcgBpAG4AZwBzACwAIAAxACwAIAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIABSAGUAcwBoAGEAcABlACAAYQByAHIAYQB5ACAAaQBuAHQAbwAgAHAAYQBpAHIAcwAuACAATwBkAGQALQBsAGUAbgBnAHQAaAAgAGEAcgByAGEAeQBzACAAYQByAGUAIABzAGEAZgBlAGwAeQAgAHAAYQBkAGQAZQBkACAAdwBpAHQAaAAgAHQAaABlACAAbQB1AGwAdABpAHAAbABpAGMAYQB0AGkAdgBlACAAaQBkAGUAbgB0AGkAdAB5ACAAXAAiADEAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHAAYQBpAHIAZQBkAF8AcwB0AHIAaQBuAGcAcwAsACAAVwBSAEEAUABSAE8AVwBTACgAYQByAHIAXwBzAHQAcgBpAG4AZwBzACwAIAAyACwAIABcACIAMQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAFYAZQBjAHQAbwByAGkAegBlAGQAIABtAHUAbAB0AGkAcABsAGkAYwBhAHQAaQBvAG4AIABhAGMAcgBvAHMAcwAgAGEAbABsACAAcABhAGkAcgBzACAAcwBpAG0AdQBsAHQAYQBuAGUAbwB1AHMAbAB5AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHIAZQBkAHUAYwBlAGQAXwBhAHIAcgBhAHkALAAgAEIAWQBSAE8AVwAoAHAAYQBpAHIAZQBkAF8AcwB0AHIAaQBuAGcAcwAsACAATABBAE0AQgBEAEEAKAByAG8AdwAsACAAVQBUAGUAeAB0AE0AdQBsACgASQBOAEQARQBYACgAcgBvAHcALAAgADEALAAgADEAKQAsACAASQBOAEQARQBYACgAcgBvAHcALAAgADEALAAgADIAKQApACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAFMAaABhAGwAbABvAHcAIAByAGUAYwB1AHIAcwBpAG8AbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBUAGUAeAB0AFQAcgBlAGUAUAByAG8AZAAoAHIAZQBkAHUAYwBlAGQAXwBhAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFsASQBuAHQAZQByAG4AYQBsAF0AIABDAGEAbABjAHUAbABhAHQAZQBzACAAdABoAGUAIABlAHgAcABvAG4AZQBuAHQAIABmAG8AcgAgAGEAbgAgAGEAcgByAGEAeQAgAG8AZgAgAHAAcgBpAG0AZQBzACAAaQBuACAAdABoAGUAIABTAHcAaQBuAGcAIAB0AGUAcgBtACAAbwBmACAAYQAgAGYAYQBjAHQAbwByAGkAYQBsAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAbgAgAFQAaABlACAAYwB1AHIAcgBlAG4AdAAgAGYAYQBjAHQAbwByAGkAYQBsACAAbQBhAGcAbgBpAHQAdQBkAGUAIAAoADwAPQAgADkAMgA3ADMAKQAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAHAAcgBpAG0AZQBzACAAQQAgAHYAZQByAHQAaQBjAGEAbAAgAGEAcgByAGEAeQAgAG8AZgAgAHAAcgBpAG0AZQAgAG4AdQBtAGIAZQByAHMAIAAoADwAPQAgAG4AKQAuAFwAbgAgACoALwBcAG4ATgBhAHQAaQB2AGUAUwB3AGkAbgBnAEUAeABwAG8AbgBlAG4AdABzACAAPQAgAEwAQQBNAEIARABBACgAbgAsACAAcAByAGkAbQBlAHMALABcAG4AIAAgACAAIABNAEEAUAAoAHAAcgBpAG0AZQBzACwAIABMAEEATQBCAEQAQQAoAHAALABcAG4AIAAgACAAIAAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAG0AYQB4AF8AcABvAHcAZQByAF8AawAsACAASQBOAFQAKABMAE8ARwAoAG4ALAAgAHAAKQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHAAcgBpAG0AZQBfAHAAbwB3AGUAcgBzACwAIABwACAAXgAgAFMARQBRAFUARQBOAEMARQAoAG0AYQB4AF8AcABvAHcAZQByAF8AawApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFMAVQBNACgATQBPAEQAKABJAE4AVAAoAG4AIAAvACAAcAByAGkAbQBlAF8AcABvAHcAZQByAHMAKQAsACAAMgApACkAXABuACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFsASQBuAHQAZQByAG4AYQBsAF0AIABDAGEAbABjAHUAbABhAHQAZQBzACAAdABoAGUAIABtAGEAcwBzAGkAdgBlACAAQgBpAGcASQBuAHQAIABzAHQAcgBpAG4AZwAgAGYAbwByACAAdABoAGUAIABTAHcAaQBuAGcAIAB0AGUAcgBtACAAbwBmACAAYQAgAGYAYQBjAHQAbwByAGkAYQBsAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAbgAgAFQAaABlACAAYwB1AHIAcgBlAG4AdAAgAGYAYQBjAHQAbwByAGkAYQBsACAAbQBhAGcAbgBpAHQAdQBkAGUALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIAB0AGkAZQByAF8AcAByAGkAbQBlAHMAIABBACAAdgBlAHIAdABpAGMAYQBsACAAYQByAHIAYQB5ACAAbwBmACAAcAByAGkAbQBlACAAbgB1AG0AYgBlAHIAcwAgACgAPAA9ACAAbgApAC4AXABuACAAKgAvAFwAbgBTAHcAaQBuAGcAVABlAHIAbQAgAD0AIABMAEEATQBCAEQAQQAoAG4ALAAgAHQAaQBlAHIAXwBwAHIAaQBtAGUAcwAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABzAHcAaQBuAGcAXwBlAHgAcABvAG4AZQBuAHQAcwAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4ATgBhAHQAaQB2AGUAUwB3AGkAbgBnAEUAeABwAG8AbgBlAG4AdABzACgAbgAsACAAdABpAGUAcgBfAHAAcgBpAG0AZQBzACkALABcAG4AIAAgACAAIAAgACAAIAAgAGgAYQBzAF8AbgBhAHQAaQB2AGUAXwBlAHgAcABvAG4AZQBuAHQALAAgAHMAdwBpAG4AZwBfAGUAeABwAG8AbgBlAG4AdABzACAAPgAgADAALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAALwAvACAASQBmACAAYQBsAGwAIABlAHgAcABvAG4AZQBuAHQAcwAgAGEAcgBlACAAMAAsACAAdABoAGUAIABzAHcAaQBuAGcAIAB0AGUAcgBtACAAaQBzACAAMQAuAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAQQBOAEQAKABOAE8AVAAoAGgAYQBzAF8AbgBhAHQAaQB2AGUAXwBlAHgAcABvAG4AZQBuAHQAKQApACwAIABcACIAMQBcACIALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABhAGMAdABpAHYAZQBfAHAAcgBpAG0AZQBzACwAIABGAEkATABUAEUAUgAoAHQAaQBlAHIAXwBwAHIAaQBtAGUAcwAsACAAaABhAHMAXwBuAGEAdABpAHYAZQBfAGUAeABwAG8AbgBlAG4AdAApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAYQBjAHQAaQB2AGUAXwBlAHgAcABvAG4AZQBuAHQAcwAsACAARgBJAEwAVABFAFIAKABzAHcAaQBuAGcAXwBlAHgAcABvAG4AZQBuAHQAcwAsACAAaABhAHMAXwBuAGEAdABpAHYAZQBfAGUAeABwAG8AbgBlAG4AdAApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAZQB2AGEAbAB1AHQAYQB0AGUAZABfAHAAcgBpAG0AZQBfAHAAbwB3AGUAcgBzACwAIABNAEEAUAAoAGEAYwB0AGkAdgBlAF8AcAByAGkAbQBlAHMALAAgAGEAYwB0AGkAdgBlAF8AZQB4AHAAbwBuAGUAbgB0AHMALAAgAEwAQQBNAEIARABBACgAcAAsACAAZQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABlACAAPQAgADEALAAgAHAAIAAmACAAXAAiAFwAIgAsACAAQgBpAGcASQBuAHQALgBQAG8AdwAoAHAAIAAmACAAXAAiAFwAIgAsACAAZQAgACYAIABcACIAXAAiACkAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBUAGUAeAB0AFQAcgBlAGUAUAByAG8AZAAoAGUAdgBhAGwAdQB0AGEAdABlAGQAXwBwAHIAaQBtAGUAXwBwAG8AdwBlAHIAcwApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAAWwBJAG4AdABlAHIAbgBhAGwAXQAgAFIAZQBjAHUAcgBzAGkAdgBlACAAdABvAHAALQBkAG8AdwBuACAATABBAE0AQgBEAEEAIABjAGEAbABjAHUAbABhAHQAaQBuAGcAIAB0AGgAZQAgAFAAcgBpAG0AZQAgAFMAdwBpAG4AZwAgAGYAYQBjAHQAbwByAGkAYQBsAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAbgAgAFQAaABlACAAYwB1AHIAcgBlAG4AdAAgAGYAYQBjAHQAbwByAGkAYQBsACAAbQBhAGcAbgBpAHQAdQBkAGUALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABnAGwAbwBiAGEAbABfAHAAcgBpAG0AZQBzACAAVABoAGUAIAB1AG4AaQBmAGkAZQBkACAAdgBlAHIAdABpAGMAYQBsACAAYQByAHIAYQB5ACAAbwBmACAAYQBsAGwAIABwAHIAaQBtAGUAcwAgAHUAcAAgAHQAbwAgAHQAaABlACAAdABhAHIAZwBlAHQAIABmAGEAYwB0AG8AcgBpAGEAbAAuAFwAbgAgACoALwBcAG4AUAByAGkAbQBlAFMAdwBpAG4AZwBLAGUAcgBuAGUAbAAgAD0AIABMAEEATQBCAEQAQQAoAG4ALAAgAGcAbABvAGIAYQBsAF8AcAByAGkAbQBlAHMALABcAG4AIAAgACAAIABJAEYAKABuACAAPAAgADIALAAgAFwAIgAxAFwAIgAsAFwAbgAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAZgBsAG8AbwByAF8AaABhAGwAZgBfAG4ALAAgAEkATgBUACgAbgAgAC8AIAAyACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAZgBhAGMAdABvAHIAaQBhAGwAXwBoAGEAbABmAF8AbgAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUAByAGkAbQBlAFMAdwBpAG4AZwBLAGUAcgBuAGUAbAAoAGYAbABvAG8AcgBfAGgAYQBsAGYAXwBuACwAIABnAGwAbwBiAGEAbABfAHAAcgBpAG0AZQBzACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAFMAcQB1AGEAcgBlACAAdABoAGUAIABoAGEAbABmAHcAYQB5ACAAcABvAGkAbgB0ACAAdQBzAGkAbgBnACAAdABoAGUAIAB1AG4AcwBhAGYAZQAgAGsAZQByAG4AZQBsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABzAHEAdQBhAHIAZQBkAF8AaABhAGwAZgBfAGYAYQBjAHQAbwByAGkAYQBsACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAFQAZQB4AHQATQB1AGwAKABmAGEAYwB0AG8AcgBpAGEAbABfAGgAYQBsAGYAXwBuACwAIABmAGEAYwB0AG8AcgBpAGEAbABfAGgAYQBsAGYAXwBuACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAEkAcwBvAGwAYQB0AGUAIAB0AGgAZQAgAHAAcgBpAG0AZQBzACAAbgBlAGUAZABlAGQAIABmAG8AcgAgAHQAaABpAHMAIAB0AGkAZQByACAAYQBuAGQAIABjAGEAbABjAHUAbABhAHQAZQAgAHQAaABlACAAcwB3AGkAbgBnACAAdABlAHIAbQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAYQBwAHAAbABpAGMAYQBiAGwAZQBfAHQAaQBlAHIAXwBwAHIAaQBtAGUAcwAsACAARgBJAEwAVABFAFIAKABnAGwAbwBiAGEAbABfAHAAcgBpAG0AZQBzACwAIABnAGwAbwBiAGEAbABfAHAAcgBpAG0AZQBzACAAPAA9ACAAbgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHMAdAByAF8AcwB3AGkAbgBnAF8AdABlAHIAbQAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwB3AGkAbgBnAFQAZQByAG0AKABuACwAIABhAHAAcABsAGkAYwBhAGIAbABlAF8AdABpAGUAcgBfAHAAcgBpAG0AZQBzACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFUAVABlAHgAdABNAHUAbAAoAHMAcQB1AGEAcgBlAGQAXwBoAGEAbABmAF8AZgBhAGMAdABvAHIAaQBhAGwALAAgAHMAdAByAF8AcwB3AGkAbgBnAF8AdABlAHIAbQApAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAAWwBJAG4AdABlAHIAbgBhAGwAXQAgAFIAZQBjAHUAcgBzAGkAdgBlACAAdABvAHUAcgBuAGEAbQBlAG4AdAAgAHQAcgBlAGUAIABmAG8AcgAgAE0AaQBuAC8ATQBhAHgAIABlAHYAYQBsAHUAYQB0AGkAbwBuAHMALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABjAG8AbAAgAEEAIAAxAEQAIAB2AGUAcgB0AGkAYwBhAGwAIABhAHIAcgBhAHkAIABvAGYAIABuAG8AcgBtAGEAbABpAHoAZQBkACAAQgBpAGcASQBuAHQAIABzAHQAcgBpAG4AZwBzAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAbQBvAGQAZQAgADEAIABmAG8AcgAgAE0AYQB4AGkAbQB1AG0ALAAgAC0AMQAgAGYAbwByACAATQBpAG4AaQBtAHUAbQAuAFwAbgAgACoALwBcAG4AVAByAGUAZQBDAG8AbQBwAGEAcgBlACAAPQAgAEwAQQBNAEIARABBACgAcwB0AHIAXwBuAG8AcgBtAHMALAAgAGMAbwBtAHAAYQByAGkAcwBvAG4AXwBtAG8AZABlACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG4AdQBtAF8AcgBvAHcAcwAsACAAUgBPAFcAUwAoAHMAdAByAF8AbgBvAHIAbQBzACkALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAbgB1AG0AXwByAG8AdwBzACAAPQAgADEALAAgAEkATgBEAEUAWAAoAHMAdAByAF8AbgBvAHIAbQBzACwAIAAxACwAIAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAB0AG8AdQByAG4AYQBtAGUAbgB0AF8AcABhAGkAcgBzACwAIABXAFIAQQBQAFIATwBXAFMAKABzAHQAcgBfAG4AbwByAG0AcwAsACAAMgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAYwBvAG0AcABlAHQAaQB0AG8AcgBzAF8AYQAsACAAVABBAEsARQAoAHQAbwB1AHIAbgBhAG0AZQBuAHQAXwBwAGEAaQByAHMALAAgACwAIAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABjAG8AbQBwAGUAdABpAHQAbwByAHMAXwBiACwAIABUAEEASwBFACgAdABvAHUAcgBuAGEAbQBlAG4AdABfAHAAYQBpAHIAcwAsACAALAAgAC0AMQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcgBvAHUAbgBkAF8AdwBpAG4AbgBlAHIAcwAsACAATQBBAFAAKABjAG8AbQBwAGUAdABpAHQAbwByAHMAXwBhACwAIABjAG8AbQBwAGUAdABpAHQAbwByAHMAXwBiACwAIABMAEEATQBCAEQAQQAoAGEALAAgAGIALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEkARgAoAEkAUwBOAEEAKABiACkALAAgAGEALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABjAG8AbQBwAGEAcgBpAHMAbwBuAF8AcgBlAHMAdQBsAHQALAAgAEIAaQBnAEkAbgB0AC4AQwBvAG0AcABhAHIAZQAoAGEALAAgAGIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEkARgAoAGMAbwBtAHAAYQByAGkAcwBvAG4AXwByAGUAcwB1AGwAdAAgACoAIABjAG8AbQBwAGEAcgBpAHMAbwBuAF8AbQBvAGQAZQAgAD4APQAgADAALAAgAGEALAAgAGIAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVAByAGUAZQBDAG8AbQBwAGEAcgBlACgAcgBvAHUAbgBkAF8AdwBpAG4AbgBlAHIAcwAsACAAYwBvAG0AcABhAHIAaQBzAG8AbgBfAG0AbwBkAGUAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQgBpAGcASQBuAHQAIgAsACIAdABlAHgAdAAiADoAIgAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwBcAG4ALwAvACAAQgBpAGcAIABJAG4AdABlAGcAZQByACAAQQByAGkAdABoAG0AZQB0AGkAYwAgAEwAaQBiAHIAYQByAHkAIAAvAC8AXABuAC8ALwAgACAAIAAgACAAIAAgACAAQgBpAGcASQBuAHQAIABNAG8AZAB1AGwAZQAgACAAIAAgACAAIAAgACAAIAAgACAALwAvAFwAbgAvAC8AIAAgACAAIAAgACAAIAAgACAAIABQAHUAYgBsAGkAYwAgAEEAUABJACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwBcAG4ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8AXABuAFwAbgAvACoAKgBcAG4AIAAqACAATgBvAHIAbQBhAGwAaQBzAGUAcwAgAGEAIABCAGkAZwBJAG4AdAAgAHMAdAByAGkAbgBnAC4AIABTAHQAcgBpAHAAcwAgAGwAZQBhAGQAaQBuAGcAIAB6AGUAcgBvAHMALAAgAHIAZQBzAG8AbAB2AGUAcwAgAFwAIgAtADAAXAAiACAAdABvACAAXAAiADAAXAAiACwAIABhAG4AZAAgAHQAaAByAG8AdwBzACAAIwBWAEEATABVAEUAIQAgAG8AbgAgAGkAbgB2AGEAbABpAGQAIABjAGgAYQByAGEAYwB0AGUAcgBzAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAaQBuAHAAdQB0ACAAVABoAGUAIABCAGkAZwBJAG4AdAAgAHMAdAByAGkAbgBnAC4AXABuACAAKgAvAFwAbgBOAG8AcgBtACAAPQAgAEwAQQBNAEIARABBACgAaQBuAHAAdQB0ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAHMAdAByAF8AaQBuAHAAdQB0ACwAIABJAEYAKABPAFIAKABJAFMATwBNAEkAVABUAEUARAAoAGkAbgBwAHUAdAApACwAIABpAG4AcAB1AHQAIAA9ACAAXAAiAFwAIgApACwAIABcACIAMABcACIALAAgAGkAbgBwAHUAdAAgACYAIABcACIAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAGkAcwBfAHYAYQBsAHUAZQBfAGYAbwByAG0AYQB0ACwAIABSAEUARwBFAFgAVABFAFMAVAAoAHMAdAByAF8AaQBuAHAAdQB0ACwAIABcACIAXgAtAD8AXABcAGQAKwAkAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAcgBfAG4AbwByAG0ALAAgAFIARQBHAEUAWABSAEUAUABMAEEAQwBFACgAcwB0AHIAXwBpAG4AcAB1AHQALAAgAFwAIgBeACgALQA/ACkAMAArACgAPwA9AFwAXABkACkAXAAiACwAIABcACIAJAAxAFwAIgApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgATgBPAFQAKABpAHMAXwB2AGEAbAB1AGUAXwBmAG8AcgBtAGEAdAApACwAIABWAEEATABVAEUAKABcACIAIwBWAEEATABVAEUAIQBcACIAKQAsACAASQBGACgAcwB0AHIAXwBuAG8AcgBtACAAPQAgAFwAIgAtADAAXAAiACwAIABcACIAMABcACIALAAgAHMAdAByAF8AbgBvAHIAbQApACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFIAZQB0AHUAcgBuAHMAIAB0AGgAZQAgAHMAaQBnAG4AIABvAGYAIABhACAAQgBpAGcASQBuAHQAOgAgADEAIAAoAHAAbwBzAGkAdABpAHYAZQApACwAIAAtADEAIAAoAG4AZQBnAGEAdABpAHYAZQApACwAIABvAHIAIAAwACAAKAB6AGUAcgBvACkALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABiAGkAZwBfAGkAbgB0ACAAVABoAGUAIABCAGkAZwBJAG4AdAAgAHMAdAByAGkAbgBnAC4AXABuACAAKgAvAFwAbgBTAGkAZwBuACAAPQAgAEwAQQBNAEIARABBACgAaQBuAHAAdQB0ACwAIABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AHIAXwBuAG8AcgBtACwAIABOAG8AcgBtACgAaQBuAHAAdQB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFMAVwBJAFQAQwBIACgATABFAEYAVAAoAHMAdAByAF8AbgBvAHIAbQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAwAFwAIgAsACAAMAAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIALQBcACIALAAgAC0AMQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvAC8AIAAtAC0ALQAgAFAAcgBlAGQAaQBjAGEAdABlAHMAIAAtAC0ALQAgAFwAXABcAFwAXABuAFwAbgAvACoAKgBcAG4AIAAqACAAUgBlAHQAdQByAG4AcwAgAFQAUgBVAEUAIABpAGYAIAB0AGgAZQAgAEIAaQBnAEkAbgB0ACAAaQBzACAAZQB4AGEAYwB0AGwAeQAgAHoAZQByAG8ALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABpAG4AcAB1AHQAIABUAGgAZQAgAEIAaQBnAEkAbgB0ACAAcwB0AHIAaQBuAGcALgBcAG4AIAAqAC8AXABuAEkAcwBaAGUAcgBvACAAPQAgAEwAQQBNAEIARABBACgAaQBuAHAAdQB0ACwAIABOAG8AcgBtACgAaQBuAHAAdQB0ACkAIAA9ACAAXAAiADAAXAAiACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABSAGUAdAB1AHIAbgBzACAAVABSAFUARQAgAGkAZgAgAHQAaABlACAAQgBpAGcASQBuAHQAIABpAHMAIABuAGUAZwBhAHQAaQB2AGUALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABpAG4AcAB1AHQAIABUAGgAZQAgAEIAaQBnAEkAbgB0ACAAcwB0AHIAaQBuAGcALgBcAG4AIAAqAC8AXABuAEkAcwBOAGUAZwAgAD0AIABMAEEATQBCAEQAQQAoAGkAbgBwAHUAdAAsACAATABFAEYAVAAoAE4AbwByAG0AKABpAG4AcAB1AHQAKQApACAAPQAgAFwAIgAtAFwAIgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAAUgBlAHQAdQByAG4AcwAgAFQAUgBVAEUAIABpAGYAIAB0AGgAZQAgAEIAaQBnAEkAbgB0ACAAaQBzACAAZQB2AGUAbgAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGkAbgBwAHUAdAAgAFQAaABlACAAQgBpAGcASQBuAHQAIABzAHQAcgBpAG4AZwAuAFwAbgAgACoALwBcAG4ASQBzAEUAdgBlAG4AIAA9ACAATABBAE0AQgBEAEEAKABpAG4AcAB1AHQALAAgAEkAUwBFAFYARQBOACgAVgBBAEwAVQBFACgAUgBJAEcASABUACgATgBvAHIAbQAoAGkAbgBwAHUAdAApACkAKQApACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABSAGUAdAB1AHIAbgBzACAAVABSAFUARQAgAGkAZgAgAHQAaABlACAAQgBpAGcASQBuAHQAIABpAHMAIABvAGQAZAAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGkAbgBwAHUAdAAgAFQAaABlACAAQgBpAGcASQBuAHQAIABzAHQAcgBpAG4AZwAuAFwAbgAgACoALwBcAG4ASQBzAE8AZABkACAAPQAgAEwAQQBNAEIARABBACgAaQBuAHAAdQB0ACwAIABJAFMATwBEAEQAKABWAEEATABVAEUAKABSAEkARwBIAFQAKABOAG8AcgBtACgAaQBuAHAAdQB0ACkAKQApACkAKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFIAZQB0AHUAcgBuAHMAIAB0AGgAZQAgAHUAbgBzAGkAZwBuAGUAZAAgAG0AYQBnAG4AaQB0AHUAZABlACAAbwBmACAAYQAgAEIAaQBnAEkAbgB0ACAAcwB0AHIAaQBuAGcAIAAoAGEAYgBzAG8AbAB1AHQAZQAgAHYAYQBsAHUAZQApAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAaQBuAHAAdQB0ACAAVABoAGUAIABCAGkAZwBJAG4AdAAgAHMAdAByAGkAbgBnAC4AXABuACAAKgAvAFwAbgBBAGIAcwAgAD0AIABMAEEATQBCAEQAQQAoAGkAbgBwAHUAdAAsACAAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAHMAdAByAF8AbgBvAHIAbQAsACAATgBvAHIAbQAoAGkAbgBwAHUAdAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABMAEUARgBUACgAcwB0AHIAXwBuAG8AcgBtACkAIAA9ACAAXAAiAC0AXAAiACwAIABNAEkARAAoAHMAdAByAF8AbgBvAHIAbQAsACAAMgAsACAATABFAE4AKABzAHQAcgBfAG4AbwByAG0AKQAgAC0AIAAxACkALAAgAHMAdAByAF8AbgBvAHIAbQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABDAG8AbQBwAGEAcgBlAHMAIAB0AHcAbwAgAEIAaQBnAEkAbgB0ACAAcwB0AHIAaQBuAGcAcwAuACAAUgBlAHQAdQByAG4AcwAgADEAIAAoAGEAIAA+ACAAYgApACwAIAAtADEAIAAoAGEAIAA8ACAAYgApACwAIABvAHIAIAAwACAAKABhACAAPQAgAGIAKQAuAFwAbgAgACoAIABFAHYAYQBsAHUAYQB0AGUAcwAgAHMAaQBnAG4AcwAgAGEAbgBkACAAbABlAG4AZwB0AGgAcwAuACAASQBmACAAaQBkAGUAbgB0AGkAYwBhAGwALAAgAGQAZQBsAGUAZwBhAHQAZQBzACAAdABvACAAbgBhAHQAaQB2AGUAIABsAGkAbQBiACAAYQByAHIAYQB5ACAAYwBvAG0AcABhAHIAaQBzAG8AbgAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGkAbgBwAHUAdABfAGEAIABUAGgAZQAgAGYAaQByAHMAdAAgAEIAaQBnAEkAbgB0ACAAcwB0AHIAaQBuAGcALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABpAG4AcAB1AHQAXwBiACAAVABoAGUAIABzAGUAYwBvAG4AZAAgAEIAaQBnAEkAbgB0ACAAcwB0AHIAaQBuAGcALgBcAG4AIAAqAC8AXABuAEMAbwBtAHAAYQByAGUAIAA9ACAATABBAE0AQgBEAEEAKABpAG4AcAB1AHQAXwBhACwAIABpAG4AcAB1AHQAXwBiACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAHMAdAByAF8AbgBvAHIAbQBfAGEALAAgAE4AbwByAG0AKABpAG4AcAB1AHQAXwBhACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAdAByAF8AbgBvAHIAbQBfAGIALAAgAE4AbwByAG0AKABpAG4AcAB1AHQAXwBiACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAaQBnAG4AXwBhACwAIABCAGkAZwBJAG4AdAAuAFMAaQBnAG4AKABzAHQAcgBfAG4AbwByAG0AXwBhACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAaQBnAG4AXwBiACwAIABCAGkAZwBpAG4AdAAuAFMAaQBnAG4AKABzAHQAcgBfAG4AbwByAG0AXwBiACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIABJAEYAKABzAGkAZwBuAF8AYQAgADwAPgAgAHMAaQBnAG4AXwBiACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFMASQBHAE4AKABzAGkAZwBuAF8AYQAgAC0AIABzAGkAZwBuAF8AYgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEkARgAoAHMAaQBnAG4AXwBhACAAPQAgADAALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAwACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAZQBuAF8AYQAsACAATABFAE4AKABzAHQAcgBfAG4AbwByAG0AXwBhACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAZQBuAF8AYgAsACAATABFAE4AKABzAHQAcgBfAG4AbwByAG0AXwBiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgAbABlAG4AXwBhACAAPAA+ACAAbABlAG4AXwBiACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFMASQBHAE4AKABsAGUAbgBfAGEAIAAtACAAbABlAG4AXwBiACkAIAAqACAAcwBpAGcAbgBfAGEALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABrACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBTAGEAZgBlAEsAKABcACIAQQBEAEQAXAAiACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGEALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFMAcABsAGkAdAAoAEIAaQBnAEkAbgB0AC4AQQBiAHMAKABzAHQAcgBfAG4AbwByAG0AXwBhACkALAAgAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGIALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFMAcABsAGkAdAAoAEIAaQBnAEkAbgB0AC4AQQBiAHMAKABzAHQAcgBfAG4AbwByAG0AXwBiACkALAAgAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAG0AYQBnAG4AaQB0AHUAZABlAF8AYwBvAG0AcABhAHIAaQBzAG8AbgAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBDAG8AbQBwAGEAcgBlACgAbABpAG0AYgBzAF8AYQAsACAAbABpAG0AYgBzAF8AYgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbQBhAGcAbgBpAHQAdQBkAGUAXwBjAG8AbQBwAGEAcgBpAHMAbwBuACAAKgAgAHMAaQBnAG4AXwBhAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvAC8AIAAgACAAIAAgACAAIAAgACAAIAAtACAAQQBkAGQAaQB0AGkAbwBuACAAJgAgAFMAdQBiAHQAcgBhAGMAdABpAG8AbgAgAC0AIAAgACAAIAAgACAAIABcAFwAXABcAFwAbgBcAG4ALwAqACoAXABuACAAKgAgAEEAZABkAHMAIAB0AHcAbwAgAEIAaQBnAEkAbgB0ACAAcwB0AHIAaQBuAGcAcwAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGkAbgBwAHUAdABfAGEAIABUAGgAZQAgAGYAaQByAHMAdAAgAEIAaQBnAEkAbgB0ACAAcwB0AHIAaQBuAGcALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABpAG4AcAB1AHQAXwBiACAAVABoAGUAIABzAGUAYwBvAG4AZAAgAEIAaQBnAEkAbgB0ACAAcwB0AHIAaQBuAGcALgBcAG4AIAAqAC8AXABuAEEAZABkACAAPQAgAEwAQQBNAEIARABBACgAaQBuAHAAdQB0AF8AYQAsACAAaQBuAHAAdQB0AF8AYgAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABzAHQAcgBfAG4AbwByAG0AXwBhACwAIABOAG8AcgBtACgAaQBuAHAAdQB0AF8AYQApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAcgBfAG4AbwByAG0AXwBiACwAIABOAG8AcgBtACgAaQBuAHAAdQB0AF8AYgApACwAXABuACAAIAAgACAAIAAgACAAIABzAGkAZwBuAF8AYQAsACAAQgBpAGcAaQBuAHQALgBTAGkAZwBuACgAcwB0AHIAXwBuAG8AcgBtAF8AYQApACwAXABuACAAIAAgACAAIAAgACAAIABzAGkAZwBuAF8AYgAsACAAQgBpAGcASQBuAHQALgBTAGkAZwBuACgAcwB0AHIAXwBuAG8AcgBtAF8AYgApACwAXABuACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgAGsALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFMAYQBmAGUASwAoAFwAIgBBAEQARABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYQAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwBwAGwAaQB0ACgAQgBpAGcASQBuAHQALgBBAGIAcwAoAHMAdAByAF8AbgBvAHIAbQBfAGEAKQAsACAAawApACwAXABuACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBiACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBTAHAAbABpAHQAKABCAGkAZwBJAG4AdAAuAEEAYgBzACgAcwB0AHIAXwBuAG8AcgBtAF8AYgApACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAcABhAGMAawBlAGQAXwByAGUAcwB1AGwAdAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AQQBkAGQAUwB1AGIAUgBvAHUAdABlAHIAKABsAGkAbQBiAHMAXwBhACwAIABsAGkAbQBiAHMAXwBiACwAIABzAGkAZwBuAF8AYQAsACAAcwBpAGcAbgBfAGIALAAgAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAG4AYQBsAF8AcwBpAGcAbgAsACAAQwBIAE8ATwBTAEUAUgBPAFcAUwAoAHAAYQBjAGsAZQBkAF8AcgBlAHMAdQBsAHQALAAgAC0AMQApACwAXABuACAAIAAgACAAIAAgACAAIABmAGkAbgBhAGwAXwBsAGkAbQBiAHMALAAgAEQAUgBPAFAAKABwAGEAYwBrAGUAZABfAHIAZQBzAHUAbAB0ACwAIAAtADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIABzAHQAcgBfAG0AZQByAGcAZQBkACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBNAGUAcgBnAGUAKABmAGkAbgBhAGwAXwBsAGkAbQBiAHMALAAgAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABmAGkAbgBhAGwAXwBzAGkAZwBuACAAPQAgAC0AMQAsACAAXAAiAC0AXAAiACAAJgAgAHMAdAByAF8AbQBlAHIAZwBlAGQALAAgAHMAdAByAF8AbQBlAHIAZwBlAGQAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAAUwB1AGIAdAByAGEAYwB0AHMAIAB0AGgAZQAgAHMAZQBjAG8AbgBkACAAQgBpAGcASQBuAHQAIABzAHQAcgBpAG4AZwAgAGYAcgBvAG0AIAB0AGgAZQAgAGYAaQByAHMAdAAgACgAQQAgAC0AIABCACkALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABpAG4AcAB1AHQAXwBhACAAVABoAGUAIABtAGkAbgB1AGUAbgBkACAAQgBpAGcASQBuAHQAIABzAHQAcgBpAG4AZwAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGkAbgBwAHUAdABfAGIAIABUAGgAZQAgAHMAdQBiAHQAcgBhAGgAZQBuAGQAIABCAGkAZwBJAG4AdAAgAHMAdAByAGkAbgBnAC4AXABuACAAKgAvAFwAbgBTAHUAYgAgAD0AIABMAEEATQBCAEQAQQAoAGkAbgBwAHUAdABfAGEALAAgAGkAbgBwAHUAdABfAGIALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AHIAXwBuAG8AcgBtAF8AYgAsACAATgBvAHIAbQAoAGkAbgBwAHUAdABfAGIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABJAG4AdgBlAHIAdAAgAHQAaABlACAAcwBpAGcAbgAgAG8AZgAgAEIAIABhAHQAIAB0AGgAZQAgAHQAZQB4AHQAIABsAGUAdgBlAGwAXABuACAAIAAgACAAIAAgACAAIABzAHQAcgBfAGkAbgB2AGUAcgBzAGUAXwBiACwAIABJAEYAKABzAHQAcgBfAG4AbwByAG0AXwBiACAAPQAgAFwAIgAwAFwAIgAsACAAXAAiADAAXAAiACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgATABFAEYAVAAoAHMAdAByAF8AbgBvAHIAbQBfAGIAKQAgAD0AIABcACIALQBcACIALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAE0ASQBEACgAcwB0AHIAXwBuAG8AcgBtAF8AYgAsACAAMgAsACAATABFAE4AKABzAHQAcgBfAG4AbwByAG0AXwBiACkAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAC0AXAAiACAAJgAgAHMAdAByAF8AbgBvAHIAbQBfAGIAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgAC8ALwAgAFAAYQBzAHMAIAB0AG8AIABBAGQAZABcAG4AIAAgACAAIAAgACAAIAAgAEEAZABkACgAaQBuAHAAdQB0AF8AYQAsACAAcwB0AHIAXwBpAG4AdgBlAHIAcwBlAF8AYgApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABTAHUAbQBzACAAYQBuACAAYQByAHIAYQB5ACAAbwByACAAcgBhAG4AZwBlACAAbwBmACAAQgBpAGcASQBuAHQAIABzAHQAcgBpAG4AZwBzACAAdgBpAGEAIAB2AGUAYwB0AG8AcgBpAHoAZQBkACAAZwByAG8AdQBwACAAbQBhAHQAcgBpAGMAZQBzAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAaQBuAHAAdQB0AF8AcgBhAG4AZwBlACAAQQAgAGMAbwBuAHQAaQBnAHUAbwB1AHMAIAByAGEAbgBnAGUAIABvAHIAIABhAHIAcgBhAHkAIABvAGYAIABCAGkAZwBJAG4AdAAgAHMAdAByAGkAbgBnAHMALgBcAG4AIAAqAC8AXABuAFMAdQBtACAAPQAgAEwAQQBNAEIARABBACgAaQBuAHAAdQB0AF8AcgBhAG4AZwBlACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAC8ALwAgAFMAZQB0AHUAcAAgAGYAbwByACAAbABpAHQAdABsAGUALQBlAG4AZABpAGEAbgAgAGEAbABpAGcAbgBtAGUAbgB0ACAAaQBuACAAbQBhAHQAcgBpAHgAIABzAHUAbQBcAG4AIAAgACAAIAAgACAAIAAgAGYAbABhAHQAdABlAG4AZQBkAF8AaQBuAHAAdQB0ACwAIABUAE8AUgBPAFcAKABpAG4AcAB1AHQAXwByAGEAbgBnAGUALAAgADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABPAFIAKABJAFMARQBSAFIATwBSACgAZgBsAGEAdAB0AGUAbgBlAGQAXwBpAG4AcAB1AHQAKQAsACAAQwBPAEwAVQBNAE4AUwAoAGYAbABhAHQAdABlAG4AZQBkAF8AaQBuAHAAdQB0ACkAIAA9ACAAMAApACwAIABcACIAMABcACIALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABzAHQAcgBfAG4AbwByAG0AcwAsACAATQBBAFAAKABmAGwAYQB0AHQAZQBuAGUAZABfAGkAbgBwAHUAdAAsACAATABBAE0AQgBEAEEAKAB4ACwAIABOAG8AcgBtACgAeAApACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGEAcgByAF8AcwBpAGcAbgBzACwAIABNAEEAUAAoAEwARQBGAFQAKABzAHQAcgBfAG4AbwByAG0AcwApACwAIABMAEEATQBCAEQAQQAoAHgALAAgAEkARgAoAHgAIAA9ACAAXAAiADAAXAAiACwAIAAwACwAIABpAGYAKAB4ACAAPQAgAFwAIgAtAFwAIgAsACAALQAxACwAIAAxACkAKQApACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABzAHQAcgBfAGEAYgBzACwAIABNAEEAUAAoAHMAdAByAF8AbgBvAHIAbQBzACwAIABhAHIAcgBfAHMAaQBnAG4AcwAsACAATABBAE0AQgBEAEEAKAB4ACwAIABzAGkAZwBuACwAIABJAEYAKABzAGkAZwBuACAAPQAgAC0AMQAsACAATQBJAEQAKAB4ACwAIAAyACwAIABMAEUATgAoAHgAKQAtADEAKQAsACAAeAApACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHMAdAByAF8AcABvAHMALAAgAEYASQBMAFQARQBSACgAcwB0AHIAXwBhAGIAcwAsACAAYQByAHIAXwBzAGkAZwBuAHMAIAA9ACAAMQAsACAAewBcACIAMABcACIAfQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcwB0AHIAXwBuAGUAZwBzACwAIABGAEkATABUAEUAUgAoAHMAdAByAF8AYQBiAHMALAAgAGEAcgByAF8AcwBpAGcAbgBzACAAPQAgAC0AMQAsACAAewBcACIAMABcACIAfQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAdQBuAGkAZgBpAGUAZABfAGsALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFMAYQBmAGUASwAoAFwAIgBBAEQARABcACIALAAgAEMATwBMAFUATQBOAFMAKABmAGwAYQB0AHQAZQBuAGUAZABfAGkAbgBwAHUAdAApACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBwAG8AcwBfAHMAdQBtACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAE0AYQB0AHIAaQB4AFMAdQBtACgAcwB0AHIAXwBwAG8AcwAsACAAdQBuAGkAZgBpAGUAZABfAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAG4AZQBnAF8AcwB1AG0ALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFUATQBhAHQAcgBpAHgAUwB1AG0AKABzAHQAcgBfAG4AZQBnAHMALAAgAHUAbgBpAGYAaQBlAGQAXwBrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABwAGEAYwBrAGUAZABfAHIAZQBzAHUAbAB0ACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBBAGQAZABTAHUAYgBSAG8AdQB0AGUAcgAoAGwAaQBtAGIAcwBfAHAAbwBzAF8AcwB1AG0ALAAgAGwAaQBtAGIAcwBfAG4AZQBnAF8AcwB1AG0ALAAgADEALAAgAC0AMQAsACAAdQBuAGkAZgBpAGUAZABfAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGYAaQBuAGEAbABfAHMAaQBnAG4ALAAgAEMASABPAE8AUwBFAFIATwBXAFMAKABwAGEAYwBrAGUAZABfAHIAZQBzAHUAbAB0ACwAIAAtADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGYAaQBuAGEAbABfAGwAaQBtAGIAcwAsACAARABSAE8AUAAoAHAAYQBjAGsAZQBkAF8AcgBlAHMAdQBsAHQALAAgAC0AMQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcwB0AHIAXwBtAGUAcgBnAGUAZAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4ATQBlAHIAZwBlACgAZgBpAG4AYQBsAF8AbABpAG0AYgBzACwAIAB1AG4AaQBmAGkAZQBkAF8AawApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgAZgBpAG4AYQBsAF8AcwBpAGcAbgAgAD0AIAAtADEALAAgAFwAIgAtAFwAIgAgACYAIABzAHQAcgBfAG0AZQByAGcAZQBkACwAIABzAHQAcgBfAG0AZQByAGcAZQBkACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABNAHUAbAB0AGkAcABsAGkAZQBzACAAdAB3AG8AIABCAGkAZwBJAG4AdAAgAHMAdAByAGkAbgBnAHMALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABpAG4AcAB1AHQAXwBhACAAVABoAGUAIABmAGkAcgBzAHQAIABCAGkAZwBJAG4AdAAgAHMAdAByAGkAbgBnAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAaQBuAHAAdQB0AF8AYgAgAFQAaABlACAAcwBlAGMAbwBuAGQAIABCAGkAZwBJAG4AdAAgAHMAdAByAGkAbgBnAC4AXABuACAAKgAvAFwAbgBNAHUAbAAgAD0AIABMAEEATQBCAEQAQQAoAGkAbgBwAHUAdABfAGEALAAgAGkAbgBwAHUAdABfAGIALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AHIAXwBuAG8AcgBtAF8AYQAsACAATgBvAHIAbQAoAGkAbgBwAHUAdABfAGEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AHIAXwBuAG8AcgBtAF8AYgAsACAATgBvAHIAbQAoAGkAbgBwAHUAdABfAGIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwBpAGcAbgBfAGEALAAgAEIAaQBnAEkAbgB0AC4AUwBpAGcAbgAoAHMAdAByAF8AbgBvAHIAbQBfAGEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwBpAGcAbgBfAGIALAAgAEIAaQBnAEkAbgB0AC4AUwBpAGcAbgAoAHMAdAByAF8AbgBvAHIAbQBfAGIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABlAG4AXwBhACwAIABMAEUATgAoAHMAdAByAF8AbgBvAHIAbQBfAGEAKQAgAC0AIABJAEYAKABzAGkAZwBuAF8AYQAgAD0AIAAtADEALAAgADEALAAgADAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABlAG4AXwBiACwAIABMAEUATgAoAHMAdAByAF8AbgBvAHIAbQBfAGIAKQAgAC0AIABJAEYAKABzAGkAZwBuAF8AYgAgAD0AIAAtADEALAAgADEALAAgADAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABQAHIAbwBkAHUAYwB0ACAAbwBmACAAdwBpAHQAaAAgADAAIABpAHMAIAAwAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgATwBSACgAcwBpAGcAbgBfAGEAIAA9ACAAMAAsACAAcwBpAGcAbgBfAGIAIAA9ACAAMAApACwAIABcACIAMABcACIALABcAG4AIAAgACAAIAAgACAAIAAgAC8ALwAgAFQAaABlACAAcgBlAHMAdQBsAHQAIAB3AGkAbABsACAAZQB4AGMAZQBlAGQAIABjAGgAYQByACAAbABpAG0AaQB0AFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAbABlAG4AXwBhACAAKwAgAGwAZQBuAF8AYgAgAD4AIAAzADIANwA2ADYALAAgACMATgBVAE0AIQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGsALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFMAYQBmAGUASwAoAFwAIgBNAFUATABcACIALAAgAE0ASQBOACgAbABlAG4AXwBhACwAIABsAGUAbgBfAGIAKQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYQAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwBwAGwAaQB0ACgAQgBpAGcASQBuAHQALgBBAGIAcwAoAHMAdAByAF8AbgBvAHIAbQBfAGEAKQAsACAAawApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYgAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwBwAGwAaQB0ACgAQgBpAGcASQBuAHQALgBBAGIAcwAoAHMAdAByAF8AbgBvAHIAbQBfAGIAKQAsACAAawApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAZgBpAG4AYQBsAF8AbABpAG0AYgBzACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAE0AdQBsACgAbABpAG0AYgBzAF8AYQAsACAAbABpAG0AYgBzAF8AYgAsACAAawApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAZgBpAG4AYQBsAF8AcwBpAGcAbgAsACAAcwBpAGcAbgBfAGEAIAAqACAAcwBpAGcAbgBfAGIALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABzAHQAcgBfAG0AZQByAGcAZQBkACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBNAGUAcgBnAGUAKABmAGkAbgBhAGwAXwBsAGkAbQBiAHMALAAgAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEkARgAoAGYAaQBuAGEAbABfAHMAaQBnAG4AIAA9ACAALQAxACwAIABcACIALQBcACIAIAAmACAAcwB0AHIAXwBtAGUAcgBnAGUAZAAsACAAcwB0AHIAXwBtAGUAcgBnAGUAZAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABbAFYATwBMAEEAVABJAEwARQBdACAARwBlAG4AZQByAGEAdABlAHMAIABhACAAZAB5AG4AYQBtAGkAYwAgAGEAcgByAGEAeQAgAG8AZgAgAGkAbgB0AGUAZwBlAHIAcwAgAGEAcwAgAHQAZQB4AHQALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABbAG4AdQBtAF8AcgBvAHcAcwBdACAAYQByAHIAYQB5ACAAaABlAGkAZwBoAHQALAAgAGQAZQBmAGEAdQBsAHQAIAAxAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAWwBuAHUAbQBfAGMAbwBsAHMAXQAgAGEAcgByAGEAeQAgAHcAaQBkAHQAaAAsACAAZABlAGYAYQB1AGwAdAAgADEALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABbAG0AaQBuAF8AZABpAGcAaQB0AHMAXQAgAG0AaQBuAGkAbQB1AG0AIABuAHUAbQBiAGUAcgAgAG8AZgAgAGQAaQBnAGkAdABzACwAIABkAGUAZgBhAHUAbAB0ACAAMQA2ACAAKABtAGkAbgAgADEAIABkAGkAZwBpAHQAKQBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABbAG0AYQB4AF8AZABpAGcAaQB0AHMAXQAgAG0AYQB4AGkAbQB1AG0AIABuAHUAbQBiAGUAcgAgAG8AZgAgAGQAaQBnAGkAdABzACwAIABkAGUAZgBhAHUAbAB0ACAANQAwACAAKABtAGEAeAAgADMAMgAsADcANgA3ACAAYwBoAGEAcgBzACwAIABpAG4AYwBsAHUAZABpAG4AZwAgAHMAaQBnAG4AKQBcAG4AIAAqAC8AXABuAFIAYQBuAGQAQQByAHIAYQB5ACAAPQAgAEwAQQBNAEIARABBACgAWwBuAHUAbQBfAHIAbwB3AHMAXQAsACAAWwBuAHUAbQBfAGMAbwBsAHMAXQAsACAAWwBtAGkAbgBfAGQAaQBnAGkAdABzAF0ALAAgAFsAbQBhAHgAXwBkAGkAZwBpAHQAcwBdACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG4AXwByAG8AdwBzACwAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAG4AdQBtAF8AcgBvAHcAcwApACwAIAAxACwAIABuAHUAbQBfAHIAbwB3AHMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbgBfAGMAbwBsAHMALAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAbgB1AG0AXwBjAG8AbABzACkALAAgADEALAAgAG4AdQBtAF8AYwBvAGwAcwApACwAIABcAG4AIAAgACAAIAAgACAAIAAgAG0AaQBuAF8AbABlAG4ALAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAbQBpAG4AXwBkAGkAZwBpAHQAcwApACwAIAAxADYALAAgAE0ASQBOACgAMwAyADcANgA3ACwAIABNAEEAWAAoADEALAAgAG0AaQBuAF8AZABpAGcAaQB0AHMAKQApACkALABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQB4AF8AbABlAG4ALAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAbQBhAHgAXwBkAGkAZwBpAHQAcwApACwAIAA1ADAALAAgAE0AQQBYACgAMQAsACAATQBJAE4AKAAzADIANwA2ADYALAAgAG0AYQB4AF8AZABpAGcAaQB0AHMAKQApACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIABNAEEAUAAoAFIAQQBOAEQAQQBSAFIAQQBZACgAbgBfAHIAbwB3AHMALAAgAG4AXwBjAG8AbABzACwAIABtAGkAbgBfAGwAZQBuACwAIABtAGEAeABfAGwAZQBuACwAIABUAFIAVQBFACkALAAgAEwAQQBNAEIARABBACgAbABlAG4AZwB0AGgALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABzAGkAZwBuAF8AcAByAGUAZgBpAHgALAAgAEMASABPAE8AUwBFACgAUgBBAE4ARABCAEUAVABXAEUARQBOACgAMQAsACAAMgApACwAIABcACIAXAAiACwAIABcACIALQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHIAYQBuAGQAXwBkAGkAZwBpAHQAcwAsACAAQwBPAE4AQwBBAFQAKABSAEEATgBEAEEAUgBSAEEAWQAoADEALAAgAGwAZQBuAGcAdABoACwAIAAwACwAIAA5ACwAIABUAFIAVQBFACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHMAaQBnAG4AXwBwAHIAZQBmAGkAeAAgACYAIABSAEUARwBFAFgAUgBFAFAATABBAEMARQAoAHIAYQBuAGQAXwBkAGkAZwBpAHQAcwAsACAAXAAiAF4AMAAqAFwAIgAsACAAXAAiAFwAIgApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABEAGkAdgBpAGQAZQBzACAAdABoAGUAIABmAGkAcgBzAHQAIABCAGkAZwBJAG4AdAAgAGIAeQAgAHQAaABlACAAcwBlAGMAbwBuAGQAIAAoAEEAIAAvACAAQgApAC4AIABcAG4AIAAqACAAUgBlAHQAdQByAG4AcwAgAHQAaABlACAAcQB1AG8AdABpAGUAbgB0ACAAYQBuAGQAIABtAG8AZAB1AGwAdQBzACAAaQBuACAAcgBvAHcAcwAgADEAIABhAG4AZAAgADIALAAgAHIAZQBzAHAAZQBjAHQAaQB2AGUAbAB5AC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAaQBuAHAAdQB0AF8AYQAgAFQAaABlACAAZABpAHYAaQBkAGUAbgBkACAAQgBpAGcASQBuAHQAIABzAHQAcgBpAG4AZwAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGkAbgBwAHUAdABfAGIAIABUAGgAZQAgAGQAaQB2AGkAcwBvAHIAIABCAGkAZwBJAG4AdAAgAHMAdAByAGkAbgBnAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAWwB1AHMAZQBfAGYAbABvAG8AcgBdACAATwBwAHQAaQBvAG4AYQBsACAAYgBvAG8AbABlAGEAbgAuACAAVABSAFUARQAgAGYAbwByACAAUAB5AHQAaABvAG4ALQBzAHQAeQBsAGUAIABGAGwAbwBvAHIAIABkAGkAdgBpAHMAaQBvAG4ALAAgAEYAQQBMAFMARQAgAGYAbwByACAAVAByAHUAbgBjAGEAdABlAGQALgAgAEQAZQBmAGEAdQBsAHQAcwAgAHQAbwAgAEYAQQBMAFMARQAuAFwAbgAgACoALwBcAG4ARABpAHYATQBvAGQAIAA9ACAATABBAE0AQgBEAEEAKABpAG4AcAB1AHQAXwBhACwAIABpAG4AcAB1AHQAXwBiACwAIABbAHUAcwBlAF8AZgBsAG8AbwByAF0ALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AHIAXwBuAG8AcgBtAF8AYQAsACAATgBvAHIAbQAoAGkAbgBwAHUAdABfAGEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AHIAXwBuAG8AcgBtAF8AYgAsACAATgBvAHIAbQAoAGkAbgBwAHUAdABfAGIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwBpAGcAbgBfAGEALAAgAEIAaQBnAEkAbgB0AC4AUwBpAGcAbgAoAHMAdAByAF8AbgBvAHIAbQBfAGEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwBpAGcAbgBfAGIALAAgAEIAaQBnAEkAbgB0AC4AUwBpAGcAbgAoAHMAdAByAF8AbgBvAHIAbQBfAGIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAaQBzAF8AZgBsAG8AbwByAF8AZABpAHYALAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAdQBzAGUAXwBmAGwAbwBvAHIAKQAsACAARgBBAEwAUwBFACwAIAB1AHMAZQBfAGYAbABvAG8AcgApACwAXABuACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAHMAaQBnAG4AXwBiACAAPQAgADAALAAgACMARABJAFYALwAwACEALABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAHMAaQBnAG4AXwBhACAAPQAgADAALAAgAHsAXAAiADAAXAAiADsAXAAiADAAXAAiAH0ALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABrACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBTAGEAZgBlAEsAKABcACIARABJAFYAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBhACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBTAHAAbABpAHQAKABCAGkAZwBJAG4AdAAuAEEAYgBzACgAcwB0AHIAXwBuAG8AcgBtAF8AYQApACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBiACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBTAHAAbABpAHQAKABCAGkAZwBJAG4AdAAuAEEAYgBzACgAcwB0AHIAXwBuAG8AcgBtAF8AYgApACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABwAGEAYwBrAGUAZABfAHIAZQBzAHUAbAB0ACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBEAGkAdgBSAG8AdQB0AGUAcgAoAGwAaQBtAGIAcwBfAGEALAAgAGwAaQBtAGIAcwBfAGIALAAgAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAZQBuAF8AcgBlAG0AYQBpAG4AZABlAHIALAAgAEkATgBEAEUAWAAoAHAAYQBjAGsAZQBkAF8AcgBlAHMAdQBsAHQALAAgADEALAAgADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAHIAZQBtAGEAaQBuAGQAZQByACwAIABDAEgATwBPAFMARQBSAE8AVwBTACgAcABhAGMAawBlAGQAXwByAGUAcwB1AGwAdAAsACAAUwBFAFEAVQBFAE4AQwBFACgAbABlAG4AXwByAGUAbQBhAGkAbgBkAGUAcgAsACAAMQAsACAAMgApACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBxAHUAbwB0AGkAZQBuAHQALAAgAEQAUgBPAFAAKABwAGEAYwBrAGUAZABfAHIAZQBzAHUAbAB0ACwAIABsAGUAbgBfAHIAZQBtAGEAaQBuAGQAZQByACAAKwAgADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGYAaQBuAGEAbABfAHMAaQBnAG4ALAAgAHMAaQBnAG4AXwBhACAAKgAgAHMAaQBnAG4AXwBiACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcwB0AHIAXwBtAGUAcgBnAGUAZABfAHEALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAE0AZQByAGcAZQAoAGwAaQBtAGIAcwBfAHEAdQBvAHQAaQBlAG4AdAAsACAAawApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcwB0AHIAXwBtAGUAcgBnAGUAZABfAHIALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAE0AZQByAGcAZQAoAGwAaQBtAGIAcwBfAHIAZQBtAGEAaQBuAGQAZQByACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABzAHQAcgBfAHQAcgB1AG4AYwBfAHEALAAgAEkARgAoAEEATgBEACgAZgBpAG4AYQBsAF8AcwBpAGcAbgAgAD0AIAAtADEALAAgAHMAdAByAF8AbQBlAHIAZwBlAGQAXwBxACAAPAA+ACAAXAAiADAAXAAiACkAIAAsACAAXAAiAC0AXAAiACAAJgAgAHMAdAByAF8AbQBlAHIAZwBlAGQAXwBxACwAIABzAHQAcgBfAG0AZQByAGcAZQBkAF8AcQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcwB0AHIAXwB0AHIAdQBuAGMAXwByACwAIABJAEYAKABhAG4AZAAoAHMAaQBnAG4AXwBhACAAPQAgAC0AMQAsACAAcwB0AHIAXwBtAGUAcgBnAGUAZABfAHIAIAA8AD4AIABcACIAMABcACIAKQAsACAAXAAiAC0AXAAiACAAJgAgAHMAdAByAF8AbQBlAHIAZwBlAGQAXwByACwAIABzAHQAcgBfAG0AZQByAGcAZQBkAF8AcgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAARgBsAG8AbwByACAAQwBvAHIAcgBlAGMAdABpAG8AbgAgAGkAZgAgAGYAbABvAG8AcgAgAGkAcwAgAHIAZQBxAHUAZQBzAHQAZQBkACwAIABzAGkAZwBuAHMAIABkAGkAZgBmAGUAcgAsACAAYQBuAGQAIAByAGUAbQBhAGkAbgBkAGUAcgAgAGkAcwAgAG4AbwBuAC0AegBlAHIAbwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABuAGUAZQBkAHMAXwBmAGwAbwBvAHIAXwBjAG8AcgByAGUAYwB0AGkAbwBuACwAIABBAE4ARAAoAGkAcwBfAGYAbABvAG8AcgBfAGQAaQB2ACwAIABmAGkAbgBhAGwAXwBzAGkAZwBuACAAPQAgAC0AMQAsACAAcwB0AHIAXwBtAGUAcgBnAGUAZABfAHIAIAA8AD4AIABcACIAMABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHMAdAByAF8AZgBpAG4AYQBsAF8AcQAsACAASQBGACgAbgBlAGUAZABzAF8AZgBsAG8AbwByAF8AYwBvAHIAcgBlAGMAdABpAG8AbgAsACAAUwB1AGIAKABzAHQAcgBfAHQAcgB1AG4AYwBfAHEALAAgAFwAIgAxAFwAIgApACwAIABzAHQAcgBfAHQAcgB1AG4AYwBfAHEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHMAdAByAF8AZgBpAG4AYQBsAF8AcgAsACAASQBGACgAbgBlAGUAZABzAF8AZgBsAG8AbwByAF8AYwBvAHIAcgBlAGMAdABpAG8AbgAsACAAQQBkAGQAKABzAHQAcgBfAHQAcgB1AG4AYwBfAHIALAAgAHMAdAByAF8AbgBvAHIAbQBfAGIAKQAsACAAcwB0AHIAXwB0AHIAdQBuAGMAXwByACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABWAFMAVABBAEMASwAoAHMAdAByAF8AZgBpAG4AYQBsAF8AcQAsACAAcwB0AHIAXwBmAGkAbgBhAGwAXwByACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAApACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAEQAaQB2AGkAZABlAHMAIAB0AGgAZQAgAGYAaQByAHMAdAAgAEIAaQBnAEkAbgB0ACAAYgB5ACAAdABoAGUAIABzAGUAYwBvAG4AZAAgACgAQQAgAC8AIABCACkALgAgAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGkAbgBwAHUAdABfAGEAIABUAGgAZQAgAGQAaQB2AGkAZABlAG4AZAAgAEIAaQBnAEkAbgB0ACAAcwB0AHIAaQBuAGcALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABpAG4AcAB1AHQAXwBiACAAVABoAGUAIABkAGkAdgBpAHMAbwByACAAQgBpAGcASQBuAHQAIABzAHQAcgBpAG4AZwAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAFsAdQBzAGUAXwBmAGwAbwBvAHIAXQAgAE8AcAB0AGkAbwBuAGEAbAAgAGIAbwBvAGwAZQBhAG4ALgAgAFQAUgBVAEUAIABmAG8AcgAgAFAAeQB0AGgAbwBuAC0AcwB0AHkAbABlACAARgBsAG8AbwByACAAZABpAHYAaQBzAGkAbwBuAC4AIABEAGUAZgBhAHUAbAB0AHMAIAB0AG8AIABGAEEATABTAEUALgBcAG4AIAAqAC8AXABuAEQAaQB2ACAAPQAgAEwAQQBNAEIARABBACgAaQBuAHAAdQB0AF8AYQAsACAAaQBuAHAAdQB0AF8AYgAsACAAWwB1AHMAZQBfAGYAbABvAG8AcgBdACwAXABuACAAIAAgACAASQBOAEQARQBYACgARABpAHYATQBvAGQAKABpAG4AcAB1AHQAXwBhACwAIABpAG4AcAB1AHQAXwBiACwAIAB1AHMAZQBfAGYAbABvAG8AcgApACwAIAAxACwAIAAxACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABDAG8AbQBwAHUAdABlAHMAIAB0AGgAZQAgAHIAZQBtAGEAaQBuAGQAZQByACAAbwBmACAAQQAgAC8AIABCAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAaQBuAHAAdQB0AF8AYQAgAFQAaABlACAAZABpAHYAaQBkAGUAbgBkACAAQgBpAGcASQBuAHQAIABzAHQAcgBpAG4AZwAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGkAbgBwAHUAdABfAGIAIABUAGgAZQAgAGQAaQB2AGkAcwBvAHIAIABCAGkAZwBJAG4AdAAgAHMAdAByAGkAbgBnAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAWwB1AHMAZQBfAGYAbABvAG8AcgBdACAATwBwAHQAaQBvAG4AYQBsACAAYgBvAG8AbABlAGEAbgAuACAAVABSAFUARQAgAGYAbwByACAAUAB5AHQAaABvAG4ALQBzAHQAeQBsAGUAIABNAG8AZAB1AGwAbwAuACAARABlAGYAYQB1AGwAdABzACAAdABvACAARgBBAEwAUwBFAC4AXABuACAAKgAvAFwAbgBNAG8AZAAgAD0AIABMAEEATQBCAEQAQQAoAGkAbgBwAHUAdABfAGEALAAgAGkAbgBwAHUAdABfAGIALAAgAFsAdQBzAGUAXwBmAGwAbwBvAHIAXQAsAFwAbgAgACAAIAAgAEkATgBEAEUAWAAoAEQAaQB2AE0AbwBkACgAaQBuAHAAdQB0AF8AYQAsACAAaQBuAHAAdQB0AF8AYgAsACAAdQBzAGUAXwBmAGwAbwBvAHIAKQAsACAAMgAsACAAMQApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAAUgBhAGkAcwBlAHMAIABhACAAQgBpAGcASQBuAHQAIABiAGEAcwBlACAAdABvACAAdABoAGUAIABwAG8AdwBlAHIAIABvAGYAIABhACAAQgBpAGcASQBuAHQAIABlAHgAcABvAG4AZQBuAHQALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABiAGEAcwBlACAAVABoAGUAIABiAGEAcwBlACAAQgBpAGcASQBuAHQAIABzAHQAcgBpAG4AZwAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGUAeABwAG8AbgBlAG4AdAAgAFQAaABlACAAZQB4AHAAbwBuAGUAbgB0ACAAQgBpAGcASQBuAHQAIABzAHQAcgBpAG4AZwAuAFwAbgAgACoALwBcAG4AUABvAHcAIAA9ACAATABBAE0AQgBEAEEAKABiAGEAcwBlACwAIABlAHgAcABvAG4AZQBuAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AHIAXwBuAG8AcgBtAF8AYgBhAHMAZQAsACAATgBvAHIAbQAoAGIAYQBzAGUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AHIAXwBuAG8AcgBtAF8AZQB4AHAALAAgAE4AbwByAG0AKABlAHgAcABvAG4AZQBuAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwBpAGcAbgBfAGIAYQBzAGUALAAgAEIAaQBnAEkAbgB0AC4AUwBpAGcAbgAoAHMAdAByAF8AbgBvAHIAbQBfAGIAYQBzAGUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwBpAGcAbgBfAGUAeABwACwAIABCAGkAZwBJAG4AdAAuAFMAaQBnAG4AKABzAHQAcgBfAG4AbwByAG0AXwBlAHgAcAApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AHIAXwBhAGIAcwBfAGIAYQBzAGUALAAgAEIAaQBnAEkAbgB0AC4AQQBiAHMAKABzAHQAcgBfAG4AbwByAG0AXwBiAGEAcwBlACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAdAByAF8AYQBiAHMAXwBlAHgAcAAsACAAQgBpAGcASQBuAHQALgBBAGIAcwAoAHMAdAByAF8AbgBvAHIAbQBfAGUAeABwACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIABpAHMAXwBlAHgAcABfAGUAdgBlAG4ALAAgAEkAUwBFAFYARQBOACgAVgBBAEwAVQBFACgAUgBJAEcASABUACgAcwB0AHIAXwBuAG8AcgBtAF8AZQB4AHAALAAgADEAKQApACkALABcAG4AIAAgACAAIAAgACAAIAAgAGYAaQBuAGEAbABfAHMAaQBnAG4ALAAgAEkARgAoAHMAaQBnAG4AXwBiAGEAcwBlACAAPQAgAC0AMQAsACAASQBGACgAaQBzAF8AZQB4AHAAXwBlAHYAZQBuACwAIAAxACwAIAAtADEAKQAsACAAcwBpAGcAbgBfAGIAYQBzAGUAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAC8ALwAgAEgAYQBuAGQAbABlACAAbQBhAHQAaABlAG0AYQB0AGkAYwBhAGwAIABiAG8AdQBuAGQAYQByAGkAZQBzACAAYQBuAGQAIABiAGEAcwBlACAAbABpAG0AaQB0AHMAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABzAHQAcgBfAGEAYgBzAF8AYgBhAHMAZQAgAD0AIABcACIAMABcACIALAAgAEkARgAoAHMAdAByAF8AbgBvAHIAbQBfAGUAeABwACAAPQAgAFwAIgAwAFwAIgAsACAAIwBOAFUATQAhACwAIABcACIAMABcACIAKQAsACAALwAvACAAMABeADAAIABpAHMAIAB1AG4AZABlAGYAaQBuAGUAZABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAHMAdAByAF8AYQBiAHMAXwBiAGEAcwBlACAAPQAgAFwAIgAxAFwAIgAsACAASQBGACgAZgBpAG4AYQBsAF8AcwBpAGcAbgAgAD0AIAAtADEALAAgAFwAIgAtADEAXAAiACwAIABcACIAMQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAcwBpAGcAbgBfAGUAeABwACAAPQAgAC0AMQAsACAAXAAiADAAXAAiACwAIAAvAC8AIABJAG4AdABlAGcAZQByACAAdAByAHUAbgBjAGEAdABpAG8AbgA6ACAAbgBlAGcAYQB0AGkAdgBlACAAZQB4AHAAbwBuAGUAbgB0AHMAIAB5AGkAZQBsAGQAIAAwACAAZgBvAHIAIABiAGEAcwBlAHMAIAA+AD0AIAAyAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAcwB0AHIAXwBuAG8AcgBtAF8AZQB4AHAAIAA9ACAAXAAiADAAXAAiACwAIABcACIAMQBcACIALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABSAGUAcwB1AGwAdABzACAAZgByAG8AbQAgAGUAeABwAG8AbgBlAG4AdABzACAAZwByAGUAYQB0AGUAcgAgAHQAaABhAG4AIAA2ACAAZABpAGcAaQB0AHMAIABjAGEAbgBuAG8AdAAgAGIAZQAgAGQAaQBzAHAAbABhAHkAZQBkAC4AXABuACAAIAAgACAAIAAgACAAIABJAEYAKABMAEUATgAoAHMAdAByAF8AbgBvAHIAbQBfAGUAeABwACkAIAA+ACAANgAsACAAIwBOAFUATQAhACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbgB1AG0AXwBlAHgAcAAsACAAVgBBAEwAVQBFACgAcwB0AHIAXwBuAG8AcgBtAF8AZQB4AHAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAEEAcABwAHIAbwB4AGkAbQBhAHQAZQAgAHQAaABlACAAZgBpAG4AYQBsACAAYwBoAGEAcgBhAGMAdABlAHIAIABjAG8AdQBuAHQAOgAgAEIAIAAqACAATABvAGcAMQAwACgAQQApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGIAYQBzAGUAXwBsAG8AZwAxADAALAAgAEwATwBHADEAMAAoAFYAQQBMAFUARQAoAEwARQBGAFQAKABzAHQAcgBfAGEAYgBzAF8AYgBhAHMAZQAsACAAMQA0ACkAKQApACAAKwAgAE0AQQBYACgAMAAsACAATABFAE4AKABzAHQAcgBfAGEAYgBzAF8AYgBhAHMAZQApACAALQAgADEANAApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAYQBwAHAAcgBvAHgAXwBkAGkAZwBpAHQAcwAsACAAbgB1AG0AXwBlAHgAcAAgACoAIABiAGEAcwBlAF8AbABvAGcAMQAwACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEkARgAoAGEAcABwAHIAbwB4AF8AZABpAGcAaQB0AHMAIAA+ACAAMwAyADcANgA2ACwAIAAjAE4AVQBNACEALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGsALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFMAYQBmAGUASwAoAFwAIgBNAFUATABcACIALAAgAGEAcABwAHIAbwB4AF8AZABpAGcAaQB0AHMAIAAvACAAMgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGIAYQBzAGUALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFMAcABsAGkAdAAoAHMAdAByAF8AYQBiAHMAXwBiAGEAcwBlACwAIABrACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGYAaQBuAGEAbAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBQAG8AdwAoAGwAaQBtAGIAcwBfAGIAYQBzAGUALAAgAHMAdAByAF8AbgBvAHIAbQBfAGUAeABwACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcwB0AHIAXwBtAGUAcgBnAGUAZAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4ATQBlAHIAZwBlACgAbABpAG0AYgBzAF8AZgBpAG4AYQBsACwAIABrACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEkARgAoAGYAaQBuAGEAbABfAHMAaQBnAG4AIAA9ACAALQAxACwAIABcACIALQBcACIAIAAmACAAcwB0AHIAXwBtAGUAcgBnAGUAZAAsACAAcwB0AHIAXwBtAGUAcgBnAGUAZAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAKQApACkAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4ALwAvADEAMgAzADQANQA2ADcAOAA5ADAAMQAyADMANAA1ADYANwA4ADkAMAAxADIAMwA0ADUANgA3ADgAOQAwADEAMgAzADQANQA2ADcAOAA5ADAAMQAyADMANAA1ADYANwA4ADkAMAAxADIAMwA0ADUANgA3ADgAOQAwADEAMgAzADQANQA2ADcAOAA5AC0AMQAyADMANAA1ADYANwAtADkAMAAxADIAMwA0ADUANgA3ADgAOQAwADEAMgAzADQANQA2ADcAOAA5ADAAMQAyADMANAA1ADYANwA4ADkAMAAxADIAMwA0ADUANgA3AC0AXABuAC8AKgAqAFwAbgAgACoAIABDAGEAbABjAHUAbABhAHQAZQBzACAAdABoAGUAIABpAG4AdABlAGcAZQByACAAcwBxAHUAYQByAGUAIAByAG8AbwB0ACAAKABmAGwAbwBvAHIAKQAgAG8AZgAgAGEAIABCAGkAZwBJAG4AdAAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGkAbgBwAHUAdAAgAFQAaABlACAAcgBhAGQAaQBjAGEAbgBkACAAQgBpAGcASQBuAHQAIABzAHQAcgBpAG4AZwAuAFwAbgAgACoALwBcAG4AUwBxAHIAdAAgAD0AIABMAEEATQBCAEQAQQAoAGkAbgBwAHUAdAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABzAHQAcgBfAG4AbwByAG0ALAAgAE4AbwByAG0AKABpAG4AcAB1AHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwBpAGcAbgBfAG4ALAAgAEIAaQBnAEkAbgB0AC4AUwBpAGcAbgAoAHMAdAByAF8AbgBvAHIAbQApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAcwBpAGcAbgBfAG4AIAA9ACAALQAxACwAIAAjAE4AVQBNACEALABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAHMAdAByAF8AbgBvAHIAbQAgAD0AIABcACIAMABcACIALAAgAFwAIgAwAFwAIgAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAcwB0AHIAXwBuAG8AcgBtACAAPQAgAFwAIgAxAFwAIgAsACAAXAAiADEAXAAiACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABlAG4AXwBuAG8AcgBtACwAIABMAEUATgAoAHMAdAByAF8AbgBvAHIAbQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbgB1AG0AXwBzAGUAZQBkAF8AcAByAGUAYwBpAHMAaQBvAG4ALAAgAEkARgAoAGwAZQBuAF8AbgBvAHIAbQAgADwAPQAgADEANAAsACAAbABlAG4AXwBuAG8AcgBtACwAIABJAEYAKABJAFMARQBWAEUATgAoAGwAZQBuAF8AbgBvAHIAbQApACwAIAAxADQALAAgADEAMwApACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABzAHQAcgBfAG4AYQB0AGkAdgBlAF8AcAByAGUAYwBpAHMAaQBvAG4ALAAgAEwARQBGAFQAKABzAHQAcgBfAG4AbwByAG0ALAAgAG4AdQBtAF8AcwBlAGUAZABfAHAAcgBlAGMAaQBzAGkAbwBuACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABuAHUAbQBfAG4AYQB0AGkAdgBlAF8AcAByAGUAYwBpAHMAaQBvAG4ALAAgAFYAQQBMAFUARQAoAHMAdAByAF8AbgBhAHQAaQB2AGUAXwBwAHIAZQBjAGkAcwBpAG8AbgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbgB1AG0AXwBtAGEAZwBuAGkAdAB1AGQAZQBfAHoAZQByAG8AZQBzACwAIAAoAGwAZQBuAF8AbgBvAHIAbQAgAC0AIABuAHUAbQBfAHMAZQBlAGQAXwBwAHIAZQBjAGkAcwBpAG8AbgApACAALwAgADIALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcwB0AHIAXwBwAHIAZQBmAGkAeAAsACAAVABFAFgAVAAoAFIATwBVAE4ARABVAFAAKABTAFEAUgBUACgAbgB1AG0AXwBuAGEAdABpAHYAZQBfAHAAcgBlAGMAaQBzAGkAbwBuACkALAAgADAAKQAgACsAIAAxACwAIABcACIAMABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHMAdAByAF8AcwBlAGUAZAAsACAAcwB0AHIAXwBwAHIAZQBmAGkAeAAgACYAIABSAEUAUABUACgAXAAiADAAXAAiACwAIABuAHUAbQBfAG0AYQBnAG4AaQB0AHUAZABlAF8AegBlAHIAbwBlAHMAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIABTAGMAYQBsAGUAcwAgAGsAIABiAHkAIAB0AGgAZQAgAG0AYQB4AGkAbQB1AG0AIABvAHYAZQByAGwAYQBwACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAawAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwBhAGYAZQBLACgAXAAiAE0AVQBMAFwAIgAsACAAbABlAG4AXwBuAG8AcgBtACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwByAGEAZABpAGMAYQBuAGQALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFMAcABsAGkAdAAoAHMAdAByAF8AbgBvAHIAbQAsACAAawApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AcwBlAGUAZAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwBwAGwAaQB0ACgAcwB0AHIAXwBzAGUAZQBkACwAIABrACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AZgBpAG4AYQBsACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAFMAcQByAHQAKABsAGkAbQBiAHMAXwByAGEAZABpAGMAYQBuAGQALAAgAGwAaQBtAGIAcwBfAHMAZQBlAGQALAAgAGsAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBNAGUAcgBnAGUAKABsAGkAbQBiAHMAXwBmAGkAbgBhAGwALAAgAGsAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACkAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABDAG8AbQBwAHUAdABlAHMAIAB0AGgAZQAgAGYAYQBjAHQAbwByAGkAYQBsACAAbwBmACAAYQAgAEIAaQBnAEkAbgB0ACAAKABuACEAKQAgAHUAcwBpAG4AZwAgAFAAZQB0AGUAcgAgAEwAdQBzAGMAaABuAHkAJwBzACAAUAByAGkAbQBlACAAUwB3AGkAbgBnACAAYQBsAGcAbwByAGkAdABoAG0ALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABpAG4AcAB1AHQAIABUAGgAZQAgAEIAaQBnAEkAbgB0ACAAcwB0AHIAaQBuAGcALgAgAE0AYQB4AGkAbQB1AG0AIABzAHUAcABwAG8AcgB0AGUAZAAgAGkAbgBwAHUAdAAgAGkAcwAgADkAMgA3ADMALgBcAG4AIAAqAC8AXABuAEYAYQBjAHQAIAA9ACAATABBAE0AQgBEAEEAKABpAG4AcAB1AHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AHIAXwBuAG8AcgBtACwAIABOAG8AcgBtACgAaQBuAHAAdQB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAaQBnAG4AXwBuACwAIABCAGkAZwBJAG4AdAAuAFMAaQBnAG4AKABzAHQAcgBfAG4AbwByAG0AKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAHMAaQBnAG4AXwBuACAAPQAgAC0AMQAsACAAIwBOAFUATQAhACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABzAHQAcgBfAG4AbwByAG0AIAA9ACAAXAAiADAAXAAiACwAIABcACIAMQBcACIALABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAHMAdAByAF8AbgBvAHIAbQAgAD0AIABcACIAMQBcACIALAAgAFwAIgAxAFwAIgAsAFwAbgAgACAAIAAgACAAIAAgACAALwAvACAARgBpAHIAZQB3AGEAbABsACAAMQA6ACAAVAByAGEAcAAgAG0AYQBzAHMAaQB2AGUAIABzAHQAcgBpAG4AZwBzACAAYgBlAGYAbwByAGUAIAB0AGgAZQB5ACAAaABpAHQAIABWAEEATABVAEUAKAApAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgATABFAE4AKABzAHQAcgBfAG4AbwByAG0AKQAgAD4AIAA0ACwAIAAjAE4AVQBNACEALAAgAFwAbgAgACAAIAAgACAAIAAgACAALwAvACAARgBpAHIAZQB3AGEAbABsACAAMgA6ACAAVAByAGEAcAAgAG0AYQB0AGgAZQBtAGEAdABpAGMAYQBsACAAYwBlAGkAbABpAG4AZwBcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAFYAQQBMAFUARQAoAHMAdAByAF8AbgBvAHIAbQApACAAPgAgADkAMgA3ADMALAAgACMATgBVAE0AIQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAG4AdQBtAF8AbgAsACAAVgBBAEwAVQBFACgAcwB0AHIAXwBuAG8AcgBtACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABnAGwAbwBiAGEAbABfAHAAcgBpAG0AZQBzACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBOAGEAdABpAHYAZQBQAHIAaQBtAGUAcwAoAG4AdQBtAF8AbgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUAByAGkAbQBlAFMAdwBpAG4AZwBLAGUAcgBuAGUAbAAoAG4AdQBtAF8AbgAsACAAZwBsAG8AYgBhAGwAXwBwAHIAaQBtAGUAcwApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAKQApACkAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABSAGUAdAB1AHIAbgBzACAAdABoAGUAIABtAGkAbgBpAG0AdQBtACAAQgBpAGcASQBuAHQAIABmAHIAbwBtACAAYQBuACAAYQByAHIAYQB5ACAAbwByACAAcgBhAG4AZwBlAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAcgBhAG4AZwBlACAAQQAgAGMAbwBuAHQAaQBnAHUAbwB1AHMAIAByAGEAbgBnAGUAIABvAHIAIABhAHIAcgBhAHkAIABvAGYAIABCAGkAZwBJAG4AdAAgAHMAdAByAGkAbgBnAHMALgBcAG4AIAAqAC8AXABuAE0AaQBuACAAPQAgAEwAQQBNAEIARABBACgAcgBhAG4AZwBlACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAGYAbABhAHQAdABlAG4AZQBkAF8AYwBvAGwALAAgAFQATwBDAE8ATAAoAHIAYQBuAGcAZQAsACAAMQApACwAXABuACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAE8AUgAoAEkAUwBFAFIAUgBPAFIAKABmAGwAYQB0AHQAZQBuAGUAZABfAGMAbwBsACkALAAgAFIATwBXAFMAKABmAGwAYQB0AHQAZQBuAGUAZABfAGMAbwBsACkAIAA9ACAAMAApACwAIABcACIAMABcACIALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVAByAGUAZQBDAG8AbQBwAGEAcgBlACgATQBBAFAAKABmAGwAYQB0AHQAZQBuAGUAZABfAGMAbwBsACwAIABCAGkAZwBJAG4AdAAuAE4AbwByAG0AKQAsACAALQAxACkAXABuACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABSAGUAdAB1AHIAbgBzACAAdABoAGUAIABtAGEAeABpAG0AdQBtACAAQgBpAGcASQBuAHQAIABmAHIAbwBtACAAYQBuACAAYQByAHIAYQB5ACAAbwByACAAcgBhAG4AZwBlAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAcgBhAG4AZwBlACAAQQAgAGMAbwBuAHQAaQBnAHUAbwB1AHMAIAByAGEAbgBnAGUAIABvAHIAIABhAHIAcgBhAHkAIABvAGYAIABCAGkAZwBJAG4AdAAgAHMAdAByAGkAbgBnAHMALgBcAG4AIAAqAC8AXABuAE0AYQB4ACAAPQAgAEwAQQBNAEIARABBACgAcgBhAG4AZwBlACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAGYAbABhAHQAdABlAG4AZQBkAF8AYwBvAGwALAAgAFQATwBDAE8ATAAoAHIAYQBuAGcAZQAsACAAMQApACwAXABuACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAE8AUgAoAEkAUwBFAFIAUgBPAFIAKABmAGwAYQB0AHQAZQBuAGUAZABfAGMAbwBsACkALAAgAFIATwBXAFMAKABmAGwAYQB0AHQAZQBuAGUAZABfAGMAbwBsACkAIAA9ACAAMAApACwAIABcACIAMABcACIALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVAByAGUAZQBDAG8AbQBwAGEAcgBlACgATQBBAFAAKABmAGwAYQB0AHQAZQBuAGUAZABfAGMAbwBsACwAIABCAGkAZwBJAG4AdAAuAE4AbwByAG0AKQAsACAAMQApAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAIgB9AF0ALAAiAHAAcgBvAGoAZQBjAHQATgBhAG0AZQBzACIAOgBbACIAdABlAHMAdABfAEIAaQBnAEkAbgB0AC4ASwBuAHUAdABoAEQAaQB2AGkAcwBpAG8AbgAiACwAIgB0AGUAcwB0AF8AQgBpAGcASQBuAHQALgBOAGUAdwB0AG8AbgBSAGEAcABoAHMAbwBuAEQAaQB2AGkAcwBpAG8AbgAiACwAIgB0AGUAcwB0AF8AQgBpAGcASQBuAHQALgBEAGkAdgBpAHMAaQBvAG4AQQBsAGcAbwByAGkAdABoAG0AcwAiACwAIgB0AGUAcwB0AF8AQgBpAGcASQBuAHQALgBEAGkAdgBpAHMAaQBvAG4AQQBsAGcAbwByAGkAdABoAG0AQwBvAG0AcABhAHIAaQBzAG8AbgAiACwAIgB0AGUAcwB0AF8AQgBpAGcASQBuAHQALgBEAGkAdgBpAHMAaQBvAG4AQgBlAG4AYwBoAG0AYQByAGsAQwBhAHMAZQBzACIALAAiAHQAZQBzAHQAXwBCAGkAZwBJAG4AdAAuAEEAcwB5AG0AbQBlAHQAcgBpAGMAQQBCAEcAcgBpAGQAIgAsACIAdABlAHMAdABfAEIAaQBnAEkAbgB0AC4ARgBhAGMAdABvAHIAaQBhAGwAQQBsAGcAbwByAGkAdABoAG0AcwAiACwAIgB0AGUAcwB0AF8AQgBpAGcASQBuAHQALgBGAGEAYwB0AG8AcgBpAGEAbABDAG8AbQBwAGEAcgBpAHMAbwBuACIALAAiAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFMAYQBmAGUASwAiACwAIgBjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBTAHAAbABpAHQAIgAsACIAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4ATQBlAHIAZwBlACIALAAiAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAEMAYQByAHIAeQAiACwAIgBjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAEMAbwBtAHAAYQByAGUAIgAsACIAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBBAGQAZAAiACwAIgBjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAFMAdQBiACIALAAiAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFUATQBhAHQAcgBpAHgAUwB1AG0AIgAsACIAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AQQBkAGQAUwB1AGIAUgBvAHUAdABlAHIAIgAsACIAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBNAHUAbAAiACwAIgBjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBGAGkAbgBkAFEAdQBvAHQAaQBlAG4AdABMAGkAbQBiACIALAAiAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAEsAbgB1AHQAaABEAGkAdgAiACwAIgBjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBEAGkAdgBSAG8AdQB0AGUAcgAiACwAIgBjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBOAGUAdwB0AG8AbgBSAGEAcABoAHMAbwBuAFMAZQBlAGQAIgAsACIAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4ATgBlAHcAdABvAG4AUgBhAHAAaABzAG8AbgBSAGUAYwBpAHAAcgBvAGMAYQBsACIALAAiAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAE4AZQB3AHQAbwBuAFIAYQBwAGgAcwBvAG4ARABpAHYAIgAsACIAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBQAG8AdwAiACwAIgBjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAFMAcQByAHQAIgAsACIAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4ATgBhAHQAaQB2AGUAUAByAGkAbQBlAHMAIgAsACIAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBUAGUAeAB0AE0AdQBsACIALAAiAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFQAZQB4AHQAVAByAGUAZQBQAHIAbwBkACIALAAiAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAE4AYQB0AGkAdgBlAFMAdwBpAG4AZwBFAHgAcABvAG4AZQBuAHQAcwAiACwAIgBjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBTAHcAaQBuAGcAVABlAHIAbQAiACwAIgBjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBQAHIAaQBtAGUAUwB3AGkAbgBnAEsAZQByAG4AZQBsACIALAAiAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFQAcgBlAGUAQwBvAG0AcABhAHIAZQAiACwAIgBCAGkAZwBJAG4AdAAuAE4AbwByAG0AIgAsACIAQgBpAGcASQBuAHQALgBTAGkAZwBuACIALAAiAEIAaQBnAEkAbgB0AC4ASQBzAFoAZQByAG8AIgAsACIAQgBpAGcASQBuAHQALgBJAHMATgBlAGcAIgAsACIAQgBpAGcASQBuAHQALgBJAHMARQB2AGUAbgAiACwAIgBCAGkAZwBJAG4AdAAuAEkAcwBPAGQAZAAiACwAIgBCAGkAZwBJAG4AdAAuAEEAYgBzACIALAAiAEIAaQBnAEkAbgB0AC4AQwBvAG0AcABhAHIAZQAiACwAIgBCAGkAZwBJAG4AdAAuAEEAZABkACIALAAiAEIAaQBnAEkAbgB0AC4AUwB1AGIAIgAsACIAQgBpAGcASQBuAHQALgBTAHUAbQAiACwAIgBCAGkAZwBJAG4AdAAuAE0AdQBsACIALAAiAEIAaQBnAEkAbgB0AC4AUgBhAG4AZABBAHIAcgBhAHkAIgAsACIAQgBpAGcASQBuAHQALgBEAGkAdgBNAG8AZAAiACwAIgBCAGkAZwBJAG4AdAAuAEQAaQB2ACIALAAiAEIAaQBnAEkAbgB0AC4ATQBvAGQAIgAsACIAQgBpAGcASQBuAHQALgBQAG8AdwAiACwAIgBCAGkAZwBJAG4AdAAuAFMAcQByAHQAIgAsACIAQgBpAGcASQBuAHQALgBGAGEAYwB0ACIALAAiAEIAaQBnAEkAbgB0AC4ATQBpAG4AIgAsACIAQgBpAGcASQBuAHQALgBNAGEAeAAiAF0ALAAiAGwAbwBjAGEAbABlACIAOgB7ACIAbABpAHMAdABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHIAbwB3AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiADsAIgAsACIAYwBvAGwAdQBtAG4AUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgB0AGgAbwB1AHMAYQBuAGQAcwBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHQAaABvAHUAcwBhAG4AZABzAFAAbwBzAGkAdABpAG8AbgBzACIAOgBbADMAXQAsACIAZABlAGMAaQBtAGEAbABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAuACIALAAiAGQAYQB0AGUATwByAGQAZQByACIAOgAiAEQATQBZACIALAAiAGMAdQByAHIAZQBuAGMAeQBTAHkAbQBiAG8AbAAiADoAIgAkACIALAAiAGkAcwBDAHUAcgByAGUAbgBjAHkAUwB5AG0AYgBvAGwATABlAGEAZAAiADoAdAByAHUAZQAsACIAaQBzAEMAdQByAHIAZQBuAGMAeQBTAGUAcABCAHkAUwBwAGEAYwBlACIAOgBmAGEAbABzAGUALAAiAHIAbwB3AEwAZQB0AHQAZQByACIAOgAiAFIAIgAsACIAYwBvAGwAdQBtAG4ATABlAHQAdABlAHIAIgA6ACIAQwAiACwAIgByAGMATABlAGYAdABCAHIAYQBjAGsAZQB0ACIAOgAiAFsAIgAsACIAcgBjAFIAaQBnAGgAdABCAHIAYQBjAGsAZQB0ACIAOgAiAF0AIgAsACIAcwB0AGEAdABlAG0AZQBuAHQAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIAOwAiACwAIgBsAG8AYwBhAGwAZQBOAGEAbQBlACIAOgAiAGUAbgAtAHUAcwAiAH0AfQA=</AFEJSONBlob>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
chore: updated doc-strings and inline comments
</commit_message>
<xml_diff>
--- a/XL-Int.xlsx
+++ b/XL-Int.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30014"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30021"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\foolu\Workspace\Excel\xl-int\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61FEFC49-7320-41B5-95F3-BA9301FA05E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA122BA5-CB32-4C09-82A7-A2CDFE16C591}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="24580" windowHeight="21000" xr2:uid="{36490472-0618-4E80-9469-F609392FABC8}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21220" xr2:uid="{36490472-0618-4E80-9469-F609392FABC8}"/>
   </bookViews>
   <sheets>
     <sheet name="Tests" sheetId="1" r:id="rId1"/>
@@ -19,52 +19,52 @@
     <sheet name="Sheet1" sheetId="6" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="BigInt.Abs" comment="Returns the unsigned magnitude of a BigInt string (absolute value)._x000a_@param input The BigInt string.">_xlfn.LAMBDA(_xlpm.input, _xlfn.LET(_xlpm.str_norm, BigInt.Norm(_xlpm.input), IF(LEFT(_xlpm.str_norm) = "-", MID(_xlpm.str_norm, 2, LEN(_xlpm.str_norm) - 1), _xlpm.str_norm)))</definedName>
-    <definedName name="BigInt.Add" comment="Adds two BigInt strings._x000a_@param input_a The first BigInt string._x000a_@param input_b The second BigInt string.">_xlfn.LAMBDA(_xlpm.input_a,_xlpm.input_b, _xlfn.LET(_xlpm.str_norm_a, BigInt.Norm(_xlpm.input_a), _xlpm.str_norm_b, BigInt.Norm(_xlpm.input_b), _xlpm.sign_a, BigInt.Sign(_xlpm.str_norm_a), _xlpm.sign_b, BigInt.Sign(_xlpm.str_norm_b), _xlpm.k, core_BigInt.SafeK("ADD"), _xlpm.limbs_a, core_BigInt.Split(BigInt.Abs(_xlpm.str_norm_a), _xlpm.k), _xlpm.limbs_b, core_BigInt.Split(BigInt.Abs(_xlpm.str_norm_b), _xlpm.k), _xlpm.packed_result, core_BigInt.AddSubRouter(_xlpm.limbs_a, _xlpm.limbs_b, _xlpm.sign_a, _xlpm.sign_b, _xlpm.k), _xlpm.final_sign, _xlfn.CHOOSEROWS(_xlpm.packed_result, -1), _xlpm.final_limbs, _xlfn.DROP(_xlpm.packed_result, -1), _xlpm.str_merged, core_BigInt.Merge(_xlpm.final_limbs, _xlpm.k), IF(_xlpm.final_sign = -1, "-" &amp; _xlpm.str_merged, _xlpm.str_merged)))</definedName>
-    <definedName name="BigInt.Compare" comment="Compares two BigInt strings. Returns 1 (a &gt; b), -1 (a &lt; b), or 0 (a = b)._x000a_Evaluates signs and lengths. If identical, delegates to native limb array comparison._x000a_@param input_a The first BigInt string._x000a_@param input_b The second BigInt string.">_xlfn.LAMBDA(_xlpm.input_a,_xlpm.input_b, _xlfn.LET(_xlpm.str_norm_a, BigInt.Norm(_xlpm.input_a), _xlpm.str_norm_b, BigInt.Norm(_xlpm.input_b), _xlpm.sign_a, BigInt.Sign(_xlpm.str_norm_a), _xlpm.sign_b, BigInt.Sign(_xlpm.str_norm_b), IF(_xlpm.sign_a &lt;&gt; _xlpm.sign_b, SIGN(_xlpm.sign_a - _xlpm.sign_b), IF(_xlpm.sign_a = 0, 0, _xlfn.LET(_xlpm.len_a, LEN(_xlpm.str_norm_a), _xlpm.len_b, LEN(_xlpm.str_norm_b), IF(_xlpm.len_a &lt;&gt; _xlpm.len_b, SIGN(_xlpm.len_a - _xlpm.len_b) * _xlpm.sign_a, _xlfn.LET(_xlpm.k, core_BigInt.SafeK("ADD"), _xlpm.limbs_a, core_BigInt.Split(BigInt.Abs(_xlpm.str_norm_a), _xlpm.k), _xlpm.limbs_b, core_BigInt.Split(BigInt.Abs(_xlpm.str_norm_b), _xlpm.k), _xlpm.magnitude_comparison, core_BigInt.UCompare(_xlpm.limbs_a, _xlpm.limbs_b), _xlpm.magnitude_comparison * _xlpm.sign_a)))))))</definedName>
-    <definedName name="BigInt.Div" comment="Divides the first BigInt by the second (A / B). _x000a_@param input_a The dividend BigInt string._x000a_@param input_b The divisor BigInt string._x000a_@param [use_floor] Optional boolean. TRUE for Python-style Floor division. Defaults to FALSE.">_xlfn.LAMBDA(_xlpm.input_a,_xlpm.input_b,_xlop.use_floor, INDEX(BigInt.DivMod(_xlpm.input_a, _xlpm.input_b, _xlpm.use_floor), 1, 1))</definedName>
-    <definedName name="BigInt.DivMod" comment="Divides the first BigInt by the second (A / B). _x000a_Returns the quotient and modulus in rows 1 and 2, respectively._x000a_@param input_a The dividend BigInt string._x000a_@param input_b The divisor BigInt string._x000a_@param [use_floor] Optional boolean. TRUE for Python-styl">_xlfn.LAMBDA(_xlpm.input_a,_xlpm.input_b,_xlop.use_floor, _xlfn.LET(_xlpm.str_norm_a, BigInt.Norm(_xlpm.input_a), _xlpm.str_norm_b, BigInt.Norm(_xlpm.input_b), _xlpm.sign_a, BigInt.Sign(_xlpm.str_norm_a), _xlpm.sign_b, BigInt.Sign(_xlpm.str_norm_b), _xlpm.is_floor_div, IF(_xlfn.ISOMITTED(_xlpm.use_floor), FALSE, _xlpm.use_floor), IF(_xlpm.sign_b = 0, #DIV/0!, IF(_xlpm.sign_a = 0, {"0";"0"}, _xlfn.LET(_xlpm.k, core_BigInt.SafeK("DIV"), _xlpm.limbs_a, core_BigInt.Split(BigInt.Abs(_xlpm.str_norm_a), _xlpm.k), _xlpm.limbs_b, core_BigInt.Split(BigInt.Abs(_xlpm.str_norm_b), _xlpm.k), _xlpm.packed_result, core_BigInt.DivRouter(_xlpm.limbs_a, _xlpm.limbs_b, _xlpm.k), _xlpm.len_remainder, INDEX(_xlpm.packed_result, 1, 1), _xlpm.limbs_remainder, _xlfn.CHOOSEROWS(_xlpm.packed_result, _xlfn.SEQUENCE(_xlpm.len_remainder, 1, 2)), _xlpm.limbs_quotient, _xlfn.DROP(_xlpm.packed_result, _xlpm.len_remainder + 1), _xlpm.final_sign, _xlpm.sign_a * _xlpm.sign_b, _xlpm.str_merged_q, core_BigInt.Merge(_xlpm.limbs_quotient, _xlpm.k), _xlpm.str_merged_r, core_BigInt.Merge(_xlpm.limbs_remainder, _xlpm.k), _xlpm.str_trunc_q, IF(AND(_xlpm.final_sign = -1, _xlpm.str_merged_q &lt;&gt; "0"), "-" &amp; _xlpm.str_merged_q, _xlpm.str_merged_q), _xlpm.str_trunc_r, IF(AND(_xlpm.sign_a = -1, _xlpm.str_merged_r &lt;&gt; "0"), "-" &amp; _xlpm.str_merged_r, _xlpm.str_merged_r), _xlpm.needs_floor_correction, AND(_xlpm.is_floor_div, _xlpm.final_sign = -1, _xlpm.str_merged_r &lt;&gt; "0"), _xlpm.str_final_q, IF(_xlpm.needs_floor_correction, BigInt.Sub(_xlpm.str_trunc_q, "1"), _xlpm.str_trunc_q), _xlpm.str_final_r, IF(_xlpm.needs_floor_correction, BigInt.Add(_xlpm.str_trunc_r, _xlpm.str_norm_b), _xlpm.str_trunc_r), _xlfn.VSTACK(_xlpm.str_final_q, _xlpm.str_final_r))))))</definedName>
-    <definedName name="BigInt.Fact" comment="Computes the factorial of a BigInt (n!) using Peter Luschny's Prime Swing algorithm._x000a_@param input The BigInt string. Maximum supported input is 9273.">_xlfn.LAMBDA(_xlpm.input, _xlfn.LET(_xlpm.str_norm, BigInt.Norm(_xlpm.input), _xlpm.sign_n, BigInt.Sign(_xlpm.str_norm), IF(_xlpm.sign_n = -1, #NUM!, IF(_xlpm.str_norm = "0", "1", IF(_xlpm.str_norm = "1", "1", IF(LEN(_xlpm.str_norm) &gt; 4, #NUM!, IF(VALUE(_xlpm.str_norm) &gt; 9273, #NUM!, _xlfn.LET(_xlpm.num_n, VALUE(_xlpm.str_norm), _xlpm.global_primes, core_BigInt.NativePrimes(_xlpm.num_n), core_BigInt.PrimeSwingKernel(_xlpm.num_n, _xlpm.global_primes)))))))))</definedName>
-    <definedName name="BigInt.IsEven" comment="Returns TRUE if the BigInt is even._x000a_@param input The BigInt string.">_xlfn.LAMBDA(_xlpm.input, ISEVEN(VALUE(RIGHT(BigInt.Norm(_xlpm.input)))))</definedName>
-    <definedName name="BigInt.IsNeg" comment="Returns TRUE if the BigInt is negative._x000a_@param input The BigInt string.">_xlfn.LAMBDA(_xlpm.input, LEFT(BigInt.Norm(_xlpm.input)) = "-")</definedName>
-    <definedName name="BigInt.IsOdd" comment="Returns TRUE if the BigInt is odd._x000a_@param input The BigInt string.">_xlfn.LAMBDA(_xlpm.input, ISODD(VALUE(RIGHT(BigInt.Norm(_xlpm.input)))))</definedName>
-    <definedName name="BigInt.IsZero" comment="Returns TRUE if the BigInt is exactly zero._x000a_@param input The BigInt string.">_xlfn.LAMBDA(_xlpm.input, BigInt.Norm(_xlpm.input) = "0")</definedName>
-    <definedName name="BigInt.Max" comment="Returns the maximum BigInt from an array or range._x000a_@param range A contiguous range or array of BigInt strings.">_xlfn.LAMBDA(_xlpm.range, _xlfn.LET(_xlpm.flattened_col, _xlfn.TOCOL(_xlpm.range, 1), IF(OR(ISERROR(_xlpm.flattened_col), ROWS(_xlpm.flattened_col) = 0), "0", core_BigInt.TreeCompare(_xlfn.MAP(_xlpm.flattened_col, BigInt.Norm), 1))))</definedName>
-    <definedName name="BigInt.Min" comment="Returns the minimum BigInt from an array or range._x000a_@param range A contiguous range or array of BigInt strings.">_xlfn.LAMBDA(_xlpm.range, _xlfn.LET(_xlpm.flattened_col, _xlfn.TOCOL(_xlpm.range, 1), IF(OR(ISERROR(_xlpm.flattened_col), ROWS(_xlpm.flattened_col) = 0), "0", core_BigInt.TreeCompare(_xlfn.MAP(_xlpm.flattened_col, BigInt.Norm), -1))))</definedName>
-    <definedName name="BigInt.Mod" comment="Computes the remainder of A / B._x000a_@param input_a The dividend BigInt string._x000a_@param input_b The divisor BigInt string._x000a_@param [use_floor] Optional boolean. TRUE for Python-style Modulo. Defaults to FALSE.">_xlfn.LAMBDA(_xlpm.input_a,_xlpm.input_b,_xlop.use_floor, INDEX(BigInt.DivMod(_xlpm.input_a, _xlpm.input_b, _xlpm.use_floor), 2, 1))</definedName>
-    <definedName name="BigInt.Mul" comment="Multiplies two BigInt strings._x000a_@param input_a The first BigInt string._x000a_@param input_b The second BigInt string.">_xlfn.LAMBDA(_xlpm.input_a,_xlpm.input_b, _xlfn.LET(_xlpm.str_norm_a, BigInt.Norm(_xlpm.input_a), _xlpm.str_norm_b, BigInt.Norm(_xlpm.input_b), _xlpm.sign_a, BigInt.Sign(_xlpm.str_norm_a), _xlpm.sign_b, BigInt.Sign(_xlpm.str_norm_b), _xlpm.len_a, LEN(_xlpm.str_norm_a) - IF(_xlpm.sign_a = -1, 1, 0), _xlpm.len_b, LEN(_xlpm.str_norm_b) - IF(_xlpm.sign_b = -1, 1, 0), IF(OR(_xlpm.sign_a = 0, _xlpm.sign_b = 0), "0", IF(_xlpm.len_a + _xlpm.len_b &gt; 32766, #NUM!, _xlfn.LET(_xlpm.k, core_BigInt.SafeK("MUL", MIN(_xlpm.len_a, _xlpm.len_b)), _xlpm.limbs_a, core_BigInt.Split(BigInt.Abs(_xlpm.str_norm_a), _xlpm.k), _xlpm.limbs_b, core_BigInt.Split(BigInt.Abs(_xlpm.str_norm_b), _xlpm.k), _xlpm.final_limbs, core_BigInt.UMul(_xlpm.limbs_a, _xlpm.limbs_b, _xlpm.k), _xlpm.final_sign, _xlpm.sign_a * _xlpm.sign_b, _xlpm.str_merged, core_BigInt.Merge(_xlpm.final_limbs, _xlpm.k), IF(_xlpm.final_sign = -1, "-" &amp; _xlpm.str_merged, _xlpm.str_merged))))))</definedName>
-    <definedName name="BigInt.Norm" comment="Normalises a BigInt string. Strips leading zeros, resolves &quot;-0&quot; to &quot;0&quot;, and throws #VALUE! on invalid characters._x000a_@param input The BigInt string.">_xlfn.LAMBDA(_xlpm.input, _xlfn.LET(_xlpm.str_input, IF(OR(_xlfn.ISOMITTED(_xlpm.input), _xlpm.input = ""), "0", _xlpm.input &amp; ""), _xlpm.is_value_format, _xlfn.REGEXTEST(_xlpm.str_input, "^-?\d+$"), _xlpm.str_norm, _xlfn.REGEXREPLACE(_xlpm.str_input, "^(-?)0+(?=\d)", "$1"), IF(NOT(_xlpm.is_value_format), VALUE("#VALUE!"), IF(_xlpm.str_norm = "-0", "0", _xlpm.str_norm))))</definedName>
-    <definedName name="BigInt.Pow" comment="Raises a BigInt base to the power of a BigInt exponent._x000a_@param base The base BigInt string._x000a_@param exponent The exponent BigInt string.">_xlfn.LAMBDA(_xlpm.base,_xlpm.exponent, _xlfn.LET(_xlpm.str_norm_base, BigInt.Norm(_xlpm.base), _xlpm.str_norm_exp, BigInt.Norm(_xlpm.exponent), _xlpm.sign_base, BigInt.Sign(_xlpm.str_norm_base), _xlpm.sign_exp, BigInt.Sign(_xlpm.str_norm_exp), _xlpm.str_abs_base, BigInt.Abs(_xlpm.str_norm_base), _xlpm.str_abs_exp, BigInt.Abs(_xlpm.str_norm_exp), _xlpm.is_exp_even, ISEVEN(VALUE(RIGHT(_xlpm.str_norm_exp, 1))), _xlpm.final_sign, IF(_xlpm.sign_base = -1, IF(_xlpm.is_exp_even, 1, -1), _xlpm.sign_base), IF(_xlpm.str_abs_base = "0", IF(_xlpm.str_norm_exp = "0", #NUM!, "0"), IF(_xlpm.str_abs_base = "1", IF(_xlpm.final_sign = -1, "-1", "1"), IF(_xlpm.sign_exp = -1, "0", IF(_xlpm.str_norm_exp = "0", "1", IF(LEN(_xlpm.str_norm_exp) &gt; 6, #NUM!, _xlfn.LET(_xlpm.num_exp, VALUE(_xlpm.str_norm_exp), _xlpm.base_log10,LOG10(VALUE(LEFT(_xlpm.str_abs_base, 14))) + MAX(0, LEN(_xlpm.str_abs_base) - 14), _xlpm.approx_digits, _xlpm.num_exp * _xlpm.base_log10, IF(_xlpm.approx_digits &gt; 32766, #NUM!, _xlfn.LET(_xlpm.k, core_BigInt.SafeK("MUL", _xlpm.approx_digits / 2), _xlpm.limbs_base, core_BigInt.Split(_xlpm.str_abs_base, _xlpm.k), _xlpm.limbs_final, core_BigInt.UPow(_xlpm.limbs_base, _xlpm.str_norm_exp, _xlpm.k), _xlpm.str_merged, core_BigInt.Merge(_xlpm.limbs_final, _xlpm.k), IF(_xlpm.final_sign = -1, "-" &amp; _xlpm.str_merged, _xlpm.str_merged)))))))))))</definedName>
-    <definedName name="BigInt.RandArray" comment="[VOLATILE] Generates a dynamic array of integers as text._x000a_@param [num_rows] array height, default 1._x000a_@param [num_cols] array width, default 1._x000a_@param [min_digits] minimum number of digits, default 16 (min 1 digit)_x000a_@param [max_digits] maximum number of dig">_xlfn.LAMBDA(_xlop.num_rows,_xlop.num_cols,_xlop.min_digits,_xlop.max_digits, _xlfn.LET(_xlpm.n_rows, IF(_xlfn.ISOMITTED(_xlpm.num_rows), 1, _xlpm.num_rows), _xlpm.n_cols, IF(_xlfn.ISOMITTED(_xlpm.num_cols), 1, _xlpm.num_cols), _xlpm.min_len, IF(_xlfn.ISOMITTED(_xlpm.min_digits), 16, MIN(32767, MAX(1, _xlpm.min_digits))), _xlpm.max_len, IF(_xlfn.ISOMITTED(_xlpm.max_digits), 50, MAX(1, MIN(32766, _xlpm.max_digits))), _xlfn.MAP(_xlfn.RANDARRAY(_xlpm.n_rows, _xlpm.n_cols, _xlpm.min_len, _xlpm.max_len, TRUE), _xlfn.LAMBDA(_xlpm.length, _xlfn.LET(_xlpm.sign_prefix, CHOOSE(RANDBETWEEN(1, 2), "", "-"), _xlpm.rand_digits, _xlfn.CONCAT(_xlfn.RANDARRAY(1, _xlpm.length, 0, 9, TRUE)), _xlpm.sign_prefix &amp; _xlfn.REGEXREPLACE(_xlpm.rand_digits, "^0*", ""))))))</definedName>
-    <definedName name="BigInt.Sign" comment="Returns the sign of a BigInt: 1 (positive), -1 (negative), or 0 (zero)._x000a_@param big_int The BigInt string.">_xlfn.LAMBDA(_xlpm.input, _xlfn.LET(_xlpm.str_norm, BigInt.Norm(_xlpm.input), _xlfn.SWITCH(LEFT(_xlpm.str_norm), "0", 0, "-", -1, 1)))</definedName>
-    <definedName name="BigInt.Sqrt" comment="Calculates the integer square root (floor) of a BigInt._x000a_@param input The radicand BigInt string.">_xlfn.LAMBDA(_xlpm.input, _xlfn.LET(_xlpm.str_norm, BigInt.Norm(_xlpm.input), _xlpm.sign_n, BigInt.Sign(_xlpm.str_norm), IF(_xlpm.sign_n = -1, #NUM!, IF(_xlpm.str_norm = "0", "0", IF(_xlpm.str_norm = "1", "1", _xlfn.LET(_xlpm.len_norm, LEN(_xlpm.str_norm), _xlpm.num_seed_precision, IF(_xlpm.len_norm &lt;= 14, _xlpm.len_norm, IF(ISEVEN(_xlpm.len_norm), 14, 13)), _xlpm.str_native_precision, LEFT(_xlpm.str_norm, _xlpm.num_seed_precision), _xlpm.num_native_precision, VALUE(_xlpm.str_native_precision), _xlpm.num_magnitude_zeroes, (_xlpm.len_norm - _xlpm.num_seed_precision) / 2, _xlpm.str_prefix, TEXT(ROUNDUP(SQRT(_xlpm.num_native_precision), 0) + 1, "0"), _xlpm.str_seed, _xlpm.str_prefix &amp; REPT("0", _xlpm.num_magnitude_zeroes), _xlpm.k, core_BigInt.SafeK("MUL", _xlpm.len_norm), _xlpm.limbs_radicand, core_BigInt.Split(_xlpm.str_norm, _xlpm.k), _xlpm.limbs_seed, core_BigInt.Split(_xlpm.str_seed, _xlpm.k), _xlpm.limbs_final, core_BigInt.USqrt(_xlpm.limbs_radicand, _xlpm.limbs_seed, _xlpm.k), core_BigInt.Merge(_xlpm.limbs_final, _xlpm.k)))))))</definedName>
-    <definedName name="BigInt.Sub" comment="Subtracts the second BigInt string from the first (A - B)._x000a_@param input_a The minuend BigInt string._x000a_@param input_b The subtrahend BigInt string.">_xlfn.LAMBDA(_xlpm.input_a,_xlpm.input_b, _xlfn.LET(_xlpm.str_norm_b, BigInt.Norm(_xlpm.input_b), _xlpm.str_inverse_b, IF(_xlpm.str_norm_b = "0", "0", IF(LEFT(_xlpm.str_norm_b) = "-", MID(_xlpm.str_norm_b, 2, LEN(_xlpm.str_norm_b)), "-" &amp; _xlpm.str_norm_b)), BigInt.Add(_xlpm.input_a, _xlpm.str_inverse_b)))</definedName>
-    <definedName name="BigInt.Sum" comment="Sums an array or range of BigInt strings via vectorized group matrices._x000a_@param input_range A contiguous range or array of BigInt strings.">_xlfn.LAMBDA(_xlpm.input_range, _xlfn.LET(_xlpm.flattened_input, _xlfn.TOROW(_xlpm.input_range, 1), IF(OR(ISERROR(_xlpm.flattened_input), COLUMNS(_xlpm.flattened_input) = 0), "0", _xlfn.LET(_xlpm.str_norms, _xlfn.MAP(_xlpm.flattened_input, _xlfn.LAMBDA(_xlpm.x, BigInt.Norm(_xlpm.x))), _xlpm.arr_signs, _xlfn.MAP(LEFT(_xlpm.str_norms), _xlfn.LAMBDA(_xlpm.x, IF(_xlpm.x = "0", 0, IF(_xlpm.x = "-", -1, 1)))), _xlpm.str_abs, _xlfn.MAP(_xlpm.str_norms, _xlpm.arr_signs, _xlfn.LAMBDA(_xlpm.x,_xlpm.sign, IF(_xlpm.sign = -1, MID(_xlpm.x, 2, LEN(_xlpm.x) - 1), _xlpm.x))), _xlpm.str_pos, _xlfn._xlws.FILTER(_xlpm.str_abs, _xlpm.arr_signs = 1, {"0"}), _xlpm.str_negs, _xlfn._xlws.FILTER(_xlpm.str_abs, _xlpm.arr_signs = -1, {"0"}), _xlpm.unified_k, core_BigInt.SafeK("ADD", COLUMNS(_xlpm.flattened_input)), _xlpm.limbs_pos_sum, core_BigInt.UMatrixSum(_xlpm.str_pos, _xlpm.unified_k), _xlpm.limbs_neg_sum, core_BigInt.UMatrixSum(_xlpm.str_negs, _xlpm.unified_k), _xlpm.packed_result, core_BigInt.AddSubRouter(_xlpm.limbs_pos_sum, _xlpm.limbs_neg_sum, 1, -1, _xlpm.unified_k), _xlpm.final_sign, _xlfn.CHOOSEROWS(_xlpm.packed_result, -1), _xlpm.final_limbs, _xlfn.DROP(_xlpm.packed_result, -1), _xlpm.str_merged, core_BigInt.Merge(_xlpm.final_limbs, _xlpm.unified_k), IF(_xlpm.final_sign = -1, "-" &amp; _xlpm.str_merged, _xlpm.str_merged)))))</definedName>
-    <definedName name="core_BigInt.AddSubRouter" comment="[Internal] Routes addition/subtraction based on signs and magnitudes._x000a_Returns a tuple array: VSTACK(limbs, final_sign) where the final row is the scalar sign._x000a_@param limbs_a The first little-endian limb array._x000a_@param limbs_b The second little-endian limb ">_xlfn.LAMBDA(_xlpm.limbs_a,_xlpm.limbs_b,_xlpm.sign_a,_xlpm.sign_b,_xlpm.k, _xlfn.LET(_xlpm.is_addition, _xlpm.sign_a = _xlpm.sign_b, IF(_xlpm.is_addition, _xlfn.VSTACK(core_BigInt.UAdd(_xlpm.limbs_a, _xlpm.limbs_b, _xlpm.k), _xlpm.sign_a), _xlfn.LET(_xlpm.magnitude_comparison, core_BigInt.UCompare(_xlpm.limbs_a, _xlpm.limbs_b), IF(_xlpm.magnitude_comparison = 0, {0;0}, IF(_xlpm.magnitude_comparison &gt; 0, _xlfn.VSTACK(core_BigInt.USub(_xlpm.limbs_a, _xlpm.limbs_b, _xlpm.k), _xlpm.sign_a), _xlfn.VSTACK(core_BigInt.USub(_xlpm.limbs_b, _xlpm.limbs_a, _xlpm.k), _xlpm.sign_b)))))))</definedName>
-    <definedName name="core_BigInt.Carry" comment="[Internal] Resolves carries right-to-left across a vertical array of base-10^k limbs._x000a_@param limbs The array of numeric limbs._x000a_@param k The limb size.">_xlfn.LAMBDA(_xlpm.limbs,_xlpm.k, _xlfn.LET(_xlpm.num_limbs, ROWS(_xlpm.limbs), _xlpm.radix_base, 10 ^ _xlpm.k, _xlpm.arr_carries, _xlfn.SCAN(0, _xlpm.limbs, _xlfn.LAMBDA(_xlpm.acc,_xlpm.val, _xlpm.val + INT(_xlpm.acc / _xlpm.radix_base))), _xlpm.remainders, MOD(_xlpm.arr_carries, _xlpm.radix_base), _xlpm.final_carry, INT(INDEX(_xlpm.arr_carries, _xlpm.num_limbs, 1) / _xlpm.radix_base), IF(_xlpm.final_carry &gt; 0, _xlfn.VSTACK(_xlpm.remainders, _xlpm.final_carry), _xlpm.remainders)))</definedName>
-    <definedName name="core_BigInt.DivRouter" comment=" * [Internal] Hybrid Division Router._x000a_ * Directs division to the optimal kernel based on Dividend length._x000a_ * @param limbs_a The dividend array._x000a_ * @param limbs_b The divisor array._x000a_ * @param k The dynamic chunk size context._x000a_ ">_xlfn.LAMBDA(_xlpm.limbs_a,_xlpm.limbs_b,_xlpm.k, _xlfn.LET(_xlpm.approx_digits_a, ROWS(_xlpm.limbs_a) * _xlpm.k, _xlpm.approx_digits_b, ROWS(_xlpm.limbs_b) * _xlpm.k, _xlpm.regression_slope_m, 0.107821194271297, _xlpm.regression_intercept_c, -221.902189462068, _xlpm.threshold_digits, (_xlpm.regression_slope_m * _xlpm.approx_digits_a) + _xlpm.regression_intercept_c, IF(_xlpm.approx_digits_b &lt;= _xlpm.threshold_digits, core_BigInt.KnuthDiv(_xlpm.limbs_a, _xlpm.limbs_b, _xlpm.k), core_BigInt.NewtonRaphsonDiv(_xlpm.limbs_a, _xlpm.limbs_b, _xlpm.k))))</definedName>
-    <definedName name="core_BigInt.FindQuotientLimb" comment=" * [Internal] Binary search to find the highest scalar quotient limb q (0 &lt;= q &lt; 10^k)_x000a_ * such that B * q &lt;= limbs_r. Eliminates the need for Knuth D float-estimation._x000a_ * @param limbs_r The current remainder array._x000a_ * @param b The divisor array._x000a_ * @param">_xlfn.LAMBDA(_xlpm.limbs_r,_xlpm.limbs_b,_xlpm.k, _xlfn.LET(_xlpm.required_bits, _xlfn.CEILING.MATH(LOG(10 ^ _xlpm.k, 2)), _xlpm.powers_of_two, 2 ^ _xlfn.SEQUENCE(_xlpm.required_bits, 1, _xlpm.required_bits - 1, -1), _xlfn.REDUCE(0, _xlpm.powers_of_two, _xlfn.LAMBDA(_xlpm.current_q,_xlpm.current_power, _xlfn.LET(_xlpm.test_q, _xlpm.current_q + _xlpm.current_power, IF(_xlpm.test_q &gt;= 10 ^ _xlpm.k, _xlpm.current_q, _xlfn.LET(_xlpm.limbs_bq, core_BigInt.Carry(_xlpm.limbs_b * _xlpm.test_q, _xlpm.k), _xlpm.magnitude_comparison, core_BigInt.UCompare(_xlpm.limbs_r, _xlpm.limbs_bq), IF(_xlpm.magnitude_comparison &gt;= 0, _xlpm.test_q, _xlpm.current_q))))))))</definedName>
-    <definedName name="core_BigInt.KnuthDiv" comment=" * [Internal] Basecase Division via sequential shift-and-subtract._x000a_ * Returns a packed 1D array: VSTACK(Length_R, R_limbs, Q_limbs)._x000a_ * Eliminates 2D array padding to strictly preserve memory efficiency._x000a_ * @param limbs_a The dividend array._x000a_ * @param lim">_xlfn.LAMBDA(_xlpm.limbs_a,_xlpm.limbs_b,_xlpm.k, _xlfn.LET(_xlpm.magnitude_comparison, core_BigInt.UCompare(_xlpm.limbs_a, _xlpm.limbs_b), IF(_xlpm.magnitude_comparison &lt; 0, _xlfn.VSTACK(ROWS(_xlpm.limbs_a), _xlpm.limbs_a, 0), IF(_xlpm.magnitude_comparison = 0, _xlfn.VSTACK(1, 0, 1), _xlfn.LET(_xlpm.num_limbs_a, ROWS(_xlpm.limbs_a), _xlpm.big_endian_a, _xlfn.CHOOSEROWS(_xlpm.limbs_a, _xlfn.SEQUENCE(_xlpm.num_limbs_a, 1, _xlpm.num_limbs_a, -1)), _xlpm.final_packed_state, _xlfn.REDUCE(_xlfn.VSTACK(1, 0, 0), _xlpm.big_endian_a, _xlfn.LAMBDA(_xlpm.packed_state,_xlpm.val, _xlfn.LET(_xlpm.num_limbs_r, INDEX(_xlpm.packed_state, 1, 1), _xlpm.limbs_r, _xlfn.CHOOSEROWS(_xlpm.packed_state, _xlfn.SEQUENCE(_xlpm.num_limbs_r, 1, 2)), _xlpm.limbs_q, _xlfn.DROP(_xlpm.packed_state, _xlpm.num_limbs_r + 1), _xlpm.limbs_shifted_r, IF(AND(ROWS(_xlpm.limbs_r) = 1, INDEX(_xlpm.limbs_r, 1, 1) = 0), _xlpm.val, _xlfn.VSTACK(_xlpm.val, _xlpm.limbs_r)), _xlpm.q_limb, core_BigInt.FindQuotientLimb(_xlpm.limbs_shifted_r, _xlpm.limbs_b, _xlpm.k), _xlpm.limbs_bq, core_BigInt.Carry(_xlpm.limbs_b * _xlpm.q_limb, _xlpm.k), _xlpm.limbs_next_r, core_BigInt.USub(_xlpm.limbs_shifted_r, _xlpm.limbs_bq, _xlpm.k), _xlpm.has_q, OR(ROWS(_xlpm.limbs_q) &gt; 1, INDEX(_xlpm.limbs_q, 1, 1) &gt; 0), _xlpm.limbs_next_q, IF(_xlpm.has_q, _xlfn.VSTACK(_xlpm.limbs_q, _xlpm.q_limb), _xlpm.q_limb), _xlfn.VSTACK(ROWS(_xlpm.limbs_next_r), _xlpm.limbs_next_r, _xlpm.limbs_next_q)))), _xlpm.num_limbs_r, INDEX(_xlpm.final_packed_state, 1, 1), _xlpm.limbs_r, _xlfn.CHOOSEROWS(_xlpm.final_packed_state, _xlfn.SEQUENCE(_xlpm.num_limbs_r, 1, 2)), _xlpm.big_endian_q, _xlfn.DROP(_xlpm.final_packed_state, _xlpm.num_limbs_r + 1), _xlpm.len_q, ROWS(_xlpm.big_endian_q), _xlpm.limbs_q, _xlfn.CHOOSEROWS(_xlpm.big_endian_q, _xlfn.SEQUENCE(_xlpm.len_q, 1, _xlpm.len_q, -1)), _xlfn.VSTACK(_xlpm.num_limbs_r, _xlpm.limbs_r, _xlpm.limbs_q))))))</definedName>
-    <definedName name="core_BigInt.Merge" comment="[Internal] Concatenates an array of numeric limbs into a BigInt string, zero-padding all but the first limb._x000a_@param limbs The vertical array of numeric limbs._x000a_@param k The limb size used during calculation.">_xlfn.LAMBDA(_xlpm.limbs,_xlpm.k, _xlfn.LET(_xlpm.num_limbs, ROWS(_xlpm.limbs), _xlpm.rev_limbs, _xlfn.CHOOSEROWS(_xlpm.limbs, _xlfn.SEQUENCE(_xlpm.num_limbs, 1, _xlpm.num_limbs, -1)), IF(_xlpm.num_limbs = 1, _xlpm.rev_limbs &amp; "", _xlfn.CONCAT(_xlfn.VSTACK(_xlfn.TAKE(_xlpm.rev_limbs, 1) &amp; "", TEXT(_xlfn.DROP(_xlpm.rev_limbs, 1), REPT("0", _xlpm.k)))))))</definedName>
-    <definedName name="core_BigInt.NativePrimes" comment="[Internal] Generates a 1D vertical array of all prime numbers up to n._x000a_Evaluates purely in native C++ using a dynamic sieve._x000a_@param n The upper bound integer (assumed &lt;= 9273).">_xlfn.LAMBDA(_xlpm.n, IF(_xlpm.n &lt; 2, #NUM!, _xlfn.LET(_xlpm.candidate_sequence, _xlfn.SEQUENCE(_xlpm.n - 1, 1, 2), _xlfn._xlws.FILTER(_xlpm.candidate_sequence, _xlfn.MAP(_xlpm.candidate_sequence, _xlfn.LAMBDA(_xlpm.current_candidate, _xlfn.LET(_xlpm.limit, INT(SQRT(_xlpm.current_candidate)), IF(_xlpm.limit &lt; 2, TRUE, MIN(MOD(_xlpm.current_candidate, _xlfn.SEQUENCE(_xlpm.limit - 1, 1, 2))) &gt; 0))))))))</definedName>
-    <definedName name="core_BigInt.NativeSwingExponents" comment="[Internal] Calculates the exponent for an array of primes in the Swing term of a factorial._x000a_@param n The current factorial magnitude (&lt;= 9273)._x000a_@param primes A vertical array of prime numbers (&lt;= n).">_xlfn.LAMBDA(_xlpm.n,_xlpm.primes, _xlfn.MAP(_xlpm.primes, _xlfn.LAMBDA(_xlpm.p, _xlfn.LET(_xlpm.max_power_k, INT(LOG(_xlpm.n, _xlpm.p)), _xlpm.prime_powers, _xlpm.p ^ _xlfn.SEQUENCE(_xlpm.max_power_k), SUM(MOD(INT(_xlpm.n / _xlpm.prime_powers), 2))))))</definedName>
-    <definedName name="core_BigInt.NewtonRaphsonDiv" comment="[Internal] Heavyweight Newton-Raphson Division._x000a_Implements progressive scaling bounded to MAX(len_a, len_b)._x000a_@param limbs_a The dividend array._x000a_@param limbs_b The divisor array._x000a_@param k The dynamic chunk size context.">_xlfn.LAMBDA(_xlpm.limbs_a,_xlpm.limbs_b,_xlpm.k, _xlfn.LET(_xlpm.num_limbs_a, ROWS(_xlpm.limbs_a), _xlpm.num_limbs_b, ROWS(_xlpm.limbs_b), _xlpm.num_limbs_target, MAX(_xlpm.num_limbs_a, _xlpm.num_limbs_b), _xlpm.limbs_reciprocal, core_BigInt.NewtonRaphsonReciprocal(_xlpm.limbs_b, _xlpm.num_limbs_target, _xlpm.k), _xlpm.right_shift_limbs, 2 * _xlpm.num_limbs_target, _xlpm.limbs_q_unscaled, core_BigInt.UMul(_xlpm.limbs_a, _xlpm.limbs_reciprocal, _xlpm.k), _xlpm.limbs_q_approx, IF(ROWS(_xlpm.limbs_q_unscaled) &lt;= _xlpm.right_shift_limbs, {0}, _xlfn.DROP(_xlpm.limbs_q_unscaled, _xlpm.right_shift_limbs)), _xlpm.limbs_p_baseline, core_BigInt.UMul(_xlpm.limbs_b, _xlpm.limbs_q_approx, _xlpm.k), _xlpm.initial_packed_state, _xlfn.VSTACK(ROWS(_xlpm.limbs_q_approx), _xlpm.limbs_q_approx, _xlpm.limbs_p_baseline), _xlpm.packed_state_swept_down, _xlfn.REDUCE(_xlpm.initial_packed_state, {1;2}, _xlfn.LAMBDA(_xlpm.packed_state,_xlpm.i, _xlfn.LET(_xlpm.len_q, INDEX(_xlpm.packed_state, 1, 1), _xlpm.limbs_current_q, _xlfn.CHOOSEROWS(_xlpm.packed_state, _xlfn.SEQUENCE(_xlpm.len_q, 1, 2)), _xlpm.limbs_current_p, _xlfn.DROP(_xlpm.packed_state, _xlpm.len_q + 1), IF(core_BigInt.UCompare(_xlpm.limbs_current_p, _xlpm.limbs_a) &lt;= 0, _xlpm.packed_state, _xlfn.LET(_xlpm.limbs_next_q, core_BigInt.USub(_xlpm.limbs_current_q, {1}, _xlpm.k), _xlpm.limbs_next_p, core_BigInt.USub(_xlpm.limbs_current_p, _xlpm.limbs_b, _xlpm.k), _xlfn.VSTACK(ROWS(_xlpm.limbs_next_q), _xlpm.limbs_next_q, _xlpm.limbs_next_p)))))), _xlpm.packed_state_swept_up, _xlfn.REDUCE(_xlpm.packed_state_swept_down, {1;2}, _xlfn.LAMBDA(_xlpm.packed_state,_xlpm.i, _xlfn.LET(_xlpm.len_q, INDEX(_xlpm.packed_state, 1, 1), _xlpm.limbs_current_q, _xlfn.CHOOSEROWS(_xlpm.packed_state, _xlfn.SEQUENCE(_xlpm.len_q, 1, 2)), _xlpm.limbs_current_p, _xlfn.DROP(_xlpm.packed_state, _xlpm.len_q + 1), _xlpm.limbs_next_p_test, core_BigInt.UAdd(_xlpm.limbs_current_p, _xlpm.limbs_b, _xlpm.k), IF(core_BigInt.UCompare(_xlpm.limbs_next_p_test, _xlpm.limbs_a) &gt; 0, _xlpm.packed_state, _xlfn.LET(_xlpm.limbs_next_q, core_BigInt.UAdd(_xlpm.limbs_current_q, {1}, _xlpm.k), _xlfn.VSTACK(ROWS(_xlpm.limbs_next_q), _xlpm.limbs_next_q, _xlpm.limbs_next_p_test)))))), _xlpm.len_q, INDEX(_xlpm.packed_state_swept_up, 1, 1), _xlpm.limbs_q, _xlfn.CHOOSEROWS(_xlpm.packed_state_swept_up, _xlfn.SEQUENCE(_xlpm.len_q, 1, 2)), _xlpm.limbs_p, _xlfn.DROP(_xlpm.packed_state_swept_up, _xlpm.len_q + 1), _xlpm.limbs_r, core_BigInt.USub(_xlpm.limbs_a, _xlpm.limbs_p, _xlpm.k), _xlfn.VSTACK(ROWS(_xlpm.limbs_r), _xlpm.limbs_r, _xlpm.limbs_q)))</definedName>
-    <definedName name="core_BigInt.NewtonRaphsonReciprocal" comment="[Internal] Computes the Reciprocal progressively scaling up to the Dividend's precision._x000a_@param limbs_b The divisor limb array._x000a_@param target_len The limb-length of Dividend A._x000a_@param k The dynamic chunk size context.">_xlfn.LAMBDA(_xlpm.limbs_b,_xlpm.target_len,_xlpm.k, _xlfn.LET(_xlpm.num_limbs_b, ROWS(_xlpm.limbs_b), _xlpm.num_seed_limbs, MIN(3, _xlpm.num_limbs_b), _xlpm.limbs_r_seed, core_BigInt.NewtonRaphsonSeed(_xlpm.limbs_b, _xlpm.k), _xlpm.required_iterations, MAX(0, _xlfn.CEILING.MATH(LN(_xlpm.target_len / _xlpm.num_seed_limbs) / LN(2))) + 1, IF(_xlpm.required_iterations = 0, _xlpm.limbs_r_seed, _xlfn.LET(_xlpm.iterations, _xlfn.SEQUENCE(_xlpm.required_iterations), _xlpm.final_packed_state, _xlfn.REDUCE(_xlfn.VSTACK(_xlpm.num_seed_limbs, _xlpm.limbs_r_seed), _xlpm.iterations, _xlfn.LAMBDA(_xlpm.packed_state,_xlpm.i, _xlfn.LET(_xlpm.current_len, INDEX(_xlpm.packed_state, 1, 1), _xlpm.limbs_current_r, _xlfn.DROP(_xlpm.packed_state, 1), _xlpm.next_len, MIN(_xlpm.current_len * 2, _xlpm.target_len), _xlpm.active_b_limbs_current, MIN(_xlpm.current_len, _xlpm.num_limbs_b), _xlpm.active_b_limbs_next, MIN(_xlpm.next_len, _xlpm.num_limbs_b), _xlpm.required_shift_limbs, 2 * (_xlpm.next_len - _xlpm.current_len) - (_xlpm.active_b_limbs_next - _xlpm.active_b_limbs_current), _xlpm.limbs_r_prime, IF(_xlpm.required_shift_limbs &gt; 0, _xlfn.VSTACK(_xlfn.EXPAND(0, _xlpm.required_shift_limbs, , 0), _xlpm.limbs_current_r), _xlpm.limbs_current_r), _xlpm.limbs_b_active, _xlfn.TAKE(_xlpm.limbs_b, -_xlpm.active_b_limbs_next), _xlpm.limbs_p, core_BigInt.UMul(_xlpm.limbs_b_active, _xlpm.limbs_r_prime, _xlpm.k), _xlpm.limbs_two_beta, _xlfn.VSTACK(_xlfn.EXPAND(0, 2 * _xlpm.next_len, , 0), 2), _xlpm.limbs_error_term, core_BigInt.USub(_xlpm.limbs_two_beta, _xlpm.limbs_p, _xlpm.k), _xlpm.limbs_next_r_unscaled, core_BigInt.UMul(_xlpm.limbs_r_prime, _xlpm.limbs_error_term, _xlpm.k), _xlpm.limbs_next_r, IF(ROWS(_xlpm.limbs_next_r_unscaled) &lt;= 2 * _xlpm.next_len, {0}, _xlfn.DROP(_xlpm.limbs_next_r_unscaled, 2 * _xlpm.next_len)), _xlfn.VSTACK(_xlpm.next_len, _xlpm.limbs_next_r)))), _xlfn.DROP(_xlpm.final_packed_state, 1)))))</definedName>
-    <definedName name="core_BigInt.NewtonRaphsonSeed" comment="[Internal] Generates the exact reciprocal seed for Newton-Raphson Division using Knuth Basecase._x000a_Extracts up to the top 3 limbs of B and calculates floor(Beta^(2*len) / B_top)._x000a_@param limbs_b The divisor limb array._x000a_@param k The dynamic chunk size context">_xlfn.LAMBDA(_xlpm.limbs_b,_xlpm.k, _xlfn.LET(_xlpm.num_limbs_b, ROWS(_xlpm.limbs_b), _xlpm.num_seed_limbs, MIN(3, _xlpm.num_limbs_b), _xlpm.limbs_b_top, _xlfn.TAKE(_xlpm.limbs_b, -_xlpm.num_seed_limbs), _xlpm.limbs_beta_2m, _xlfn.VSTACK(_xlfn.EXPAND(0, 2 * _xlpm.num_seed_limbs, , 0), 1), _xlpm.packed_basecase_result, core_BigInt.KnuthDiv(_xlpm.limbs_beta_2m, _xlpm.limbs_b_top, _xlpm.k), _xlpm.num_limbs_r, INDEX(_xlpm.packed_basecase_result, 1, 1), _xlfn.DROP(_xlpm.packed_basecase_result, _xlpm.num_limbs_r + 1)))</definedName>
-    <definedName name="core_BigInt.PrimeSwingKernel" comment="[Internal] Recursive top-down LAMBDA calculating the Prime Swing factorial._x000a_@param n The current factorial magnitude._x000a_@param global_primes The unified vertical array of all primes up to the target factorial.">_xlfn.LAMBDA(_xlpm.n,_xlpm.global_primes, IF(_xlpm.n &lt; 2, "1", _xlfn.LET(_xlpm.floor_half_n, INT(_xlpm.n / 2), _xlpm.factorial_half_n, core_BigInt.PrimeSwingKernel(_xlpm.floor_half_n, _xlpm.global_primes), _xlpm.squared_half_factorial, core_BigInt.UTextMul(_xlpm.factorial_half_n, _xlpm.factorial_half_n), _xlpm.applicable_tier_primes, _xlfn._xlws.FILTER(_xlpm.global_primes, _xlpm.global_primes &lt;= _xlpm.n), _xlpm.str_swing_term, core_BigInt.SwingTerm(_xlpm.n, _xlpm.applicable_tier_primes), core_BigInt.UTextMul(_xlpm.squared_half_factorial, _xlpm.str_swing_term))))</definedName>
-    <definedName name="core_BigInt.SafeK" comment="[Internal] Computes the maximum safe base-10 limb size (k) to avoid IEEE-754 precision loss._x000a_@param operation: &quot;ADD&quot;, &quot;MUL&quot;, or &quot;DIV&quot;._x000a_@param [max_items] ADD: number of operands. MUL: shortest string digits count.">_xlfn.LAMBDA(_xlpm.operation,_xlop.operand_or_digits, _xlfn.LET(_xlpm.resolved_count, IF(OR(_xlpm.operand_or_digits = "", _xlfn.ISOMITTED(_xlpm.operand_or_digits)), 2, MAX(2, _xlpm.operand_or_digits)), _xlfn.SWITCH(_xlpm.operation, "ADD", 15 - LEN(_xlpm.resolved_count), "MUL", _xlfn.LET(_xlpm.test_k, {7;6;5;4;3;2;1}, _xlpm.max_overlap, ROUNDUP(_xlpm.resolved_count / _xlpm.test_k, 0), _xlpm.uncarried_max, _xlpm.max_overlap * (10 ^ _xlpm.test_k - 1) ^ 2, _xlpm.max_carry, INT(_xlpm.uncarried_max / 10 ^ _xlpm.test_k), _xlpm.peak_val, _xlpm.uncarried_max + _xlpm.max_carry, MAX(_xlfn._xlws.FILTER(_xlpm.test_k, _xlpm.peak_val &lt;= (10 ^ 15 - 1)))), "DIV", 7, #NAME?)))</definedName>
-    <definedName name="core_BigInt.Split" comment="[Internal] Unified Splitter. Splits both scalars and arrays into Little-Endian limbs._x000a_Uses MAX() to guarantee scalar inputs to the SEQUENCE engine._x000a_@param big_ints The string or array of strings._x000a_@param k The dynamic chunk size context.">_xlfn.LAMBDA(_xlpm.str_norms,_xlpm.k, _xlfn.LET(_xlpm.flattened_norms, _xlfn.TOROW(_xlpm.str_norms), _xlpm.lengths, LEN(_xlpm.flattened_norms), _xlpm.max_len, MAX(_xlpm.lengths), _xlpm.pad_len, ROUNDUP(_xlpm.max_len / _xlpm.k, 0) * _xlpm.k, _xlpm.padded_norms, REPT("0", _xlpm.pad_len - _xlpm.lengths) &amp; _xlpm.flattened_norms, _xlpm.limb_start_indices, _xlfn.SEQUENCE(_xlpm.pad_len / _xlpm.k, 1, _xlpm.pad_len - _xlpm.k + 1, -_xlpm.k), --MID(_xlpm.padded_norms, _xlpm.limb_start_indices, _xlpm.k)))</definedName>
-    <definedName name="core_BigInt.SwingTerm" comment="[Internal] Calculates the massive BigInt string for the Swing term of a factorial._x000a_@param n The current factorial magnitude._x000a_@param tier_primes A vertical array of prime numbers (&lt;= n).">_xlfn.LAMBDA(_xlpm.n,_xlpm.tier_primes, _xlfn.LET(_xlpm.swing_exponents, core_BigInt.NativeSwingExponents(_xlpm.n, _xlpm.tier_primes), _xlpm.has_native_exponent, _xlpm.swing_exponents &gt; 0, IF(AND(NOT(_xlpm.has_native_exponent)), "1", _xlfn.LET(_xlpm.active_primes, _xlfn._xlws.FILTER(_xlpm.tier_primes, _xlpm.has_native_exponent), _xlpm.active_exponents, _xlfn._xlws.FILTER(_xlpm.swing_exponents, _xlpm.has_native_exponent), _xlpm.evalutated_prime_powers, _xlfn.MAP(_xlpm.active_primes, _xlpm.active_exponents, _xlfn.LAMBDA(_xlpm.p,_xlpm.e, IF(_xlpm.e = 1, _xlpm.p &amp; "", BigInt.Pow(_xlpm.p &amp; "", _xlpm.e &amp; "")))), core_BigInt.TextTreeProd(_xlpm.evalutated_prime_powers)))))</definedName>
-    <definedName name="core_BigInt.TextTreeProd" comment="[Internal] Vectorized logarithmic product of an array of BigInt strings._x000a_Recursively cuts the array in half to bypass REDUCE sequential memory allocations._x000a_@param arr_strings A 1D vertical array of BigInt strings.">_xlfn.LAMBDA(_xlpm.arr_strings, _xlfn.LET(_xlpm.num_elements, ROWS(_xlpm.arr_strings), IF(_xlpm.num_elements = 1, INDEX(_xlpm.arr_strings, 1, 1), _xlfn.LET(_xlpm.paired_strings, _xlfn.WRAPROWS(_xlpm.arr_strings, 2, "1"), _xlpm.reduced_array, _xlfn.BYROW(_xlpm.paired_strings, _xlfn.LAMBDA(_xlpm.row, core_BigInt.UTextMul(INDEX(_xlpm.row, 1, 1), INDEX(_xlpm.row, 1, 2)))), core_BigInt.TextTreeProd(_xlpm.reduced_array)))))</definedName>
-    <definedName name="core_BigInt.TreeCompare" comment="[Internal] Recursive tournament tree for Min/Max evaluations._x000a_@param col A 1D vertical array of normalized BigInt strings._x000a_@param mode 1 for Maximum, -1 for Minimum.">_xlfn.LAMBDA(_xlpm.str_norms,_xlpm.comparison_mode, _xlfn.LET(_xlpm.num_rows, ROWS(_xlpm.str_norms), IF(_xlpm.num_rows = 1, INDEX(_xlpm.str_norms, 1, 1), _xlfn.LET(_xlpm.tournament_pairs, _xlfn.WRAPROWS(_xlpm.str_norms, 2), _xlpm.competitors_a, _xlfn.TAKE(_xlpm.tournament_pairs, , 1), _xlpm.competitors_b, _xlfn.TAKE(_xlpm.tournament_pairs, , -1), _xlpm.round_winners, _xlfn.MAP(_xlpm.competitors_a, _xlpm.competitors_b, _xlfn.LAMBDA(_xlpm.a,_xlpm.b, IF(ISNA(_xlpm.b), _xlpm.a, _xlfn.LET(_xlpm.comparison_result, BigInt.Compare(_xlpm.a, _xlpm.b), IF(_xlpm.comparison_result * _xlpm.comparison_mode &gt;= 0, _xlpm.a, _xlpm.b))))), core_BigInt.TreeCompare(_xlpm.round_winners, _xlpm.comparison_mode)))))</definedName>
-    <definedName name="core_BigInt.UAdd" comment="[Internal] Unsigned addition of two Little-Endian limb arrays._x000a_@param limbs_a The first limb array._x000a_@param limbs_b The second limb array._x000a_@param k The dynamic chunk size context.">_xlfn.LAMBDA(_xlpm.a,_xlpm.b,_xlpm.k, _xlfn.LET(_xlpm.max_rows, MAX(ROWS(_xlpm.a), ROWS(_xlpm.b)), _xlpm.limbs_a_aligned, _xlfn.EXPAND(_xlpm.a, _xlpm.max_rows, 1, 0), _xlpm.limbs_b_aligned, _xlfn.EXPAND(_xlpm.b, _xlpm.max_rows, 1, 0), core_BigInt.Carry(_xlpm.limbs_a_aligned + _xlpm.limbs_b_aligned, _xlpm.k)))</definedName>
-    <definedName name="core_BigInt.UCompare" comment="[Internal] Unsigned comparison of two Little-Endian limb arrays._x000a_Returns 1 (a &gt; b), -1 (a &lt; b), or 0 (a = b)._x000a_@param limbs_a The first limb array._x000a_@param limbs_b The second limb array.">_xlfn.LAMBDA(_xlpm.limbs_a,_xlpm.limbs_b, _xlfn.LET(_xlpm.max_rows, MAX(ROWS(_xlpm.limbs_a), ROWS(_xlpm.limbs_b)), _xlpm.limbs_a_aligned, _xlfn.EXPAND(_xlpm.limbs_a, _xlpm.max_rows, 1, 0), _xlpm.limbs_b_aligned, _xlfn.EXPAND(_xlpm.limbs_b, _xlpm.max_rows, 1, 0), _xlpm.differences, _xlpm.limbs_a_aligned - _xlpm.limbs_b_aligned, _xlpm.highest_non_zero_index, _xlfn.XMATCH(TRUE, _xlpm.differences &lt;&gt; 0, 0, -1), IF(ISNA(_xlpm.highest_non_zero_index), 0, SIGN(INDEX(_xlpm.differences, _xlpm.highest_non_zero_index, 1)))))</definedName>
-    <definedName name="core_BigInt.UMatrixSum" comment="[Internal] Vectorized matrix sum of unsigned BigInt strings._x000a_@param str_norms Horizontal array (1xN) of normalized magnitude strings._x000a_@param k The unified dynamic chunk size context.">_xlfn.LAMBDA(_xlpm.str_norms,_xlpm.k, _xlfn.LET(_xlpm.grid, core_BigInt.Split(_xlpm.str_norms, _xlpm.k), _xlpm.raw_limbs, _xlfn.BYROW(_xlpm.grid, _xleta.SUM), core_BigInt.Carry(_xlpm.raw_limbs, _xlpm.k)))</definedName>
-    <definedName name="core_BigInt.UMul" comment="[Internal] Unsigned multiplication of two Little-Endian limb arrays._x000a_Utilizes a 1D Discrete Convolution (Cauchy Product) array-slicing strategy._x000a_Zero dynamic memory reallocation. $O(N+M)$ memory footprint._x000a_@param limbs_a The multiplicand limb array._x000a_@para">_xlfn.LAMBDA(_xlpm.limbs_a,_xlpm.limbs_b,_xlpm.k, _xlfn.LET(_xlpm.num_limbs_a, ROWS(_xlpm.limbs_a), _xlpm.num_limbs_b, ROWS(_xlpm.limbs_b), _xlpm.convolution_length, _xlpm.num_limbs_a + _xlpm.num_limbs_b - 1, _xlpm.raw_convolution, _xlfn.MAKEARRAY(_xlpm.convolution_length, 1, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, _xlfn.LET(_xlpm.window_start_i, MAX(1, _xlpm.r - _xlpm.num_limbs_b + 1), _xlpm.window_end_i, MIN(_xlpm.r, _xlpm.num_limbs_a), _xlpm.overlap_rows, _xlpm.window_end_i - _xlpm.window_start_i + 1, _xlpm.seq_i, _xlfn.SEQUENCE(_xlpm.overlap_rows, 1, _xlpm.window_start_i, 1), _xlpm.seq_j, _xlfn.SEQUENCE(_xlpm.overlap_rows, 1, _xlpm.r - _xlpm.window_start_i + 1, -1), SUM(INDEX(_xlpm.limbs_a, _xlpm.seq_i, 1) * INDEX(_xlpm.limbs_b, _xlpm.seq_j, 1))))), core_BigInt.Carry(_xlpm.raw_convolution, _xlpm.k)))</definedName>
-    <definedName name="core_BigInt.UPow" comment="[Internal] Unsigned Base-10 Left-to-Right Exponentiation._x000a_Evaluates the exponent iteratively using a pre-computed 1-9 cache._x000a_@param limbs_base The little-endian limb array of the base._x000a_@param exp_string The exact text string of the exponent._x000a_@param k The ">_xlfn.LAMBDA(_xlpm.limbs_base,_xlpm.exponent_string,_xlpm.k, _xlfn.LET(_xlpm.limbs_base1, _xlpm.limbs_base, _xlpm.limbs_base2, core_BigInt.UMul(_xlpm.limbs_base1, _xlpm.limbs_base1, _xlpm.k), _xlpm.limbs_base3, core_BigInt.UMul(_xlpm.limbs_base2, _xlpm.limbs_base1, _xlpm.k), _xlpm.limbs_base4, core_BigInt.UMul(_xlpm.limbs_base2, _xlpm.limbs_base2, _xlpm.k), _xlpm.limbs_base5, core_BigInt.UMul(_xlpm.limbs_base4, _xlpm.limbs_base1, _xlpm.k), _xlpm.limbs_base6, core_BigInt.UMul(_xlpm.limbs_base3, _xlpm.limbs_base3, _xlpm.k), _xlpm.limbs_base7, core_BigInt.UMul(_xlpm.limbs_base6, _xlpm.limbs_base1, _xlpm.k), _xlpm.limbs_base8, core_BigInt.UMul(_xlpm.limbs_base4, _xlpm.limbs_base4, _xlpm.k), _xlpm.limbs_base9, core_BigInt.UMul(_xlpm.limbs_base8, _xlpm.limbs_base1, _xlpm.k), _xlpm.exponent_digits, --MID(_xlpm.exponent_string, _xlfn.SEQUENCE(LEN(_xlpm.exponent_string)), 1), _xlfn.REDUCE(1, _xlpm.exponent_digits, _xlfn.LAMBDA(_xlpm.limbs_accumulator,_xlpm.current_digit, _xlfn.LET(_xlpm.is_one, AND(ROWS(_xlpm.limbs_accumulator) = 1, INDEX(_xlpm.limbs_accumulator, 1, 1) = 1), _xlpm.limbs_acc_10, IF(_xlpm.is_one, _xlpm.limbs_accumulator, _xlfn.LET(_xlpm.limbs_acc_2, core_BigInt.UMul(_xlpm.limbs_accumulator, _xlpm.limbs_accumulator, _xlpm.k), _xlpm.limbs_acc_4, core_BigInt.UMul(_xlpm.limbs_acc_2, _xlpm.limbs_acc_2, _xlpm.k), _xlpm.limbs_acc_8, core_BigInt.UMul(_xlpm.limbs_acc_4, _xlpm.limbs_acc_4, _xlpm.k), core_BigInt.UMul(_xlpm.limbs_acc_8, _xlpm.limbs_acc_2, _xlpm.k))), IF(_xlpm.current_digit = 0, _xlpm.limbs_acc_10, _xlfn.LET(_xlpm.limbs_cache_multiplier, CHOOSE(_xlpm.current_digit, _xlpm.limbs_base1, _xlpm.limbs_base2, _xlpm.limbs_base3, _xlpm.limbs_base4, _xlpm.limbs_base5, _xlpm.limbs_base6, _xlpm.limbs_base7, _xlpm.limbs_base8, _xlpm.limbs_base9), IF(_xlpm.is_one, _xlpm.limbs_cache_multiplier, core_BigInt.UMul(_xlpm.limbs_acc_10, _xlpm.limbs_cache_multiplier, _xlpm.k)))))))))</definedName>
-    <definedName name="core_BigInt.USqrt" comment="[Internal] Unsigned Integer Square Root using Newton's Method._x000a_@param limbs_radicand._x000a_@param limbs_initial_x Over-estimated seed array._x000a_@param k The dynamic chunk size context.">_xlfn.LAMBDA(_xlpm.limbs_radicand,_xlpm.limbs_initial_x,_xlpm.k, _xlfn.LET(_xlpm.maximum_iterations, 35, _xlpm.final_packed_state, _xlfn.REDUCE(_xlfn.VSTACK(0, _xlpm.limbs_initial_x), _xlfn.SEQUENCE(_xlpm.maximum_iterations), _xlfn.LAMBDA(_xlpm.packed_state,_xlpm.i, _xlfn.LET(_xlpm.has_converged, INDEX(_xlpm.packed_state, 1, 1), _xlpm.limbs_current_x, _xlfn.DROP(_xlpm.packed_state, 1), IF(_xlpm.has_converged, _xlpm.packed_state, _xlfn.LET(_xlpm.packed_division_result, core_BigInt.DivRouter(_xlpm.limbs_radicand, _xlpm.limbs_current_x, _xlpm.k), _xlpm.num_limbs_r, INDEX(_xlpm.packed_division_result, 1, 1), _xlpm.limbs_q, _xlfn.DROP(_xlpm.packed_division_result, _xlpm.num_limbs_r + 1), _xlpm.limbs_sum_xq, core_BigInt.UAdd(_xlpm.limbs_current_x, _xlpm.limbs_q, _xlpm.k), _xlpm.packed_half_result, core_BigInt.KnuthDiv(_xlpm.limbs_sum_xq, {2}, _xlpm.k), _xlpm.num_limbs_halfed, INDEX(_xlpm.packed_half_result, 1, 1), _xlpm.limbs_next_x, _xlfn.DROP(_xlpm.packed_half_result, _xlpm.num_limbs_halfed + 1), _xlpm.convergence_comparison, core_BigInt.UCompare(_xlpm.limbs_next_x, _xlpm.limbs_current_x), IF(_xlpm.convergence_comparison &gt;= 0, _xlfn.VSTACK(1, _xlpm.limbs_current_x), _xlfn.VSTACK(0, _xlpm.limbs_next_x))))))), _xlfn.DROP(_xlpm.final_packed_state, 1)))</definedName>
-    <definedName name="core_BigInt.USub" comment="[Internal] Unsigned subtraction of two Little-Endian limb arrays._x000a_Assumes magnitudes A &gt;= B. Resolves borrows top-to-bottom and trims trailing zeros._x000a_@param limbs_a The minuend limb array (must be &gt;= limbs_b)._x000a_@param limbs_b The subtrahend limb array._x000a_@pa">_xlfn.LAMBDA(_xlpm.limbs_a,_xlpm.limbs_b,_xlpm.k, _xlfn.LET(_xlpm.max_rows, MAX(ROWS(_xlpm.limbs_a), ROWS(_xlpm.limbs_b)), _xlpm.limbs_a_aligned, _xlfn.EXPAND(_xlpm.limbs_a, _xlpm.max_rows, 1, 0), _xlpm.limbs_b_aligned, _xlfn.EXPAND(_xlpm.limbs_b, _xlpm.max_rows, 1, 0), _xlpm.differences, _xlpm.limbs_a_aligned - _xlpm.limbs_b_aligned, _xlpm.carried_differences, core_BigInt.Carry(_xlpm.differences, _xlpm.k), _xlpm.highest_non_zero_index, _xlfn.XMATCH(TRUE, _xlpm.carried_differences &lt;&gt; 0, 0, -1), IF(ISNA(_xlpm.highest_non_zero_index), {0}, _xlfn.TAKE(_xlpm.carried_differences, _xlpm.highest_non_zero_index))))</definedName>
-    <definedName name="core_BigInt.UTextMul" comment="[Internal] Unsafe, high-performance text multiplication for normalised, positive BigInt strings._x000a_Bypasses Layer 0 validation. Implements strict short-circuits for padding optimization._x000a_@param norm_a_x000a_@param norm_b">_xlfn.LAMBDA(_xlpm.norm_a,_xlpm.norm_b, IF(OR(_xlpm.norm_a = "0", _xlpm.norm_b = "0"), "0", IF(_xlpm.norm_a = "1", _xlpm.norm_b, IF(_xlpm.norm_b = "1", _xlpm.norm_a, _xlfn.LET(_xlpm.len_a, LEN(_xlpm.norm_a), _xlpm.len_b, LEN(_xlpm.norm_b), _xlpm.k, core_BigInt.SafeK("MUL", MIN(_xlpm.len_a, _xlpm.len_b)), _xlpm.limbs_a, core_BigInt.Split(_xlpm.norm_a, _xlpm.k), _xlpm.limbs_b, core_BigInt.Split(_xlpm.norm_b, _xlpm.k), _xlpm.final_limbs, core_BigInt.UMul(_xlpm.limbs_a, _xlpm.limbs_b, _xlpm.k), core_BigInt.Merge(_xlpm.final_limbs, _xlpm.k))))))</definedName>
+    <definedName name="BigInt.Abs" comment="Returns the unsigned magnitude of a BigInt string (absolute value)._x000a_[input: Text]">_xlfn.LAMBDA(_xlpm.input, _xlfn.LET(_xlpm.str_norm, BigInt.Norm(_xlpm.input), IF(LEFT(_xlpm.str_norm) = "-", MID(_xlpm.str_norm, 2, LEN(_xlpm.str_norm) - 1), _xlpm.str_norm)))</definedName>
+    <definedName name="BigInt.Add" comment="Returns the sum of two BigInt strings._x000a_[input_a: Text, input_b: Text]">_xlfn.LAMBDA(_xlpm.input_a,_xlpm.input_b, _xlfn.LET(_xlpm.str_norm_a, BigInt.Norm(_xlpm.input_a), _xlpm.str_norm_b, BigInt.Norm(_xlpm.input_b), _xlpm.sign_a, BigInt.Sign(_xlpm.str_norm_a), _xlpm.sign_b, BigInt.Sign(_xlpm.str_norm_b), _xlpm.k, core_BigInt.SafeK("ADD"), _xlpm.limbs_a, core_BigInt.Split(BigInt.Abs(_xlpm.str_norm_a), _xlpm.k), _xlpm.limbs_b, core_BigInt.Split(BigInt.Abs(_xlpm.str_norm_b), _xlpm.k), _xlpm.packed_result, core_BigInt.AddSubRouter(_xlpm.limbs_a, _xlpm.limbs_b, _xlpm.sign_a, _xlpm.sign_b, _xlpm.k), _xlpm.final_sign, _xlfn.CHOOSEROWS(_xlpm.packed_result, -1), _xlpm.final_limbs, _xlfn.DROP(_xlpm.packed_result, -1), _xlpm.str_merged, core_BigInt.Merge(_xlpm.final_limbs, _xlpm.k), IF(_xlpm.final_sign = -1, "-" &amp; _xlpm.str_merged, _xlpm.str_merged)))</definedName>
+    <definedName name="BigInt.Compare" comment="Returns 1 (a &gt; b), -1 (a &lt; b), or 0 (a = b). Compares signs and lengths before limb analysis._x000a_[input_a: Text, input_b: Text]">_xlfn.LAMBDA(_xlpm.input_a,_xlpm.input_b, _xlfn.LET(_xlpm.str_norm_a, BigInt.Norm(_xlpm.input_a), _xlpm.str_norm_b, BigInt.Norm(_xlpm.input_b), _xlpm.sign_a, BigInt.Sign(_xlpm.str_norm_a), _xlpm.sign_b, BigInt.Sign(_xlpm.str_norm_b), IF(_xlpm.sign_a &lt;&gt; _xlpm.sign_b, SIGN(_xlpm.sign_a - _xlpm.sign_b), IF(_xlpm.sign_a = 0, 0, _xlfn.LET(_xlpm.len_a, LEN(_xlpm.str_norm_a), _xlpm.len_b, LEN(_xlpm.str_norm_b), IF(_xlpm.len_a &lt;&gt; _xlpm.len_b, SIGN(_xlpm.len_a - _xlpm.len_b) * _xlpm.sign_a, _xlfn.LET(_xlpm.k, core_BigInt.SafeK("ADD"), _xlpm.limbs_a, core_BigInt.Split(BigInt.Abs(_xlpm.str_norm_a), _xlpm.k), _xlpm.limbs_b, core_BigInt.Split(BigInt.Abs(_xlpm.str_norm_b), _xlpm.k), _xlpm.magnitude_comparison, core_BigInt.UCompare(_xlpm.limbs_a, _xlpm.limbs_b), _xlpm.magnitude_comparison * _xlpm.sign_a)))))))</definedName>
+    <definedName name="BigInt.Div" comment="Returns the quotient of A / B. Defaults to Truncated division._x000a_[input_a: Text, input_b: Text, use_floor: Bool]">_xlfn.LAMBDA(_xlpm.input_a,_xlpm.input_b,_xlop.use_floor, INDEX(BigInt.DivMod(_xlpm.input_a, _xlpm.input_b, _xlpm.use_floor), 1, 1))</definedName>
+    <definedName name="BigInt.DivMod" comment="Returns 2-row array: [Quotient; Remainder]. Supports Truncated or Floor division._x000a_[input_a: Text, input_b: Text, use_floor: Bool]">_xlfn.LAMBDA(_xlpm.input_a,_xlpm.input_b,_xlop.use_floor, _xlfn.LET(_xlpm.str_norm_a, BigInt.Norm(_xlpm.input_a), _xlpm.str_norm_b, BigInt.Norm(_xlpm.input_b), _xlpm.sign_a, BigInt.Sign(_xlpm.str_norm_a), _xlpm.sign_b, BigInt.Sign(_xlpm.str_norm_b), _xlpm.is_floor_div, IF(_xlfn.ISOMITTED(_xlpm.use_floor), FALSE, _xlpm.use_floor), IF(_xlpm.sign_b = 0, #DIV/0!, IF(_xlpm.sign_a = 0, {"0";"0"}, _xlfn.LET(_xlpm.k, core_BigInt.SafeK("DIV"), _xlpm.limbs_a, core_BigInt.Split(BigInt.Abs(_xlpm.str_norm_a), _xlpm.k), _xlpm.limbs_b, core_BigInt.Split(BigInt.Abs(_xlpm.str_norm_b), _xlpm.k), _xlpm.packed_result, core_BigInt.DivRouter(_xlpm.limbs_a, _xlpm.limbs_b, _xlpm.k), _xlpm.len_remainder, INDEX(_xlpm.packed_result, 1, 1), _xlpm.limbs_remainder, _xlfn.CHOOSEROWS(_xlpm.packed_result, _xlfn.SEQUENCE(_xlpm.len_remainder, 1, 2)), _xlpm.limbs_quotient, _xlfn.DROP(_xlpm.packed_result, _xlpm.len_remainder + 1), _xlpm.final_sign, _xlpm.sign_a * _xlpm.sign_b, _xlpm.str_merged_q, core_BigInt.Merge(_xlpm.limbs_quotient, _xlpm.k), _xlpm.str_merged_r, core_BigInt.Merge(_xlpm.limbs_remainder, _xlpm.k), _xlpm.str_trunc_q, IF(AND(_xlpm.final_sign = -1, _xlpm.str_merged_q &lt;&gt; "0"), "-" &amp; _xlpm.str_merged_q, _xlpm.str_merged_q), _xlpm.str_trunc_r, IF(AND(_xlpm.sign_a = -1, _xlpm.str_merged_r &lt;&gt; "0"), "-" &amp; _xlpm.str_merged_r, _xlpm.str_merged_r), _xlpm.needs_floor_correction, AND(_xlpm.is_floor_div, _xlpm.final_sign = -1, _xlpm.str_merged_r &lt;&gt; "0"), _xlpm.str_final_q, IF(_xlpm.needs_floor_correction, BigInt.Sub(_xlpm.str_trunc_q, "1"), _xlpm.str_trunc_q), _xlpm.str_final_r, IF(_xlpm.needs_floor_correction, BigInt.Add(_xlpm.str_trunc_r, _xlpm.str_norm_b), _xlpm.str_trunc_r), _xlfn.VSTACK(_xlpm.str_final_q, _xlpm.str_final_r))))))</definedName>
+    <definedName name="BigInt.Fact" comment="Returns the factorial (n!) using Prime Swing. Max input: 9273._x000a_[input: Text]">_xlfn.LAMBDA(_xlpm.input, _xlfn.LET(_xlpm.str_norm, BigInt.Norm(_xlpm.input), _xlpm.sign_n, BigInt.Sign(_xlpm.str_norm), IF(_xlpm.sign_n = -1, #NUM!, IF(_xlpm.str_norm = "0", "1", IF(_xlpm.str_norm = "1", "1", IF(LEN(_xlpm.str_norm) &gt; 4, #NUM!, IF(VALUE(_xlpm.str_norm) &gt; 9273, #NUM!, _xlfn.LET(_xlpm.num_n, VALUE(_xlpm.str_norm), _xlpm.global_primes, core_BigInt.NativePrimes(_xlpm.num_n), core_BigInt.PrimeSwingKernel(_xlpm.num_n, _xlpm.global_primes)))))))))</definedName>
+    <definedName name="BigInt.IsEven" comment="Returns TRUE if the BigInt is even._x000a_[input: Text]">_xlfn.LAMBDA(_xlpm.input, ISEVEN(VALUE(RIGHT(BigInt.Norm(_xlpm.input)))))</definedName>
+    <definedName name="BigInt.IsNeg" comment="Returns TRUE if the BigInt is negative._x000a_[input: Text]">_xlfn.LAMBDA(_xlpm.input, LEFT(BigInt.Norm(_xlpm.input)) = "-")</definedName>
+    <definedName name="BigInt.IsOdd" comment="Returns TRUE if the BigInt is odd._x000a_[input: Text]">_xlfn.LAMBDA(_xlpm.input, ISODD(VALUE(RIGHT(BigInt.Norm(_xlpm.input)))))</definedName>
+    <definedName name="BigInt.IsZero" comment="Returns TRUE if the BigInt is exactly zero._x000a_[input: Text]">_xlfn.LAMBDA(_xlpm.input, BigInt.Norm(_xlpm.input) = "0")</definedName>
+    <definedName name="BigInt.Max" comment="Returns the maximum BigInt from a range or array._x000a_[range: Range/Array]">_xlfn.LAMBDA(_xlpm.range, _xlfn.LET(_xlpm.flattened_col, _xlfn.TOCOL(_xlpm.range, 1), IF(OR(ISERROR(_xlpm.flattened_col), ROWS(_xlpm.flattened_col) = 0), "0", core_BigInt.TreeCompare(_xlfn.MAP(_xlpm.flattened_col, BigInt.Norm), 1))))</definedName>
+    <definedName name="BigInt.Min" comment="Returns the minimum BigInt from a range or array._x000a_[range: Range/Array]">_xlfn.LAMBDA(_xlpm.range, _xlfn.LET(_xlpm.flattened_col, _xlfn.TOCOL(_xlpm.range, 1), IF(OR(ISERROR(_xlpm.flattened_col), ROWS(_xlpm.flattened_col) = 0), "0", core_BigInt.TreeCompare(_xlfn.MAP(_xlpm.flattened_col, BigInt.Norm), -1))))</definedName>
+    <definedName name="BigInt.Mod" comment="Returns the remainder of A / B. Defaults to Truncated division._x000a_[input_a: Text, input_b: Text, use_floor: Bool]">_xlfn.LAMBDA(_xlpm.input_a,_xlpm.input_b,_xlop.use_floor, INDEX(BigInt.DivMod(_xlpm.input_a, _xlpm.input_b, _xlpm.use_floor), 2, 1))</definedName>
+    <definedName name="BigInt.Mul" comment="Returns the product of two BigInt strings._x000a_[input_a: Text, input_b: Text]">_xlfn.LAMBDA(_xlpm.input_a,_xlpm.input_b, _xlfn.LET(_xlpm.str_norm_a, BigInt.Norm(_xlpm.input_a), _xlpm.str_norm_b, BigInt.Norm(_xlpm.input_b), _xlpm.sign_a, BigInt.Sign(_xlpm.str_norm_a), _xlpm.sign_b, BigInt.Sign(_xlpm.str_norm_b), _xlpm.len_a, LEN(_xlpm.str_norm_a) - IF(_xlpm.sign_a = -1, 1, 0), _xlpm.len_b, LEN(_xlpm.str_norm_b) - IF(_xlpm.sign_b = -1, 1, 0), IF(OR(_xlpm.sign_a = 0, _xlpm.sign_b = 0), "0", IF(_xlpm.len_a + _xlpm.len_b &gt; 32766, #NUM!, _xlfn.LET(_xlpm.k, core_BigInt.SafeK("MUL", MIN(_xlpm.len_a, _xlpm.len_b)), _xlpm.limbs_a, core_BigInt.Split(BigInt.Abs(_xlpm.str_norm_a), _xlpm.k), _xlpm.limbs_b, core_BigInt.Split(BigInt.Abs(_xlpm.str_norm_b), _xlpm.k), _xlpm.final_limbs, core_BigInt.UMul(_xlpm.limbs_a, _xlpm.limbs_b, _xlpm.k), _xlpm.final_sign, _xlpm.sign_a * _xlpm.sign_b, _xlpm.str_merged, core_BigInt.Merge(_xlpm.final_limbs, _xlpm.k), IF(_xlpm.final_sign = -1, "-" &amp; _xlpm.str_merged, _xlpm.str_merged))))))</definedName>
+    <definedName name="BigInt.Norm" comment="Normalises a BigInt string. Strips leading zeros, resolves &quot;-0&quot; to &quot;0&quot;, and throws #VALUE! on invalid characters._x000a_[input: Text]">_xlfn.LAMBDA(_xlpm.input, _xlfn.LET(_xlpm.str_input, IF(OR(_xlfn.ISOMITTED(_xlpm.input), _xlpm.input = ""), "0", _xlpm.input &amp; ""), _xlpm.is_value_format, _xlfn.REGEXTEST(_xlpm.str_input, "^-?\d+$"), _xlpm.str_norm, _xlfn.REGEXREPLACE(_xlpm.str_input, "^(-?)0+(?=\d)", "$1"), IF(NOT(_xlpm.is_value_format), VALUE("#VALUE!"), IF(_xlpm.str_norm = "-0", "0", _xlpm.str_norm))))</definedName>
+    <definedName name="BigInt.Pow" comment="Returns base raised to the power of exponent._x000a_[base: Text, exponent: Text]">_xlfn.LAMBDA(_xlpm.base,_xlpm.exponent, _xlfn.LET(_xlpm.str_norm_base, BigInt.Norm(_xlpm.base), _xlpm.str_norm_exp, BigInt.Norm(_xlpm.exponent), _xlpm.sign_base, BigInt.Sign(_xlpm.str_norm_base), _xlpm.sign_exp, BigInt.Sign(_xlpm.str_norm_exp), _xlpm.str_abs_base, BigInt.Abs(_xlpm.str_norm_base), _xlpm.str_abs_exp, BigInt.Abs(_xlpm.str_norm_exp), _xlpm.is_exp_even, ISEVEN(VALUE(RIGHT(_xlpm.str_norm_exp, 1))), _xlpm.final_sign, IF(_xlpm.sign_base = -1, IF(_xlpm.is_exp_even, 1, -1), _xlpm.sign_base), IF(_xlpm.str_abs_base = "0", IF(_xlpm.str_norm_exp = "0", #NUM!, "0"), IF(_xlpm.str_abs_base = "1", IF(_xlpm.final_sign = -1, "-1", "1"), IF(_xlpm.sign_exp = -1, "0", IF(_xlpm.str_norm_exp = "0", "1", IF(LEN(_xlpm.str_norm_exp) &gt; 6, #NUM!, _xlfn.LET(_xlpm.num_exp, VALUE(_xlpm.str_norm_exp), _xlpm.base_log10,LOG10(VALUE(LEFT(_xlpm.str_abs_base, 14))) + MAX(0, LEN(_xlpm.str_abs_base) - 14), _xlpm.approx_digits, _xlpm.num_exp * _xlpm.base_log10, IF(_xlpm.approx_digits &gt; 32766, #NUM!, _xlfn.LET(_xlpm.k, core_BigInt.SafeK("MUL", _xlpm.approx_digits / 2), _xlpm.limbs_base, core_BigInt.Split(_xlpm.str_abs_base, _xlpm.k), _xlpm.limbs_final, core_BigInt.UPow(_xlpm.limbs_base, _xlpm.str_norm_exp, _xlpm.k), _xlpm.str_merged, core_BigInt.Merge(_xlpm.limbs_final, _xlpm.k), IF(_xlpm.final_sign = -1, "-" &amp; _xlpm.str_merged, _xlpm.str_merged)))))))))))</definedName>
+    <definedName name="BigInt.RandArray" comment="[VOLATILE] Generates a dynamic array of random BigInt strings._x000a_[num_rows: int, num_cols: int, min_digits: int, max_digits: int]">_xlfn.LAMBDA(_xlop.num_rows,_xlop.num_cols,_xlop.min_digits,_xlop.max_digits, _xlfn.LET(_xlpm.n_rows, IF(_xlfn.ISOMITTED(_xlpm.num_rows), 1, _xlpm.num_rows), _xlpm.n_cols, IF(_xlfn.ISOMITTED(_xlpm.num_cols), 1, _xlpm.num_cols), _xlpm.min_len, IF(_xlfn.ISOMITTED(_xlpm.min_digits), 16, MIN(32767, MAX(1, _xlpm.min_digits))), _xlpm.max_len, IF(_xlfn.ISOMITTED(_xlpm.max_digits), 50, MAX(1, MIN(32766, _xlpm.max_digits))), _xlfn.MAP(_xlfn.RANDARRAY(_xlpm.n_rows, _xlpm.n_cols, _xlpm.min_len, _xlpm.max_len, TRUE), _xlfn.LAMBDA(_xlpm.length, _xlfn.LET(_xlpm.sign_prefix, CHOOSE(RANDBETWEEN(1, 2), "", "-"), _xlpm.rand_digits, _xlfn.CONCAT(_xlfn.RANDARRAY(1, _xlpm.length, 0, 9, TRUE)), _xlpm.sign_prefix &amp; _xlfn.REGEXREPLACE(_xlpm.rand_digits, "^0*", ""))))))</definedName>
+    <definedName name="BigInt.Sign" comment="Returns the sign of a BigInt: 1 (positive), -1 (negative), or 0 (zero)._x000a_[input: Text]">_xlfn.LAMBDA(_xlpm.input, _xlfn.LET(_xlpm.str_norm, BigInt.Norm(_xlpm.input), _xlfn.SWITCH(LEFT(_xlpm.str_norm), "0", 0, "-", -1, 1)))</definedName>
+    <definedName name="BigInt.Sqrt" comment="Returns the integer square root (floor) of a BigInt._x000a_[input: Text]">_xlfn.LAMBDA(_xlpm.input, _xlfn.LET(_xlpm.str_norm, BigInt.Norm(_xlpm.input), _xlpm.sign_n, BigInt.Sign(_xlpm.str_norm), IF(_xlpm.sign_n = -1, #NUM!, IF(_xlpm.str_norm = "0", "0", IF(_xlpm.str_norm = "1", "1", _xlfn.LET(_xlpm.len_norm, LEN(_xlpm.str_norm), _xlpm.num_seed_precision, IF(_xlpm.len_norm &lt;= 14, _xlpm.len_norm, IF(ISEVEN(_xlpm.len_norm), 14, 13)), _xlpm.str_native_precision, LEFT(_xlpm.str_norm, _xlpm.num_seed_precision), _xlpm.num_native_precision, VALUE(_xlpm.str_native_precision), _xlpm.num_magnitude_zeroes, (_xlpm.len_norm - _xlpm.num_seed_precision) / 2, _xlpm.str_prefix, TEXT(ROUNDUP(SQRT(_xlpm.num_native_precision), 0) + 1, "0"), _xlpm.str_seed, _xlpm.str_prefix &amp; REPT("0", _xlpm.num_magnitude_zeroes), _xlpm.k, core_BigInt.SafeK("MUL", _xlpm.len_norm), _xlpm.limbs_radicand, core_BigInt.Split(_xlpm.str_norm, _xlpm.k), _xlpm.limbs_seed, core_BigInt.Split(_xlpm.str_seed, _xlpm.k), _xlpm.limbs_final, core_BigInt.USqrt(_xlpm.limbs_radicand, _xlpm.limbs_seed, _xlpm.k), core_BigInt.Merge(_xlpm.limbs_final, _xlpm.k)))))))</definedName>
+    <definedName name="BigInt.Sub" comment="Returns the difference of two BigInt strings (A - B)._x000a_[input_a: Text, input_b: Text]">_xlfn.LAMBDA(_xlpm.input_a,_xlpm.input_b, _xlfn.LET(_xlpm.str_norm_b, BigInt.Norm(_xlpm.input_b), _xlpm.str_inverse_b, IF(_xlpm.str_norm_b = "0", "0", IF(LEFT(_xlpm.str_norm_b) = "-", MID(_xlpm.str_norm_b, 2, LEN(_xlpm.str_norm_b)), "-" &amp; _xlpm.str_norm_b)), BigInt.Add(_xlpm.input_a, _xlpm.str_inverse_b)))</definedName>
+    <definedName name="BigInt.Sum" comment="Sums a range or array of BigInt strings._x000a_[input_range: Range/Array]">_xlfn.LAMBDA(_xlpm.input_range, _xlfn.LET(_xlpm.flattened_input, _xlfn.TOROW(_xlpm.input_range, 1), IF(OR(ISERROR(_xlpm.flattened_input), COLUMNS(_xlpm.flattened_input) = 0), "0", _xlfn.LET(_xlpm.str_norms, _xlfn.MAP(_xlpm.flattened_input, _xlfn.LAMBDA(_xlpm.x, BigInt.Norm(_xlpm.x))), _xlpm.arr_signs, _xlfn.MAP(LEFT(_xlpm.str_norms), _xlfn.LAMBDA(_xlpm.x, IF(_xlpm.x = "0", 0, IF(_xlpm.x = "-", -1, 1)))), _xlpm.str_abs, _xlfn.MAP(_xlpm.str_norms, _xlpm.arr_signs, _xlfn.LAMBDA(_xlpm.x,_xlpm.sign, IF(_xlpm.sign = -1, MID(_xlpm.x, 2, LEN(_xlpm.x) - 1), _xlpm.x))), _xlpm.str_pos, _xlfn._xlws.FILTER(_xlpm.str_abs, _xlpm.arr_signs = 1, {"0"}), _xlpm.str_negs, _xlfn._xlws.FILTER(_xlpm.str_abs, _xlpm.arr_signs = -1, {"0"}), _xlpm.unified_k, core_BigInt.SafeK("ADD", COLUMNS(_xlpm.flattened_input)), _xlpm.limbs_pos_sum, core_BigInt.UMatrixSum(_xlpm.str_pos, _xlpm.unified_k), _xlpm.limbs_neg_sum, core_BigInt.UMatrixSum(_xlpm.str_negs, _xlpm.unified_k), _xlpm.packed_result, core_BigInt.AddSubRouter(_xlpm.limbs_pos_sum, _xlpm.limbs_neg_sum, 1, -1, _xlpm.unified_k), _xlpm.final_sign, _xlfn.CHOOSEROWS(_xlpm.packed_result, -1), _xlpm.final_limbs, _xlfn.DROP(_xlpm.packed_result, -1), _xlpm.str_merged, core_BigInt.Merge(_xlpm.final_limbs, _xlpm.unified_k), IF(_xlpm.final_sign = -1, "-" &amp; _xlpm.str_merged, _xlpm.str_merged)))))</definedName>
+    <definedName name="core_BigInt.AddSubRouter" comment="[Internal] Returns packed array: [limbs; final_sign]. Resolves sign logic for Add/Sub._x000a_[limbs_a: Array, limbs_b: Array, sign_a: int, sign_b: int, k: int]">_xlfn.LAMBDA(_xlpm.limbs_a,_xlpm.limbs_b,_xlpm.sign_a,_xlpm.sign_b,_xlpm.k, _xlfn.LET(_xlpm.is_addition, _xlpm.sign_a = _xlpm.sign_b, IF(_xlpm.is_addition, _xlfn.VSTACK(core_BigInt.UAdd(_xlpm.limbs_a, _xlpm.limbs_b, _xlpm.k), _xlpm.sign_a), _xlfn.LET(_xlpm.magnitude_comparison, core_BigInt.UCompare(_xlpm.limbs_a, _xlpm.limbs_b), IF(_xlpm.magnitude_comparison = 0, {0;0}, IF(_xlpm.magnitude_comparison &gt; 0, _xlfn.VSTACK(core_BigInt.USub(_xlpm.limbs_a, _xlpm.limbs_b, _xlpm.k), _xlpm.sign_a), _xlfn.VSTACK(core_BigInt.USub(_xlpm.limbs_b, _xlpm.limbs_a, _xlpm.k), _xlpm.sign_b)))))))</definedName>
+    <definedName name="core_BigInt.Carry" comment="[Internal] Resolves carries right-to-left across a vertical array of base-10^k limbs._x000a_[limbs: Array, k: int]">_xlfn.LAMBDA(_xlpm.limbs,_xlpm.k, _xlfn.LET(_xlpm.num_limbs, ROWS(_xlpm.limbs), _xlpm.radix_base, 10 ^ _xlpm.k, _xlpm.arr_carries, _xlfn.SCAN(0, _xlpm.limbs, _xlfn.LAMBDA(_xlpm.acc,_xlpm.val, _xlpm.val + INT(_xlpm.acc / _xlpm.radix_base))), _xlpm.remainders, MOD(_xlpm.arr_carries, _xlpm.radix_base), _xlpm.final_carry, INT(INDEX(_xlpm.arr_carries, _xlpm.num_limbs, 1) / _xlpm.radix_base), IF(_xlpm.final_carry &gt; 0, _xlfn.VSTACK(_xlpm.remainders, _xlpm.final_carry), _xlpm.remainders)))</definedName>
+    <definedName name="core_BigInt.DivRouter" comment="[Internal] Routes division to Knuth or Newton-Raphson based on Dividend length._x000a_[limbs_a: Array, limbs_b: Array, k: int]">_xlfn.LAMBDA(_xlpm.limbs_a,_xlpm.limbs_b,_xlpm.k, _xlfn.LET(_xlpm.approx_digits_a, ROWS(_xlpm.limbs_a) * _xlpm.k, _xlpm.approx_digits_b, ROWS(_xlpm.limbs_b) * _xlpm.k, _xlpm.regression_slope_m, 0.107821194271297, _xlpm.regression_intercept_c, -221.902189462068, _xlpm.threshold_digits, (_xlpm.regression_slope_m * _xlpm.approx_digits_a) + _xlpm.regression_intercept_c, IF(_xlpm.approx_digits_b &lt;= _xlpm.threshold_digits, core_BigInt.KnuthDiv(_xlpm.limbs_a, _xlpm.limbs_b, _xlpm.k), core_BigInt.NewtonRaphsonDiv(_xlpm.limbs_a, _xlpm.limbs_b, _xlpm.k))))</definedName>
+    <definedName name="core_BigInt.FindQuotientLimb" comment="[Internal] Returns highest scalar quotient limb q (0 &lt;= q &lt; 10^k) where B * q &lt;= R._x000a_[limbs_r: Array, limbs_b: Array, k: int]">_xlfn.LAMBDA(_xlpm.limbs_r,_xlpm.limbs_b,_xlpm.k, _xlfn.LET(_xlpm.required_bits, _xlfn.CEILING.MATH(LOG(10 ^ _xlpm.k, 2)), _xlpm.powers_of_two, 2 ^ _xlfn.SEQUENCE(_xlpm.required_bits, 1, _xlpm.required_bits - 1, -1), _xlfn.REDUCE(0, _xlpm.powers_of_two, _xlfn.LAMBDA(_xlpm.current_q,_xlpm.current_power, _xlfn.LET(_xlpm.test_q, _xlpm.current_q + _xlpm.current_power, IF(_xlpm.test_q &gt;= 10 ^ _xlpm.k, _xlpm.current_q, _xlfn.LET(_xlpm.limbs_bq, core_BigInt.Carry(_xlpm.limbs_b * _xlpm.test_q, _xlpm.k), _xlpm.magnitude_comparison, core_BigInt.UCompare(_xlpm.limbs_r, _xlpm.limbs_bq), IF(_xlpm.magnitude_comparison &gt;= 0, _xlpm.test_q, _xlpm.current_q))))))))</definedName>
+    <definedName name="core_BigInt.KnuthDiv" comment="[Internal] Returns packed array: [Len_R; R_limbs; Q_limbs] using sequential long division._x000a_[limbs_a: Array, limbs_b: Array, k: int]">_xlfn.LAMBDA(_xlpm.limbs_a,_xlpm.limbs_b,_xlpm.k, _xlfn.LET(_xlpm.magnitude_comparison, core_BigInt.UCompare(_xlpm.limbs_a, _xlpm.limbs_b), IF(_xlpm.magnitude_comparison &lt; 0, _xlfn.VSTACK(ROWS(_xlpm.limbs_a), _xlpm.limbs_a, 0), IF(_xlpm.magnitude_comparison = 0, _xlfn.VSTACK(1, 0, 1), _xlfn.LET(_xlpm.num_limbs_a, ROWS(_xlpm.limbs_a), _xlpm.big_endian_a, _xlfn.CHOOSEROWS(_xlpm.limbs_a, _xlfn.SEQUENCE(_xlpm.num_limbs_a, 1, _xlpm.num_limbs_a, -1)), _xlpm.final_packed_state, _xlfn.REDUCE(_xlfn.VSTACK(1, 0, 0), _xlpm.big_endian_a, _xlfn.LAMBDA(_xlpm.packed_state,_xlpm.val, _xlfn.LET(_xlpm.num_limbs_r, INDEX(_xlpm.packed_state, 1, 1), _xlpm.limbs_r, _xlfn.CHOOSEROWS(_xlpm.packed_state, _xlfn.SEQUENCE(_xlpm.num_limbs_r, 1, 2)), _xlpm.limbs_q, _xlfn.DROP(_xlpm.packed_state, _xlpm.num_limbs_r + 1), _xlpm.limbs_shifted_r, IF(AND(ROWS(_xlpm.limbs_r) = 1, INDEX(_xlpm.limbs_r, 1, 1) = 0), _xlpm.val, _xlfn.VSTACK(_xlpm.val, _xlpm.limbs_r)), _xlpm.q_limb, core_BigInt.FindQuotientLimb(_xlpm.limbs_shifted_r, _xlpm.limbs_b, _xlpm.k), _xlpm.limbs_bq, core_BigInt.Carry(_xlpm.limbs_b * _xlpm.q_limb, _xlpm.k), _xlpm.limbs_next_r, core_BigInt.USub(_xlpm.limbs_shifted_r, _xlpm.limbs_bq, _xlpm.k), _xlpm.has_q, OR(ROWS(_xlpm.limbs_q) &gt; 1, INDEX(_xlpm.limbs_q, 1, 1) &gt; 0), _xlpm.limbs_next_q, IF(_xlpm.has_q, _xlfn.VSTACK(_xlpm.limbs_q, _xlpm.q_limb), _xlpm.q_limb), _xlfn.VSTACK(ROWS(_xlpm.limbs_next_r), _xlpm.limbs_next_r, _xlpm.limbs_next_q)))), _xlpm.num_limbs_r, INDEX(_xlpm.final_packed_state, 1, 1), _xlpm.limbs_r, _xlfn.CHOOSEROWS(_xlpm.final_packed_state, _xlfn.SEQUENCE(_xlpm.num_limbs_r, 1, 2)), _xlpm.big_endian_q, _xlfn.DROP(_xlpm.final_packed_state, _xlpm.num_limbs_r + 1), _xlpm.len_q, ROWS(_xlpm.big_endian_q), _xlpm.limbs_q, _xlfn.CHOOSEROWS(_xlpm.big_endian_q, _xlfn.SEQUENCE(_xlpm.len_q, 1, _xlpm.len_q, -1)), _xlfn.VSTACK(_xlpm.num_limbs_r, _xlpm.limbs_r, _xlpm.limbs_q))))))</definedName>
+    <definedName name="core_BigInt.Merge" comment="[Internal] Merges Little-Endian limb arrays into a Big-Endian BigInt string._x000a_[limbs: Array, k: int]">_xlfn.LAMBDA(_xlpm.limbs,_xlpm.k, _xlfn.LET(_xlpm.num_limbs, ROWS(_xlpm.limbs), _xlpm.rev_limbs, _xlfn.CHOOSEROWS(_xlpm.limbs, _xlfn.SEQUENCE(_xlpm.num_limbs, 1, _xlpm.num_limbs, -1)), IF(_xlpm.num_limbs = 1, _xlpm.rev_limbs &amp; "", _xlfn.CONCAT(_xlfn.VSTACK(_xlfn.TAKE(_xlpm.rev_limbs, 1) &amp; "", TEXT(_xlfn.DROP(_xlpm.rev_limbs, 1), REPT("0", _xlpm.k)))))))</definedName>
+    <definedName name="core_BigInt.NativePrimes" comment="[Internal] Returns a vertical array of prime numbers up to n._x000a_[n: int]">_xlfn.LAMBDA(_xlpm.n, IF(_xlpm.n &lt; 2, #NUM!, _xlfn.LET(_xlpm.candidate_sequence, _xlfn.SEQUENCE(_xlpm.n - 1, 1, 2), _xlfn._xlws.FILTER(_xlpm.candidate_sequence, _xlfn.MAP(_xlpm.candidate_sequence, _xlfn.LAMBDA(_xlpm.current_candidate, _xlfn.LET(_xlpm.limit, INT(SQRT(_xlpm.current_candidate)), IF(_xlpm.limit &lt; 2, TRUE, MIN(MOD(_xlpm.current_candidate, _xlfn.SEQUENCE(_xlpm.limit - 1, 1, 2))) &gt; 0))))))))</definedName>
+    <definedName name="core_BigInt.NativeSwingExponents" comment="[Internal] Returns the exponent for each prime in the Prime Swing term._x000a_[n: int, primes: Array]">_xlfn.LAMBDA(_xlpm.n,_xlpm.primes, _xlfn.MAP(_xlpm.primes, _xlfn.LAMBDA(_xlpm.p, _xlfn.LET(_xlpm.max_power_k, INT(LOG(_xlpm.n, _xlpm.p)), _xlpm.prime_powers, _xlpm.p ^ _xlfn.SEQUENCE(_xlpm.max_power_k), SUM(MOD(INT(_xlpm.n / _xlpm.prime_powers), 2))))))</definedName>
+    <definedName name="core_BigInt.NewtonRaphsonDiv" comment="[Internal] Returns packed array: [Len_R; R_limbs; Q_limbs] using Newton-Raphson._x000a_[limbs_a: Array, limbs_b: Array, k: int]">_xlfn.LAMBDA(_xlpm.limbs_a,_xlpm.limbs_b,_xlpm.k, _xlfn.LET(_xlpm.num_limbs_a, ROWS(_xlpm.limbs_a), _xlpm.num_limbs_b, ROWS(_xlpm.limbs_b), _xlpm.num_limbs_target, MAX(_xlpm.num_limbs_a, _xlpm.num_limbs_b), _xlpm.limbs_reciprocal, core_BigInt.NewtonRaphsonReciprocal(_xlpm.limbs_b, _xlpm.num_limbs_target, _xlpm.k), _xlpm.right_shift_limbs, 2 * _xlpm.num_limbs_target, _xlpm.limbs_q_unscaled, core_BigInt.UMul(_xlpm.limbs_a, _xlpm.limbs_reciprocal, _xlpm.k), _xlpm.limbs_q_approx, IF(ROWS(_xlpm.limbs_q_unscaled) &lt;= _xlpm.right_shift_limbs, {0}, _xlfn.DROP(_xlpm.limbs_q_unscaled, _xlpm.right_shift_limbs)), _xlpm.limbs_p_baseline, core_BigInt.UMul(_xlpm.limbs_b, _xlpm.limbs_q_approx, _xlpm.k), _xlpm.initial_packed_state, _xlfn.VSTACK(ROWS(_xlpm.limbs_q_approx), _xlpm.limbs_q_approx, _xlpm.limbs_p_baseline), _xlpm.packed_state_swept_down, _xlfn.REDUCE(_xlpm.initial_packed_state, {1;2}, _xlfn.LAMBDA(_xlpm.packed_state,_xlpm.i, _xlfn.LET(_xlpm.len_q, INDEX(_xlpm.packed_state, 1, 1), _xlpm.limbs_current_q, _xlfn.CHOOSEROWS(_xlpm.packed_state, _xlfn.SEQUENCE(_xlpm.len_q, 1, 2)), _xlpm.limbs_current_p, _xlfn.DROP(_xlpm.packed_state, _xlpm.len_q + 1), IF(core_BigInt.UCompare(_xlpm.limbs_current_p, _xlpm.limbs_a) &lt;= 0, _xlpm.packed_state, _xlfn.LET(_xlpm.limbs_next_q, core_BigInt.USub(_xlpm.limbs_current_q, {1}, _xlpm.k), _xlpm.limbs_next_p, core_BigInt.USub(_xlpm.limbs_current_p, _xlpm.limbs_b, _xlpm.k), _xlfn.VSTACK(ROWS(_xlpm.limbs_next_q), _xlpm.limbs_next_q, _xlpm.limbs_next_p)))))), _xlpm.packed_state_swept_up, _xlfn.REDUCE(_xlpm.packed_state_swept_down, {1;2}, _xlfn.LAMBDA(_xlpm.packed_state,_xlpm.i, _xlfn.LET(_xlpm.len_q, INDEX(_xlpm.packed_state, 1, 1), _xlpm.limbs_current_q, _xlfn.CHOOSEROWS(_xlpm.packed_state, _xlfn.SEQUENCE(_xlpm.len_q, 1, 2)), _xlpm.limbs_current_p, _xlfn.DROP(_xlpm.packed_state, _xlpm.len_q + 1), _xlpm.limbs_next_p_test, core_BigInt.UAdd(_xlpm.limbs_current_p, _xlpm.limbs_b, _xlpm.k), IF(core_BigInt.UCompare(_xlpm.limbs_next_p_test, _xlpm.limbs_a) &gt; 0, _xlpm.packed_state, _xlfn.LET(_xlpm.limbs_next_q, core_BigInt.UAdd(_xlpm.limbs_current_q, {1}, _xlpm.k), _xlfn.VSTACK(ROWS(_xlpm.limbs_next_q), _xlpm.limbs_next_q, _xlpm.limbs_next_p_test)))))), _xlpm.len_q, INDEX(_xlpm.packed_state_swept_up, 1, 1), _xlpm.limbs_q, _xlfn.CHOOSEROWS(_xlpm.packed_state_swept_up, _xlfn.SEQUENCE(_xlpm.len_q, 1, 2)), _xlpm.limbs_p, _xlfn.DROP(_xlpm.packed_state_swept_up, _xlpm.len_q + 1), _xlpm.limbs_r, core_BigInt.USub(_xlpm.limbs_a, _xlpm.limbs_p, _xlpm.k), _xlfn.VSTACK(ROWS(_xlpm.limbs_r), _xlpm.limbs_r, _xlpm.limbs_q)))</definedName>
+    <definedName name="core_BigInt.NewtonRaphsonReciprocal" comment="[Internal] Returns the Reciprocal R scaled progressively to the Dividend's precision._x000a_[limbs_b: Array, target_len: int, k: int]">_xlfn.LAMBDA(_xlpm.limbs_b,_xlpm.target_len,_xlpm.k, _xlfn.LET(_xlpm.num_limbs_b, ROWS(_xlpm.limbs_b), _xlpm.num_seed_limbs, MIN(3, _xlpm.num_limbs_b), _xlpm.limbs_r_seed, core_BigInt.NewtonRaphsonSeed(_xlpm.limbs_b, _xlpm.k), _xlpm.required_iterations, MAX(0, _xlfn.CEILING.MATH(LN(_xlpm.target_len / _xlpm.num_seed_limbs) / LN(2))) + 1, IF(_xlpm.required_iterations = 0, _xlpm.limbs_r_seed, _xlfn.LET(_xlpm.iterations, _xlfn.SEQUENCE(_xlpm.required_iterations), _xlpm.final_packed_state, _xlfn.REDUCE(_xlfn.VSTACK(_xlpm.num_seed_limbs, _xlpm.limbs_r_seed), _xlpm.iterations, _xlfn.LAMBDA(_xlpm.packed_state,_xlpm.i, _xlfn.LET(_xlpm.current_len, INDEX(_xlpm.packed_state, 1, 1), _xlpm.limbs_current_r, _xlfn.DROP(_xlpm.packed_state, 1), _xlpm.next_len, MIN(_xlpm.current_len * 2, _xlpm.target_len), _xlpm.active_b_limbs_current, MIN(_xlpm.current_len, _xlpm.num_limbs_b), _xlpm.active_b_limbs_next, MIN(_xlpm.next_len, _xlpm.num_limbs_b), _xlpm.required_shift_limbs, 2 * (_xlpm.next_len - _xlpm.current_len) - (_xlpm.active_b_limbs_next - _xlpm.active_b_limbs_current), _xlpm.limbs_r_prime, IF(_xlpm.required_shift_limbs &gt; 0, _xlfn.VSTACK(_xlfn.EXPAND(0, _xlpm.required_shift_limbs, , 0), _xlpm.limbs_current_r), _xlpm.limbs_current_r), _xlpm.limbs_b_active, _xlfn.TAKE(_xlpm.limbs_b, -_xlpm.active_b_limbs_next), _xlpm.limbs_p, core_BigInt.UMul(_xlpm.limbs_b_active, _xlpm.limbs_r_prime, _xlpm.k), _xlpm.limbs_two_beta, _xlfn.VSTACK(_xlfn.EXPAND(0, 2 * _xlpm.next_len, , 0), 2), _xlpm.limbs_error_term, core_BigInt.USub(_xlpm.limbs_two_beta, _xlpm.limbs_p, _xlpm.k), _xlpm.limbs_next_r_unscaled, core_BigInt.UMul(_xlpm.limbs_r_prime, _xlpm.limbs_error_term, _xlpm.k), _xlpm.limbs_next_r, IF(ROWS(_xlpm.limbs_next_r_unscaled) &lt;= 2 * _xlpm.next_len, {0}, _xlfn.DROP(_xlpm.limbs_next_r_unscaled, 2 * _xlpm.next_len)), _xlfn.VSTACK(_xlpm.next_len, _xlpm.limbs_next_r)))), _xlfn.DROP(_xlpm.final_packed_state, 1)))))</definedName>
+    <definedName name="core_BigInt.NewtonRaphsonSeed" comment="[Internal] Returns the reciprocal seed floor(Beta^(2*len) / B_top) via Knuth Basecase._x000a_[limbs_b: Array, k: int]">_xlfn.LAMBDA(_xlpm.limbs_b,_xlpm.k, _xlfn.LET(_xlpm.num_limbs_b, ROWS(_xlpm.limbs_b), _xlpm.num_seed_limbs, MIN(3, _xlpm.num_limbs_b), _xlpm.limbs_b_top, _xlfn.TAKE(_xlpm.limbs_b, -_xlpm.num_seed_limbs), _xlpm.limbs_beta_2m, _xlfn.VSTACK(_xlfn.EXPAND(0, 2 * _xlpm.num_seed_limbs, , 0), 1), _xlpm.packed_basecase_result, core_BigInt.KnuthDiv(_xlpm.limbs_beta_2m, _xlpm.limbs_b_top, _xlpm.k), _xlpm.num_limbs_r, INDEX(_xlpm.packed_basecase_result, 1, 1), _xlfn.DROP(_xlpm.packed_basecase_result, _xlpm.num_limbs_r + 1)))</definedName>
+    <definedName name="core_BigInt.PrimeSwingKernel" comment="[Internal] Returns n! as a string using the recursive Prime Swing algorithm._x000a_[n: int, global_primes: Array]">_xlfn.LAMBDA(_xlpm.n,_xlpm.global_primes, IF(_xlpm.n &lt; 2, "1", _xlfn.LET(_xlpm.floor_half_n, INT(_xlpm.n / 2), _xlpm.factorial_half_n, core_BigInt.PrimeSwingKernel(_xlpm.floor_half_n, _xlpm.global_primes), _xlpm.squared_half_factorial, core_BigInt.UTextMul(_xlpm.factorial_half_n, _xlpm.factorial_half_n), _xlpm.applicable_tier_primes, _xlfn._xlws.FILTER(_xlpm.global_primes, _xlpm.global_primes &lt;= _xlpm.n), _xlpm.str_swing_term, core_BigInt.SwingTerm(_xlpm.n, _xlpm.applicable_tier_primes), core_BigInt.UTextMul(_xlpm.squared_half_factorial, _xlpm.str_swing_term))))</definedName>
+    <definedName name="core_BigInt.SafeK" comment="[Internal] Returns max safe base-10 limb size (k) to prevent IEEE-754 precision loss._x000a_[operation: Text, operand_or_digits: int]">_xlfn.LAMBDA(_xlpm.operation,_xlop.operand_or_digits, _xlfn.LET(_xlpm.resolved_count, IF(OR(_xlpm.operand_or_digits = "", _xlfn.ISOMITTED(_xlpm.operand_or_digits)), 2, MAX(2, _xlpm.operand_or_digits)), _xlfn.SWITCH(_xlpm.operation, "ADD", 15 - LEN(_xlpm.resolved_count), "MUL", _xlfn.LET(_xlpm.test_k, {7;6;5;4;3;2;1}, _xlpm.max_overlap, ROUNDUP(_xlpm.resolved_count / _xlpm.test_k, 0), _xlpm.uncarried_max, _xlpm.max_overlap * (10 ^ _xlpm.test_k - 1) ^ 2, _xlpm.max_carry, INT(_xlpm.uncarried_max / 10 ^ _xlpm.test_k), _xlpm.peak_val, _xlpm.uncarried_max + _xlpm.max_carry, MAX(_xlfn._xlws.FILTER(_xlpm.test_k, _xlpm.peak_val &lt;= (10 ^ 15 - 1)))), "DIV", 7, #NAME?)))</definedName>
+    <definedName name="core_BigInt.Split" comment="[Internal] Splits strings or arrays into Little-Endian numeric limb arrays._x000a_[str_norms: Text/Array, k: int]">_xlfn.LAMBDA(_xlpm.str_norms,_xlpm.k, _xlfn.LET(_xlpm.flattened_norms, _xlfn.TOROW(_xlpm.str_norms), _xlpm.lengths, LEN(_xlpm.flattened_norms), _xlpm.max_len, MAX(_xlpm.lengths), _xlpm.pad_len, ROUNDUP(_xlpm.max_len / _xlpm.k, 0) * _xlpm.k, _xlpm.padded_norms, REPT("0", _xlpm.pad_len - _xlpm.lengths) &amp; _xlpm.flattened_norms, _xlpm.limb_start_indices, _xlfn.SEQUENCE(_xlpm.pad_len / _xlpm.k, 1, _xlpm.pad_len - _xlpm.k + 1, -_xlpm.k), --MID(_xlpm.padded_norms, _xlpm.limb_start_indices, _xlpm.k)))</definedName>
+    <definedName name="core_BigInt.SwingTerm" comment="[Internal] Returns the Swing term for the current factorial tier as a string._x000a_[n: int, tier_primes: Array]">_xlfn.LAMBDA(_xlpm.n,_xlpm.tier_primes, _xlfn.LET(_xlpm.swing_exponents, core_BigInt.NativeSwingExponents(_xlpm.n, _xlpm.tier_primes), _xlpm.has_native_exponent, _xlpm.swing_exponents &gt; 0, IF(AND(NOT(_xlpm.has_native_exponent)), "1", _xlfn.LET(_xlpm.active_primes, _xlfn._xlws.FILTER(_xlpm.tier_primes, _xlpm.has_native_exponent), _xlpm.active_exponents, _xlfn._xlws.FILTER(_xlpm.swing_exponents, _xlpm.has_native_exponent), _xlpm.evalutated_prime_powers, _xlfn.MAP(_xlpm.active_primes, _xlpm.active_exponents, _xlfn.LAMBDA(_xlpm.p,_xlpm.e, IF(_xlpm.e = 1, _xlpm.p &amp; "", BigInt.Pow(_xlpm.p &amp; "", _xlpm.e &amp; "")))), core_BigInt.TextTreeProd(_xlpm.evalutated_prime_powers)))))</definedName>
+    <definedName name="core_BigInt.TextTreeProd" comment="[Internal] Returns the product of an array of strings using a recursive tournament tree._x000a_[arr_strings: Array]">_xlfn.LAMBDA(_xlpm.arr_strings, _xlfn.LET(_xlpm.num_elements, ROWS(_xlpm.arr_strings), IF(_xlpm.num_elements = 1, INDEX(_xlpm.arr_strings, 1, 1), _xlfn.LET(_xlpm.paired_strings, _xlfn.WRAPROWS(_xlpm.arr_strings, 2, "1"), _xlpm.reduced_array, _xlfn.BYROW(_xlpm.paired_strings, _xlfn.LAMBDA(_xlpm.row, core_BigInt.UTextMul(INDEX(_xlpm.row, 1, 1), INDEX(_xlpm.row, 1, 2)))), core_BigInt.TextTreeProd(_xlpm.reduced_array)))))</definedName>
+    <definedName name="core_BigInt.TreeCompare" comment="[Internal] Returns Min/Max from an array of strings using a recursive tournament tree._x000a_[str_norms: Array, comparison_mode: int]">_xlfn.LAMBDA(_xlpm.str_norms,_xlpm.comparison_mode, _xlfn.LET(_xlpm.num_rows, ROWS(_xlpm.str_norms), IF(_xlpm.num_rows = 1, INDEX(_xlpm.str_norms, 1, 1), _xlfn.LET(_xlpm.tournament_pairs, _xlfn.WRAPROWS(_xlpm.str_norms, 2), _xlpm.competitors_a, _xlfn.TAKE(_xlpm.tournament_pairs, , 1), _xlpm.competitors_b, _xlfn.TAKE(_xlpm.tournament_pairs, , -1), _xlpm.round_winners, _xlfn.MAP(_xlpm.competitors_a, _xlpm.competitors_b, _xlfn.LAMBDA(_xlpm.a,_xlpm.b, IF(ISNA(_xlpm.b), _xlpm.a, _xlfn.LET(_xlpm.comparison_result, BigInt.Compare(_xlpm.a, _xlpm.b), IF(_xlpm.comparison_result * _xlpm.comparison_mode &gt;= 0, _xlpm.a, _xlpm.b))))), core_BigInt.TreeCompare(_xlpm.round_winners, _xlpm.comparison_mode)))))</definedName>
+    <definedName name="core_BigInt.UAdd" comment="[Internal] Returns the sum of two unsigned Little-Endian limb arrays._x000a_[a: Array, b: Array, k: int]">_xlfn.LAMBDA(_xlpm.a,_xlpm.b,_xlpm.k, _xlfn.LET(_xlpm.max_rows, MAX(ROWS(_xlpm.a), ROWS(_xlpm.b)), _xlpm.limbs_a_aligned, _xlfn.EXPAND(_xlpm.a, _xlpm.max_rows, 1, 0), _xlpm.limbs_b_aligned, _xlfn.EXPAND(_xlpm.b, _xlpm.max_rows, 1, 0), core_BigInt.Carry(_xlpm.limbs_a_aligned + _xlpm.limbs_b_aligned, _xlpm.k)))</definedName>
+    <definedName name="core_BigInt.UCompare" comment="[Internal] Returns 1 (a &gt; b), -1 (a &lt; b), or 0 (a = b) for unsigned limb arrays._x000a_[limbs_a: Array, limbs_b: Array]">_xlfn.LAMBDA(_xlpm.limbs_a,_xlpm.limbs_b, _xlfn.LET(_xlpm.max_rows, MAX(ROWS(_xlpm.limbs_a), ROWS(_xlpm.limbs_b)), _xlpm.limbs_a_aligned, _xlfn.EXPAND(_xlpm.limbs_a, _xlpm.max_rows, 1, 0), _xlpm.limbs_b_aligned, _xlfn.EXPAND(_xlpm.limbs_b, _xlpm.max_rows, 1, 0), _xlpm.differences, _xlpm.limbs_a_aligned - _xlpm.limbs_b_aligned, _xlpm.highest_non_zero_index, _xlfn.XMATCH(TRUE, _xlpm.differences &lt;&gt; 0, 0, -1), IF(ISNA(_xlpm.highest_non_zero_index), 0, SIGN(INDEX(_xlpm.differences, _xlpm.highest_non_zero_index, 1)))))</definedName>
+    <definedName name="core_BigInt.UMatrixSum" comment="[Internal] Sums a horizontal array of BigInt strings via 2D matrix broadcasting._x000a_[str_norms: Array, k: int]">_xlfn.LAMBDA(_xlpm.str_norms,_xlpm.k, _xlfn.LET(_xlpm.grid, core_BigInt.Split(_xlpm.str_norms, _xlpm.k), _xlpm.raw_limbs, _xlfn.BYROW(_xlpm.grid, _xleta.SUM), core_BigInt.Carry(_xlpm.raw_limbs, _xlpm.k)))</definedName>
+    <definedName name="core_BigInt.UMul" comment="[Internal] Multiplies unsigned Little-Endian limb arrays via 1D Discrete Convolution._x000a_[limbs_a: Array, limbs_b: Array, k: int]">_xlfn.LAMBDA(_xlpm.limbs_a,_xlpm.limbs_b,_xlpm.k, _xlfn.LET(_xlpm.num_limbs_a, ROWS(_xlpm.limbs_a), _xlpm.num_limbs_b, ROWS(_xlpm.limbs_b), _xlpm.convolution_length, _xlpm.num_limbs_a + _xlpm.num_limbs_b - 1, _xlpm.raw_convolution, _xlfn.MAKEARRAY(_xlpm.convolution_length, 1, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, _xlfn.LET(_xlpm.window_start_i, MAX(1, _xlpm.r - _xlpm.num_limbs_b + 1), _xlpm.window_end_i, MIN(_xlpm.r, _xlpm.num_limbs_a), _xlpm.overlap_rows, _xlpm.window_end_i - _xlpm.window_start_i + 1, _xlpm.seq_i, _xlfn.SEQUENCE(_xlpm.overlap_rows, 1, _xlpm.window_start_i, 1), _xlpm.seq_j, _xlfn.SEQUENCE(_xlpm.overlap_rows, 1, _xlpm.r - _xlpm.window_start_i + 1, -1), SUM(INDEX(_xlpm.limbs_a, _xlpm.seq_i, 1) * INDEX(_xlpm.limbs_b, _xlpm.seq_j, 1))))), core_BigInt.Carry(_xlpm.raw_convolution, _xlpm.k)))</definedName>
+    <definedName name="core_BigInt.UPow" comment="[Internal] Returns base^exponent using Left-to-Right evaluation and a 1-9 power cache._x000a_[limbs_base: Array, exponent_string: Text, k: int]">_xlfn.LAMBDA(_xlpm.limbs_base,_xlpm.exponent_string,_xlpm.k, _xlfn.LET(_xlpm.limbs_base1, _xlpm.limbs_base, _xlpm.limbs_base2, core_BigInt.UMul(_xlpm.limbs_base1, _xlpm.limbs_base1, _xlpm.k), _xlpm.limbs_base3, core_BigInt.UMul(_xlpm.limbs_base2, _xlpm.limbs_base1, _xlpm.k), _xlpm.limbs_base4, core_BigInt.UMul(_xlpm.limbs_base2, _xlpm.limbs_base2, _xlpm.k), _xlpm.limbs_base5, core_BigInt.UMul(_xlpm.limbs_base4, _xlpm.limbs_base1, _xlpm.k), _xlpm.limbs_base6, core_BigInt.UMul(_xlpm.limbs_base3, _xlpm.limbs_base3, _xlpm.k), _xlpm.limbs_base7, core_BigInt.UMul(_xlpm.limbs_base6, _xlpm.limbs_base1, _xlpm.k), _xlpm.limbs_base8, core_BigInt.UMul(_xlpm.limbs_base4, _xlpm.limbs_base4, _xlpm.k), _xlpm.limbs_base9, core_BigInt.UMul(_xlpm.limbs_base8, _xlpm.limbs_base1, _xlpm.k), _xlpm.exponent_digits, --MID(_xlpm.exponent_string, _xlfn.SEQUENCE(LEN(_xlpm.exponent_string)), 1), _xlfn.REDUCE(1, _xlpm.exponent_digits, _xlfn.LAMBDA(_xlpm.limbs_accumulator,_xlpm.current_digit, _xlfn.LET(_xlpm.is_one, AND(ROWS(_xlpm.limbs_accumulator) = 1, INDEX(_xlpm.limbs_accumulator, 1, 1) = 1), _xlpm.limbs_acc_10, IF(_xlpm.is_one, _xlpm.limbs_accumulator, _xlfn.LET(_xlpm.limbs_acc_2, core_BigInt.UMul(_xlpm.limbs_accumulator, _xlpm.limbs_accumulator, _xlpm.k), _xlpm.limbs_acc_4, core_BigInt.UMul(_xlpm.limbs_acc_2, _xlpm.limbs_acc_2, _xlpm.k), _xlpm.limbs_acc_8, core_BigInt.UMul(_xlpm.limbs_acc_4, _xlpm.limbs_acc_4, _xlpm.k), core_BigInt.UMul(_xlpm.limbs_acc_8, _xlpm.limbs_acc_2, _xlpm.k))), IF(_xlpm.current_digit = 0, _xlpm.limbs_acc_10, _xlfn.LET(_xlpm.limbs_cache_multiplier, CHOOSE(_xlpm.current_digit, _xlpm.limbs_base1, _xlpm.limbs_base2, _xlpm.limbs_base3, _xlpm.limbs_base4, _xlpm.limbs_base5, _xlpm.limbs_base6, _xlpm.limbs_base7, _xlpm.limbs_base8, _xlpm.limbs_base9), IF(_xlpm.is_one, _xlpm.limbs_cache_multiplier, core_BigInt.UMul(_xlpm.limbs_acc_10, _xlpm.limbs_cache_multiplier, _xlpm.k)))))))))</definedName>
+    <definedName name="core_BigInt.USqrt" comment="[Internal] Returns the integer square root of the radicand using Newton's Method._x000a_[limbs_radicand: Array, limbs_initial_x: Array, k: int]">_xlfn.LAMBDA(_xlpm.limbs_radicand,_xlpm.limbs_initial_x,_xlpm.k, _xlfn.LET(_xlpm.maximum_iterations, 35, _xlpm.final_packed_state, _xlfn.REDUCE(_xlfn.VSTACK(0, _xlpm.limbs_initial_x), _xlfn.SEQUENCE(_xlpm.maximum_iterations), _xlfn.LAMBDA(_xlpm.packed_state,_xlpm.i, _xlfn.LET(_xlpm.has_converged, INDEX(_xlpm.packed_state, 1, 1), _xlpm.limbs_current_x, _xlfn.DROP(_xlpm.packed_state, 1), IF(_xlpm.has_converged, _xlpm.packed_state, _xlfn.LET(_xlpm.packed_division_result, core_BigInt.DivRouter(_xlpm.limbs_radicand, _xlpm.limbs_current_x, _xlpm.k), _xlpm.num_limbs_r, INDEX(_xlpm.packed_division_result, 1, 1), _xlpm.limbs_q, _xlfn.DROP(_xlpm.packed_division_result, _xlpm.num_limbs_r + 1), _xlpm.limbs_sum_xq, core_BigInt.UAdd(_xlpm.limbs_current_x, _xlpm.limbs_q, _xlpm.k), _xlpm.packed_half_result, core_BigInt.KnuthDiv(_xlpm.limbs_sum_xq, {2}, _xlpm.k), _xlpm.num_limbs_halfed, INDEX(_xlpm.packed_half_result, 1, 1), _xlpm.limbs_next_x, _xlfn.DROP(_xlpm.packed_half_result, _xlpm.num_limbs_halfed + 1), _xlpm.convergence_comparison, core_BigInt.UCompare(_xlpm.limbs_next_x, _xlpm.limbs_current_x), IF(_xlpm.convergence_comparison &gt;= 0, _xlfn.VSTACK(1, _xlpm.limbs_current_x), _xlfn.VSTACK(0, _xlpm.limbs_next_x))))))), _xlfn.DROP(_xlpm.final_packed_state, 1)))</definedName>
+    <definedName name="core_BigInt.USub" comment="[Internal] Returns the difference of unsigned Little-Endian arrays (A - B). Assumes A &gt;= B._x000a_[limbs_a: Array, limbs_b: Array, k: int]">_xlfn.LAMBDA(_xlpm.limbs_a,_xlpm.limbs_b,_xlpm.k, _xlfn.LET(_xlpm.max_rows, MAX(ROWS(_xlpm.limbs_a), ROWS(_xlpm.limbs_b)), _xlpm.limbs_a_aligned, _xlfn.EXPAND(_xlpm.limbs_a, _xlpm.max_rows, 1, 0), _xlpm.limbs_b_aligned, _xlfn.EXPAND(_xlpm.limbs_b, _xlpm.max_rows, 1, 0), _xlpm.differences, _xlpm.limbs_a_aligned - _xlpm.limbs_b_aligned, _xlpm.carried_differences, core_BigInt.Carry(_xlpm.differences, _xlpm.k), _xlpm.highest_non_zero_index, _xlfn.XMATCH(TRUE, _xlpm.carried_differences &lt;&gt; 0, 0, -1), IF(ISNA(_xlpm.highest_non_zero_index), {0}, _xlfn.TAKE(_xlpm.carried_differences, _xlpm.highest_non_zero_index))))</definedName>
+    <definedName name="core_BigInt.UTextMul" comment="[Internal] High-performance multiplication of normalized positive strings. Bypasses Layer 0._x000a_[norm_a: Text, norm_b: Text]">_xlfn.LAMBDA(_xlpm.norm_a,_xlpm.norm_b, IF(OR(_xlpm.norm_a = "0", _xlpm.norm_b = "0"), "0", IF(_xlpm.norm_a = "1", _xlpm.norm_b, IF(_xlpm.norm_b = "1", _xlpm.norm_a, _xlfn.LET(_xlpm.len_a, LEN(_xlpm.norm_a), _xlpm.len_b, LEN(_xlpm.norm_b), _xlpm.k, core_BigInt.SafeK("MUL", MIN(_xlpm.len_a, _xlpm.len_b)), _xlpm.limbs_a, core_BigInt.Split(_xlpm.norm_a, _xlpm.k), _xlpm.limbs_b, core_BigInt.Split(_xlpm.norm_b, _xlpm.k), _xlpm.final_limbs, core_BigInt.UMul(_xlpm.limbs_a, _xlpm.limbs_b, _xlpm.k), core_BigInt.Merge(_xlpm.final_limbs, _xlpm.k))))))</definedName>
     <definedName name="test_BigInt.AsymmetricABGrid">_xlfn.LAMBDA(_xlpm.start_a,_xlpm.max_a,_xlpm.step_a,_xlpm.start_b,_xlpm.max_b,_xlpm.step_b, _xlfn.LET(_xlpm.seq_a, _xlfn.SEQUENCE((_xlpm.max_a - _xlpm.start_a) / _xlpm.step_a + 1, 1, _xlpm.start_a, _xlpm.step_a), _xlpm.seq_b, _xlfn.SEQUENCE((_xlpm.max_b - _xlpm.start_b) / _xlpm.step_b + 1, 1, _xlpm.start_b, _xlpm.step_b), _xlpm.n_a, ROWS(_xlpm.seq_a), _xlpm.n_b, ROWS(_xlpm.seq_b), _xlpm.col_a, _xlfn.TOCOL(IF(_xlfn.SEQUENCE(1, _xlpm.n_b), _xlpm.seq_a)), _xlpm.col_b, _xlfn.TOCOL(IF(_xlfn.SEQUENCE(_xlpm.n_a), _xlfn.TOROW(_xlpm.seq_b))), _xlfn.HSTACK(_xlpm.col_a, _xlpm.col_b)))</definedName>
     <definedName name="test_BigInt.DivisionAlgorithmComparison" comment="Executes a strictly sequential benchmark suite to avoid multi-threading contamination._x000a_@param test_cases An N x 2 array of test lengths: [Length_A, Length_B]_x000a_@param iters Number of iterations per benchmark to smooth NOW() resolution.">_xlfn.LAMBDA(_xlpm.test_cases,_xlpm.iters,_xlpm.repeats, _xlfn.LET(_xlpm.n_tests, ROWS(_xlpm.test_cases), _xlpm.initial, {"Len_A","Len_B","Knuth_ms","NR_ms"}, _xlfn.REDUCE(_xlpm.initial, _xlfn.SEQUENCE(_xlpm.n_tests), _xlfn.LAMBDA(_xlpm.acc,_xlpm.i, _xlfn.LET(_xlpm.len_a, INDEX(_xlpm.test_cases, _xlpm.i, 1), _xlpm.len_b, INDEX(_xlpm.test_cases, _xlpm.i, 2), IF(_xlpm.len_b &gt; _xlpm.len_a, _xlpm.acc, _xlfn.LET(_xlpm.str_a, REPT("9", _xlpm.len_a), _xlpm.str_b, IF(_xlpm.len_b = 1, "7", "7" &amp; REPT("3", _xlpm.len_b - 1)), _xlpm.time_k, test_BigInt.DivisionAlgorithms(_xlpm.str_a, _xlpm.str_b, "KNUTH", _xlpm.iters, _xlpm.repeats), _xlpm.time_nr, test_BigInt.DivisionAlgorithms(_xlpm.str_a, _xlpm.str_b, "NR", _xlpm.iters, _xlpm.repeats), _xlfn.VSTACK(_xlpm.acc, _xlfn.HSTACK(_xlpm.len_a, _xlpm.len_b, _xlpm.time_k, _xlpm.time_nr)))))))))</definedName>
     <definedName name="test_BigInt.DivisionAlgorithms" comment="@param a The dividend string_x000a_@param b The divisor string_x000a_@param mode &quot;KNUTH&quot; or &quot;NR&quot;_x000a_@param iters Inner loop count (to defeat chunky clock resolution)_x000a_@param repeats Outer loop count (to defeat OS/Garbage Collection noise)">_xlfn.LAMBDA(_xlpm.a,_xlpm.b,_xlpm.mode,_xlpm.iters,_xlpm.repeats, _xlfn.LET(_xlpm.batch_times, _xlfn.MAP(_xlfn.SEQUENCE(_xlpm.repeats), _xlfn.LAMBDA(_xlpm.r, _xlfn.LET(_xlpm.start, NOW(), _xlpm.run, IF(_xlpm.mode = "KNUTH", _xlfn.MAP(_xlfn.SEQUENCE(_xlpm.iters), _xlfn.LAMBDA(_xlpm.i, test_BigInt.KnuthDivision(_xlpm.a, _xlpm.b))), _xlfn.MAP(_xlfn.SEQUENCE(_xlpm.iters), _xlfn.LAMBDA(_xlpm.i, test_BigInt.NewtonRaphsonDivision(_xlpm.a, _xlpm.b)))), _xlpm.stop, NOW() + (0 * LEN(INDEX(_xlpm.run, 1, 1))), (_xlpm.stop - _xlpm.start) * 86400000))), MIN(_xlpm.batch_times) / _xlpm.iters))</definedName>
@@ -12235,7 +12235,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="1659" row="6">
+  <wetp:taskpane dockstate="right" visibility="0" width="1936" row="6">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -21597,7 +21597,7 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAHQAZQBzAHQAXwBCAGkAZwBJAG4AdAAiACwAIgB0AGUAeAB0ACIAOgAiAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAFwAbgAvAC8AIABCAGkAZwAgAEkAbgB0AGUAZwBlAHIAIABBAHIAaQB0AGgAbQBlAHQAaQBjACAATABpAGIAcgBhAHIAeQAgAC8ALwBcAG4ALwAvACAAIAAgACAAIAAgACAAdABlAHMAdABfAEIAaQBnAEkAbgB0ACAATQBvAGQAdQBsAGUAIAAgACAAIAAgACAAIAAvAC8AXABuAC8ALwAgACAAIAAgACAAIAAgAFAAcgBpAHYAYQB0AGUAIABUAGUAcwB0AGkAbgBnACAAQQBQAEkAIAAgACAAIAAgACAALwAvAFwAbgAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwBcAG4AXABuAEsAbgB1AHQAaABEAGkAdgBpAHMAaQBvAG4APQBMAEEATQBCAEQAQQAoAGEALAAgAGIALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAawAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwBhAGYAZQBLACgAXAAiAEQASQBWAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABwAGEAYwBrAGUAZAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4ASwBuAHUAdABoAEQAaQB2ACgAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwBwAGwAaQB0ACgAYQAsACAAawApACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBTAHAAbABpAHQAKABiACwAIABrACkALAAgAGsAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAE0AZQByAGcAZQAoAEQAUgBPAFAAKABwAGEAYwBrAGUAZAAsACAASQBOAEQARQBYACgAcABhAGMAawBlAGQALAAgADEALAAgADEAKQAgACsAIAAxACkALAAgAGsAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBOAGUAdwB0AG8AbgBSAGEAcABoAHMAbwBuAEQAaQB2AGkAcwBpAG8AbgAgAD0AIABMAEEATQBCAEQAQQAoAGEALAAgAGIALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAawAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwBhAGYAZQBLACgAXAAiAEQASQBWAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABwAGEAYwBrAGUAZAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4ATgBlAHcAdABvAG4AUgBhAHAAaABzAG8AbgBEAGkAdgAoAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFMAcABsAGkAdAAoAGEALAAgAGsAKQAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwBwAGwAaQB0ACgAYgAsACAAawApACwAIABrACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBNAGUAcgBnAGUAKABEAFIATwBQACgAcABhAGMAawBlAGQALAAgAEkATgBEAEUAWAAoAHAAYQBjAGsAZQBkACwAIAAxACwAIAAxACkAIAArACAAMQApACwAIABrACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAEAAcABhAHIAYQBtACAAYQAgAFQAaABlACAAZABpAHYAaQBkAGUAbgBkACAAcwB0AHIAaQBuAGcAXABuACAAKgAgAEAAcABhAHIAYQBtACAAYgAgAFQAaABlACAAZABpAHYAaQBzAG8AcgAgAHMAdAByAGkAbgBnAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAG0AbwBkAGUAIABcACIASwBOAFUAVABIAFwAIgAgAG8AcgAgAFwAIgBOAFIAXAAiAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGkAdABlAHIAcwAgAEkAbgBuAGUAcgAgAGwAbwBvAHAAIABjAG8AdQBuAHQAIAAoAHQAbwAgAGQAZQBmAGUAYQB0ACAAYwBoAHUAbgBrAHkAIABjAGwAbwBjAGsAIAByAGUAcwBvAGwAdQB0AGkAbwBuACkAXABuACAAKgAgAEAAcABhAHIAYQBtACAAcgBlAHAAZQBhAHQAcwAgAE8AdQB0AGUAcgAgAGwAbwBvAHAAIABjAG8AdQBuAHQAIAAoAHQAbwAgAGQAZQBmAGUAYQB0ACAATwBTAC8ARwBhAHIAYgBhAGcAZQAgAEMAbwBsAGwAZQBjAHQAaQBvAG4AIABuAG8AaQBzAGUAKQBcAG4AIAAqAC8AXABuAEQAaQB2AGkAcwBpAG8AbgBBAGwAZwBvAHIAaQB0AGgAbQBzACAAPQAgAEwAQQBNAEIARABBACgAYQAsACAAYgAsACAAbQBvAGQAZQAsACAAaQB0AGUAcgBzACwAIAByAGUAcABlAGEAdABzACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAC8ALwAgAE0AYQBwACAAdABoAGUAIABvAHUAdABlAHIAIAByAGUAcABlAGEAdABzACAAbABvAG8AcABcAG4AIAAgACAAIAAgACAAIAAgAGIAYQB0AGMAaABfAHQAaQBtAGUAcwAsACAATQBBAFAAKABTAEUAUQBVAEUATgBDAEUAKAByAGUAcABlAGEAdABzACkALAAgAEwAQQBNAEIARABBACgAcgAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHMAdABhAHIAdAAsACAATgBPAFcAKAApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAATQBhAHAAIAB0AGgAZQAgAGkAbgBuAGUAcgAgAGUAeABlAGMAdQB0AGkAbwBuACAAbABvAG8AcABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAByAHUAbgAsACAASQBGACgAbQBvAGQAZQAgAD0AIABcACIASwBOAFUAVABIAFwAIgAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAE0AQQBQACgAUwBFAFEAVQBFAE4AQwBFACgAaQB0AGUAcgBzACkALAAgAEwAQQBNAEIARABBACgAaQAsACAASwBuAHUAdABoAEQAaQB2AGkAcwBpAG8AbgAoAGEALAAgAGIAKQApACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBBAFAAKABTAEUAUQBVAEUATgBDAEUAKABpAHQAZQByAHMAKQAsACAATABBAE0AQgBEAEEAKABpACwAIABOAGUAdwB0AG8AbgBSAGEAcABoAHMAbwBuAEQAaQB2AGkAcwBpAG8AbgAoAGEALAAgAGIAKQApACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAEYAbwByAGMAZQAgAGUAdgBhAGwAdQBhAHQAaQBvAG4AIABiAGUAZgBvAHIAZQAgAHAAdQBsAGwAaQBuAGcAIABzAHQAbwBwACAAdABpAG0AZQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABzAHQAbwBwACwAIABOAE8AVwAoACkAIAArACAAKAAwACAAKgAgAEwARQBOACgASQBOAEQARQBYACgAcgB1AG4ALAAgADEALAAgADEAKQApACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIABUAG8AdABhAGwAIABiAGEAdABjAGgAIAB0AGkAbQBlACAAaQBuACAAbQBpAGwAbABpAHMAZQBjAG8AbgBkAHMAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABzAHQAbwBwACAALQAgAHMAdABhAHIAdAApACAAKgAgADgANgA0ADAAMAAwADAAMABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABFAHgAdAByAGEAYwB0ACAAdABoAGUAIABjAGwAZQBhAG4AZQBzAHQAIAByAHUAbgAgAGEAbgBkACAAYQB2AGUAcgBhAGcAZQAgAGkAdAAgAGQAbwB3AG4AIAB0AG8AIABhACAAcwBpAG4AZwBsAGUAIABlAHgAZQBjAHUAdABpAG8AbgAgAHQAaQBtAGUAXABuACAAIAAgACAAIAAgACAAIABNAEkATgAoAGIAYQB0AGMAaABfAHQAaQBtAGUAcwApACAALwAgAGkAdABlAHIAcwBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAARQB4AGUAYwB1AHQAZQBzACAAYQAgAHMAdAByAGkAYwB0AGwAeQAgAHMAZQBxAHUAZQBuAHQAaQBhAGwAIABiAGUAbgBjAGgAbQBhAHIAawAgAHMAdQBpAHQAZQAgAHQAbwAgAGEAdgBvAGkAZAAgAG0AdQBsAHQAaQAtAHQAaAByAGUAYQBkAGkAbgBnACAAYwBvAG4AdABhAG0AaQBuAGEAdABpAG8AbgAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAHQAZQBzAHQAXwBjAGEAcwBlAHMAIABBAG4AIABOACAAeAAgADIAIABhAHIAcgBhAHkAIABvAGYAIAB0AGUAcwB0ACAAbABlAG4AZwB0AGgAcwA6ACAAWwBMAGUAbgBnAHQAaABfAEEALAAgAEwAZQBuAGcAdABoAF8AQgBdAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGkAdABlAHIAcwAgAE4AdQBtAGIAZQByACAAbwBmACAAaQB0AGUAcgBhAHQAaQBvAG4AcwAgAHAAZQByACAAYgBlAG4AYwBoAG0AYQByAGsAIAB0AG8AIABzAG0AbwBvAHQAaAAgAE4ATwBXACgAKQAgAHIAZQBzAG8AbAB1AHQAaQBvAG4ALgBcAG4AIAAqAC8AXABuAEQAaQB2AGkAcwBpAG8AbgBBAGwAZwBvAHIAaQB0AGgAbQBDAG8AbQBwAGEAcgBpAHMAbwBuACAAPQAgAEwAQQBNAEIARABBACgAdABlAHMAdABfAGMAYQBzAGUAcwAsACAAaQB0AGUAcgBzACwAIAByAGUAcABlAGEAdABzACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG4AXwB0AGUAcwB0AHMALAAgAFIATwBXAFMAKAB0AGUAcwB0AF8AYwBhAHMAZQBzACkALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAALwAvACAASQBuAGkAdABpAGEAbAAgAHMAdABhAHQAZQA6ACAARABhAHQAYQAgAGgAZQBhAGQAZQByAHMAIABmAG8AcgAgAEMAUwBWACAAZQB4AHAAbwByAHQAXABuACAAIAAgACAAIAAgACAAIABpAG4AaQB0AGkAYQBsACwAIAB7AFwAIgBMAGUAbgBfAEEAXAAiACwAIABcACIATABlAG4AXwBCAFwAIgAsACAAXAAiAEsAbgB1AHQAaABfAG0AcwBcACIALAAgAFwAIgBOAFIAXwBtAHMAXAAiAH0ALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAUgBFAEQAVQBDAEUAKABpAG4AaQB0AGkAYQBsACwAIABTAEUAUQBVAEUATgBDAEUAKABuAF8AdABlAHMAdABzACkALAAgAEwAQQBNAEIARABBACgAYQBjAGMALAAgAGkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGUAbgBfAGEALAAgAEkATgBEAEUAWAAoAHQAZQBzAHQAXwBjAGEAcwBlAHMALAAgAGkALAAgADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAZQBuAF8AYgAsACAASQBOAEQARQBYACgAdABlAHMAdABfAGMAYQBzAGUAcwAsACAAaQAsACAAMgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAAUwBrAGkAcAAgAEQAaQB2AGkAcwBvAHIAIAA+ACAARABpAHYAaQBkAGUAbgBkABQgaQB0ACcAcwAgAG4AZQB2AGUAcgAgAGEAbgAgAGkAbgB0AGUAZwBlAHIAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgAbABlAG4AXwBiACAAPgAgAGwAZQBuAF8AYQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABhAGMAYwAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAARwBlAG4AZQByAGEAdABlACAAZQB4AGEAYwB0AC0AbABlAG4AZwB0AGgAIAB0AGUAcwB0ACAAcwB0AHIAaQBuAGcAcwAgAG4AYQB0AGkAdgBlAGwAeQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcwB0AHIAXwBhACwAIABSAEUAUABUACgAXAAiADkAXAAiACwAIABsAGUAbgBfAGEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABzAHQAcgBfAGIALAAgAEkARgAoAGwAZQBuAF8AYgAgAD0AIAAxACwAIABcACIANwBcACIALAAgAFwAIgA3AFwAIgAgACYAIABSAEUAUABUACgAXAAiADMAXAAiACwAIABsAGUAbgBfAGIAIAAtACAAMQApACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAEUAeABlAGMAdQB0AGUAIABiAGUAbgBjAGgAbQBhAHIAawBzACAAcwB0AHIAaQBjAHQAbAB5ACAAbwBuAGUAIABhAGYAdABlAHIAIAB0AGgAZQAgAG8AdABoAGUAcgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAdABpAG0AZQBfAGsALAAgAEQAaQB2AGkAcwBpAG8AbgBBAGwAZwBvAHIAaQB0AGgAbQBzACgAcwB0AHIAXwBhACwAIABzAHQAcgBfAGIALAAgAFwAIgBLAE4AVQBUAEgAXAAiACwAIABpAHQAZQByAHMALAAgAHIAZQBwAGUAYQB0AHMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAB0AGkAbQBlAF8AbgByACwAIABEAGkAdgBpAHMAaQBvAG4AQQBsAGcAbwByAGkAdABoAG0AcwAoAHMAdAByAF8AYQAsACAAcwB0AHIAXwBiACwAIABcACIATgBSAFwAIgAsACAAaQB0AGUAcgBzACwAIAByAGUAcABlAGEAdABzACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAEEAcABwAGUAbgBkACAAdABoAGUAIAByAGUAcwB1AGwAdABzAC4AIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAAUgBlAGEAbABsAG8AYwBhAHQAaQBvAG4AIABkAGUAbABhAHkAIABvAGMAYwB1AHIAcwAgAGgAZQByAGUALAAgAHMAYQBmAGUAbAB5ACAAbwB1AHQAcwBpAGQAZQAgAHQAaABlACAAdABpAG0AZQBkACAAdwBpAG4AZABvAHcALgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAVgBTAFQAQQBDAEsAKABhAGMAYwAsACAASABTAFQAQQBDAEsAKABsAGUAbgBfAGEALAAgAGwAZQBuAF8AYgAsACAAdABpAG0AZQBfAGsALAAgAHQAaQBtAGUAXwBuAHIAKQApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8ALwAgAEcAZQBuAGUAcgBhAHQAZQBzACAAYQAgADIALQBjAG8AbAB1AG0AbgAgAGEAcgByAGEAeQAgAG8AZgAgAGUAdgBlAHIAeQAgAGMAbwBtAGIAaQBuAGEAdABpAG8AbgAgAG8AZgAgAGwAZQBuAGcAdABoAHMAXABuAEQAaQB2AGkAcwBpAG8AbgBCAGUAbgBjAGgAbQBhAHIAawBDAGEAcwBlAHMAIAA9ACAATABBAE0AQgBEAEEAKABzAHQAYQByAHQAXwBsAGUAbgAsACAAbQBhAHgAXwBsAGUAbgAsACAAcwB0AGUAcAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABzAGUAcQAsACAAUwBFAFEAVQBFAE4AQwBFACgAKABtAGEAeABfAGwAZQBuACAALQAgAHMAdABhAHIAdABfAGwAZQBuACkAIAAvACAAcwB0AGUAcAAgACsAIAAxACwAIAAxACwAIABzAHQAYQByAHQAXwBsAGUAbgAsACAAcwB0AGUAcAApACwAXABuACAAIAAgACAAIAAgACAAIABuACwAIABSAE8AVwBTACgAcwBlAHEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABDAGEAcgB0AGUAcwBpAGEAbgAgAEoAbwBpAG4AXABuACAAIAAgACAAIAAgACAAIABjAG8AbABfAGEALAAgAFQATwBDAE8ATAAoAEkARgAoAFMARQBRAFUARQBOAEMARQAoADEALAAgAG4AKQAsACAAcwBlAHEAKQApACwAXABuACAAIAAgACAAIAAgACAAIABjAG8AbABfAGIALAAgAFQATwBDAE8ATAAoAEkARgAoAFMARQBRAFUARQBOAEMARQAoAG4ALAAgADEAKQAsACAAVABPAFIATwBXACgAcwBlAHEAKQApACkALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAASABTAFQAQQBDAEsAKABjAG8AbABfAGEALAAgAGMAbwBsAF8AYgApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8ALwAgAEcAZQBuAGUAcgBhAHQAZQBzACAAYQAgAEMAYQByAHQAZQBzAGkAYQBuACAAZwByAGkAZAAgAGYAcgBvAG0AIAB0AHcAbwAgAGkAbgBkAGUAcABlAG4AZABlAG4AdAAgAHMAZQBxAHUAZQBuAGMAZQBzAFwAbgBBAHMAeQBtAG0AZQB0AHIAaQBjAEEAQgBHAHIAaQBkACAAPQAgAEwAQQBNAEIARABBACgAcwB0AGEAcgB0AF8AYQAsACAAbQBhAHgAXwBhACwAIABzAHQAZQBwAF8AYQAsACAAcwB0AGEAcgB0AF8AYgAsACAAbQBhAHgAXwBiACwAIABzAHQAZQBwAF8AYgAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABzAGUAcQBfAGEALAAgAFMARQBRAFUARQBOAEMARQAoACgAbQBhAHgAXwBhACAALQAgAHMAdABhAHIAdABfAGEAKQAgAC8AIABzAHQAZQBwAF8AYQAgACsAIAAxACwAIAAxACwAIABzAHQAYQByAHQAXwBhACwAIABzAHQAZQBwAF8AYQApACwAXABuACAAIAAgACAAIAAgACAAIABzAGUAcQBfAGIALAAgAFMARQBRAFUARQBOAEMARQAoACgAbQBhAHgAXwBiACAALQAgAHMAdABhAHIAdABfAGIAKQAgAC8AIABzAHQAZQBwAF8AYgAgACsAIAAxACwAIAAxACwAIABzAHQAYQByAHQAXwBiACwAIABzAHQAZQBwAF8AYgApACwAXABuACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgAG4AXwBhACwAIABSAE8AVwBTACgAcwBlAHEAXwBhACkALABcAG4AIAAgACAAIAAgACAAIAAgAG4AXwBiACwAIABSAE8AVwBTACgAcwBlAHEAXwBiACkALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAALwAvACAATwByAHQAaABvAGcAbwBuAGEAbAAgAGIAcgBvAGEAZABjAGEAcwB0ACAAdQBzAGkAbgBnACAAaQBuAGQAZQBwAGUAbgBkAGUAbgB0ACAAZABpAG0AZQBuAHMAaQBvAG4AcwBcAG4AIAAgACAAIAAgACAAIAAgAGMAbwBsAF8AYQAsACAAVABPAEMATwBMACgASQBGACgAUwBFAFEAVQBFAE4AQwBFACgAMQAsACAAbgBfAGIAKQAsACAAcwBlAHEAXwBhACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAYwBvAGwAXwBiACwAIABUAE8AQwBPAEwAKABJAEYAKABTAEUAUQBVAEUATgBDAEUAKABuAF8AYQApACwAIABUAE8AUgBPAFcAKABzAGUAcQBfAGIAKQApACkALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAASABTAFQAQQBDAEsAKABjAG8AbABfAGEALAAgAGMAbwBsAF8AYgApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAEYAYQBjAHQAbwByAGkAYQBsAEEAbABnAG8AcgBpAHQAaABtAHMAIAA9ACAATABBAE0AQgBEAEEAKABpAG4AcAB1AHQALAAgAG0AbwBkAGUALAAgAGkAdABlAHIAcwAsACAAcgBlAHAAZQBhAHQAcwAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABNAGEAcAAgAHQAaABlACAAbwB1AHQAZQByACAAcgBlAHAAZQBhAHQAcwAgAGwAbwBvAHAAXABuACAAIAAgACAAIAAgACAAIABiAGEAdABjAGgAXwB0AGkAbQBlAHMALAAgAE0AQQBQACgAUwBFAFEAVQBFAE4AQwBFACgAcgBlAHAAZQBhAHQAcwApACwAIABMAEEATQBCAEQAQQAoAHIALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQALAAgAE4ATwBXACgAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAE0AYQBwACAAdABoAGUAIABpAG4AbgBlAHIAIABlAHgAZQBjAHUAdABpAG8AbgAgAGwAbwBvAHAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcgB1AG4ALAAgAEkARgAoAG0AbwBkAGUAIAA9ACAAXAAiAEwAZQBnAGUAbgBkAHIAZQBcACIALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEEAUAAoAFMARQBRAFUARQBOAEMARQAoAGkAdABlAHIAcwApACwAIABMAEEATQBCAEQAQQAoAGkALAAgAEIAaQBnAEkAbgB0AC4ARgBhAGMAdAAoAGkAbgBwAHUAdAApACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEEAUAAoAFMARQBRAFUARQBOAEMARQAoAGkAdABlAHIAcwApACwAIABMAEEATQBCAEQAQQAoAGkALAAgAEIAaQBnAEkAbgB0AC4ARgBhAGMAdABTAHcAaQBuAGcAKABpAG4AcAB1AHQAKQApACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAEYAbwByAGMAZQAgAGUAdgBhAGwAdQBhAHQAaQBvAG4AIABiAGUAZgBvAHIAZQAgAHAAdQBsAGwAaQBuAGcAIABzAHQAbwBwACAAdABpAG0AZQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABzAHQAbwBwACwAIABOAE8AVwAoACkAIAArACAAKAAwACAAKgAgAEwARQBOACgASQBOAEQARQBYACgAcgB1AG4ALAAgADEALAAgADEAKQApACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIABUAG8AdABhAGwAIABiAGEAdABjAGgAIAB0AGkAbQBlACAAaQBuACAAbQBpAGwAbABpAHMAZQBjAG8AbgBkAHMAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABzAHQAbwBwACAALQAgAHMAdABhAHIAdAApACAAKgAgADgANgA0ADAAMAAwADAAMABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABFAHgAdAByAGEAYwB0ACAAdABoAGUAIABjAGwAZQBhAG4AZQBzAHQAIAByAHUAbgAgAGEAbgBkACAAYQB2AGUAcgBhAGcAZQAgAGkAdAAgAGQAbwB3AG4AIAB0AG8AIABhACAAcwBpAG4AZwBsAGUAIABlAHgAZQBjAHUAdABpAG8AbgAgAHQAaQBtAGUAXABuACAAIAAgACAAIAAgACAAIABNAEkATgAoAGIAYQB0AGMAaABfAHQAaQBtAGUAcwApACAALwAgAGkAdABlAHIAcwBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAARQB4AGUAYwB1AHQAZQBzACAAYQAgAHMAdAByAGkAYwB0AGwAeQAgAHMAZQBxAHUAZQBuAHQAaQBhAGwAIABiAGUAbgBjAGgAbQBhAHIAawAgAHMAdQBpAHQAZQAgAHQAbwAgAGEAdgBvAGkAZAAgAG0AdQBsAHQAaQAtAHQAaAByAGUAYQBkAGkAbgBnACAAYwBvAG4AdABhAG0AaQBuAGEAdABpAG8AbgAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAHQAZQBzAHQAXwBjAGEAcwBlAHMAIABBAG4AIABOACAAeAAgADEAIABhAHIAcgBhAHkAIABvAGYAIAB0AGUAcwB0ACAAaQBuAHAAdQB0AHMAXABuACAAKgAgAEAAcABhAHIAYQBtACAAaQB0AGUAcgBzACAATgB1AG0AYgBlAHIAIABvAGYAIABpAHQAZQByAGEAdABpAG8AbgBzACAAcABlAHIAIABzAGEAbQBwAGwAZQAgAHQAbwAgAHMAbQBvAG8AdABoACAATgBPAFcAKAApACAAcgBlAHMAbwBsAHUAdABpAG8AbgAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAHIAZQBwAGUAYQB0AHMAIABOAHUAbQBiAGUAcgAgAG8AZgAgAGkAdABlAHIAYQB0AGkAbwBuAHMAIABwAGUAcgAgAGIAZQBuAGMAaABtAGEAcgBrACAAdABvACAAcwBtAG8AbwB0AGgAIABPAFMAIABhAG4AZAAgAGIAYQBjAGsAZwByAG8AdQBuAGQAIABuAG8AaQBzAGUALgBcAG4AIAAqAC8AXABuAEYAYQBjAHQAbwByAGkAYQBsAEMAbwBtAHAAYQByAGkAcwBvAG4AIAA9ACAATABBAE0AQgBEAEEAKAB0AGUAcwB0AF8AYwBhAHMAZQBzACwAIABpAHQAZQByAHMALAAgAHIAZQBwAGUAYQB0AHMALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbgBfAHQAZQBzAHQAcwAsACAAUgBPAFcAUwAoAHQAZQBzAHQAXwBjAGEAcwBlAHMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABJAG4AaQB0AGkAYQBsACAAcwB0AGEAdABlADoAIABEAGEAdABhACAAaABlAGEAZABlAHIAcwAgAGYAbwByACAAQwBTAFYAIABlAHgAcABvAHIAdABcAG4AIAAgACAAIAAgACAAIAAgAGkAbgBpAHQAaQBhAGwALAAgAHsAXAAiAE4AXAAiACwAIABcACIATABlAGcAZQBuAGQAcgBlAFwAIgAsACAAXAAiAFMAdwBpAG4AZwBcACIAfQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIABSAEUARABVAEMARQAoAGkAbgBpAHQAaQBhAGwALAAgAFMARQBRAFUARQBOAEMARQAoAG4AXwB0AGUAcwB0AHMAKQAsACAATABBAE0AQgBEAEEAKABhAGMAYwAsACAAaQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGkAbgBwAHUAdAAsACAASQBOAEQARQBYACgAdABlAHMAdABfAGMAYQBzAGUAcwAsACAAaQAsACAAMQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAARQB4AGUAYwB1AHQAZQAgAGIAZQBuAGMAaABtAGEAcgBrAHMAIABzAHQAcgBpAGMAdABsAHkAIABvAG4AZQAgAGEAZgB0AGUAcgAgAHQAaABlACAAbwB0AGgAZQByAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHQAaQBtAGUAXwBsAGUAZwBlAG4AZAByAGUALAAgAEYAYQBjAHQAbwByAGkAYQBsAEEAbABnAG8AcgBpAHQAaABtAHMAKABpAG4AcAB1AHQALAAgAFwAIgBMAGUAZwBlAG4AZAByAGUAXAAiACwAIABpAHQAZQByAHMALAAgAHIAZQBwAGUAYQB0AHMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHQAaQBtAGUAXwBzAHcAaQBuAGcALAAgAEYAYQBjAHQAbwByAGkAYQBsAEEAbABnAG8AcgBpAHQAaABtAHMAKABpAG4AcAB1AHQALAAgAFwAIgBTAHcAaQBuAGcAXAAiACwAIABpAHQAZQByAHMALAAgAHIAZQBwAGUAYQB0AHMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAEEAcABwAGUAbgBkACAAdABoAGUAIAByAGUAcwB1AGwAdABzAC4AIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIABSAGUAYQBsAGwAbwBjAGEAdABpAG8AbgAgAGQAZQBsAGEAeQAgAG8AYwBjAHUAcgBzACAAaABlAHIAZQAsACAAcwBhAGYAZQBsAHkAIABvAHUAdABzAGkAZABlACAAdABoAGUAIAB0AGkAbQBlAGQAIAB3AGkAbgBkAG8AdwAuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFYAUwBUAEEAQwBLACgAYQBjAGMALAAgAEgAUwBUAEEAQwBLACgAaQBuAHAAdQB0ACwAIAB0AGkAbQBlAF8AbABlAGcAZQBuAGQAcgBlACwAIAB0AGkAbQBlAF8AcwB3AGkAbgBnACkAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBjAG8AcgBlAF8AQgBpAGcASQBuAHQAIgAsACIAdABlAHgAdAAiADoAIgAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwBcAG4ALwAvACAAQgBpAGcAIABJAG4AdABlAGcAZQByACAAQQByAGkAdABoAG0AZQB0AGkAYwAgAEwAaQBiAHIAYQByAHkAIAAvAC8AXABuAC8ALwAgACAAIAAgACAAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQAIABNAG8AZAB1AGwAZQAgACAAIAAgACAAIAAgACAALwAvAFwAbgAvAC8AIAAgACAAIAAgACAAIAAgACAAIABQAHIAaQB2AGEAdABlACAAQQBQAEkAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwBcAG4ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8AXABuAFwAbgAvACoAKgBcAG4AIAAqACAAWwBJAG4AdABlAHIAbgBhAGwAXQAgAEMAbwBtAHAAdQB0AGUAcwAgAHQAaABlACAAbQBhAHgAaQBtAHUAbQAgAHMAYQBmAGUAIABiAGEAcwBlAC0AMQAwACAAbABpAG0AYgAgAHMAaQB6AGUAIAAoAGsAKQAgAHQAbwAgAGEAdgBvAGkAZAAgAEkARQBFAEUALQA3ADUANAAgAHAAcgBlAGMAaQBzAGkAbwBuACAAbABvAHMAcwAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAG8AcABlAHIAYQB0AGkAbwBuADoAIABcACIAQQBEAEQAXAAiACwAIABcACIATQBVAEwAXAAiACwAIABvAHIAIABcACIARABJAFYAXAAiAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAWwBtAGEAeABfAGkAdABlAG0AcwBdACAAQQBEAEQAOgAgAG4AdQBtAGIAZQByACAAbwBmACAAbwBwAGUAcgBhAG4AZABzAC4AIABNAFUATAA6ACAAcwBoAG8AcgB0AGUAcwB0ACAAcwB0AHIAaQBuAGcAIABkAGkAZwBpAHQAcwAgAGMAbwB1AG4AdAAuAFwAbgAgACoALwBcAG4AUwBhAGYAZQBLACAAPQAgAEwAQQBNAEIARABBACgAbwBwAGUAcgBhAHQAaQBvAG4ALAAgAFsAbwBwAGUAcgBhAG4AZABfAG8AcgBfAGQAaQBnAGkAdABzAF0ALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAcgBlAHMAbwBsAHYAZQBkAF8AYwBvAHUAbgB0ACwAIABJAEYAKABPAFIAKABvAHAAZQByAGEAbgBkAF8AbwByAF8AZABpAGcAaQB0AHMAIAA9ACAAXAAiAFwAIgAsACAASQBTAE8ATQBJAFQAVABFAEQAKABvAHAAZQByAGEAbgBkAF8AbwByAF8AZABpAGcAaQB0AHMAKQApACwAIAAyACwAIABNAEEAWAAoADIALAAgAG8AcABlAHIAYQBuAGQAXwBvAHIAXwBkAGkAZwBpAHQAcwApACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIABTAFcASQBUAEMASAAoAG8AcABlAHIAYQB0AGkAbwBuACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAEQARABcACIALAAgADEANQAgAC0AIABMAEUATgAoAHIAZQBzAG8AbAB2AGUAZABfAGMAbwB1AG4AdAApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIATQBVAEwAXAAiACwAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHQAZQBzAHQAXwBrACwAIAB7ADcAOwAgADYAOwAgADUAOwAgADQAOwAgADMAOwAgADIAOwAgADEAfQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAG0AYQB4AF8AbwB2AGUAcgBsAGEAcAAsACAAUgBPAFUATgBEAFUAUAAoAHIAZQBzAG8AbAB2AGUAZABfAGMAbwB1AG4AdAAgAC8AIAB0AGUAcwB0AF8AawAsACAAMAApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAAQwBhAGwAYwB1AGwAYQB0AGUAIAB0AGgAZQAgAGEAYgBzAG8AbAB1AHQAZQAgAHAAZQBhAGsAIAB2AGEAbAB1AGUAIABpAG4AcwBpAGQAZQAgAHQAaABlACAAZQBuAGcAaQBuAGUAIAAoAEMAbwBuAHYAbwBsAHUAdABpAG8AbgAgACsAIABDAGEAcgByAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAB1AG4AYwBhAHIAcgBpAGUAZABfAG0AYQB4ACwAIABtAGEAeABfAG8AdgBlAHIAbABhAHAAIAAqACAAKAAxADAAXgB0AGUAcwB0AF8AawAgAC0AIAAxACkAXgAyACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbQBhAHgAXwBjAGEAcgByAHkALAAgAEkATgBUACgAdQBuAGMAYQByAHIAaQBlAGQAXwBtAGEAeAAgAC8AIAAxADAAXgB0AGUAcwB0AF8AawApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcABlAGEAawBfAHYAYQBsACwAIAB1AG4AYwBhAHIAcgBpAGUAZABfAG0AYQB4ACAAKwAgAG0AYQB4AF8AYwBhAHIAcgB5ACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAAUgBlAHQAdQByAG4AIAB0AGgAZQAgAG0AYQB4ACAAawAgADwAPQAgAEUAeABjAGUAbAAnAHMAIAAxADUALQBkAGkAZwBpAHQAIABjAGUAaQBsAGkAbgBnAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAE0AQQBYACgARgBJAEwAVABFAFIAKAB0AGUAcwB0AF8AawAsACAAcABlAGEAawBfAHYAYQBsACAAPAA9ACAAKAAxADAAXgAxADUAIAAtACAAMQApACkAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQASQBWAFwAIgAsACAANwAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAjAE4AQQBNAEUAPwBcAG4AIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFsASQBuAHQAZQByAG4AYQBsAF0AIABVAG4AaQBmAGkAZQBkACAAUwBwAGwAaQB0AHQAZQByAC4AIABTAHAAbABpAHQAcwAgAGIAbwB0AGgAIABzAGMAYQBsAGEAcgBzACAAYQBuAGQAIABhAHIAcgBhAHkAcwAgAGkAbgB0AG8AIABMAGkAdAB0AGwAZQAtAEUAbgBkAGkAYQBuACAAbABpAG0AYgBzAC4AXABuACAAKgAgAFUAcwBlAHMAIABNAEEAWAAoACkAIAB0AG8AIABnAHUAYQByAGEAbgB0AGUAZQAgAHMAYwBhAGwAYQByACAAaQBuAHAAdQB0AHMAIAB0AG8AIAB0AGgAZQAgAFMARQBRAFUARQBOAEMARQAgAGUAbgBnAGkAbgBlAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAYgBpAGcAXwBpAG4AdABzACAAVABoAGUAIABzAHQAcgBpAG4AZwAgAG8AcgAgAGEAcgByAGEAeQAgAG8AZgAgAHMAdAByAGkAbgBnAHMALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABrACAAVABoAGUAIABkAHkAbgBhAG0AaQBjACAAYwBoAHUAbgBrACAAcwBpAHoAZQAgAGMAbwBuAHQAZQB4AHQALgBcAG4AIAAqAC8AXABuAFMAcABsAGkAdAAgAD0AIABMAEEATQBCAEQAQQAoAHMAdAByAF8AbgBvAHIAbQBzACwAIABrACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAGYAbABhAHQAdABlAG4AZQBkAF8AbgBvAHIAbQBzACwAIABUAE8AUgBPAFcAKABzAHQAcgBfAG4AbwByAG0AcwApACwAXABuACAAIAAgACAAIAAgACAAIABsAGUAbgBnAHQAaABzACwAIABMAEUATgAoAGYAbABhAHQAdABlAG4AZQBkAF8AbgBvAHIAbQBzACkALABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQB4AF8AbABlAG4ALAAgAE0AQQBYACgAbABlAG4AZwB0AGgAcwApACwAXABuACAAIAAgACAAIAAgACAAIABwAGEAZABfAGwAZQBuACwAIABSAE8AVQBOAEQAVQBQACgAbQBhAHgAXwBsAGUAbgAgAC8AIABrACwAIAAwACkAIAAqACAAawAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIABwAGEAZABkAGUAZABfAG4AbwByAG0AcwAsACAAUgBFAFAAVAAoAFwAIgAwAFwAIgAsACAAcABhAGQAXwBsAGUAbgAgAC0AIABsAGUAbgBnAHQAaABzACkAIAAmACAAZgBsAGEAdAB0AGUAbgBlAGQAXwBuAG8AcgBtAHMALABcAG4AIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAXwBzAHQAYQByAHQAXwBpAG4AZABpAGMAZQBzACwAIABTAEUAUQBVAEUATgBDAEUAKABwAGEAZABfAGwAZQBuACAALwAgAGsALAAgADEALAAgAHAAYQBkAF8AbABlAG4AIAAtACAAawAgACsAIAAxACwAIAAtAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAtAC0ATQBJAEQAKABwAGEAZABkAGUAZABfAG4AbwByAG0AcwAsACAAbABpAG0AYgBfAHMAdABhAHIAdABfAGkAbgBkAGkAYwBlAHMALAAgAGsAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAAWwBJAG4AdABlAHIAbgBhAGwAXQAgAEMAbwBuAGMAYQB0AGUAbgBhAHQAZQBzACAAYQBuACAAYQByAHIAYQB5ACAAbwBmACAAbgB1AG0AZQByAGkAYwAgAGwAaQBtAGIAcwAgAGkAbgB0AG8AIABhACAAQgBpAGcASQBuAHQAIABzAHQAcgBpAG4AZwAsACAAegBlAHIAbwAtAHAAYQBkAGQAaQBuAGcAIABhAGwAbAAgAGIAdQB0ACAAdABoAGUAIABmAGkAcgBzAHQAIABsAGkAbQBiAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAbABpAG0AYgBzACAAVABoAGUAIAB2AGUAcgB0AGkAYwBhAGwAIABhAHIAcgBhAHkAIABvAGYAIABuAHUAbQBlAHIAaQBjACAAbABpAG0AYgBzAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAawAgAFQAaABlACAAbABpAG0AYgAgAHMAaQB6AGUAIAB1AHMAZQBkACAAZAB1AHIAaQBuAGcAIABjAGEAbABjAHUAbABhAHQAaQBvAG4ALgBcAG4AIAAqAC8AXABuAE0AZQByAGcAZQAgAD0AIABMAEEATQBCAEQAQQAoAGwAaQBtAGIAcwAsACAAawAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABuAHUAbQBfAGwAaQBtAGIAcwAsACAAUgBPAFcAUwAoAGwAaQBtAGIAcwApACwAXABuACAAIAAgACAAIAAgACAAIAByAGUAdgBfAGwAaQBtAGIAcwAsACAAQwBIAE8ATwBTAEUAUgBPAFcAUwAoAGwAaQBtAGIAcwAsACAAUwBFAFEAVQBFAE4AQwBFACgAbgB1AG0AXwBsAGkAbQBiAHMALAAgADEALAAgAG4AdQBtAF8AbABpAG0AYgBzACwAIAAtADEAKQApACwAXABuACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABuAHUAbQBfAGwAaQBtAGIAcwAgAD0AIAAxACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHIAZQB2AF8AbABpAG0AYgBzACAAJgAgAFwAIgBcACIALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAQwBPAE4AQwBBAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABWAFMAVABBAEMASwAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAVABBAEsARQAoAHIAZQB2AF8AbABpAG0AYgBzACwAIAAxACkAIAAmACAAXAAiAFwAIgAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAVABFAFgAVAAoAEQAUgBPAFAAKAByAGUAdgBfAGwAaQBtAGIAcwAsACAAMQApACwAIABSAEUAUABUACgAXAAiADAAXAAiACwAIABrACkAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAAWwBJAG4AdABlAHIAbgBhAGwAXQAgAFIAZQBzAG8AbAB2AGUAcwAgAGMAYQByAHIAaQBlAHMAIAByAGkAZwBoAHQALQB0AG8ALQBsAGUAZgB0ACAAYQBjAHIAbwBzAHMAIABhACAAdgBlAHIAdABpAGMAYQBsACAAYQByAHIAYQB5ACAAbwBmACAAYgBhAHMAZQAtADEAMABeAGsAIABsAGkAbQBiAHMALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABsAGkAbQBiAHMAIABUAGgAZQAgAGEAcgByAGEAeQAgAG8AZgAgAG4AdQBtAGUAcgBpAGMAIABsAGkAbQBiAHMALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABrACAAVABoAGUAIABsAGkAbQBiACAAcwBpAHoAZQAuAFwAbgAgACoALwBcAG4AQwBhAHIAcgB5ACAAPQAgAEwAQQBNAEIARABBACgAbABpAG0AYgBzACwAIABrACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG4AdQBtAF8AbABpAG0AYgBzACwAIABSAE8AVwBTACgAbABpAG0AYgBzACkALABcAG4AIAAgACAAIAAgACAAIAAgAHIAYQBkAGkAeABfAGIAYQBzAGUALAAgADEAMABeAGsALABcAG4AIAAgACAAIAAgACAAIAAgAGEAcgByAF8AYwBhAHIAcgBpAGUAcwAsACAAUwBDAEEATgAoADAALAAgAGwAaQBtAGIAcwAsACAATABBAE0AQgBEAEEAKABhAGMAYwAsACAAdgBhAGwALAAgAHYAYQBsACAAKwAgAEkATgBUACgAYQBjAGMAIAAvACAAcgBhAGQAaQB4AF8AYgBhAHMAZQApACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcgBlAG0AYQBpAG4AZABlAHIAcwAsACAATQBPAEQAKABhAHIAcgBfAGMAYQByAHIAaQBlAHMALAAgAHIAYQBkAGkAeABfAGIAYQBzAGUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAG4AYQBsAF8AYwBhAHIAcgB5ACwAIABJAE4AVAAoAEkATgBEAEUAWAAoAGEAcgByAF8AYwBhAHIAcgBpAGUAcwAsACAAbgB1AG0AXwBsAGkAbQBiAHMALAAgADEAKQAgAC8AIAByAGEAZABpAHgAXwBiAGEAcwBlACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIABJAEYAKABmAGkAbgBhAGwAXwBjAGEAcgByAHkAIAA+ACAAMAAsACAAVgBTAFQAQQBDAEsAKAByAGUAbQBhAGkAbgBkAGUAcgBzACwAIABmAGkAbgBhAGwAXwBjAGEAcgByAHkAKQAsACAAcgBlAG0AYQBpAG4AZABlAHIAcwApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8ALwAgAC0ALQAtACAAVQBuAHMAaQBnAG4AZQBkACAASwBlAHIAbgBlAGwAcwAgAC0ALQAtACAAXABcAFwAXABcAG4AXABuAC8AKgAqAFwAbgAgACoAIABbAEkAbgB0AGUAcgBuAGEAbABdACAAVQBuAHMAaQBnAG4AZQBkACAAYwBvAG0AcABhAHIAaQBzAG8AbgAgAG8AZgAgAHQAdwBvACAATABpAHQAdABsAGUALQBFAG4AZABpAGEAbgAgAGwAaQBtAGIAIABhAHIAcgBhAHkAcwAuAFwAbgAgACoAIABSAGUAdAB1AHIAbgBzACAAMQAgACgAYQAgAD4AIABiACkALAAgAC0AMQAgACgAYQAgADwAIABiACkALAAgAG8AcgAgADAAIAAoAGEAIAA9ACAAYgApAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAbABpAG0AYgBzAF8AYQAgAFQAaABlACAAZgBpAHIAcwB0ACAAbABpAG0AYgAgAGEAcgByAGEAeQAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGwAaQBtAGIAcwBfAGIAIABUAGgAZQAgAHMAZQBjAG8AbgBkACAAbABpAG0AYgAgAGEAcgByAGEAeQAuAFwAbgAgACoALwBcAG4AVQBDAG8AbQBwAGEAcgBlACAAPQAgAEwAQQBNAEIARABBACgAbABpAG0AYgBzAF8AYQAsACAAbABpAG0AYgBzAF8AYgAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABtAGEAeABfAHIAbwB3AHMALAAgAE0AQQBYACgAUgBPAFcAUwAoAGwAaQBtAGIAcwBfAGEAKQAsACAAUgBPAFcAUwAoAGwAaQBtAGIAcwBfAGIAKQApACwAXABuACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBhAF8AYQBsAGkAZwBuAGUAZAAsACAARQBYAFAAQQBOAEQAKABsAGkAbQBiAHMAXwBhACwAIABtAGEAeABfAHIAbwB3AHMALAAgADEALAAgADAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYgBfAGEAbABpAGcAbgBlAGQALAAgAEUAWABQAEEATgBEACgAbABpAG0AYgBzAF8AYgAsACAAbQBhAHgAXwByAG8AdwBzACwAIAAxACwAIAAwACkALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAZABpAGYAZgBlAHIAZQBuAGMAZQBzACwAIABsAGkAbQBiAHMAXwBhAF8AYQBsAGkAZwBuAGUAZAAgAC0AIABsAGkAbQBiAHMAXwBiAF8AYQBsAGkAZwBuAGUAZAAsAFwAbgAgACAAIAAgACAAIAAgACAAaABpAGcAaABlAHMAdABfAG4AbwBuAF8AegBlAHIAbwBfAGkAbgBkAGUAeAAsACAAWABNAEEAVABDAEgAKABUAFIAVQBFACwAIABkAGkAZgBmAGUAcgBlAG4AYwBlAHMAIAA8AD4AIAAwACwAIAAwACwAIAAtADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATgBBACgAaABpAGcAaABlAHMAdABfAG4AbwBuAF8AegBlAHIAbwBfAGkAbgBkAGUAeAApACwAIAAwACwAIABTAEkARwBOACgASQBOAEQARQBYACgAZABpAGYAZgBlAHIAZQBuAGMAZQBzACwAIABoAGkAZwBoAGUAcwB0AF8AbgBvAG4AXwB6AGUAcgBvAF8AaQBuAGQAZQB4ACwAIAAxACkAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABbAEkAbgB0AGUAcgBuAGEAbABdACAAVQBuAHMAaQBnAG4AZQBkACAAYQBkAGQAaQB0AGkAbwBuACAAbwBmACAAdAB3AG8AIABMAGkAdAB0AGwAZQAtAEUAbgBkAGkAYQBuACAAbABpAG0AYgAgAGEAcgByAGEAeQBzAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAbABpAG0AYgBzAF8AYQAgAFQAaABlACAAZgBpAHIAcwB0ACAAbABpAG0AYgAgAGEAcgByAGEAeQAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGwAaQBtAGIAcwBfAGIAIABUAGgAZQAgAHMAZQBjAG8AbgBkACAAbABpAG0AYgAgAGEAcgByAGEAeQAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGsAIABUAGgAZQAgAGQAeQBuAGEAbQBpAGMAIABjAGgAdQBuAGsAIABzAGkAegBlACAAYwBvAG4AdABlAHgAdAAuAFwAbgAgACoALwBcAG4AVQBBAGQAZAAgAD0AIABMAEEATQBCAEQAQQAoAGEALAAgAGIALAAgAGsALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHgAXwByAG8AdwBzACwAIABNAEEAWAAoAFIATwBXAFMAKABhACkALAAgAFIATwBXAFMAKABiACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYQBfAGEAbABpAGcAbgBlAGQALAAgAEUAWABQAEEATgBEACgAYQAsACAAbQBhAHgAXwByAG8AdwBzACwAIAAxACwAIAAwACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGIAXwBhAGwAaQBnAG4AZQBkACwAIABFAFgAUABBAE4ARAAoAGIALAAgAG0AYQB4AF8AcgBvAHcAcwAsACAAMQAsACAAMAApACwAXABuACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAYQByAHIAeQAoAGwAaQBtAGIAcwBfAGEAXwBhAGwAaQBnAG4AZQBkACAAKwAgAGwAaQBtAGIAcwBfAGIAXwBhAGwAaQBnAG4AZQBkACwAIABrACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFsASQBuAHQAZQByAG4AYQBsAF0AIABVAG4AcwBpAGcAbgBlAGQAIABzAHUAYgB0AHIAYQBjAHQAaQBvAG4AIABvAGYAIAB0AHcAbwAgAEwAaQB0AHQAbABlAC0ARQBuAGQAaQBhAG4AIABsAGkAbQBiACAAYQByAHIAYQB5AHMALgBcAG4AIAAqACAAQQBzAHMAdQBtAGUAcwAgAG0AYQBnAG4AaQB0AHUAZABlAHMAIABBACAAPgA9ACAAQgAuACAAUgBlAHMAbwBsAHYAZQBzACAAYgBvAHIAcgBvAHcAcwAgAHQAbwBwAC0AdABvAC0AYgBvAHQAdABvAG0AIABhAG4AZAAgAHQAcgBpAG0AcwAgAHQAcgBhAGkAbABpAG4AZwAgAHoAZQByAG8AcwAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGwAaQBtAGIAcwBfAGEAIABUAGgAZQAgAG0AaQBuAHUAZQBuAGQAIABsAGkAbQBiACAAYQByAHIAYQB5ACAAKABtAHUAcwB0ACAAYgBlACAAPgA9ACAAbABpAG0AYgBzAF8AYgApAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAbABpAG0AYgBzAF8AYgAgAFQAaABlACAAcwB1AGIAdAByAGEAaABlAG4AZAAgAGwAaQBtAGIAIABhAHIAcgBhAHkALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABrACAAVABoAGUAIABkAHkAbgBhAG0AaQBjACAAYwBoAHUAbgBrACAAcwBpAHoAZQAgAGMAbwBuAHQAZQB4AHQALgBcAG4AIAAqAC8AXABuAFUAUwB1AGIAIAA9ACAATABBAE0AQgBEAEEAKABsAGkAbQBiAHMAXwBhACwAIABsAGkAbQBiAHMAXwBiACwAIABrACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQB4AF8AcgBvAHcAcwAsACAATQBBAFgAKABSAE8AVwBTACgAbABpAG0AYgBzAF8AYQApACwAIABSAE8AVwBTACgAbABpAG0AYgBzAF8AYgApACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGEAXwBhAGwAaQBnAG4AZQBkACwAIABFAFgAUABBAE4ARAAoAGwAaQBtAGIAcwBfAGEALAAgAG0AYQB4AF8AcgBvAHcAcwAsACAAMQAsACAAMAApACwAXABuACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBiAF8AYQBsAGkAZwBuAGUAZAAsACAARQBYAFAAQQBOAEQAKABsAGkAbQBiAHMAXwBiACwAIABtAGEAeABfAHIAbwB3AHMALAAgADEALAAgADAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIABkAGkAZgBmAGUAcgBlAG4AYwBlAHMALAAgAGwAaQBtAGIAcwBfAGEAXwBhAGwAaQBnAG4AZQBkACAALQAgAGwAaQBtAGIAcwBfAGIAXwBhAGwAaQBnAG4AZQBkACwAXABuACAAIAAgACAAIAAgACAAIABjAGEAcgByAGkAZQBkAF8AZABpAGYAZgBlAHIAZQBuAGMAZQBzACwAIABDAGEAcgByAHkAKABkAGkAZgBmAGUAcgBlAG4AYwBlAHMALAAgAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIABoAGkAZwBoAGUAcwB0AF8AbgBvAG4AXwB6AGUAcgBvAF8AaQBuAGQAZQB4ACwAIABYAE0AQQBUAEMASAAoAFQAUgBVAEUALAAgAGMAYQByAHIAaQBlAGQAXwBkAGkAZgBmAGUAcgBlAG4AYwBlAHMAIAA8AD4AIAAwACwAIAAwACwAIAAtADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATgBBACgAaABpAGcAaABlAHMAdABfAG4AbwBuAF8AegBlAHIAbwBfAGkAbgBkAGUAeAApACwAIAB7ADAAfQAsACAAVABBAEsARQAoAGMAYQByAHIAaQBlAGQAXwBkAGkAZgBmAGUAcgBlAG4AYwBlAHMALAAgAGgAaQBnAGgAZQBzAHQAXwBuAG8AbgBfAHoAZQByAG8AXwBpAG4AZABlAHgAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABbAEkAbgB0AGUAcgBuAGEAbABdACAAVgBlAGMAdABvAHIAaQB6AGUAZAAgAG0AYQB0AHIAaQB4ACAAcwB1AG0AIABvAGYAIAB1AG4AcwBpAGcAbgBlAGQAIABCAGkAZwBJAG4AdAAgAHMAdAByAGkAbgBnAHMALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABzAHQAcgBfAG4AbwByAG0AcwAgAEgAbwByAGkAegBvAG4AdABhAGwAIABhAHIAcgBhAHkAIAAoADEAeABOACkAIABvAGYAIABuAG8AcgBtAGEAbABpAHoAZQBkACAAbQBhAGcAbgBpAHQAdQBkAGUAIABzAHQAcgBpAG4AZwBzAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAawAgAFQAaABlACAAdQBuAGkAZgBpAGUAZAAgAGQAeQBuAGEAbQBpAGMAIABjAGgAdQBuAGsAIABzAGkAegBlACAAYwBvAG4AdABlAHgAdAAuAFwAbgAgACoALwBcAG4AVQBNAGEAdAByAGkAeABTAHUAbQAgAD0AIABMAEEATQBCAEQAQQAoAHMAdAByAF8AbgBvAHIAbQBzACwAIABrACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAGcAcgBpAGQALAAgAFMAcABsAGkAdAAoAHMAdAByAF8AbgBvAHIAbQBzACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgAHIAYQB3AF8AbABpAG0AYgBzACwAIABCAFkAUgBPAFcAKABnAHIAaQBkACwAIABTAFUATQApACwAXABuACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAYQByAHIAeQAoAHIAYQB3AF8AbABpAG0AYgBzACwAIABrACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFsASQBuAHQAZQByAG4AYQBsAF0AIABSAG8AdQB0AGUAcwAgAGEAZABkAGkAdABpAG8AbgAvAHMAdQBiAHQAcgBhAGMAdABpAG8AbgAgAGIAYQBzAGUAZAAgAG8AbgAgAHMAaQBnAG4AcwAgAGEAbgBkACAAbQBhAGcAbgBpAHQAdQBkAGUAcwAuAFwAbgAgACoAIABSAGUAdAB1AHIAbgBzACAAYQAgAHQAdQBwAGwAZQAgAGEAcgByAGEAeQA6ACAAVgBTAFQAQQBDAEsAKABsAGkAbQBiAHMALAAgAGYAaQBuAGEAbABfAHMAaQBnAG4AKQAgAHcAaABlAHIAZQAgAHQAaABlACAAZgBpAG4AYQBsACAAcgBvAHcAIABpAHMAIAB0AGgAZQAgAHMAYwBhAGwAYQByACAAcwBpAGcAbgAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGwAaQBtAGIAcwBfAGEAIABUAGgAZQAgAGYAaQByAHMAdAAgAGwAaQB0AHQAbABlAC0AZQBuAGQAaQBhAG4AIABsAGkAbQBiACAAYQByAHIAYQB5AC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAbABpAG0AYgBzAF8AYgAgAFQAaABlACAAcwBlAGMAbwBuAGQAIABsAGkAdAB0AGwAZQAtAGUAbgBkAGkAYQBuACAAbABpAG0AYgAgAGEAcgByAGEAeQAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAHMAaQBnAG4AXwBhACAAVABoAGUAIABzAGkAZwBuACAAbwBmACAAdABoAGUAIABmAGkAcgBzAHQAIABhAHIAcgBhAHkAIAAoADEALAAgAC0AMQAsACAAMAApAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAcwBpAGcAbgBfAGIAIABUAGgAZQAgAHMAaQBnAG4AIABvAGYAIAB0AGgAZQAgAHMAZQBjAG8AbgBkACAAYQByAHIAYQB5ACAAKAAxACwAIAAtADEALAAgADAAKQAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGsAIABUAGgAZQAgAGQAeQBuAGEAbQBpAGMAIABjAGgAdQBuAGsAIABzAGkAegBlACAAYwBvAG4AdABlAHgAdAAuAFwAbgAgACoALwBcAG4AQQBkAGQAUwB1AGIAUgBvAHUAdABlAHIAIAA9ACAATABBAE0AQgBEAEEAKABsAGkAbQBiAHMAXwBhACwAIABsAGkAbQBiAHMAXwBiACwAIABzAGkAZwBuAF8AYQAsACAAcwBpAGcAbgBfAGIALAAgAGsALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAaQBzAF8AYQBkAGQAaQB0AGkAbwBuACwAIABzAGkAZwBuAF8AYQAgAD0AIABzAGkAZwBuAF8AYgAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABpAHMAXwBhAGQAZABpAHQAaQBvAG4ALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAVgBTAFQAQQBDAEsAKABVAEEAZABkACgAbABpAG0AYgBzAF8AYQAsACAAbABpAG0AYgBzAF8AYgAsACAAawApACwAIABzAGkAZwBuAF8AYQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAG0AYQBnAG4AaQB0AHUAZABlAF8AYwBvAG0AcABhAHIAaQBzAG8AbgAsACAAVQBDAG8AbQBwAGEAcgBlACgAbABpAG0AYgBzAF8AYQAsACAAbABpAG0AYgBzAF8AYgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgAbQBhAGcAbgBpAHQAdQBkAGUAXwBjAG8AbQBwAGEAcgBpAHMAbwBuACAAPQAgADAALAAgAC8ALwAgAFQAbwB0AGEAbAAgAGMAYQBuAGMAZQBsAGwAYQB0AGkAbwBuADoAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAB7ADAAOwAwAH0ALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgAbQBhAGcAbgBpAHQAdQBkAGUAXwBjAG8AbQBwAGEAcgBpAHMAbwBuACAAPgAgADAALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAAQQAgAGkAcwAgAGwAYQByAGcAZQByADoAIABzAGkAZwBuACAAYgBlAGwAbwBuAGcAcwAgAHQAbwAgAEEALgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAVgBTAFQAQQBDAEsAKABVAFMAdQBiACgAbABpAG0AYgBzAF8AYQAsACAAbABpAG0AYgBzAF8AYgAsACAAawApACwAIABzAGkAZwBuAF8AYQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIABCACAAaQBzACAAbABhAHIAZwBlAHIAOgAgAHIAbwB1AHQAZQAgAEIAIABmAGkAcgBzAHQALAAgAHMAaQBnAG4AIABiAGUAbABvAG4AZwBzACAAdABvACAAQgAuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABWAFMAVABBAEMASwAoAFUAUwB1AGIAKABsAGkAbQBiAHMAXwBiACwAIABsAGkAbQBiAHMAXwBhACwAIABrACkALAAgAHMAaQBnAG4AXwBiACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABbAEkAbgB0AGUAcgBuAGEAbABdACAAVQBuAHMAaQBnAG4AZQBkACAAbQB1AGwAdABpAHAAbABpAGMAYQB0AGkAbwBuACAAbwBmACAAdAB3AG8AIABMAGkAdAB0AGwAZQAtAEUAbgBkAGkAYQBuACAAbABpAG0AYgAgAGEAcgByAGEAeQBzAC4AXABuACAAKgAgAFUAdABpAGwAaQB6AGUAcwAgAGEAIAAxAEQAIABEAGkAcwBjAHIAZQB0AGUAIABDAG8AbgB2AG8AbAB1AHQAaQBvAG4AIAAoAEMAYQB1AGMAaAB5ACAAUAByAG8AZAB1AGMAdAApACAAYQByAHIAYQB5AC0AcwBsAGkAYwBpAG4AZwAgAHMAdAByAGEAdABlAGcAeQAuAFwAbgAgACoAIABaAGUAcgBvACAAZAB5AG4AYQBtAGkAYwAgAG0AZQBtAG8AcgB5ACAAcgBlAGEAbABsAG8AYwBhAHQAaQBvAG4ALgAgACQATwAoAE4AKwBNACkAJAAgAG0AZQBtAG8AcgB5ACAAZgBvAG8AdABwAHIAaQBuAHQALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABsAGkAbQBiAHMAXwBhACAAVABoAGUAIABtAHUAbAB0AGkAcABsAGkAYwBhAG4AZAAgAGwAaQBtAGIAIABhAHIAcgBhAHkALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABsAGkAbQBiAHMAXwBiACAAVABoAGUAIABtAHUAbAB0AGkAcABsAGkAZQByACAAbABpAG0AYgAgAGEAcgByAGEAeQAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGsAIABUAGgAZQAgAGQAeQBuAGEAbQBpAGMAIABjAGgAdQBuAGsAIABzAGkAegBlACAAYwBvAG4AdABlAHgAdAAuAFwAbgAgACoALwBcAG4AVQBNAHUAbAAgAD0AIABMAEEATQBCAEQAQQAoAGwAaQBtAGIAcwBfAGEALAAgAGwAaQBtAGIAcwBfAGIALAAgAGsALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbgB1AG0AXwBsAGkAbQBiAHMAXwBhACwAIABSAE8AVwBTACgAbABpAG0AYgBzAF8AYQApACwAXABuACAAIAAgACAAIAAgACAAIABuAHUAbQBfAGwAaQBtAGIAcwBfAGIALAAgAFIATwBXAFMAKABsAGkAbQBiAHMAXwBiACkALABcAG4AIAAgACAAIAAgACAAIAAgAGMAbwBuAHYAbwBsAHUAdABpAG8AbgBfAGwAZQBuAGcAdABoACwAIABuAHUAbQBfAGwAaQBtAGIAcwBfAGEAIAArACAAbgB1AG0AXwBsAGkAbQBiAHMAXwBiACAALQAgADEALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAcgBhAHcAXwBjAG8AbgB2AG8AbAB1AHQAaQBvAG4ALAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAYwBvAG4AdgBvAGwAdQB0AGkAbwBuAF8AbABlAG4AZwB0AGgALAAgADEALAAgAEwAQQBNAEIARABBACgAcgAsACAAYwAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHcAaQBuAGQAbwB3AF8AcwB0AGEAcgB0AF8AaQAsACAATQBBAFgAKAAxACwAIAByACAALQAgAG4AdQBtAF8AbABpAG0AYgBzAF8AYgAgACsAIAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAB3AGkAbgBkAG8AdwBfAGUAbgBkAF8AaQAsACAATQBJAE4AKAByACwAIABuAHUAbQBfAGwAaQBtAGIAcwBfAGEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAG8AdgBlAHIAbABhAHAAXwByAG8AdwBzACwAIAB3AGkAbgBkAG8AdwBfAGUAbgBkAF8AaQAgAC0AIAB3AGkAbgBkAG8AdwBfAHMAdABhAHIAdABfAGkAIAArACAAMQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHMAZQBxAF8AaQAsACAAUwBFAFEAVQBFAE4AQwBFACgAbwB2AGUAcgBsAGEAcABfAHIAbwB3AHMALAAgADEALAAgAHcAaQBuAGQAbwB3AF8AcwB0AGEAcgB0AF8AaQAsACAAMQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcwBlAHEAXwBqACwAIABTAEUAUQBVAEUATgBDAEUAKABvAHYAZQByAGwAYQBwAF8AcgBvAHcAcwAsACAAMQAsACAAcgAgAC0AIAB3AGkAbgBkAG8AdwBfAHMAdABhAHIAdABfAGkAIAArACAAMQAsACAALQAxACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABTAFUATQAoAEkATgBEAEUAWAAoAGwAaQBtAGIAcwBfAGEALAAgAHMAZQBxAF8AaQAsACAAMQApACAAKgAgAEkATgBEAEUAWAAoAGwAaQBtAGIAcwBfAGIALAAgAHMAZQBxAF8AagAsACAAMQApACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAApACkALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBhAHIAcgB5ACgAcgBhAHcAXwBjAG8AbgB2AG8AbAB1AHQAaQBvAG4ALAAgAGsAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AoAAqACAAWwBJAG4AdABlAHIAbgBhAGwAXQAgAEIAaQBuAGEAcgB5ACAAcwBlAGEAcgBjAGgAIAB0AG8AIABmAGkAbgBkACAAdABoAGUAIABoAGkAZwBoAGUAcwB0ACAAcwBjAGEAbABhAHIAIABxAHUAbwB0AGkAZQBuAHQAIABsAGkAbQBiACAAcQAgACgAMAAgADwAPQAgAHEAIAA8ACAAMQAwAF4AawApAFwAbgCgACoAIABzAHUAYwBoACAAdABoAGEAdAAgAEIAIAAqACAAcQAgADwAPQAgAGwAaQBtAGIAcwBfAHIALgAgAEUAbABpAG0AaQBuAGEAdABlAHMAIAB0AGgAZQAgAG4AZQBlAGQAIABmAG8AcgAgAEsAbgB1AHQAaAAgAEQAIABmAGwAbwBhAHQALQBlAHMAdABpAG0AYQB0AGkAbwBuAC4AXABuAKAAKgAgAEAAcABhAHIAYQBtACAAbABpAG0AYgBzAF8AcgAgAFQAaABlACAAYwB1AHIAcgBlAG4AdAAgAHIAZQBtAGEAaQBuAGQAZQByACAAYQByAHIAYQB5AC4AXABuAKAAKgAgAEAAcABhAHIAYQBtACAAYgAgAFQAaABlACAAZABpAHYAaQBzAG8AcgAgAGEAcgByAGEAeQAuAFwAbgCgACoAIABAAHAAYQByAGEAbQAgAGsAIABUAGgAZQAgAGQAeQBuAGEAbQBpAGMAIABjAGgAdQBuAGsAIABzAGkAegBlACAAYwBvAG4AdABlAHgAdAAuAFwAbgCgACoALwBcAG4ARgBpAG4AZABRAHUAbwB0AGkAZQBuAHQATABpAG0AYgAgAD0AIABMAEEATQBCAEQAQQAoAGwAaQBtAGIAcwBfAHIALAAgAGwAaQBtAGIAcwBfAGIALAAgAGsALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAcgBlAHEAdQBpAHIAZQBkAF8AYgBpAHQAcwAsACAAQwBFAEkATABJAE4ARwAuAE0AQQBUAEgAKABMAE8ARwAoADEAMABeAGsALAAgADIAKQApACwAXABuACAAIAAgACAAIAAgACAAIABwAG8AdwBlAHIAcwBfAG8AZgBfAHQAdwBvACwAIAAyACAAXgAgAFMARQBRAFUARQBOAEMARQAoAHIAZQBxAHUAaQByAGUAZABfAGIAaQB0AHMALAAgADEALAAgAHIAZQBxAHUAaQByAGUAZABfAGIAaQB0AHMAIAAtACAAMQAsACAALQAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAUgBFAEQAVQBDAEUAKAAwACwAIABwAG8AdwBlAHIAcwBfAG8AZgBfAHQAdwBvACwAIABMAEEATQBCAEQAQQAoAGMAdQByAHIAZQBuAHQAXwBxACwAIABjAHUAcgByAGUAbgB0AF8AcABvAHcAZQByACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAdABlAHMAdABfAHEALAAgAGMAdQByAHIAZQBuAHQAXwBxACAAKwAgAGMAdQByAHIAZQBuAHQAXwBwAG8AdwBlAHIALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKAB0AGUAcwB0AF8AcQAgAD4APQAgADEAMABeAGsALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAYwB1AHIAcgBlAG4AdABfAHEALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGIAcQAsACAAQwBhAHIAcgB5ACgAbABpAG0AYgBzAF8AYgAgACoAIAB0AGUAcwB0AF8AcQAsACAAawApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAG0AYQBnAG4AaQB0AHUAZABlAF8AYwBvAG0AcABhAHIAaQBzAG8AbgAsACAAVQBDAG8AbQBwAGEAcgBlACgAbABpAG0AYgBzAF8AcgAsACAAbABpAG0AYgBzAF8AYgBxACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEkARgAoAG0AYQBnAG4AaQB0AHUAZABlAF8AYwBvAG0AcABhAHIAaQBzAG8AbgAgAD4APQAgADAALAAgAHQAZQBzAHQAXwBxACwAIABjAHUAcgByAGUAbgB0AF8AcQApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgCgACoAIABbAEkAbgB0AGUAcgBuAGEAbABdACAAQgBhAHMAZQBjAGEAcwBlACAARABpAHYAaQBzAGkAbwBuACAAdgBpAGEAIABzAGUAcQB1AGUAbgB0AGkAYQBsACAAcwBoAGkAZgB0AC0AYQBuAGQALQBzAHUAYgB0AHIAYQBjAHQALgBcAG4AoAAqACAAUgBlAHQAdQByAG4AcwAgAGEAIABwAGEAYwBrAGUAZAAgADEARAAgAGEAcgByAGEAeQA6ACAAVgBTAFQAQQBDAEsAKABMAGUAbgBnAHQAaABfAFIALAAgAFIAXwBsAGkAbQBiAHMALAAgAFEAXwBsAGkAbQBiAHMAKQAuAFwAbgCgACoAIABFAGwAaQBtAGkAbgBhAHQAZQBzACAAMgBEACAAYQByAHIAYQB5ACAAcABhAGQAZABpAG4AZwAgAHQAbwAgAHMAdAByAGkAYwB0AGwAeQAgAHAAcgBlAHMAZQByAHYAZQAgAG0AZQBtAG8AcgB5ACAAZQBmAGYAaQBjAGkAZQBuAGMAeQAuAFwAbgCgACoAIABAAHAAYQByAGEAbQAgAGwAaQBtAGIAcwBfAGEAIABUAGgAZQAgAGQAaQB2AGkAZABlAG4AZAAgAGEAcgByAGEAeQAuAFwAbgCgACoAIABAAHAAYQByAGEAbQAgAGwAaQBtAGIAcwBfAGIAIABUAGgAZQAgAGQAaQB2AGkAcwBvAHIAIABhAHIAcgBhAHkAIAAoAGEAcwBzAHUAbQBlAGQAIABuAG8AbgAtAHoAZQByAG8AKQAuAFwAbgCgACoAIABAAHAAYQByAGEAbQAgAGsAIABUAGgAZQAgAGQAeQBuAGEAbQBpAGMAIABjAGgAdQBuAGsAIABzAGkAegBlACAAYwBvAG4AdABlAHgAdAAuAFwAbgCgACoALwBcAG4ASwBuAHUAdABoAEQAaQB2ACAAPQAgAEwAQQBNAEIARABBACgAbABpAG0AYgBzAF8AYQAsACAAbABpAG0AYgBzAF8AYgAsACAAawAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABtAGEAZwBuAGkAdAB1AGQAZQBfAGMAbwBtAHAAYQByAGkAcwBvAG4ALAAgAFUAQwBvAG0AcABhAHIAZQAoAGwAaQBtAGIAcwBfAGEALAAgAGwAaQBtAGIAcwBfAGIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABtAGEAZwBuAGkAdAB1AGQAZQBfAGMAbwBtAHAAYQByAGkAcwBvAG4AIAA8ACAAMAAsACAAVgBTAFQAQQBDAEsAKABSAE8AVwBTACgAbABpAG0AYgBzAF8AYQApACwAIABsAGkAbQBiAHMAXwBhACwAIAAwACkALABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAG0AYQBnAG4AaQB0AHUAZABlAF8AYwBvAG0AcABhAHIAaQBzAG8AbgAgAD0AIAAwACwAIABWAFMAVABBAEMASwAoADEALAAgADAALAAgADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAG4AdQBtAF8AbABpAG0AYgBzAF8AYQAsACAAUgBPAFcAUwAoAGwAaQBtAGIAcwBfAGEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGIAaQBnAF8AZQBuAGQAaQBhAG4AXwBhACwAIABDAEgATwBPAFMARQBSAE8AVwBTACgAbABpAG0AYgBzAF8AYQAsACAAUwBFAFEAVQBFAE4AQwBFACgAbgB1AG0AXwBsAGkAbQBiAHMAXwBhACwAIAAxACwAIABuAHUAbQBfAGwAaQBtAGIAcwBfAGEALAAgAC0AMQApACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABmAGkAbgBhAGwAXwBwAGEAYwBrAGUAZABfAHMAdABhAHQAZQAsACAAUgBFAEQAVQBDAEUAKABWAFMAVABBAEMASwAoADEALAAgADAALAAgADAAKQAsACAAYgBpAGcAXwBlAG4AZABpAGEAbgBfAGEALAAgAEwAQQBNAEIARABBACgAcABhAGMAawBlAGQAXwBzAHQAYQB0AGUALAAgAHYAYQBsACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABuAHUAbQBfAGwAaQBtAGIAcwBfAHIALAAgAEkATgBEAEUAWAAoAHAAYQBjAGsAZQBkAF8AcwB0AGEAdABlACwAIAAxACwAIAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AcgAsACAAQwBIAE8ATwBTAEUAUgBPAFcAUwAoAHAAYQBjAGsAZQBkAF8AcwB0AGEAdABlACwAIABTAEUAUQBVAEUATgBDAEUAKABuAHUAbQBfAGwAaQBtAGIAcwBfAHIALAAgADEALAAgADIAKQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAHEALAAgAEQAUgBPAFAAKABwAGEAYwBrAGUAZABfAHMAdABhAHQAZQAsACAAbgB1AG0AXwBsAGkAbQBiAHMAXwByACAAKwAgADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AcwBoAGkAZgB0AGUAZABfAHIALAAgAEkARgAoAEEATgBEACgAUgBPAFcAUwAoAGwAaQBtAGIAcwBfAHIAKQAgAD0AIAAxACwAIABJAE4ARABFAFgAKABsAGkAbQBiAHMAXwByACwAIAAxACwAIAAxACkAIAA9ACAAMAApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAB2AGEAbAAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAVgBTAFQAQQBDAEsAKAB2AGEAbAAsACAAbABpAG0AYgBzAF8AcgApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABxAF8AbABpAG0AYgAsACAARgBpAG4AZABRAHUAbwB0AGkAZQBuAHQATABpAG0AYgAoAGwAaQBtAGIAcwBfAHMAaABpAGYAdABlAGQAXwByACwAIABsAGkAbQBiAHMAXwBiACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYgBxACwAIABDAGEAcgByAHkAKABsAGkAbQBiAHMAXwBiACAAKgAgAHEAXwBsAGkAbQBiACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AbgBlAHgAdABfAHIALAAgAFUAUwB1AGIAKABsAGkAbQBiAHMAXwBzAGgAaQBmAHQAZQBkAF8AcgAsACAAbABpAG0AYgBzAF8AYgBxACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAaABhAHMAXwBxACwAIABPAFIAKABSAE8AVwBTACgAbABpAG0AYgBzAF8AcQApACAAPgAgADEALAAgAEkATgBEAEUAWAAoAGwAaQBtAGIAcwBfAHEALAAxACwAMQApACAAPgAgADAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AbgBlAHgAdABfAHEALAAgAEkARgAoAGgAYQBzAF8AcQAsACAAVgBTAFQAQQBDAEsAKABsAGkAbQBiAHMAXwBxACwAIABxAF8AbABpAG0AYgApACwAIABxAF8AbABpAG0AYgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABWAFMAVABBAEMASwAoAFIATwBXAFMAKABsAGkAbQBiAHMAXwBuAGUAeAB0AF8AcgApACwAIABsAGkAbQBiAHMAXwBuAGUAeAB0AF8AcgAsACAAbABpAG0AYgBzAF8AbgBlAHgAdABfAHEAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbgB1AG0AXwBsAGkAbQBiAHMAXwByACwAIABJAE4ARABFAFgAKABmAGkAbgBhAGwAXwBwAGEAYwBrAGUAZABfAHMAdABhAHQAZQAsACAAMQAsACAAMQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AcgAsACAAQwBIAE8ATwBTAEUAUgBPAFcAUwAoAGYAaQBuAGEAbABfAHAAYQBjAGsAZQBkAF8AcwB0AGEAdABlACwAIABTAEUAUQBVAEUATgBDAEUAKABuAHUAbQBfAGwAaQBtAGIAcwBfAHIALAAgADEALAAgADIAKQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAYgBpAGcAXwBlAG4AZABpAGEAbgBfAHEALAAgAEQAUgBPAFAAKABmAGkAbgBhAGwAXwBwAGEAYwBrAGUAZABfAHMAdABhAHQAZQAsACAAbgB1AG0AXwBsAGkAbQBiAHMAXwByACAAKwAgADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAZQBuAF8AcQAsACAAUgBPAFcAUwAoAGIAaQBnAF8AZQBuAGQAaQBhAG4AXwBxACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBxACwAIABDAEgATwBPAFMARQBSAE8AVwBTACgAYgBpAGcAXwBlAG4AZABpAGEAbgBfAHEALAAgAFMARQBRAFUARQBOAEMARQAoAGwAZQBuAF8AcQAsACAAMQAsACAAbABlAG4AXwBxACwAIAAtADEAKQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAVgBTAFQAQQBDAEsAKABuAHUAbQBfAGwAaQBtAGIAcwBfAHIALAAgAGwAaQBtAGIAcwBfAHIALAAgAGwAaQBtAGIAcwBfAHEAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AoAAqACAAWwBJAG4AdABlAHIAbgBhAGwAXQAgAEgAeQBiAHIAaQBkACAARABpAHYAaQBzAGkAbwBuACAAUgBvAHUAdABlAHIALgBcAG4AoAAqACAARABpAHIAZQBjAHQAcwAgAGQAaQB2AGkAcwBpAG8AbgAgAHQAbwAgAHQAaABlACAAbwBwAHQAaQBtAGEAbAAgAGsAZQByAG4AZQBsACAAYgBhAHMAZQBkACAAbwBuACAARABpAHYAaQBkAGUAbgBkACAAbABlAG4AZwB0AGgALgBcAG4AoAAqACAAQABwAGEAcgBhAG0AIABsAGkAbQBiAHMAXwBhACAAVABoAGUAIABkAGkAdgBpAGQAZQBuAGQAIABhAHIAcgBhAHkALgBcAG4AoAAqACAAQABwAGEAcgBhAG0AIABsAGkAbQBiAHMAXwBiACAAVABoAGUAIABkAGkAdgBpAHMAbwByACAAYQByAHIAYQB5AC4AXABuAKAAKgAgAEAAcABhAHIAYQBtACAAawAgAFQAaABlACAAZAB5AG4AYQBtAGkAYwAgAGMAaAB1AG4AawAgAHMAaQB6AGUAIABjAG8AbgB0AGUAeAB0AC4AXABuAKAAKgAvAFwAbgBEAGkAdgBSAG8AdQB0AGUAcgAgAD0AIABMAEEATQBCAEQAQQAoAGwAaQBtAGIAcwBfAGEALAAgAGwAaQBtAGIAcwBfAGIALAAgAGsALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAYQBwAHAAcgBvAHgAXwBkAGkAZwBpAHQAcwBfAGEALAAgAFIATwBXAFMAKABsAGkAbQBiAHMAXwBhACkAIAAqACAAawAsAFwAbgAgACAAIAAgACAAIAAgACAAYQBwAHAAcgBvAHgAXwBkAGkAZwBpAHQAcwBfAGIALAAgAFIATwBXAFMAKABsAGkAbQBiAHMAXwBiACkAIAAqACAAawAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABMAG8AZwBpAHMAdABpAGMAIABSAGUAZwByAGUAcwBzAGkAbwBuACAAYwBvAGUAZgBmAGkAYwBpAGUAbgB0AHMAXABuACAAIAAgACAAIAAgACAAIAByAGUAZwByAGUAcwBzAGkAbwBuAF8AcwBsAG8AcABlAF8AbQAsACAAMAAuADEAMAA3ADgAMgAxADEAOQA0ADIANwAxADIAOQA3ACwAXABuACAAIAAgACAAIAAgACAAIAByAGUAZwByAGUAcwBzAGkAbwBuAF8AaQBuAHQAZQByAGMAZQBwAHQAXwBjACwAIAAtADIAMgAxAC4AOQAwADIAMQA4ADkANAA2ADIAMAA2ADgALABcAG4AIAAgACAAIAAgACAAIAAgAHQAaAByAGUAcwBoAG8AbABkAF8AZABpAGcAaQB0AHMALAAgACgAcgBlAGcAcgBlAHMAcwBpAG8AbgBfAHMAbABvAHAAZQBfAG0AIAAqACAAYQBwAHAAcgBvAHgAXwBkAGkAZwBpAHQAcwBfAGEAKQAgACsAIAByAGUAZwByAGUAcwBzAGkAbwBuAF8AaQBuAHQAZQByAGMAZQBwAHQAXwBjACwAXABuACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAGEAcABwAHIAbwB4AF8AZABpAGcAaQB0AHMAXwBiACAAPAA9ACAAdABoAHIAZQBzAGgAbwBsAGQAXwBkAGkAZwBpAHQAcwAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABLAG4AdQB0AGgARABpAHYAKABsAGkAbQBiAHMAXwBhACwAIABsAGkAbQBiAHMAXwBiACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATgBlAHcAdABvAG4AUgBhAHAAaABzAG8AbgBEAGkAdgAoAGwAaQBtAGIAcwBfAGEALAAgAGwAaQBtAGIAcwBfAGIALAAgAGsAKQBcAG4AIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFsASQBuAHQAZQByAG4AYQBsAF0AIABHAGUAbgBlAHIAYQB0AGUAcwAgAHQAaABlACAAZQB4AGEAYwB0ACAAcgBlAGMAaQBwAHIAbwBjAGEAbAAgAHMAZQBlAGQAIABmAG8AcgAgAE4AZQB3AHQAbwBuAC0AUgBhAHAAaABzAG8AbgAgAEQAaQB2AGkAcwBpAG8AbgAgAHUAcwBpAG4AZwAgAEsAbgB1AHQAaAAgAEIAYQBzAGUAYwBhAHMAZQAuAFwAbgAgACoAIABFAHgAdAByAGEAYwB0AHMAIAB1AHAAIAB0AG8AIAB0AGgAZQAgAHQAbwBwACAAMwAgAGwAaQBtAGIAcwAgAG8AZgAgAEIAIABhAG4AZAAgAGMAYQBsAGMAdQBsAGEAdABlAHMAIABmAGwAbwBvAHIAKABCAGUAdABhAF4AKAAyACoAbABlAG4AKQAgAC8AIABCAF8AdABvAHAAKQAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGwAaQBtAGIAcwBfAGIAIABUAGgAZQAgAGQAaQB2AGkAcwBvAHIAIABsAGkAbQBiACAAYQByAHIAYQB5AC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAawAgAFQAaABlACAAZAB5AG4AYQBtAGkAYwAgAGMAaAB1AG4AawAgAHMAaQB6AGUAIABjAG8AbgB0AGUAeAB0AC4AXABuACAAKgAvAFwAbgBOAGUAdwB0AG8AbgBSAGEAcABoAHMAbwBuAFMAZQBlAGQAIAA9ACAATABBAE0AQgBEAEEAKABsAGkAbQBiAHMAXwBiACwAIABrACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG4AdQBtAF8AbABpAG0AYgBzAF8AYgAsACAAUgBPAFcAUwAoAGwAaQBtAGIAcwBfAGIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbgB1AG0AXwBzAGUAZQBkAF8AbABpAG0AYgBzACwAIABNAEkATgAoADMALAAgAG4AdQBtAF8AbABpAG0AYgBzAF8AYgApACwAXABuACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgAC8ALwAgAEUAeAB0AHIAYQBjAHQAIAB0AG8AcAAgACcAcwBlAGUAZABfAGwAZQBuACcAIABsAGkAbQBiAHMAIAAoAEwAaQB0AHQAbABlAC0ARQBuAGQAaQBhAG4AOgAgAHQAYQBrAGUAIABmAHIAbwBtACAAdABoAGUAIABiAG8AdAB0AG8AbQApAFwAbgAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYgBfAHQAbwBwACwAIABUAEEASwBFACgAbABpAG0AYgBzAF8AYgAsACAALQBuAHUAbQBfAHMAZQBlAGQAXwBsAGkAbQBiAHMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABDAG8AbgBzAHQAcgB1AGMAdAAgAEIAZQB0AGEAXgAoADIAIAAqACAAcwBlAGUAZABfAGwAZQBuACkAIABuAGEAdABpAHYAZQBsAHkAXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABlAC4AZwAuACwAIABpAGYAIABzAGUAZQBkAF8AbABlAG4AIAA9ACAAMQAsACAAdABoAGUAbgAgADEAIABmAG8AbABsAG8AdwBlAGQAIABiAHkAIAB0AHcAbwAgAHoAZQByAG8AIABsAGkAbQBiAHMAOgAgAFYAUwBUAEEAQwBLACgAMAAsACAAMAAsACAAMQApAFwAbgAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYgBlAHQAYQBfADIAbQAsACAAVgBTAFQAQQBDAEsAKABFAFgAUABBAE4ARAAoADAALAAgADIAIAAqACAAbgB1AG0AXwBzAGUAZQBkAF8AbABpAG0AYgBzACwAIAAsACAAMAApACwAIAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAALwAvACAASwBuAHUAdABoACAARABpAHYAaQBzAGkAbwBuACAAeQBpAGUAbABkAHMAIABlAHgAYQBjAHQAIABpAG4AaQB0AGkAYQBsACAAcgBlAGMAaQBwAHIAbwBjAGEAbABcAG4AIAAgACAAIAAgACAAIAAgAHAAYQBjAGsAZQBkAF8AYgBhAHMAZQBjAGEAcwBlAF8AcgBlAHMAdQBsAHQALAAgAEsAbgB1AHQAaABEAGkAdgAoAGwAaQBtAGIAcwBfAGIAZQB0AGEAXwAyAG0ALAAgAGwAaQBtAGIAcwBfAGIAXwB0AG8AcAAsACAAawApACwAXABuACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgAC8ALwAgAEUAeAB0AHIAYQBjAHQAIABRAHUAbwB0AGkAZQBuAHQAIABhAHIAcgBhAHkAIABmAHIAbwBtACAAdABoAGUAIABwAGEAYwBrAGUAZAAgAFYAUwBUAEEAQwBLAFwAbgAgACAAIAAgACAAIAAgACAAbgB1AG0AXwBsAGkAbQBiAHMAXwByACwAIABJAE4ARABFAFgAKABwAGEAYwBrAGUAZABfAGIAYQBzAGUAYwBhAHMAZQBfAHIAZQBzAHUAbAB0ACwAIAAxACwAIAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAEQAUgBPAFAAKABwAGEAYwBrAGUAZABfAGIAYQBzAGUAYwBhAHMAZQBfAHIAZQBzAHUAbAB0ACwAIABuAHUAbQBfAGwAaQBtAGIAcwBfAHIAIAArACAAMQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABbAEkAbgB0AGUAcgBuAGEAbABdACAAQwBvAG0AcAB1AHQAZQBzACAAdABoAGUAIABSAGUAYwBpAHAAcgBvAGMAYQBsACAAcAByAG8AZwByAGUAcwBzAGkAdgBlAGwAeQAgAHMAYwBhAGwAaQBuAGcAIAB1AHAAIAB0AG8AIAB0AGgAZQAgAEQAaQB2AGkAZABlAG4AZAAnAHMAIABwAHIAZQBjAGkAcwBpAG8AbgAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGwAaQBtAGIAcwBfAGIAIABUAGgAZQAgAGQAaQB2AGkAcwBvAHIAIABsAGkAbQBiACAAYQByAHIAYQB5AC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAdABhAHIAZwBlAHQAXwBsAGUAbgAgAFQAaABlACAAbABpAG0AYgAtAGwAZQBuAGcAdABoACAAbwBmACAARABpAHYAaQBkAGUAbgBkACAAQQAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGsAIABUAGgAZQAgAGQAeQBuAGEAbQBpAGMAIABjAGgAdQBuAGsAIABzAGkAegBlACAAYwBvAG4AdABlAHgAdAAuAFwAbgAgACoALwBcAG4ATgBlAHcAdABvAG4AUgBhAHAAaABzAG8AbgBSAGUAYwBpAHAAcgBvAGMAYQBsACAAPQAgAEwAQQBNAEIARABBACgAbABpAG0AYgBzAF8AYgAsACAAdABhAHIAZwBlAHQAXwBsAGUAbgAsACAAawAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABuAHUAbQBfAGwAaQBtAGIAcwBfAGIALAAgAFIATwBXAFMAKABsAGkAbQBiAHMAXwBiACkALABcAG4AIAAgACAAIAAgACAAIAAgAG4AdQBtAF8AcwBlAGUAZABfAGwAaQBtAGIAcwAsACAATQBJAE4AKAAzACwAIABuAHUAbQBfAGwAaQBtAGIAcwBfAGIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AcgBfAHMAZQBlAGQALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAE4AZQB3AHQAbwBuAFIAYQBwAGgAcwBvAG4AUwBlAGUAZAAoAGwAaQBtAGIAcwBfAGIALAAgAGsAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAHIAZQBxAHUAaQByAGUAZABfAGkAdABlAHIAYQB0AGkAbwBuAHMALAAgAE0AQQBYACgAMAAsACAAQwBFAEkATABJAE4ARwAuAE0AQQBUAEgAKABMAE4AKAB0AGEAcgBnAGUAdABfAGwAZQBuACAALwAgAG4AdQBtAF8AcwBlAGUAZABfAGwAaQBtAGIAcwApACAALwAgAEwATgAoADIAKQApACkAIAArACAAMQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAHIAZQBxAHUAaQByAGUAZABfAGkAdABlAHIAYQB0AGkAbwBuAHMAIAA9ACAAMAAsACAAbABpAG0AYgBzAF8AcgBfAHMAZQBlAGQALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABpAHQAZQByAGEAdABpAG8AbgBzACwAIABTAEUAUQBVAEUATgBDAEUAKAByAGUAcQB1AGkAcgBlAGQAXwBpAHQAZQByAGEAdABpAG8AbgBzACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABmAGkAbgBhAGwAXwBwAGEAYwBrAGUAZABfAHMAdABhAHQAZQAsACAAUgBFAEQAVQBDAEUAKABWAFMAVABBAEMASwAoAG4AdQBtAF8AcwBlAGUAZABfAGwAaQBtAGIAcwAsACAAbABpAG0AYgBzAF8AcgBfAHMAZQBlAGQAKQAsACAAaQB0AGUAcgBhAHQAaQBvAG4AcwAsACAATABBAE0AQgBEAEEAKABwAGEAYwBrAGUAZABfAHMAdABhAHQAZQAsACAAaQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAYwB1AHIAcgBlAG4AdABfAGwAZQBuACwAIABJAE4ARABFAFgAKABwAGEAYwBrAGUAZABfAHMAdABhAHQAZQAsACAAMQAsACAAMQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGMAdQByAHIAZQBuAHQAXwByACwAIABEAFIATwBQACgAcABhAGMAawBlAGQAXwBzAHQAYQB0AGUALAAgADEAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbgBlAHgAdABfAGwAZQBuACwAIABNAEkATgAoAGMAdQByAHIAZQBuAHQAXwBsAGUAbgAgACoAIAAyACwAIAB0AGEAcgBnAGUAdABfAGwAZQBuACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAEQAeQBuAGEAbQBpAGMAIABTAGMAYQBsAGkAbgBnACAAUwBoAGkAZgB0ADoAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAEkAZgAgAEIAIABoAGEAcwAgAHAAbABhAHQAZQBhAHUAZQBkACwAIABSACAAbQB1AHMAdAAgAHMAYwBhAGwAZQAgAGIAeQAgADIAKgAoAG4ALQBtACkALgAgAEkAZgAgAEIAIABpAHMAIABnAHIAbwB3AGkAbgBnACwAIABSACAAcwBjAGEAbABlAHMAIABiAHkAIAAoAG4ALQBtACkALgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAYQBjAHQAaQB2AGUAXwBiAF8AbABpAG0AYgBzAF8AYwB1AHIAcgBlAG4AdAAsACAATQBJAE4AKABjAHUAcgByAGUAbgB0AF8AbABlAG4ALAAgAG4AdQBtAF8AbABpAG0AYgBzAF8AYgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGEAYwB0AGkAdgBlAF8AYgBfAGwAaQBtAGIAcwBfAG4AZQB4AHQALAAgAE0ASQBOACgAbgBlAHgAdABfAGwAZQBuACwAIABuAHUAbQBfAGwAaQBtAGIAcwBfAGIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAByAGUAcQB1AGkAcgBlAGQAXwBzAGgAaQBmAHQAXwBsAGkAbQBiAHMALAAgADIAIAAqACAAKABuAGUAeAB0AF8AbABlAG4AIAAtACAAYwB1AHIAcgBlAG4AdABfAGwAZQBuACkAIAAtACAAKABhAGMAdABpAHYAZQBfAGIAXwBsAGkAbQBiAHMAXwBuAGUAeAB0ACAALQAgAGEAYwB0AGkAdgBlAF8AYgBfAGwAaQBtAGIAcwBfAGMAdQByAHIAZQBuAHQAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AcgBfAHAAcgBpAG0AZQAsACAASQBGACgAcgBlAHEAdQBpAHIAZQBkAF8AcwBoAGkAZgB0AF8AbABpAG0AYgBzACAAPgAgADAALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABWAFMAVABBAEMASwAoAEUAWABQAEEATgBEACgAMAAsACAAcgBlAHEAdQBpAHIAZQBkAF8AcwBoAGkAZgB0AF8AbABpAG0AYgBzACwAIAAsACAAMAApACwAIABsAGkAbQBiAHMAXwBjAHUAcgByAGUAbgB0AF8AcgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYwB1AHIAcgBlAG4AdABfAHIAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGIAXwBhAGMAdABpAHYAZQAsACAAVABBAEsARQAoAGwAaQBtAGIAcwBfAGIALAAgAC0AYQBjAHQAaQB2AGUAXwBiAF8AbABpAG0AYgBzAF8AbgBlAHgAdAApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIABQACAAaQBzACAAbgBhAHQAaQB2AGUAbAB5ACAAYQBsAGkAZwBuAGUAZAAgAHQAbwAgADIAKgBuAGUAeAB0AF8AbABlAG4AIABiAGUAYwBhAHUAcwBlACAAbwBmACAAdABoAGUAIABjAG8AcgByAGUAYwB0AGUAZAAgAHMAaABpAGYAdABfAGwAaQBtAGIAcwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AcAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBNAHUAbAAoAGwAaQBtAGIAcwBfAGIAXwBhAGMAdABpAHYAZQAsACAAbABpAG0AYgBzAF8AcgBfAHAAcgBpAG0AZQAsACAAawApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwB0AHcAbwBfAGIAZQB0AGEALAAgAFYAUwBUAEEAQwBLACgARQBYAFAAQQBOAEQAKAAwACwAIAAyACAAKgAgAG4AZQB4AHQAXwBsAGUAbgAsACAALAAgADAAKQAsACAAMgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGUAcgByAG8AcgBfAHQAZQByAG0ALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFUAUwB1AGIAKABsAGkAbQBiAHMAXwB0AHcAbwBfAGIAZQB0AGEALAAgAGwAaQBtAGIAcwBfAHAALAAgAGsAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AbgBlAHgAdABfAHIAXwB1AG4AcwBjAGEAbABlAGQALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFUATQB1AGwAKABsAGkAbQBiAHMAXwByAF8AcAByAGkAbQBlACwAIABsAGkAbQBiAHMAXwBlAHIAcgBvAHIAXwB0AGUAcgBtACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AbgBlAHgAdABfAHIALAAgAEkARgAoAFIATwBXAFMAKABsAGkAbQBiAHMAXwBuAGUAeAB0AF8AcgBfAHUAbgBzAGMAYQBsAGUAZAApACAAPAA9ACAAMgAgACoAIABuAGUAeAB0AF8AbABlAG4ALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAB7ADAAfQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEQAUgBPAFAAKABsAGkAbQBiAHMAXwBuAGUAeAB0AF8AcgBfAHUAbgBzAGMAYQBsAGUAZAAsACAAMgAgACoAIABuAGUAeAB0AF8AbABlAG4AKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAVgBTAFQAQQBDAEsAKABuAGUAeAB0AF8AbABlAG4ALAAgAGwAaQBtAGIAcwBfAG4AZQB4AHQAXwByACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEQAUgBPAFAAKABmAGkAbgBhAGwAXwBwAGEAYwBrAGUAZABfAHMAdABhAHQAZQAsACAAMQApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAAWwBJAG4AdABlAHIAbgBhAGwAXQAgAEgAZQBhAHYAeQB3AGUAaQBnAGgAdAAgAE4AZQB3AHQAbwBuAC0AUgBhAHAAaABzAG8AbgAgAEQAaQB2AGkAcwBpAG8AbgAuAFwAbgAgACoAIABJAG0AcABsAGUAbQBlAG4AdABzACAAcAByAG8AZwByAGUAcwBzAGkAdgBlACAAcwBjAGEAbABpAG4AZwAgAGIAbwB1AG4AZABlAGQAIAB0AG8AIABNAEEAWAAoAGwAZQBuAF8AYQAsACAAbABlAG4AXwBiACkALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABsAGkAbQBiAHMAXwBhACAAVABoAGUAIABkAGkAdgBpAGQAZQBuAGQAIABhAHIAcgBhAHkALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABsAGkAbQBiAHMAXwBiACAAVABoAGUAIABkAGkAdgBpAHMAbwByACAAYQByAHIAYQB5AC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAawAgAFQAaABlACAAZAB5AG4AYQBtAGkAYwAgAGMAaAB1AG4AawAgAHMAaQB6AGUAIABjAG8AbgB0AGUAeAB0AC4AXABuACAAKgAvAFwAbgBOAGUAdwB0AG8AbgBSAGEAcABoAHMAbwBuAEQAaQB2ACAAPQAgAEwAQQBNAEIARABBACgAbABpAG0AYgBzAF8AYQAsACAAbABpAG0AYgBzAF8AYgAsACAAawAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABuAHUAbQBfAGwAaQBtAGIAcwBfAGEALAAgAFIATwBXAFMAKABsAGkAbQBiAHMAXwBhACkALABcAG4AIAAgACAAIAAgACAAIAAgAG4AdQBtAF8AbABpAG0AYgBzAF8AYgAsACAAUgBPAFcAUwAoAGwAaQBtAGIAcwBfAGIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbgB1AG0AXwBsAGkAbQBiAHMAXwB0AGEAcgBnAGUAdAAsACAATQBBAFgAKABuAHUAbQBfAGwAaQBtAGIAcwBfAGEALAAgAG4AdQBtAF8AbABpAG0AYgBzAF8AYgApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAALwAvACAAMQAuACAAQwBhAGwAYwB1AGwAYQB0AGUAIAByAGUAYwBpAHAAcgBvAGMAYQBsACAAUgAgAHMAYwBhAGwAZQBkACAAZAB5AG4AYQBtAGkAYwBhAGwAbAB5ACAAdABvACAAMgAgACoAIAB0AGEAcgBnAGUAdABfAGwAZQBuAFwAbgAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AcgBlAGMAaQBwAHIAbwBjAGEAbAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4ATgBlAHcAdABvAG4AUgBhAHAAaABzAG8AbgBSAGUAYwBpAHAAcgBvAGMAYQBsACgAbABpAG0AYgBzAF8AYgAsACAAbgB1AG0AXwBsAGkAbQBiAHMAXwB0AGEAcgBnAGUAdAAsACAAawApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAALwAvACAAMgAuACAAQQBwAHAAcgBvAHgAaQBtAGEAdABlACAAUQB1AG8AdABpAGUAbgB0ADoAIABRAF8AYQBwAHAAcgBvAHgAIAA9ACAAQQAgACoAIABSACAALwAgAEIAZQB0AGEAXgAoADIAIAAqACAAdABhAHIAZwBlAHQAXwBsAGUAbgApAFwAbgAgACAAIAAgACAAIAAgACAAcgBpAGcAaAB0AF8AcwBoAGkAZgB0AF8AbABpAG0AYgBzACwAIAAyACAAKgAgAG4AdQBtAF8AbABpAG0AYgBzAF8AdABhAHIAZwBlAHQALABcAG4AIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAHEAXwB1AG4AcwBjAGEAbABlAGQALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFUATQB1AGwAKABsAGkAbQBiAHMAXwBhACwAIABsAGkAbQBiAHMAXwByAGUAYwBpAHAAcgBvAGMAYQBsACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAHEAXwBhAHAAcAByAG8AeAAsACAASQBGACgAUgBPAFcAUwAoAGwAaQBtAGIAcwBfAHEAXwB1AG4AcwBjAGEAbABlAGQAKQAgADwAPQAgAHIAaQBnAGgAdABfAHMAaABpAGYAdABfAGwAaQBtAGIAcwAsACAAewAwAH0ALAAgAEQAUgBPAFAAKABsAGkAbQBiAHMAXwBxAF8AdQBuAHMAYwBhAGwAZQBkACwAIAByAGkAZwBoAHQAXwBzAGgAaQBmAHQAXwBsAGkAbQBiAHMAKQApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAALwAvACAAQwBhAGwAYwB1AGwAYQB0AGUAIAB0AGgAZQAgAG0AYQBzAHMAaQB2AGUAIABiAGEAcwBlAGwAaQBuAGUAIABwAHIAbwBkAHUAYwB0ACAAZQB4AGEAYwB0AGwAeQAgAE8ATgBDAEUAXABuACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBwAF8AYgBhAHMAZQBsAGkAbgBlACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAE0AdQBsACgAbABpAG0AYgBzAF8AYgAsACAAbABpAG0AYgBzAF8AcQBfAGEAcABwAHIAbwB4ACwAIABrACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAvAC8AIAAzAC4AIABCAG8AdQBuAGQAZQBkACAARQByAHIAbwByACAAQwBvAHIAcgBlAGMAdABpAG8AbgAgAFMAdwBlAGUAcAAgACgATwBwAHQAaQBtAGkAegBlAGQAIABPACgATgApACAAUwB0AGUAcABwAGkAbgBnACkAXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABTAHQAYQB0AGUAIABwAGEAYwBrAGkAbgBnADoAIABWAFMAVABBAEMASwAoAEwAZQBuAGcAdABoAF8AUQAsACAAUQBfAGwAaQBtAGIAcwAsACAAUABfAGwAaQBtAGIAcwApAFwAbgAgACAAIAAgACAAIAAgACAAaQBuAGkAdABpAGEAbABfAHAAYQBjAGsAZQBkAF8AcwB0AGEAdABlACwAIABWAFMAVABBAEMASwAoAFIATwBXAFMAKABsAGkAbQBiAHMAXwBxAF8AYQBwAHAAcgBvAHgAKQAsACAAbABpAG0AYgBzAF8AcQBfAGEAcABwAHIAbwB4ACwAIABsAGkAbQBiAHMAXwBwAF8AYgBhAHMAZQBsAGkAbgBlACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABTAHcAZQBlAHAAIABEAG8AdwBuADoAIABJAGYAIABQACAAPgAgAEEALAAgAFEAIABpAHMAIAB0AG8AbwAgAGIAaQBnAC4AIABTAHQAZQBwACAAUQAgAGQAbwB3AG4AIABiAHkAIAAxACwAIABhAG4AZAAgAFAAIABkAG8AdwBuACAAYgB5ACAAQgAuAFwAbgAgACAAIAAgACAAIAAgACAAcABhAGMAawBlAGQAXwBzAHQAYQB0AGUAXwBzAHcAZQBwAHQAXwBkAG8AdwBuACwAIABSAEUARABVAEMARQAoAGkAbgBpAHQAaQBhAGwAXwBwAGEAYwBrAGUAZABfAHMAdABhAHQAZQAsACAAewAxADsAIAAyAH0ALAAgAEwAQQBNAEIARABBACgAcABhAGMAawBlAGQAXwBzAHQAYQB0AGUALAAgAGkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGUAbgBfAHEALAAgAEkATgBEAEUAWAAoAHAAYQBjAGsAZQBkAF8AcwB0AGEAdABlACwAIAAxACwAIAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBjAHUAcgByAGUAbgB0AF8AcQAsACAAQwBIAE8ATwBTAEUAUgBPAFcAUwAoAHAAYQBjAGsAZQBkAF8AcwB0AGEAdABlACwAIABTAEUAUQBVAEUATgBDAEUAKABsAGUAbgBfAHEALAAgADEALAAgADIAKQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYwB1AHIAcgBlAG4AdABfAHAALAAgAEQAUgBPAFAAKABwAGEAYwBrAGUAZABfAHMAdABhAHQAZQAsACAAbABlAG4AXwBxACAAKwAgADEAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAEMAbwBtAHAAYQByAGUAKABsAGkAbQBiAHMAXwBjAHUAcgByAGUAbgB0AF8AcAAsACAAbABpAG0AYgBzAF8AYQApACAAPAA9ACAAMAAsACAAcABhAGMAawBlAGQAXwBzAHQAYQB0AGUALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAG4AZQB4AHQAXwBxACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAFMAdQBiACgAbABpAG0AYgBzAF8AYwB1AHIAcgBlAG4AdABfAHEALAAgAHsAMQB9ACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AbgBlAHgAdABfAHAALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFUAUwB1AGIAKABsAGkAbQBiAHMAXwBjAHUAcgByAGUAbgB0AF8AcAAsACAAbABpAG0AYgBzAF8AYgAsACAAawApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFYAUwBUAEEAQwBLACgAUgBPAFcAUwAoAGwAaQBtAGIAcwBfAG4AZQB4AHQAXwBxACkALAAgAGwAaQBtAGIAcwBfAG4AZQB4AHQAXwBxACwAIABsAGkAbQBiAHMAXwBuAGUAeAB0AF8AcAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACkAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAC8ALwAgAFMAdwBlAGUAcAAgAFUAcAA6ACAASQBmACAAUAAgACsAIABCACAAPAA9ACAAQQAsACAAUQAgAGkAcwAgAHQAbwBvACAAcwBtAGEAbABsAC4AIABTAHQAZQBwACAAUQAgAHUAcAAgAGIAeQAgADEALAAgAGEAbgBkACAAUAAgAHUAcAAgAGIAeQAgAEIALgBcAG4AIAAgACAAIAAgACAAIAAgAHAAYQBjAGsAZQBkAF8AcwB0AGEAdABlAF8AcwB3AGUAcAB0AF8AdQBwACwAIABSAEUARABVAEMARQAoAHAAYQBjAGsAZQBkAF8AcwB0AGEAdABlAF8AcwB3AGUAcAB0AF8AZABvAHcAbgAsACAAewAxADsAIAAyAH0ALAAgAEwAQQBNAEIARABBACgAcABhAGMAawBlAGQAXwBzAHQAYQB0AGUALAAgAGkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGUAbgBfAHEALAAgAEkATgBEAEUAWAAoAHAAYQBjAGsAZQBkAF8AcwB0AGEAdABlACwAIAAxACwAIAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBjAHUAcgByAGUAbgB0AF8AcQAsACAAQwBIAE8ATwBTAEUAUgBPAFcAUwAoAHAAYQBjAGsAZQBkAF8AcwB0AGEAdABlACwAIABTAEUAUQBVAEUATgBDAEUAKABsAGUAbgBfAHEALAAgADEALAAgADIAKQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYwB1AHIAcgBlAG4AdABfAHAALAAgAEQAUgBPAFAAKABwAGEAYwBrAGUAZABfAHMAdABhAHQAZQAsACAAbABlAG4AXwBxACAAKwAgADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAG4AZQB4AHQAXwBwAF8AdABlAHMAdAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBBAGQAZAAoAGwAaQBtAGIAcwBfAGMAdQByAHIAZQBuAHQAXwBwACwAIABsAGkAbQBiAHMAXwBiACwAIABrACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBDAG8AbQBwAGEAcgBlACgAbABpAG0AYgBzAF8AbgBlAHgAdABfAHAAXwB0AGUAcwB0ACwAIABsAGkAbQBiAHMAXwBhACkAIAA+ACAAMAAsACAAcABhAGMAawBlAGQAXwBzAHQAYQB0AGUALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAG4AZQB4AHQAXwBxACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAEEAZABkACgAbABpAG0AYgBzAF8AYwB1AHIAcgBlAG4AdABfAHEALAAgAHsAMQB9ACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAVgBTAFQAQQBDAEsAKABSAE8AVwBTACgAbABpAG0AYgBzAF8AbgBlAHgAdABfAHEAKQAsACAAbABpAG0AYgBzAF8AbgBlAHgAdABfAHEALAAgAGwAaQBtAGIAcwBfAG4AZQB4AHQAXwBwAF8AdABlAHMAdAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACkAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAC8ALwAgAEUAeAB0AHIAYQBjAHQAIABGAGkAbgBhAGwAIABRACAAYQBuAGQAIABQAFwAbgAgACAAIAAgACAAIAAgACAAbABlAG4AXwBxACwAIABJAE4ARABFAFgAKABwAGEAYwBrAGUAZABfAHMAdABhAHQAZQBfAHMAdwBlAHAAdABfAHUAcAAsACAAMQAsACAAMQApACwAXABuACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBxACwAIABDAEgATwBPAFMARQBSAE8AVwBTACgAcABhAGMAawBlAGQAXwBzAHQAYQB0AGUAXwBzAHcAZQBwAHQAXwB1AHAALAAgAFMARQBRAFUARQBOAEMARQAoAGwAZQBuAF8AcQAsACAAMQAsACAAMgApACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAHAALAAgAEQAUgBPAFAAKABwAGEAYwBrAGUAZABfAHMAdABhAHQAZQBfAHMAdwBlAHAAdABfAHUAcAAsACAAbABlAG4AXwBxACAAKwAgADEAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAC8ALwAgADQALgAgAEUAeAB0AHIAYQBjAHQAIABUAHIAdQBlACAAUgBlAG0AYQBpAG4AZABlAHIAIABTAGEAZgBlAGwAeQAgACgAQQAgAC0AIABGAGkAbgBhAGwAXwBQACkAXABuACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwByACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAFMAdQBiACgAbABpAG0AYgBzAF8AYQAsACAAbABpAG0AYgBzAF8AcAAsACAAawApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAVgBTAFQAQQBDAEsAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBPAFcAUwAoAGwAaQBtAGIAcwBfAHIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwByACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAHEAXABuACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABbAEkAbgB0AGUAcgBuAGEAbABdACAAVQBuAHMAaQBnAG4AZQBkACAAQgBhAHMAZQAtADEAMAAgAEwAZQBmAHQALQB0AG8ALQBSAGkAZwBoAHQAIABFAHgAcABvAG4AZQBuAHQAaQBhAHQAaQBvAG4ALgBcAG4AIAAqACAARQB2AGEAbAB1AGEAdABlAHMAIAB0AGgAZQAgAGUAeABwAG8AbgBlAG4AdAAgAGkAdABlAHIAYQB0AGkAdgBlAGwAeQAgAHUAcwBpAG4AZwAgAGEAIABwAHIAZQAtAGMAbwBtAHAAdQB0AGUAZAAgADEALQA5ACAAYwBhAGMAaABlAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAbABpAG0AYgBzAF8AYgBhAHMAZQAgAFQAaABlACAAbABpAHQAdABsAGUALQBlAG4AZABpAGEAbgAgAGwAaQBtAGIAIABhAHIAcgBhAHkAIABvAGYAIAB0AGgAZQAgAGIAYQBzAGUALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABlAHgAcABfAHMAdAByAGkAbgBnACAAVABoAGUAIABlAHgAYQBjAHQAIAB0AGUAeAB0ACAAcwB0AHIAaQBuAGcAIABvAGYAIAB0AGgAZQAgAGUAeABwAG8AbgBlAG4AdAAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGsAIABUAGgAZQAgAGQAeQBuAGEAbQBpAGMAIABjAGgAdQBuAGsAIABzAGkAegBlACAAYwBvAG4AdABlAHgAdAAuAFwAbgAgACoALwBcAG4AVQBQAG8AdwAgAD0AIABMAEEATQBCAEQAQQAoAGwAaQBtAGIAcwBfAGIAYQBzAGUALAAgAGUAeABwAG8AbgBlAG4AdABfAHMAdAByAGkAbgBnACwAIABrACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAC8ALwAgAFAAcgBlAC0AYwBvAG0AcAB1AHQAZQAgAHAAbwB3AGUAcgBzACAAMQAgAHQAaAByAG8AdQBnAGgAIAA5AC4AXABuACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBiAGEAcwBlADEALAAgAGwAaQBtAGIAcwBfAGIAYQBzAGUALABcAG4AIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGIAYQBzAGUAMgAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBNAHUAbAAoAGwAaQBtAGIAcwBfAGIAYQBzAGUAMQAsACAAbABpAG0AYgBzAF8AYgBhAHMAZQAxACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGIAYQBzAGUAMwAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBNAHUAbAAoAGwAaQBtAGIAcwBfAGIAYQBzAGUAMgAsACAAbABpAG0AYgBzAF8AYgBhAHMAZQAxACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGIAYQBzAGUANAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBNAHUAbAAoAGwAaQBtAGIAcwBfAGIAYQBzAGUAMgAsACAAbABpAG0AYgBzAF8AYgBhAHMAZQAyACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGIAYQBzAGUANQAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBNAHUAbAAoAGwAaQBtAGIAcwBfAGIAYQBzAGUANAAsACAAbABpAG0AYgBzAF8AYgBhAHMAZQAxACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGIAYQBzAGUANgAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBNAHUAbAAoAGwAaQBtAGIAcwBfAGIAYQBzAGUAMwAsACAAbABpAG0AYgBzAF8AYgBhAHMAZQAzACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGIAYQBzAGUANwAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBNAHUAbAAoAGwAaQBtAGIAcwBfAGIAYQBzAGUANgAsACAAbABpAG0AYgBzAF8AYgBhAHMAZQAxACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGIAYQBzAGUAOAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBNAHUAbAAoAGwAaQBtAGIAcwBfAGIAYQBzAGUANAAsACAAbABpAG0AYgBzAF8AYgBhAHMAZQA0ACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGIAYQBzAGUAOQAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBNAHUAbAAoAGwAaQBtAGIAcwBfAGIAYQBzAGUAOAAsACAAbABpAG0AYgBzAF8AYgBhAHMAZQAxACwAIABrACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIABlAHgAcABvAG4AZQBuAHQAXwBkAGkAZwBpAHQAcwAsACAALQAtAE0ASQBEACgAZQB4AHAAbwBuAGUAbgB0AF8AcwB0AHIAaQBuAGcALAAgAFMARQBRAFUARQBOAEMARQAoAEwARQBOACgAZQB4AHAAbwBuAGUAbgB0AF8AcwB0AHIAaQBuAGcAKQApACwAIAAxACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIABSAEUARABVAEMARQAoADEALAAgAGUAeABwAG8AbgBlAG4AdABfAGQAaQBnAGkAdABzACwAIABMAEEATQBCAEQAQQAoAGwAaQBtAGIAcwBfAGEAYwBjAHUAbQB1AGwAYQB0AG8AcgAsACAAYwB1AHIAcgBlAG4AdABfAGQAaQBnAGkAdAAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAFMAaABvAHIAdAAtAGMAaQByAGMAdQBpAHQAOgAgAFMAawBpAHAAIABjAGEAbABjAHUAbABhAHQAaQBuAGcAIAAxAF4AMQAwACAAZAB1AHIAaQBuAGcAIABsAGUAYQBkAGkAbgBnACAAaQB0AGUAcgBhAHQAaQBvAG4AcwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABpAHMAXwBvAG4AZQAsACAAQQBOAEQAKABSAE8AVwBTACgAbABpAG0AYgBzAF8AYQBjAGMAdQBtAHUAbABhAHQAbwByACkAIAA9ACAAMQAsACAASQBOAEQARQBYACgAbABpAG0AYgBzAF8AYQBjAGMAdQBtAHUAbABhAHQAbwByACwAIAAxACwAIAAxACkAIAA9ACAAMQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAAMQAuACAAUgBhAGkAcwBlACAAQQBjAGMAIAB0AG8AIAB0AGgAZQAgADEAMAB0AGgAIABwAG8AdwBlAHIAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYQBjAGMAXwAxADAALAAgAEkARgAoAGkAcwBfAG8AbgBlACwAIABsAGkAbQBiAHMAXwBhAGMAYwB1AG0AdQBsAGEAdABvAHIALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGEAYwBjAF8AMgAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBNAHUAbAAoAGwAaQBtAGIAcwBfAGEAYwBjAHUAbQB1AGwAYQB0AG8AcgAsACAAbABpAG0AYgBzAF8AYQBjAGMAdQBtAHUAbABhAHQAbwByACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYQBjAGMAXwA0ACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAE0AdQBsACgAbABpAG0AYgBzAF8AYQBjAGMAXwAyACwAIABsAGkAbQBiAHMAXwBhAGMAYwBfADIALAAgAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBhAGMAYwBfADgALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFUATQB1AGwAKABsAGkAbQBiAHMAXwBhAGMAYwBfADQALAAgAGwAaQBtAGIAcwBfAGEAYwBjAF8ANAAsACAAawApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFUATQB1AGwAKABsAGkAbQBiAHMAXwBhAGMAYwBfADgALAAgAGwAaQBtAGIAcwBfAGEAYwBjAF8AMgAsACAAawApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgADIALgAgAE0AdQBsAHQAaQBwAGwAeQAgAGIAeQAgAHQAaABlACAAYwBvAHIAcgBlAHMAcABvAG4AZABpAG4AZwAgAGMAYQBjAGgAZQBkACAAdgBhAGwAdQBlAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEkARgAoAGMAdQByAHIAZQBuAHQAXwBkAGkAZwBpAHQAIAA9ACAAMAAsACAAbABpAG0AYgBzAF8AYQBjAGMAXwAxADAALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGMAYQBjAGgAZQBfAG0AdQBsAHQAaQBwAGwAaQBlAHIALAAgAEMASABPAE8AUwBFACgAYwB1AHIAcgBlAG4AdABfAGQAaQBnAGkAdAAsACAAbABpAG0AYgBzAF8AYgBhAHMAZQAxACwAIABsAGkAbQBiAHMAXwBiAGEAcwBlADIALAAgAGwAaQBtAGIAcwBfAGIAYQBzAGUAMwAsACAAbABpAG0AYgBzAF8AYgBhAHMAZQA0ACwAIABsAGkAbQBiAHMAXwBiAGEAcwBlADUALAAgAGwAaQBtAGIAcwBfAGIAYQBzAGUANgAsACAAbABpAG0AYgBzAF8AYgBhAHMAZQA3ACwAIABsAGkAbQBiAHMAXwBiAGEAcwBlADgALAAgAGwAaQBtAGIAcwBfAGIAYQBzAGUAOQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEkARgAoAGkAcwBfAG8AbgBlACwAIABsAGkAbQBiAHMAXwBjAGEAYwBoAGUAXwBtAHUAbAB0AGkAcABsAGkAZQByACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAE0AdQBsACgAbABpAG0AYgBzAF8AYQBjAGMAXwAxADAALAAgAGwAaQBtAGIAcwBfAGMAYQBjAGgAZQBfAG0AdQBsAHQAaQBwAGwAaQBlAHIALAAgAGsAKQApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABbAEkAbgB0AGUAcgBuAGEAbABdACAAVQBuAHMAaQBnAG4AZQBkACAASQBuAHQAZQBnAGUAcgAgAFMAcQB1AGEAcgBlACAAUgBvAG8AdAAgAHUAcwBpAG4AZwAgAE4AZQB3AHQAbwBuACcAcwAgAE0AZQB0AGgAbwBkAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAbABpAG0AYgBzAF8AcgBhAGQAaQBjAGEAbgBkAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAbABpAG0AYgBzAF8AaQBuAGkAdABpAGEAbABfAHgAIABPAHYAZQByAC0AZQBzAHQAaQBtAGEAdABlAGQAIABzAGUAZQBkACAAYQByAHIAYQB5AC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAawAgAFQAaABlACAAZAB5AG4AYQBtAGkAYwAgAGMAaAB1AG4AawAgAHMAaQB6AGUAIABjAG8AbgB0AGUAeAB0AC4AXABuACAAKgAvAFwAbgBVAFMAcQByAHQAIAA9ACAATABBAE0AQgBEAEEAKABsAGkAbQBiAHMAXwByAGEAZABpAGMAYQBuAGQALAAgAGwAaQBtAGIAcwBfAGkAbgBpAHQAaQBhAGwAXwB4ACwAIABrACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQB4AGkAbQB1AG0AXwBpAHQAZQByAGEAdABpAG8AbgBzACwAIAAzADUALABcAG4AXABuACAAIAAgACAAIAAgACAAIABmAGkAbgBhAGwAXwBwAGEAYwBrAGUAZABfAHMAdABhAHQAZQAsACAAUgBFAEQAVQBDAEUAKABWAFMAVABBAEMASwAoADAALAAgAGwAaQBtAGIAcwBfAGkAbgBpAHQAaQBhAGwAXwB4ACkALAAgAFMARQBRAFUARQBOAEMARQAoAG0AYQB4AGkAbQB1AG0AXwBpAHQAZQByAGEAdABpAG8AbgBzACkALAAgAEwAQQBNAEIARABBACgAcABhAGMAawBlAGQAXwBzAHQAYQB0AGUALAAgAGkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABoAGEAcwBfAGMAbwBuAHYAZQByAGcAZQBkACwAIABJAE4ARABFAFgAKABwAGEAYwBrAGUAZABfAHMAdABhAHQAZQAsACAAMQAsACAAMQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYwB1AHIAcgBlAG4AdABfAHgALAAgAEQAUgBPAFAAKABwAGEAYwBrAGUAZABfAHMAdABhAHQAZQAsACAAMQApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEkARgAoAGgAYQBzAF8AYwBvAG4AdgBlAHIAZwBlAGQALAAgAHAAYQBjAGsAZQBkAF8AcwB0AGEAdABlACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIAAxAC4AIABEAGkAdgBpAHMAaQBvAG4AOgAgAG4AIAAvACAAeABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcABhAGMAawBlAGQAXwBkAGkAdgBpAHMAaQBvAG4AXwByAGUAcwB1AGwAdAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4ARABpAHYAUgBvAHUAdABlAHIAKABsAGkAbQBiAHMAXwByAGEAZABpAGMAYQBuAGQALAAgAGwAaQBtAGIAcwBfAGMAdQByAHIAZQBuAHQAXwB4ACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbgB1AG0AXwBsAGkAbQBiAHMAXwByACwAIABJAE4ARABFAFgAKABwAGEAYwBrAGUAZABfAGQAaQB2AGkAcwBpAG8AbgBfAHIAZQBzAHUAbAB0ACwAIAAxACwAIAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AcQAsACAARABSAE8AUAAoAHAAYQBjAGsAZQBkAF8AZABpAHYAaQBzAGkAbwBuAF8AcgBlAHMAdQBsAHQALAAgAG4AdQBtAF8AbABpAG0AYgBzAF8AcgAgACsAIAAxACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgADIALgAgAEEAZABkAGkAdABpAG8AbgA6ACAAeAAgACsAIAAoAG4AIAAvACAAeAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBzAHUAbQBfAHgAcQAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBBAGQAZAAoAGwAaQBtAGIAcwBfAGMAdQByAHIAZQBuAHQAXwB4ACwAIABsAGkAbQBiAHMAXwBxACwAIABrACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgADMALgAgAEgAYQBsAHYAaQBuAGcAOgAgACgAeAAgACsAIAAoAG4AIAAvACAAeAApACkAIAAvACAAMgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAASwBuAHUAdABoAEQAaQB2ACAAaQBuAGgAZQByAGUAbgB0AGwAeQAgAHMAdQBwAHAAbwByAHQAcwAgAHMAYwBhAGwAYQByACAAZABpAHYAaQBzAG8AcgBzACAAdwBpAHQAaAAgAHoAZQByAG8AIABvAHYAZQByAGgAZQBhAGQAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHAAYQBjAGsAZQBkAF8AaABhAGwAZgBfAHIAZQBzAHUAbAB0ACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBLAG4AdQB0AGgARABpAHYAKABsAGkAbQBiAHMAXwBzAHUAbQBfAHgAcQAsACAAewAyAH0ALAAgAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABuAHUAbQBfAGwAaQBtAGIAcwBfAGgAYQBsAGYAZQBkACwAIABJAE4ARABFAFgAKABwAGEAYwBrAGUAZABfAGgAYQBsAGYAXwByAGUAcwB1AGwAdAAsACAAMQAsACAAMQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAG4AZQB4AHQAXwB4ACwAIABEAFIATwBQACgAcABhAGMAawBlAGQAXwBoAGEAbABmAF8AcgBlAHMAdQBsAHQALAAgAG4AdQBtAF8AbABpAG0AYgBzAF8AaABhAGwAZgBlAGQAIAArACAAMQApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIAA0AC4AIABDAG8AbgB2AGUAcgBnAGUAbgBjAGUAIABDAGgAZQBjAGsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGMAbwBuAHYAZQByAGcAZQBuAGMAZQBfAGMAbwBtAHAAYQByAGkAcwBvAG4ALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFUAQwBvAG0AcABhAHIAZQAoAGwAaQBtAGIAcwBfAG4AZQB4AHQAXwB4ACwAIABsAGkAbQBiAHMAXwBjAHUAcgByAGUAbgB0AF8AeAApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIABOAGUAdwB0AG8AbgAnAHMAIABtAGUAdABoAG8AZAAgAGMAbwBuAHYAZQByAGcAZQBzACAAbwBuACAAdABoAGUAIABmAGwAbwBvAHIAIAByAG8AbwB0ACwAIABhAG4AZAAgAHMAdABhAGIAaQBsAGkAegBlAHMAIABvAHIAIABvAHMAYwBpAGwAbABhAHQAZQBzACAAdQBwACAAYgB5ACAAMQAuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIABUAGgAZQByAGUAZgBvAHIAZQAsACAAaQBmACAAeABfAG4AZQB4AHQAIAA+AD0AIABjAHUAcgByAF8AeAAsACAAdABoAGUAIABhAGwAZwBvAHIAaQB0AGgAbQAgAGgAYQBzACAAYwBvAG4AdgBlAHIAZwBlAGQALgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgAYwBvAG4AdgBlAHIAZwBlAG4AYwBlAF8AYwBvAG0AcABhAHIAaQBzAG8AbgAgAD4APQAgADAALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABWAFMAVABBAEMASwAoADEALAAgAGwAaQBtAGIAcwBfAGMAdQByAHIAZQBuAHQAXwB4ACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABWAFMAVABBAEMASwAoADAALAAgAGwAaQBtAGIAcwBfAG4AZQB4AHQAXwB4ACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAApACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIABEAFIATwBQACgAZgBpAG4AYQBsAF8AcABhAGMAawBlAGQAXwBzAHQAYQB0AGUALAAgADEAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAAWwBJAG4AdABlAHIAbgBhAGwAXQAgAEcAZQBuAGUAcgBhAHQAZQBzACAAYQAgADEARAAgAHYAZQByAHQAaQBjAGEAbAAgAGEAcgByAGEAeQAgAG8AZgAgAGEAbABsACAAcAByAGkAbQBlACAAbgB1AG0AYgBlAHIAcwAgAHUAcAAgAHQAbwAgAG4ALgBcAG4AIAAqACAARQB2AGEAbAB1AGEAdABlAHMAIABwAHUAcgBlAGwAeQAgAGkAbgAgAG4AYQB0AGkAdgBlACAAQwArACsAIAB1AHMAaQBuAGcAIABhACAAZAB5AG4AYQBtAGkAYwAgAHMAaQBlAHYAZQAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAG4AIABUAGgAZQAgAHUAcABwAGUAcgAgAGIAbwB1AG4AZAAgAGkAbgB0AGUAZwBlAHIAIAAoAGEAcwBzAHUAbQBlAGQAIAA8AD0AIAA5ADIANwAzACkALgBcAG4AIAAqAC8AXABuAE4AYQB0AGkAdgBlAFAAcgBpAG0AZQBzACAAPQAgAEwAQQBNAEIARABBACgAbgAsAFwAbgAgACAAIAAgAEkARgAoAG4AIAA8ACAAMgAsACAAIwBOAFUATQAhACwAXABuACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABjAGEAbgBkAGkAZABhAHQAZQBfAHMAZQBxAHUAZQBuAGMAZQAsACAAUwBFAFEAVQBFAE4AQwBFACgAbgAgAC0AIAAxACwAIAAxACwAIAAyACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABjAGEAbgBkAGkAZABhAHQAZQBfAHMAZQBxAHUAZQBuAGMAZQAsACAATQBBAFAAKABjAGEAbgBkAGkAZABhAHQAZQBfAHMAZQBxAHUAZQBuAGMAZQAsACAATABBAE0AQgBEAEEAKABjAHUAcgByAGUAbgB0AF8AYwBhAG4AZABpAGQAYQB0AGUALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AaQB0ACwAIABJAE4AVAAoAFMAUQBSAFQAKABjAHUAcgByAGUAbgB0AF8AYwBhAG4AZABpAGQAYQB0AGUAKQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABsAGkAbQBpAHQAIAA8ACAAMgAsACAAVABSAFUARQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEkATgAoAE0ATwBEACgAYwB1AHIAcgBlAG4AdABfAGMAYQBuAGQAaQBkAGEAdABlACwAIABTAEUAUQBVAEUATgBDAEUAKABsAGkAbQBpAHQAIAAtACAAMQAsACAAMQAsACAAMgApACkAKQAgAD4AIAAwAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAApACkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFsASQBuAHQAZQByAG4AYQBsAF0AIABVAG4AcwBhAGYAZQAsACAAaABpAGcAaAAtAHAAZQByAGYAbwByAG0AYQBuAGMAZQAgAHQAZQB4AHQAIABtAHUAbAB0AGkAcABsAGkAYwBhAHQAaQBvAG4AIABmAG8AcgAgAG4AbwByAG0AYQBsAGkAcwBlAGQALAAgAHAAbwBzAGkAdABpAHYAZQAgAEIAaQBnAEkAbgB0ACAAcwB0AHIAaQBuAGcAcwAuAFwAbgAgACoAIABCAHkAcABhAHMAcwBlAHMAIABMAGEAeQBlAHIAIAAwACAAdgBhAGwAaQBkAGEAdABpAG8AbgAuACAASQBtAHAAbABlAG0AZQBuAHQAcwAgAHMAdAByAGkAYwB0ACAAcwBoAG8AcgB0AC0AYwBpAHIAYwB1AGkAdABzACAAZgBvAHIAIABwAGEAZABkAGkAbgBnACAAbwBwAHQAaQBtAGkAegBhAHQAaQBvAG4ALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABuAG8AcgBtAF8AYQBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABuAG8AcgBtAF8AYgBcAG4AIAAqAC8AXABuAFUAVABlAHgAdABNAHUAbAAgAD0AIABMAEEATQBCAEQAQQAoAG4AbwByAG0AXwBhACwAIABuAG8AcgBtAF8AYgAsAFwAbgAgACAAIAAgAEkARgAoAE8AUgAoAG4AbwByAG0AXwBhACAAPQAgAFwAIgAwAFwAIgAsACAAbgBvAHIAbQBfAGIAIAA9ACAAXAAiADAAXAAiACkALAAgAFwAIgAwAFwAIgAsAFwAbgAgACAAIAAgAEkARgAoAG4AbwByAG0AXwBhACAAPQAgAFwAIgAxAFwAIgAsACAAbgBvAHIAbQBfAGIALABcAG4AIAAgACAAIABJAEYAKABuAG8AcgBtAF8AYgAgAD0AIABcACIAMQBcACIALAAgAG4AbwByAG0AXwBhACwAXABuACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGUAbgBfAGEALAAgAEwARQBOACgAbgBvAHIAbQBfAGEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGUAbgBfAGIALAAgAEwARQBOACgAbgBvAHIAbQBfAGIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABrACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBTAGEAZgBlAEsAKABcACIATQBVAEwAXAAiACwAIABNAEkATgAoAGwAZQBuAF8AYQAsACAAbABlAG4AXwBiACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYQAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwBwAGwAaQB0ACgAbgBvAHIAbQBfAGEALAAgAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBiACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBTAHAAbABpAHQAKABuAG8AcgBtAF8AYgAsACAAawApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABmAGkAbgBhAGwAXwBsAGkAbQBiAHMALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFUATQB1AGwAKABsAGkAbQBiAHMAXwBhACwAIABsAGkAbQBiAHMAXwBiACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAE0AZQByAGcAZQAoAGYAaQBuAGEAbABfAGwAaQBtAGIAcwAsACAAawApAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApACkAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFsASQBuAHQAZQByAG4AYQBsAF0AIABWAGUAYwB0AG8AcgBpAHoAZQBkACAAbABvAGcAYQByAGkAdABoAG0AaQBjACAAcAByAG8AZAB1AGMAdAAgAG8AZgAgAGEAbgAgAGEAcgByAGEAeQAgAG8AZgAgAEIAaQBnAEkAbgB0ACAAcwB0AHIAaQBuAGcAcwAuAFwAbgAgACoAIABSAGUAYwB1AHIAcwBpAHYAZQBsAHkAIABjAHUAdABzACAAdABoAGUAIABhAHIAcgBhAHkAIABpAG4AIABoAGEAbABmACAAdABvACAAYgB5AHAAYQBzAHMAIABSAEUARABVAEMARQAgAHMAZQBxAHUAZQBuAHQAaQBhAGwAIABtAGUAbQBvAHIAeQAgAGEAbABsAG8AYwBhAHQAaQBvAG4AcwAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGEAcgByAF8AcwB0AHIAaQBuAGcAcwAgAEEAIAAxAEQAIAB2AGUAcgB0AGkAYwBhAGwAIABhAHIAcgBhAHkAIABvAGYAIABCAGkAZwBJAG4AdAAgAHMAdAByAGkAbgBnAHMALgBcAG4AIAAqAC8AXABuAFQAZQB4AHQAVAByAGUAZQBQAHIAbwBkACAAPQAgAEwAQQBNAEIARABBACgAYQByAHIAXwBzAHQAcgBpAG4AZwBzACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG4AdQBtAF8AZQBsAGUAbQBlAG4AdABzACwAIABSAE8AVwBTACgAYQByAHIAXwBzAHQAcgBpAG4AZwBzACkALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAbgB1AG0AXwBlAGwAZQBtAGUAbgB0AHMAIAA9ACAAMQAsACAASQBOAEQARQBYACgAYQByAHIAXwBzAHQAcgBpAG4AZwBzACwAIAAxACwAIAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIABSAGUAcwBoAGEAcABlACAAYQByAHIAYQB5ACAAaQBuAHQAbwAgAHAAYQBpAHIAcwAuACAATwBkAGQALQBsAGUAbgBnAHQAaAAgAGEAcgByAGEAeQBzACAAYQByAGUAIABzAGEAZgBlAGwAeQAgAHAAYQBkAGQAZQBkACAAdwBpAHQAaAAgAHQAaABlACAAbQB1AGwAdABpAHAAbABpAGMAYQB0AGkAdgBlACAAaQBkAGUAbgB0AGkAdAB5ACAAXAAiADEAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHAAYQBpAHIAZQBkAF8AcwB0AHIAaQBuAGcAcwAsACAAVwBSAEEAUABSAE8AVwBTACgAYQByAHIAXwBzAHQAcgBpAG4AZwBzACwAIAAyACwAIABcACIAMQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAFYAZQBjAHQAbwByAGkAegBlAGQAIABtAHUAbAB0AGkAcABsAGkAYwBhAHQAaQBvAG4AIABhAGMAcgBvAHMAcwAgAGEAbABsACAAcABhAGkAcgBzACAAcwBpAG0AdQBsAHQAYQBuAGUAbwB1AHMAbAB5AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHIAZQBkAHUAYwBlAGQAXwBhAHIAcgBhAHkALAAgAEIAWQBSAE8AVwAoAHAAYQBpAHIAZQBkAF8AcwB0AHIAaQBuAGcAcwAsACAATABBAE0AQgBEAEEAKAByAG8AdwAsACAAVQBUAGUAeAB0AE0AdQBsACgASQBOAEQARQBYACgAcgBvAHcALAAgADEALAAgADEAKQAsACAASQBOAEQARQBYACgAcgBvAHcALAAgADEALAAgADIAKQApACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAFMAaABhAGwAbABvAHcAIAByAGUAYwB1AHIAcwBpAG8AbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBUAGUAeAB0AFQAcgBlAGUAUAByAG8AZAAoAHIAZQBkAHUAYwBlAGQAXwBhAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFsASQBuAHQAZQByAG4AYQBsAF0AIABDAGEAbABjAHUAbABhAHQAZQBzACAAdABoAGUAIABlAHgAcABvAG4AZQBuAHQAIABmAG8AcgAgAGEAbgAgAGEAcgByAGEAeQAgAG8AZgAgAHAAcgBpAG0AZQBzACAAaQBuACAAdABoAGUAIABTAHcAaQBuAGcAIAB0AGUAcgBtACAAbwBmACAAYQAgAGYAYQBjAHQAbwByAGkAYQBsAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAbgAgAFQAaABlACAAYwB1AHIAcgBlAG4AdAAgAGYAYQBjAHQAbwByAGkAYQBsACAAbQBhAGcAbgBpAHQAdQBkAGUAIAAoADwAPQAgADkAMgA3ADMAKQAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAHAAcgBpAG0AZQBzACAAQQAgAHYAZQByAHQAaQBjAGEAbAAgAGEAcgByAGEAeQAgAG8AZgAgAHAAcgBpAG0AZQAgAG4AdQBtAGIAZQByAHMAIAAoADwAPQAgAG4AKQAuAFwAbgAgACoALwBcAG4ATgBhAHQAaQB2AGUAUwB3AGkAbgBnAEUAeABwAG8AbgBlAG4AdABzACAAPQAgAEwAQQBNAEIARABBACgAbgAsACAAcAByAGkAbQBlAHMALABcAG4AIAAgACAAIABNAEEAUAAoAHAAcgBpAG0AZQBzACwAIABMAEEATQBCAEQAQQAoAHAALABcAG4AIAAgACAAIAAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAG0AYQB4AF8AcABvAHcAZQByAF8AawAsACAASQBOAFQAKABMAE8ARwAoAG4ALAAgAHAAKQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHAAcgBpAG0AZQBfAHAAbwB3AGUAcgBzACwAIABwACAAXgAgAFMARQBRAFUARQBOAEMARQAoAG0AYQB4AF8AcABvAHcAZQByAF8AawApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFMAVQBNACgATQBPAEQAKABJAE4AVAAoAG4AIAAvACAAcAByAGkAbQBlAF8AcABvAHcAZQByAHMAKQAsACAAMgApACkAXABuACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFsASQBuAHQAZQByAG4AYQBsAF0AIABDAGEAbABjAHUAbABhAHQAZQBzACAAdABoAGUAIABtAGEAcwBzAGkAdgBlACAAQgBpAGcASQBuAHQAIABzAHQAcgBpAG4AZwAgAGYAbwByACAAdABoAGUAIABTAHcAaQBuAGcAIAB0AGUAcgBtACAAbwBmACAAYQAgAGYAYQBjAHQAbwByAGkAYQBsAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAbgAgAFQAaABlACAAYwB1AHIAcgBlAG4AdAAgAGYAYQBjAHQAbwByAGkAYQBsACAAbQBhAGcAbgBpAHQAdQBkAGUALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIAB0AGkAZQByAF8AcAByAGkAbQBlAHMAIABBACAAdgBlAHIAdABpAGMAYQBsACAAYQByAHIAYQB5ACAAbwBmACAAcAByAGkAbQBlACAAbgB1AG0AYgBlAHIAcwAgACgAPAA9ACAAbgApAC4AXABuACAAKgAvAFwAbgBTAHcAaQBuAGcAVABlAHIAbQAgAD0AIABMAEEATQBCAEQAQQAoAG4ALAAgAHQAaQBlAHIAXwBwAHIAaQBtAGUAcwAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABzAHcAaQBuAGcAXwBlAHgAcABvAG4AZQBuAHQAcwAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4ATgBhAHQAaQB2AGUAUwB3AGkAbgBnAEUAeABwAG8AbgBlAG4AdABzACgAbgAsACAAdABpAGUAcgBfAHAAcgBpAG0AZQBzACkALABcAG4AIAAgACAAIAAgACAAIAAgAGgAYQBzAF8AbgBhAHQAaQB2AGUAXwBlAHgAcABvAG4AZQBuAHQALAAgAHMAdwBpAG4AZwBfAGUAeABwAG8AbgBlAG4AdABzACAAPgAgADAALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAALwAvACAASQBmACAAYQBsAGwAIABlAHgAcABvAG4AZQBuAHQAcwAgAGEAcgBlACAAMAAsACAAdABoAGUAIABzAHcAaQBuAGcAIAB0AGUAcgBtACAAaQBzACAAMQAuAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAQQBOAEQAKABOAE8AVAAoAGgAYQBzAF8AbgBhAHQAaQB2AGUAXwBlAHgAcABvAG4AZQBuAHQAKQApACwAIABcACIAMQBcACIALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABhAGMAdABpAHYAZQBfAHAAcgBpAG0AZQBzACwAIABGAEkATABUAEUAUgAoAHQAaQBlAHIAXwBwAHIAaQBtAGUAcwAsACAAaABhAHMAXwBuAGEAdABpAHYAZQBfAGUAeABwAG8AbgBlAG4AdAApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAYQBjAHQAaQB2AGUAXwBlAHgAcABvAG4AZQBuAHQAcwAsACAARgBJAEwAVABFAFIAKABzAHcAaQBuAGcAXwBlAHgAcABvAG4AZQBuAHQAcwAsACAAaABhAHMAXwBuAGEAdABpAHYAZQBfAGUAeABwAG8AbgBlAG4AdAApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAZQB2AGEAbAB1AHQAYQB0AGUAZABfAHAAcgBpAG0AZQBfAHAAbwB3AGUAcgBzACwAIABNAEEAUAAoAGEAYwB0AGkAdgBlAF8AcAByAGkAbQBlAHMALAAgAGEAYwB0AGkAdgBlAF8AZQB4AHAAbwBuAGUAbgB0AHMALAAgAEwAQQBNAEIARABBACgAcAAsACAAZQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABlACAAPQAgADEALAAgAHAAIAAmACAAXAAiAFwAIgAsACAAQgBpAGcASQBuAHQALgBQAG8AdwAoAHAAIAAmACAAXAAiAFwAIgAsACAAZQAgACYAIABcACIAXAAiACkAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBUAGUAeAB0AFQAcgBlAGUAUAByAG8AZAAoAGUAdgBhAGwAdQB0AGEAdABlAGQAXwBwAHIAaQBtAGUAXwBwAG8AdwBlAHIAcwApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAAWwBJAG4AdABlAHIAbgBhAGwAXQAgAFIAZQBjAHUAcgBzAGkAdgBlACAAdABvAHAALQBkAG8AdwBuACAATABBAE0AQgBEAEEAIABjAGEAbABjAHUAbABhAHQAaQBuAGcAIAB0AGgAZQAgAFAAcgBpAG0AZQAgAFMAdwBpAG4AZwAgAGYAYQBjAHQAbwByAGkAYQBsAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAbgAgAFQAaABlACAAYwB1AHIAcgBlAG4AdAAgAGYAYQBjAHQAbwByAGkAYQBsACAAbQBhAGcAbgBpAHQAdQBkAGUALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABnAGwAbwBiAGEAbABfAHAAcgBpAG0AZQBzACAAVABoAGUAIAB1AG4AaQBmAGkAZQBkACAAdgBlAHIAdABpAGMAYQBsACAAYQByAHIAYQB5ACAAbwBmACAAYQBsAGwAIABwAHIAaQBtAGUAcwAgAHUAcAAgAHQAbwAgAHQAaABlACAAdABhAHIAZwBlAHQAIABmAGEAYwB0AG8AcgBpAGEAbAAuAFwAbgAgACoALwBcAG4AUAByAGkAbQBlAFMAdwBpAG4AZwBLAGUAcgBuAGUAbAAgAD0AIABMAEEATQBCAEQAQQAoAG4ALAAgAGcAbABvAGIAYQBsAF8AcAByAGkAbQBlAHMALABcAG4AIAAgACAAIABJAEYAKABuACAAPAAgADIALAAgAFwAIgAxAFwAIgAsAFwAbgAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAZgBsAG8AbwByAF8AaABhAGwAZgBfAG4ALAAgAEkATgBUACgAbgAgAC8AIAAyACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAZgBhAGMAdABvAHIAaQBhAGwAXwBoAGEAbABmAF8AbgAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUAByAGkAbQBlAFMAdwBpAG4AZwBLAGUAcgBuAGUAbAAoAGYAbABvAG8AcgBfAGgAYQBsAGYAXwBuACwAIABnAGwAbwBiAGEAbABfAHAAcgBpAG0AZQBzACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAFMAcQB1AGEAcgBlACAAdABoAGUAIABoAGEAbABmAHcAYQB5ACAAcABvAGkAbgB0ACAAdQBzAGkAbgBnACAAdABoAGUAIAB1AG4AcwBhAGYAZQAgAGsAZQByAG4AZQBsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABzAHEAdQBhAHIAZQBkAF8AaABhAGwAZgBfAGYAYQBjAHQAbwByAGkAYQBsACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAFQAZQB4AHQATQB1AGwAKABmAGEAYwB0AG8AcgBpAGEAbABfAGgAYQBsAGYAXwBuACwAIABmAGEAYwB0AG8AcgBpAGEAbABfAGgAYQBsAGYAXwBuACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAEkAcwBvAGwAYQB0AGUAIAB0AGgAZQAgAHAAcgBpAG0AZQBzACAAbgBlAGUAZABlAGQAIABmAG8AcgAgAHQAaABpAHMAIAB0AGkAZQByACAAYQBuAGQAIABjAGEAbABjAHUAbABhAHQAZQAgAHQAaABlACAAcwB3AGkAbgBnACAAdABlAHIAbQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAYQBwAHAAbABpAGMAYQBiAGwAZQBfAHQAaQBlAHIAXwBwAHIAaQBtAGUAcwAsACAARgBJAEwAVABFAFIAKABnAGwAbwBiAGEAbABfAHAAcgBpAG0AZQBzACwAIABnAGwAbwBiAGEAbABfAHAAcgBpAG0AZQBzACAAPAA9ACAAbgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHMAdAByAF8AcwB3AGkAbgBnAF8AdABlAHIAbQAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwB3AGkAbgBnAFQAZQByAG0AKABuACwAIABhAHAAcABsAGkAYwBhAGIAbABlAF8AdABpAGUAcgBfAHAAcgBpAG0AZQBzACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFUAVABlAHgAdABNAHUAbAAoAHMAcQB1AGEAcgBlAGQAXwBoAGEAbABmAF8AZgBhAGMAdABvAHIAaQBhAGwALAAgAHMAdAByAF8AcwB3AGkAbgBnAF8AdABlAHIAbQApAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAAWwBJAG4AdABlAHIAbgBhAGwAXQAgAFIAZQBjAHUAcgBzAGkAdgBlACAAdABvAHUAcgBuAGEAbQBlAG4AdAAgAHQAcgBlAGUAIABmAG8AcgAgAE0AaQBuAC8ATQBhAHgAIABlAHYAYQBsAHUAYQB0AGkAbwBuAHMALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABjAG8AbAAgAEEAIAAxAEQAIAB2AGUAcgB0AGkAYwBhAGwAIABhAHIAcgBhAHkAIABvAGYAIABuAG8AcgBtAGEAbABpAHoAZQBkACAAQgBpAGcASQBuAHQAIABzAHQAcgBpAG4AZwBzAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAbQBvAGQAZQAgADEAIABmAG8AcgAgAE0AYQB4AGkAbQB1AG0ALAAgAC0AMQAgAGYAbwByACAATQBpAG4AaQBtAHUAbQAuAFwAbgAgACoALwBcAG4AVAByAGUAZQBDAG8AbQBwAGEAcgBlACAAPQAgAEwAQQBNAEIARABBACgAcwB0AHIAXwBuAG8AcgBtAHMALAAgAGMAbwBtAHAAYQByAGkAcwBvAG4AXwBtAG8AZABlACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG4AdQBtAF8AcgBvAHcAcwAsACAAUgBPAFcAUwAoAHMAdAByAF8AbgBvAHIAbQBzACkALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAbgB1AG0AXwByAG8AdwBzACAAPQAgADEALAAgAEkATgBEAEUAWAAoAHMAdAByAF8AbgBvAHIAbQBzACwAIAAxACwAIAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAB0AG8AdQByAG4AYQBtAGUAbgB0AF8AcABhAGkAcgBzACwAIABXAFIAQQBQAFIATwBXAFMAKABzAHQAcgBfAG4AbwByAG0AcwAsACAAMgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAYwBvAG0AcABlAHQAaQB0AG8AcgBzAF8AYQAsACAAVABBAEsARQAoAHQAbwB1AHIAbgBhAG0AZQBuAHQAXwBwAGEAaQByAHMALAAgACwAIAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABjAG8AbQBwAGUAdABpAHQAbwByAHMAXwBiACwAIABUAEEASwBFACgAdABvAHUAcgBuAGEAbQBlAG4AdABfAHAAYQBpAHIAcwAsACAALAAgAC0AMQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcgBvAHUAbgBkAF8AdwBpAG4AbgBlAHIAcwAsACAATQBBAFAAKABjAG8AbQBwAGUAdABpAHQAbwByAHMAXwBhACwAIABjAG8AbQBwAGUAdABpAHQAbwByAHMAXwBiACwAIABMAEEATQBCAEQAQQAoAGEALAAgAGIALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEkARgAoAEkAUwBOAEEAKABiACkALAAgAGEALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABjAG8AbQBwAGEAcgBpAHMAbwBuAF8AcgBlAHMAdQBsAHQALAAgAEIAaQBnAEkAbgB0AC4AQwBvAG0AcABhAHIAZQAoAGEALAAgAGIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEkARgAoAGMAbwBtAHAAYQByAGkAcwBvAG4AXwByAGUAcwB1AGwAdAAgACoAIABjAG8AbQBwAGEAcgBpAHMAbwBuAF8AbQBvAGQAZQAgAD4APQAgADAALAAgAGEALAAgAGIAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVAByAGUAZQBDAG8AbQBwAGEAcgBlACgAcgBvAHUAbgBkAF8AdwBpAG4AbgBlAHIAcwAsACAAYwBvAG0AcABhAHIAaQBzAG8AbgBfAG0AbwBkAGUAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQgBpAGcASQBuAHQAIgAsACIAdABlAHgAdAAiADoAIgAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwBcAG4ALwAvACAAQgBpAGcAIABJAG4AdABlAGcAZQByACAAQQByAGkAdABoAG0AZQB0AGkAYwAgAEwAaQBiAHIAYQByAHkAIAAvAC8AXABuAC8ALwAgACAAIAAgACAAIAAgACAAQgBpAGcASQBuAHQAIABNAG8AZAB1AGwAZQAgACAAIAAgACAAIAAgACAAIAAgACAALwAvAFwAbgAvAC8AIAAgACAAIAAgACAAIAAgACAAIABQAHUAYgBsAGkAYwAgAEEAUABJACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwBcAG4ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8AXABuAFwAbgAvACoAKgBcAG4AIAAqACAATgBvAHIAbQBhAGwAaQBzAGUAcwAgAGEAIABCAGkAZwBJAG4AdAAgAHMAdAByAGkAbgBnAC4AIABTAHQAcgBpAHAAcwAgAGwAZQBhAGQAaQBuAGcAIAB6AGUAcgBvAHMALAAgAHIAZQBzAG8AbAB2AGUAcwAgAFwAIgAtADAAXAAiACAAdABvACAAXAAiADAAXAAiACwAIABhAG4AZAAgAHQAaAByAG8AdwBzACAAIwBWAEEATABVAEUAIQAgAG8AbgAgAGkAbgB2AGEAbABpAGQAIABjAGgAYQByAGEAYwB0AGUAcgBzAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAaQBuAHAAdQB0ACAAVABoAGUAIABCAGkAZwBJAG4AdAAgAHMAdAByAGkAbgBnAC4AXABuACAAKgAvAFwAbgBOAG8AcgBtACAAPQAgAEwAQQBNAEIARABBACgAaQBuAHAAdQB0ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAHMAdAByAF8AaQBuAHAAdQB0ACwAIABJAEYAKABPAFIAKABJAFMATwBNAEkAVABUAEUARAAoAGkAbgBwAHUAdAApACwAIABpAG4AcAB1AHQAIAA9ACAAXAAiAFwAIgApACwAIABcACIAMABcACIALAAgAGkAbgBwAHUAdAAgACYAIABcACIAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAGkAcwBfAHYAYQBsAHUAZQBfAGYAbwByAG0AYQB0ACwAIABSAEUARwBFAFgAVABFAFMAVAAoAHMAdAByAF8AaQBuAHAAdQB0ACwAIABcACIAXgAtAD8AXABcAGQAKwAkAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAcgBfAG4AbwByAG0ALAAgAFIARQBHAEUAWABSAEUAUABMAEEAQwBFACgAcwB0AHIAXwBpAG4AcAB1AHQALAAgAFwAIgBeACgALQA/ACkAMAArACgAPwA9AFwAXABkACkAXAAiACwAIABcACIAJAAxAFwAIgApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgATgBPAFQAKABpAHMAXwB2AGEAbAB1AGUAXwBmAG8AcgBtAGEAdAApACwAIABWAEEATABVAEUAKABcACIAIwBWAEEATABVAEUAIQBcACIAKQAsACAASQBGACgAcwB0AHIAXwBuAG8AcgBtACAAPQAgAFwAIgAtADAAXAAiACwAIABcACIAMABcACIALAAgAHMAdAByAF8AbgBvAHIAbQApACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFIAZQB0AHUAcgBuAHMAIAB0AGgAZQAgAHMAaQBnAG4AIABvAGYAIABhACAAQgBpAGcASQBuAHQAOgAgADEAIAAoAHAAbwBzAGkAdABpAHYAZQApACwAIAAtADEAIAAoAG4AZQBnAGEAdABpAHYAZQApACwAIABvAHIAIAAwACAAKAB6AGUAcgBvACkALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABiAGkAZwBfAGkAbgB0ACAAVABoAGUAIABCAGkAZwBJAG4AdAAgAHMAdAByAGkAbgBnAC4AXABuACAAKgAvAFwAbgBTAGkAZwBuACAAPQAgAEwAQQBNAEIARABBACgAaQBuAHAAdQB0ACwAIABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AHIAXwBuAG8AcgBtACwAIABOAG8AcgBtACgAaQBuAHAAdQB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFMAVwBJAFQAQwBIACgATABFAEYAVAAoAHMAdAByAF8AbgBvAHIAbQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAwAFwAIgAsACAAMAAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIALQBcACIALAAgAC0AMQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvAC8AIAAtAC0ALQAgAFAAcgBlAGQAaQBjAGEAdABlAHMAIAAtAC0ALQAgAFwAXABcAFwAXABuAFwAbgAvACoAKgBcAG4AIAAqACAAUgBlAHQAdQByAG4AcwAgAFQAUgBVAEUAIABpAGYAIAB0AGgAZQAgAEIAaQBnAEkAbgB0ACAAaQBzACAAZQB4AGEAYwB0AGwAeQAgAHoAZQByAG8ALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABpAG4AcAB1AHQAIABUAGgAZQAgAEIAaQBnAEkAbgB0ACAAcwB0AHIAaQBuAGcALgBcAG4AIAAqAC8AXABuAEkAcwBaAGUAcgBvACAAPQAgAEwAQQBNAEIARABBACgAaQBuAHAAdQB0ACwAIABOAG8AcgBtACgAaQBuAHAAdQB0ACkAIAA9ACAAXAAiADAAXAAiACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABSAGUAdAB1AHIAbgBzACAAVABSAFUARQAgAGkAZgAgAHQAaABlACAAQgBpAGcASQBuAHQAIABpAHMAIABuAGUAZwBhAHQAaQB2AGUALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABpAG4AcAB1AHQAIABUAGgAZQAgAEIAaQBnAEkAbgB0ACAAcwB0AHIAaQBuAGcALgBcAG4AIAAqAC8AXABuAEkAcwBOAGUAZwAgAD0AIABMAEEATQBCAEQAQQAoAGkAbgBwAHUAdAAsACAATABFAEYAVAAoAE4AbwByAG0AKABpAG4AcAB1AHQAKQApACAAPQAgAFwAIgAtAFwAIgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAAUgBlAHQAdQByAG4AcwAgAFQAUgBVAEUAIABpAGYAIAB0AGgAZQAgAEIAaQBnAEkAbgB0ACAAaQBzACAAZQB2AGUAbgAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGkAbgBwAHUAdAAgAFQAaABlACAAQgBpAGcASQBuAHQAIABzAHQAcgBpAG4AZwAuAFwAbgAgACoALwBcAG4ASQBzAEUAdgBlAG4AIAA9ACAATABBAE0AQgBEAEEAKABpAG4AcAB1AHQALAAgAEkAUwBFAFYARQBOACgAVgBBAEwAVQBFACgAUgBJAEcASABUACgATgBvAHIAbQAoAGkAbgBwAHUAdAApACkAKQApACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABSAGUAdAB1AHIAbgBzACAAVABSAFUARQAgAGkAZgAgAHQAaABlACAAQgBpAGcASQBuAHQAIABpAHMAIABvAGQAZAAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGkAbgBwAHUAdAAgAFQAaABlACAAQgBpAGcASQBuAHQAIABzAHQAcgBpAG4AZwAuAFwAbgAgACoALwBcAG4ASQBzAE8AZABkACAAPQAgAEwAQQBNAEIARABBACgAaQBuAHAAdQB0ACwAIABJAFMATwBEAEQAKABWAEEATABVAEUAKABSAEkARwBIAFQAKABOAG8AcgBtACgAaQBuAHAAdQB0ACkAKQApACkAKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFIAZQB0AHUAcgBuAHMAIAB0AGgAZQAgAHUAbgBzAGkAZwBuAGUAZAAgAG0AYQBnAG4AaQB0AHUAZABlACAAbwBmACAAYQAgAEIAaQBnAEkAbgB0ACAAcwB0AHIAaQBuAGcAIAAoAGEAYgBzAG8AbAB1AHQAZQAgAHYAYQBsAHUAZQApAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAaQBuAHAAdQB0ACAAVABoAGUAIABCAGkAZwBJAG4AdAAgAHMAdAByAGkAbgBnAC4AXABuACAAKgAvAFwAbgBBAGIAcwAgAD0AIABMAEEATQBCAEQAQQAoAGkAbgBwAHUAdAAsACAAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAHMAdAByAF8AbgBvAHIAbQAsACAATgBvAHIAbQAoAGkAbgBwAHUAdAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABMAEUARgBUACgAcwB0AHIAXwBuAG8AcgBtACkAIAA9ACAAXAAiAC0AXAAiACwAIABNAEkARAAoAHMAdAByAF8AbgBvAHIAbQAsACAAMgAsACAATABFAE4AKABzAHQAcgBfAG4AbwByAG0AKQAgAC0AIAAxACkALAAgAHMAdAByAF8AbgBvAHIAbQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABDAG8AbQBwAGEAcgBlAHMAIAB0AHcAbwAgAEIAaQBnAEkAbgB0ACAAcwB0AHIAaQBuAGcAcwAuACAAUgBlAHQAdQByAG4AcwAgADEAIAAoAGEAIAA+ACAAYgApACwAIAAtADEAIAAoAGEAIAA8ACAAYgApACwAIABvAHIAIAAwACAAKABhACAAPQAgAGIAKQAuAFwAbgAgACoAIABFAHYAYQBsAHUAYQB0AGUAcwAgAHMAaQBnAG4AcwAgAGEAbgBkACAAbABlAG4AZwB0AGgAcwAuACAASQBmACAAaQBkAGUAbgB0AGkAYwBhAGwALAAgAGQAZQBsAGUAZwBhAHQAZQBzACAAdABvACAAbgBhAHQAaQB2AGUAIABsAGkAbQBiACAAYQByAHIAYQB5ACAAYwBvAG0AcABhAHIAaQBzAG8AbgAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGkAbgBwAHUAdABfAGEAIABUAGgAZQAgAGYAaQByAHMAdAAgAEIAaQBnAEkAbgB0ACAAcwB0AHIAaQBuAGcALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABpAG4AcAB1AHQAXwBiACAAVABoAGUAIABzAGUAYwBvAG4AZAAgAEIAaQBnAEkAbgB0ACAAcwB0AHIAaQBuAGcALgBcAG4AIAAqAC8AXABuAEMAbwBtAHAAYQByAGUAIAA9ACAATABBAE0AQgBEAEEAKABpAG4AcAB1AHQAXwBhACwAIABpAG4AcAB1AHQAXwBiACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAHMAdAByAF8AbgBvAHIAbQBfAGEALAAgAE4AbwByAG0AKABpAG4AcAB1AHQAXwBhACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAdAByAF8AbgBvAHIAbQBfAGIALAAgAE4AbwByAG0AKABpAG4AcAB1AHQAXwBiACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAaQBnAG4AXwBhACwAIABCAGkAZwBJAG4AdAAuAFMAaQBnAG4AKABzAHQAcgBfAG4AbwByAG0AXwBhACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAaQBnAG4AXwBiACwAIABCAGkAZwBpAG4AdAAuAFMAaQBnAG4AKABzAHQAcgBfAG4AbwByAG0AXwBiACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIABJAEYAKABzAGkAZwBuAF8AYQAgADwAPgAgAHMAaQBnAG4AXwBiACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFMASQBHAE4AKABzAGkAZwBuAF8AYQAgAC0AIABzAGkAZwBuAF8AYgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEkARgAoAHMAaQBnAG4AXwBhACAAPQAgADAALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAwACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAZQBuAF8AYQAsACAATABFAE4AKABzAHQAcgBfAG4AbwByAG0AXwBhACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAZQBuAF8AYgAsACAATABFAE4AKABzAHQAcgBfAG4AbwByAG0AXwBiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgAbABlAG4AXwBhACAAPAA+ACAAbABlAG4AXwBiACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFMASQBHAE4AKABsAGUAbgBfAGEAIAAtACAAbABlAG4AXwBiACkAIAAqACAAcwBpAGcAbgBfAGEALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABrACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBTAGEAZgBlAEsAKABcACIAQQBEAEQAXAAiACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGEALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFMAcABsAGkAdAAoAEIAaQBnAEkAbgB0AC4AQQBiAHMAKABzAHQAcgBfAG4AbwByAG0AXwBhACkALAAgAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGIALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFMAcABsAGkAdAAoAEIAaQBnAEkAbgB0AC4AQQBiAHMAKABzAHQAcgBfAG4AbwByAG0AXwBiACkALAAgAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAG0AYQBnAG4AaQB0AHUAZABlAF8AYwBvAG0AcABhAHIAaQBzAG8AbgAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBDAG8AbQBwAGEAcgBlACgAbABpAG0AYgBzAF8AYQAsACAAbABpAG0AYgBzAF8AYgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbQBhAGcAbgBpAHQAdQBkAGUAXwBjAG8AbQBwAGEAcgBpAHMAbwBuACAAKgAgAHMAaQBnAG4AXwBhAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvAC8AIAAgACAAIAAgACAAIAAgACAAIAAtACAAQQBkAGQAaQB0AGkAbwBuACAAJgAgAFMAdQBiAHQAcgBhAGMAdABpAG8AbgAgAC0AIAAgACAAIAAgACAAIABcAFwAXABcAFwAbgBcAG4ALwAqACoAXABuACAAKgAgAEEAZABkAHMAIAB0AHcAbwAgAEIAaQBnAEkAbgB0ACAAcwB0AHIAaQBuAGcAcwAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGkAbgBwAHUAdABfAGEAIABUAGgAZQAgAGYAaQByAHMAdAAgAEIAaQBnAEkAbgB0ACAAcwB0AHIAaQBuAGcALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABpAG4AcAB1AHQAXwBiACAAVABoAGUAIABzAGUAYwBvAG4AZAAgAEIAaQBnAEkAbgB0ACAAcwB0AHIAaQBuAGcALgBcAG4AIAAqAC8AXABuAEEAZABkACAAPQAgAEwAQQBNAEIARABBACgAaQBuAHAAdQB0AF8AYQAsACAAaQBuAHAAdQB0AF8AYgAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABzAHQAcgBfAG4AbwByAG0AXwBhACwAIABOAG8AcgBtACgAaQBuAHAAdQB0AF8AYQApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAcgBfAG4AbwByAG0AXwBiACwAIABOAG8AcgBtACgAaQBuAHAAdQB0AF8AYgApACwAXABuACAAIAAgACAAIAAgACAAIABzAGkAZwBuAF8AYQAsACAAQgBpAGcAaQBuAHQALgBTAGkAZwBuACgAcwB0AHIAXwBuAG8AcgBtAF8AYQApACwAXABuACAAIAAgACAAIAAgACAAIABzAGkAZwBuAF8AYgAsACAAQgBpAGcASQBuAHQALgBTAGkAZwBuACgAcwB0AHIAXwBuAG8AcgBtAF8AYgApACwAXABuACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgAGsALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFMAYQBmAGUASwAoAFwAIgBBAEQARABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYQAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwBwAGwAaQB0ACgAQgBpAGcASQBuAHQALgBBAGIAcwAoAHMAdAByAF8AbgBvAHIAbQBfAGEAKQAsACAAawApACwAXABuACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBiACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBTAHAAbABpAHQAKABCAGkAZwBJAG4AdAAuAEEAYgBzACgAcwB0AHIAXwBuAG8AcgBtAF8AYgApACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAcABhAGMAawBlAGQAXwByAGUAcwB1AGwAdAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AQQBkAGQAUwB1AGIAUgBvAHUAdABlAHIAKABsAGkAbQBiAHMAXwBhACwAIABsAGkAbQBiAHMAXwBiACwAIABzAGkAZwBuAF8AYQAsACAAcwBpAGcAbgBfAGIALAAgAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAG4AYQBsAF8AcwBpAGcAbgAsACAAQwBIAE8ATwBTAEUAUgBPAFcAUwAoAHAAYQBjAGsAZQBkAF8AcgBlAHMAdQBsAHQALAAgAC0AMQApACwAXABuACAAIAAgACAAIAAgACAAIABmAGkAbgBhAGwAXwBsAGkAbQBiAHMALAAgAEQAUgBPAFAAKABwAGEAYwBrAGUAZABfAHIAZQBzAHUAbAB0ACwAIAAtADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIABzAHQAcgBfAG0AZQByAGcAZQBkACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBNAGUAcgBnAGUAKABmAGkAbgBhAGwAXwBsAGkAbQBiAHMALAAgAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABmAGkAbgBhAGwAXwBzAGkAZwBuACAAPQAgAC0AMQAsACAAXAAiAC0AXAAiACAAJgAgAHMAdAByAF8AbQBlAHIAZwBlAGQALAAgAHMAdAByAF8AbQBlAHIAZwBlAGQAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAAUwB1AGIAdAByAGEAYwB0AHMAIAB0AGgAZQAgAHMAZQBjAG8AbgBkACAAQgBpAGcASQBuAHQAIABzAHQAcgBpAG4AZwAgAGYAcgBvAG0AIAB0AGgAZQAgAGYAaQByAHMAdAAgACgAQQAgAC0AIABCACkALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABpAG4AcAB1AHQAXwBhACAAVABoAGUAIABtAGkAbgB1AGUAbgBkACAAQgBpAGcASQBuAHQAIABzAHQAcgBpAG4AZwAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGkAbgBwAHUAdABfAGIAIABUAGgAZQAgAHMAdQBiAHQAcgBhAGgAZQBuAGQAIABCAGkAZwBJAG4AdAAgAHMAdAByAGkAbgBnAC4AXABuACAAKgAvAFwAbgBTAHUAYgAgAD0AIABMAEEATQBCAEQAQQAoAGkAbgBwAHUAdABfAGEALAAgAGkAbgBwAHUAdABfAGIALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AHIAXwBuAG8AcgBtAF8AYgAsACAATgBvAHIAbQAoAGkAbgBwAHUAdABfAGIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABJAG4AdgBlAHIAdAAgAHQAaABlACAAcwBpAGcAbgAgAG8AZgAgAEIAIABhAHQAIAB0AGgAZQAgAHQAZQB4AHQAIABsAGUAdgBlAGwAXABuACAAIAAgACAAIAAgACAAIABzAHQAcgBfAGkAbgB2AGUAcgBzAGUAXwBiACwAIABJAEYAKABzAHQAcgBfAG4AbwByAG0AXwBiACAAPQAgAFwAIgAwAFwAIgAsACAAXAAiADAAXAAiACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgATABFAEYAVAAoAHMAdAByAF8AbgBvAHIAbQBfAGIAKQAgAD0AIABcACIALQBcACIALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAE0ASQBEACgAcwB0AHIAXwBuAG8AcgBtAF8AYgAsACAAMgAsACAATABFAE4AKABzAHQAcgBfAG4AbwByAG0AXwBiACkAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAC0AXAAiACAAJgAgAHMAdAByAF8AbgBvAHIAbQBfAGIAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgAC8ALwAgAFAAYQBzAHMAIAB0AG8AIABBAGQAZABcAG4AIAAgACAAIAAgACAAIAAgAEEAZABkACgAaQBuAHAAdQB0AF8AYQAsACAAcwB0AHIAXwBpAG4AdgBlAHIAcwBlAF8AYgApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABTAHUAbQBzACAAYQBuACAAYQByAHIAYQB5ACAAbwByACAAcgBhAG4AZwBlACAAbwBmACAAQgBpAGcASQBuAHQAIABzAHQAcgBpAG4AZwBzACAAdgBpAGEAIAB2AGUAYwB0AG8AcgBpAHoAZQBkACAAZwByAG8AdQBwACAAbQBhAHQAcgBpAGMAZQBzAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAaQBuAHAAdQB0AF8AcgBhAG4AZwBlACAAQQAgAGMAbwBuAHQAaQBnAHUAbwB1AHMAIAByAGEAbgBnAGUAIABvAHIAIABhAHIAcgBhAHkAIABvAGYAIABCAGkAZwBJAG4AdAAgAHMAdAByAGkAbgBnAHMALgBcAG4AIAAqAC8AXABuAFMAdQBtACAAPQAgAEwAQQBNAEIARABBACgAaQBuAHAAdQB0AF8AcgBhAG4AZwBlACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAC8ALwAgAFMAZQB0AHUAcAAgAGYAbwByACAAbABpAHQAdABsAGUALQBlAG4AZABpAGEAbgAgAGEAbABpAGcAbgBtAGUAbgB0ACAAaQBuACAAbQBhAHQAcgBpAHgAIABzAHUAbQBcAG4AIAAgACAAIAAgACAAIAAgAGYAbABhAHQAdABlAG4AZQBkAF8AaQBuAHAAdQB0ACwAIABUAE8AUgBPAFcAKABpAG4AcAB1AHQAXwByAGEAbgBnAGUALAAgADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABPAFIAKABJAFMARQBSAFIATwBSACgAZgBsAGEAdAB0AGUAbgBlAGQAXwBpAG4AcAB1AHQAKQAsACAAQwBPAEwAVQBNAE4AUwAoAGYAbABhAHQAdABlAG4AZQBkAF8AaQBuAHAAdQB0ACkAIAA9ACAAMAApACwAIABcACIAMABcACIALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABzAHQAcgBfAG4AbwByAG0AcwAsACAATQBBAFAAKABmAGwAYQB0AHQAZQBuAGUAZABfAGkAbgBwAHUAdAAsACAATABBAE0AQgBEAEEAKAB4ACwAIABOAG8AcgBtACgAeAApACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGEAcgByAF8AcwBpAGcAbgBzACwAIABNAEEAUAAoAEwARQBGAFQAKABzAHQAcgBfAG4AbwByAG0AcwApACwAIABMAEEATQBCAEQAQQAoAHgALAAgAEkARgAoAHgAIAA9ACAAXAAiADAAXAAiACwAIAAwACwAIABpAGYAKAB4ACAAPQAgAFwAIgAtAFwAIgAsACAALQAxACwAIAAxACkAKQApACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABzAHQAcgBfAGEAYgBzACwAIABNAEEAUAAoAHMAdAByAF8AbgBvAHIAbQBzACwAIABhAHIAcgBfAHMAaQBnAG4AcwAsACAATABBAE0AQgBEAEEAKAB4ACwAIABzAGkAZwBuACwAIABJAEYAKABzAGkAZwBuACAAPQAgAC0AMQAsACAATQBJAEQAKAB4ACwAIAAyACwAIABMAEUATgAoAHgAKQAtADEAKQAsACAAeAApACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHMAdAByAF8AcABvAHMALAAgAEYASQBMAFQARQBSACgAcwB0AHIAXwBhAGIAcwAsACAAYQByAHIAXwBzAGkAZwBuAHMAIAA9ACAAMQAsACAAewBcACIAMABcACIAfQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcwB0AHIAXwBuAGUAZwBzACwAIABGAEkATABUAEUAUgAoAHMAdAByAF8AYQBiAHMALAAgAGEAcgByAF8AcwBpAGcAbgBzACAAPQAgAC0AMQAsACAAewBcACIAMABcACIAfQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAdQBuAGkAZgBpAGUAZABfAGsALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFMAYQBmAGUASwAoAFwAIgBBAEQARABcACIALAAgAEMATwBMAFUATQBOAFMAKABmAGwAYQB0AHQAZQBuAGUAZABfAGkAbgBwAHUAdAApACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBwAG8AcwBfAHMAdQBtACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAE0AYQB0AHIAaQB4AFMAdQBtACgAcwB0AHIAXwBwAG8AcwAsACAAdQBuAGkAZgBpAGUAZABfAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAG4AZQBnAF8AcwB1AG0ALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFUATQBhAHQAcgBpAHgAUwB1AG0AKABzAHQAcgBfAG4AZQBnAHMALAAgAHUAbgBpAGYAaQBlAGQAXwBrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABwAGEAYwBrAGUAZABfAHIAZQBzAHUAbAB0ACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBBAGQAZABTAHUAYgBSAG8AdQB0AGUAcgAoAGwAaQBtAGIAcwBfAHAAbwBzAF8AcwB1AG0ALAAgAGwAaQBtAGIAcwBfAG4AZQBnAF8AcwB1AG0ALAAgADEALAAgAC0AMQAsACAAdQBuAGkAZgBpAGUAZABfAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGYAaQBuAGEAbABfAHMAaQBnAG4ALAAgAEMASABPAE8AUwBFAFIATwBXAFMAKABwAGEAYwBrAGUAZABfAHIAZQBzAHUAbAB0ACwAIAAtADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGYAaQBuAGEAbABfAGwAaQBtAGIAcwAsACAARABSAE8AUAAoAHAAYQBjAGsAZQBkAF8AcgBlAHMAdQBsAHQALAAgAC0AMQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcwB0AHIAXwBtAGUAcgBnAGUAZAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4ATQBlAHIAZwBlACgAZgBpAG4AYQBsAF8AbABpAG0AYgBzACwAIAB1AG4AaQBmAGkAZQBkAF8AawApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgAZgBpAG4AYQBsAF8AcwBpAGcAbgAgAD0AIAAtADEALAAgAFwAIgAtAFwAIgAgACYAIABzAHQAcgBfAG0AZQByAGcAZQBkACwAIABzAHQAcgBfAG0AZQByAGcAZQBkACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABNAHUAbAB0AGkAcABsAGkAZQBzACAAdAB3AG8AIABCAGkAZwBJAG4AdAAgAHMAdAByAGkAbgBnAHMALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABpAG4AcAB1AHQAXwBhACAAVABoAGUAIABmAGkAcgBzAHQAIABCAGkAZwBJAG4AdAAgAHMAdAByAGkAbgBnAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAaQBuAHAAdQB0AF8AYgAgAFQAaABlACAAcwBlAGMAbwBuAGQAIABCAGkAZwBJAG4AdAAgAHMAdAByAGkAbgBnAC4AXABuACAAKgAvAFwAbgBNAHUAbAAgAD0AIABMAEEATQBCAEQAQQAoAGkAbgBwAHUAdABfAGEALAAgAGkAbgBwAHUAdABfAGIALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AHIAXwBuAG8AcgBtAF8AYQAsACAATgBvAHIAbQAoAGkAbgBwAHUAdABfAGEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AHIAXwBuAG8AcgBtAF8AYgAsACAATgBvAHIAbQAoAGkAbgBwAHUAdABfAGIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwBpAGcAbgBfAGEALAAgAEIAaQBnAEkAbgB0AC4AUwBpAGcAbgAoAHMAdAByAF8AbgBvAHIAbQBfAGEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwBpAGcAbgBfAGIALAAgAEIAaQBnAEkAbgB0AC4AUwBpAGcAbgAoAHMAdAByAF8AbgBvAHIAbQBfAGIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABlAG4AXwBhACwAIABMAEUATgAoAHMAdAByAF8AbgBvAHIAbQBfAGEAKQAgAC0AIABJAEYAKABzAGkAZwBuAF8AYQAgAD0AIAAtADEALAAgADEALAAgADAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABlAG4AXwBiACwAIABMAEUATgAoAHMAdAByAF8AbgBvAHIAbQBfAGIAKQAgAC0AIABJAEYAKABzAGkAZwBuAF8AYgAgAD0AIAAtADEALAAgADEALAAgADAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABQAHIAbwBkAHUAYwB0ACAAbwBmACAAdwBpAHQAaAAgADAAIABpAHMAIAAwAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgATwBSACgAcwBpAGcAbgBfAGEAIAA9ACAAMAAsACAAcwBpAGcAbgBfAGIAIAA9ACAAMAApACwAIABcACIAMABcACIALABcAG4AIAAgACAAIAAgACAAIAAgAC8ALwAgAFQAaABlACAAcgBlAHMAdQBsAHQAIAB3AGkAbABsACAAZQB4AGMAZQBlAGQAIABjAGgAYQByACAAbABpAG0AaQB0AFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAbABlAG4AXwBhACAAKwAgAGwAZQBuAF8AYgAgAD4AIAAzADIANwA2ADYALAAgACMATgBVAE0AIQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGsALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFMAYQBmAGUASwAoAFwAIgBNAFUATABcACIALAAgAE0ASQBOACgAbABlAG4AXwBhACwAIABsAGUAbgBfAGIAKQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYQAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwBwAGwAaQB0ACgAQgBpAGcASQBuAHQALgBBAGIAcwAoAHMAdAByAF8AbgBvAHIAbQBfAGEAKQAsACAAawApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYgAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwBwAGwAaQB0ACgAQgBpAGcASQBuAHQALgBBAGIAcwAoAHMAdAByAF8AbgBvAHIAbQBfAGIAKQAsACAAawApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAZgBpAG4AYQBsAF8AbABpAG0AYgBzACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAE0AdQBsACgAbABpAG0AYgBzAF8AYQAsACAAbABpAG0AYgBzAF8AYgAsACAAawApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAZgBpAG4AYQBsAF8AcwBpAGcAbgAsACAAcwBpAGcAbgBfAGEAIAAqACAAcwBpAGcAbgBfAGIALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABzAHQAcgBfAG0AZQByAGcAZQBkACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBNAGUAcgBnAGUAKABmAGkAbgBhAGwAXwBsAGkAbQBiAHMALAAgAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEkARgAoAGYAaQBuAGEAbABfAHMAaQBnAG4AIAA9ACAALQAxACwAIABcACIALQBcACIAIAAmACAAcwB0AHIAXwBtAGUAcgBnAGUAZAAsACAAcwB0AHIAXwBtAGUAcgBnAGUAZAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABbAFYATwBMAEEAVABJAEwARQBdACAARwBlAG4AZQByAGEAdABlAHMAIABhACAAZAB5AG4AYQBtAGkAYwAgAGEAcgByAGEAeQAgAG8AZgAgAGkAbgB0AGUAZwBlAHIAcwAgAGEAcwAgAHQAZQB4AHQALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABbAG4AdQBtAF8AcgBvAHcAcwBdACAAYQByAHIAYQB5ACAAaABlAGkAZwBoAHQALAAgAGQAZQBmAGEAdQBsAHQAIAAxAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAWwBuAHUAbQBfAGMAbwBsAHMAXQAgAGEAcgByAGEAeQAgAHcAaQBkAHQAaAAsACAAZABlAGYAYQB1AGwAdAAgADEALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABbAG0AaQBuAF8AZABpAGcAaQB0AHMAXQAgAG0AaQBuAGkAbQB1AG0AIABuAHUAbQBiAGUAcgAgAG8AZgAgAGQAaQBnAGkAdABzACwAIABkAGUAZgBhAHUAbAB0ACAAMQA2ACAAKABtAGkAbgAgADEAIABkAGkAZwBpAHQAKQBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABbAG0AYQB4AF8AZABpAGcAaQB0AHMAXQAgAG0AYQB4AGkAbQB1AG0AIABuAHUAbQBiAGUAcgAgAG8AZgAgAGQAaQBnAGkAdABzACwAIABkAGUAZgBhAHUAbAB0ACAANQAwACAAKABtAGEAeAAgADMAMgAsADcANgA3ACAAYwBoAGEAcgBzACwAIABpAG4AYwBsAHUAZABpAG4AZwAgAHMAaQBnAG4AKQBcAG4AIAAqAC8AXABuAFIAYQBuAGQAQQByAHIAYQB5ACAAPQAgAEwAQQBNAEIARABBACgAWwBuAHUAbQBfAHIAbwB3AHMAXQAsACAAWwBuAHUAbQBfAGMAbwBsAHMAXQAsACAAWwBtAGkAbgBfAGQAaQBnAGkAdABzAF0ALAAgAFsAbQBhAHgAXwBkAGkAZwBpAHQAcwBdACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG4AXwByAG8AdwBzACwAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAG4AdQBtAF8AcgBvAHcAcwApACwAIAAxACwAIABuAHUAbQBfAHIAbwB3AHMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbgBfAGMAbwBsAHMALAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAbgB1AG0AXwBjAG8AbABzACkALAAgADEALAAgAG4AdQBtAF8AYwBvAGwAcwApACwAIABcAG4AIAAgACAAIAAgACAAIAAgAG0AaQBuAF8AbABlAG4ALAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAbQBpAG4AXwBkAGkAZwBpAHQAcwApACwAIAAxADYALAAgAE0ASQBOACgAMwAyADcANgA3ACwAIABNAEEAWAAoADEALAAgAG0AaQBuAF8AZABpAGcAaQB0AHMAKQApACkALABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQB4AF8AbABlAG4ALAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAbQBhAHgAXwBkAGkAZwBpAHQAcwApACwAIAA1ADAALAAgAE0AQQBYACgAMQAsACAATQBJAE4AKAAzADIANwA2ADYALAAgAG0AYQB4AF8AZABpAGcAaQB0AHMAKQApACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIABNAEEAUAAoAFIAQQBOAEQAQQBSAFIAQQBZACgAbgBfAHIAbwB3AHMALAAgAG4AXwBjAG8AbABzACwAIABtAGkAbgBfAGwAZQBuACwAIABtAGEAeABfAGwAZQBuACwAIABUAFIAVQBFACkALAAgAEwAQQBNAEIARABBACgAbABlAG4AZwB0AGgALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABzAGkAZwBuAF8AcAByAGUAZgBpAHgALAAgAEMASABPAE8AUwBFACgAUgBBAE4ARABCAEUAVABXAEUARQBOACgAMQAsACAAMgApACwAIABcACIAXAAiACwAIABcACIALQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHIAYQBuAGQAXwBkAGkAZwBpAHQAcwAsACAAQwBPAE4AQwBBAFQAKABSAEEATgBEAEEAUgBSAEEAWQAoADEALAAgAGwAZQBuAGcAdABoACwAIAAwACwAIAA5ACwAIABUAFIAVQBFACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHMAaQBnAG4AXwBwAHIAZQBmAGkAeAAgACYAIABSAEUARwBFAFgAUgBFAFAATABBAEMARQAoAHIAYQBuAGQAXwBkAGkAZwBpAHQAcwAsACAAXAAiAF4AMAAqAFwAIgAsACAAXAAiAFwAIgApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABEAGkAdgBpAGQAZQBzACAAdABoAGUAIABmAGkAcgBzAHQAIABCAGkAZwBJAG4AdAAgAGIAeQAgAHQAaABlACAAcwBlAGMAbwBuAGQAIAAoAEEAIAAvACAAQgApAC4AIABcAG4AIAAqACAAUgBlAHQAdQByAG4AcwAgAHQAaABlACAAcQB1AG8AdABpAGUAbgB0ACAAYQBuAGQAIABtAG8AZAB1AGwAdQBzACAAaQBuACAAcgBvAHcAcwAgADEAIABhAG4AZAAgADIALAAgAHIAZQBzAHAAZQBjAHQAaQB2AGUAbAB5AC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAaQBuAHAAdQB0AF8AYQAgAFQAaABlACAAZABpAHYAaQBkAGUAbgBkACAAQgBpAGcASQBuAHQAIABzAHQAcgBpAG4AZwAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGkAbgBwAHUAdABfAGIAIABUAGgAZQAgAGQAaQB2AGkAcwBvAHIAIABCAGkAZwBJAG4AdAAgAHMAdAByAGkAbgBnAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAWwB1AHMAZQBfAGYAbABvAG8AcgBdACAATwBwAHQAaQBvAG4AYQBsACAAYgBvAG8AbABlAGEAbgAuACAAVABSAFUARQAgAGYAbwByACAAUAB5AHQAaABvAG4ALQBzAHQAeQBsAGUAIABGAGwAbwBvAHIAIABkAGkAdgBpAHMAaQBvAG4ALAAgAEYAQQBMAFMARQAgAGYAbwByACAAVAByAHUAbgBjAGEAdABlAGQALgAgAEQAZQBmAGEAdQBsAHQAcwAgAHQAbwAgAEYAQQBMAFMARQAuAFwAbgAgACoALwBcAG4ARABpAHYATQBvAGQAIAA9ACAATABBAE0AQgBEAEEAKABpAG4AcAB1AHQAXwBhACwAIABpAG4AcAB1AHQAXwBiACwAIABbAHUAcwBlAF8AZgBsAG8AbwByAF0ALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AHIAXwBuAG8AcgBtAF8AYQAsACAATgBvAHIAbQAoAGkAbgBwAHUAdABfAGEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AHIAXwBuAG8AcgBtAF8AYgAsACAATgBvAHIAbQAoAGkAbgBwAHUAdABfAGIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwBpAGcAbgBfAGEALAAgAEIAaQBnAEkAbgB0AC4AUwBpAGcAbgAoAHMAdAByAF8AbgBvAHIAbQBfAGEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwBpAGcAbgBfAGIALAAgAEIAaQBnAEkAbgB0AC4AUwBpAGcAbgAoAHMAdAByAF8AbgBvAHIAbQBfAGIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAaQBzAF8AZgBsAG8AbwByAF8AZABpAHYALAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAdQBzAGUAXwBmAGwAbwBvAHIAKQAsACAARgBBAEwAUwBFACwAIAB1AHMAZQBfAGYAbABvAG8AcgApACwAXABuACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAHMAaQBnAG4AXwBiACAAPQAgADAALAAgACMARABJAFYALwAwACEALABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAHMAaQBnAG4AXwBhACAAPQAgADAALAAgAHsAXAAiADAAXAAiADsAXAAiADAAXAAiAH0ALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABrACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBTAGEAZgBlAEsAKABcACIARABJAFYAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBhACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBTAHAAbABpAHQAKABCAGkAZwBJAG4AdAAuAEEAYgBzACgAcwB0AHIAXwBuAG8AcgBtAF8AYQApACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBiACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBTAHAAbABpAHQAKABCAGkAZwBJAG4AdAAuAEEAYgBzACgAcwB0AHIAXwBuAG8AcgBtAF8AYgApACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABwAGEAYwBrAGUAZABfAHIAZQBzAHUAbAB0ACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBEAGkAdgBSAG8AdQB0AGUAcgAoAGwAaQBtAGIAcwBfAGEALAAgAGwAaQBtAGIAcwBfAGIALAAgAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAZQBuAF8AcgBlAG0AYQBpAG4AZABlAHIALAAgAEkATgBEAEUAWAAoAHAAYQBjAGsAZQBkAF8AcgBlAHMAdQBsAHQALAAgADEALAAgADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAHIAZQBtAGEAaQBuAGQAZQByACwAIABDAEgATwBPAFMARQBSAE8AVwBTACgAcABhAGMAawBlAGQAXwByAGUAcwB1AGwAdAAsACAAUwBFAFEAVQBFAE4AQwBFACgAbABlAG4AXwByAGUAbQBhAGkAbgBkAGUAcgAsACAAMQAsACAAMgApACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBxAHUAbwB0AGkAZQBuAHQALAAgAEQAUgBPAFAAKABwAGEAYwBrAGUAZABfAHIAZQBzAHUAbAB0ACwAIABsAGUAbgBfAHIAZQBtAGEAaQBuAGQAZQByACAAKwAgADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGYAaQBuAGEAbABfAHMAaQBnAG4ALAAgAHMAaQBnAG4AXwBhACAAKgAgAHMAaQBnAG4AXwBiACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcwB0AHIAXwBtAGUAcgBnAGUAZABfAHEALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAE0AZQByAGcAZQAoAGwAaQBtAGIAcwBfAHEAdQBvAHQAaQBlAG4AdAAsACAAawApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcwB0AHIAXwBtAGUAcgBnAGUAZABfAHIALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAE0AZQByAGcAZQAoAGwAaQBtAGIAcwBfAHIAZQBtAGEAaQBuAGQAZQByACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABzAHQAcgBfAHQAcgB1AG4AYwBfAHEALAAgAEkARgAoAEEATgBEACgAZgBpAG4AYQBsAF8AcwBpAGcAbgAgAD0AIAAtADEALAAgAHMAdAByAF8AbQBlAHIAZwBlAGQAXwBxACAAPAA+ACAAXAAiADAAXAAiACkAIAAsACAAXAAiAC0AXAAiACAAJgAgAHMAdAByAF8AbQBlAHIAZwBlAGQAXwBxACwAIABzAHQAcgBfAG0AZQByAGcAZQBkAF8AcQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcwB0AHIAXwB0AHIAdQBuAGMAXwByACwAIABJAEYAKABhAG4AZAAoAHMAaQBnAG4AXwBhACAAPQAgAC0AMQAsACAAcwB0AHIAXwBtAGUAcgBnAGUAZABfAHIAIAA8AD4AIABcACIAMABcACIAKQAsACAAXAAiAC0AXAAiACAAJgAgAHMAdAByAF8AbQBlAHIAZwBlAGQAXwByACwAIABzAHQAcgBfAG0AZQByAGcAZQBkAF8AcgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAARgBsAG8AbwByACAAQwBvAHIAcgBlAGMAdABpAG8AbgAgAGkAZgAgAGYAbABvAG8AcgAgAGkAcwAgAHIAZQBxAHUAZQBzAHQAZQBkACwAIABzAGkAZwBuAHMAIABkAGkAZgBmAGUAcgAsACAAYQBuAGQAIAByAGUAbQBhAGkAbgBkAGUAcgAgAGkAcwAgAG4AbwBuAC0AegBlAHIAbwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABuAGUAZQBkAHMAXwBmAGwAbwBvAHIAXwBjAG8AcgByAGUAYwB0AGkAbwBuACwAIABBAE4ARAAoAGkAcwBfAGYAbABvAG8AcgBfAGQAaQB2ACwAIABmAGkAbgBhAGwAXwBzAGkAZwBuACAAPQAgAC0AMQAsACAAcwB0AHIAXwBtAGUAcgBnAGUAZABfAHIAIAA8AD4AIABcACIAMABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHMAdAByAF8AZgBpAG4AYQBsAF8AcQAsACAASQBGACgAbgBlAGUAZABzAF8AZgBsAG8AbwByAF8AYwBvAHIAcgBlAGMAdABpAG8AbgAsACAAUwB1AGIAKABzAHQAcgBfAHQAcgB1AG4AYwBfAHEALAAgAFwAIgAxAFwAIgApACwAIABzAHQAcgBfAHQAcgB1AG4AYwBfAHEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHMAdAByAF8AZgBpAG4AYQBsAF8AcgAsACAASQBGACgAbgBlAGUAZABzAF8AZgBsAG8AbwByAF8AYwBvAHIAcgBlAGMAdABpAG8AbgAsACAAQQBkAGQAKABzAHQAcgBfAHQAcgB1AG4AYwBfAHIALAAgAHMAdAByAF8AbgBvAHIAbQBfAGIAKQAsACAAcwB0AHIAXwB0AHIAdQBuAGMAXwByACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABWAFMAVABBAEMASwAoAHMAdAByAF8AZgBpAG4AYQBsAF8AcQAsACAAcwB0AHIAXwBmAGkAbgBhAGwAXwByACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAApACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAEQAaQB2AGkAZABlAHMAIAB0AGgAZQAgAGYAaQByAHMAdAAgAEIAaQBnAEkAbgB0ACAAYgB5ACAAdABoAGUAIABzAGUAYwBvAG4AZAAgACgAQQAgAC8AIABCACkALgAgAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGkAbgBwAHUAdABfAGEAIABUAGgAZQAgAGQAaQB2AGkAZABlAG4AZAAgAEIAaQBnAEkAbgB0ACAAcwB0AHIAaQBuAGcALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABpAG4AcAB1AHQAXwBiACAAVABoAGUAIABkAGkAdgBpAHMAbwByACAAQgBpAGcASQBuAHQAIABzAHQAcgBpAG4AZwAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAFsAdQBzAGUAXwBmAGwAbwBvAHIAXQAgAE8AcAB0AGkAbwBuAGEAbAAgAGIAbwBvAGwAZQBhAG4ALgAgAFQAUgBVAEUAIABmAG8AcgAgAFAAeQB0AGgAbwBuAC0AcwB0AHkAbABlACAARgBsAG8AbwByACAAZABpAHYAaQBzAGkAbwBuAC4AIABEAGUAZgBhAHUAbAB0AHMAIAB0AG8AIABGAEEATABTAEUALgBcAG4AIAAqAC8AXABuAEQAaQB2ACAAPQAgAEwAQQBNAEIARABBACgAaQBuAHAAdQB0AF8AYQAsACAAaQBuAHAAdQB0AF8AYgAsACAAWwB1AHMAZQBfAGYAbABvAG8AcgBdACwAXABuACAAIAAgACAASQBOAEQARQBYACgARABpAHYATQBvAGQAKABpAG4AcAB1AHQAXwBhACwAIABpAG4AcAB1AHQAXwBiACwAIAB1AHMAZQBfAGYAbABvAG8AcgApACwAIAAxACwAIAAxACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABDAG8AbQBwAHUAdABlAHMAIAB0AGgAZQAgAHIAZQBtAGEAaQBuAGQAZQByACAAbwBmACAAQQAgAC8AIABCAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAaQBuAHAAdQB0AF8AYQAgAFQAaABlACAAZABpAHYAaQBkAGUAbgBkACAAQgBpAGcASQBuAHQAIABzAHQAcgBpAG4AZwAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGkAbgBwAHUAdABfAGIAIABUAGgAZQAgAGQAaQB2AGkAcwBvAHIAIABCAGkAZwBJAG4AdAAgAHMAdAByAGkAbgBnAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAWwB1AHMAZQBfAGYAbABvAG8AcgBdACAATwBwAHQAaQBvAG4AYQBsACAAYgBvAG8AbABlAGEAbgAuACAAVABSAFUARQAgAGYAbwByACAAUAB5AHQAaABvAG4ALQBzAHQAeQBsAGUAIABNAG8AZAB1AGwAbwAuACAARABlAGYAYQB1AGwAdABzACAAdABvACAARgBBAEwAUwBFAC4AXABuACAAKgAvAFwAbgBNAG8AZAAgAD0AIABMAEEATQBCAEQAQQAoAGkAbgBwAHUAdABfAGEALAAgAGkAbgBwAHUAdABfAGIALAAgAFsAdQBzAGUAXwBmAGwAbwBvAHIAXQAsAFwAbgAgACAAIAAgAEkATgBEAEUAWAAoAEQAaQB2AE0AbwBkACgAaQBuAHAAdQB0AF8AYQAsACAAaQBuAHAAdQB0AF8AYgAsACAAdQBzAGUAXwBmAGwAbwBvAHIAKQAsACAAMgAsACAAMQApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAAUgBhAGkAcwBlAHMAIABhACAAQgBpAGcASQBuAHQAIABiAGEAcwBlACAAdABvACAAdABoAGUAIABwAG8AdwBlAHIAIABvAGYAIABhACAAQgBpAGcASQBuAHQAIABlAHgAcABvAG4AZQBuAHQALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABiAGEAcwBlACAAVABoAGUAIABiAGEAcwBlACAAQgBpAGcASQBuAHQAIABzAHQAcgBpAG4AZwAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGUAeABwAG8AbgBlAG4AdAAgAFQAaABlACAAZQB4AHAAbwBuAGUAbgB0ACAAQgBpAGcASQBuAHQAIABzAHQAcgBpAG4AZwAuAFwAbgAgACoALwBcAG4AUABvAHcAIAA9ACAATABBAE0AQgBEAEEAKABiAGEAcwBlACwAIABlAHgAcABvAG4AZQBuAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AHIAXwBuAG8AcgBtAF8AYgBhAHMAZQAsACAATgBvAHIAbQAoAGIAYQBzAGUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AHIAXwBuAG8AcgBtAF8AZQB4AHAALAAgAE4AbwByAG0AKABlAHgAcABvAG4AZQBuAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwBpAGcAbgBfAGIAYQBzAGUALAAgAEIAaQBnAEkAbgB0AC4AUwBpAGcAbgAoAHMAdAByAF8AbgBvAHIAbQBfAGIAYQBzAGUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwBpAGcAbgBfAGUAeABwACwAIABCAGkAZwBJAG4AdAAuAFMAaQBnAG4AKABzAHQAcgBfAG4AbwByAG0AXwBlAHgAcAApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AHIAXwBhAGIAcwBfAGIAYQBzAGUALAAgAEIAaQBnAEkAbgB0AC4AQQBiAHMAKABzAHQAcgBfAG4AbwByAG0AXwBiAGEAcwBlACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAdAByAF8AYQBiAHMAXwBlAHgAcAAsACAAQgBpAGcASQBuAHQALgBBAGIAcwAoAHMAdAByAF8AbgBvAHIAbQBfAGUAeABwACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIABpAHMAXwBlAHgAcABfAGUAdgBlAG4ALAAgAEkAUwBFAFYARQBOACgAVgBBAEwAVQBFACgAUgBJAEcASABUACgAcwB0AHIAXwBuAG8AcgBtAF8AZQB4AHAALAAgADEAKQApACkALABcAG4AIAAgACAAIAAgACAAIAAgAGYAaQBuAGEAbABfAHMAaQBnAG4ALAAgAEkARgAoAHMAaQBnAG4AXwBiAGEAcwBlACAAPQAgAC0AMQAsACAASQBGACgAaQBzAF8AZQB4AHAAXwBlAHYAZQBuACwAIAAxACwAIAAtADEAKQAsACAAcwBpAGcAbgBfAGIAYQBzAGUAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAC8ALwAgAEgAYQBuAGQAbABlACAAbQBhAHQAaABlAG0AYQB0AGkAYwBhAGwAIABiAG8AdQBuAGQAYQByAGkAZQBzACAAYQBuAGQAIABiAGEAcwBlACAAbABpAG0AaQB0AHMAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABzAHQAcgBfAGEAYgBzAF8AYgBhAHMAZQAgAD0AIABcACIAMABcACIALAAgAEkARgAoAHMAdAByAF8AbgBvAHIAbQBfAGUAeABwACAAPQAgAFwAIgAwAFwAIgAsACAAIwBOAFUATQAhACwAIABcACIAMABcACIAKQAsACAALwAvACAAMABeADAAIABpAHMAIAB1AG4AZABlAGYAaQBuAGUAZABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAHMAdAByAF8AYQBiAHMAXwBiAGEAcwBlACAAPQAgAFwAIgAxAFwAIgAsACAASQBGACgAZgBpAG4AYQBsAF8AcwBpAGcAbgAgAD0AIAAtADEALAAgAFwAIgAtADEAXAAiACwAIABcACIAMQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAcwBpAGcAbgBfAGUAeABwACAAPQAgAC0AMQAsACAAXAAiADAAXAAiACwAIAAvAC8AIABJAG4AdABlAGcAZQByACAAdAByAHUAbgBjAGEAdABpAG8AbgA6ACAAbgBlAGcAYQB0AGkAdgBlACAAZQB4AHAAbwBuAGUAbgB0AHMAIAB5AGkAZQBsAGQAIAAwACAAZgBvAHIAIABiAGEAcwBlAHMAIAA+AD0AIAAyAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAcwB0AHIAXwBuAG8AcgBtAF8AZQB4AHAAIAA9ACAAXAAiADAAXAAiACwAIABcACIAMQBcACIALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABSAGUAcwB1AGwAdABzACAAZgByAG8AbQAgAGUAeABwAG8AbgBlAG4AdABzACAAZwByAGUAYQB0AGUAcgAgAHQAaABhAG4AIAA2ACAAZABpAGcAaQB0AHMAIABjAGEAbgBuAG8AdAAgAGIAZQAgAGQAaQBzAHAAbABhAHkAZQBkAC4AXABuACAAIAAgACAAIAAgACAAIABJAEYAKABMAEUATgAoAHMAdAByAF8AbgBvAHIAbQBfAGUAeABwACkAIAA+ACAANgAsACAAIwBOAFUATQAhACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbgB1AG0AXwBlAHgAcAAsACAAVgBBAEwAVQBFACgAcwB0AHIAXwBuAG8AcgBtAF8AZQB4AHAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAEEAcABwAHIAbwB4AGkAbQBhAHQAZQAgAHQAaABlACAAZgBpAG4AYQBsACAAYwBoAGEAcgBhAGMAdABlAHIAIABjAG8AdQBuAHQAOgAgAEIAIAAqACAATABvAGcAMQAwACgAQQApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGIAYQBzAGUAXwBsAG8AZwAxADAALAAgAEwATwBHADEAMAAoAFYAQQBMAFUARQAoAEwARQBGAFQAKABzAHQAcgBfAGEAYgBzAF8AYgBhAHMAZQAsACAAMQA0ACkAKQApACAAKwAgAE0AQQBYACgAMAAsACAATABFAE4AKABzAHQAcgBfAGEAYgBzAF8AYgBhAHMAZQApACAALQAgADEANAApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAYQBwAHAAcgBvAHgAXwBkAGkAZwBpAHQAcwAsACAAbgB1AG0AXwBlAHgAcAAgACoAIABiAGEAcwBlAF8AbABvAGcAMQAwACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEkARgAoAGEAcABwAHIAbwB4AF8AZABpAGcAaQB0AHMAIAA+ACAAMwAyADcANgA2ACwAIAAjAE4AVQBNACEALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGsALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFMAYQBmAGUASwAoAFwAIgBNAFUATABcACIALAAgAGEAcABwAHIAbwB4AF8AZABpAGcAaQB0AHMAIAAvACAAMgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGIAYQBzAGUALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFMAcABsAGkAdAAoAHMAdAByAF8AYQBiAHMAXwBiAGEAcwBlACwAIABrACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGYAaQBuAGEAbAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBQAG8AdwAoAGwAaQBtAGIAcwBfAGIAYQBzAGUALAAgAHMAdAByAF8AbgBvAHIAbQBfAGUAeABwACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcwB0AHIAXwBtAGUAcgBnAGUAZAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4ATQBlAHIAZwBlACgAbABpAG0AYgBzAF8AZgBpAG4AYQBsACwAIABrACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEkARgAoAGYAaQBuAGEAbABfAHMAaQBnAG4AIAA9ACAALQAxACwAIABcACIALQBcACIAIAAmACAAcwB0AHIAXwBtAGUAcgBnAGUAZAAsACAAcwB0AHIAXwBtAGUAcgBnAGUAZAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAKQApACkAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4ALwAvADEAMgAzADQANQA2ADcAOAA5ADAAMQAyADMANAA1ADYANwA4ADkAMAAxADIAMwA0ADUANgA3ADgAOQAwADEAMgAzADQANQA2ADcAOAA5ADAAMQAyADMANAA1ADYANwA4ADkAMAAxADIAMwA0ADUANgA3ADgAOQAwADEAMgAzADQANQA2ADcAOAA5AC0AMQAyADMANAA1ADYANwAtADkAMAAxADIAMwA0ADUANgA3ADgAOQAwADEAMgAzADQANQA2ADcAOAA5ADAAMQAyADMANAA1ADYANwA4ADkAMAAxADIAMwA0ADUANgA3AC0AXABuAC8AKgAqAFwAbgAgACoAIABDAGEAbABjAHUAbABhAHQAZQBzACAAdABoAGUAIABpAG4AdABlAGcAZQByACAAcwBxAHUAYQByAGUAIAByAG8AbwB0ACAAKABmAGwAbwBvAHIAKQAgAG8AZgAgAGEAIABCAGkAZwBJAG4AdAAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGkAbgBwAHUAdAAgAFQAaABlACAAcgBhAGQAaQBjAGEAbgBkACAAQgBpAGcASQBuAHQAIABzAHQAcgBpAG4AZwAuAFwAbgAgACoALwBcAG4AUwBxAHIAdAAgAD0AIABMAEEATQBCAEQAQQAoAGkAbgBwAHUAdAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABzAHQAcgBfAG4AbwByAG0ALAAgAE4AbwByAG0AKABpAG4AcAB1AHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwBpAGcAbgBfAG4ALAAgAEIAaQBnAEkAbgB0AC4AUwBpAGcAbgAoAHMAdAByAF8AbgBvAHIAbQApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAcwBpAGcAbgBfAG4AIAA9ACAALQAxACwAIAAjAE4AVQBNACEALABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAHMAdAByAF8AbgBvAHIAbQAgAD0AIABcACIAMABcACIALAAgAFwAIgAwAFwAIgAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAcwB0AHIAXwBuAG8AcgBtACAAPQAgAFwAIgAxAFwAIgAsACAAXAAiADEAXAAiACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABlAG4AXwBuAG8AcgBtACwAIABMAEUATgAoAHMAdAByAF8AbgBvAHIAbQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbgB1AG0AXwBzAGUAZQBkAF8AcAByAGUAYwBpAHMAaQBvAG4ALAAgAEkARgAoAGwAZQBuAF8AbgBvAHIAbQAgADwAPQAgADEANAAsACAAbABlAG4AXwBuAG8AcgBtACwAIABJAEYAKABJAFMARQBWAEUATgAoAGwAZQBuAF8AbgBvAHIAbQApACwAIAAxADQALAAgADEAMwApACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABzAHQAcgBfAG4AYQB0AGkAdgBlAF8AcAByAGUAYwBpAHMAaQBvAG4ALAAgAEwARQBGAFQAKABzAHQAcgBfAG4AbwByAG0ALAAgAG4AdQBtAF8AcwBlAGUAZABfAHAAcgBlAGMAaQBzAGkAbwBuACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABuAHUAbQBfAG4AYQB0AGkAdgBlAF8AcAByAGUAYwBpAHMAaQBvAG4ALAAgAFYAQQBMAFUARQAoAHMAdAByAF8AbgBhAHQAaQB2AGUAXwBwAHIAZQBjAGkAcwBpAG8AbgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbgB1AG0AXwBtAGEAZwBuAGkAdAB1AGQAZQBfAHoAZQByAG8AZQBzACwAIAAoAGwAZQBuAF8AbgBvAHIAbQAgAC0AIABuAHUAbQBfAHMAZQBlAGQAXwBwAHIAZQBjAGkAcwBpAG8AbgApACAALwAgADIALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcwB0AHIAXwBwAHIAZQBmAGkAeAAsACAAVABFAFgAVAAoAFIATwBVAE4ARABVAFAAKABTAFEAUgBUACgAbgB1AG0AXwBuAGEAdABpAHYAZQBfAHAAcgBlAGMAaQBzAGkAbwBuACkALAAgADAAKQAgACsAIAAxACwAIABcACIAMABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHMAdAByAF8AcwBlAGUAZAAsACAAcwB0AHIAXwBwAHIAZQBmAGkAeAAgACYAIABSAEUAUABUACgAXAAiADAAXAAiACwAIABuAHUAbQBfAG0AYQBnAG4AaQB0AHUAZABlAF8AegBlAHIAbwBlAHMAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIABTAGMAYQBsAGUAcwAgAGsAIABiAHkAIAB0AGgAZQAgAG0AYQB4AGkAbQB1AG0AIABvAHYAZQByAGwAYQBwACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAawAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwBhAGYAZQBLACgAXAAiAE0AVQBMAFwAIgAsACAAbABlAG4AXwBuAG8AcgBtACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwByAGEAZABpAGMAYQBuAGQALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFMAcABsAGkAdAAoAHMAdAByAF8AbgBvAHIAbQAsACAAawApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AcwBlAGUAZAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwBwAGwAaQB0ACgAcwB0AHIAXwBzAGUAZQBkACwAIABrACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AZgBpAG4AYQBsACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAFMAcQByAHQAKABsAGkAbQBiAHMAXwByAGEAZABpAGMAYQBuAGQALAAgAGwAaQBtAGIAcwBfAHMAZQBlAGQALAAgAGsAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBNAGUAcgBnAGUAKABsAGkAbQBiAHMAXwBmAGkAbgBhAGwALAAgAGsAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACkAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABDAG8AbQBwAHUAdABlAHMAIAB0AGgAZQAgAGYAYQBjAHQAbwByAGkAYQBsACAAbwBmACAAYQAgAEIAaQBnAEkAbgB0ACAAKABuACEAKQAgAHUAcwBpAG4AZwAgAFAAZQB0AGUAcgAgAEwAdQBzAGMAaABuAHkAJwBzACAAUAByAGkAbQBlACAAUwB3AGkAbgBnACAAYQBsAGcAbwByAGkAdABoAG0ALgBcAG4AIAAqACAAQABwAGEAcgBhAG0AIABpAG4AcAB1AHQAIABUAGgAZQAgAEIAaQBnAEkAbgB0ACAAcwB0AHIAaQBuAGcALgAgAE0AYQB4AGkAbQB1AG0AIABzAHUAcABwAG8AcgB0AGUAZAAgAGkAbgBwAHUAdAAgAGkAcwAgADkAMgA3ADMALgBcAG4AIAAqAC8AXABuAEYAYQBjAHQAIAA9ACAATABBAE0AQgBEAEEAKABpAG4AcAB1AHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AHIAXwBuAG8AcgBtACwAIABOAG8AcgBtACgAaQBuAHAAdQB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAaQBnAG4AXwBuACwAIABCAGkAZwBJAG4AdAAuAFMAaQBnAG4AKABzAHQAcgBfAG4AbwByAG0AKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAHMAaQBnAG4AXwBuACAAPQAgAC0AMQAsACAAIwBOAFUATQAhACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABzAHQAcgBfAG4AbwByAG0AIAA9ACAAXAAiADAAXAAiACwAIABcACIAMQBcACIALABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAHMAdAByAF8AbgBvAHIAbQAgAD0AIABcACIAMQBcACIALAAgAFwAIgAxAFwAIgAsAFwAbgAgACAAIAAgACAAIAAgACAALwAvACAARgBpAHIAZQB3AGEAbABsACAAMQA6ACAAVAByAGEAcAAgAG0AYQBzAHMAaQB2AGUAIABzAHQAcgBpAG4AZwBzACAAYgBlAGYAbwByAGUAIAB0AGgAZQB5ACAAaABpAHQAIABWAEEATABVAEUAKAApAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgATABFAE4AKABzAHQAcgBfAG4AbwByAG0AKQAgAD4AIAA0ACwAIAAjAE4AVQBNACEALAAgAFwAbgAgACAAIAAgACAAIAAgACAALwAvACAARgBpAHIAZQB3AGEAbABsACAAMgA6ACAAVAByAGEAcAAgAG0AYQB0AGgAZQBtAGEAdABpAGMAYQBsACAAYwBlAGkAbABpAG4AZwBcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAFYAQQBMAFUARQAoAHMAdAByAF8AbgBvAHIAbQApACAAPgAgADkAMgA3ADMALAAgACMATgBVAE0AIQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAG4AdQBtAF8AbgAsACAAVgBBAEwAVQBFACgAcwB0AHIAXwBuAG8AcgBtACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABnAGwAbwBiAGEAbABfAHAAcgBpAG0AZQBzACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBOAGEAdABpAHYAZQBQAHIAaQBtAGUAcwAoAG4AdQBtAF8AbgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUAByAGkAbQBlAFMAdwBpAG4AZwBLAGUAcgBuAGUAbAAoAG4AdQBtAF8AbgAsACAAZwBsAG8AYgBhAGwAXwBwAHIAaQBtAGUAcwApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAKQApACkAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABSAGUAdAB1AHIAbgBzACAAdABoAGUAIABtAGkAbgBpAG0AdQBtACAAQgBpAGcASQBuAHQAIABmAHIAbwBtACAAYQBuACAAYQByAHIAYQB5ACAAbwByACAAcgBhAG4AZwBlAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAcgBhAG4AZwBlACAAQQAgAGMAbwBuAHQAaQBnAHUAbwB1AHMAIAByAGEAbgBnAGUAIABvAHIAIABhAHIAcgBhAHkAIABvAGYAIABCAGkAZwBJAG4AdAAgAHMAdAByAGkAbgBnAHMALgBcAG4AIAAqAC8AXABuAE0AaQBuACAAPQAgAEwAQQBNAEIARABBACgAcgBhAG4AZwBlACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAGYAbABhAHQAdABlAG4AZQBkAF8AYwBvAGwALAAgAFQATwBDAE8ATAAoAHIAYQBuAGcAZQAsACAAMQApACwAXABuACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAE8AUgAoAEkAUwBFAFIAUgBPAFIAKABmAGwAYQB0AHQAZQBuAGUAZABfAGMAbwBsACkALAAgAFIATwBXAFMAKABmAGwAYQB0AHQAZQBuAGUAZABfAGMAbwBsACkAIAA9ACAAMAApACwAIABcACIAMABcACIALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVAByAGUAZQBDAG8AbQBwAGEAcgBlACgATQBBAFAAKABmAGwAYQB0AHQAZQBuAGUAZABfAGMAbwBsACwAIABCAGkAZwBJAG4AdAAuAE4AbwByAG0AKQAsACAALQAxACkAXABuACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABSAGUAdAB1AHIAbgBzACAAdABoAGUAIABtAGEAeABpAG0AdQBtACAAQgBpAGcASQBuAHQAIABmAHIAbwBtACAAYQBuACAAYQByAHIAYQB5ACAAbwByACAAcgBhAG4AZwBlAC4AXABuACAAKgAgAEAAcABhAHIAYQBtACAAcgBhAG4AZwBlACAAQQAgAGMAbwBuAHQAaQBnAHUAbwB1AHMAIAByAGEAbgBnAGUAIABvAHIAIABhAHIAcgBhAHkAIABvAGYAIABCAGkAZwBJAG4AdAAgAHMAdAByAGkAbgBnAHMALgBcAG4AIAAqAC8AXABuAE0AYQB4ACAAPQAgAEwAQQBNAEIARABBACgAcgBhAG4AZwBlACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAGYAbABhAHQAdABlAG4AZQBkAF8AYwBvAGwALAAgAFQATwBDAE8ATAAoAHIAYQBuAGcAZQAsACAAMQApACwAXABuACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAE8AUgAoAEkAUwBFAFIAUgBPAFIAKABmAGwAYQB0AHQAZQBuAGUAZABfAGMAbwBsACkALAAgAFIATwBXAFMAKABmAGwAYQB0AHQAZQBuAGUAZABfAGMAbwBsACkAIAA9ACAAMAApACwAIABcACIAMABcACIALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVAByAGUAZQBDAG8AbQBwAGEAcgBlACgATQBBAFAAKABmAGwAYQB0AHQAZQBuAGUAZABfAGMAbwBsACwAIABCAGkAZwBJAG4AdAAuAE4AbwByAG0AKQAsACAAMQApAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAIgB9AF0ALAAiAHAAcgBvAGoAZQBjAHQATgBhAG0AZQBzACIAOgBbACIAdABlAHMAdABfAEIAaQBnAEkAbgB0AC4ASwBuAHUAdABoAEQAaQB2AGkAcwBpAG8AbgAiACwAIgB0AGUAcwB0AF8AQgBpAGcASQBuAHQALgBOAGUAdwB0AG8AbgBSAGEAcABoAHMAbwBuAEQAaQB2AGkAcwBpAG8AbgAiACwAIgB0AGUAcwB0AF8AQgBpAGcASQBuAHQALgBEAGkAdgBpAHMAaQBvAG4AQQBsAGcAbwByAGkAdABoAG0AcwAiACwAIgB0AGUAcwB0AF8AQgBpAGcASQBuAHQALgBEAGkAdgBpAHMAaQBvAG4AQQBsAGcAbwByAGkAdABoAG0AQwBvAG0AcABhAHIAaQBzAG8AbgAiACwAIgB0AGUAcwB0AF8AQgBpAGcASQBuAHQALgBEAGkAdgBpAHMAaQBvAG4AQgBlAG4AYwBoAG0AYQByAGsAQwBhAHMAZQBzACIALAAiAHQAZQBzAHQAXwBCAGkAZwBJAG4AdAAuAEEAcwB5AG0AbQBlAHQAcgBpAGMAQQBCAEcAcgBpAGQAIgAsACIAdABlAHMAdABfAEIAaQBnAEkAbgB0AC4ARgBhAGMAdABvAHIAaQBhAGwAQQBsAGcAbwByAGkAdABoAG0AcwAiACwAIgB0AGUAcwB0AF8AQgBpAGcASQBuAHQALgBGAGEAYwB0AG8AcgBpAGEAbABDAG8AbQBwAGEAcgBpAHMAbwBuACIALAAiAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFMAYQBmAGUASwAiACwAIgBjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBTAHAAbABpAHQAIgAsACIAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4ATQBlAHIAZwBlACIALAAiAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAEMAYQByAHIAeQAiACwAIgBjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAEMAbwBtAHAAYQByAGUAIgAsACIAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBBAGQAZAAiACwAIgBjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAFMAdQBiACIALAAiAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFUATQBhAHQAcgBpAHgAUwB1AG0AIgAsACIAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AQQBkAGQAUwB1AGIAUgBvAHUAdABlAHIAIgAsACIAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBNAHUAbAAiACwAIgBjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBGAGkAbgBkAFEAdQBvAHQAaQBlAG4AdABMAGkAbQBiACIALAAiAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAEsAbgB1AHQAaABEAGkAdgAiACwAIgBjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBEAGkAdgBSAG8AdQB0AGUAcgAiACwAIgBjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBOAGUAdwB0AG8AbgBSAGEAcABoAHMAbwBuAFMAZQBlAGQAIgAsACIAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4ATgBlAHcAdABvAG4AUgBhAHAAaABzAG8AbgBSAGUAYwBpAHAAcgBvAGMAYQBsACIALAAiAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAE4AZQB3AHQAbwBuAFIAYQBwAGgAcwBvAG4ARABpAHYAIgAsACIAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBQAG8AdwAiACwAIgBjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAFMAcQByAHQAIgAsACIAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4ATgBhAHQAaQB2AGUAUAByAGkAbQBlAHMAIgAsACIAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBUAGUAeAB0AE0AdQBsACIALAAiAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFQAZQB4AHQAVAByAGUAZQBQAHIAbwBkACIALAAiAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAE4AYQB0AGkAdgBlAFMAdwBpAG4AZwBFAHgAcABvAG4AZQBuAHQAcwAiACwAIgBjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBTAHcAaQBuAGcAVABlAHIAbQAiACwAIgBjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBQAHIAaQBtAGUAUwB3AGkAbgBnAEsAZQByAG4AZQBsACIALAAiAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFQAcgBlAGUAQwBvAG0AcABhAHIAZQAiACwAIgBCAGkAZwBJAG4AdAAuAE4AbwByAG0AIgAsACIAQgBpAGcASQBuAHQALgBTAGkAZwBuACIALAAiAEIAaQBnAEkAbgB0AC4ASQBzAFoAZQByAG8AIgAsACIAQgBpAGcASQBuAHQALgBJAHMATgBlAGcAIgAsACIAQgBpAGcASQBuAHQALgBJAHMARQB2AGUAbgAiACwAIgBCAGkAZwBJAG4AdAAuAEkAcwBPAGQAZAAiACwAIgBCAGkAZwBJAG4AdAAuAEEAYgBzACIALAAiAEIAaQBnAEkAbgB0AC4AQwBvAG0AcABhAHIAZQAiACwAIgBCAGkAZwBJAG4AdAAuAEEAZABkACIALAAiAEIAaQBnAEkAbgB0AC4AUwB1AGIAIgAsACIAQgBpAGcASQBuAHQALgBTAHUAbQAiACwAIgBCAGkAZwBJAG4AdAAuAE0AdQBsACIALAAiAEIAaQBnAEkAbgB0AC4AUgBhAG4AZABBAHIAcgBhAHkAIgAsACIAQgBpAGcASQBuAHQALgBEAGkAdgBNAG8AZAAiACwAIgBCAGkAZwBJAG4AdAAuAEQAaQB2ACIALAAiAEIAaQBnAEkAbgB0AC4ATQBvAGQAIgAsACIAQgBpAGcASQBuAHQALgBQAG8AdwAiACwAIgBCAGkAZwBJAG4AdAAuAFMAcQByAHQAIgAsACIAQgBpAGcASQBuAHQALgBGAGEAYwB0ACIALAAiAEIAaQBnAEkAbgB0AC4ATQBpAG4AIgAsACIAQgBpAGcASQBuAHQALgBNAGEAeAAiAF0ALAAiAGwAbwBjAGEAbABlACIAOgB7ACIAbABpAHMAdABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHIAbwB3AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiADsAIgAsACIAYwBvAGwAdQBtAG4AUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgB0AGgAbwB1AHMAYQBuAGQAcwBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHQAaABvAHUAcwBhAG4AZABzAFAAbwBzAGkAdABpAG8AbgBzACIAOgBbADMAXQAsACIAZABlAGMAaQBtAGEAbABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAuACIALAAiAGQAYQB0AGUATwByAGQAZQByACIAOgAiAEQATQBZACIALAAiAGMAdQByAHIAZQBuAGMAeQBTAHkAbQBiAG8AbAAiADoAIgAkACIALAAiAGkAcwBDAHUAcgByAGUAbgBjAHkAUwB5AG0AYgBvAGwATABlAGEAZAAiADoAdAByAHUAZQAsACIAaQBzAEMAdQByAHIAZQBuAGMAeQBTAGUAcABCAHkAUwBwAGEAYwBlACIAOgBmAGEAbABzAGUALAAiAHIAbwB3AEwAZQB0AHQAZQByACIAOgAiAFIAIgAsACIAYwBvAGwAdQBtAG4ATABlAHQAdABlAHIAIgA6ACIAQwAiACwAIgByAGMATABlAGYAdABCAHIAYQBjAGsAZQB0ACIAOgAiAFsAIgAsACIAcgBjAFIAaQBnAGgAdABCAHIAYQBjAGsAZQB0ACIAOgAiAF0AIgAsACIAcwB0AGEAdABlAG0AZQBuAHQAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIAOwAiACwAIgBsAG8AYwBhAGwAZQBOAGEAbQBlACIAOgAiAGUAbgAtAHUAcwAiAH0AfQA=</AFEJSONBlob>
+<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAHQAZQBzAHQAXwBCAGkAZwBJAG4AdAAiACwAIgB0AGUAeAB0ACIAOgAiAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAFwAbgAvAC8AIABCAGkAZwAgAEkAbgB0AGUAZwBlAHIAIABBAHIAaQB0AGgAbQBlAHQAaQBjACAATABpAGIAcgBhAHIAeQAgAC8ALwBcAG4ALwAvACAAIAAgACAAIAAgACAAdABlAHMAdABfAEIAaQBnAEkAbgB0ACAATQBvAGQAdQBsAGUAIAAgACAAIAAgACAAIAAvAC8AXABuAC8ALwAgACAAIAAgACAAIAAgAFAAcgBpAHYAYQB0AGUAIABUAGUAcwB0AGkAbgBnACAAQQBQAEkAIAAgACAAIAAgACAALwAvAFwAbgAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwBcAG4AXABuAEsAbgB1AHQAaABEAGkAdgBpAHMAaQBvAG4APQBMAEEATQBCAEQAQQAoAGEALAAgAGIALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAawAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwBhAGYAZQBLACgAXAAiAEQASQBWAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABwAGEAYwBrAGUAZAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4ASwBuAHUAdABoAEQAaQB2ACgAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwBwAGwAaQB0ACgAYQAsACAAawApACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBTAHAAbABpAHQAKABiACwAIABrACkALAAgAGsAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAE0AZQByAGcAZQAoAEQAUgBPAFAAKABwAGEAYwBrAGUAZAAsACAASQBOAEQARQBYACgAcABhAGMAawBlAGQALAAgADEALAAgADEAKQAgACsAIAAxACkALAAgAGsAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBOAGUAdwB0AG8AbgBSAGEAcABoAHMAbwBuAEQAaQB2AGkAcwBpAG8AbgAgAD0AIABMAEEATQBCAEQAQQAoAGEALAAgAGIALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAawAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwBhAGYAZQBLACgAXAAiAEQASQBWAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABwAGEAYwBrAGUAZAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4ATgBlAHcAdABvAG4AUgBhAHAAaABzAG8AbgBEAGkAdgAoAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFMAcABsAGkAdAAoAGEALAAgAGsAKQAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwBwAGwAaQB0ACgAYgAsACAAawApACwAIABrACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBNAGUAcgBnAGUAKABEAFIATwBQACgAcABhAGMAawBlAGQALAAgAEkATgBEAEUAWAAoAHAAYQBjAGsAZQBkACwAIAAxACwAIAAxACkAIAArACAAMQApACwAIABrACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAEAAcABhAHIAYQBtACAAYQAgAFQAaABlACAAZABpAHYAaQBkAGUAbgBkACAAcwB0AHIAaQBuAGcAXABuACAAKgAgAEAAcABhAHIAYQBtACAAYgAgAFQAaABlACAAZABpAHYAaQBzAG8AcgAgAHMAdAByAGkAbgBnAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAG0AbwBkAGUAIABcACIASwBOAFUAVABIAFwAIgAgAG8AcgAgAFwAIgBOAFIAXAAiAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGkAdABlAHIAcwAgAEkAbgBuAGUAcgAgAGwAbwBvAHAAIABjAG8AdQBuAHQAIAAoAHQAbwAgAGQAZQBmAGUAYQB0ACAAYwBoAHUAbgBrAHkAIABjAGwAbwBjAGsAIAByAGUAcwBvAGwAdQB0AGkAbwBuACkAXABuACAAKgAgAEAAcABhAHIAYQBtACAAcgBlAHAAZQBhAHQAcwAgAE8AdQB0AGUAcgAgAGwAbwBvAHAAIABjAG8AdQBuAHQAIAAoAHQAbwAgAGQAZQBmAGUAYQB0ACAATwBTAC8ARwBhAHIAYgBhAGcAZQAgAEMAbwBsAGwAZQBjAHQAaQBvAG4AIABuAG8AaQBzAGUAKQBcAG4AIAAqAC8AXABuAEQAaQB2AGkAcwBpAG8AbgBBAGwAZwBvAHIAaQB0AGgAbQBzACAAPQAgAEwAQQBNAEIARABBACgAYQAsACAAYgAsACAAbQBvAGQAZQAsACAAaQB0AGUAcgBzACwAIAByAGUAcABlAGEAdABzACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAC8ALwAgAE0AYQBwACAAdABoAGUAIABvAHUAdABlAHIAIAByAGUAcABlAGEAdABzACAAbABvAG8AcABcAG4AIAAgACAAIAAgACAAIAAgAGIAYQB0AGMAaABfAHQAaQBtAGUAcwAsACAATQBBAFAAKABTAEUAUQBVAEUATgBDAEUAKAByAGUAcABlAGEAdABzACkALAAgAEwAQQBNAEIARABBACgAcgAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHMAdABhAHIAdAAsACAATgBPAFcAKAApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAATQBhAHAAIAB0AGgAZQAgAGkAbgBuAGUAcgAgAGUAeABlAGMAdQB0AGkAbwBuACAAbABvAG8AcABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAByAHUAbgAsACAASQBGACgAbQBvAGQAZQAgAD0AIABcACIASwBOAFUAVABIAFwAIgAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAE0AQQBQACgAUwBFAFEAVQBFAE4AQwBFACgAaQB0AGUAcgBzACkALAAgAEwAQQBNAEIARABBACgAaQAsACAASwBuAHUAdABoAEQAaQB2AGkAcwBpAG8AbgAoAGEALAAgAGIAKQApACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBBAFAAKABTAEUAUQBVAEUATgBDAEUAKABpAHQAZQByAHMAKQAsACAATABBAE0AQgBEAEEAKABpACwAIABOAGUAdwB0AG8AbgBSAGEAcABoAHMAbwBuAEQAaQB2AGkAcwBpAG8AbgAoAGEALAAgAGIAKQApACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAEYAbwByAGMAZQAgAGUAdgBhAGwAdQBhAHQAaQBvAG4AIABiAGUAZgBvAHIAZQAgAHAAdQBsAGwAaQBuAGcAIABzAHQAbwBwACAAdABpAG0AZQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABzAHQAbwBwACwAIABOAE8AVwAoACkAIAArACAAKAAwACAAKgAgAEwARQBOACgASQBOAEQARQBYACgAcgB1AG4ALAAgADEALAAgADEAKQApACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIABUAG8AdABhAGwAIABiAGEAdABjAGgAIAB0AGkAbQBlACAAaQBuACAAbQBpAGwAbABpAHMAZQBjAG8AbgBkAHMAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABzAHQAbwBwACAALQAgAHMAdABhAHIAdAApACAAKgAgADgANgA0ADAAMAAwADAAMABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABFAHgAdAByAGEAYwB0ACAAdABoAGUAIABjAGwAZQBhAG4AZQBzAHQAIAByAHUAbgAgAGEAbgBkACAAYQB2AGUAcgBhAGcAZQAgAGkAdAAgAGQAbwB3AG4AIAB0AG8AIABhACAAcwBpAG4AZwBsAGUAIABlAHgAZQBjAHUAdABpAG8AbgAgAHQAaQBtAGUAXABuACAAIAAgACAAIAAgACAAIABNAEkATgAoAGIAYQB0AGMAaABfAHQAaQBtAGUAcwApACAALwAgAGkAdABlAHIAcwBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAARQB4AGUAYwB1AHQAZQBzACAAYQAgAHMAdAByAGkAYwB0AGwAeQAgAHMAZQBxAHUAZQBuAHQAaQBhAGwAIABiAGUAbgBjAGgAbQBhAHIAawAgAHMAdQBpAHQAZQAgAHQAbwAgAGEAdgBvAGkAZAAgAG0AdQBsAHQAaQAtAHQAaAByAGUAYQBkAGkAbgBnACAAYwBvAG4AdABhAG0AaQBuAGEAdABpAG8AbgAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAHQAZQBzAHQAXwBjAGEAcwBlAHMAIABBAG4AIABOACAAeAAgADIAIABhAHIAcgBhAHkAIABvAGYAIAB0AGUAcwB0ACAAbABlAG4AZwB0AGgAcwA6ACAAWwBMAGUAbgBnAHQAaABfAEEALAAgAEwAZQBuAGcAdABoAF8AQgBdAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAGkAdABlAHIAcwAgAE4AdQBtAGIAZQByACAAbwBmACAAaQB0AGUAcgBhAHQAaQBvAG4AcwAgAHAAZQByACAAYgBlAG4AYwBoAG0AYQByAGsAIAB0AG8AIABzAG0AbwBvAHQAaAAgAE4ATwBXACgAKQAgAHIAZQBzAG8AbAB1AHQAaQBvAG4ALgBcAG4AIAAqAC8AXABuAEQAaQB2AGkAcwBpAG8AbgBBAGwAZwBvAHIAaQB0AGgAbQBDAG8AbQBwAGEAcgBpAHMAbwBuACAAPQAgAEwAQQBNAEIARABBACgAdABlAHMAdABfAGMAYQBzAGUAcwAsACAAaQB0AGUAcgBzACwAIAByAGUAcABlAGEAdABzACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG4AXwB0AGUAcwB0AHMALAAgAFIATwBXAFMAKAB0AGUAcwB0AF8AYwBhAHMAZQBzACkALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAALwAvACAASQBuAGkAdABpAGEAbAAgAHMAdABhAHQAZQA6ACAARABhAHQAYQAgAGgAZQBhAGQAZQByAHMAIABmAG8AcgAgAEMAUwBWACAAZQB4AHAAbwByAHQAXABuACAAIAAgACAAIAAgACAAIABpAG4AaQB0AGkAYQBsACwAIAB7AFwAIgBMAGUAbgBfAEEAXAAiACwAIABcACIATABlAG4AXwBCAFwAIgAsACAAXAAiAEsAbgB1AHQAaABfAG0AcwBcACIALAAgAFwAIgBOAFIAXwBtAHMAXAAiAH0ALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAUgBFAEQAVQBDAEUAKABpAG4AaQB0AGkAYQBsACwAIABTAEUAUQBVAEUATgBDAEUAKABuAF8AdABlAHMAdABzACkALAAgAEwAQQBNAEIARABBACgAYQBjAGMALAAgAGkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGUAbgBfAGEALAAgAEkATgBEAEUAWAAoAHQAZQBzAHQAXwBjAGEAcwBlAHMALAAgAGkALAAgADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAZQBuAF8AYgAsACAASQBOAEQARQBYACgAdABlAHMAdABfAGMAYQBzAGUAcwAsACAAaQAsACAAMgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAAUwBrAGkAcAAgAEQAaQB2AGkAcwBvAHIAIAA+ACAARABpAHYAaQBkAGUAbgBkABQgaQB0ACcAcwAgAG4AZQB2AGUAcgAgAGEAbgAgAGkAbgB0AGUAZwBlAHIAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgAbABlAG4AXwBiACAAPgAgAGwAZQBuAF8AYQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABhAGMAYwAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAARwBlAG4AZQByAGEAdABlACAAZQB4AGEAYwB0AC0AbABlAG4AZwB0AGgAIAB0AGUAcwB0ACAAcwB0AHIAaQBuAGcAcwAgAG4AYQB0AGkAdgBlAGwAeQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcwB0AHIAXwBhACwAIABSAEUAUABUACgAXAAiADkAXAAiACwAIABsAGUAbgBfAGEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABzAHQAcgBfAGIALAAgAEkARgAoAGwAZQBuAF8AYgAgAD0AIAAxACwAIABcACIANwBcACIALAAgAFwAIgA3AFwAIgAgACYAIABSAEUAUABUACgAXAAiADMAXAAiACwAIABsAGUAbgBfAGIAIAAtACAAMQApACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAEUAeABlAGMAdQB0AGUAIABiAGUAbgBjAGgAbQBhAHIAawBzACAAcwB0AHIAaQBjAHQAbAB5ACAAbwBuAGUAIABhAGYAdABlAHIAIAB0AGgAZQAgAG8AdABoAGUAcgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAdABpAG0AZQBfAGsALAAgAEQAaQB2AGkAcwBpAG8AbgBBAGwAZwBvAHIAaQB0AGgAbQBzACgAcwB0AHIAXwBhACwAIABzAHQAcgBfAGIALAAgAFwAIgBLAE4AVQBUAEgAXAAiACwAIABpAHQAZQByAHMALAAgAHIAZQBwAGUAYQB0AHMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAB0AGkAbQBlAF8AbgByACwAIABEAGkAdgBpAHMAaQBvAG4AQQBsAGcAbwByAGkAdABoAG0AcwAoAHMAdAByAF8AYQAsACAAcwB0AHIAXwBiACwAIABcACIATgBSAFwAIgAsACAAaQB0AGUAcgBzACwAIAByAGUAcABlAGEAdABzACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAEEAcABwAGUAbgBkACAAdABoAGUAIAByAGUAcwB1AGwAdABzAC4AIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAAUgBlAGEAbABsAG8AYwBhAHQAaQBvAG4AIABkAGUAbABhAHkAIABvAGMAYwB1AHIAcwAgAGgAZQByAGUALAAgAHMAYQBmAGUAbAB5ACAAbwB1AHQAcwBpAGQAZQAgAHQAaABlACAAdABpAG0AZQBkACAAdwBpAG4AZABvAHcALgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAVgBTAFQAQQBDAEsAKABhAGMAYwAsACAASABTAFQAQQBDAEsAKABsAGUAbgBfAGEALAAgAGwAZQBuAF8AYgAsACAAdABpAG0AZQBfAGsALAAgAHQAaQBtAGUAXwBuAHIAKQApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8ALwAgAEcAZQBuAGUAcgBhAHQAZQBzACAAYQAgADIALQBjAG8AbAB1AG0AbgAgAGEAcgByAGEAeQAgAG8AZgAgAGUAdgBlAHIAeQAgAGMAbwBtAGIAaQBuAGEAdABpAG8AbgAgAG8AZgAgAGwAZQBuAGcAdABoAHMAXABuAEQAaQB2AGkAcwBpAG8AbgBCAGUAbgBjAGgAbQBhAHIAawBDAGEAcwBlAHMAIAA9ACAATABBAE0AQgBEAEEAKABzAHQAYQByAHQAXwBsAGUAbgAsACAAbQBhAHgAXwBsAGUAbgAsACAAcwB0AGUAcAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABzAGUAcQAsACAAUwBFAFEAVQBFAE4AQwBFACgAKABtAGEAeABfAGwAZQBuACAALQAgAHMAdABhAHIAdABfAGwAZQBuACkAIAAvACAAcwB0AGUAcAAgACsAIAAxACwAIAAxACwAIABzAHQAYQByAHQAXwBsAGUAbgAsACAAcwB0AGUAcAApACwAXABuACAAIAAgACAAIAAgACAAIABuACwAIABSAE8AVwBTACgAcwBlAHEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABDAGEAcgB0AGUAcwBpAGEAbgAgAEoAbwBpAG4AXABuACAAIAAgACAAIAAgACAAIABjAG8AbABfAGEALAAgAFQATwBDAE8ATAAoAEkARgAoAFMARQBRAFUARQBOAEMARQAoADEALAAgAG4AKQAsACAAcwBlAHEAKQApACwAXABuACAAIAAgACAAIAAgACAAIABjAG8AbABfAGIALAAgAFQATwBDAE8ATAAoAEkARgAoAFMARQBRAFUARQBOAEMARQAoAG4ALAAgADEAKQAsACAAVABPAFIATwBXACgAcwBlAHEAKQApACkALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAASABTAFQAQQBDAEsAKABjAG8AbABfAGEALAAgAGMAbwBsAF8AYgApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8ALwAgAEcAZQBuAGUAcgBhAHQAZQBzACAAYQAgAEMAYQByAHQAZQBzAGkAYQBuACAAZwByAGkAZAAgAGYAcgBvAG0AIAB0AHcAbwAgAGkAbgBkAGUAcABlAG4AZABlAG4AdAAgAHMAZQBxAHUAZQBuAGMAZQBzAFwAbgBBAHMAeQBtAG0AZQB0AHIAaQBjAEEAQgBHAHIAaQBkACAAPQAgAEwAQQBNAEIARABBACgAcwB0AGEAcgB0AF8AYQAsACAAbQBhAHgAXwBhACwAIABzAHQAZQBwAF8AYQAsACAAcwB0AGEAcgB0AF8AYgAsACAAbQBhAHgAXwBiACwAIABzAHQAZQBwAF8AYgAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABzAGUAcQBfAGEALAAgAFMARQBRAFUARQBOAEMARQAoACgAbQBhAHgAXwBhACAALQAgAHMAdABhAHIAdABfAGEAKQAgAC8AIABzAHQAZQBwAF8AYQAgACsAIAAxACwAIAAxACwAIABzAHQAYQByAHQAXwBhACwAIABzAHQAZQBwAF8AYQApACwAXABuACAAIAAgACAAIAAgACAAIABzAGUAcQBfAGIALAAgAFMARQBRAFUARQBOAEMARQAoACgAbQBhAHgAXwBiACAALQAgAHMAdABhAHIAdABfAGIAKQAgAC8AIABzAHQAZQBwAF8AYgAgACsAIAAxACwAIAAxACwAIABzAHQAYQByAHQAXwBiACwAIABzAHQAZQBwAF8AYgApACwAXABuACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgAG4AXwBhACwAIABSAE8AVwBTACgAcwBlAHEAXwBhACkALABcAG4AIAAgACAAIAAgACAAIAAgAG4AXwBiACwAIABSAE8AVwBTACgAcwBlAHEAXwBiACkALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAALwAvACAATwByAHQAaABvAGcAbwBuAGEAbAAgAGIAcgBvAGEAZABjAGEAcwB0ACAAdQBzAGkAbgBnACAAaQBuAGQAZQBwAGUAbgBkAGUAbgB0ACAAZABpAG0AZQBuAHMAaQBvAG4AcwBcAG4AIAAgACAAIAAgACAAIAAgAGMAbwBsAF8AYQAsACAAVABPAEMATwBMACgASQBGACgAUwBFAFEAVQBFAE4AQwBFACgAMQAsACAAbgBfAGIAKQAsACAAcwBlAHEAXwBhACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAYwBvAGwAXwBiACwAIABUAE8AQwBPAEwAKABJAEYAKABTAEUAUQBVAEUATgBDAEUAKABuAF8AYQApACwAIABUAE8AUgBPAFcAKABzAGUAcQBfAGIAKQApACkALABcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAASABTAFQAQQBDAEsAKABjAG8AbABfAGEALAAgAGMAbwBsAF8AYgApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAEYAYQBjAHQAbwByAGkAYQBsAEEAbABnAG8AcgBpAHQAaABtAHMAIAA9ACAATABBAE0AQgBEAEEAKABpAG4AcAB1AHQALAAgAG0AbwBkAGUALAAgAGkAdABlAHIAcwAsACAAcgBlAHAAZQBhAHQAcwAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABNAGEAcAAgAHQAaABlACAAbwB1AHQAZQByACAAcgBlAHAAZQBhAHQAcwAgAGwAbwBvAHAAXABuACAAIAAgACAAIAAgACAAIABiAGEAdABjAGgAXwB0AGkAbQBlAHMALAAgAE0AQQBQACgAUwBFAFEAVQBFAE4AQwBFACgAcgBlAHAAZQBhAHQAcwApACwAIABMAEEATQBCAEQAQQAoAHIALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQALAAgAE4ATwBXACgAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAE0AYQBwACAAdABoAGUAIABpAG4AbgBlAHIAIABlAHgAZQBjAHUAdABpAG8AbgAgAGwAbwBvAHAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcgB1AG4ALAAgAEkARgAoAG0AbwBkAGUAIAA9ACAAXAAiAEwAZQBnAGUAbgBkAHIAZQBcACIALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEEAUAAoAFMARQBRAFUARQBOAEMARQAoAGkAdABlAHIAcwApACwAIABMAEEATQBCAEQAQQAoAGkALAAgAEIAaQBnAEkAbgB0AC4ARgBhAGMAdAAoAGkAbgBwAHUAdAApACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEEAUAAoAFMARQBRAFUARQBOAEMARQAoAGkAdABlAHIAcwApACwAIABMAEEATQBCAEQAQQAoAGkALAAgAEIAaQBnAEkAbgB0AC4ARgBhAGMAdABTAHcAaQBuAGcAKABpAG4AcAB1AHQAKQApACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAEYAbwByAGMAZQAgAGUAdgBhAGwAdQBhAHQAaQBvAG4AIABiAGUAZgBvAHIAZQAgAHAAdQBsAGwAaQBuAGcAIABzAHQAbwBwACAAdABpAG0AZQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABzAHQAbwBwACwAIABOAE8AVwAoACkAIAArACAAKAAwACAAKgAgAEwARQBOACgASQBOAEQARQBYACgAcgB1AG4ALAAgADEALAAgADEAKQApACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIABUAG8AdABhAGwAIABiAGEAdABjAGgAIAB0AGkAbQBlACAAaQBuACAAbQBpAGwAbABpAHMAZQBjAG8AbgBkAHMAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABzAHQAbwBwACAALQAgAHMAdABhAHIAdAApACAAKgAgADgANgA0ADAAMAAwADAAMABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABFAHgAdAByAGEAYwB0ACAAdABoAGUAIABjAGwAZQBhAG4AZQBzAHQAIAByAHUAbgAgAGEAbgBkACAAYQB2AGUAcgBhAGcAZQAgAGkAdAAgAGQAbwB3AG4AIAB0AG8AIABhACAAcwBpAG4AZwBsAGUAIABlAHgAZQBjAHUAdABpAG8AbgAgAHQAaQBtAGUAXABuACAAIAAgACAAIAAgACAAIABNAEkATgAoAGIAYQB0AGMAaABfAHQAaQBtAGUAcwApACAALwAgAGkAdABlAHIAcwBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAARQB4AGUAYwB1AHQAZQBzACAAYQAgAHMAdAByAGkAYwB0AGwAeQAgAHMAZQBxAHUAZQBuAHQAaQBhAGwAIABiAGUAbgBjAGgAbQBhAHIAawAgAHMAdQBpAHQAZQAgAHQAbwAgAGEAdgBvAGkAZAAgAG0AdQBsAHQAaQAtAHQAaAByAGUAYQBkAGkAbgBnACAAYwBvAG4AdABhAG0AaQBuAGEAdABpAG8AbgAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAHQAZQBzAHQAXwBjAGEAcwBlAHMAIABBAG4AIABOACAAeAAgADEAIABhAHIAcgBhAHkAIABvAGYAIAB0AGUAcwB0ACAAaQBuAHAAdQB0AHMAXABuACAAKgAgAEAAcABhAHIAYQBtACAAaQB0AGUAcgBzACAATgB1AG0AYgBlAHIAIABvAGYAIABpAHQAZQByAGEAdABpAG8AbgBzACAAcABlAHIAIABzAGEAbQBwAGwAZQAgAHQAbwAgAHMAbQBvAG8AdABoACAATgBPAFcAKAApACAAcgBlAHMAbwBsAHUAdABpAG8AbgAuAFwAbgAgACoAIABAAHAAYQByAGEAbQAgAHIAZQBwAGUAYQB0AHMAIABOAHUAbQBiAGUAcgAgAG8AZgAgAGkAdABlAHIAYQB0AGkAbwBuAHMAIABwAGUAcgAgAGIAZQBuAGMAaABtAGEAcgBrACAAdABvACAAcwBtAG8AbwB0AGgAIABPAFMAIABhAG4AZAAgAGIAYQBjAGsAZwByAG8AdQBuAGQAIABuAG8AaQBzAGUALgBcAG4AIAAqAC8AXABuAEYAYQBjAHQAbwByAGkAYQBsAEMAbwBtAHAAYQByAGkAcwBvAG4AIAA9ACAATABBAE0AQgBEAEEAKAB0AGUAcwB0AF8AYwBhAHMAZQBzACwAIABpAHQAZQByAHMALAAgAHIAZQBwAGUAYQB0AHMALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbgBfAHQAZQBzAHQAcwAsACAAUgBPAFcAUwAoAHQAZQBzAHQAXwBjAGEAcwBlAHMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABJAG4AaQB0AGkAYQBsACAAcwB0AGEAdABlADoAIABEAGEAdABhACAAaABlAGEAZABlAHIAcwAgAGYAbwByACAAQwBTAFYAIABlAHgAcABvAHIAdABcAG4AIAAgACAAIAAgACAAIAAgAGkAbgBpAHQAaQBhAGwALAAgAHsAXAAiAE4AXAAiACwAIABcACIATABlAGcAZQBuAGQAcgBlAFwAIgAsACAAXAAiAFMAdwBpAG4AZwBcACIAfQAsAFwAbgAgACAAIAAgACAAIAAgACAAXABuACAAIAAgACAAIAAgACAAIABSAEUARABVAEMARQAoAGkAbgBpAHQAaQBhAGwALAAgAFMARQBRAFUARQBOAEMARQAoAG4AXwB0AGUAcwB0AHMAKQAsACAATABBAE0AQgBEAEEAKABhAGMAYwAsACAAaQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGkAbgBwAHUAdAAsACAASQBOAEQARQBYACgAdABlAHMAdABfAGMAYQBzAGUAcwAsACAAaQAsACAAMQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAARQB4AGUAYwB1AHQAZQAgAGIAZQBuAGMAaABtAGEAcgBrAHMAIABzAHQAcgBpAGMAdABsAHkAIABvAG4AZQAgAGEAZgB0AGUAcgAgAHQAaABlACAAbwB0AGgAZQByAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHQAaQBtAGUAXwBsAGUAZwBlAG4AZAByAGUALAAgAEYAYQBjAHQAbwByAGkAYQBsAEEAbABnAG8AcgBpAHQAaABtAHMAKABpAG4AcAB1AHQALAAgAFwAIgBMAGUAZwBlAG4AZAByAGUAXAAiACwAIABpAHQAZQByAHMALAAgAHIAZQBwAGUAYQB0AHMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHQAaQBtAGUAXwBzAHcAaQBuAGcALAAgAEYAYQBjAHQAbwByAGkAYQBsAEEAbABnAG8AcgBpAHQAaABtAHMAKABpAG4AcAB1AHQALAAgAFwAIgBTAHcAaQBuAGcAXAAiACwAIABpAHQAZQByAHMALAAgAHIAZQBwAGUAYQB0AHMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAEEAcABwAGUAbgBkACAAdABoAGUAIAByAGUAcwB1AGwAdABzAC4AIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIABSAGUAYQBsAGwAbwBjAGEAdABpAG8AbgAgAGQAZQBsAGEAeQAgAG8AYwBjAHUAcgBzACAAaABlAHIAZQAsACAAcwBhAGYAZQBsAHkAIABvAHUAdABzAGkAZABlACAAdABoAGUAIAB0AGkAbQBlAGQAIAB3AGkAbgBkAG8AdwAuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFYAUwBUAEEAQwBLACgAYQBjAGMALAAgAEgAUwBUAEEAQwBLACgAaQBuAHAAdQB0ACwAIAB0AGkAbQBlAF8AbABlAGcAZQBuAGQAcgBlACwAIAB0AGkAbQBlAF8AcwB3AGkAbgBnACkAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBjAG8AcgBlAF8AQgBpAGcASQBuAHQAIgAsACIAdABlAHgAdAAiADoAIgAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwBcAG4ALwAvACAAQgBpAGcAIABJAG4AdABlAGcAZQByACAAQQByAGkAdABoAG0AZQB0AGkAYwAgAEwAaQBiAHIAYQByAHkAIAAvAC8AXABuAC8ALwAgACAAIAAgACAAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQAIABNAG8AZAB1AGwAZQAgACAAIAAgACAAIAAgACAALwAvAFwAbgAvAC8AIAAgACAAIAAgACAAIAAgACAAIABQAHIAaQB2AGEAdABlACAAQQBQAEkAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwBcAG4ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8AXABuAFwAbgAvACoAKgBcAG4AIAAqACAAWwBJAG4AdABlAHIAbgBhAGwAXQAgAFIAZQB0AHUAcgBuAHMAIABtAGEAeAAgAHMAYQBmAGUAIABiAGEAcwBlAC0AMQAwACAAbABpAG0AYgAgAHMAaQB6AGUAIAAoAGsAKQAgAHQAbwAgAHAAcgBlAHYAZQBuAHQAIABJAEUARQBFAC0ANwA1ADQAIABwAHIAZQBjAGkAcwBpAG8AbgAgAGwAbwBzAHMALgBcAG4AIAAqACAAWwBvAHAAZQByAGEAdABpAG8AbgA6ACAAVABlAHgAdAAsACAAbwBwAGUAcgBhAG4AZABfAG8AcgBfAGQAaQBnAGkAdABzADoAIABpAG4AdABdAFwAbgAgACoALwBcAG4AUwBhAGYAZQBLACAAPQAgAEwAQQBNAEIARABBACgAbwBwAGUAcgBhAHQAaQBvAG4ALAAgAFsAbwBwAGUAcgBhAG4AZABfAG8AcgBfAGQAaQBnAGkAdABzAF0ALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAcgBlAHMAbwBsAHYAZQBkAF8AYwBvAHUAbgB0ACwAIABJAEYAKABPAFIAKABvAHAAZQByAGEAbgBkAF8AbwByAF8AZABpAGcAaQB0AHMAIAA9ACAAXAAiAFwAIgAsACAASQBTAE8ATQBJAFQAVABFAEQAKABvAHAAZQByAGEAbgBkAF8AbwByAF8AZABpAGcAaQB0AHMAKQApACwAIAAyACwAIABNAEEAWAAoADIALAAgAG8AcABlAHIAYQBuAGQAXwBvAHIAXwBkAGkAZwBpAHQAcwApACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIABTAFcASQBUAEMASAAoAG8AcABlAHIAYQB0AGkAbwBuACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAEQARABcACIALAAgADEANQAgAC0AIABMAEUATgAoAHIAZQBzAG8AbAB2AGUAZABfAGMAbwB1AG4AdAApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIATQBVAEwAXAAiACwAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHQAZQBzAHQAXwBrACwAIAB7ADcAOwAgADYAOwAgADUAOwAgADQAOwAgADMAOwAgADIAOwAgADEAfQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABtAGEAeABfAG8AdgBlAHIAbABhAHAALAAgAFIATwBVAE4ARABVAFAAKAByAGUAcwBvAGwAdgBlAGQAXwBjAG8AdQBuAHQAIAAvACAAdABlAHMAdABfAGsALAAgADAAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIABEAGUAdABlAHIAbQBpAG4AZQAgAGsAIABiAHkAIABzAGkAbQB1AGwAYQB0AGkAbgBnACAAdABoAGUAIAB3AG8AcgBzAHQALQBjAGEAcwBlACAAYwBvAG4AdgBvAGwAdQB0AGkAbwBuACAAcABlAGEAawAgAHQAbwAgAHAAcgBlAHYAZQBuAHQAIABJAEUARQBFAC0ANwA1ADQAIABwAHIAZQBjAGkAcwBpAG8AbgAgAGIAbABlAGUAZABpAG4AZwAuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAFAAZQBhAGsAIAB2AGEAbAB1AGUAIABpAG4AYwBsAHUAZABlAHMAIAB0AGgAZQAgAG0AYQB4AGkAbQB1AG0AIABwAG8AcwBzAGkAYgBsAGUAIAB1AG4AYwBhAHIAcgBpAGUAZAAgAHAAcgBvAGQAdQBjAHQAIABwAGwAdQBzACAAdABoAGUAIABtAGEAeABpAG0AdQBtACAAcABvAHQAZQBuAHQAaQBhAGwAIABjAGEAcgByAHkALgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAB1AG4AYwBhAHIAcgBpAGUAZABfAG0AYQB4ACwAIABtAGEAeABfAG8AdgBlAHIAbABhAHAAIAAqACAAKAAxADAAXgB0AGUAcwB0AF8AawAgAC0AIAAxACkAXgAyACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbQBhAHgAXwBjAGEAcgByAHkALAAgAEkATgBUACgAdQBuAGMAYQByAHIAaQBlAGQAXwBtAGEAeAAgAC8AIAAxADAAXgB0AGUAcwB0AF8AawApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcABlAGEAawBfAHYAYQBsACwAIAB1AG4AYwBhAHIAcgBpAGUAZABfAG0AYQB4ACAAKwAgAG0AYQB4AF8AYwBhAHIAcgB5ACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAFIAZQB0AHUAcgBuACAAdABoAGUAIABtAGEAeAAgAGsAIAA8AD0AIABFAHgAYwBlAGwAJwBzACAAMQA1AC0AZABpAGcAaQB0ACAAYwBlAGkAbABpAG4AZwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEEAWAAoAEYASQBMAFQARQBSACgAdABlAHMAdABfAGsALAAgAHAAZQBhAGsAXwB2AGEAbAAgADwAPQAgACgAMQAwAF4AMQA1ACAALQAgADEAKQApACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAEkAVgBcACIALAAgADcALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIwBOAEEATQBFAD8AXABuACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABbAEkAbgB0AGUAcgBuAGEAbABdACAAUwBwAGwAaQB0AHMAIABzAHQAcgBpAG4AZwBzACAAbwByACAAYQByAHIAYQB5AHMAIABpAG4AdABvACAATABpAHQAdABsAGUALQBFAG4AZABpAGEAbgAgAG4AdQBtAGUAcgBpAGMAIABsAGkAbQBiACAAYQByAHIAYQB5AHMALgBcAG4AIAAqACAAWwBzAHQAcgBfAG4AbwByAG0AcwA6ACAAVABlAHgAdAAvAEEAcgByAGEAeQAsACAAawA6ACAAaQBuAHQAXQBcAG4AIAAqAC8AXABuAFMAcABsAGkAdAAgAD0AIABMAEEATQBCAEQAQQAoAHMAdAByAF8AbgBvAHIAbQBzACwAIABrACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAGYAbABhAHQAdABlAG4AZQBkAF8AbgBvAHIAbQBzACwAIABUAE8AUgBPAFcAKABzAHQAcgBfAG4AbwByAG0AcwApACwAXABuACAAIAAgACAAIAAgACAAIABsAGUAbgBnAHQAaABzACwAIABMAEUATgAoAGYAbABhAHQAdABlAG4AZQBkAF8AbgBvAHIAbQBzACkALABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQB4AF8AbABlAG4ALAAgAE0AQQBYACgAbABlAG4AZwB0AGgAcwApACwAXABuACAAIAAgACAAIAAgACAAIABwAGEAZABfAGwAZQBuACwAIABSAE8AVQBOAEQAVQBQACgAbQBhAHgAXwBsAGUAbgAgAC8AIABrACwAIAAwACkAIAAqACAAawAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAHAAYQBkAGQAZQBkAF8AbgBvAHIAbQBzACwAIABSAEUAUABUACgAXAAiADAAXAAiACwAIABwAGEAZABfAGwAZQBuACAALQAgAGwAZQBuAGcAdABoAHMAKQAgACYAIABmAGwAYQB0AHQAZQBuAGUAZABfAG4AbwByAG0AcwAsAFwAbgAgACAAIAAgACAAIAAgACAAbABpAG0AYgBfAHMAdABhAHIAdABfAGkAbgBkAGkAYwBlAHMALAAgAFMARQBRAFUARQBOAEMARQAoAHAAYQBkAF8AbABlAG4AIAAvACAAawAsACAAMQAsACAAcABhAGQAXwBsAGUAbgAgAC0AIABrACAAKwAgADEALAAgAC0AawApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAALQAtAE0ASQBEACgAcABhAGQAZABlAGQAXwBuAG8AcgBtAHMALAAgAGwAaQBtAGIAXwBzAHQAYQByAHQAXwBpAG4AZABpAGMAZQBzACwAIABrACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFsASQBuAHQAZQByAG4AYQBsAF0AIABNAGUAcgBnAGUAcwAgAEwAaQB0AHQAbABlAC0ARQBuAGQAaQBhAG4AIABsAGkAbQBiACAAYQByAHIAYQB5AHMAIABpAG4AdABvACAAYQAgAEIAaQBnAC0ARQBuAGQAaQBhAG4AIABCAGkAZwBJAG4AdAAgAHMAdAByAGkAbgBnAC4AXABuACAAKgAgAFsAbABpAG0AYgBzADoAIABBAHIAcgBhAHkALAAgAGsAOgAgAGkAbgB0AF0AXABuACAAKgAvAFwAbgBNAGUAcgBnAGUAIAA9ACAATABBAE0AQgBEAEEAKABsAGkAbQBiAHMALAAgAGsALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbgB1AG0AXwBsAGkAbQBiAHMALAAgAFIATwBXAFMAKABsAGkAbQBiAHMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcgBlAHYAXwBsAGkAbQBiAHMALAAgAEMASABPAE8AUwBFAFIATwBXAFMAKABsAGkAbQBiAHMALAAgAFMARQBRAFUARQBOAEMARQAoAG4AdQBtAF8AbABpAG0AYgBzACwAIAAxACwAIABuAHUAbQBfAGwAaQBtAGIAcwAsACAALQAxACkAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAG4AdQBtAF8AbABpAG0AYgBzACAAPQAgADEALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAcgBlAHYAXwBsAGkAbQBiAHMAIAAmACAAXAAiAFwAIgAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABDAE8ATgBDAEEAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFYAUwBUAEEAQwBLACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABUAEEASwBFACgAcgBlAHYAXwBsAGkAbQBiAHMALAAgADEAKQAgACYAIABcACIAXAAiACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABUAEUAWABUACgARABSAE8AUAAoAHIAZQB2AF8AbABpAG0AYgBzACwAIAAxACkALAAgAFIARQBQAFQAKABcACIAMABcACIALAAgAGsAKQApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABbAEkAbgB0AGUAcgBuAGEAbABdACAAUgBlAHMAbwBsAHYAZQBzACAAYwBhAHIAcgBpAGUAcwAgAHIAaQBnAGgAdAAtAHQAbwAtAGwAZQBmAHQAIABhAGMAcgBvAHMAcwAgAGEAIAB2AGUAcgB0AGkAYwBhAGwAIABhAHIAcgBhAHkAIABvAGYAIABiAGEAcwBlAC0AMQAwAF4AawAgAGwAaQBtAGIAcwAuAFwAbgAgACoAIABbAGwAaQBtAGIAcwA6ACAAQQByAHIAYQB5ACwAIABrADoAIABpAG4AdABdAFwAbgAgACoALwBcAG4AQwBhAHIAcgB5ACAAPQAgAEwAQQBNAEIARABBACgAbABpAG0AYgBzACwAIABrACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG4AdQBtAF8AbABpAG0AYgBzACwAIABSAE8AVwBTACgAbABpAG0AYgBzACkALABcAG4AIAAgACAAIAAgACAAIAAgAHIAYQBkAGkAeABfAGIAYQBzAGUALAAgADEAMABeAGsALABcAG4AIAAgACAAIAAgACAAIAAgAC8ALwAgAFMAQwBBAE4AIABzAGkAbQB1AGwAYQB0AGUAcwAgAHQAaABlACAAcwBlAHIAaQBhAGwAIABwAHIAbwBwAGEAZwBhAHQAaQBvAG4AIABvAGYAIABjAGEAcgByAGkAZQBzACAAdABoAHIAbwB1AGcAaAAgAHQAaABlACAAYQByAHIAYQB5ACAAaQBuACAAYQAgAHMAaQBuAGcAbABlACAAdgBlAGMAdABvAHIAaQB6AGUAZAAgAHAAYQBzAHMALgBcAG4AIAAgACAAIAAgACAAIAAgAGEAcgByAF8AYwBhAHIAcgBpAGUAcwAsACAAUwBDAEEATgAoADAALAAgAGwAaQBtAGIAcwAsACAATABBAE0AQgBEAEEAKABhAGMAYwAsACAAdgBhAGwALAAgAHYAYQBsACAAKwAgAEkATgBUACgAYQBjAGMAIAAvACAAcgBhAGQAaQB4AF8AYgBhAHMAZQApACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcgBlAG0AYQBpAG4AZABlAHIAcwAsACAATQBPAEQAKABhAHIAcgBfAGMAYQByAHIAaQBlAHMALAAgAHIAYQBkAGkAeABfAGIAYQBzAGUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAG4AYQBsAF8AYwBhAHIAcgB5ACwAIABJAE4AVAAoAEkATgBEAEUAWAAoAGEAcgByAF8AYwBhAHIAcgBpAGUAcwAsACAAbgB1AG0AXwBsAGkAbQBiAHMALAAgADEAKQAgAC8AIAByAGEAZABpAHgAXwBiAGEAcwBlACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIABJAEYAKABmAGkAbgBhAGwAXwBjAGEAcgByAHkAIAA+ACAAMAAsACAAVgBTAFQAQQBDAEsAKAByAGUAbQBhAGkAbgBkAGUAcgBzACwAIABmAGkAbgBhAGwAXwBjAGEAcgByAHkAKQAsACAAcgBlAG0AYQBpAG4AZABlAHIAcwApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8ALwAgAC0ALQAtACAAVQBuAHMAaQBnAG4AZQBkACAASwBlAHIAbgBlAGwAcwAgAC0ALQAtACAAXABcAFwAXABcAG4AXABuAC8AKgAqAFwAbgAgACoAIABbAEkAbgB0AGUAcgBuAGEAbABdACAAUgBlAHQAdQByAG4AcwAgADEAIAAoAGEAIAA+ACAAYgApACwAIAAtADEAIAAoAGEAIAA8ACAAYgApACwAIABvAHIAIAAwACAAKABhACAAPQAgAGIAKQAgAGYAbwByACAAdQBuAHMAaQBnAG4AZQBkACAAbABpAG0AYgAgAGEAcgByAGEAeQBzAC4AXABuACAAKgAgAFsAbABpAG0AYgBzAF8AYQA6ACAAQQByAHIAYQB5ACwAIABsAGkAbQBiAHMAXwBiADoAIABBAHIAcgBhAHkAXQBcAG4AIAAqAC8AXABuAFUAQwBvAG0AcABhAHIAZQAgAD0AIABMAEEATQBCAEQAQQAoAGwAaQBtAGIAcwBfAGEALAAgAGwAaQBtAGIAcwBfAGIALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHgAXwByAG8AdwBzACwAIABNAEEAWAAoAFIATwBXAFMAKABsAGkAbQBiAHMAXwBhACkALAAgAFIATwBXAFMAKABsAGkAbQBiAHMAXwBiACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYQBfAGEAbABpAGcAbgBlAGQALAAgAEUAWABQAEEATgBEACgAbABpAG0AYgBzAF8AYQAsACAAbQBhAHgAXwByAG8AdwBzACwAIAAxACwAIAAwACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGIAXwBhAGwAaQBnAG4AZQBkACwAIABFAFgAUABBAE4ARAAoAGwAaQBtAGIAcwBfAGIALAAgAG0AYQB4AF8AcgBvAHcAcwAsACAAMQAsACAAMAApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAZABpAGYAZgBlAHIAZQBuAGMAZQBzACwAIABsAGkAbQBiAHMAXwBhAF8AYQBsAGkAZwBuAGUAZAAgAC0AIABsAGkAbQBiAHMAXwBiAF8AYQBsAGkAZwBuAGUAZAAsAFwAbgAgACAAIAAgACAAIAAgACAALwAvACAAUwBlAGEAcgBjAGgAaQBuAGcAIABmAHIAbwBtACAAdABoAGUAIABiAG8AdAB0AG8AbQAgACgAaABpAGcAaABlAHMAdAAgAG0AYQBnAG4AaQB0AHUAZABlACkAIABlAG4AcwB1AHIAZQBzACAAdABoAGUAIABtAG8AcwB0ACAAcwBpAGcAbgBpAGYAaQBjAGEAbgB0ACAAZABpAGYAZgBlAHIAZQBuAGMAZQAgAGkAcwAgAGYAbwB1AG4AZAAgAGYAaQByAHMAdAAuAFwAbgAgACAAIAAgACAAIAAgACAAaABpAGcAaABlAHMAdABfAG4AbwBuAF8AegBlAHIAbwBfAGkAbgBkAGUAeAAsACAAWABNAEEAVABDAEgAKABUAFIAVQBFACwAIABkAGkAZgBmAGUAcgBlAG4AYwBlAHMAIAA8AD4AIAAwACwAIAAwACwAIAAtADEAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAEkAUwBOAEEAKABoAGkAZwBoAGUAcwB0AF8AbgBvAG4AXwB6AGUAcgBvAF8AaQBuAGQAZQB4ACkALAAgADAALAAgAFMASQBHAE4AKABJAE4ARABFAFgAKABkAGkAZgBmAGUAcgBlAG4AYwBlAHMALAAgAGgAaQBnAGgAZQBzAHQAXwBuAG8AbgBfAHoAZQByAG8AXwBpAG4AZABlAHgALAAgADEAKQApACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFsASQBuAHQAZQByAG4AYQBsAF0AIABSAGUAdAB1AHIAbgBzACAAdABoAGUAIABzAHUAbQAgAG8AZgAgAHQAdwBvACAAdQBuAHMAaQBnAG4AZQBkACAATABpAHQAdABsAGUALQBFAG4AZABpAGEAbgAgAGwAaQBtAGIAIABhAHIAcgBhAHkAcwAuAFwAbgAgACoAIABbAGEAOgAgAEEAcgByAGEAeQAsACAAYgA6ACAAQQByAHIAYQB5ACwAIABrADoAIABpAG4AdABdAFwAbgAgACoALwBcAG4AVQBBAGQAZAAgAD0AIABMAEEATQBCAEQAQQAoAGEALAAgAGIALAAgAGsALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHgAXwByAG8AdwBzACwAIABNAEEAWAAoAFIATwBXAFMAKABhACkALAAgAFIATwBXAFMAKABiACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYQBfAGEAbABpAGcAbgBlAGQALAAgAEUAWABQAEEATgBEACgAYQAsACAAbQBhAHgAXwByAG8AdwBzACwAIAAxACwAIAAwACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGIAXwBhAGwAaQBnAG4AZQBkACwAIABFAFgAUABBAE4ARAAoAGIALAAgAG0AYQB4AF8AcgBvAHcAcwAsACAAMQAsACAAMAApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAQwBhAHIAcgB5ACgAbABpAG0AYgBzAF8AYQBfAGEAbABpAGcAbgBlAGQAIAArACAAbABpAG0AYgBzAF8AYgBfAGEAbABpAGcAbgBlAGQALAAgAGsAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAAWwBJAG4AdABlAHIAbgBhAGwAXQAgAFIAZQB0AHUAcgBuAHMAIAB0AGgAZQAgAGQAaQBmAGYAZQByAGUAbgBjAGUAIABvAGYAIAB1AG4AcwBpAGcAbgBlAGQAIABMAGkAdAB0AGwAZQAtAEUAbgBkAGkAYQBuACAAYQByAHIAYQB5AHMAIAAoAEEAIAAtACAAQgApAC4AIABBAHMAcwB1AG0AZQBzACAAQQAgAD4APQAgAEIALgBcAG4AIAAqACAAWwBsAGkAbQBiAHMAXwBhADoAIABBAHIAcgBhAHkALAAgAGwAaQBtAGIAcwBfAGIAOgAgAEEAcgByAGEAeQAsACAAawA6ACAAaQBuAHQAXQBcAG4AIAAqAC8AXABuAFUAUwB1AGIAIAA9ACAATABBAE0AQgBEAEEAKABsAGkAbQBiAHMAXwBhACwAIABsAGkAbQBiAHMAXwBiACwAIABrACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQB4AF8AcgBvAHcAcwAsACAATQBBAFgAKABSAE8AVwBTACgAbABpAG0AYgBzAF8AYQApACwAIABSAE8AVwBTACgAbABpAG0AYgBzAF8AYgApACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGEAXwBhAGwAaQBnAG4AZQBkACwAIABFAFgAUABBAE4ARAAoAGwAaQBtAGIAcwBfAGEALAAgAG0AYQB4AF8AcgBvAHcAcwAsACAAMQAsACAAMAApACwAXABuACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBiAF8AYQBsAGkAZwBuAGUAZAAsACAARQBYAFAAQQBOAEQAKABsAGkAbQBiAHMAXwBiACwAIABtAGEAeABfAHIAbwB3AHMALAAgADEALAAgADAAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAGQAaQBmAGYAZQByAGUAbgBjAGUAcwAsACAAbABpAG0AYgBzAF8AYQBfAGEAbABpAGcAbgBlAGQAIAAtACAAbABpAG0AYgBzAF8AYgBfAGEAbABpAGcAbgBlAGQALABcAG4AIAAgACAAIAAgACAAIAAgAGMAYQByAHIAaQBlAGQAXwBkAGkAZgBmAGUAcgBlAG4AYwBlAHMALAAgAEMAYQByAHIAeQAoAGQAaQBmAGYAZQByAGUAbgBjAGUAcwAsACAAawApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAaABpAGcAaABlAHMAdABfAG4AbwBuAF8AegBlAHIAbwBfAGkAbgBkAGUAeAAsACAAWABNAEEAVABDAEgAKABUAFIAVQBFACwAIABjAGEAcgByAGkAZQBkAF8AZABpAGYAZgBlAHIAZQBuAGMAZQBzACAAPAA+ACAAMAAsACAAMAAsACAALQAxACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATgBBACgAaABpAGcAaABlAHMAdABfAG4AbwBuAF8AegBlAHIAbwBfAGkAbgBkAGUAeAApACwAIAB7ADAAfQAsACAAVABBAEsARQAoAGMAYQByAHIAaQBlAGQAXwBkAGkAZgBmAGUAcgBlAG4AYwBlAHMALAAgAGgAaQBnAGgAZQBzAHQAXwBuAG8AbgBfAHoAZQByAG8AXwBpAG4AZABlAHgAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABbAEkAbgB0AGUAcgBuAGEAbABdACAAUwB1AG0AcwAgAGEAIABoAG8AcgBpAHoAbwBuAHQAYQBsACAAYQByAHIAYQB5ACAAbwBmACAAQgBpAGcASQBuAHQAIABzAHQAcgBpAG4AZwBzACAAdgBpAGEAIAAyAEQAIABtAGEAdAByAGkAeAAgAGIAcgBvAGEAZABjAGEAcwB0AGkAbgBnAC4AXABuACAAKgAgAFsAcwB0AHIAXwBuAG8AcgBtAHMAOgAgAEEAcgByAGEAeQAsACAAawA6ACAAaQBuAHQAXQBcAG4AIAAqAC8AXABuAFUATQBhAHQAcgBpAHgAUwB1AG0AIAA9ACAATABBAE0AQgBEAEEAKABzAHQAcgBfAG4AbwByAG0AcwAsACAAawAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABnAHIAaQBkACwAIABTAHAAbABpAHQAKABzAHQAcgBfAG4AbwByAG0AcwAsACAAawApACwAXABuACAAIAAgACAAIAAgACAAIAByAGEAdwBfAGwAaQBtAGIAcwAsACAAQgBZAFIATwBXACgAZwByAGkAZAAsACAAUwBVAE0AKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAEMAYQByAHIAeQAoAHIAYQB3AF8AbABpAG0AYgBzACwAIABrACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFsASQBuAHQAZQByAG4AYQBsAF0AIABSAGUAdAB1AHIAbgBzACAAcABhAGMAawBlAGQAIABhAHIAcgBhAHkAOgAgAFsAbABpAG0AYgBzADsAIABmAGkAbgBhAGwAXwBzAGkAZwBuAF0ALgAgAFIAZQBzAG8AbAB2AGUAcwAgAHMAaQBnAG4AIABsAG8AZwBpAGMAIABmAG8AcgAgAEEAZABkAC8AUwB1AGIALgBcAG4AIAAqACAAWwBsAGkAbQBiAHMAXwBhADoAIABBAHIAcgBhAHkALAAgAGwAaQBtAGIAcwBfAGIAOgAgAEEAcgByAGEAeQAsACAAcwBpAGcAbgBfAGEAOgAgAGkAbgB0ACwAIABzAGkAZwBuAF8AYgA6ACAAaQBuAHQALAAgAGsAOgAgAGkAbgB0AF0AXABuACAAKgAvAFwAbgBBAGQAZABTAHUAYgBSAG8AdQB0AGUAcgAgAD0AIABMAEEATQBCAEQAQQAoAGwAaQBtAGIAcwBfAGEALAAgAGwAaQBtAGIAcwBfAGIALAAgAHMAaQBnAG4AXwBhACwAIABzAGkAZwBuAF8AYgAsACAAawAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABpAHMAXwBhAGQAZABpAHQAaQBvAG4ALAAgAHMAaQBnAG4AXwBhACAAPQAgAHMAaQBnAG4AXwBiACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAaQBzAF8AYQBkAGQAaQB0AGkAbwBuACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFYAUwBUAEEAQwBLACgAVQBBAGQAZAAoAGwAaQBtAGIAcwBfAGEALAAgAGwAaQBtAGIAcwBfAGIALAAgAGsAKQAsACAAcwBpAGcAbgBfAGEAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABtAGEAZwBuAGkAdAB1AGQAZQBfAGMAbwBtAHAAYQByAGkAcwBvAG4ALAAgAFUAQwBvAG0AcABhAHIAZQAoAGwAaQBtAGIAcwBfAGEALAAgAGwAaQBtAGIAcwBfAGIAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABtAGEAZwBuAGkAdAB1AGQAZQBfAGMAbwBtAHAAYQByAGkAcwBvAG4AIAA9ACAAMAAsACAALwAvACAAVABvAHQAYQBsACAAYwBhAG4AYwBlAGwAbABhAHQAaQBvAG4AOgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAEEAIAAyAC0AcgBvAHcAIABhAHIAcgBhAHkAIABbADAAOwAgADAAXQAgAGkAcwAgAHIAZQB0AHUAcgBuAGUAZAAgAHQAbwAgAHMAYQB0AGkAcwBmAHkAIAB0AGgAZQAgAHAAYQBjAGsAZQBkACAAWwBsAGkAbQBiAHMAOwAgAHMAaQBnAG4AXQAgAGMAbwBuAHQAcgBhAGMAdAAuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAewAwADsAMAB9ACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgAbQBhAGcAbgBpAHQAdQBkAGUAXwBjAG8AbQBwAGEAcgBpAHMAbwBuACAAPgAgADAALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAAQQAgAGkAcwAgAGwAYQByAGcAZQByADoAIABzAGkAZwBuACAAYgBlAGwAbwBuAGcAcwAgAHQAbwAgAEEALgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAVgBTAFQAQQBDAEsAKABVAFMAdQBiACgAbABpAG0AYgBzAF8AYQAsACAAbABpAG0AYgBzAF8AYgAsACAAawApACwAIABzAGkAZwBuAF8AYQApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIABCACAAaQBzACAAbABhAHIAZwBlAHIAOgAgAHIAbwB1AHQAZQAgAEIAIABmAGkAcgBzAHQALAAgAHMAaQBnAG4AIABiAGUAbABvAG4AZwBzACAAdABvACAAQgAuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABWAFMAVABBAEMASwAoAFUAUwB1AGIAKABsAGkAbQBiAHMAXwBiACwAIABsAGkAbQBiAHMAXwBhACwAIABrACkALAAgAHMAaQBnAG4AXwBiACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABbAEkAbgB0AGUAcgBuAGEAbABdACAATQB1AGwAdABpAHAAbABpAGUAcwAgAHUAbgBzAGkAZwBuAGUAZAAgAEwAaQB0AHQAbABlAC0ARQBuAGQAaQBhAG4AIABsAGkAbQBiACAAYQByAHIAYQB5AHMAIAB2AGkAYQAgADEARAAgAEQAaQBzAGMAcgBlAHQAZQAgAEMAbwBuAHYAbwBsAHUAdABpAG8AbgAuAFwAbgAgACoAIABbAGwAaQBtAGIAcwBfAGEAOgAgAEEAcgByAGEAeQAsACAAbABpAG0AYgBzAF8AYgA6ACAAQQByAHIAYQB5ACwAIABrADoAIABpAG4AdABdAFwAbgAgACoALwBcAG4AVQBNAHUAbAAgAD0AIABMAEEATQBCAEQAQQAoAGwAaQBtAGIAcwBfAGEALAAgAGwAaQBtAGIAcwBfAGIALAAgAGsALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbgB1AG0AXwBsAGkAbQBiAHMAXwBhACwAIABSAE8AVwBTACgAbABpAG0AYgBzAF8AYQApACwAXABuACAAIAAgACAAIAAgACAAIABuAHUAbQBfAGwAaQBtAGIAcwBfAGIALAAgAFIATwBXAFMAKABsAGkAbQBiAHMAXwBiACkALABcAG4AIAAgACAAIAAgACAAIAAgAGMAbwBuAHYAbwBsAHUAdABpAG8AbgBfAGwAZQBuAGcAdABoACwAIABuAHUAbQBfAGwAaQBtAGIAcwBfAGEAIAArACAAbgB1AG0AXwBsAGkAbQBiAHMAXwBiACAALQAgADEALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABDAGEAdQBjAGgAeQAgAFAAcgBvAGQAdQBjAHQAIABhAHYAbwBpAGQAcwAgAGUAeABwAGUAbgBzAGkAdgBlACAAMgBEACAAbQBhAHQAcgBpAHgAIABnAGUAbgBlAHIAYQB0AGkAbwBuACAAYgB5ACAAYwBhAGwAYwB1AGwAYQB0AGkAbgBnACAAZQBhAGMAaAAgAGwAaQBtAGIAJwBzACAAbQBhAGcAbgBpAHQAdQBkAGUAIABpAG4AZABlAHAAZQBuAGQAZQBuAHQAbAB5AC4AXABuACAAIAAgACAAIAAgACAAIAByAGEAdwBfAGMAbwBuAHYAbwBsAHUAdABpAG8AbgAsACAATQBBAEsARQBBAFIAUgBBAFkAKABjAG8AbgB2AG8AbAB1AHQAaQBvAG4AXwBsAGUAbgBnAHQAaAAsACAAMQAsACAATABBAE0AQgBEAEEAKAByACwAIABjACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAdwBpAG4AZABvAHcAXwBzAHQAYQByAHQAXwBpACwAIABNAEEAWAAoADEALAAgAHIAIAAtACAAbgB1AG0AXwBsAGkAbQBiAHMAXwBiACAAKwAgADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHcAaQBuAGQAbwB3AF8AZQBuAGQAXwBpACwAIABNAEkATgAoAHIALAAgAG4AdQBtAF8AbABpAG0AYgBzAF8AYQApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAG8AdgBlAHIAbABhAHAAXwByAG8AdwBzACwAIAB3AGkAbgBkAG8AdwBfAGUAbgBkAF8AaQAgAC0AIAB3AGkAbgBkAG8AdwBfAHMAdABhAHIAdABfAGkAIAArACAAMQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABzAGUAcQBfAGkALAAgAFMARQBRAFUARQBOAEMARQAoAG8AdgBlAHIAbABhAHAAXwByAG8AdwBzACwAIAAxACwAIAB3AGkAbgBkAG8AdwBfAHMAdABhAHIAdABfAGkALAAgADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHMAZQBxAF8AagAsACAAUwBFAFEAVQBFAE4AQwBFACgAbwB2AGUAcgBsAGEAcABfAHIAbwB3AHMALAAgADEALAAgAHIAIAAtACAAdwBpAG4AZABvAHcAXwBzAHQAYQByAHQAXwBpACAAKwAgADEALAAgAC0AMQApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFMAVQBNACgASQBOAEQARQBYACgAbABpAG0AYgBzAF8AYQAsACAAcwBlAHEAXwBpACwAIAAxACkAIAAqACAASQBOAEQARQBYACgAbABpAG0AYgBzAF8AYgAsACAAcwBlAHEAXwBqACwAIAAxACkAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACkAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAEMAYQByAHIAeQAoAHIAYQB3AF8AYwBvAG4AdgBvAGwAdQB0AGkAbwBuACwAIABrACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFsASQBuAHQAZQByAG4AYQBsAF0AIABSAGUAdAB1AHIAbgBzACAAaABpAGcAaABlAHMAdAAgAHMAYwBhAGwAYQByACAAcQB1AG8AdABpAGUAbgB0ACAAbABpAG0AYgAgAHEAIAAoADAAIAA8AD0AIABxACAAPAAgADEAMABeAGsAKQAgAHcAaABlAHIAZQAgAEIAIAAqACAAcQAgADwAPQAgAFIALgBcAG4AIAAqACAAWwBsAGkAbQBiAHMAXwByADoAIABBAHIAcgBhAHkALAAgAGwAaQBtAGIAcwBfAGIAOgAgAEEAcgByAGEAeQAsACAAawA6ACAAaQBuAHQAXQBcAG4AIAAqAC8AXABuAEYAaQBuAGQAUQB1AG8AdABpAGUAbgB0AEwAaQBtAGIAIAA9ACAATABBAE0AQgBEAEEAKABsAGkAbQBiAHMAXwByACwAIABsAGkAbQBiAHMAXwBiACwAIABrACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAHIAZQBxAHUAaQByAGUAZABfAGIAaQB0AHMALAAgAEMARQBJAEwASQBOAEcALgBNAEEAVABIACgATABPAEcAKAAxADAAXgBrACwAIAAyACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcABvAHcAZQByAHMAXwBvAGYAXwB0AHcAbwAsACAAMgAgAF4AIABTAEUAUQBVAEUATgBDAEUAKAByAGUAcQB1AGkAcgBlAGQAXwBiAGkAdABzACwAIAAxACwAIAByAGUAcQB1AGkAcgBlAGQAXwBiAGkAdABzACAALQAgADEALAAgAC0AMQApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAUgBFAEQAVQBDAEUAKAAwACwAIABwAG8AdwBlAHIAcwBfAG8AZgBfAHQAdwBvACwAIABMAEEATQBCAEQAQQAoAGMAdQByAHIAZQBuAHQAXwBxACwAIABjAHUAcgByAGUAbgB0AF8AcABvAHcAZQByACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAdABlAHMAdABfAHEALAAgAGMAdQByAHIAZQBuAHQAXwBxACAAKwAgAGMAdQByAHIAZQBuAHQAXwBwAG8AdwBlAHIALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgAdABlAHMAdABfAHEAIAA+AD0AIAAxADAAXgBrACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABjAHUAcgByAGUAbgB0AF8AcQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYgBxACwAIABDAGEAcgByAHkAKABsAGkAbQBiAHMAXwBiACAAKgAgAHQAZQBzAHQAXwBxACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbQBhAGcAbgBpAHQAdQBkAGUAXwBjAG8AbQBwAGEAcgBpAHMAbwBuACwAIABVAEMAbwBtAHAAYQByAGUAKABsAGkAbQBiAHMAXwByACwAIABsAGkAbQBiAHMAXwBiAHEAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgAbQBhAGcAbgBpAHQAdQBkAGUAXwBjAG8AbQBwAGEAcgBpAHMAbwBuACAAPgA9ACAAMAAsACAAdABlAHMAdABfAHEALAAgAGMAdQByAHIAZQBuAHQAXwBxACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAApACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFsASQBuAHQAZQByAG4AYQBsAF0AIABSAGUAdAB1AHIAbgBzACAAcABhAGMAawBlAGQAIABhAHIAcgBhAHkAOgAgAFsATABlAG4AXwBSADsAIABSAF8AbABpAG0AYgBzADsAIABRAF8AbABpAG0AYgBzAF0AIAB1AHMAaQBuAGcAIABzAGUAcQB1AGUAbgB0AGkAYQBsACAAbABvAG4AZwAgAGQAaQB2AGkAcwBpAG8AbgAuAFwAbgAgACoAIABbAGwAaQBtAGIAcwBfAGEAOgAgAEEAcgByAGEAeQAsACAAbABpAG0AYgBzAF8AYgA6ACAAQQByAHIAYQB5ACwAIABrADoAIABpAG4AdABdAFwAbgAgACoALwBcAG4ASwBuAHUAdABoAEQAaQB2ACAAPQAgAEwAQQBNAEIARABBACgAbABpAG0AYgBzAF8AYQAsACAAbABpAG0AYgBzAF8AYgAsACAAawAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABtAGEAZwBuAGkAdAB1AGQAZQBfAGMAbwBtAHAAYQByAGkAcwBvAG4ALAAgAFUAQwBvAG0AcABhAHIAZQAoAGwAaQBtAGIAcwBfAGEALAAgAGwAaQBtAGIAcwBfAGIAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAG0AYQBnAG4AaQB0AHUAZABlAF8AYwBvAG0AcABhAHIAaQBzAG8AbgAgADwAIAAwACwAIABWAFMAVABBAEMASwAoAFIATwBXAFMAKABsAGkAbQBiAHMAXwBhACkALAAgAGwAaQBtAGIAcwBfAGEALAAgADAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAbQBhAGcAbgBpAHQAdQBkAGUAXwBjAG8AbQBwAGEAcgBpAHMAbwBuACAAPQAgADAALAAgAFYAUwBUAEEAQwBLACgAMQAsACAAMAAsACAAMQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbgB1AG0AXwBsAGkAbQBiAHMAXwBhACwAIABSAE8AVwBTACgAbABpAG0AYgBzAF8AYQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAYgBpAGcAXwBlAG4AZABpAGEAbgBfAGEALAAgAEMASABPAE8AUwBFAFIATwBXAFMAKABsAGkAbQBiAHMAXwBhACwAIABTAEUAUQBVAEUATgBDAEUAKABuAHUAbQBfAGwAaQBtAGIAcwBfAGEALAAgADEALAAgAG4AdQBtAF8AbABpAG0AYgBzAF8AYQAsACAALQAxACkAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIABTAHQAYQB0AGUAIABpAHMAIABwAGEAYwBrAGUAZAAgAGkAbgB0AG8AIABhACAAMQBEACAAdgBlAHIAdABpAGMAYQBsACAAYQByAHIAYQB5ACAAYgBlAGMAYQB1AHMAZQAgAEUAeABjAGUAbAAgAGMAYQBuACAAbwBuAGwAeQAgAHIAZQB0AHUAcgBuACAAbwBuAGUAIABvAGIAagBlAGMAdAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAHAAcgBlAGYAaQB4AGkAbgBnACAAdABoAGUAIAByAGUAbQBhAGkAbgBkAGUAcgAnAHMAIABsAGUAbgBnAHQAaAAgAGEAbABsAG8AdwBzACAAZQBmAGYAaQBjAGkAZQBuAHQAIAB1AG4AcABhAGMAawBpAG4AZwAgAG8AZgAgAGIAbwB0AGgAIABSACAAYQBuAGQAIABRACAAYwBvAG0AcABvAG4AZQBuAHQAcwAuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGYAaQBuAGEAbABfAHAAYQBjAGsAZQBkAF8AcwB0AGEAdABlACwAIABSAEUARABVAEMARQAoAFYAUwBUAEEAQwBLACgAMQAsACAAMAAsACAAMAApACwAIABiAGkAZwBfAGUAbgBkAGkAYQBuAF8AYQAsACAATABBAE0AQgBEAEEAKABwAGEAYwBrAGUAZABfAHMAdABhAHQAZQAsACAAdgBhAGwALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAG4AdQBtAF8AbABpAG0AYgBzAF8AcgAsACAASQBOAEQARQBYACgAcABhAGMAawBlAGQAXwBzAHQAYQB0AGUALAAgADEALAAgADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwByACwAIABDAEgATwBPAFMARQBSAE8AVwBTACgAcABhAGMAawBlAGQAXwBzAHQAYQB0AGUALAAgAFMARQBRAFUARQBOAEMARQAoAG4AdQBtAF8AbABpAG0AYgBzAF8AcgAsACAAMQAsACAAMgApACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AcQAsACAARABSAE8AUAAoAHAAYQBjAGsAZQBkAF8AcwB0AGEAdABlACwAIABuAHUAbQBfAGwAaQBtAGIAcwBfAHIAIAArACAAMQApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBzAGgAaQBmAHQAZQBkAF8AcgAsACAASQBGACgAQQBOAEQAKABSAE8AVwBTACgAbABpAG0AYgBzAF8AcgApACAAPQAgADEALAAgAEkATgBEAEUAWAAoAGwAaQBtAGIAcwBfAHIALAAgADEALAAgADEAKQAgAD0AIAAwACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAB2AGEAbAAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFYAUwBUAEEAQwBLACgAdgBhAGwALAAgAGwAaQBtAGIAcwBfAHIAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcQBfAGwAaQBtAGIALAAgAEYAaQBuAGQAUQB1AG8AdABpAGUAbgB0AEwAaQBtAGIAKABsAGkAbQBiAHMAXwBzAGgAaQBmAHQAZQBkAF8AcgAsACAAbABpAG0AYgBzAF8AYgAsACAAawApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGIAcQAsACAAQwBhAHIAcgB5ACgAbABpAG0AYgBzAF8AYgAgACoAIABxAF8AbABpAG0AYgAsACAAawApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAG4AZQB4AHQAXwByACwAIABVAFMAdQBiACgAbABpAG0AYgBzAF8AcwBoAGkAZgB0AGUAZABfAHIALAAgAGwAaQBtAGIAcwBfAGIAcQAsACAAawApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGgAYQBzAF8AcQAsACAATwBSACgAUgBPAFcAUwAoAGwAaQBtAGIAcwBfAHEAKQAgAD4AIAAxACwAIABJAE4ARABFAFgAKABsAGkAbQBiAHMAXwBxACwAMQAsADEAKQAgAD4AIAAwACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAG4AZQB4AHQAXwBxACwAIABJAEYAKABoAGEAcwBfAHEALAAgAFYAUwBUAEEAQwBLACgAbABpAG0AYgBzAF8AcQAsACAAcQBfAGwAaQBtAGIAKQAsACAAcQBfAGwAaQBtAGIAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAVgBTAFQAQQBDAEsAKABSAE8AVwBTACgAbABpAG0AYgBzAF8AbgBlAHgAdABfAHIAKQAsACAAbABpAG0AYgBzAF8AbgBlAHgAdABfAHIALAAgAGwAaQBtAGIAcwBfAG4AZQB4AHQAXwBxACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABuAHUAbQBfAGwAaQBtAGIAcwBfAHIALAAgAEkATgBEAEUAWAAoAGYAaQBuAGEAbABfAHAAYQBjAGsAZQBkAF8AcwB0AGEAdABlACwAIAAxACwAIAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwByACwAIABDAEgATwBPAFMARQBSAE8AVwBTACgAZgBpAG4AYQBsAF8AcABhAGMAawBlAGQAXwBzAHQAYQB0AGUALAAgAFMARQBRAFUARQBOAEMARQAoAG4AdQBtAF8AbABpAG0AYgBzAF8AcgAsACAAMQAsACAAMgApACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABiAGkAZwBfAGUAbgBkAGkAYQBuAF8AcQAsACAARABSAE8AUAAoAGYAaQBuAGEAbABfAHAAYQBjAGsAZQBkAF8AcwB0AGEAdABlACwAIABuAHUAbQBfAGwAaQBtAGIAcwBfAHIAIAArACAAMQApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAZQBuAF8AcQAsACAAUgBPAFcAUwAoAGIAaQBnAF8AZQBuAGQAaQBhAG4AXwBxACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBxACwAIABDAEgATwBPAFMARQBSAE8AVwBTACgAYgBpAGcAXwBlAG4AZABpAGEAbgBfAHEALAAgAFMARQBRAFUARQBOAEMARQAoAGwAZQBuAF8AcQAsACAAMQAsACAAbABlAG4AXwBxACwAIAAtADEAKQApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFYAUwBUAEEAQwBLACgAbgB1AG0AXwBsAGkAbQBiAHMAXwByACwAIABsAGkAbQBiAHMAXwByACwAIABsAGkAbQBiAHMAXwBxACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAApACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFsASQBuAHQAZQByAG4AYQBsAF0AIABSAG8AdQB0AGUAcwAgAGQAaQB2AGkAcwBpAG8AbgAgAHQAbwAgAEsAbgB1AHQAaAAgAG8AcgAgAE4AZQB3AHQAbwBuAC0AUgBhAHAAaABzAG8AbgAgAGIAYQBzAGUAZAAgAG8AbgAgAEQAaQB2AGkAZABlAG4AZAAgAGwAZQBuAGcAdABoAC4AXABuACAAKgAgAFsAbABpAG0AYgBzAF8AYQA6ACAAQQByAHIAYQB5ACwAIABsAGkAbQBiAHMAXwBiADoAIABBAHIAcgBhAHkALAAgAGsAOgAgAGkAbgB0AF0AXABuACAAKgAvAFwAbgBEAGkAdgBSAG8AdQB0AGUAcgAgAD0AIABMAEEATQBCAEQAQQAoAGwAaQBtAGIAcwBfAGEALAAgAGwAaQBtAGIAcwBfAGIALAAgAGsALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAYQBwAHAAcgBvAHgAXwBkAGkAZwBpAHQAcwBfAGEALAAgAFIATwBXAFMAKABsAGkAbQBiAHMAXwBhACkAIAAqACAAawAsAFwAbgAgACAAIAAgACAAIAAgACAAYQBwAHAAcgBvAHgAXwBkAGkAZwBpAHQAcwBfAGIALAAgAFIATwBXAFMAKABsAGkAbQBiAHMAXwBiACkAIAAqACAAawAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAC8ALwAgAEwAbwBnAGkAcwB0AGkAYwAgAFIAZQBnAHIAZQBzAHMAaQBvAG4AIABjAG8AZQBmAGYAaQBjAGkAZQBuAHQAcwAgAGQAZQB0AGUAcgBtAGkAbgBlACAAdABoAGUAIABjAHIAbwBzAHMAbwB2AGUAcgAgAHcAaABlAHIAZQAgAHMAZQBxAHUAZQBuAHQAaQBhAGwAIAByAGUAYQBsAGwAbwBjAGEAdABpAG8AbgAgAGsAaQBsAGwAcwAgAHAAZQByAGYAbwByAG0AYQBuAGMAZQAuAFwAbgAgACAAIAAgACAAIAAgACAAcgBlAGcAcgBlAHMAcwBpAG8AbgBfAHMAbABvAHAAZQBfAG0ALAAgADAALgAxADAANwA4ADIAMQAxADkANAAyADcAMQAyADkANwAsAFwAbgAgACAAIAAgACAAIAAgACAAcgBlAGcAcgBlAHMAcwBpAG8AbgBfAGkAbgB0AGUAcgBjAGUAcAB0AF8AYwAsACAALQAyADIAMQAuADkAMAAyADEAOAA5ADQANgAyADAANgA4ACwAXABuACAAIAAgACAAIAAgACAAIAB0AGgAcgBlAHMAaABvAGwAZABfAGQAaQBnAGkAdABzACwAIAAoAHIAZQBnAHIAZQBzAHMAaQBvAG4AXwBzAGwAbwBwAGUAXwBtACAAKgAgAGEAcABwAHIAbwB4AF8AZABpAGcAaQB0AHMAXwBhACkAIAArACAAcgBlAGcAcgBlAHMAcwBpAG8AbgBfAGkAbgB0AGUAcgBjAGUAcAB0AF8AYwAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAGEAcABwAHIAbwB4AF8AZABpAGcAaQB0AHMAXwBiACAAPAA9ACAAdABoAHIAZQBzAGgAbwBsAGQAXwBkAGkAZwBpAHQAcwAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABLAG4AdQB0AGgARABpAHYAKABsAGkAbQBiAHMAXwBhACwAIABsAGkAbQBiAHMAXwBiACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATgBlAHcAdABvAG4AUgBhAHAAaABzAG8AbgBEAGkAdgAoAGwAaQBtAGIAcwBfAGEALAAgAGwAaQBtAGIAcwBfAGIALAAgAGsAKQBcAG4AIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFsASQBuAHQAZQByAG4AYQBsAF0AIABSAGUAdAB1AHIAbgBzACAAdABoAGUAIAByAGUAYwBpAHAAcgBvAGMAYQBsACAAcwBlAGUAZAAgAGYAbABvAG8AcgAoAEIAZQB0AGEAXgAoADIAKgBsAGUAbgApACAALwAgAEIAXwB0AG8AcAApACAAdgBpAGEAIABLAG4AdQB0AGgAIABCAGEAcwBlAGMAYQBzAGUALgBcAG4AIAAqACAAWwBsAGkAbQBiAHMAXwBiADoAIABBAHIAcgBhAHkALAAgAGsAOgAgAGkAbgB0AF0AXABuACAAKgAvAFwAbgBOAGUAdwB0AG8AbgBSAGEAcABoAHMAbwBuAFMAZQBlAGQAIAA9ACAATABBAE0AQgBEAEEAKABsAGkAbQBiAHMAXwBiACwAIABrACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG4AdQBtAF8AbABpAG0AYgBzAF8AYgAsACAAUgBPAFcAUwAoAGwAaQBtAGIAcwBfAGIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbgB1AG0AXwBzAGUAZQBkAF8AbABpAG0AYgBzACwAIABNAEkATgAoADMALAAgAG4AdQBtAF8AbABpAG0AYgBzAF8AYgApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAALwAvACAARQB4AHQAcgBhAGMAdAAgAHQAbwBwACAAbABpAG0AYgBzACAAKABMAGkAdAB0AGwAZQAtAEUAbgBkAGkAYQBuADoAIAB0AGEAawBlACAAZgByAG8AbQAgAHQAaABlACAAYgBvAHQAdABvAG0AKQBcAG4AIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGIAXwB0AG8AcAAsACAAVABBAEsARQAoAGwAaQBtAGIAcwBfAGIALAAgAC0AbgB1AG0AXwBzAGUAZQBkAF8AbABpAG0AYgBzACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABDAG8AbgBzAHQAcgB1AGMAdAAgAEIAZQB0AGEAXgAoADIAIAAqACAAcwBlAGUAZABfAGwAZQBuACkAIABuAGEAdABpAHYAZQBsAHkAXABuACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBiAGUAdABhAF8AMgBtACwAIABWAFMAVABBAEMASwAoAEUAWABQAEEATgBEACgAMAAsACAAMgAgACoAIABuAHUAbQBfAHMAZQBlAGQAXwBsAGkAbQBiAHMALAAgACwAIAAwACkALAAgADEAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAC8ALwAgAEsAbgB1AHQAaAAgAEQAaQB2AGkAcwBpAG8AbgAgAHkAaQBlAGwAZABzACAAZQB4AGEAYwB0ACAAaQBuAGkAdABpAGEAbAAgAHIAZQBjAGkAcAByAG8AYwBhAGwAXABuACAAIAAgACAAIAAgACAAIABwAGEAYwBrAGUAZABfAGIAYQBzAGUAYwBhAHMAZQBfAHIAZQBzAHUAbAB0ACwAIABLAG4AdQB0AGgARABpAHYAKABsAGkAbQBiAHMAXwBiAGUAdABhAF8AMgBtACwAIABsAGkAbQBiAHMAXwBiAF8AdABvAHAALAAgAGsAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAC8ALwAgAEUAeAB0AHIAYQBjAHQAIABRAHUAbwB0AGkAZQBuAHQAIABhAHIAcgBhAHkAIABmAHIAbwBtACAAdABoAGUAIABwAGEAYwBrAGUAZAAgAFYAUwBUAEEAQwBLAFwAbgAgACAAIAAgACAAIAAgACAAbgB1AG0AXwBsAGkAbQBiAHMAXwByACwAIABJAE4ARABFAFgAKABwAGEAYwBrAGUAZABfAGIAYQBzAGUAYwBhAHMAZQBfAHIAZQBzAHUAbAB0ACwAIAAxACwAIAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAEQAUgBPAFAAKABwAGEAYwBrAGUAZABfAGIAYQBzAGUAYwBhAHMAZQBfAHIAZQBzAHUAbAB0ACwAIABuAHUAbQBfAGwAaQBtAGIAcwBfAHIAIAArACAAMQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABbAEkAbgB0AGUAcgBuAGEAbABdACAAUgBlAHQAdQByAG4AcwAgAHQAaABlACAAUgBlAGMAaQBwAHIAbwBjAGEAbAAgAFIAIABzAGMAYQBsAGUAZAAgAHAAcgBvAGcAcgBlAHMAcwBpAHYAZQBsAHkAIAB0AG8AIAB0AGgAZQAgAEQAaQB2AGkAZABlAG4AZAAnAHMAIABwAHIAZQBjAGkAcwBpAG8AbgAuAFwAbgAgACoAIABbAGwAaQBtAGIAcwBfAGIAOgAgAEEAcgByAGEAeQAsACAAdABhAHIAZwBlAHQAXwBsAGUAbgA6ACAAaQBuAHQALAAgAGsAOgAgAGkAbgB0AF0AXABuACAAKgAvAFwAbgBOAGUAdwB0AG8AbgBSAGEAcABoAHMAbwBuAFIAZQBjAGkAcAByAG8AYwBhAGwAIAA9ACAATABBAE0AQgBEAEEAKABsAGkAbQBiAHMAXwBiACwAIAB0AGEAcgBnAGUAdABfAGwAZQBuACwAIABrACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG4AdQBtAF8AbABpAG0AYgBzAF8AYgAsACAAUgBPAFcAUwAoAGwAaQBtAGIAcwBfAGIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbgB1AG0AXwBzAGUAZQBkAF8AbABpAG0AYgBzACwAIABNAEkATgAoADMALAAgAG4AdQBtAF8AbABpAG0AYgBzAF8AYgApACwAXABuACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwByAF8AcwBlAGUAZAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4ATgBlAHcAdABvAG4AUgBhAHAAaABzAG8AbgBTAGUAZQBkACgAbABpAG0AYgBzAF8AYgAsACAAawApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAcgBlAHEAdQBpAHIAZQBkAF8AaQB0AGUAcgBhAHQAaQBvAG4AcwAsACAATQBBAFgAKAAwACwAIABDAEUASQBMAEkATgBHAC4ATQBBAFQASAAoAEwATgAoAHQAYQByAGcAZQB0AF8AbABlAG4AIAAvACAAbgB1AG0AXwBzAGUAZQBkAF8AbABpAG0AYgBzACkAIAAvACAATABOACgAMgApACkAKQAgACsAIAAxACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAcgBlAHEAdQBpAHIAZQBkAF8AaQB0AGUAcgBhAHQAaQBvAG4AcwAgAD0AIAAwACwAIABsAGkAbQBiAHMAXwByAF8AcwBlAGUAZAAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGkAdABlAHIAYQB0AGkAbwBuAHMALAAgAFMARQBRAFUARQBOAEMARQAoAHIAZQBxAHUAaQByAGUAZABfAGkAdABlAHIAYQB0AGkAbwBuAHMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAFAAYQBjAGsAaQBuAGcAIABbAEwAZQBuAF8AUgA7ACAAUgBfAGwAaQBtAGIAcwBdACAAaQBuAHQAbwAgAGEAIAAxAEQAIAB2AGUAcgB0AGkAYwBhAGwAIABhAHIAcgBhAHkAIABhAGwAbABvAHcAcwAgAHIAZQB0AHUAcgBuAGkAbgBnACAAbQB1AGwAdABpAHAAbABlACAAYwBvAG0AcABvAG4AZQBuAHQAcwAgAHcAaQB0AGgAaQBuACAAUgBFAEQAVQBDAEUALgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABmAGkAbgBhAGwAXwBwAGEAYwBrAGUAZABfAHMAdABhAHQAZQAsACAAUgBFAEQAVQBDAEUAKABWAFMAVABBAEMASwAoAG4AdQBtAF8AcwBlAGUAZABfAGwAaQBtAGIAcwAsACAAbABpAG0AYgBzAF8AcgBfAHMAZQBlAGQAKQAsACAAaQB0AGUAcgBhAHQAaQBvAG4AcwAsACAATABBAE0AQgBEAEEAKABwAGEAYwBrAGUAZABfAHMAdABhAHQAZQAsACAAaQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAYwB1AHIAcgBlAG4AdABfAGwAZQBuACwAIABJAE4ARABFAFgAKABwAGEAYwBrAGUAZABfAHMAdABhAHQAZQAsACAAMQAsACAAMQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGMAdQByAHIAZQBuAHQAXwByACwAIABEAFIATwBQACgAcABhAGMAawBlAGQAXwBzAHQAYQB0AGUALAAgADEAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbgBlAHgAdABfAGwAZQBuACwAIABNAEkATgAoAGMAdQByAHIAZQBuAHQAXwBsAGUAbgAgACoAIAAyACwAIAB0AGEAcgBnAGUAdABfAGwAZQBuACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAEkAZgAgAEIAIABoAGEAcwAgAHAAbABhAHQAZQBhAHUAZQBkACwAIABSACAAbQB1AHMAdAAgAHMAYwBhAGwAZQAgAGIAeQAgADIAKgAoAG4ALQBtACkALgAgAEkAZgAgAEIAIABpAHMAIABnAHIAbwB3AGkAbgBnACwAIABSACAAcwBjAGEAbABlAHMAIABiAHkAIAAoAG4ALQBtACkALgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAYQBjAHQAaQB2AGUAXwBiAF8AbABpAG0AYgBzAF8AYwB1AHIAcgBlAG4AdAAsACAATQBJAE4AKABjAHUAcgByAGUAbgB0AF8AbABlAG4ALAAgAG4AdQBtAF8AbABpAG0AYgBzAF8AYgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGEAYwB0AGkAdgBlAF8AYgBfAGwAaQBtAGIAcwBfAG4AZQB4AHQALAAgAE0ASQBOACgAbgBlAHgAdABfAGwAZQBuACwAIABuAHUAbQBfAGwAaQBtAGIAcwBfAGIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAByAGUAcQB1AGkAcgBlAGQAXwBzAGgAaQBmAHQAXwBsAGkAbQBiAHMALAAgADIAIAAqACAAKABuAGUAeAB0AF8AbABlAG4AIAAtACAAYwB1AHIAcgBlAG4AdABfAGwAZQBuACkAIAAtACAAKABhAGMAdABpAHYAZQBfAGIAXwBsAGkAbQBiAHMAXwBuAGUAeAB0ACAALQAgAGEAYwB0AGkAdgBlAF8AYgBfAGwAaQBtAGIAcwBfAGMAdQByAHIAZQBuAHQAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AcgBfAHAAcgBpAG0AZQAsACAASQBGACgAcgBlAHEAdQBpAHIAZQBkAF8AcwBoAGkAZgB0AF8AbABpAG0AYgBzACAAPgAgADAALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABWAFMAVABBAEMASwAoAEUAWABQAEEATgBEACgAMAAsACAAcgBlAHEAdQBpAHIAZQBkAF8AcwBoAGkAZgB0AF8AbABpAG0AYgBzACwAIAAsACAAMAApACwAIABsAGkAbQBiAHMAXwBjAHUAcgByAGUAbgB0AF8AcgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYwB1AHIAcgBlAG4AdABfAHIAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGIAXwBhAGMAdABpAHYAZQAsACAAVABBAEsARQAoAGwAaQBtAGIAcwBfAGIALAAgAC0AYQBjAHQAaQB2AGUAXwBiAF8AbABpAG0AYgBzAF8AbgBlAHgAdAApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIABQACAAaQBzACAAbgBhAHQAaQB2AGUAbAB5ACAAYQBsAGkAZwBuAGUAZAAgAHQAbwAgADIAKgBuAGUAeAB0AF8AbABlAG4AIABiAGUAYwBhAHUAcwBlACAAbwBmACAAdABoAGUAIABjAG8AcgByAGUAYwB0AGUAZAAgAHMAaABpAGYAdABfAGwAaQBtAGIAcwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AcAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBNAHUAbAAoAGwAaQBtAGIAcwBfAGIAXwBhAGMAdABpAHYAZQAsACAAbABpAG0AYgBzAF8AcgBfAHAAcgBpAG0AZQAsACAAawApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwB0AHcAbwBfAGIAZQB0AGEALAAgAFYAUwBUAEEAQwBLACgARQBYAFAAQQBOAEQAKAAwACwAIAAyACAAKgAgAG4AZQB4AHQAXwBsAGUAbgAsACAALAAgADAAKQAsACAAMgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGUAcgByAG8AcgBfAHQAZQByAG0ALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFUAUwB1AGIAKABsAGkAbQBiAHMAXwB0AHcAbwBfAGIAZQB0AGEALAAgAGwAaQBtAGIAcwBfAHAALAAgAGsAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AbgBlAHgAdABfAHIAXwB1AG4AcwBjAGEAbABlAGQALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFUATQB1AGwAKABsAGkAbQBiAHMAXwByAF8AcAByAGkAbQBlACwAIABsAGkAbQBiAHMAXwBlAHIAcgBvAHIAXwB0AGUAcgBtACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AbgBlAHgAdABfAHIALAAgAEkARgAoAFIATwBXAFMAKABsAGkAbQBiAHMAXwBuAGUAeAB0AF8AcgBfAHUAbgBzAGMAYQBsAGUAZAApACAAPAA9ACAAMgAgACoAIABuAGUAeAB0AF8AbABlAG4ALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAB7ADAAfQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEQAUgBPAFAAKABsAGkAbQBiAHMAXwBuAGUAeAB0AF8AcgBfAHUAbgBzAGMAYQBsAGUAZAAsACAAMgAgACoAIABuAGUAeAB0AF8AbABlAG4AKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAVgBTAFQAQQBDAEsAKABuAGUAeAB0AF8AbABlAG4ALAAgAGwAaQBtAGIAcwBfAG4AZQB4AHQAXwByACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEQAUgBPAFAAKABmAGkAbgBhAGwAXwBwAGEAYwBrAGUAZABfAHMAdABhAHQAZQAsACAAMQApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAAWwBJAG4AdABlAHIAbgBhAGwAXQAgAFIAZQB0AHUAcgBuAHMAIABwAGEAYwBrAGUAZAAgAGEAcgByAGEAeQA6ACAAWwBMAGUAbgBfAFIAOwAgAFIAXwBsAGkAbQBiAHMAOwAgAFEAXwBsAGkAbQBiAHMAXQAgAHUAcwBpAG4AZwAgAE4AZQB3AHQAbwBuAC0AUgBhAHAAaABzAG8AbgAuAFwAbgAgACoAIABbAGwAaQBtAGIAcwBfAGEAOgAgAEEAcgByAGEAeQAsACAAbABpAG0AYgBzAF8AYgA6ACAAQQByAHIAYQB5ACwAIABrADoAIABpAG4AdABdAFwAbgAgACoALwBcAG4ATgBlAHcAdABvAG4AUgBhAHAAaABzAG8AbgBEAGkAdgAgAD0AIABMAEEATQBCAEQAQQAoAGwAaQBtAGIAcwBfAGEALAAgAGwAaQBtAGIAcwBfAGIALAAgAGsALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbgB1AG0AXwBsAGkAbQBiAHMAXwBhACwAIABSAE8AVwBTACgAbABpAG0AYgBzAF8AYQApACwAXABuACAAIAAgACAAIAAgACAAIABuAHUAbQBfAGwAaQBtAGIAcwBfAGIALAAgAFIATwBXAFMAKABsAGkAbQBiAHMAXwBiACkALABcAG4AIAAgACAAIAAgACAAIAAgAG4AdQBtAF8AbABpAG0AYgBzAF8AdABhAHIAZwBlAHQALAAgAE0AQQBYACgAbgB1AG0AXwBsAGkAbQBiAHMAXwBhACwAIABuAHUAbQBfAGwAaQBtAGIAcwBfAGIAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAC8ALwAgADEALgAgAEMAYQBsAGMAdQBsAGEAdABlACAAcgBlAGMAaQBwAHIAbwBjAGEAbAAgAFIAIABzAGMAYQBsAGUAZAAgAGQAeQBuAGEAbQBpAGMAYQBsAGwAeQAgAHQAbwAgADIAIAAqACAAdABhAHIAZwBlAHQAXwBsAGUAbgBcAG4AIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAHIAZQBjAGkAcAByAG8AYwBhAGwALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAE4AZQB3AHQAbwBuAFIAYQBwAGgAcwBvAG4AUgBlAGMAaQBwAHIAbwBjAGEAbAAoAGwAaQBtAGIAcwBfAGIALAAgAG4AdQBtAF8AbABpAG0AYgBzAF8AdABhAHIAZwBlAHQALAAgAGsAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAC8ALwAgADIALgAgAEEAcABwAHIAbwB4AGkAbQBhAHQAZQAgAFEAdQBvAHQAaQBlAG4AdAA6ACAAUQBfAGEAcABwAHIAbwB4ACAAPQAgAEEAIAAqACAAUgAgAC8AIABCAGUAdABhAF4AKAAyACAAKgAgAHQAYQByAGcAZQB0AF8AbABlAG4AKQBcAG4AIAAgACAAIAAgACAAIAAgAHIAaQBnAGgAdABfAHMAaABpAGYAdABfAGwAaQBtAGIAcwAsACAAMgAgACoAIABuAHUAbQBfAGwAaQBtAGIAcwBfAHQAYQByAGcAZQB0ACwAXABuACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBxAF8AdQBuAHMAYwBhAGwAZQBkACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAE0AdQBsACgAbABpAG0AYgBzAF8AYQAsACAAbABpAG0AYgBzAF8AcgBlAGMAaQBwAHIAbwBjAGEAbAAsACAAawApACwAXABuACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBxAF8AYQBwAHAAcgBvAHgALAAgAEkARgAoAFIATwBXAFMAKABsAGkAbQBiAHMAXwBxAF8AdQBuAHMAYwBhAGwAZQBkACkAIAA8AD0AIAByAGkAZwBoAHQAXwBzAGgAaQBmAHQAXwBsAGkAbQBiAHMALAAgAHsAMAB9ACwAIABEAFIATwBQACgAbABpAG0AYgBzAF8AcQBfAHUAbgBzAGMAYQBsAGUAZAAsACAAcgBpAGcAaAB0AF8AcwBoAGkAZgB0AF8AbABpAG0AYgBzACkAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAC8ALwAgAEMAYQBsAGMAdQBsAGEAdABlACAAdABoAGUAIABtAGEAcwBzAGkAdgBlACAAYgBhAHMAZQBsAGkAbgBlACAAcAByAG8AZAB1AGMAdAAgAGUAeABhAGMAdABsAHkAIABPAE4AQwBFACAAdABvACAAcAByAGUAdgBlAG4AdAAgAHIAZQBkAHUAbgBkAGEAbgB0ACAAVQBNAHUAbAAgAGMAYQBsAGwAcwAuAFwAbgAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AcABfAGIAYQBzAGUAbABpAG4AZQAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBNAHUAbAAoAGwAaQBtAGIAcwBfAGIALAAgAGwAaQBtAGIAcwBfAHEAXwBhAHAAcAByAG8AeAAsACAAawApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAALwAvACAAMwAuACAAQgBvAHUAbgBkAGUAZAAgAEUAcgByAG8AcgAgAEMAbwByAHIAZQBjAHQAaQBvAG4AIABTAHcAZQBlAHAAIAAoAE8AcAB0AGkAbQBpAHoAZQBkACAATwAoAE4AKQAgAFMAdABlAHAAcABpAG4AZwApAFwAbgAgACAAIAAgACAAIAAgACAALwAvACAAUwB0AGEAdABlACAAaQBzACAAcABhAGMAawBlAGQAIABpAG4AdABvACAAYQAgADEARAAgAHYAZQByAHQAaQBjAGEAbAAgAGEAcgByAGEAeQAgAGIAZQBjAGEAdQBzAGUAIABFAHgAYwBlAGwAIABjAGEAbgAgAG8AbgBsAHkAIAByAGUAdAB1AHIAbgAgAG8AbgBlACAAbwBiAGoAZQBjAHQAOwBcAG4AIAAgACAAIAAgACAAIAAgAC8ALwAgAHAAcgBlAGYAaQB4AGkAbgBnACAAdABoAGUAIAByAGUAbQBhAGkAbgBkAGUAcgAnAHMAIABsAGUAbgBnAHQAaAAgAGEAbABsAG8AdwBzACAAZQBmAGYAaQBjAGkAZQBuAHQAIAB1AG4AcABhAGMAawBpAG4AZwAgAG8AZgAgAGIAbwB0AGgAIABSACAAYQBuAGQAIABRACAAYwBvAG0AcABvAG4AZQBuAHQAcwAuAFwAbgAgACAAIAAgACAAIAAgACAAaQBuAGkAdABpAGEAbABfAHAAYQBjAGsAZQBkAF8AcwB0AGEAdABlACwAIABWAFMAVABBAEMASwAoAFIATwBXAFMAKABsAGkAbQBiAHMAXwBxAF8AYQBwAHAAcgBvAHgAKQAsACAAbABpAG0AYgBzAF8AcQBfAGEAcABwAHIAbwB4ACwAIABsAGkAbQBiAHMAXwBwAF8AYgBhAHMAZQBsAGkAbgBlACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABTAHcAZQBlAHAAIABEAG8AdwBuADoAIABJAGYAIABQACAAPgAgAEEALAAgAFEAIABpAHMAIAB0AG8AbwAgAGIAaQBnAC4AIABTAHQAZQBwACAAUQAgAGQAbwB3AG4AIABiAHkAIAAxACwAIABhAG4AZAAgAFAAIABkAG8AdwBuACAAYgB5ACAAQgAuAFwAbgAgACAAIAAgACAAIAAgACAAcABhAGMAawBlAGQAXwBzAHQAYQB0AGUAXwBzAHcAZQBwAHQAXwBkAG8AdwBuACwAIABSAEUARABVAEMARQAoAGkAbgBpAHQAaQBhAGwAXwBwAGEAYwBrAGUAZABfAHMAdABhAHQAZQAsACAAewAxADsAIAAyAH0ALAAgAEwAQQBNAEIARABBACgAcABhAGMAawBlAGQAXwBzAHQAYQB0AGUALAAgAGkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGUAbgBfAHEALAAgAEkATgBEAEUAWAAoAHAAYQBjAGsAZQBkAF8AcwB0AGEAdABlACwAIAAxACwAIAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBjAHUAcgByAGUAbgB0AF8AcQAsACAAQwBIAE8ATwBTAEUAUgBPAFcAUwAoAHAAYQBjAGsAZQBkAF8AcwB0AGEAdABlACwAIABTAEUAUQBVAEUATgBDAEUAKABsAGUAbgBfAHEALAAgADEALAAgADIAKQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYwB1AHIAcgBlAG4AdABfAHAALAAgAEQAUgBPAFAAKABwAGEAYwBrAGUAZABfAHMAdABhAHQAZQAsACAAbABlAG4AXwBxACAAKwAgADEAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAEMAbwBtAHAAYQByAGUAKABsAGkAbQBiAHMAXwBjAHUAcgByAGUAbgB0AF8AcAAsACAAbABpAG0AYgBzAF8AYQApACAAPAA9ACAAMAAsACAAcABhAGMAawBlAGQAXwBzAHQAYQB0AGUALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAG4AZQB4AHQAXwBxACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAFMAdQBiACgAbABpAG0AYgBzAF8AYwB1AHIAcgBlAG4AdABfAHEALAAgAHsAMQB9ACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AbgBlAHgAdABfAHAALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFUAUwB1AGIAKABsAGkAbQBiAHMAXwBjAHUAcgByAGUAbgB0AF8AcAAsACAAbABpAG0AYgBzAF8AYgAsACAAawApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFYAUwBUAEEAQwBLACgAUgBPAFcAUwAoAGwAaQBtAGIAcwBfAG4AZQB4AHQAXwBxACkALAAgAGwAaQBtAGIAcwBfAG4AZQB4AHQAXwBxACwAIABsAGkAbQBiAHMAXwBuAGUAeAB0AF8AcAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAKQApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAALwAvACAAUwB3AGUAZQBwACAAVQBwADoAIABJAGYAIABQACAAKwAgAEIAIAA8AD0AIABBACwAIABRACAAaQBzACAAdABvAG8AIABzAG0AYQBsAGwALgAgAFMAdABlAHAAIABRACAAdQBwACAAYgB5ACAAMQAsACAAYQBuAGQAIABQACAAdQBwACAAYgB5ACAAQgAuAFwAbgAgACAAIAAgACAAIAAgACAAcABhAGMAawBlAGQAXwBzAHQAYQB0AGUAXwBzAHcAZQBwAHQAXwB1AHAALAAgAFIARQBEAFUAQwBFACgAcABhAGMAawBlAGQAXwBzAHQAYQB0AGUAXwBzAHcAZQBwAHQAXwBkAG8AdwBuACwAIAB7ADEAOwAgADIAfQAsACAATABBAE0AQgBEAEEAKABwAGEAYwBrAGUAZABfAHMAdABhAHQAZQAsACAAaQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAZQBuAF8AcQAsACAASQBOAEQARQBYACgAcABhAGMAawBlAGQAXwBzAHQAYQB0AGUALAAgADEALAAgADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGMAdQByAHIAZQBuAHQAXwBxACwAIABDAEgATwBPAFMARQBSAE8AVwBTACgAcABhAGMAawBlAGQAXwBzAHQAYQB0AGUALAAgAFMARQBRAFUARQBOAEMARQAoAGwAZQBuAF8AcQAsACAAMQAsACAAMgApACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBjAHUAcgByAGUAbgB0AF8AcAAsACAARABSAE8AUAAoAHAAYQBjAGsAZQBkAF8AcwB0AGEAdABlACwAIABsAGUAbgBfAHEAIAArACAAMQApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAG4AZQB4AHQAXwBwAF8AdABlAHMAdAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBBAGQAZAAoAGwAaQBtAGIAcwBfAGMAdQByAHIAZQBuAHQAXwBwACwAIABsAGkAbQBiAHMAXwBiACwAIABrACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBDAG8AbQBwAGEAcgBlACgAbABpAG0AYgBzAF8AbgBlAHgAdABfAHAAXwB0AGUAcwB0ACwAIABsAGkAbQBiAHMAXwBhACkAIAA+ACAAMAAsACAAcABhAGMAawBlAGQAXwBzAHQAYQB0AGUALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAG4AZQB4AHQAXwBxACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAEEAZABkACgAbABpAG0AYgBzAF8AYwB1AHIAcgBlAG4AdABfAHEALAAgAHsAMQB9ACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAVgBTAFQAQQBDAEsAKABSAE8AVwBTACgAbABpAG0AYgBzAF8AbgBlAHgAdABfAHEAKQAsACAAbABpAG0AYgBzAF8AbgBlAHgAdABfAHEALAAgAGwAaQBtAGIAcwBfAG4AZQB4AHQAXwBwAF8AdABlAHMAdAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAKQApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAALwAvACAARQB4AHQAcgBhAGMAdAAgAEYAaQBuAGEAbAAgAFEAIABhAG4AZAAgAFAAXABuACAAIAAgACAAIAAgACAAIABsAGUAbgBfAHEALAAgAEkATgBEAEUAWAAoAHAAYQBjAGsAZQBkAF8AcwB0AGEAdABlAF8AcwB3AGUAcAB0AF8AdQBwACwAIAAxACwAIAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAHEALAAgAEMASABPAE8AUwBFAFIATwBXAFMAKABwAGEAYwBrAGUAZABfAHMAdABhAHQAZQBfAHMAdwBlAHAAdABfAHUAcAAsACAAUwBFAFEAVQBFAE4AQwBFACgAbABlAG4AXwBxACwAIAAxACwAIAAyACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AcAAsACAARABSAE8AUAAoAHAAYQBjAGsAZQBkAF8AcwB0AGEAdABlAF8AcwB3AGUAcAB0AF8AdQBwACwAIABsAGUAbgBfAHEAIAArACAAMQApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAALwAvACAANAAuACAARQB4AHQAcgBhAGMAdAAgAFQAcgB1AGUAIABSAGUAbQBhAGkAbgBkAGUAcgAgAFMAYQBmAGUAbAB5ACAAKABBACAALQAgAEYAaQBuAGEAbABfAFAAKQBcAG4AIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAHIALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFUAUwB1AGIAKABsAGkAbQBiAHMAXwBhACwAIABsAGkAbQBiAHMAXwBwACwAIABrACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIABWAFMAVABBAEMASwAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAE8AVwBTACgAbABpAG0AYgBzAF8AcgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAHIALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AcQBcAG4AIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFsASQBuAHQAZQByAG4AYQBsAF0AIABSAGUAdAB1AHIAbgBzACAAYgBhAHMAZQBeAGUAeABwAG8AbgBlAG4AdAAgAHUAcwBpAG4AZwAgAEwAZQBmAHQALQB0AG8ALQBSAGkAZwBoAHQAIABlAHYAYQBsAHUAYQB0AGkAbwBuACAAYQBuAGQAIABhACAAMQAtADkAIABwAG8AdwBlAHIAIABjAGEAYwBoAGUALgBcAG4AIAAqACAAWwBsAGkAbQBiAHMAXwBiAGEAcwBlADoAIABBAHIAcgBhAHkALAAgAGUAeABwAG8AbgBlAG4AdABfAHMAdAByAGkAbgBnADoAIABUAGUAeAB0ACwAIABrADoAIABpAG4AdABdAFwAbgAgACoALwBcAG4AVQBQAG8AdwAgAD0AIABMAEEATQBCAEQAQQAoAGwAaQBtAGIAcwBfAGIAYQBzAGUALAAgAGUAeABwAG8AbgBlAG4AdABfAHMAdAByAGkAbgBnACwAIABrACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAC8ALwAgAFAAcgBlAC0AYwBvAG0AcAB1AHQAZQAgAHAAbwB3AGUAcgBzACAAMQAgAHQAaAByAG8AdQBnAGgAIAA5ACAAdABvACAAbQBpAG4AaQBtAGkAegBlACAAbQB1AGwAdABpAHAAbABpAGMAYQB0AGkAbwBuAHMAIABpAG4AcwBpAGQAZQAgAHQAaABlACAAbQBhAGkAbgAgAGQAaQBnAGkAdAAgAGwAbwBvAHAALgBcAG4AIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGIAYQBzAGUAMQAsACAAbABpAG0AYgBzAF8AYgBhAHMAZQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYgBhAHMAZQAyACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAE0AdQBsACgAbABpAG0AYgBzAF8AYgBhAHMAZQAxACwAIABsAGkAbQBiAHMAXwBiAGEAcwBlADEALAAgAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYgBhAHMAZQAzACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAE0AdQBsACgAbABpAG0AYgBzAF8AYgBhAHMAZQAyACwAIABsAGkAbQBiAHMAXwBiAGEAcwBlADEALAAgAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYgBhAHMAZQA0ACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAE0AdQBsACgAbABpAG0AYgBzAF8AYgBhAHMAZQAyACwAIABsAGkAbQBiAHMAXwBiAGEAcwBlADIALAAgAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYgBhAHMAZQA1ACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAE0AdQBsACgAbABpAG0AYgBzAF8AYgBhAHMAZQA0ACwAIABsAGkAbQBiAHMAXwBiAGEAcwBlADEALAAgAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYgBhAHMAZQA2ACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAE0AdQBsACgAbABpAG0AYgBzAF8AYgBhAHMAZQAzACwAIABsAGkAbQBiAHMAXwBiAGEAcwBlADMALAAgAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYgBhAHMAZQA3ACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAE0AdQBsACgAbABpAG0AYgBzAF8AYgBhAHMAZQA2ACwAIABsAGkAbQBiAHMAXwBiAGEAcwBlADEALAAgAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYgBhAHMAZQA4ACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAE0AdQBsACgAbABpAG0AYgBzAF8AYgBhAHMAZQA0ACwAIABsAGkAbQBiAHMAXwBiAGEAcwBlADQALAAgAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYgBhAHMAZQA5ACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAE0AdQBsACgAbABpAG0AYgBzAF8AYgBhAHMAZQA4ACwAIABsAGkAbQBiAHMAXwBiAGEAcwBlADEALAAgAGsAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAGUAeABwAG8AbgBlAG4AdABfAGQAaQBnAGkAdABzACwAIAAtAC0ATQBJAEQAKABlAHgAcABvAG4AZQBuAHQAXwBzAHQAcgBpAG4AZwAsACAAUwBFAFEAVQBFAE4AQwBFACgATABFAE4AKABlAHgAcABvAG4AZQBuAHQAXwBzAHQAcgBpAG4AZwApACkALAAgADEAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAFIARQBEAFUAQwBFACgAMQAsACAAZQB4AHAAbwBuAGUAbgB0AF8AZABpAGcAaQB0AHMALAAgAEwAQQBNAEIARABBACgAbABpAG0AYgBzAF8AYQBjAGMAdQBtAHUAbABhAHQAbwByACwAIABjAHUAcgByAGUAbgB0AF8AZABpAGcAaQB0ACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAATwBwAHQAaQBtAGkAegBlACAAdABoAGUAIABsAGUAYQBkAGkAbgBnACAAZQBkAGcAZQAgAHQAbwAgAGEAdgBvAGkAZAAgAHIAZQBkAHUAbgBkAGEAbgB0ACAAbQB1AGwAdABpAHAAbABpAGMAYQB0AGkAbwBuAHMAIABiAHkAIAAxAC4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAaQBzAF8AbwBuAGUALAAgAEEATgBEACgAUgBPAFcAUwAoAGwAaQBtAGIAcwBfAGEAYwBjAHUAbQB1AGwAYQB0AG8AcgApACAAPQAgADEALAAgAEkATgBEAEUAWAAoAGwAaQBtAGIAcwBfAGEAYwBjAHUAbQB1AGwAYQB0AG8AcgAsACAAMQAsACAAMQApACAAPQAgADEAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIAAxAC4AIABSAGEAaQBzAGUAIABBAGMAYwAgAHQAbwAgAHQAaABlACAAMQAwAHQAaAAgAHAAbwB3AGUAcgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBhAGMAYwBfADEAMAAsACAASQBGACgAaQBzAF8AbwBuAGUALAAgAGwAaQBtAGIAcwBfAGEAYwBjAHUAbQB1AGwAYQB0AG8AcgAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYQBjAGMAXwAyACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAE0AdQBsACgAbABpAG0AYgBzAF8AYQBjAGMAdQBtAHUAbABhAHQAbwByACwAIABsAGkAbQBiAHMAXwBhAGMAYwB1AG0AdQBsAGEAdABvAHIALAAgAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBhAGMAYwBfADQALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFUATQB1AGwAKABsAGkAbQBiAHMAXwBhAGMAYwBfADIALAAgAGwAaQBtAGIAcwBfAGEAYwBjAF8AMgAsACAAawApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGEAYwBjAF8AOAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBNAHUAbAAoAGwAaQBtAGIAcwBfAGEAYwBjAF8ANAAsACAAbABpAG0AYgBzAF8AYQBjAGMAXwA0ACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBNAHUAbAAoAGwAaQBtAGIAcwBfAGEAYwBjAF8AOAAsACAAbABpAG0AYgBzAF8AYQBjAGMAXwAyACwAIABrACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAAMgAuACAATQB1AGwAdABpAHAAbAB5ACAAYgB5ACAAdABoAGUAIABjAG8AcgByAGUAcwBwAG8AbgBkAGkAbgBnACAAYwBhAGMAaABlAGQAIAB2AGEAbAB1AGUAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgAYwB1AHIAcgBlAG4AdABfAGQAaQBnAGkAdAAgAD0AIAAwACwAIABsAGkAbQBiAHMAXwBhAGMAYwBfADEAMAAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYwBhAGMAaABlAF8AbQB1AGwAdABpAHAAbABpAGUAcgAsACAAQwBIAE8ATwBTAEUAKABjAHUAcgByAGUAbgB0AF8AZABpAGcAaQB0ACwAIABsAGkAbQBiAHMAXwBiAGEAcwBlADEALAAgAGwAaQBtAGIAcwBfAGIAYQBzAGUAMgAsACAAbABpAG0AYgBzAF8AYgBhAHMAZQAzACwAIABsAGkAbQBiAHMAXwBiAGEAcwBlADQALAAgAGwAaQBtAGIAcwBfAGIAYQBzAGUANQAsACAAbABpAG0AYgBzAF8AYgBhAHMAZQA2ACwAIABsAGkAbQBiAHMAXwBiAGEAcwBlADcALAAgAGwAaQBtAGIAcwBfAGIAYQBzAGUAOAAsACAAbABpAG0AYgBzAF8AYgBhAHMAZQA5ACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgAaQBzAF8AbwBuAGUALAAgAGwAaQBtAGIAcwBfAGMAYQBjAGgAZQBfAG0AdQBsAHQAaQBwAGwAaQBlAHIALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFUATQB1AGwAKABsAGkAbQBiAHMAXwBhAGMAYwBfADEAMAAsACAAbABpAG0AYgBzAF8AYwBhAGMAaABlAF8AbQB1AGwAdABpAHAAbABpAGUAcgAsACAAawApACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAApACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFsASQBuAHQAZQByAG4AYQBsAF0AIABSAGUAdAB1AHIAbgBzACAAdABoAGUAIABpAG4AdABlAGcAZQByACAAcwBxAHUAYQByAGUAIAByAG8AbwB0ACAAbwBmACAAdABoAGUAIAByAGEAZABpAGMAYQBuAGQAIAB1AHMAaQBuAGcAIABOAGUAdwB0AG8AbgAnAHMAIABNAGUAdABoAG8AZAAuAFwAbgAgACoAIABbAGwAaQBtAGIAcwBfAHIAYQBkAGkAYwBhAG4AZAA6ACAAQQByAHIAYQB5ACwAIABsAGkAbQBiAHMAXwBpAG4AaQB0AGkAYQBsAF8AeAA6ACAAQQByAHIAYQB5ACwAIABrADoAIABpAG4AdABdAFwAbgAgACoALwBcAG4AVQBTAHEAcgB0ACAAPQAgAEwAQQBNAEIARABBACgAbABpAG0AYgBzAF8AcgBhAGQAaQBjAGEAbgBkACwAIABsAGkAbQBiAHMAXwBpAG4AaQB0AGkAYQBsAF8AeAAsACAAawAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABtAGEAeABpAG0AdQBtAF8AaQB0AGUAcgBhAHQAaQBvAG4AcwAsACAAMwA1ACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAG4AYQBsAF8AcABhAGMAawBlAGQAXwBzAHQAYQB0AGUALAAgAFIARQBEAFUAQwBFACgAVgBTAFQAQQBDAEsAKAAwACwAIABsAGkAbQBiAHMAXwBpAG4AaQB0AGkAYQBsAF8AeAApACwAIABTAEUAUQBVAEUATgBDAEUAKABtAGEAeABpAG0AdQBtAF8AaQB0AGUAcgBhAHQAaQBvAG4AcwApACwAIABMAEEATQBCAEQAQQAoAHAAYQBjAGsAZQBkAF8AcwB0AGEAdABlACwAIABpACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAaABhAHMAXwBjAG8AbgB2AGUAcgBnAGUAZAAsACAASQBOAEQARQBYACgAcABhAGMAawBlAGQAXwBzAHQAYQB0AGUALAAgADEALAAgADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGMAdQByAHIAZQBuAHQAXwB4ACwAIABEAFIATwBQACgAcABhAGMAawBlAGQAXwBzAHQAYQB0AGUALAAgADEAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABoAGEAcwBfAGMAbwBuAHYAZQByAGcAZQBkACwAIABwAGEAYwBrAGUAZABfAHMAdABhAHQAZQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAAMQAuACAARABpAHYAaQBzAGkAbwBuADoAIABuACAALwAgAHgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHAAYQBjAGsAZQBkAF8AZABpAHYAaQBzAGkAbwBuAF8AcgBlAHMAdQBsAHQALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAEQAaQB2AFIAbwB1AHQAZQByACgAbABpAG0AYgBzAF8AcgBhAGQAaQBjAGEAbgBkACwAIABsAGkAbQBiAHMAXwBjAHUAcgByAGUAbgB0AF8AeAAsACAAawApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAG4AdQBtAF8AbABpAG0AYgBzAF8AcgAsACAASQBOAEQARQBYACgAcABhAGMAawBlAGQAXwBkAGkAdgBpAHMAaQBvAG4AXwByAGUAcwB1AGwAdAAsACAAMQAsACAAMQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAHEALAAgAEQAUgBPAFAAKABwAGEAYwBrAGUAZABfAGQAaQB2AGkAcwBpAG8AbgBfAHIAZQBzAHUAbAB0ACwAIABuAHUAbQBfAGwAaQBtAGIAcwBfAHIAIAArACAAMQApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIAAyAC4AIABBAGQAZABpAHQAaQBvAG4AOgAgAHgAIAArACAAKABuACAALwAgAHgAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AcwB1AG0AXwB4AHEALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFUAQQBkAGQAKABsAGkAbQBiAHMAXwBjAHUAcgByAGUAbgB0AF8AeAAsACAAbABpAG0AYgBzAF8AcQAsACAAawApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIAAzAC4AIABIAGEAbAB2AGkAbgBnADoAIAAoAHgAIAArACAAKABuACAALwAgAHgAKQApACAALwAgADIAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAEsAbgB1AHQAaABEAGkAdgAgAGkAbgBoAGUAcgBlAG4AdABsAHkAIABzAHUAcABwAG8AcgB0AHMAIABzAGMAYQBsAGEAcgAgAGQAaQB2AGkAcwBvAHIAcwAgAHcAaQB0AGgAIAB6AGUAcgBvACAAbwB2AGUAcgBoAGUAYQBkAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABwAGEAYwBrAGUAZABfAGgAYQBsAGYAXwByAGUAcwB1AGwAdAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4ASwBuAHUAdABoAEQAaQB2ACgAbABpAG0AYgBzAF8AcwB1AG0AXwB4AHEALAAgAHsAMgB9ACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbgB1AG0AXwBsAGkAbQBiAHMAXwBoAGEAbABmAGUAZAAsACAASQBOAEQARQBYACgAcABhAGMAawBlAGQAXwBoAGEAbABmAF8AcgBlAHMAdQBsAHQALAAgADEALAAgADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBuAGUAeAB0AF8AeAAsACAARABSAE8AUAAoAHAAYQBjAGsAZQBkAF8AaABhAGwAZgBfAHIAZQBzAHUAbAB0ACwAIABuAHUAbQBfAGwAaQBtAGIAcwBfAGgAYQBsAGYAZQBkACAAKwAgADEAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAANAAuACAAQwBvAG4AdgBlAHIAZwBlAG4AYwBlACAAQwBoAGUAYwBrAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABjAG8AbgB2AGUAcgBnAGUAbgBjAGUAXwBjAG8AbQBwAGEAcgBpAHMAbwBuACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAEMAbwBtAHAAYQByAGUAKABsAGkAbQBiAHMAXwBuAGUAeAB0AF8AeAAsACAAbABpAG0AYgBzAF8AYwB1AHIAcgBlAG4AdABfAHgAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAATgBlAHcAdABvAG4AJwBzACAAbQBlAHQAaABvAGQAIABjAG8AbgB2AGUAcgBnAGUAcwAgAG8AbgAgAHQAaABlACAAZgBsAG8AbwByACAAcgBvAG8AdAAgAGEAbgBkACAAcwB0AGEAYgBpAGwAaQB6AGUAcwAgAG8AcgAgAG8AcwBjAGkAbABsAGEAdABlAHMAIAB1AHAAIABiAHkAIAAxAC4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAFQAaABlAHIAZQBmAG8AcgBlACwAIABpAGYAIAB4AF8AbgBlAHgAdAAgAD4APQAgAGMAdQByAHIAXwB4ACwAIAB0AGgAZQAgAGEAbABnAG8AcgBpAHQAaABtACAAaABhAHMAIABjAG8AbgB2AGUAcgBnAGUAZAAuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABjAG8AbgB2AGUAcgBnAGUAbgBjAGUAXwBjAG8AbQBwAGEAcgBpAHMAbwBuACAAPgA9ACAAMAAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFYAUwBUAEEAQwBLACgAMQAsACAAbABpAG0AYgBzAF8AYwB1AHIAcgBlAG4AdABfAHgAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFYAUwBUAEEAQwBLACgAMAAsACAAbABpAG0AYgBzAF8AbgBlAHgAdABfAHgAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACkAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAEQAUgBPAFAAKABmAGkAbgBhAGwAXwBwAGEAYwBrAGUAZABfAHMAdABhAHQAZQAsACAAMQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABbAEkAbgB0AGUAcgBuAGEAbABdACAAUgBlAHQAdQByAG4AcwAgAGEAIAB2AGUAcgB0AGkAYwBhAGwAIABhAHIAcgBhAHkAIABvAGYAIABwAHIAaQBtAGUAIABuAHUAbQBiAGUAcgBzACAAdQBwACAAdABvACAAbgAuAFwAbgAgACoAIABbAG4AOgAgAGkAbgB0AF0AXABuACAAKgAvAFwAbgBOAGEAdABpAHYAZQBQAHIAaQBtAGUAcwAgAD0AIABMAEEATQBCAEQAQQAoAG4ALABcAG4AIAAgACAAIABJAEYAKABuACAAPAAgADIALAAgACMATgBVAE0AIQAsAFwAbgAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAYwBhAG4AZABpAGQAYQB0AGUAXwBzAGUAcQB1AGUAbgBjAGUALAAgAFMARQBRAFUARQBOAEMARQAoAG4AIAAtACAAMQAsACAAMQAsACAAMgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSACgAYwBhAG4AZABpAGQAYQB0AGUAXwBzAGUAcQB1AGUAbgBjAGUALAAgAE0AQQBQACgAYwBhAG4AZABpAGQAYQB0AGUAXwBzAGUAcQB1AGUAbgBjAGUALAAgAEwAQQBNAEIARABBACgAYwB1AHIAcgBlAG4AdABfAGMAYQBuAGQAaQBkAGEAdABlACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGkAdAAsACAASQBOAFQAKABTAFEAUgBUACgAYwB1AHIAcgBlAG4AdABfAGMAYQBuAGQAaQBkAGEAdABlACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgAbABpAG0AaQB0ACAAPAAgADIALAAgAFQAUgBVAEUALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBJAE4AKABNAE8ARAAoAGMAdQByAHIAZQBuAHQAXwBjAGEAbgBkAGkAZABhAHQAZQAsACAAUwBFAFEAVQBFAE4AQwBFACgAbABpAG0AaQB0ACAALQAgADEALAAgADEALAAgADIAKQApACkAIAA+ACAAMABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQApACkAXABuACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABbAEkAbgB0AGUAcgBuAGEAbABdACAASABpAGcAaAAtAHAAZQByAGYAbwByAG0AYQBuAGMAZQAgAG0AdQBsAHQAaQBwAGwAaQBjAGEAdABpAG8AbgAgAG8AZgAgAG4AbwByAG0AYQBsAGkAegBlAGQAIABwAG8AcwBpAHQAaQB2AGUAIABzAHQAcgBpAG4AZwBzAC4AIABCAHkAcABhAHMAcwBlAHMAIABMAGEAeQBlAHIAIAAwAC4AXABuACAAKgAgAFsAbgBvAHIAbQBfAGEAOgAgAFQAZQB4AHQALAAgAG4AbwByAG0AXwBiADoAIABUAGUAeAB0AF0AXABuACAAKgAvAFwAbgBVAFQAZQB4AHQATQB1AGwAIAA9ACAATABBAE0AQgBEAEEAKABuAG8AcgBtAF8AYQAsACAAbgBvAHIAbQBfAGIALABcAG4AIAAgACAAIABJAEYAKABPAFIAKABuAG8AcgBtAF8AYQAgAD0AIABcACIAMABcACIALAAgAG4AbwByAG0AXwBiACAAPQAgAFwAIgAwAFwAIgApACwAIABcACIAMABcACIALABcAG4AIAAgACAAIABJAEYAKABuAG8AcgBtAF8AYQAgAD0AIABcACIAMQBcACIALAAgAG4AbwByAG0AXwBiACwAXABuACAAIAAgACAASQBGACgAbgBvAHIAbQBfAGIAIAA9ACAAXAAiADEAXAAiACwAIABuAG8AcgBtAF8AYQAsAFwAbgAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABlAG4AXwBhACwAIABMAEUATgAoAG4AbwByAG0AXwBhACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABlAG4AXwBiACwAIABMAEUATgAoAG4AbwByAG0AXwBiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAawAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwBhAGYAZQBLACgAXAAiAE0AVQBMAFwAIgAsACAATQBJAE4AKABsAGUAbgBfAGEALAAgAGwAZQBuAF8AYgApACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGEALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFMAcABsAGkAdAAoAG4AbwByAG0AXwBhACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYgAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwBwAGwAaQB0ACgAbgBvAHIAbQBfAGIALAAgAGsAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAZgBpAG4AYQBsAF8AbABpAG0AYgBzACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAE0AdQBsACgAbABpAG0AYgBzAF8AYQAsACAAbABpAG0AYgBzAF8AYgAsACAAawApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBNAGUAcgBnAGUAKABmAGkAbgBhAGwAXwBsAGkAbQBiAHMALAAgAGsAKQBcAG4AIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQApACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABbAEkAbgB0AGUAcgBuAGEAbABdACAAUgBlAHQAdQByAG4AcwAgAHQAaABlACAAcAByAG8AZAB1AGMAdAAgAG8AZgAgAGEAbgAgAGEAcgByAGEAeQAgAG8AZgAgAHMAdAByAGkAbgBnAHMAIAB1AHMAaQBuAGcAIABhACAAcgBlAGMAdQByAHMAaQB2AGUAIAB0AG8AdQByAG4AYQBtAGUAbgB0ACAAdAByAGUAZQAuAFwAbgAgACoAIABbAGEAcgByAF8AcwB0AHIAaQBuAGcAcwA6ACAAQQByAHIAYQB5AF0AXABuACAAKgAvAFwAbgBUAGUAeAB0AFQAcgBlAGUAUAByAG8AZAAgAD0AIABMAEEATQBCAEQAQQAoAGEAcgByAF8AcwB0AHIAaQBuAGcAcwAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABuAHUAbQBfAGUAbABlAG0AZQBuAHQAcwAsACAAUgBPAFcAUwAoAGEAcgByAF8AcwB0AHIAaQBuAGcAcwApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAbgB1AG0AXwBlAGwAZQBtAGUAbgB0AHMAIAA9ACAAMQAsACAASQBOAEQARQBYACgAYQByAHIAXwBzAHQAcgBpAG4AZwBzACwAIAAxACwAIAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIABSAGUAcwBoAGEAcABlACAAYQByAHIAYQB5ACAAaQBuAHQAbwAgAHAAYQBpAHIAcwAuACAATwBkAGQALQBsAGUAbgBnAHQAaAAgAGEAcgByAGEAeQBzACAAYQByAGUAIABzAGEAZgBlAGwAeQAgAHAAYQBkAGQAZQBkACAAdwBpAHQAaAAgAHQAaABlACAAbQB1AGwAdABpAHAAbABpAGMAYQB0AGkAdgBlACAAaQBkAGUAbgB0AGkAdAB5ACAAXAAiADEAXAAiAC4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcABhAGkAcgBlAGQAXwBzAHQAcgBpAG4AZwBzACwAIABXAFIAQQBQAFIATwBXAFMAKABhAHIAcgBfAHMAdAByAGkAbgBnAHMALAAgADIALAAgAFwAIgAxAFwAIgApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAFYAZQBjAHQAbwByAGkAegBlAGQAIABtAHUAbAB0AGkAcABsAGkAYwBhAHQAaQBvAG4AIABhAGMAcgBvAHMAcwAgAGEAbABsACAAcABhAGkAcgBzACAAcwBpAG0AdQBsAHQAYQBuAGUAbwB1AHMAbAB5ACAAbQBpAG4AaQBtAGkAegBlAHMAIAByAGUAYwB1AHIAcwBpAHYAZQAgAGQAZQBwAHQAaAAuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHIAZQBkAHUAYwBlAGQAXwBhAHIAcgBhAHkALAAgAEIAWQBSAE8AVwAoAHAAYQBpAHIAZQBkAF8AcwB0AHIAaQBuAGcAcwAsACAATABBAE0AQgBEAEEAKAByAG8AdwAsACAAVQBUAGUAeAB0AE0AdQBsACgASQBOAEQARQBYACgAcgBvAHcALAAgADEALAAgADEAKQAsACAASQBOAEQARQBYACgAcgBvAHcALAAgADEALAAgADIAKQApACkAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBUAGUAeAB0AFQAcgBlAGUAUAByAG8AZAAoAHIAZQBkAHUAYwBlAGQAXwBhAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFsASQBuAHQAZQByAG4AYQBsAF0AIABSAGUAdAB1AHIAbgBzACAAdABoAGUAIABlAHgAcABvAG4AZQBuAHQAIABmAG8AcgAgAGUAYQBjAGgAIABwAHIAaQBtAGUAIABpAG4AIAB0AGgAZQAgAFAAcgBpAG0AZQAgAFMAdwBpAG4AZwAgAHQAZQByAG0ALgBcAG4AIAAqACAAWwBuADoAIABpAG4AdAAsACAAcAByAGkAbQBlAHMAOgAgAEEAcgByAGEAeQBdAFwAbgAgACoALwBcAG4ATgBhAHQAaQB2AGUAUwB3AGkAbgBnAEUAeABwAG8AbgBlAG4AdABzACAAPQAgAEwAQQBNAEIARABBACgAbgAsACAAcAByAGkAbQBlAHMALABcAG4AIAAgACAAIABNAEEAUAAoAHAAcgBpAG0AZQBzACwAIABMAEEATQBCAEQAQQAoAHAALABcAG4AIAAgACAAIAAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAG0AYQB4AF8AcABvAHcAZQByAF8AawAsACAASQBOAFQAKABMAE8ARwAoAG4ALAAgAHAAKQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHAAcgBpAG0AZQBfAHAAbwB3AGUAcgBzACwAIABwACAAXgAgAFMARQBRAFUARQBOAEMARQAoAG0AYQB4AF8AcABvAHcAZQByAF8AawApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFMAVQBNACgATQBPAEQAKABJAE4AVAAoAG4AIAAvACAAcAByAGkAbQBlAF8AcABvAHcAZQByAHMAKQAsACAAMgApACkAXABuACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFsASQBuAHQAZQByAG4AYQBsAF0AIABSAGUAdAB1AHIAbgBzACAAdABoAGUAIABTAHcAaQBuAGcAIAB0AGUAcgBtACAAZgBvAHIAIAB0AGgAZQAgAGMAdQByAHIAZQBuAHQAIABmAGEAYwB0AG8AcgBpAGEAbAAgAHQAaQBlAHIAIABhAHMAIABhACAAcwB0AHIAaQBuAGcALgBcAG4AIAAqACAAWwBuADoAIABpAG4AdAAsACAAdABpAGUAcgBfAHAAcgBpAG0AZQBzADoAIABBAHIAcgBhAHkAXQBcAG4AIAAqAC8AXABuAFMAdwBpAG4AZwBUAGUAcgBtACAAPQAgAEwAQQBNAEIARABBACgAbgAsACAAdABpAGUAcgBfAHAAcgBpAG0AZQBzACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAHMAdwBpAG4AZwBfAGUAeABwAG8AbgBlAG4AdABzACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBOAGEAdABpAHYAZQBTAHcAaQBuAGcARQB4AHAAbwBuAGUAbgB0AHMAKABuACwAIAB0AGkAZQByAF8AcAByAGkAbQBlAHMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAaABhAHMAXwBuAGEAdABpAHYAZQBfAGUAeABwAG8AbgBlAG4AdAAsACAAcwB3AGkAbgBnAF8AZQB4AHAAbwBuAGUAbgB0AHMAIAA+ACAAMAAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAC8ALwAgAFAAcgBpAG0AZQBzACAAdwBpAHQAaAAgAGUAeABwAG8AbgBlAG4AdAAgADAAIABkAG8AIABuAG8AdAAgAGMAbwBuAHQAcgBpAGIAdQB0AGUAIAB0AG8AIAB0AGgAZQAgAHMAdwBpAG4AZwAgAHQAZQByAG0ALgBcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAEEATgBEACgATgBPAFQAKABoAGEAcwBfAG4AYQB0AGkAdgBlAF8AZQB4AHAAbwBuAGUAbgB0ACkAKQAsACAAXAAiADEAXAAiACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAYQBjAHQAaQB2AGUAXwBwAHIAaQBtAGUAcwAsACAARgBJAEwAVABFAFIAKAB0AGkAZQByAF8AcAByAGkAbQBlAHMALAAgAGgAYQBzAF8AbgBhAHQAaQB2AGUAXwBlAHgAcABvAG4AZQBuAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGEAYwB0AGkAdgBlAF8AZQB4AHAAbwBuAGUAbgB0AHMALAAgAEYASQBMAFQARQBSACgAcwB3AGkAbgBnAF8AZQB4AHAAbwBuAGUAbgB0AHMALAAgAGgAYQBzAF8AbgBhAHQAaQB2AGUAXwBlAHgAcABvAG4AZQBuAHQAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABlAHYAYQBsAHUAdABhAHQAZQBkAF8AcAByAGkAbQBlAF8AcABvAHcAZQByAHMALAAgAE0AQQBQACgAYQBjAHQAaQB2AGUAXwBwAHIAaQBtAGUAcwAsACAAYQBjAHQAaQB2AGUAXwBlAHgAcABvAG4AZQBuAHQAcwAsACAATABBAE0AQgBEAEEAKABwACwAIABlACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABlACAAPQAgADEALAAgAHAAIAAmACAAXAAiAFwAIgAsACAAQgBpAGcASQBuAHQALgBQAG8AdwAoAHAAIAAmACAAXAAiAFwAIgAsACAAZQAgACYAIABcACIAXAAiACkAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVABlAHgAdABUAHIAZQBlAFAAcgBvAGQAKABlAHYAYQBsAHUAdABhAHQAZQBkAF8AcAByAGkAbQBlAF8AcABvAHcAZQByAHMAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFsASQBuAHQAZQByAG4AYQBsAF0AIABSAGUAdAB1AHIAbgBzACAAbgAhACAAYQBzACAAYQAgAHMAdAByAGkAbgBnACAAdQBzAGkAbgBnACAAdABoAGUAIAByAGUAYwB1AHIAcwBpAHYAZQAgAFAAcgBpAG0AZQAgAFMAdwBpAG4AZwAgAGEAbABnAG8AcgBpAHQAaABtAC4AXABuACAAKgAgAFsAbgA6ACAAaQBuAHQALAAgAGcAbABvAGIAYQBsAF8AcAByAGkAbQBlAHMAOgAgAEEAcgByAGEAeQBdAFwAbgAgACoALwBcAG4AUAByAGkAbQBlAFMAdwBpAG4AZwBLAGUAcgBuAGUAbAAgAD0AIABMAEEATQBCAEQAQQAoAG4ALAAgAGcAbABvAGIAYQBsAF8AcAByAGkAbQBlAHMALABcAG4AIAAgACAAIABJAEYAKABuACAAPAAgADIALAAgAFwAIgAxAFwAIgAsAFwAbgAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAZgBsAG8AbwByAF8AaABhAGwAZgBfAG4ALAAgAEkATgBUACgAbgAgAC8AIAAyACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAZgBhAGMAdABvAHIAaQBhAGwAXwBoAGEAbABmAF8AbgAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUAByAGkAbQBlAFMAdwBpAG4AZwBLAGUAcgBuAGUAbAAoAGYAbABvAG8AcgBfAGgAYQBsAGYAXwBuACwAIABnAGwAbwBiAGEAbABfAHAAcgBpAG0AZQBzACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAEYAYQBjAHQAbwByAGkAYQBsAHMAIABhAHIAZQAgAGIAdQBpAGwAdAAgAGIAeQAgAHMAcQB1AGEAcgBpAG4AZwAgAHQAaABlACAAcAByAGUAdgBpAG8AdQBzACAAdABpAGUAcgAgACgAbgAvADIAKQAhACAAYQBuAGQAIABtAHUAbAB0AGkAcABsAHkAaQBuAGcAIABiAHkAIAB0AGgAZQAgAHMAdwBpAG4AZwAgAHQAZQByAG0ALgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAcwBxAHUAYQByAGUAZABfAGgAYQBsAGYAXwBmAGEAYwB0AG8AcgBpAGEAbAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBUAGUAeAB0AE0AdQBsACgAZgBhAGMAdABvAHIAaQBhAGwAXwBoAGEAbABmAF8AbgAsACAAZgBhAGMAdABvAHIAaQBhAGwAXwBoAGEAbABmAF8AbgApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABhAHAAcABsAGkAYwBhAGIAbABlAF8AdABpAGUAcgBfAHAAcgBpAG0AZQBzACwAIABGAEkATABUAEUAUgAoAGcAbABvAGIAYQBsAF8AcAByAGkAbQBlAHMALAAgAGcAbABvAGIAYQBsAF8AcAByAGkAbQBlAHMAIAA8AD0AIABuACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAcwB0AHIAXwBzAHcAaQBuAGcAXwB0AGUAcgBtACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBTAHcAaQBuAGcAVABlAHIAbQAoAG4ALAAgAGEAcABwAGwAaQBjAGEAYgBsAGUAXwB0AGkAZQByAF8AcAByAGkAbQBlAHMAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBUAGUAeAB0AE0AdQBsACgAcwBxAHUAYQByAGUAZABfAGgAYQBsAGYAXwBmAGEAYwB0AG8AcgBpAGEAbAAsACAAcwB0AHIAXwBzAHcAaQBuAGcAXwB0AGUAcgBtACkAXABuACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABbAEkAbgB0AGUAcgBuAGEAbABdACAAUgBlAHQAdQByAG4AcwAgAE0AaQBuAC8ATQBhAHgAIABmAHIAbwBtACAAYQBuACAAYQByAHIAYQB5ACAAbwBmACAAcwB0AHIAaQBuAGcAcwAgAHUAcwBpAG4AZwAgAGEAIAByAGUAYwB1AHIAcwBpAHYAZQAgAHQAbwB1AHIAbgBhAG0AZQBuAHQAIAB0AHIAZQBlAC4AXABuACAAKgAgAFsAcwB0AHIAXwBuAG8AcgBtAHMAOgAgAEEAcgByAGEAeQAsACAAYwBvAG0AcABhAHIAaQBzAG8AbgBfAG0AbwBkAGUAOgAgAGkAbgB0AF0AXABuACAAKgAvAFwAbgBUAHIAZQBlAEMAbwBtAHAAYQByAGUAIAA9ACAATABBAE0AQgBEAEEAKABzAHQAcgBfAG4AbwByAG0AcwAsACAAYwBvAG0AcABhAHIAaQBzAG8AbgBfAG0AbwBkAGUALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbgB1AG0AXwByAG8AdwBzACwAIABSAE8AVwBTACgAcwB0AHIAXwBuAG8AcgBtAHMAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAG4AdQBtAF8AcgBvAHcAcwAgAD0AIAAxACwAIABJAE4ARABFAFgAKABzAHQAcgBfAG4AbwByAG0AcwAsACAAMQAsACAAMQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAdABvAHUAcgBuAGEAbQBlAG4AdABfAHAAYQBpAHIAcwAsACAAVwBSAEEAUABSAE8AVwBTACgAcwB0AHIAXwBuAG8AcgBtAHMALAAgADIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGMAbwBtAHAAZQB0AGkAdABvAHIAcwBfAGEALAAgAFQAQQBLAEUAKAB0AG8AdQByAG4AYQBtAGUAbgB0AF8AcABhAGkAcgBzACwAIAAsACAAMQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAYwBvAG0AcABlAHQAaQB0AG8AcgBzAF8AYgAsACAAVABBAEsARQAoAHQAbwB1AHIAbgBhAG0AZQBuAHQAXwBwAGEAaQByAHMALAAgACwAIAAtADEAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAByAG8AdQBuAGQAXwB3AGkAbgBuAGUAcgBzACwAIABNAEEAUAAoAGMAbwBtAHAAZQB0AGkAdABvAHIAcwBfAGEALAAgAGMAbwBtAHAAZQB0AGkAdABvAHIAcwBfAGIALAAgAEwAQQBNAEIARABBACgAYQAsACAAYgAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgASQBTAE4AQQAoAGIAKQAsACAAYQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGMAbwBtAHAAYQByAGkAcwBvAG4AXwByAGUAcwB1AGwAdAAsACAAQgBpAGcASQBuAHQALgBDAG8AbQBwAGEAcgBlACgAYQAsACAAYgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgAYwBvAG0AcABhAHIAaQBzAG8AbgBfAHIAZQBzAHUAbAB0ACAAKgAgAGMAbwBtAHAAYQByAGkAcwBvAG4AXwBtAG8AZABlACAAPgA9ACAAMAAsACAAYQAsACAAYgApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVAByAGUAZQBDAG8AbQBwAGEAcgBlACgAcgBvAHUAbgBkAF8AdwBpAG4AbgBlAHIAcwAsACAAYwBvAG0AcABhAHIAaQBzAG8AbgBfAG0AbwBkAGUAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQgBpAGcASQBuAHQAIgAsACIAdABlAHgAdAAiADoAIgAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwBcAG4ALwAvACAAQgBpAGcAIABJAG4AdABlAGcAZQByACAAQQByAGkAdABoAG0AZQB0AGkAYwAgAEwAaQBiAHIAYQByAHkAIAAvAC8AXABuAC8ALwAgACAAIAAgACAAIAAgACAAQgBpAGcASQBuAHQAIABNAG8AZAB1AGwAZQAgACAAIAAgACAAIAAgACAAIAAgACAALwAvAFwAbgAvAC8AIAAgACAAIAAgACAAIAAgACAAIABQAHUAYgBsAGkAYwAgAEEAUABJACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwBcAG4ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8ALwAvAC8AXABuAFwAbgAvACoAKgBcAG4AIAAqACAATgBvAHIAbQBhAGwAaQBzAGUAcwAgAGEAIABCAGkAZwBJAG4AdAAgAHMAdAByAGkAbgBnAC4AIABTAHQAcgBpAHAAcwAgAGwAZQBhAGQAaQBuAGcAIAB6AGUAcgBvAHMALAAgAHIAZQBzAG8AbAB2AGUAcwAgAFwAIgAtADAAXAAiACAAdABvACAAXAAiADAAXAAiACwAIABhAG4AZAAgAHQAaAByAG8AdwBzACAAIwBWAEEATABVAEUAIQAgAG8AbgAgAGkAbgB2AGEAbABpAGQAIABjAGgAYQByAGEAYwB0AGUAcgBzAC4AXABuACAAKgAgAFsAaQBuAHAAdQB0ADoAIABUAGUAeAB0AF0AXABuACAAKgAvAFwAbgBOAG8AcgBtACAAPQAgAEwAQQBNAEIARABBACgAaQBuAHAAdQB0ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAHMAdAByAF8AaQBuAHAAdQB0ACwAIABJAEYAKABPAFIAKABJAFMATwBNAEkAVABUAEUARAAoAGkAbgBwAHUAdAApACwAIABpAG4AcAB1AHQAIAA9ACAAXAAiAFwAIgApACwAIABcACIAMABcACIALAAgAGkAbgBwAHUAdAAgACYAIABcACIAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAGkAcwBfAHYAYQBsAHUAZQBfAGYAbwByAG0AYQB0ACwAIABSAEUARwBFAFgAVABFAFMAVAAoAHMAdAByAF8AaQBuAHAAdQB0ACwAIABcACIAXgAtAD8AXABcAGQAKwAkAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAcgBfAG4AbwByAG0ALAAgAFIARQBHAEUAWABSAEUAUABMAEEAQwBFACgAcwB0AHIAXwBpAG4AcAB1AHQALAAgAFwAIgBeACgALQA/ACkAMAArACgAPwA9AFwAXABkACkAXAAiACwAIABcACIAJAAxAFwAIgApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgATgBPAFQAKABpAHMAXwB2AGEAbAB1AGUAXwBmAG8AcgBtAGEAdAApACwAIABWAEEATABVAEUAKABcACIAIwBWAEEATABVAEUAIQBcACIAKQAsACAASQBGACgAcwB0AHIAXwBuAG8AcgBtACAAPQAgAFwAIgAtADAAXAAiACwAIABcACIAMABcACIALAAgAHMAdAByAF8AbgBvAHIAbQApACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFIAZQB0AHUAcgBuAHMAIAB0AGgAZQAgAHMAaQBnAG4AIABvAGYAIABhACAAQgBpAGcASQBuAHQAOgAgADEAIAAoAHAAbwBzAGkAdABpAHYAZQApACwAIAAtADEAIAAoAG4AZQBnAGEAdABpAHYAZQApACwAIABvAHIAIAAwACAAKAB6AGUAcgBvACkALgBcAG4AIAAqACAAWwBpAG4AcAB1AHQAOgAgAFQAZQB4AHQAXQBcAG4AIAAqAC8AXABuAFMAaQBnAG4AIAA9ACAATABBAE0AQgBEAEEAKABpAG4AcAB1AHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AHIAXwBuAG8AcgBtACwAIABOAG8AcgBtACgAaQBuAHAAdQB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFMAVwBJAFQAQwBIACgATABFAEYAVAAoAHMAdAByAF8AbgBvAHIAbQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAwAFwAIgAsACAAMAAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIALQBcACIALAAgAC0AMQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvAC8AIAAtAC0ALQAgAFAAcgBlAGQAaQBjAGEAdABlAHMAIAAtAC0ALQAgAFwAXABcAFwAXABuAFwAbgAvACoAKgBcAG4AIAAqACAAUgBlAHQAdQByAG4AcwAgAFQAUgBVAEUAIABpAGYAIAB0AGgAZQAgAEIAaQBnAEkAbgB0ACAAaQBzACAAZQB4AGEAYwB0AGwAeQAgAHoAZQByAG8ALgBcAG4AIAAqACAAWwBpAG4AcAB1AHQAOgAgAFQAZQB4AHQAXQBcAG4AIAAqAC8AXABuAEkAcwBaAGUAcgBvACAAPQAgAEwAQQBNAEIARABBACgAaQBuAHAAdQB0ACwAIABOAG8AcgBtACgAaQBuAHAAdQB0ACkAIAA9ACAAXAAiADAAXAAiACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABSAGUAdAB1AHIAbgBzACAAVABSAFUARQAgAGkAZgAgAHQAaABlACAAQgBpAGcASQBuAHQAIABpAHMAIABuAGUAZwBhAHQAaQB2AGUALgBcAG4AIAAqACAAWwBpAG4AcAB1AHQAOgAgAFQAZQB4AHQAXQBcAG4AIAAqAC8AXABuAEkAcwBOAGUAZwAgAD0AIABMAEEATQBCAEQAQQAoAGkAbgBwAHUAdAAsACAATABFAEYAVAAoAE4AbwByAG0AKABpAG4AcAB1AHQAKQApACAAPQAgAFwAIgAtAFwAIgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAAUgBlAHQAdQByAG4AcwAgAFQAUgBVAEUAIABpAGYAIAB0AGgAZQAgAEIAaQBnAEkAbgB0ACAAaQBzACAAZQB2AGUAbgAuAFwAbgAgACoAIABbAGkAbgBwAHUAdAA6ACAAVABlAHgAdABdAFwAbgAgACoALwBcAG4ASQBzAEUAdgBlAG4AIAA9ACAATABBAE0AQgBEAEEAKABpAG4AcAB1AHQALAAgAEkAUwBFAFYARQBOACgAVgBBAEwAVQBFACgAUgBJAEcASABUACgATgBvAHIAbQAoAGkAbgBwAHUAdAApACkAKQApACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABSAGUAdAB1AHIAbgBzACAAVABSAFUARQAgAGkAZgAgAHQAaABlACAAQgBpAGcASQBuAHQAIABpAHMAIABvAGQAZAAuAFwAbgAgACoAIABbAGkAbgBwAHUAdAA6ACAAVABlAHgAdABdAFwAbgAgACoALwBcAG4ASQBzAE8AZABkACAAPQAgAEwAQQBNAEIARABBACgAaQBuAHAAdQB0ACwAIABJAFMATwBEAEQAKABWAEEATABVAEUAKABSAEkARwBIAFQAKABOAG8AcgBtACgAaQBuAHAAdQB0ACkAKQApACkAKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFIAZQB0AHUAcgBuAHMAIAB0AGgAZQAgAHUAbgBzAGkAZwBuAGUAZAAgAG0AYQBnAG4AaQB0AHUAZABlACAAbwBmACAAYQAgAEIAaQBnAEkAbgB0ACAAcwB0AHIAaQBuAGcAIAAoAGEAYgBzAG8AbAB1AHQAZQAgAHYAYQBsAHUAZQApAC4AXABuACAAKgAgAFsAaQBuAHAAdQB0ADoAIABUAGUAeAB0AF0AXABuACAAKgAvAFwAbgBBAGIAcwAgAD0AIABMAEEATQBCAEQAQQAoAGkAbgBwAHUAdAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABzAHQAcgBfAG4AbwByAG0ALAAgAE4AbwByAG0AKABpAG4AcAB1AHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgATABFAEYAVAAoAHMAdAByAF8AbgBvAHIAbQApACAAPQAgAFwAIgAtAFwAIgAsACAATQBJAEQAKABzAHQAcgBfAG4AbwByAG0ALAAgADIALAAgAEwARQBOACgAcwB0AHIAXwBuAG8AcgBtACkAIAAtACAAMQApACwAIABzAHQAcgBfAG4AbwByAG0AKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAAUgBlAHQAdQByAG4AcwAgADEAIAAoAGEAIAA+ACAAYgApACwAIAAtADEAIAAoAGEAIAA8ACAAYgApACwAIABvAHIAIAAwACAAKABhACAAPQAgAGIAKQAuACAAQwBvAG0AcABhAHIAZQBzACAAcwBpAGcAbgBzACAAYQBuAGQAIABsAGUAbgBnAHQAaABzACAAYgBlAGYAbwByAGUAIABsAGkAbQBiACAAYQBuAGEAbAB5AHMAaQBzAC4AXABuACAAKgAgAFsAaQBuAHAAdQB0AF8AYQA6ACAAVABlAHgAdAAsACAAaQBuAHAAdQB0AF8AYgA6ACAAVABlAHgAdABdAFwAbgAgACoALwBcAG4AQwBvAG0AcABhAHIAZQAgAD0AIABMAEEATQBCAEQAQQAoAGkAbgBwAHUAdABfAGEALAAgAGkAbgBwAHUAdABfAGIALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AHIAXwBuAG8AcgBtAF8AYQAsACAATgBvAHIAbQAoAGkAbgBwAHUAdABfAGEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AHIAXwBuAG8AcgBtAF8AYgAsACAATgBvAHIAbQAoAGkAbgBwAHUAdABfAGIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwBpAGcAbgBfAGEALAAgAEIAaQBnAEkAbgB0AC4AUwBpAGcAbgAoAHMAdAByAF8AbgBvAHIAbQBfAGEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwBpAGcAbgBfAGIALAAgAEIAaQBnAGkAbgB0AC4AUwBpAGcAbgAoAHMAdAByAF8AbgBvAHIAbQBfAGIAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAHMAaQBnAG4AXwBhACAAPAA+ACAAcwBpAGcAbgBfAGIALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUwBJAEcATgAoAHMAaQBnAG4AXwBhACAALQAgAHMAaQBnAG4AXwBiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgAcwBpAGcAbgBfAGEAIAA9ACAAMAAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgADAALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABlAG4AXwBhACwAIABMAEUATgAoAHMAdAByAF8AbgBvAHIAbQBfAGEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABlAG4AXwBiACwAIABMAEUATgAoAHMAdAByAF8AbgBvAHIAbQBfAGIAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEkARgAoAGwAZQBuAF8AYQAgADwAPgAgAGwAZQBuAF8AYgAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABTAEkARwBOACgAbABlAG4AXwBhACAALQAgAGwAZQBuAF8AYgApACAAKgAgAHMAaQBnAG4AXwBhACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAAXAAiAEEARABEAFwAIgAgAGMAbwBuAHQAZQB4AHQAIABtAGEAeABpAG0AaQB6AGUAcwAgAGwAaQBtAGIAIABzAGkAegBlACAAdwBoAGkAbABlACAAcAByAGUAdgBlAG4AdABpAG4AZwAgAG8AdgBlAHIAZgBsAG8AdwAuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGsALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFMAYQBmAGUASwAoAFwAIgBBAEQARABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGEALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFMAcABsAGkAdAAoAEIAaQBnAEkAbgB0AC4AQQBiAHMAKABzAHQAcgBfAG4AbwByAG0AXwBhACkALAAgAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGIALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFMAcABsAGkAdAAoAEIAaQBnAEkAbgB0AC4AQQBiAHMAKABzAHQAcgBfAG4AbwByAG0AXwBiACkALAAgAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAG0AYQBnAG4AaQB0AHUAZABlAF8AYwBvAG0AcABhAHIAaQBzAG8AbgAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBDAG8AbQBwAGEAcgBlACgAbABpAG0AYgBzAF8AYQAsACAAbABpAG0AYgBzAF8AYgApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAG0AYQBnAG4AaQB0AHUAZABlAF8AYwBvAG0AcABhAHIAaQBzAG8AbgAgACoAIABzAGkAZwBuAF8AYQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAvACAAIAAgACAAIAAgACAAIAAgACAALQAgAEEAZABkAGkAdABpAG8AbgAgACYAIABTAHUAYgB0AHIAYQBjAHQAaQBvAG4AIAAtACAAIAAgACAAIAAgACAAXABcAFwAXABcAG4AXABuAC8AKgAqAFwAbgAgACoAIABSAGUAdAB1AHIAbgBzACAAdABoAGUAIABzAHUAbQAgAG8AZgAgAHQAdwBvACAAQgBpAGcASQBuAHQAIABzAHQAcgBpAG4AZwBzAC4AXABuACAAKgAgAFsAaQBuAHAAdQB0AF8AYQA6ACAAVABlAHgAdAAsACAAaQBuAHAAdQB0AF8AYgA6ACAAVABlAHgAdABdAFwAbgAgACoALwBcAG4AQQBkAGQAIAA9ACAATABBAE0AQgBEAEEAKABpAG4AcAB1AHQAXwBhACwAIABpAG4AcAB1AHQAXwBiACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAHMAdAByAF8AbgBvAHIAbQBfAGEALAAgAE4AbwByAG0AKABpAG4AcAB1AHQAXwBhACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAdAByAF8AbgBvAHIAbQBfAGIALAAgAE4AbwByAG0AKABpAG4AcAB1AHQAXwBiACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAaQBnAG4AXwBhACwAIABCAGkAZwBpAG4AdAAuAFMAaQBnAG4AKABzAHQAcgBfAG4AbwByAG0AXwBhACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAaQBnAG4AXwBiACwAIABCAGkAZwBJAG4AdAAuAFMAaQBnAG4AKABzAHQAcgBfAG4AbwByAG0AXwBiACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIABrACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBTAGEAZgBlAEsAKABcACIAQQBEAEQAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGEALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFMAcABsAGkAdAAoAEIAaQBnAEkAbgB0AC4AQQBiAHMAKABzAHQAcgBfAG4AbwByAG0AXwBhACkALAAgAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYgAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwBwAGwAaQB0ACgAQgBpAGcASQBuAHQALgBBAGIAcwAoAHMAdAByAF8AbgBvAHIAbQBfAGIAKQAsACAAawApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAALwAvACAAQQBkAGQAUwB1AGIAUgBvAHUAdABlAHIAIAByAGUAcwBvAGwAdgBlAHMAIABzAGkAZwBuACAAbABvAGcAaQBjACAAYQBuAGQAIAByAGUAdAB1AHIAbgBzACAAYQAgAHAAYQBjAGsAZQBkACAAYQByAHIAYQB5ACAAWwBsAGkAbQBiAHMAOwAgAHMAaQBnAG4AXQBcAG4AIAAgACAAIAAgACAAIAAgAHAAYQBjAGsAZQBkAF8AcgBlAHMAdQBsAHQALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAEEAZABkAFMAdQBiAFIAbwB1AHQAZQByACgAbABpAG0AYgBzAF8AYQAsACAAbABpAG0AYgBzAF8AYgAsACAAcwBpAGcAbgBfAGEALAAgAHMAaQBnAG4AXwBiACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgAGYAaQBuAGEAbABfAHMAaQBnAG4ALAAgAEMASABPAE8AUwBFAFIATwBXAFMAKABwAGEAYwBrAGUAZABfAHIAZQBzAHUAbAB0ACwAIAAtADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAG4AYQBsAF8AbABpAG0AYgBzACwAIABEAFIATwBQACgAcABhAGMAawBlAGQAXwByAGUAcwB1AGwAdAAsACAALQAxACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIABzAHQAcgBfAG0AZQByAGcAZQBkACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBNAGUAcgBnAGUAKABmAGkAbgBhAGwAXwBsAGkAbQBiAHMALAAgAGsAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAGYAaQBuAGEAbABfAHMAaQBnAG4AIAA9ACAALQAxACwAIABcACIALQBcACIAIAAmACAAcwB0AHIAXwBtAGUAcgBnAGUAZAAsACAAcwB0AHIAXwBtAGUAcgBnAGUAZAApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABSAGUAdAB1AHIAbgBzACAAdABoAGUAIABkAGkAZgBmAGUAcgBlAG4AYwBlACAAbwBmACAAdAB3AG8AIABCAGkAZwBJAG4AdAAgAHMAdAByAGkAbgBnAHMAIAAoAEEAIAAtACAAQgApAC4AXABuACAAKgAgAFsAaQBuAHAAdQB0AF8AYQA6ACAAVABlAHgAdAAsACAAaQBuAHAAdQB0AF8AYgA6ACAAVABlAHgAdABdAFwAbgAgACoALwBcAG4AUwB1AGIAIAA9ACAATABBAE0AQgBEAEEAKABpAG4AcAB1AHQAXwBhACwAIABpAG4AcAB1AHQAXwBiACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAHMAdAByAF8AbgBvAHIAbQBfAGIALAAgAE4AbwByAG0AKABpAG4AcAB1AHQAXwBiACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABBAGQAZABpAHQAaQBvAG4AIABvAHIAYwBoAGUAcwB0AHIAYQB0AGUAcwA7ACAAcwB1AGIAdAByAGEAYwB0AGkAbwBuACAAagB1AHMAdAAgAGkAbgB2AGUAcgB0AHMAIAB0AGgAZQAgAHMAdQBiAHQAcgBhAGgAZQBuAGQAIABmAG8AcgAgAGEAZABkAGkAdABpAG8AbgAuAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AHIAXwBpAG4AdgBlAHIAcwBlAF8AYgAsACAASQBGACgAcwB0AHIAXwBuAG8AcgBtAF8AYgAgAD0AIABcACIAMABcACIALAAgAFwAIgAwAFwAIgAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABMAEUARgBUACgAcwB0AHIAXwBuAG8AcgBtAF8AYgApACAAPQAgAFwAIgAtAFwAIgAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAE0ASQBEACgAcwB0AHIAXwBuAG8AcgBtAF8AYgAsACAAMgAsACAATABFAE4AKABzAHQAcgBfAG4AbwByAG0AXwBiACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAtAFwAIgAgACYAIABzAHQAcgBfAG4AbwByAG0AXwBiAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAEEAZABkACgAaQBuAHAAdQB0AF8AYQAsACAAcwB0AHIAXwBpAG4AdgBlAHIAcwBlAF8AYgApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABTAHUAbQBzACAAYQAgAHIAYQBuAGcAZQAgAG8AcgAgAGEAcgByAGEAeQAgAG8AZgAgAEIAaQBnAEkAbgB0ACAAcwB0AHIAaQBuAGcAcwAuAFwAbgAgACoAIABbAGkAbgBwAHUAdABfAHIAYQBuAGcAZQA6ACAAUgBhAG4AZwBlAC8AQQByAHIAYQB5AF0AXABuACAAKgAvAFwAbgBTAHUAbQAgAD0AIABMAEEATQBCAEQAQQAoAGkAbgBwAHUAdABfAHIAYQBuAGcAZQAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABUAE8AUgBPAFcAIABlAG4AcwB1AHIAZQBzACAAaQBuAHAAdQB0ACAAaQBzACAAaABvAHIAaQB6AG8AbgB0AGEAbAAgAGYAbwByACAAdABoAGUAIABzAHUAYgBzAGUAcQB1AGUAbgB0ACAAUwBwAGwAaQB0ACAAYgByAG8AYQBkAGMAYQBzAHQALgBcAG4AIAAgACAAIAAgACAAIAAgAGYAbABhAHQAdABlAG4AZQBkAF8AaQBuAHAAdQB0ACwAIABUAE8AUgBPAFcAKABpAG4AcAB1AHQAXwByAGEAbgBnAGUALAAgADEAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAE8AUgAoAEkAUwBFAFIAUgBPAFIAKABmAGwAYQB0AHQAZQBuAGUAZABfAGkAbgBwAHUAdAApACwAIABDAE8ATABVAE0ATgBTACgAZgBsAGEAdAB0AGUAbgBlAGQAXwBpAG4AcAB1AHQAKQAgAD0AIAAwACkALAAgAFwAIgAwAFwAIgAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHMAdAByAF8AbgBvAHIAbQBzACwAIABNAEEAUAAoAGYAbABhAHQAdABlAG4AZQBkAF8AaQBuAHAAdQB0ACwAIABMAEEATQBCAEQAQQAoAHgALAAgAE4AbwByAG0AKAB4ACkAKQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAYQByAHIAXwBzAGkAZwBuAHMALAAgAE0AQQBQACgATABFAEYAVAAoAHMAdAByAF8AbgBvAHIAbQBzACkALAAgAEwAQQBNAEIARABBACgAeAAsACAASQBGACgAeAAgAD0AIABcACIAMABcACIALAAgADAALAAgAGkAZgAoAHgAIAA9ACAAXAAiAC0AXAAiACwAIAAtADEALAAgADEAKQApACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHMAdAByAF8AYQBiAHMALAAgAE0AQQBQACgAcwB0AHIAXwBuAG8AcgBtAHMALAAgAGEAcgByAF8AcwBpAGcAbgBzACwAIABMAEEATQBCAEQAQQAoAHgALAAgAHMAaQBnAG4ALAAgAEkARgAoAHMAaQBnAG4AIAA9ACAALQAxACwAIABNAEkARAAoAHgALAAgADIALAAgAEwARQBOACgAeAApAC0AMQApACwAIAB4ACkAKQApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHMAdAByAF8AcABvAHMALAAgAEYASQBMAFQARQBSACgAcwB0AHIAXwBhAGIAcwAsACAAYQByAHIAXwBzAGkAZwBuAHMAIAA9ACAAMQAsACAAewBcACIAMABcACIAfQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcwB0AHIAXwBuAGUAZwBzACwAIABGAEkATABUAEUAUgAoAHMAdAByAF8AYQBiAHMALAAgAGEAcgByAF8AcwBpAGcAbgBzACAAPQAgAC0AMQAsACAAewBcACIAMABcACIAfQApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHUAbgBpAGYAaQBlAGQAXwBrACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBTAGEAZgBlAEsAKABcACIAQQBEAEQAXAAiACwAIABDAE8ATABVAE0ATgBTACgAZgBsAGEAdAB0AGUAbgBlAGQAXwBpAG4AcAB1AHQAKQApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAHAAbwBzAF8AcwB1AG0ALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFUATQBhAHQAcgBpAHgAUwB1AG0AKABzAHQAcgBfAHAAbwBzACwAIAB1AG4AaQBmAGkAZQBkAF8AawApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AbgBlAGcAXwBzAHUAbQAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBNAGEAdAByAGkAeABTAHUAbQAoAHMAdAByAF8AbgBlAGcAcwAsACAAdQBuAGkAZgBpAGUAZABfAGsAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABwAGEAYwBrAGUAZABfAHIAZQBzAHUAbAB0ACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBBAGQAZABTAHUAYgBSAG8AdQB0AGUAcgAoAGwAaQBtAGIAcwBfAHAAbwBzAF8AcwB1AG0ALAAgAGwAaQBtAGIAcwBfAG4AZQBnAF8AcwB1AG0ALAAgADEALAAgAC0AMQAsACAAdQBuAGkAZgBpAGUAZABfAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGYAaQBuAGEAbABfAHMAaQBnAG4ALAAgAEMASABPAE8AUwBFAFIATwBXAFMAKABwAGEAYwBrAGUAZABfAHIAZQBzAHUAbAB0ACwAIAAtADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGYAaQBuAGEAbABfAGwAaQBtAGIAcwAsACAARABSAE8AUAAoAHAAYQBjAGsAZQBkAF8AcgBlAHMAdQBsAHQALAAgAC0AMQApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHMAdAByAF8AbQBlAHIAZwBlAGQALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAE0AZQByAGcAZQAoAGYAaQBuAGEAbABfAGwAaQBtAGIAcwAsACAAdQBuAGkAZgBpAGUAZABfAGsAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABmAGkAbgBhAGwAXwBzAGkAZwBuACAAPQAgAC0AMQAsACAAXAAiAC0AXAAiACAAJgAgAHMAdAByAF8AbQBlAHIAZwBlAGQALAAgAHMAdAByAF8AbQBlAHIAZwBlAGQAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFIAZQB0AHUAcgBuAHMAIAB0AGgAZQAgAHAAcgBvAGQAdQBjAHQAIABvAGYAIAB0AHcAbwAgAEIAaQBnAEkAbgB0ACAAcwB0AHIAaQBuAGcAcwAuAFwAbgAgACoAIABbAGkAbgBwAHUAdABfAGEAOgAgAFQAZQB4AHQALAAgAGkAbgBwAHUAdABfAGIAOgAgAFQAZQB4AHQAXQBcAG4AIAAqAC8AXABuAE0AdQBsACAAPQAgAEwAQQBNAEIARABBACgAaQBuAHAAdQB0AF8AYQAsACAAaQBuAHAAdQB0AF8AYgAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABzAHQAcgBfAG4AbwByAG0AXwBhACwAIABOAG8AcgBtACgAaQBuAHAAdQB0AF8AYQApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAcgBfAG4AbwByAG0AXwBiACwAIABOAG8AcgBtACgAaQBuAHAAdQB0AF8AYgApACwAXABuACAAIAAgACAAIAAgACAAIABzAGkAZwBuAF8AYQAsACAAQgBpAGcASQBuAHQALgBTAGkAZwBuACgAcwB0AHIAXwBuAG8AcgBtAF8AYQApACwAXABuACAAIAAgACAAIAAgACAAIABzAGkAZwBuAF8AYgAsACAAQgBpAGcASQBuAHQALgBTAGkAZwBuACgAcwB0AHIAXwBuAG8AcgBtAF8AYgApACwAXABuACAAIAAgACAAIAAgACAAIABsAGUAbgBfAGEALAAgAEwARQBOACgAcwB0AHIAXwBuAG8AcgBtAF8AYQApACAALQAgAEkARgAoAHMAaQBnAG4AXwBhACAAPQAgAC0AMQAsACAAMQAsACAAMAApACwAXABuACAAIAAgACAAIAAgACAAIABsAGUAbgBfAGIALAAgAEwARQBOACgAcwB0AHIAXwBuAG8AcgBtAF8AYgApACAALQAgAEkARgAoAHMAaQBnAG4AXwBiACAAPQAgAC0AMQAsACAAMQAsACAAMAApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAALwAvACAAUAByAG8AZAB1AGMAdAAgAG8AZgAgAHcAaQB0AGgAIAAwACAAaQBzACAAMABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAE8AUgAoAHMAaQBnAG4AXwBhACAAPQAgADAALAAgAHMAaQBnAG4AXwBiACAAPQAgADAAKQAsACAAXAAiADAAXAAiACwAXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABUAHIAYQBwACAAcwB0AHIAaQBuAGcAIABvAHYAZQByAGYAbABvAHcAcwAgAGIAZQBmAG8AcgBlACAAZQBuAHQAZQByAGkAbgBnACAAdABoAGUAIABjAG8AbgB2AG8AbAB1AHQAaQBvAG4AIABlAG4AZwBpAG4AZQAuAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAbABlAG4AXwBhACAAKwAgAGwAZQBuAF8AYgAgAD4AIAAzADIANwA2ADYALAAgACMATgBVAE0AIQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGsALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFMAYQBmAGUASwAoAFwAIgBNAFUATABcACIALAAgAE0ASQBOACgAbABlAG4AXwBhACwAIABsAGUAbgBfAGIAKQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYQAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwBwAGwAaQB0ACgAQgBpAGcASQBuAHQALgBBAGIAcwAoAHMAdAByAF8AbgBvAHIAbQBfAGEAKQAsACAAawApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYgAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwBwAGwAaQB0ACgAQgBpAGcASQBuAHQALgBBAGIAcwAoAHMAdAByAF8AbgBvAHIAbQBfAGIAKQAsACAAawApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGYAaQBuAGEAbABfAGwAaQBtAGIAcwAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBNAHUAbAAoAGwAaQBtAGIAcwBfAGEALAAgAGwAaQBtAGIAcwBfAGIALAAgAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGYAaQBuAGEAbABfAHMAaQBnAG4ALAAgAHMAaQBnAG4AXwBhACAAKgAgAHMAaQBnAG4AXwBiACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHMAdAByAF8AbQBlAHIAZwBlAGQALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAE0AZQByAGcAZQAoAGYAaQBuAGEAbABfAGwAaQBtAGIAcwAsACAAawApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEkARgAoAGYAaQBuAGEAbABfAHMAaQBnAG4AIAA9ACAALQAxACwAIABcACIALQBcACIAIAAmACAAcwB0AHIAXwBtAGUAcgBnAGUAZAAsACAAcwB0AHIAXwBtAGUAcgBnAGUAZAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABbAFYATwBMAEEAVABJAEwARQBdACAARwBlAG4AZQByAGEAdABlAHMAIABhACAAZAB5AG4AYQBtAGkAYwAgAGEAcgByAGEAeQAgAG8AZgAgAHIAYQBuAGQAbwBtACAAQgBpAGcASQBuAHQAIABzAHQAcgBpAG4AZwBzAC4AXABuACAAKgAgAFsAbgB1AG0AXwByAG8AdwBzADoAIABpAG4AdAAsACAAbgB1AG0AXwBjAG8AbABzADoAIABpAG4AdAAsACAAbQBpAG4AXwBkAGkAZwBpAHQAcwA6ACAAaQBuAHQALAAgAG0AYQB4AF8AZABpAGcAaQB0AHMAOgAgAGkAbgB0AF0AXABuACAAKgAvAFwAbgBSAGEAbgBkAEEAcgByAGEAeQAgAD0AIABMAEEATQBCAEQAQQAoAFsAbgB1AG0AXwByAG8AdwBzAF0ALAAgAFsAbgB1AG0AXwBjAG8AbABzAF0ALAAgAFsAbQBpAG4AXwBkAGkAZwBpAHQAcwBdACwAIABbAG0AYQB4AF8AZABpAGcAaQB0AHMAXQAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABuAF8AcgBvAHcAcwAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABuAHUAbQBfAHIAbwB3AHMAKQAsACAAMQAsACAAbgB1AG0AXwByAG8AdwBzACkALABcAG4AIAAgACAAIAAgACAAIAAgAG4AXwBjAG8AbABzACwAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAG4AdQBtAF8AYwBvAGwAcwApACwAIAAxACwAIABuAHUAbQBfAGMAbwBsAHMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbQBpAG4AXwBsAGUAbgAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABtAGkAbgBfAGQAaQBnAGkAdABzACkALAAgADEANgAsACAATQBJAE4AKAAzADIANwA2ADcALAAgAE0AQQBYACgAMQAsACAAbQBpAG4AXwBkAGkAZwBpAHQAcwApACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHgAXwBsAGUAbgAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABtAGEAeABfAGQAaQBnAGkAdABzACkALAAgADUAMAAsACAATQBBAFgAKAAxACwAIABNAEkATgAoADMAMgA3ADYANgAsACAAbQBhAHgAXwBkAGkAZwBpAHQAcwApACkAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAE0AQQBQACgAUgBBAE4ARABBAFIAUgBBAFkAKABuAF8AcgBvAHcAcwAsACAAbgBfAGMAbwBsAHMALAAgAG0AaQBuAF8AbABlAG4ALAAgAG0AYQB4AF8AbABlAG4ALAAgAFQAUgBVAEUAKQAsACAATABBAE0AQgBEAEEAKABsAGUAbgBnAHQAaAAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHMAaQBnAG4AXwBwAHIAZQBmAGkAeAAsACAAQwBIAE8ATwBTAEUAKABSAEEATgBEAEIARQBUAFcARQBFAE4AKAAxACwAIAAyACkALAAgAFwAIgBcACIALAAgAFwAIgAtAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcgBhAG4AZABfAGQAaQBnAGkAdABzACwAIABDAE8ATgBDAEEAVAAoAFIAQQBOAEQAQQBSAFIAQQBZACgAMQAsACAAbABlAG4AZwB0AGgALAAgADAALAAgADkALAAgAFQAUgBVAEUAKQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcwBpAGcAbgBfAHAAcgBlAGYAaQB4ACAAJgAgAFIARQBHAEUAWABSAEUAUABMAEEAQwBFACgAcgBhAG4AZABfAGQAaQBnAGkAdABzACwAIABcACIAXgAwACoAXAAiACwAIABcACIAXAAiACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAApACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFIAZQB0AHUAcgBuAHMAIAAyAC0AcgBvAHcAIABhAHIAcgBhAHkAOgAgAFsAUQB1AG8AdABpAGUAbgB0ADsAIABSAGUAbQBhAGkAbgBkAGUAcgBdAC4AIABTAHUAcABwAG8AcgB0AHMAIABUAHIAdQBuAGMAYQB0AGUAZAAgAG8AcgAgAEYAbABvAG8AcgAgAGQAaQB2AGkAcwBpAG8AbgAuAFwAbgAgACoAIABbAGkAbgBwAHUAdABfAGEAOgAgAFQAZQB4AHQALAAgAGkAbgBwAHUAdABfAGIAOgAgAFQAZQB4AHQALAAgAHUAcwBlAF8AZgBsAG8AbwByADoAIABCAG8AbwBsAF0AXABuACAAKgAvAFwAbgBEAGkAdgBNAG8AZAAgAD0AIABMAEEATQBCAEQAQQAoAGkAbgBwAHUAdABfAGEALAAgAGkAbgBwAHUAdABfAGIALAAgAFsAdQBzAGUAXwBmAGwAbwBvAHIAXQAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABzAHQAcgBfAG4AbwByAG0AXwBhACwAIABOAG8AcgBtACgAaQBuAHAAdQB0AF8AYQApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAcgBfAG4AbwByAG0AXwBiACwAIABOAG8AcgBtACgAaQBuAHAAdQB0AF8AYgApACwAXABuACAAIAAgACAAIAAgACAAIABzAGkAZwBuAF8AYQAsACAAQgBpAGcASQBuAHQALgBTAGkAZwBuACgAcwB0AHIAXwBuAG8AcgBtAF8AYQApACwAXABuACAAIAAgACAAIAAgACAAIABzAGkAZwBuAF8AYgAsACAAQgBpAGcASQBuAHQALgBTAGkAZwBuACgAcwB0AHIAXwBuAG8AcgBtAF8AYgApACwAXABuACAAIAAgACAAIAAgACAAIABpAHMAXwBmAGwAbwBvAHIAXwBkAGkAdgAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKAB1AHMAZQBfAGYAbABvAG8AcgApACwAIABGAEEATABTAEUALAAgAHUAcwBlAF8AZgBsAG8AbwByACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIABJAEYAKABzAGkAZwBuAF8AYgAgAD0AIAAwACwAIAAjAEQASQBWAC8AMAAhACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABzAGkAZwBuAF8AYQAgAD0AIAAwACwAIAB7AFwAIgAwAFwAIgA7AFwAIgAwAFwAIgB9ACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAawAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwBhAGYAZQBLACgAXAAiAEQASQBWAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYQAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwBwAGwAaQB0ACgAQgBpAGcASQBuAHQALgBBAGIAcwAoAHMAdAByAF8AbgBvAHIAbQBfAGEAKQAsACAAawApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AYgAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwBwAGwAaQB0ACgAQgBpAGcASQBuAHQALgBBAGIAcwAoAHMAdAByAF8AbgBvAHIAbQBfAGIAKQAsACAAawApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHAAYQBjAGsAZQBkAF8AcgBlAHMAdQBsAHQALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAEQAaQB2AFIAbwB1AHQAZQByACgAbABpAG0AYgBzAF8AYQAsACAAbABpAG0AYgBzAF8AYgAsACAAawApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAZQBuAF8AcgBlAG0AYQBpAG4AZABlAHIALAAgAEkATgBEAEUAWAAoAHAAYQBjAGsAZQBkAF8AcgBlAHMAdQBsAHQALAAgADEALAAgADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAHIAZQBtAGEAaQBuAGQAZQByACwAIABDAEgATwBPAFMARQBSAE8AVwBTACgAcABhAGMAawBlAGQAXwByAGUAcwB1AGwAdAAsACAAUwBFAFEAVQBFAE4AQwBFACgAbABlAG4AXwByAGUAbQBhAGkAbgBkAGUAcgAsACAAMQAsACAAMgApACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABsAGkAbQBiAHMAXwBxAHUAbwB0AGkAZQBuAHQALAAgAEQAUgBPAFAAKABwAGEAYwBrAGUAZABfAHIAZQBzAHUAbAB0ACwAIABsAGUAbgBfAHIAZQBtAGEAaQBuAGQAZQByACAAKwAgADEAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABmAGkAbgBhAGwAXwBzAGkAZwBuACwAIABzAGkAZwBuAF8AYQAgACoAIABzAGkAZwBuAF8AYgAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHMAdAByAF8AbQBlAHIAZwBlAGQAXwBxACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBNAGUAcgBnAGUAKABsAGkAbQBiAHMAXwBxAHUAbwB0AGkAZQBuAHQALAAgAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHMAdAByAF8AbQBlAHIAZwBlAGQAXwByACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBNAGUAcgBnAGUAKABsAGkAbQBiAHMAXwByAGUAbQBhAGkAbgBkAGUAcgAsACAAawApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHMAdAByAF8AdAByAHUAbgBjAF8AcQAsACAASQBGACgAQQBOAEQAKABmAGkAbgBhAGwAXwBzAGkAZwBuACAAPQAgAC0AMQAsACAAcwB0AHIAXwBtAGUAcgBnAGUAZABfAHEAIAA8AD4AIABcACIAMABcACIAKQAgACwAIABcACIALQBcACIAIAAmACAAcwB0AHIAXwBtAGUAcgBnAGUAZABfAHEALAAgAHMAdAByAF8AbQBlAHIAZwBlAGQAXwBxACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABzAHQAcgBfAHQAcgB1AG4AYwBfAHIALAAgAEkARgAoAGEAbgBkACgAcwBpAGcAbgBfAGEAIAA9ACAALQAxACwAIABzAHQAcgBfAG0AZQByAGcAZQBkAF8AcgAgADwAPgAgAFwAIgAwAFwAIgApACwAIABcACIALQBcACIAIAAmACAAcwB0AHIAXwBtAGUAcgBnAGUAZABfAHIALAAgAHMAdAByAF8AbQBlAHIAZwBlAGQAXwByACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAAUAB5AHQAaABvAG4ALQBzAHQAeQBsAGUAIABmAGwAbwBvAHIAIABkAGkAdgBpAHMAaQBvAG4AIAByAGUAcQB1AGkAcgBlAHMAIABhACAAYwBvAHIAcgBlAGMAdABpAG8AbgAgAHMAdABlAHAAIAB3AGgAZQBuACAAcwBpAGcAbgBzACAAYQByAGUAIABtAGkAeABlAGQAIABhAG4AZAAgAHIAZQBtAGEAaQBuAGQAZQByACAAaQBzACAAbgBvAG4ALQB6AGUAcgBvAC4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbgBlAGUAZABzAF8AZgBsAG8AbwByAF8AYwBvAHIAcgBlAGMAdABpAG8AbgAsACAAQQBOAEQAKABpAHMAXwBmAGwAbwBvAHIAXwBkAGkAdgAsACAAZgBpAG4AYQBsAF8AcwBpAGcAbgAgAD0AIAAtADEALAAgAHMAdAByAF8AbQBlAHIAZwBlAGQAXwByACAAPAA+ACAAXAAiADAAXAAiACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcwB0AHIAXwBmAGkAbgBhAGwAXwBxACwAIABJAEYAKABuAGUAZQBkAHMAXwBmAGwAbwBvAHIAXwBjAG8AcgByAGUAYwB0AGkAbwBuACwAIABTAHUAYgAoAHMAdAByAF8AdAByAHUAbgBjAF8AcQAsACAAXAAiADEAXAAiACkALAAgAHMAdAByAF8AdAByAHUAbgBjAF8AcQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcwB0AHIAXwBmAGkAbgBhAGwAXwByACwAIABJAEYAKABuAGUAZQBkAHMAXwBmAGwAbwBvAHIAXwBjAG8AcgByAGUAYwB0AGkAbwBuACwAIABBAGQAZAAoAHMAdAByAF8AdAByAHUAbgBjAF8AcgAsACAAcwB0AHIAXwBuAG8AcgBtAF8AYgApACwAIABzAHQAcgBfAHQAcgB1AG4AYwBfAHIAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABWAFMAVABBAEMASwAoAHMAdAByAF8AZgBpAG4AYQBsAF8AcQAsACAAcwB0AHIAXwBmAGkAbgBhAGwAXwByACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAApACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFIAZQB0AHUAcgBuAHMAIAB0AGgAZQAgAHEAdQBvAHQAaQBlAG4AdAAgAG8AZgAgAEEAIAAvACAAQgAuACAARABlAGYAYQB1AGwAdABzACAAdABvACAAVAByAHUAbgBjAGEAdABlAGQAIABkAGkAdgBpAHMAaQBvAG4ALgBcAG4AIAAqACAAWwBpAG4AcAB1AHQAXwBhADoAIABUAGUAeAB0ACwAIABpAG4AcAB1AHQAXwBiADoAIABUAGUAeAB0ACwAIAB1AHMAZQBfAGYAbABvAG8AcgA6ACAAQgBvAG8AbABdAFwAbgAgACoALwBcAG4ARABpAHYAIAA9ACAATABBAE0AQgBEAEEAKABpAG4AcAB1AHQAXwBhACwAIABpAG4AcAB1AHQAXwBiACwAIABbAHUAcwBlAF8AZgBsAG8AbwByAF0ALABcAG4AIAAgACAAIABJAE4ARABFAFgAKABEAGkAdgBNAG8AZAAoAGkAbgBwAHUAdABfAGEALAAgAGkAbgBwAHUAdABfAGIALAAgAHUAcwBlAF8AZgBsAG8AbwByACkALAAgADEALAAgADEAKQBcAG4AKQA7AFwAbgBcAG4ALwAqACoAXABuACAAKgAgAFIAZQB0AHUAcgBuAHMAIAB0AGgAZQAgAHIAZQBtAGEAaQBuAGQAZQByACAAbwBmACAAQQAgAC8AIABCAC4AIABEAGUAZgBhAHUAbAB0AHMAIAB0AG8AIABUAHIAdQBuAGMAYQB0AGUAZAAgAGQAaQB2AGkAcwBpAG8AbgAuAFwAbgAgACoAIABbAGkAbgBwAHUAdABfAGEAOgAgAFQAZQB4AHQALAAgAGkAbgBwAHUAdABfAGIAOgAgAFQAZQB4AHQALAAgAHUAcwBlAF8AZgBsAG8AbwByADoAIABCAG8AbwBsAF0AXABuACAAKgAvAFwAbgBNAG8AZAAgAD0AIABMAEEATQBCAEQAQQAoAGkAbgBwAHUAdABfAGEALAAgAGkAbgBwAHUAdABfAGIALAAgAFsAdQBzAGUAXwBmAGwAbwBvAHIAXQAsAFwAbgAgACAAIAAgAEkATgBEAEUAWAAoAEQAaQB2AE0AbwBkACgAaQBuAHAAdQB0AF8AYQAsACAAaQBuAHAAdQB0AF8AYgAsACAAdQBzAGUAXwBmAGwAbwBvAHIAKQAsACAAMgAsACAAMQApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAAUgBlAHQAdQByAG4AcwAgAGIAYQBzAGUAIAByAGEAaQBzAGUAZAAgAHQAbwAgAHQAaABlACAAcABvAHcAZQByACAAbwBmACAAZQB4AHAAbwBuAGUAbgB0AC4AXABuACAAKgAgAFsAYgBhAHMAZQA6ACAAVABlAHgAdAAsACAAZQB4AHAAbwBuAGUAbgB0ADoAIABUAGUAeAB0AF0AXABuACAAKgAvAFwAbgBQAG8AdwAgAD0AIABMAEEATQBCAEQAQQAoAGIAYQBzAGUALAAgAGUAeABwAG8AbgBlAG4AdAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABzAHQAcgBfAG4AbwByAG0AXwBiAGEAcwBlACwAIABOAG8AcgBtACgAYgBhAHMAZQApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAcgBfAG4AbwByAG0AXwBlAHgAcAAsACAATgBvAHIAbQAoAGUAeABwAG8AbgBlAG4AdAApACwAXABuACAAIAAgACAAIAAgACAAIABzAGkAZwBuAF8AYgBhAHMAZQAsACAAQgBpAGcASQBuAHQALgBTAGkAZwBuACgAcwB0AHIAXwBuAG8AcgBtAF8AYgBhAHMAZQApACwAXABuACAAIAAgACAAIAAgACAAIABzAGkAZwBuAF8AZQB4AHAALAAgAEIAaQBnAEkAbgB0AC4AUwBpAGcAbgAoAHMAdAByAF8AbgBvAHIAbQBfAGUAeABwACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIABzAHQAcgBfAGEAYgBzAF8AYgBhAHMAZQAsACAAQgBpAGcASQBuAHQALgBBAGIAcwAoAHMAdAByAF8AbgBvAHIAbQBfAGIAYQBzAGUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AHIAXwBhAGIAcwBfAGUAeABwACwAIABCAGkAZwBJAG4AdAAuAEEAYgBzACgAcwB0AHIAXwBuAG8AcgBtAF8AZQB4AHAAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAGkAcwBfAGUAeABwAF8AZQB2AGUAbgAsACAASQBTAEUAVgBFAE4AKABWAEEATABVAEUAKABSAEkARwBIAFQAKABzAHQAcgBfAG4AbwByAG0AXwBlAHgAcAAsACAAMQApACkAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAG4AYQBsAF8AcwBpAGcAbgAsACAASQBGACgAcwBpAGcAbgBfAGIAYQBzAGUAIAA9ACAALQAxACwAIABJAEYAKABpAHMAXwBlAHgAcABfAGUAdgBlAG4ALAAgADEALAAgAC0AMQApACwAIABzAGkAZwBuAF8AYgBhAHMAZQApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAALwAvACAATQBhAHQAaABlAG0AYQB0AGkAYwBhAGwAIABpAGQAZQBuAHQAaQB0AGkAZQBzACAAYQBuAGQAIABmAGwAbwBvAHIALQBpAG4AdABlAGcAZQByACAAYgBvAHUAbgBkAGEAcgB5ACAAYwBvAG4AZABpAHQAaQBvAG4AcwAuAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAcwB0AHIAXwBhAGIAcwBfAGIAYQBzAGUAIAA9ACAAXAAiADAAXAAiACwAIABJAEYAKABzAHQAcgBfAG4AbwByAG0AXwBlAHgAcAAgAD0AIABcACIAMABcACIALAAgACMATgBVAE0AIQAsACAAXAAiADAAXAAiACkALAAgAC8ALwAgADAAXgAwACAAaQBzACAAdQBuAGQAZQBmAGkAbgBlAGQAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABzAHQAcgBfAGEAYgBzAF8AYgBhAHMAZQAgAD0AIABcACIAMQBcACIALAAgAEkARgAoAGYAaQBuAGEAbABfAHMAaQBnAG4AIAA9ACAALQAxACwAIABcACIALQAxAFwAIgAsACAAXAAiADEAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAHMAaQBnAG4AXwBlAHgAcAAgAD0AIAAtADEALAAgAFwAIgAwAFwAIgAsACAALwAvACAASQBuAHQAZQBnAGUAcgAgAHQAcgB1AG4AYwBhAHQAaQBvAG4AOgAgAG4AZQBnAGEAdABpAHYAZQAgAGUAeABwAG8AbgBlAG4AdABzACAAeQBpAGUAbABkACAAMAAgAGYAbwByACAAYgBhAHMAZQBzACAAPgA9ACAAMgBcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAHMAdAByAF8AbgBvAHIAbQBfAGUAeABwACAAPQAgAFwAIgAwAFwAIgAsACAAXAAiADEAXAAiACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAALwAvACAAVAByAGEAcAAgAGUAeABwAG8AbgBlAG4AdABzACAAdABoAGEAdAAgAGEAcgBlACAAZwB1AGEAcgBhAG4AdABlAGUAZAAgAHQAbwAgAGUAeABjAGUAZQBkACAARQB4AGMAZQBsACcAcwAgAHMAdAByAGkAbgBnACAAbABpAG0AaQB0AHMALgBcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAEwARQBOACgAcwB0AHIAXwBuAG8AcgBtAF8AZQB4AHAAKQAgAD4AIAA2ACwAIAAjAE4AVQBNACEALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABuAHUAbQBfAGUAeABwACwAIABWAEEATABVAEUAKABzAHQAcgBfAG4AbwByAG0AXwBlAHgAcAApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAC8ALwAgAEQAZQB0AGUAcgBtAGkAbgBlACAAaQBmACAAdABoAGkAcwAgAGMAYQBsAGMAdQBsAGEAdABpAG8AbgAgAHcAaQBsAGwAIABlAHgAYwBlAGUAZAAgAEUAeABjAGUAbAAnAHMAIABzAHQAcgBpAG4AZwAgAGwAaQBtAGkAdABzAC4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAYgBhAHMAZQBfAGwAbwBnADEAMAAsACAATABPAEcAMQAwACgAVgBBAEwAVQBFACgATABFAEYAVAAoAHMAdAByAF8AYQBiAHMAXwBiAGEAcwBlACwAIAAxADQAKQApACkAIAArACAATQBBAFgAKAAwACwAIABMAEUATgAoAHMAdAByAF8AYQBiAHMAXwBiAGEAcwBlACkAIAAtACAAMQA0ACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABhAHAAcAByAG8AeABfAGQAaQBnAGkAdABzACwAIABuAHUAbQBfAGUAeABwACAAKgAgAGIAYQBzAGUAXwBsAG8AZwAxADAALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgAYQBwAHAAcgBvAHgAXwBkAGkAZwBpAHQAcwAgAD4AIAAzADIANwA2ADYALAAgACMATgBVAE0AIQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAALwAvACAARQB4AHAAbwBuAGUAbgB0AGkAYQB0AGkAbwBuACAAYwBvAG4AdABlAHgAdAAgAHUAcwBlAHMAIABhAHAAcAByAG8AeABfAGQAaQBnAGkAdABzACAALwAgADIAIABmAG8AcgAgAFMAYQBmAGUASwAgAHQAbwAgAGEAYwBjAG8AdQBuAHQAIABmAG8AcgAgAGMAbwBuAHYAbwBsAHUAdABpAG8AbgAgAG8AdgBlAHIAbABhAHAAIABpAG4AIABVAE0AdQBsAC4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGsALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFMAYQBmAGUASwAoAFwAIgBNAFUATABcACIALAAgAGEAcABwAHIAbwB4AF8AZABpAGcAaQB0AHMAIAAvACAAMgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGIAYQBzAGUALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFMAcABsAGkAdAAoAHMAdAByAF8AYQBiAHMAXwBiAGEAcwBlACwAIABrACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGYAaQBuAGEAbAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBQAG8AdwAoAGwAaQBtAGIAcwBfAGIAYQBzAGUALAAgAHMAdAByAF8AbgBvAHIAbQBfAGUAeABwACwAIABrACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcwB0AHIAXwBtAGUAcgBnAGUAZAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4ATQBlAHIAZwBlACgAbABpAG0AYgBzAF8AZgBpAG4AYQBsACwAIABrACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEkARgAoAGYAaQBuAGEAbABfAHMAaQBnAG4AIAA9ACAALQAxACwAIABcACIALQBcACIAIAAmACAAcwB0AHIAXwBtAGUAcgBnAGUAZAAsACAAcwB0AHIAXwBtAGUAcgBnAGUAZAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACAAIAAgACAAKQApACkAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAC8AKgAqAFwAbgAgACoAIABSAGUAdAB1AHIAbgBzACAAdABoAGUAIABpAG4AdABlAGcAZQByACAAcwBxAHUAYQByAGUAIAByAG8AbwB0ACAAKABmAGwAbwBvAHIAKQAgAG8AZgAgAGEAIABCAGkAZwBJAG4AdAAuAFwAbgAgACoAIABbAGkAbgBwAHUAdAA6ACAAVABlAHgAdABdAFwAbgAgACoALwBcAG4AUwBxAHIAdAAgAD0AIABMAEEATQBCAEQAQQAoAGkAbgBwAHUAdAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABzAHQAcgBfAG4AbwByAG0ALAAgAE4AbwByAG0AKABpAG4AcAB1AHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwBpAGcAbgBfAG4ALAAgAEIAaQBnAEkAbgB0AC4AUwBpAGcAbgAoAHMAdAByAF8AbgBvAHIAbQApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAcwBpAGcAbgBfAG4AIAA9ACAALQAxACwAIAAjAE4AVQBNACEALABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAHMAdAByAF8AbgBvAHIAbQAgAD0AIABcACIAMABcACIALAAgAFwAIgAwAFwAIgAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAcwB0AHIAXwBuAG8AcgBtACAAPQAgAFwAIgAxAFwAIgAsACAAXAAiADEAXAAiACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABlAG4AXwBuAG8AcgBtACwAIABMAEUATgAoAHMAdAByAF8AbgBvAHIAbQApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbgB1AG0AXwBzAGUAZQBkAF8AcAByAGUAYwBpAHMAaQBvAG4ALAAgAEkARgAoAGwAZQBuAF8AbgBvAHIAbQAgADwAPQAgADEANAAsACAAbABlAG4AXwBuAG8AcgBtACwAIABJAEYAKABJAFMARQBWAEUATgAoAGwAZQBuAF8AbgBvAHIAbQApACwAIAAxADQALAAgADEAMwApACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABzAHQAcgBfAG4AYQB0AGkAdgBlAF8AcAByAGUAYwBpAHMAaQBvAG4ALAAgAEwARQBGAFQAKABzAHQAcgBfAG4AbwByAG0ALAAgAG4AdQBtAF8AcwBlAGUAZABfAHAAcgBlAGMAaQBzAGkAbwBuACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABuAHUAbQBfAG4AYQB0AGkAdgBlAF8AcAByAGUAYwBpAHMAaQBvAG4ALAAgAFYAQQBMAFUARQAoAHMAdAByAF8AbgBhAHQAaQB2AGUAXwBwAHIAZQBjAGkAcwBpAG8AbgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbgB1AG0AXwBtAGEAZwBuAGkAdAB1AGQAZQBfAHoAZQByAG8AZQBzACwAIAAoAGwAZQBuAF8AbgBvAHIAbQAgAC0AIABuAHUAbQBfAHMAZQBlAGQAXwBwAHIAZQBjAGkAcwBpAG8AbgApACAALwAgADIALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAcwB0AHIAXwBwAHIAZQBmAGkAeAAsACAAVABFAFgAVAAoAFIATwBVAE4ARABVAFAAKABTAFEAUgBUACgAbgB1AG0AXwBuAGEAdABpAHYAZQBfAHAAcgBlAGMAaQBzAGkAbwBuACkALAAgADAAKQAgACsAIAAxACwAIABcACIAMABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAHMAdAByAF8AcwBlAGUAZAAsACAAcwB0AHIAXwBwAHIAZQBmAGkAeAAgACYAIABSAEUAUABUACgAXAAiADAAXAAiACwAIABuAHUAbQBfAG0AYQBnAG4AaQB0AHUAZABlAF8AegBlAHIAbwBlAHMAKQAsAFwAbgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAvAC8AIABTAFEAUgBUACAAcgBlAHEAdQBpAHIAZQBzACAAYQAgAGcAbABvAGIAYQBsACAAawAgAHQAbwAgAHAAcgBlAHYAZQBuAHQAIABwAHIAZQBjAGkAcwBpAG8AbgAgAGQAcgBpAGYAdAAgAGEAYwByAG8AcwBzACAAdABoAGUAIABpAHQAZQByAGEAdABpAHYAZQAgAE4AZQB3AHQAbwBuACAAcwB0AGUAcABzAC4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAawAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwBhAGYAZQBLACgAXAAiAE0AVQBMAFwAIgAsACAAbABlAG4AXwBuAG8AcgBtACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAbABpAG0AYgBzAF8AcgBhAGQAaQBjAGEAbgBkACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBTAHAAbABpAHQAKABzAHQAcgBfAG4AbwByAG0ALAAgAGsAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAHMAZQBlAGQALAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFMAcABsAGkAdAAoAHMAdAByAF8AcwBlAGUAZAAsACAAawApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGwAaQBtAGIAcwBfAGYAaQBuAGEAbAAsACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBTAHEAcgB0ACgAbABpAG0AYgBzAF8AcgBhAGQAaQBjAGEAbgBkACwAIABsAGkAbQBiAHMAXwBzAGUAZQBkACwAIABrACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4ATQBlAHIAZwBlACgAbABpAG0AYgBzAF8AZgBpAG4AYQBsACwAIABrACkAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAIAAgACAAIAApACkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAAUgBlAHQAdQByAG4AcwAgAHQAaABlACAAZgBhAGMAdABvAHIAaQBhAGwAIAAoAG4AIQApACAAdQBzAGkAbgBnACAAUAByAGkAbQBlACAAUwB3AGkAbgBnAC4AIABNAGEAeAAgAGkAbgBwAHUAdAA6ACAAOQAyADcAMwAuAFwAbgAgACoAIABbAGkAbgBwAHUAdAA6ACAAVABlAHgAdABdAFwAbgAgACoALwBcAG4ARgBhAGMAdAAgAD0AIABMAEEATQBCAEQAQQAoAGkAbgBwAHUAdAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABzAHQAcgBfAG4AbwByAG0ALAAgAE4AbwByAG0AKABpAG4AcAB1AHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwBpAGcAbgBfAG4ALAAgAEIAaQBnAEkAbgB0AC4AUwBpAGcAbgAoAHMAdAByAF8AbgBvAHIAbQApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAcwBpAGcAbgBfAG4AIAA9ACAALQAxACwAIAAjAE4AVQBNACEALABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAHMAdAByAF8AbgBvAHIAbQAgAD0AIABcACIAMABcACIALAAgAFwAIgAxAFwAIgAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAcwB0AHIAXwBuAG8AcgBtACAAPQAgAFwAIgAxAFwAIgAsACAAXAAiADEAXAAiACwAXABuACAAIAAgACAAIAAgACAAIAAvAC8AIABUAHIAYQBwACAAZgBhAGMAYwB0AG8AcgBpAGEAbABzACAAdABoAGEAdAAgAGEAcgBlACAAZwB1AGEAcgBhAG4AdABlAGUAZAAgAHQAbwAgAGUAeABjAGUAZQBkACAARQB4AGMAZQBsACcAcwAgAHMAdAByAGkAbgBnACAAbABpAG0AaQB0AHMALgBcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAEwARQBOACgAcwB0AHIAXwBuAG8AcgBtACkAIAA+ACAANAAsACAAIwBOAFUATQAhACwAXABuACAAIAAgACAAIAAgACAAIAAvAC8AIAA5ADIANwAzACEAIABpAHMAIAB0AGgAZQAgAGEAYgBzAG8AbAB1AHQAZQAgAHAAaAB5AHMAaQBjAGEAbAAgAGMAZQBpAGwAaQBuAGcAIABmAG8AcgAgAGEAIAAzADIALAA3ADYANgAgAGMAaABhAHIAYQBjAHQAZQByACAAcwB0AHIAaQBuAGcALgBcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAFYAQQBMAFUARQAoAHMAdAByAF8AbgBvAHIAbQApACAAPgAgADkAMgA3ADMALAAgACMATgBVAE0AIQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAG4AdQBtAF8AbgAsACAAVgBBAEwAVQBFACgAcwB0AHIAXwBuAG8AcgBtACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIABnAGwAbwBiAGEAbABfAHAAcgBpAG0AZQBzACwAIABjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBOAGEAdABpAHYAZQBQAHIAaQBtAGUAcwAoAG4AdQBtAF8AbgApACwAXABuAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFAAcgBpAG0AZQBTAHcAaQBuAGcASwBlAHIAbgBlAGwAKABuAHUAbQBfAG4ALAAgAGcAbABvAGIAYQBsAF8AcAByAGkAbQBlAHMAKQBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAAgACAAIAAgACkAKQApACkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAAUgBlAHQAdQByAG4AcwAgAHQAaABlACAAbQBpAG4AaQBtAHUAbQAgAEIAaQBnAEkAbgB0ACAAZgByAG8AbQAgAGEAIAByAGEAbgBnAGUAIABvAHIAIABhAHIAcgBhAHkALgBcAG4AIAAqACAAWwByAGEAbgBnAGUAOgAgAFIAYQBuAGcAZQAvAEEAcgByAGEAeQBdAFwAbgAgACoALwBcAG4ATQBpAG4AIAA9ACAATABBAE0AQgBEAEEAKAByAGEAbgBnAGUALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAZgBsAGEAdAB0AGUAbgBlAGQAXwBjAG8AbAAsACAAVABPAEMATwBMACgAcgBhAG4AZwBlACwAIAAxACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIABJAEYAKABPAFIAKABJAFMARQBSAFIATwBSACgAZgBsAGEAdAB0AGUAbgBlAGQAXwBjAG8AbAApACwAIABSAE8AVwBTACgAZgBsAGEAdAB0AGUAbgBlAGQAXwBjAG8AbAApACAAPQAgADAAKQAsACAAXAAiADAAXAAiACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFQAcgBlAGUAQwBvAG0AcABhAHIAZQAoAE0AQQBQACgAZgBsAGEAdAB0AGUAbgBlAGQAXwBjAG8AbAAsACAAQgBpAGcASQBuAHQALgBOAG8AcgBtACkALAAgAC0AMQApAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgAvACoAKgBcAG4AIAAqACAAUgBlAHQAdQByAG4AcwAgAHQAaABlACAAbQBhAHgAaQBtAHUAbQAgAEIAaQBnAEkAbgB0ACAAZgByAG8AbQAgAGEAIAByAGEAbgBnAGUAIABvAHIAIABhAHIAcgBhAHkALgBcAG4AIAAqACAAWwByAGEAbgBnAGUAOgAgAFIAYQBuAGcAZQAvAEEAcgByAGEAeQBdAFwAbgAgACoALwBcAG4ATQBhAHgAIAA9ACAATABBAE0AQgBEAEEAKAByAGEAbgBnAGUALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAZgBsAGEAdAB0AGUAbgBlAGQAXwBjAG8AbAAsACAAVABPAEMATwBMACgAcgBhAG4AZwBlACwAIAAxACkALABcAG4AXABuACAAIAAgACAAIAAgACAAIABJAEYAKABPAFIAKABJAFMARQBSAFIATwBSACgAZgBsAGEAdAB0AGUAbgBlAGQAXwBjAG8AbAApACwAIABSAE8AVwBTACgAZgBsAGEAdAB0AGUAbgBlAGQAXwBjAG8AbAApACAAPQAgADAAKQAsACAAXAAiADAAXAAiACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFQAcgBlAGUAQwBvAG0AcABhAHIAZQAoAE0AQQBQACgAZgBsAGEAdAB0AGUAbgBlAGQAXwBjAG8AbAAsACAAQgBpAGcASQBuAHQALgBOAG8AcgBtACkALAAgADEAKQBcAG4AIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AKQA7ACIAfQBdACwAIgBwAHIAbwBqAGUAYwB0AE4AYQBtAGUAcwAiADoAWwAiAHQAZQBzAHQAXwBCAGkAZwBJAG4AdAAuAEsAbgB1AHQAaABEAGkAdgBpAHMAaQBvAG4AIgAsACIAdABlAHMAdABfAEIAaQBnAEkAbgB0AC4ATgBlAHcAdABvAG4AUgBhAHAAaABzAG8AbgBEAGkAdgBpAHMAaQBvAG4AIgAsACIAdABlAHMAdABfAEIAaQBnAEkAbgB0AC4ARABpAHYAaQBzAGkAbwBuAEEAbABnAG8AcgBpAHQAaABtAHMAIgAsACIAdABlAHMAdABfAEIAaQBnAEkAbgB0AC4ARABpAHYAaQBzAGkAbwBuAEEAbABnAG8AcgBpAHQAaABtAEMAbwBtAHAAYQByAGkAcwBvAG4AIgAsACIAdABlAHMAdABfAEIAaQBnAEkAbgB0AC4ARABpAHYAaQBzAGkAbwBuAEIAZQBuAGMAaABtAGEAcgBrAEMAYQBzAGUAcwAiACwAIgB0AGUAcwB0AF8AQgBpAGcASQBuAHQALgBBAHMAeQBtAG0AZQB0AHIAaQBjAEEAQgBHAHIAaQBkACIALAAiAHQAZQBzAHQAXwBCAGkAZwBJAG4AdAAuAEYAYQBjAHQAbwByAGkAYQBsAEEAbABnAG8AcgBpAHQAaABtAHMAIgAsACIAdABlAHMAdABfAEIAaQBnAEkAbgB0AC4ARgBhAGMAdABvAHIAaQBhAGwAQwBvAG0AcABhAHIAaQBzAG8AbgAiACwAIgBjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBTAGEAZgBlAEsAIgAsACIAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwBwAGwAaQB0ACIALAAiAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAE0AZQByAGcAZQAiACwAIgBjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBDAGEAcgByAHkAIgAsACIAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBDAG8AbQBwAGEAcgBlACIALAAiAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFUAQQBkAGQAIgAsACIAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBTAHUAYgAiACwAIgBjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBVAE0AYQB0AHIAaQB4AFMAdQBtACIALAAiAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAEEAZABkAFMAdQBiAFIAbwB1AHQAZQByACIALAAiAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFUATQB1AGwAIgAsACIAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4ARgBpAG4AZABRAHUAbwB0AGkAZQBuAHQATABpAG0AYgAiACwAIgBjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBLAG4AdQB0AGgARABpAHYAIgAsACIAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4ARABpAHYAUgBvAHUAdABlAHIAIgAsACIAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4ATgBlAHcAdABvAG4AUgBhAHAAaABzAG8AbgBTAGUAZQBkACIALAAiAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAE4AZQB3AHQAbwBuAFIAYQBwAGgAcwBvAG4AUgBlAGMAaQBwAHIAbwBjAGEAbAAiACwAIgBjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBOAGUAdwB0AG8AbgBSAGEAcABoAHMAbwBuAEQAaQB2ACIALAAiAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFUAUABvAHcAIgAsACIAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AVQBTAHEAcgB0ACIALAAiAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAE4AYQB0AGkAdgBlAFAAcgBpAG0AZQBzACIALAAiAGMAbwByAGUAXwBCAGkAZwBJAG4AdAAuAFUAVABlAHgAdABNAHUAbAAiACwAIgBjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBUAGUAeAB0AFQAcgBlAGUAUAByAG8AZAAiACwAIgBjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBOAGEAdABpAHYAZQBTAHcAaQBuAGcARQB4AHAAbwBuAGUAbgB0AHMAIgAsACIAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUwB3AGkAbgBnAFQAZQByAG0AIgAsACIAYwBvAHIAZQBfAEIAaQBnAEkAbgB0AC4AUAByAGkAbQBlAFMAdwBpAG4AZwBLAGUAcgBuAGUAbAAiACwAIgBjAG8AcgBlAF8AQgBpAGcASQBuAHQALgBUAHIAZQBlAEMAbwBtAHAAYQByAGUAIgAsACIAQgBpAGcASQBuAHQALgBOAG8AcgBtACIALAAiAEIAaQBnAEkAbgB0AC4AUwBpAGcAbgAiACwAIgBCAGkAZwBJAG4AdAAuAEkAcwBaAGUAcgBvACIALAAiAEIAaQBnAEkAbgB0AC4ASQBzAE4AZQBnACIALAAiAEIAaQBnAEkAbgB0AC4ASQBzAEUAdgBlAG4AIgAsACIAQgBpAGcASQBuAHQALgBJAHMATwBkAGQAIgAsACIAQgBpAGcASQBuAHQALgBBAGIAcwAiACwAIgBCAGkAZwBJAG4AdAAuAEMAbwBtAHAAYQByAGUAIgAsACIAQgBpAGcASQBuAHQALgBBAGQAZAAiACwAIgBCAGkAZwBJAG4AdAAuAFMAdQBiACIALAAiAEIAaQBnAEkAbgB0AC4AUwB1AG0AIgAsACIAQgBpAGcASQBuAHQALgBNAHUAbAAiACwAIgBCAGkAZwBJAG4AdAAuAFIAYQBuAGQAQQByAHIAYQB5ACIALAAiAEIAaQBnAEkAbgB0AC4ARABpAHYATQBvAGQAIgAsACIAQgBpAGcASQBuAHQALgBEAGkAdgAiACwAIgBCAGkAZwBJAG4AdAAuAE0AbwBkACIALAAiAEIAaQBnAEkAbgB0AC4AUABvAHcAIgAsACIAQgBpAGcASQBuAHQALgBTAHEAcgB0ACIALAAiAEIAaQBnAEkAbgB0AC4ARgBhAGMAdAAiACwAIgBCAGkAZwBJAG4AdAAuAE0AaQBuACIALAAiAEIAaQBnAEkAbgB0AC4ATQBhAHgAIgBdACwAIgBsAG8AYwBhAGwAZQAiADoAewAiAGwAaQBzAHQAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgByAG8AdwBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGMAbwBsAHUAbQBuAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgB0AGgAbwB1AHMAYQBuAGQAcwBQAG8AcwBpAHQAaQBvAG4AcwAiADoAWwAzAF0ALAAiAGQAZQBjAGkAbQBhAGwAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALgAiACwAIgBkAGEAdABlAE8AcgBkAGUAcgAiADoAIgBEAE0AWQAiACwAIgBjAHUAcgByAGUAbgBjAHkAUwB5AG0AYgBvAGwAIgA6ACIAJAAiACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsAEwAZQBhAGQAIgA6AHQAcgB1AGUALAAiAGkAcwBDAHUAcgByAGUAbgBjAHkAUwBlAHAAQgB5AFMAcABhAGMAZQAiADoAZgBhAGwAcwBlACwAIgByAG8AdwBMAGUAdAB0AGUAcgAiADoAIgBSACIALAAiAGMAbwBsAHUAbQBuAEwAZQB0AHQAZQByACIAOgAiAEMAIgAsACIAcgBjAEwAZQBmAHQAQgByAGEAYwBrAGUAdAAiADoAIgBbACIALAAiAHIAYwBSAGkAZwBoAHQAQgByAGEAYwBrAGUAdAAiADoAIgBdACIALAAiAHMAdABhAHQAZQBtAGUAbgB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiADsAIgAsACIAbABvAGMAYQBsAGUATgBhAG0AZQAiADoAIgBlAG4ALQB1AHMAIgB9AH0A</AFEJSONBlob>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>